<commit_message>
Aggiornamento dati Dynamica 2026-07-21
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 17/07/2026  |  Ultimo aggiornamento: 20/07/2026 11:37</t>
+          <t>Periodo: 01/07/2026 - 20/07/2026  |  Ultimo aggiornamento: 21/07/2026 12:02</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1054,26 +1054,26 @@
       <c r="L5" s="119" t="n"/>
       <c r="M5" s="119" t="n"/>
       <c r="N5" s="119" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="O5" s="119" t="n"/>
       <c r="P5" s="117" t="n">
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>5209.677419354838</v>
+        <v>6129.032258064516</v>
       </c>
       <c r="R5" s="117" t="n">
         <v>5794.215866</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>584.5384466451615</v>
+        <v>-334.8163920645165</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.1122024262910217</v>
+        <v>-0.0546279376526316</v>
       </c>
       <c r="U5" s="117" t="n">
-        <v>98.20704857627118</v>
+        <v>87.79114948484848</v>
       </c>
       <c r="V5" s="117" t="n"/>
       <c r="W5" s="120" t="inlineStr">
@@ -1117,7 +1117,7 @@
       <c r="L6" s="119" t="n"/>
       <c r="M6" s="119" t="n"/>
       <c r="N6" s="119" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="O6" s="119" t="n"/>
       <c r="P6" s="117" t="n"/>
@@ -1168,26 +1168,26 @@
       <c r="L7" s="119" t="n"/>
       <c r="M7" s="119" t="n"/>
       <c r="N7" s="119" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="O7" s="119" t="n"/>
       <c r="P7" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>822.5806451612904</v>
+        <v>967.741935483871</v>
       </c>
       <c r="R7" s="117" t="n">
         <v>1074.27638</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>251.6957348387096</v>
+        <v>106.534444516129</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>0.3059830501960784</v>
+        <v>0.1100855926666666</v>
       </c>
       <c r="U7" s="117" t="n">
-        <v>18.52200655172414</v>
+        <v>16.27691484848485</v>
       </c>
       <c r="V7" s="117" t="n"/>
       <c r="W7" s="120" t="inlineStr">
@@ -1231,7 +1231,7 @@
       <c r="L8" s="119" t="n"/>
       <c r="M8" s="119" t="n"/>
       <c r="N8" s="119" t="n">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="O8" s="119" t="n"/>
       <c r="P8" s="117" t="n"/>
@@ -1282,26 +1282,26 @@
       <c r="L9" s="119" t="n"/>
       <c r="M9" s="119" t="n"/>
       <c r="N9" s="119" t="n">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="O9" s="119" t="n"/>
       <c r="P9" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>5483.870967741936</v>
+        <v>6451.612903225806</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>5657.94</v>
+        <v>6251.68</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>174.069032258064</v>
+        <v>-199.9329032258056</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.0317419999999999</v>
+        <v>-0.0309895999999998</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>97.55068965517241</v>
+        <v>96.17969230769231</v>
       </c>
       <c r="V9" s="117" t="n"/>
       <c r="W9" s="120" t="inlineStr">
@@ -1328,33 +1328,45 @@
       </c>
       <c r="H10" s="123" t="n"/>
       <c r="I10" s="125" t="n"/>
-      <c r="J10" s="123" t="n"/>
-      <c r="K10" s="125" t="n"/>
-      <c r="L10" s="125" t="n"/>
-      <c r="M10" s="125" t="n"/>
+      <c r="J10" s="123" t="n">
+        <v>45</v>
+      </c>
+      <c r="K10" s="125" t="n">
+        <v>466.6666666666667</v>
+      </c>
+      <c r="L10" s="125" t="n">
+        <v>15.05376344086022</v>
+      </c>
+      <c r="M10" s="125" t="n">
+        <v>301.0752688172043</v>
+      </c>
       <c r="N10" s="125" t="n">
-        <v>291</v>
-      </c>
-      <c r="O10" s="125" t="n"/>
+        <v>328</v>
+      </c>
+      <c r="O10" s="125" t="n">
+        <v>26.92473118279565</v>
+      </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>11516.12903225806</v>
+        <v>13548.38709677419</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>12526.432246</v>
+        <v>13120.172246</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>1010.303213741934</v>
+        <v>-428.2148507741931</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>0.0877294107170867</v>
+        <v>-0.0316063342238094</v>
       </c>
       <c r="U10" s="123" t="n">
-        <v>43.04615892096219</v>
-      </c>
-      <c r="V10" s="123" t="n"/>
+        <v>40.0005251402439</v>
+      </c>
+      <c r="V10" s="123" t="n">
+        <v>-4.999474859756099</v>
+      </c>
       <c r="W10" s="126" t="n"/>
     </row>
     <row r="11" ht="36" customHeight="1" s="74">
@@ -1405,28 +1417,28 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>128.1943862589024</v>
+        <v>150.8169250104734</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>61</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-67.19438625890237</v>
+        <v>-89.8169250104734</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>4935.483870967741</v>
+        <v>5806.451612903225</v>
       </c>
       <c r="R11" s="117" t="n">
         <v>5490.756616000001</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>555.2727450322591</v>
+        <v>-315.6949969032248</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.1125062424575165</v>
+        <v>-0.0543696939111109</v>
       </c>
       <c r="U11" s="117" t="n">
         <v>90.01240354098361</v>
@@ -1475,7 +1487,7 @@
       <c r="L12" s="119" t="n"/>
       <c r="M12" s="119" t="n"/>
       <c r="N12" s="119" t="n">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="O12" s="119" t="n"/>
       <c r="P12" s="117" t="n"/>
@@ -1535,34 +1547,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>64.51612903225806</v>
+        <v>75.90132827324479</v>
       </c>
       <c r="N13" s="119" t="n">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>33.48387096774194</v>
+        <v>35.09867172675521</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>2193.548387096774</v>
+        <v>2580.645161290322</v>
       </c>
       <c r="R13" s="117" t="n">
         <v>3069.617174</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>876.0687869032258</v>
+        <v>488.9720127096775</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.3993842999117647</v>
+        <v>0.189476654925</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>31.3226242244898</v>
+        <v>27.65420877477477</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>-2.677375775510203</v>
+        <v>-6.345791225225227</v>
       </c>
       <c r="W13" s="120" t="inlineStr">
         <is>
@@ -1618,28 +1630,28 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>14.43123938879457</v>
+        <v>16.97792869269949</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>5</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-9.431239388794566</v>
+        <v>-11.97792869269949</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>548.3870967741935</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="R14" s="117" t="n">
         <v>510.988722</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-37.39837477419354</v>
+        <v>-134.1725683225806</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.0681970363529411</v>
+        <v>-0.2079674808999999</v>
       </c>
       <c r="U14" s="117" t="n">
         <v>102.1977444</v>
@@ -1701,28 +1713,28 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>2.193548387096774</v>
+        <v>2.580645161290323</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-0.193548387096774</v>
+        <v>-0.5806451612903225</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>548.3870967741935</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="R15" s="117" t="n">
         <v>630.160373</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>81.77327622580651</v>
+        <v>-15.00091732258056</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>0.1491159742941177</v>
+        <v>-0.0232514218499998</v>
       </c>
       <c r="U15" s="117" t="n">
         <v>315.0801865</v>
@@ -1818,7 +1830,7 @@
       <c r="L17" s="119" t="n"/>
       <c r="M17" s="119" t="n"/>
       <c r="N17" s="119" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O17" s="119" t="n"/>
       <c r="P17" s="117" t="n"/>
@@ -1878,34 +1890,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>2.28494623655914</v>
+        <v>2.688172043010753</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>4</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>1.71505376344086</v>
+        <v>1.311827956989247</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>274.1935483870968</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>283.27</v>
+        <v>311.38</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>9.076451612903211</v>
+        <v>-11.20064516129031</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>0.0331023529411764</v>
+        <v>-0.0347219999999999</v>
       </c>
       <c r="U18" s="117" t="n">
-        <v>70.8175</v>
+        <v>77.845</v>
       </c>
       <c r="V18" s="117" t="n">
-        <v>-49.1825</v>
+        <v>-42.155</v>
       </c>
       <c r="W18" s="120" t="inlineStr"/>
     </row>
@@ -1957,34 +1969,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>6.854838709677419</v>
+        <v>8.064516129032258</v>
       </c>
       <c r="N19" s="119" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>24.14516129032258</v>
+        <v>23.93548387096774</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>274.1935483870968</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>322.95</v>
+        <v>355.21</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>48.75645161290322</v>
+        <v>32.62935483870967</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>0.1778176470588235</v>
+        <v>0.1011509999999999</v>
       </c>
       <c r="U19" s="117" t="n">
-        <v>10.41774193548387</v>
+        <v>11.1003125</v>
       </c>
       <c r="V19" s="117" t="n">
-        <v>-29.58225806451613</v>
+        <v>-28.8996875</v>
       </c>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
@@ -2036,34 +2048,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>6.093189964157706</v>
+        <v>7.168458781362007</v>
       </c>
       <c r="N20" s="119" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>10.9068100358423</v>
+        <v>11.83154121863799</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>548.3870967741935</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>581.76</v>
+        <v>639.04</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>33.37290322580645</v>
+        <v>-6.121290322580649</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>0.0608564705882353</v>
+        <v>-0.009488</v>
       </c>
       <c r="U20" s="117" t="n">
-        <v>34.22117647058823</v>
+        <v>33.63368421052631</v>
       </c>
       <c r="V20" s="117" t="n">
-        <v>-55.77882352941177</v>
+        <v>-56.36631578947369</v>
       </c>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
@@ -2115,34 +2127,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>428.4274193548387</v>
+        <v>504.0322580645162</v>
       </c>
       <c r="N21" s="119" t="n">
-        <v>367</v>
+        <v>417</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-61.42741935483872</v>
+        <v>-87.03225806451616</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>5483.870967741936</v>
+        <v>6451.612903225806</v>
       </c>
       <c r="R21" s="117" t="n">
-        <v>7444.1</v>
+        <v>8745.66</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>1960.229032258065</v>
+        <v>2294.047096774194</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>0.3574535294117647</v>
+        <v>0.3555773000000001</v>
       </c>
       <c r="U21" s="117" t="n">
-        <v>20.28365122615804</v>
+        <v>20.97280575539568</v>
       </c>
       <c r="V21" s="117" t="n">
-        <v>7.483651226158038</v>
+        <v>8.172805755395682</v>
       </c>
       <c r="W21" s="120" t="inlineStr">
         <is>
@@ -2198,34 +2210,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>20.56451612903226</v>
+        <v>24.19354838709678</v>
       </c>
       <c r="N22" s="119" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>0.4354838709677402</v>
+        <v>-2.193548387096776</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>822.5806451612904</v>
+        <v>967.741935483871</v>
       </c>
       <c r="R22" s="117" t="n">
         <v>1057.013242</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>234.4325968387096</v>
+        <v>89.27130651612902</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>0.2849964902745097</v>
+        <v>0.0922470167333333</v>
       </c>
       <c r="U22" s="117" t="n">
-        <v>50.3339639047619</v>
+        <v>48.04605645454546</v>
       </c>
       <c r="V22" s="117" t="n">
-        <v>10.3339639047619</v>
+        <v>8.046056454545457</v>
       </c>
       <c r="W22" s="120" t="inlineStr"/>
     </row>
@@ -2277,34 +2289,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>54.83870967741935</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="N23" s="119" t="n">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>47.16129032258065</v>
+        <v>49.48387096774194</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>822.5806451612904</v>
+        <v>967.741935483871</v>
       </c>
       <c r="R23" s="117" t="n">
         <v>1241.040684</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>418.4600388387097</v>
+        <v>273.2987485161291</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.5087161256470588</v>
+        <v>0.2824087068000001</v>
       </c>
       <c r="U23" s="117" t="n">
-        <v>12.16706552941176</v>
+        <v>10.88632178947368</v>
       </c>
       <c r="V23" s="117" t="n">
-        <v>-2.832934470588235</v>
+        <v>-4.113678210526315</v>
       </c>
       <c r="W23" s="120" t="inlineStr">
         <is>
@@ -2360,34 +2372,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>21.09181141439206</v>
+        <v>24.81389578163772</v>
       </c>
       <c r="N24" s="119" t="n">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>37.90818858560795</v>
+        <v>42.18610421836229</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>548.3870967741935</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="R24" s="117" t="n">
-        <v>1016.68</v>
+        <v>1107.29</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>468.2929032258064</v>
+        <v>462.1287096774194</v>
       </c>
       <c r="T24" s="118" t="n">
-        <v>0.8539458823529411</v>
+        <v>0.7162995</v>
       </c>
       <c r="U24" s="117" t="n">
-        <v>17.23186440677966</v>
+        <v>16.52671641791045</v>
       </c>
       <c r="V24" s="117" t="n">
-        <v>-8.76813559322034</v>
+        <v>-9.473283582089554</v>
       </c>
       <c r="W24" s="120" t="inlineStr"/>
     </row>
@@ -2428,17 +2440,19 @@
       <c r="L25" s="119" t="n"/>
       <c r="M25" s="119" t="n"/>
       <c r="N25" s="119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O25" s="119" t="n"/>
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>144.47</v>
+        <v>334.82</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
-      <c r="U25" s="117" t="n"/>
+      <c r="U25" s="117" t="n">
+        <v>334.82</v>
+      </c>
       <c r="V25" s="117" t="n"/>
       <c r="W25" s="120" t="inlineStr"/>
     </row>
@@ -2474,34 +2488,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>749.4907345531284</v>
+        <v>881.7538053566217</v>
       </c>
       <c r="N26" s="125" t="n">
-        <v>863</v>
+        <v>967</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>113.5092654468716</v>
+        <v>85.24619464337832</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>17000</v>
+        <v>20000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>21792.806811</v>
+        <v>23492.976811</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>4792.806811000002</v>
+        <v>3492.976811</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>0.2819298124117648</v>
+        <v>0.17464884055</v>
       </c>
       <c r="U26" s="123" t="n">
-        <v>25.25238332676709</v>
+        <v>24.29470197621509</v>
       </c>
       <c r="V26" s="123" t="n">
-        <v>2.570315068597139</v>
+        <v>1.612633718045142</v>
       </c>
       <c r="W26" s="126" t="n"/>
     </row>
@@ -2549,28 +2563,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>243.7275985663082</v>
+        <v>286.7383512544803</v>
       </c>
       <c r="N27" s="119" t="n">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-68.72759856630825</v>
+        <v>-99.73835125448028</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>2193.548387096774</v>
+        <v>2580.645161290322</v>
       </c>
       <c r="R27" s="117" t="n">
-        <v>1575</v>
+        <v>1683</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-618.5483870967741</v>
+        <v>-897.6451612903224</v>
       </c>
       <c r="T27" s="118" t="n">
-        <v>-0.281985294117647</v>
+        <v>-0.3478374999999999</v>
       </c>
       <c r="U27" s="117" t="n">
         <v>9</v>
@@ -2624,28 +2638,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>360.7809847198643</v>
+        <v>424.4482173174873</v>
       </c>
       <c r="N28" s="119" t="n">
-        <v>360</v>
+        <v>371</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-0.7809847198642501</v>
+        <v>-53.44821731748732</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>161.2903225806452</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>2741.935483870968</v>
+        <v>3225.806451612903</v>
       </c>
       <c r="R28" s="117" t="n">
-        <v>2736</v>
+        <v>2819.6</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-5.935483870967801</v>
+        <v>-406.206451612903</v>
       </c>
       <c r="T28" s="118" t="n">
-        <v>-0.0021647058823529</v>
+        <v>-0.1259239999999999</v>
       </c>
       <c r="U28" s="117" t="n">
         <v>7.6</v>
@@ -2699,28 +2713,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>137.0967741935484</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="N29" s="119" t="n">
-        <v>223</v>
+        <v>240</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>85.90322580645162</v>
+        <v>78.70967741935485</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>1096.774193548387</v>
+        <v>1290.322580645161</v>
       </c>
       <c r="R29" s="117" t="n">
-        <v>1784</v>
+        <v>1920</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>687.2258064516129</v>
+        <v>629.6774193548388</v>
       </c>
       <c r="T29" s="118" t="n">
-        <v>0.6265882352941177</v>
+        <v>0.4880000000000001</v>
       </c>
       <c r="U29" s="117" t="n">
         <v>8</v>
@@ -2762,34 +2776,34 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>741.6053574797209</v>
+        <v>872.4768911526128</v>
       </c>
       <c r="N30" s="125" t="n">
-        <v>758</v>
+        <v>798</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>16.39464252027915</v>
+        <v>-74.47689115261278</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>354.8387096774193</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>6032.258064516129</v>
+        <v>7096.774193548386</v>
       </c>
       <c r="R30" s="123" t="n">
-        <v>6095</v>
+        <v>6422.6</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>62.7419354838712</v>
+        <v>-674.174193548386</v>
       </c>
       <c r="T30" s="124" t="n">
-        <v>0.0104010695187166</v>
+        <v>-0.0949972727272725</v>
       </c>
       <c r="U30" s="123" t="n">
-        <v>8.040897097625329</v>
+        <v>8.048370927318297</v>
       </c>
       <c r="V30" s="123" t="n">
-        <v>-0.0931569564287251</v>
+        <v>-0.0856831267357574</v>
       </c>
       <c r="W30" s="126" t="n"/>
     </row>
@@ -2816,43 +2830,43 @@
         <v>84.56183862433862</v>
       </c>
       <c r="J31" s="129" t="n">
-        <v>23.16979253139447</v>
+        <v>19.77572292204534</v>
       </c>
       <c r="K31" s="131" t="n">
-        <v>2719.057579589313</v>
+        <v>3185.72424625598</v>
       </c>
       <c r="L31" s="131" t="n">
-        <v>87.71153482546173</v>
+        <v>102.7652982663219</v>
       </c>
       <c r="M31" s="131" t="n">
-        <v>1491.096092032849</v>
+        <v>2055.305965326439</v>
       </c>
       <c r="N31" s="131" t="n">
-        <v>1912</v>
+        <v>2093</v>
       </c>
       <c r="O31" s="131" t="n">
-        <v>420.9039079671506</v>
+        <v>37.69403467356096</v>
       </c>
       <c r="P31" s="129" t="n">
         <v>2032.258064516129</v>
       </c>
       <c r="Q31" s="129" t="n">
-        <v>34548.38709677419</v>
+        <v>40645.16129032258</v>
       </c>
       <c r="R31" s="129" t="n">
-        <v>40414.239057</v>
+        <v>43035.749057</v>
       </c>
       <c r="S31" s="129" t="n">
-        <v>5865.851960225809</v>
+        <v>2390.587766677425</v>
       </c>
       <c r="T31" s="130" t="n">
-        <v>0.1697865646750701</v>
+        <v>0.0588160482277779</v>
       </c>
       <c r="U31" s="129" t="n">
-        <v>21.13715431851464</v>
+        <v>20.56175301337793</v>
       </c>
       <c r="V31" s="129" t="n">
-        <v>-2.032638212879828</v>
+        <v>0.7860300913325879</v>
       </c>
       <c r="W31" s="132" t="n"/>
     </row>
@@ -3115,13 +3129,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3155,25 +3169,25 @@
       <c r="L2" s="135" t="n"/>
       <c r="N2" s="135" t="n"/>
       <c r="R2" t="n">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="T2" s="135" t="n">
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>5209.677419354838</v>
+        <v>6129.032258064516</v>
       </c>
       <c r="V2" s="135" t="n">
         <v>5794.215866</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>584.5384466451615</v>
+        <v>-334.8163920645165</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.1122024262910217</v>
+        <v>-0.0546279376526316</v>
       </c>
       <c r="Y2" s="135" t="n">
-        <v>98.20704857627118</v>
+        <v>87.79114948484848</v>
       </c>
       <c r="Z2" s="135" t="n"/>
       <c r="AA2" t="inlineStr">
@@ -3190,7 +3204,7 @@
       <c r="AD2" s="137" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>google:stale;google:includes_excel_row_3</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -3206,13 +3220,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3242,7 +3256,7 @@
       <c r="L3" s="135" t="n"/>
       <c r="N3" s="135" t="n"/>
       <c r="R3" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="T3" s="135" t="n"/>
       <c r="U3" s="135" t="n"/>
@@ -3260,7 +3274,7 @@
       <c r="AD3" s="137" t="inlineStr"/>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>google:rolled_up_to_excel_row_2</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -3276,13 +3290,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3316,25 +3330,25 @@
       <c r="L4" s="135" t="n"/>
       <c r="N4" s="135" t="n"/>
       <c r="R4" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="T4" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>822.5806451612904</v>
+        <v>967.741935483871</v>
       </c>
       <c r="V4" s="135" t="n">
         <v>1074.27638</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>251.6957348387096</v>
+        <v>106.534444516129</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>0.3059830501960784</v>
+        <v>0.1100855926666666</v>
       </c>
       <c r="Y4" s="135" t="n">
-        <v>18.52200655172414</v>
+        <v>16.27691484848485</v>
       </c>
       <c r="Z4" s="135" t="n"/>
       <c r="AA4" t="inlineStr">
@@ -3351,7 +3365,7 @@
       <c r="AD4" s="137" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>google:stale;google:includes_excel_row_5</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -3367,13 +3381,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3403,7 +3417,7 @@
       <c r="L5" s="135" t="n"/>
       <c r="N5" s="135" t="n"/>
       <c r="R5" t="n">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="T5" s="135" t="n"/>
       <c r="U5" s="135" t="n"/>
@@ -3421,7 +3435,7 @@
       <c r="AD5" s="137" t="inlineStr"/>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>google:rolled_up_to_excel_row_4</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -3437,13 +3451,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3477,25 +3491,25 @@
       <c r="L6" s="135" t="n"/>
       <c r="N6" s="135" t="n"/>
       <c r="R6" t="n">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>5483.870967741936</v>
+        <v>6451.612903225806</v>
       </c>
       <c r="V6" s="135" t="n">
-        <v>5657.94</v>
+        <v>6251.68</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>174.069032258064</v>
+        <v>-199.9329032258056</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>0.0317419999999999</v>
+        <v>-0.0309895999999998</v>
       </c>
       <c r="Y6" s="135" t="n">
-        <v>97.55068965517241</v>
+        <v>96.17969230769231</v>
       </c>
       <c r="Z6" s="135" t="n"/>
       <c r="AA6" t="inlineStr">
@@ -3512,7 +3526,7 @@
       <c r="AD6" s="137" t="inlineStr"/>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -3528,13 +3542,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E7" t="n">
         <v>26</v>
@@ -3581,28 +3595,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q7" t="n">
-        <v>243.7275985663082</v>
+        <v>286.7383512544803</v>
       </c>
       <c r="R7" t="n">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="S7" t="n">
-        <v>-68.72759856630825</v>
+        <v>-99.73835125448028</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>2193.548387096774</v>
+        <v>2580.645161290322</v>
       </c>
       <c r="V7" s="135" t="n">
-        <v>1575</v>
+        <v>1683</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>-618.5483870967741</v>
+        <v>-897.6451612903224</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>-0.281985294117647</v>
+        <v>-0.3478374999999999</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>9</v>
@@ -3615,7 +3629,7 @@
       <c r="AD7" s="137" t="inlineStr"/>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -3631,13 +3645,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E8" t="n">
         <v>25</v>
@@ -3684,28 +3698,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q8" t="n">
-        <v>360.7809847198643</v>
+        <v>424.4482173174873</v>
       </c>
       <c r="R8" t="n">
-        <v>360</v>
+        <v>371</v>
       </c>
       <c r="S8" t="n">
-        <v>-0.7809847198642501</v>
+        <v>-53.44821731748732</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>161.2903225806452</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>2741.935483870968</v>
+        <v>3225.806451612903</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>2736</v>
+        <v>2819.6</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>-5.935483870967801</v>
+        <v>-406.206451612903</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>-0.0021647058823529</v>
+        <v>-0.1259239999999999</v>
       </c>
       <c r="Y8" s="135" t="n">
         <v>7.6</v>
@@ -3718,7 +3732,7 @@
       <c r="AD8" s="137" t="inlineStr"/>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -3734,13 +3748,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3787,28 +3801,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>137.0967741935484</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="R9" t="n">
-        <v>223</v>
+        <v>240</v>
       </c>
       <c r="S9" t="n">
-        <v>85.90322580645162</v>
+        <v>78.70967741935485</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>1096.774193548387</v>
+        <v>1290.322580645161</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>1784</v>
+        <v>1920</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>687.2258064516129</v>
+        <v>629.6774193548388</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.6265882352941177</v>
+        <v>0.4880000000000001</v>
       </c>
       <c r="Y9" s="135" t="n">
         <v>8</v>
@@ -3821,7 +3835,7 @@
       <c r="AD9" s="137" t="inlineStr"/>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -3837,13 +3851,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E10" t="n">
         <v>9</v>
@@ -3890,28 +3904,28 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q10" t="n">
-        <v>128.1943862589024</v>
+        <v>150.8169250104734</v>
       </c>
       <c r="R10" t="n">
         <v>61</v>
       </c>
       <c r="S10" t="n">
-        <v>-67.19438625890237</v>
+        <v>-89.8169250104734</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>4935.483870967741</v>
+        <v>5806.451612903225</v>
       </c>
       <c r="V10" s="135" t="n">
         <v>5490.756616000001</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>555.2727450322591</v>
+        <v>-315.6949969032248</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.1125062424575165</v>
+        <v>-0.0543696939111109</v>
       </c>
       <c r="Y10" s="135" t="n">
         <v>90.01240354098361</v>
@@ -3933,7 +3947,7 @@
       <c r="AD10" s="137" t="inlineStr"/>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>google:stale;google:includes_excel_row_10</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -3949,13 +3963,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E11" t="n">
         <v>10</v>
@@ -3985,7 +3999,7 @@
       <c r="L11" s="135" t="n"/>
       <c r="N11" s="135" t="n"/>
       <c r="R11" t="n">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="T11" s="135" t="n"/>
       <c r="U11" s="135" t="n"/>
@@ -4003,7 +4017,7 @@
       <c r="AD11" s="137" t="inlineStr"/>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>google:rolled_up_to_excel_row_9</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -4019,13 +4033,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E12" t="n">
         <v>8</v>
@@ -4072,34 +4086,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q12" t="n">
-        <v>64.51612903225806</v>
+        <v>75.90132827324479</v>
       </c>
       <c r="R12" t="n">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="S12" t="n">
-        <v>33.48387096774194</v>
+        <v>35.09867172675521</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>2193.548387096774</v>
+        <v>2580.645161290322</v>
       </c>
       <c r="V12" s="135" t="n">
         <v>3069.617174</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>876.0687869032258</v>
+        <v>488.9720127096775</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.3993842999117647</v>
+        <v>0.189476654925</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>31.3226242244898</v>
+        <v>27.65420877477477</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>-2.677375775510203</v>
+        <v>-6.345791225225227</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
@@ -4115,7 +4129,7 @@
       <c r="AD12" s="137" t="inlineStr"/>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>google:stale</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -4131,13 +4145,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4184,28 +4198,28 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>14.43123938879457</v>
+        <v>16.97792869269949</v>
       </c>
       <c r="R13" t="n">
         <v>5</v>
       </c>
       <c r="S13" t="n">
-        <v>-9.431239388794566</v>
+        <v>-11.97792869269949</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>548.3870967741935</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="V13" s="135" t="n">
         <v>510.988722</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-37.39837477419354</v>
+        <v>-134.1725683225806</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.0681970363529411</v>
+        <v>-0.2079674808999999</v>
       </c>
       <c r="Y13" s="135" t="n">
         <v>102.1977444</v>
@@ -4227,7 +4241,7 @@
       <c r="AD13" s="137" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>google:stale;google:includes_excel_row_12</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -4243,13 +4257,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -4296,28 +4310,28 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q14" t="n">
-        <v>2.193548387096774</v>
+        <v>2.580645161290323</v>
       </c>
       <c r="R14" t="n">
         <v>2</v>
       </c>
       <c r="S14" t="n">
-        <v>-0.193548387096774</v>
+        <v>-0.5806451612903225</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>548.3870967741935</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="V14" s="135" t="n">
         <v>630.160373</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>81.77327622580651</v>
+        <v>-15.00091732258056</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>0.1491159742941177</v>
+        <v>-0.0232514218499998</v>
       </c>
       <c r="Y14" s="135" t="n">
         <v>315.0801865</v>
@@ -4339,7 +4353,7 @@
       <c r="AD14" s="137" t="inlineStr"/>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>google:stale;google:includes_excel_row_14</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -4355,13 +4369,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E15" t="n">
         <v>14</v>
@@ -4409,7 +4423,7 @@
       <c r="AD15" s="137" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>google:rolled_up_to_excel_row_13</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -4425,13 +4439,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E16" t="n">
         <v>12</v>
@@ -4461,7 +4475,7 @@
       <c r="L16" s="135" t="n"/>
       <c r="N16" s="135" t="n"/>
       <c r="R16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T16" s="135" t="n"/>
       <c r="U16" s="135" t="n"/>
@@ -4479,7 +4493,7 @@
       <c r="AD16" s="137" t="inlineStr"/>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>google:rolled_up_to_excel_row_11</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -4495,13 +4509,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E17" t="n">
         <v>21</v>
@@ -4548,34 +4562,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q17" t="n">
-        <v>2.28494623655914</v>
+        <v>2.688172043010753</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
       </c>
       <c r="S17" t="n">
-        <v>1.71505376344086</v>
+        <v>1.311827956989247</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>274.1935483870968</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>283.27</v>
+        <v>311.38</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>9.076451612903211</v>
+        <v>-11.20064516129031</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>0.0331023529411764</v>
+        <v>-0.0347219999999999</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>70.8175</v>
+        <v>77.845</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>-49.1825</v>
+        <v>-42.155</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr">
@@ -4586,7 +4600,7 @@
       <c r="AD17" s="137" t="inlineStr"/>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
@@ -4602,13 +4616,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4655,34 +4669,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>6.854838709677419</v>
+        <v>8.064516129032258</v>
       </c>
       <c r="R18" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S18" t="n">
-        <v>24.14516129032258</v>
+        <v>23.93548387096774</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>274.1935483870968</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>322.95</v>
+        <v>355.21</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>48.75645161290322</v>
+        <v>32.62935483870967</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>0.1778176470588235</v>
+        <v>0.1011509999999999</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>10.41774193548387</v>
+        <v>11.1003125</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>-29.58225806451613</v>
+        <v>-28.8996875</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr">
@@ -4693,7 +4707,7 @@
       <c r="AD18" s="137" t="inlineStr"/>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
@@ -4709,13 +4723,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4762,34 +4776,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>6.093189964157706</v>
+        <v>7.168458781362007</v>
       </c>
       <c r="R19" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="S19" t="n">
-        <v>10.9068100358423</v>
+        <v>11.83154121863799</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>548.3870967741935</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="V19" s="135" t="n">
-        <v>581.76</v>
+        <v>639.04</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>33.37290322580645</v>
+        <v>-6.121290322580649</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>0.0608564705882353</v>
+        <v>-0.009488</v>
       </c>
       <c r="Y19" s="135" t="n">
-        <v>34.22117647058823</v>
+        <v>33.63368421052631</v>
       </c>
       <c r="Z19" s="135" t="n">
-        <v>-55.77882352941177</v>
+        <v>-56.36631578947369</v>
       </c>
       <c r="AB19" s="137" t="inlineStr"/>
       <c r="AC19" s="137" t="inlineStr">
@@ -4800,7 +4814,7 @@
       <c r="AD19" s="137" t="inlineStr"/>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
@@ -4816,13 +4830,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E20" t="n">
         <v>17</v>
@@ -4869,34 +4883,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q20" t="n">
-        <v>428.4274193548387</v>
+        <v>504.0322580645162</v>
       </c>
       <c r="R20" t="n">
-        <v>367</v>
+        <v>417</v>
       </c>
       <c r="S20" t="n">
-        <v>-61.42741935483872</v>
+        <v>-87.03225806451616</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>5483.870967741936</v>
+        <v>6451.612903225806</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>7444.1</v>
+        <v>8745.66</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>1960.229032258065</v>
+        <v>2294.047096774194</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>0.3574535294117647</v>
+        <v>0.3555773000000001</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>20.28365122615804</v>
+        <v>20.97280575539568</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>7.483651226158038</v>
+        <v>8.172805755395682</v>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
@@ -4912,7 +4926,7 @@
       <c r="AD20" s="137" t="inlineStr"/>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr">
@@ -4928,13 +4942,13 @@
         </is>
       </c>
       <c r="B21" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C21" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D21" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4981,34 +4995,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>20.56451612903226</v>
+        <v>24.19354838709678</v>
       </c>
       <c r="R21" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S21" t="n">
-        <v>0.4354838709677402</v>
+        <v>-2.193548387096776</v>
       </c>
       <c r="T21" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="135" t="n">
-        <v>822.5806451612904</v>
+        <v>967.741935483871</v>
       </c>
       <c r="V21" s="135" t="n">
         <v>1057.013242</v>
       </c>
       <c r="W21" s="135" t="n">
-        <v>234.4325968387096</v>
+        <v>89.27130651612902</v>
       </c>
       <c r="X21" s="136" t="n">
-        <v>0.2849964902745097</v>
+        <v>0.0922470167333333</v>
       </c>
       <c r="Y21" s="135" t="n">
-        <v>50.3339639047619</v>
+        <v>48.04605645454546</v>
       </c>
       <c r="Z21" s="135" t="n">
-        <v>10.3339639047619</v>
+        <v>8.046056454545457</v>
       </c>
       <c r="AB21" s="137" t="inlineStr">
         <is>
@@ -5019,7 +5033,7 @@
       <c r="AD21" s="137" t="inlineStr"/>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>google:stale</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
@@ -5035,13 +5049,13 @@
         </is>
       </c>
       <c r="B22" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C22" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D22" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -5088,34 +5102,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>54.83870967741935</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="R22" t="n">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="S22" t="n">
-        <v>47.16129032258065</v>
+        <v>49.48387096774194</v>
       </c>
       <c r="T22" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="135" t="n">
-        <v>822.5806451612904</v>
+        <v>967.741935483871</v>
       </c>
       <c r="V22" s="135" t="n">
         <v>1241.040684</v>
       </c>
       <c r="W22" s="135" t="n">
-        <v>418.4600388387097</v>
+        <v>273.2987485161291</v>
       </c>
       <c r="X22" s="136" t="n">
-        <v>0.5087161256470588</v>
+        <v>0.2824087068000001</v>
       </c>
       <c r="Y22" s="135" t="n">
-        <v>12.16706552941176</v>
+        <v>10.88632178947368</v>
       </c>
       <c r="Z22" s="135" t="n">
-        <v>-2.832934470588235</v>
+        <v>-4.113678210526315</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -5131,7 +5145,7 @@
       <c r="AD22" s="137" t="inlineStr"/>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>google:stale</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
@@ -5147,13 +5161,13 @@
         </is>
       </c>
       <c r="B23" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C23" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D23" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5200,34 +5214,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>21.09181141439206</v>
+        <v>24.81389578163772</v>
       </c>
       <c r="R23" t="n">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="S23" t="n">
-        <v>37.90818858560795</v>
+        <v>42.18610421836229</v>
       </c>
       <c r="T23" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="135" t="n">
-        <v>548.3870967741935</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="V23" s="135" t="n">
-        <v>1016.68</v>
+        <v>1107.29</v>
       </c>
       <c r="W23" s="135" t="n">
-        <v>468.2929032258064</v>
+        <v>462.1287096774194</v>
       </c>
       <c r="X23" s="136" t="n">
-        <v>0.8539458823529411</v>
+        <v>0.7162995</v>
       </c>
       <c r="Y23" s="135" t="n">
-        <v>17.23186440677966</v>
+        <v>16.52671641791045</v>
       </c>
       <c r="Z23" s="135" t="n">
-        <v>-8.76813559322034</v>
+        <v>-9.473283582089554</v>
       </c>
       <c r="AB23" s="137" t="inlineStr"/>
       <c r="AC23" s="137" t="inlineStr">
@@ -5238,7 +5252,7 @@
       <c r="AD23" s="137" t="inlineStr"/>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -5254,13 +5268,13 @@
         </is>
       </c>
       <c r="B24" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C24" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D24" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5292,16 +5306,18 @@
       <c r="L24" s="135" t="n"/>
       <c r="N24" s="135" t="n"/>
       <c r="R24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T24" s="135" t="n"/>
       <c r="U24" s="135" t="n"/>
       <c r="V24" s="135" t="n">
-        <v>144.47</v>
+        <v>334.82</v>
       </c>
       <c r="W24" s="135" t="n"/>
       <c r="X24" s="136" t="n"/>
-      <c r="Y24" s="135" t="n"/>
+      <c r="Y24" s="135" t="n">
+        <v>334.82</v>
+      </c>
       <c r="Z24" s="135" t="n"/>
       <c r="AB24" s="137" t="inlineStr"/>
       <c r="AC24" s="137" t="inlineStr">
@@ -5312,7 +5328,7 @@
       <c r="AD24" s="137" t="inlineStr"/>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
@@ -5328,13 +5344,13 @@
         </is>
       </c>
       <c r="B25" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C25" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D25" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5353,35 +5369,51 @@
         <v>0.3333333333333333</v>
       </c>
       <c r="L25" s="135" t="n"/>
-      <c r="N25" s="135" t="n"/>
+      <c r="N25" s="135" t="n">
+        <v>45</v>
+      </c>
+      <c r="O25" t="n">
+        <v>466.6666666666667</v>
+      </c>
+      <c r="P25" t="n">
+        <v>15.05376344086022</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>301.0752688172043</v>
+      </c>
       <c r="R25" t="n">
-        <v>291</v>
+        <v>328</v>
+      </c>
+      <c r="S25" t="n">
+        <v>26.92473118279565</v>
       </c>
       <c r="T25" s="135" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="135" t="n">
-        <v>11516.12903225806</v>
+        <v>13548.38709677419</v>
       </c>
       <c r="V25" s="135" t="n">
-        <v>12526.432246</v>
+        <v>13120.172246</v>
       </c>
       <c r="W25" s="135" t="n">
-        <v>1010.303213741934</v>
+        <v>-428.2148507741931</v>
       </c>
       <c r="X25" s="136" t="n">
-        <v>0.0877294107170867</v>
+        <v>-0.0316063342238094</v>
       </c>
       <c r="Y25" s="135" t="n">
-        <v>43.04615892096219</v>
-      </c>
-      <c r="Z25" s="135" t="n"/>
+        <v>40.0005251402439</v>
+      </c>
+      <c r="Z25" s="135" t="n">
+        <v>-4.999474859756099</v>
+      </c>
       <c r="AB25" s="137" t="inlineStr"/>
       <c r="AC25" s="137" t="inlineStr"/>
       <c r="AD25" s="137" t="inlineStr"/>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>partial</t>
         </is>
       </c>
     </row>
@@ -5392,13 +5424,13 @@
         </is>
       </c>
       <c r="B26" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C26" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D26" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5432,41 +5464,41 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>749.4907345531284</v>
+        <v>881.7538053566217</v>
       </c>
       <c r="R26" t="n">
-        <v>863</v>
+        <v>967</v>
       </c>
       <c r="S26" t="n">
-        <v>113.5092654468716</v>
+        <v>85.24619464337832</v>
       </c>
       <c r="T26" s="135" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="135" t="n">
-        <v>17000</v>
+        <v>20000</v>
       </c>
       <c r="V26" s="135" t="n">
-        <v>21792.806811</v>
+        <v>23492.976811</v>
       </c>
       <c r="W26" s="135" t="n">
-        <v>4792.806811000002</v>
+        <v>3492.976811</v>
       </c>
       <c r="X26" s="136" t="n">
-        <v>0.2819298124117648</v>
+        <v>0.17464884055</v>
       </c>
       <c r="Y26" s="135" t="n">
-        <v>25.25238332676709</v>
+        <v>24.29470197621509</v>
       </c>
       <c r="Z26" s="135" t="n">
-        <v>2.570315068597139</v>
+        <v>1.612633718045142</v>
       </c>
       <c r="AB26" s="137" t="inlineStr"/>
       <c r="AC26" s="137" t="inlineStr"/>
       <c r="AD26" s="137" t="inlineStr"/>
       <c r="AE26" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>partial</t>
         </is>
       </c>
     </row>
@@ -5477,13 +5509,13 @@
         </is>
       </c>
       <c r="B27" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C27" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D27" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5517,41 +5549,41 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>741.6053574797209</v>
+        <v>872.4768911526128</v>
       </c>
       <c r="R27" t="n">
-        <v>758</v>
+        <v>798</v>
       </c>
       <c r="S27" t="n">
-        <v>16.39464252027915</v>
+        <v>-74.47689115261278</v>
       </c>
       <c r="T27" s="135" t="n">
         <v>354.8387096774193</v>
       </c>
       <c r="U27" s="135" t="n">
-        <v>6032.258064516129</v>
+        <v>7096.774193548386</v>
       </c>
       <c r="V27" s="135" t="n">
-        <v>6095</v>
+        <v>6422.6</v>
       </c>
       <c r="W27" s="135" t="n">
-        <v>62.7419354838712</v>
+        <v>-674.174193548386</v>
       </c>
       <c r="X27" s="136" t="n">
-        <v>0.0104010695187166</v>
+        <v>-0.0949972727272725</v>
       </c>
       <c r="Y27" s="135" t="n">
-        <v>8.040897097625329</v>
+        <v>8.048370927318297</v>
       </c>
       <c r="Z27" s="135" t="n">
-        <v>-0.0931569564287251</v>
+        <v>-0.0856831267357574</v>
       </c>
       <c r="AB27" s="137" t="inlineStr"/>
       <c r="AC27" s="137" t="inlineStr"/>
       <c r="AD27" s="137" t="inlineStr"/>
       <c r="AE27" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -5562,13 +5594,13 @@
         </is>
       </c>
       <c r="B28" s="134" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="C28" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D28" s="134" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5593,43 +5625,43 @@
         <v>84.56183862433862</v>
       </c>
       <c r="N28" s="135" t="n">
-        <v>23.16979253139447</v>
+        <v>19.77572292204534</v>
       </c>
       <c r="O28" t="n">
-        <v>2719.057579589313</v>
+        <v>3185.72424625598</v>
       </c>
       <c r="P28" t="n">
-        <v>87.71153482546173</v>
+        <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>1491.096092032849</v>
+        <v>2055.305965326439</v>
       </c>
       <c r="R28" t="n">
-        <v>1912</v>
+        <v>2093</v>
       </c>
       <c r="S28" t="n">
-        <v>420.9039079671506</v>
+        <v>37.69403467356096</v>
       </c>
       <c r="T28" s="135" t="n">
         <v>2032.258064516129</v>
       </c>
       <c r="U28" s="135" t="n">
-        <v>34548.38709677419</v>
+        <v>40645.16129032258</v>
       </c>
       <c r="V28" s="135" t="n">
-        <v>40414.239057</v>
+        <v>43035.749057</v>
       </c>
       <c r="W28" s="135" t="n">
-        <v>5865.851960225809</v>
+        <v>2390.587766677425</v>
       </c>
       <c r="X28" s="136" t="n">
-        <v>0.1697865646750701</v>
+        <v>0.0588160482277779</v>
       </c>
       <c r="Y28" s="135" t="n">
-        <v>21.13715431851464</v>
+        <v>20.56175301337793</v>
       </c>
       <c r="Z28" s="135" t="n">
-        <v>-2.032638212879828</v>
+        <v>0.7860300913325879</v>
       </c>
       <c r="AB28" s="137" t="inlineStr"/>
       <c r="AC28" s="137" t="inlineStr"/>
@@ -5732,7 +5764,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46220</v>
+        <v>46223</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5772,7 +5804,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5792,7 +5824,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46223.48444444445</v>
+        <v>46224.50170138889</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-07-22
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 20/07/2026  |  Ultimo aggiornamento: 21/07/2026 12:09</t>
+          <t>Periodo: 01/07/2026 - 21/07/2026  |  Ultimo aggiornamento: 22/07/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1061,19 +1061,19 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>6129.032258064516</v>
+        <v>6435.483870967741</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>6634.492993</v>
+        <v>6924.614962</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>505.4607349354837</v>
+        <v>489.1310910322582</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0824699093842105</v>
+        <v>0.0760053324411027</v>
       </c>
       <c r="U5" s="117" t="n">
-        <v>100.5226211060606</v>
+        <v>104.9184085151515</v>
       </c>
       <c r="V5" s="117" t="n"/>
       <c r="W5" s="120" t="inlineStr">
@@ -1175,19 +1175,19 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>967.741935483871</v>
+        <v>1016.129032258065</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>1196.140528</v>
+        <v>1236.075099</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>228.3985925161289</v>
+        <v>219.9460667419353</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>0.2360118789333332</v>
+        <v>0.2164548593333331</v>
       </c>
       <c r="U7" s="117" t="n">
-        <v>18.12334133333333</v>
+        <v>18.72841059090909</v>
       </c>
       <c r="V7" s="117" t="n"/>
       <c r="W7" s="120" t="inlineStr">
@@ -1289,19 +1289,19 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>6451.612903225806</v>
+        <v>6774.193548387097</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>6251.69</v>
+        <v>6483.86</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-199.9229032258063</v>
+        <v>-290.3335483870969</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.0309880499999999</v>
+        <v>-0.0428587619047619</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>96.17984615384614</v>
+        <v>99.75169230769232</v>
       </c>
       <c r="V9" s="117" t="n"/>
       <c r="W9" s="120" t="inlineStr">
@@ -1338,34 +1338,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>301.0752688172043</v>
+        <v>316.1290322580645</v>
       </c>
       <c r="N10" s="125" t="n">
         <v>328</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>26.92473118279565</v>
+        <v>11.87096774193549</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>13548.38709677419</v>
+        <v>14225.8064516129</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>14082.323521</v>
+        <v>14644.550061</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>533.9364242258052</v>
+        <v>418.7436093870965</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>0.0394095932166665</v>
+        <v>0.0294354918163265</v>
       </c>
       <c r="U10" s="123" t="n">
-        <v>42.93391317378048</v>
+        <v>44.64801847865854</v>
       </c>
       <c r="V10" s="123" t="n">
-        <v>-2.066086826219518</v>
+        <v>-0.3519815213414645</v>
       </c>
       <c r="W10" s="126" t="n"/>
     </row>
@@ -1417,34 +1417,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>150.8169250104734</v>
+        <v>158.357771260997</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>61</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-89.8169250104734</v>
+        <v>-97.35777126099704</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>5806.451612903225</v>
+        <v>6096.774193548387</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>6318.986418</v>
+        <v>6653.326913999999</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>512.534805096775</v>
+        <v>556.552720451612</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0882698831000001</v>
+        <v>0.0912864250476189</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>103.5899412786885</v>
+        <v>109.0709330163934</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>65.08994127868853</v>
+        <v>70.57093301639343</v>
       </c>
       <c r="W11" s="120" t="inlineStr">
         <is>
@@ -1547,34 +1547,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>75.90132827324479</v>
+        <v>79.69639468690701</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>111</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>35.09867172675521</v>
+        <v>31.30360531309299</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>2580.645161290322</v>
+        <v>2709.677419354839</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>3441.920792</v>
+        <v>3552.685198</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>861.2756307096774</v>
+        <v>843.0077786451616</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.3337443069</v>
+        <v>0.3111100135476192</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>31.00829542342342</v>
+        <v>32.00617295495496</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>-2.991704576576577</v>
+        <v>-1.993827045045045</v>
       </c>
       <c r="W13" s="120" t="inlineStr">
         <is>
@@ -1630,34 +1630,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>16.97792869269949</v>
+        <v>17.82682512733446</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>5</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-11.97792869269949</v>
+        <v>-12.82682512733446</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>645.1612903225806</v>
+        <v>677.4193548387096</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>626.3617840000001</v>
+        <v>667.311784</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-18.79950632258056</v>
+        <v>-10.10757083870965</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.0291392347999998</v>
+        <v>-0.0149206998095237</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>125.2723568</v>
+        <v>133.4623568</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>87.27235680000001</v>
+        <v>95.46235679999999</v>
       </c>
       <c r="W14" s="120" t="inlineStr">
         <is>
@@ -1713,34 +1713,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>2.580645161290323</v>
+        <v>2.709677419354839</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-0.5806451612903225</v>
+        <v>-0.7096774193548385</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>645.1612903225806</v>
+        <v>677.4193548387096</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>666.632657</v>
+        <v>704.740261</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>21.47136667741938</v>
+        <v>27.3209061612904</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>0.03328061835</v>
+        <v>0.0403308614761905</v>
       </c>
       <c r="U15" s="117" t="n">
-        <v>333.3163285</v>
+        <v>352.3701305</v>
       </c>
       <c r="V15" s="117" t="n">
-        <v>83.3163285</v>
+        <v>102.3701305</v>
       </c>
       <c r="W15" s="120" t="inlineStr">
         <is>
@@ -1890,34 +1890,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>2.688172043010753</v>
+        <v>2.822580645161291</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>4</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>1.311827956989247</v>
+        <v>1.177419354838709</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>322.5806451612903</v>
+        <v>338.7096774193548</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>311.38</v>
+        <v>323.59</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>-11.20064516129031</v>
+        <v>-15.11967741935484</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>-0.0347219999999999</v>
+        <v>-0.0446390476190476</v>
       </c>
       <c r="U18" s="117" t="n">
-        <v>77.845</v>
+        <v>80.89749999999999</v>
       </c>
       <c r="V18" s="117" t="n">
-        <v>-42.155</v>
+        <v>-39.10250000000001</v>
       </c>
       <c r="W18" s="120" t="inlineStr"/>
     </row>
@@ -1969,34 +1969,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>8.064516129032258</v>
+        <v>8.46774193548387</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>32</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>23.93548387096774</v>
+        <v>23.53225806451613</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>322.5806451612903</v>
+        <v>338.7096774193548</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>355.21</v>
+        <v>365.93</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>32.62935483870967</v>
+        <v>27.22032258064519</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>0.1011509999999999</v>
+        <v>0.08036476190476199</v>
       </c>
       <c r="U19" s="117" t="n">
-        <v>11.1003125</v>
+        <v>11.4353125</v>
       </c>
       <c r="V19" s="117" t="n">
-        <v>-28.8996875</v>
+        <v>-28.5646875</v>
       </c>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
@@ -2048,34 +2048,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>7.168458781362007</v>
+        <v>7.526881720430107</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>11.83154121863799</v>
+        <v>11.47311827956989</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>645.1612903225806</v>
+        <v>677.4193548387096</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>639.04</v>
+        <v>660.22</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-6.121290322580649</v>
+        <v>-17.19935483870961</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.009488</v>
+        <v>-0.0253895238095237</v>
       </c>
       <c r="U20" s="117" t="n">
-        <v>33.63368421052631</v>
+        <v>34.74842105263158</v>
       </c>
       <c r="V20" s="117" t="n">
-        <v>-56.36631578947369</v>
+        <v>-55.25157894736842</v>
       </c>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
@@ -2127,34 +2127,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>504.0322580645162</v>
+        <v>529.233870967742</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>417</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-87.03225806451616</v>
+        <v>-112.233870967742</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>6451.612903225806</v>
+        <v>6774.193548387097</v>
       </c>
       <c r="R21" s="117" t="n">
-        <v>8745.66</v>
+        <v>9220.65</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>2294.047096774194</v>
+        <v>2446.456451612903</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>0.3555773000000001</v>
+        <v>0.3611435714285714</v>
       </c>
       <c r="U21" s="117" t="n">
-        <v>20.97280575539568</v>
+        <v>22.11187050359712</v>
       </c>
       <c r="V21" s="117" t="n">
-        <v>8.172805755395682</v>
+        <v>9.31187050359712</v>
       </c>
       <c r="W21" s="120" t="inlineStr">
         <is>
@@ -2210,34 +2210,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>24.19354838709678</v>
+        <v>25.40322580645161</v>
       </c>
       <c r="N22" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-2.193548387096776</v>
+        <v>-3.403225806451612</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>967.741935483871</v>
+        <v>1016.129032258065</v>
       </c>
       <c r="R22" s="117" t="n">
-        <v>1189.161543</v>
+        <v>1239.425384</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>221.419607516129</v>
+        <v>223.2963517419353</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>0.2288002610999999</v>
+        <v>0.2197519652063489</v>
       </c>
       <c r="U22" s="117" t="n">
-        <v>54.05279740909091</v>
+        <v>56.33751745454545</v>
       </c>
       <c r="V22" s="117" t="n">
-        <v>14.05279740909091</v>
+        <v>16.33751745454545</v>
       </c>
       <c r="W22" s="120" t="inlineStr"/>
     </row>
@@ -2289,34 +2289,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>64.51612903225806</v>
+        <v>67.74193548387096</v>
       </c>
       <c r="N23" s="119" t="n">
         <v>114</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>49.48387096774194</v>
+        <v>46.25806451612904</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>967.741935483871</v>
+        <v>1016.129032258065</v>
       </c>
       <c r="R23" s="117" t="n">
-        <v>1385.782038</v>
+        <v>1455.378526</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>418.0401025161291</v>
+        <v>439.2494937419353</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.4319747726</v>
+        <v>0.4322772795555554</v>
       </c>
       <c r="U23" s="117" t="n">
-        <v>12.15598278947368</v>
+        <v>12.76647829824561</v>
       </c>
       <c r="V23" s="117" t="n">
-        <v>-2.844017210526316</v>
+        <v>-2.233521701754386</v>
       </c>
       <c r="W23" s="120" t="inlineStr">
         <is>
@@ -2372,34 +2372,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>24.81389578163772</v>
+        <v>26.0545905707196</v>
       </c>
       <c r="N24" s="119" t="n">
         <v>67</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>42.18610421836229</v>
+        <v>40.9454094292804</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>645.1612903225806</v>
+        <v>677.4193548387096</v>
       </c>
       <c r="R24" s="117" t="n">
-        <v>1107.29</v>
+        <v>1144.15</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>462.1287096774194</v>
+        <v>466.7306451612905</v>
       </c>
       <c r="T24" s="118" t="n">
-        <v>0.7162995</v>
+        <v>0.6889833333333336</v>
       </c>
       <c r="U24" s="117" t="n">
-        <v>16.52671641791045</v>
+        <v>17.07686567164179</v>
       </c>
       <c r="V24" s="117" t="n">
-        <v>-9.473283582089554</v>
+        <v>-8.923134328358209</v>
       </c>
       <c r="W24" s="120" t="inlineStr"/>
     </row>
@@ -2446,12 +2446,12 @@
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>334.82</v>
+        <v>400.4</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
       <c r="U25" s="117" t="n">
-        <v>334.82</v>
+        <v>400.4</v>
       </c>
       <c r="V25" s="117" t="n"/>
       <c r="W25" s="120" t="inlineStr"/>
@@ -2488,34 +2488,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>881.7538053566217</v>
+        <v>925.8414956244528</v>
       </c>
       <c r="N26" s="125" t="n">
         <v>967</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>85.24619464337832</v>
+        <v>41.1585043755473</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>20000</v>
+        <v>21000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>25122.245232</v>
+        <v>26387.808067</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>5122.245232000001</v>
+        <v>5387.808066999998</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>0.2561122616</v>
+        <v>0.2565622889047618</v>
       </c>
       <c r="U26" s="123" t="n">
-        <v>25.97957107755946</v>
+        <v>27.28832271664943</v>
       </c>
       <c r="V26" s="123" t="n">
-        <v>3.297502819389507</v>
+        <v>4.606254458479473</v>
       </c>
       <c r="W26" s="126" t="n"/>
     </row>
@@ -2563,28 +2563,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>286.7383512544803</v>
+        <v>301.0752688172043</v>
       </c>
       <c r="N27" s="119" t="n">
         <v>187</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-99.73835125448028</v>
+        <v>-114.0752688172043</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>2580.645161290322</v>
+        <v>2709.677419354839</v>
       </c>
       <c r="R27" s="117" t="n">
         <v>1683</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-897.6451612903224</v>
+        <v>-1026.677419354838</v>
       </c>
       <c r="T27" s="118" t="n">
-        <v>-0.3478374999999999</v>
+        <v>-0.3788928571428571</v>
       </c>
       <c r="U27" s="117" t="n">
         <v>9</v>
@@ -2638,28 +2638,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>424.4482173174873</v>
+        <v>445.6706281833617</v>
       </c>
       <c r="N28" s="119" t="n">
         <v>371</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-53.44821731748732</v>
+        <v>-74.67062818336171</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>161.2903225806452</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>3225.806451612903</v>
+        <v>3387.096774193548</v>
       </c>
       <c r="R28" s="117" t="n">
         <v>2819.6</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-406.206451612903</v>
+        <v>-567.4967741935484</v>
       </c>
       <c r="T28" s="118" t="n">
-        <v>-0.1259239999999999</v>
+        <v>-0.1675466666666666</v>
       </c>
       <c r="U28" s="117" t="n">
         <v>7.6</v>
@@ -2713,28 +2713,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>161.2903225806452</v>
+        <v>169.3548387096774</v>
       </c>
       <c r="N29" s="119" t="n">
         <v>240</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>78.70967741935485</v>
+        <v>70.64516129032259</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>1290.322580645161</v>
+        <v>1354.838709677419</v>
       </c>
       <c r="R29" s="117" t="n">
         <v>1920</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>629.6774193548388</v>
+        <v>565.1612903225807</v>
       </c>
       <c r="T29" s="118" t="n">
-        <v>0.4880000000000001</v>
+        <v>0.4171428571428572</v>
       </c>
       <c r="U29" s="117" t="n">
         <v>8</v>
@@ -2776,28 +2776,28 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>872.4768911526128</v>
+        <v>916.1007357102434</v>
       </c>
       <c r="N30" s="125" t="n">
         <v>798</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-74.47689115261278</v>
+        <v>-118.1007357102434</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>354.8387096774193</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>7096.774193548386</v>
+        <v>7451.612903225806</v>
       </c>
       <c r="R30" s="123" t="n">
         <v>6422.6</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>-674.174193548386</v>
+        <v>-1029.012903225806</v>
       </c>
       <c r="T30" s="124" t="n">
-        <v>-0.0949972727272725</v>
+        <v>-0.1380926406926405</v>
       </c>
       <c r="U30" s="123" t="n">
         <v>8.048370927318297</v>
@@ -2839,34 +2839,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="131" t="n">
-        <v>2055.305965326439</v>
+        <v>2158.071263592761</v>
       </c>
       <c r="N31" s="131" t="n">
         <v>2093</v>
       </c>
       <c r="O31" s="131" t="n">
-        <v>37.69403467356096</v>
+        <v>-65.07126359276072</v>
       </c>
       <c r="P31" s="129" t="n">
         <v>2032.258064516129</v>
       </c>
       <c r="Q31" s="129" t="n">
-        <v>40645.16129032258</v>
+        <v>42677.41935483871</v>
       </c>
       <c r="R31" s="129" t="n">
-        <v>45627.168753</v>
+        <v>47454.958128</v>
       </c>
       <c r="S31" s="129" t="n">
-        <v>4982.007462677422</v>
+        <v>4777.538773161286</v>
       </c>
       <c r="T31" s="130" t="n">
-        <v>0.1225731994785715</v>
+        <v>0.1119453529614511</v>
       </c>
       <c r="U31" s="129" t="n">
-        <v>21.7998895140946</v>
+        <v>22.67317636311515</v>
       </c>
       <c r="V31" s="129" t="n">
-        <v>2.024166592049262</v>
+        <v>2.897453441069807</v>
       </c>
       <c r="W31" s="132" t="n"/>
     </row>
@@ -3129,13 +3129,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3175,19 +3175,19 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>6129.032258064516</v>
+        <v>6435.483870967741</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>6634.492993</v>
+        <v>6924.614962</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>505.4607349354837</v>
+        <v>489.1310910322582</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0824699093842105</v>
+        <v>0.0760053324411027</v>
       </c>
       <c r="Y2" s="135" t="n">
-        <v>100.5226211060606</v>
+        <v>104.9184085151515</v>
       </c>
       <c r="Z2" s="135" t="n"/>
       <c r="AA2" t="inlineStr">
@@ -3204,7 +3204,7 @@
       <c r="AD2" s="137" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_3</t>
+          <t>google:ok;google:includes_excel_row_3;crm:stale</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -3220,13 +3220,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3274,7 +3274,7 @@
       <c r="AD3" s="137" t="inlineStr"/>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_2</t>
+          <t>google:rolled_up_to_excel_row_2;crm:stale</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -3290,13 +3290,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3336,19 +3336,19 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>967.741935483871</v>
+        <v>1016.129032258065</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>1196.140528</v>
+        <v>1236.075099</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>228.3985925161289</v>
+        <v>219.9460667419353</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>0.2360118789333332</v>
+        <v>0.2164548593333331</v>
       </c>
       <c r="Y4" s="135" t="n">
-        <v>18.12334133333333</v>
+        <v>18.72841059090909</v>
       </c>
       <c r="Z4" s="135" t="n"/>
       <c r="AA4" t="inlineStr">
@@ -3365,7 +3365,7 @@
       <c r="AD4" s="137" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_5</t>
+          <t>google:ok;google:includes_excel_row_5;crm:stale</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -3381,13 +3381,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3435,7 +3435,7 @@
       <c r="AD5" s="137" t="inlineStr"/>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_4</t>
+          <t>google:rolled_up_to_excel_row_4;crm:stale</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -3451,13 +3451,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3497,19 +3497,19 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>6451.612903225806</v>
+        <v>6774.193548387097</v>
       </c>
       <c r="V6" s="135" t="n">
-        <v>6251.69</v>
+        <v>6483.86</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-199.9229032258063</v>
+        <v>-290.3335483870969</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.0309880499999999</v>
+        <v>-0.0428587619047619</v>
       </c>
       <c r="Y6" s="135" t="n">
-        <v>96.17984615384614</v>
+        <v>99.75169230769232</v>
       </c>
       <c r="Z6" s="135" t="n"/>
       <c r="AA6" t="inlineStr">
@@ -3526,7 +3526,7 @@
       <c r="AD6" s="137" t="inlineStr"/>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -3542,13 +3542,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E7" t="n">
         <v>26</v>
@@ -3595,28 +3595,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q7" t="n">
-        <v>286.7383512544803</v>
+        <v>301.0752688172043</v>
       </c>
       <c r="R7" t="n">
         <v>187</v>
       </c>
       <c r="S7" t="n">
-        <v>-99.73835125448028</v>
+        <v>-114.0752688172043</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>2580.645161290322</v>
+        <v>2709.677419354839</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>1683</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>-897.6451612903224</v>
+        <v>-1026.677419354838</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>-0.3478374999999999</v>
+        <v>-0.3788928571428571</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>9</v>
@@ -3629,7 +3629,7 @@
       <c r="AD7" s="137" t="inlineStr"/>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -3645,13 +3645,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E8" t="n">
         <v>25</v>
@@ -3698,28 +3698,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q8" t="n">
-        <v>424.4482173174873</v>
+        <v>445.6706281833617</v>
       </c>
       <c r="R8" t="n">
         <v>371</v>
       </c>
       <c r="S8" t="n">
-        <v>-53.44821731748732</v>
+        <v>-74.67062818336171</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>161.2903225806452</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>3225.806451612903</v>
+        <v>3387.096774193548</v>
       </c>
       <c r="V8" s="135" t="n">
         <v>2819.6</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>-406.206451612903</v>
+        <v>-567.4967741935484</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>-0.1259239999999999</v>
+        <v>-0.1675466666666666</v>
       </c>
       <c r="Y8" s="135" t="n">
         <v>7.6</v>
@@ -3732,7 +3732,7 @@
       <c r="AD8" s="137" t="inlineStr"/>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -3748,13 +3748,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3801,28 +3801,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>161.2903225806452</v>
+        <v>169.3548387096774</v>
       </c>
       <c r="R9" t="n">
         <v>240</v>
       </c>
       <c r="S9" t="n">
-        <v>78.70967741935485</v>
+        <v>70.64516129032259</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>1290.322580645161</v>
+        <v>1354.838709677419</v>
       </c>
       <c r="V9" s="135" t="n">
         <v>1920</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>629.6774193548388</v>
+        <v>565.1612903225807</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.4880000000000001</v>
+        <v>0.4171428571428572</v>
       </c>
       <c r="Y9" s="135" t="n">
         <v>8</v>
@@ -3835,7 +3835,7 @@
       <c r="AD9" s="137" t="inlineStr"/>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -3851,13 +3851,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E10" t="n">
         <v>9</v>
@@ -3904,34 +3904,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q10" t="n">
-        <v>150.8169250104734</v>
+        <v>158.357771260997</v>
       </c>
       <c r="R10" t="n">
         <v>61</v>
       </c>
       <c r="S10" t="n">
-        <v>-89.8169250104734</v>
+        <v>-97.35777126099704</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>5806.451612903225</v>
+        <v>6096.774193548387</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>6318.986418</v>
+        <v>6653.326913999999</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>512.534805096775</v>
+        <v>556.552720451612</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0882698831000001</v>
+        <v>0.0912864250476189</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>103.5899412786885</v>
+        <v>109.0709330163934</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>65.08994127868853</v>
+        <v>70.57093301639343</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -3947,7 +3947,7 @@
       <c r="AD10" s="137" t="inlineStr"/>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_10</t>
+          <t>google:ok;google:includes_excel_row_10;crm:stale</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -3963,13 +3963,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E11" t="n">
         <v>10</v>
@@ -4017,7 +4017,7 @@
       <c r="AD11" s="137" t="inlineStr"/>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_9</t>
+          <t>google:rolled_up_to_excel_row_9;crm:stale</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -4033,13 +4033,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E12" t="n">
         <v>8</v>
@@ -4086,34 +4086,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q12" t="n">
-        <v>75.90132827324479</v>
+        <v>79.69639468690701</v>
       </c>
       <c r="R12" t="n">
         <v>111</v>
       </c>
       <c r="S12" t="n">
-        <v>35.09867172675521</v>
+        <v>31.30360531309299</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>2580.645161290322</v>
+        <v>2709.677419354839</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>3441.920792</v>
+        <v>3552.685198</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>861.2756307096774</v>
+        <v>843.0077786451616</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.3337443069</v>
+        <v>0.3111100135476192</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>31.00829542342342</v>
+        <v>32.00617295495496</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>-2.991704576576577</v>
+        <v>-1.993827045045045</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
@@ -4129,7 +4129,7 @@
       <c r="AD12" s="137" t="inlineStr"/>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -4145,13 +4145,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4198,34 +4198,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>16.97792869269949</v>
+        <v>17.82682512733446</v>
       </c>
       <c r="R13" t="n">
         <v>5</v>
       </c>
       <c r="S13" t="n">
-        <v>-11.97792869269949</v>
+        <v>-12.82682512733446</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>645.1612903225806</v>
+        <v>677.4193548387096</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>626.3617840000001</v>
+        <v>667.311784</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-18.79950632258056</v>
+        <v>-10.10757083870965</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.0291392347999998</v>
+        <v>-0.0149206998095237</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>125.2723568</v>
+        <v>133.4623568</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>87.27235680000001</v>
+        <v>95.46235679999999</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -4241,7 +4241,7 @@
       <c r="AD13" s="137" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_12</t>
+          <t>google:ok;google:includes_excel_row_12;crm:stale</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -4257,13 +4257,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -4310,34 +4310,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q14" t="n">
-        <v>2.580645161290323</v>
+        <v>2.709677419354839</v>
       </c>
       <c r="R14" t="n">
         <v>2</v>
       </c>
       <c r="S14" t="n">
-        <v>-0.5806451612903225</v>
+        <v>-0.7096774193548385</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>645.1612903225806</v>
+        <v>677.4193548387096</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>666.632657</v>
+        <v>704.740261</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>21.47136667741938</v>
+        <v>27.3209061612904</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>0.03328061835</v>
+        <v>0.0403308614761905</v>
       </c>
       <c r="Y14" s="135" t="n">
-        <v>333.3163285</v>
+        <v>352.3701305</v>
       </c>
       <c r="Z14" s="135" t="n">
-        <v>83.3163285</v>
+        <v>102.3701305</v>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
@@ -4353,7 +4353,7 @@
       <c r="AD14" s="137" t="inlineStr"/>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_14</t>
+          <t>google:ok;google:includes_excel_row_14;crm:stale</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -4369,13 +4369,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E15" t="n">
         <v>14</v>
@@ -4423,7 +4423,7 @@
       <c r="AD15" s="137" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_13</t>
+          <t>google:rolled_up_to_excel_row_13;crm:stale</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -4439,13 +4439,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E16" t="n">
         <v>12</v>
@@ -4493,7 +4493,7 @@
       <c r="AD16" s="137" t="inlineStr"/>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_11</t>
+          <t>google:rolled_up_to_excel_row_11;crm:stale</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -4509,13 +4509,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E17" t="n">
         <v>21</v>
@@ -4562,34 +4562,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q17" t="n">
-        <v>2.688172043010753</v>
+        <v>2.822580645161291</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
       </c>
       <c r="S17" t="n">
-        <v>1.311827956989247</v>
+        <v>1.177419354838709</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>322.5806451612903</v>
+        <v>338.7096774193548</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>311.38</v>
+        <v>323.59</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-11.20064516129031</v>
+        <v>-15.11967741935484</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0347219999999999</v>
+        <v>-0.0446390476190476</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>77.845</v>
+        <v>80.89749999999999</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>-42.155</v>
+        <v>-39.10250000000001</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr">
@@ -4600,7 +4600,7 @@
       <c r="AD17" s="137" t="inlineStr"/>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
@@ -4616,13 +4616,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4669,34 +4669,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>8.064516129032258</v>
+        <v>8.46774193548387</v>
       </c>
       <c r="R18" t="n">
         <v>32</v>
       </c>
       <c r="S18" t="n">
-        <v>23.93548387096774</v>
+        <v>23.53225806451613</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>322.5806451612903</v>
+        <v>338.7096774193548</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>355.21</v>
+        <v>365.93</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>32.62935483870967</v>
+        <v>27.22032258064519</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>0.1011509999999999</v>
+        <v>0.08036476190476199</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>11.1003125</v>
+        <v>11.4353125</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>-28.8996875</v>
+        <v>-28.5646875</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr">
@@ -4707,7 +4707,7 @@
       <c r="AD18" s="137" t="inlineStr"/>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
@@ -4723,13 +4723,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4776,34 +4776,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>7.168458781362007</v>
+        <v>7.526881720430107</v>
       </c>
       <c r="R19" t="n">
         <v>19</v>
       </c>
       <c r="S19" t="n">
-        <v>11.83154121863799</v>
+        <v>11.47311827956989</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>645.1612903225806</v>
+        <v>677.4193548387096</v>
       </c>
       <c r="V19" s="135" t="n">
-        <v>639.04</v>
+        <v>660.22</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-6.121290322580649</v>
+        <v>-17.19935483870961</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.009488</v>
+        <v>-0.0253895238095237</v>
       </c>
       <c r="Y19" s="135" t="n">
-        <v>33.63368421052631</v>
+        <v>34.74842105263158</v>
       </c>
       <c r="Z19" s="135" t="n">
-        <v>-56.36631578947369</v>
+        <v>-55.25157894736842</v>
       </c>
       <c r="AB19" s="137" t="inlineStr"/>
       <c r="AC19" s="137" t="inlineStr">
@@ -4814,7 +4814,7 @@
       <c r="AD19" s="137" t="inlineStr"/>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
@@ -4830,13 +4830,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E20" t="n">
         <v>17</v>
@@ -4883,34 +4883,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q20" t="n">
-        <v>504.0322580645162</v>
+        <v>529.233870967742</v>
       </c>
       <c r="R20" t="n">
         <v>417</v>
       </c>
       <c r="S20" t="n">
-        <v>-87.03225806451616</v>
+        <v>-112.233870967742</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>6451.612903225806</v>
+        <v>6774.193548387097</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>8745.66</v>
+        <v>9220.65</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>2294.047096774194</v>
+        <v>2446.456451612903</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>0.3555773000000001</v>
+        <v>0.3611435714285714</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>20.97280575539568</v>
+        <v>22.11187050359712</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>8.172805755395682</v>
+        <v>9.31187050359712</v>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
@@ -4926,7 +4926,7 @@
       <c r="AD20" s="137" t="inlineStr"/>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr">
@@ -4942,13 +4942,13 @@
         </is>
       </c>
       <c r="B21" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C21" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D21" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4995,34 +4995,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>24.19354838709678</v>
+        <v>25.40322580645161</v>
       </c>
       <c r="R21" t="n">
         <v>22</v>
       </c>
       <c r="S21" t="n">
-        <v>-2.193548387096776</v>
+        <v>-3.403225806451612</v>
       </c>
       <c r="T21" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="135" t="n">
-        <v>967.741935483871</v>
+        <v>1016.129032258065</v>
       </c>
       <c r="V21" s="135" t="n">
-        <v>1189.161543</v>
+        <v>1239.425384</v>
       </c>
       <c r="W21" s="135" t="n">
-        <v>221.419607516129</v>
+        <v>223.2963517419353</v>
       </c>
       <c r="X21" s="136" t="n">
-        <v>0.2288002610999999</v>
+        <v>0.2197519652063489</v>
       </c>
       <c r="Y21" s="135" t="n">
-        <v>54.05279740909091</v>
+        <v>56.33751745454545</v>
       </c>
       <c r="Z21" s="135" t="n">
-        <v>14.05279740909091</v>
+        <v>16.33751745454545</v>
       </c>
       <c r="AB21" s="137" t="inlineStr">
         <is>
@@ -5033,7 +5033,7 @@
       <c r="AD21" s="137" t="inlineStr"/>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
@@ -5049,13 +5049,13 @@
         </is>
       </c>
       <c r="B22" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C22" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D22" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -5102,34 +5102,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>64.51612903225806</v>
+        <v>67.74193548387096</v>
       </c>
       <c r="R22" t="n">
         <v>114</v>
       </c>
       <c r="S22" t="n">
-        <v>49.48387096774194</v>
+        <v>46.25806451612904</v>
       </c>
       <c r="T22" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="135" t="n">
-        <v>967.741935483871</v>
+        <v>1016.129032258065</v>
       </c>
       <c r="V22" s="135" t="n">
-        <v>1385.782038</v>
+        <v>1455.378526</v>
       </c>
       <c r="W22" s="135" t="n">
-        <v>418.0401025161291</v>
+        <v>439.2494937419353</v>
       </c>
       <c r="X22" s="136" t="n">
-        <v>0.4319747726</v>
+        <v>0.4322772795555554</v>
       </c>
       <c r="Y22" s="135" t="n">
-        <v>12.15598278947368</v>
+        <v>12.76647829824561</v>
       </c>
       <c r="Z22" s="135" t="n">
-        <v>-2.844017210526316</v>
+        <v>-2.233521701754386</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -5145,7 +5145,7 @@
       <c r="AD22" s="137" t="inlineStr"/>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
@@ -5161,13 +5161,13 @@
         </is>
       </c>
       <c r="B23" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C23" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D23" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5214,34 +5214,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>24.81389578163772</v>
+        <v>26.0545905707196</v>
       </c>
       <c r="R23" t="n">
         <v>67</v>
       </c>
       <c r="S23" t="n">
-        <v>42.18610421836229</v>
+        <v>40.9454094292804</v>
       </c>
       <c r="T23" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="135" t="n">
-        <v>645.1612903225806</v>
+        <v>677.4193548387096</v>
       </c>
       <c r="V23" s="135" t="n">
-        <v>1107.29</v>
+        <v>1144.15</v>
       </c>
       <c r="W23" s="135" t="n">
-        <v>462.1287096774194</v>
+        <v>466.7306451612905</v>
       </c>
       <c r="X23" s="136" t="n">
-        <v>0.7162995</v>
+        <v>0.6889833333333336</v>
       </c>
       <c r="Y23" s="135" t="n">
-        <v>16.52671641791045</v>
+        <v>17.07686567164179</v>
       </c>
       <c r="Z23" s="135" t="n">
-        <v>-9.473283582089554</v>
+        <v>-8.923134328358209</v>
       </c>
       <c r="AB23" s="137" t="inlineStr"/>
       <c r="AC23" s="137" t="inlineStr">
@@ -5252,7 +5252,7 @@
       <c r="AD23" s="137" t="inlineStr"/>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -5268,13 +5268,13 @@
         </is>
       </c>
       <c r="B24" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C24" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D24" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5311,12 +5311,12 @@
       <c r="T24" s="135" t="n"/>
       <c r="U24" s="135" t="n"/>
       <c r="V24" s="135" t="n">
-        <v>334.82</v>
+        <v>400.4</v>
       </c>
       <c r="W24" s="135" t="n"/>
       <c r="X24" s="136" t="n"/>
       <c r="Y24" s="135" t="n">
-        <v>334.82</v>
+        <v>400.4</v>
       </c>
       <c r="Z24" s="135" t="n"/>
       <c r="AB24" s="137" t="inlineStr"/>
@@ -5328,7 +5328,7 @@
       <c r="AD24" s="137" t="inlineStr"/>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
@@ -5344,13 +5344,13 @@
         </is>
       </c>
       <c r="B25" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C25" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D25" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5379,41 +5379,41 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>301.0752688172043</v>
+        <v>316.1290322580645</v>
       </c>
       <c r="R25" t="n">
         <v>328</v>
       </c>
       <c r="S25" t="n">
-        <v>26.92473118279565</v>
+        <v>11.87096774193549</v>
       </c>
       <c r="T25" s="135" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="135" t="n">
-        <v>13548.38709677419</v>
+        <v>14225.8064516129</v>
       </c>
       <c r="V25" s="135" t="n">
-        <v>14082.323521</v>
+        <v>14644.550061</v>
       </c>
       <c r="W25" s="135" t="n">
-        <v>533.9364242258052</v>
+        <v>418.7436093870965</v>
       </c>
       <c r="X25" s="136" t="n">
-        <v>0.0394095932166665</v>
+        <v>0.0294354918163265</v>
       </c>
       <c r="Y25" s="135" t="n">
-        <v>42.93391317378048</v>
+        <v>44.64801847865854</v>
       </c>
       <c r="Z25" s="135" t="n">
-        <v>-2.066086826219518</v>
+        <v>-0.3519815213414645</v>
       </c>
       <c r="AB25" s="137" t="inlineStr"/>
       <c r="AC25" s="137" t="inlineStr"/>
       <c r="AD25" s="137" t="inlineStr"/>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5424,13 +5424,13 @@
         </is>
       </c>
       <c r="B26" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C26" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D26" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5464,41 +5464,41 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>881.7538053566217</v>
+        <v>925.8414956244528</v>
       </c>
       <c r="R26" t="n">
         <v>967</v>
       </c>
       <c r="S26" t="n">
-        <v>85.24619464337832</v>
+        <v>41.1585043755473</v>
       </c>
       <c r="T26" s="135" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="135" t="n">
-        <v>20000</v>
+        <v>21000</v>
       </c>
       <c r="V26" s="135" t="n">
-        <v>25122.245232</v>
+        <v>26387.808067</v>
       </c>
       <c r="W26" s="135" t="n">
-        <v>5122.245232000001</v>
+        <v>5387.808066999998</v>
       </c>
       <c r="X26" s="136" t="n">
-        <v>0.2561122616</v>
+        <v>0.2565622889047618</v>
       </c>
       <c r="Y26" s="135" t="n">
-        <v>25.97957107755946</v>
+        <v>27.28832271664943</v>
       </c>
       <c r="Z26" s="135" t="n">
-        <v>3.297502819389507</v>
+        <v>4.606254458479473</v>
       </c>
       <c r="AB26" s="137" t="inlineStr"/>
       <c r="AC26" s="137" t="inlineStr"/>
       <c r="AD26" s="137" t="inlineStr"/>
       <c r="AE26" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5509,13 +5509,13 @@
         </is>
       </c>
       <c r="B27" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C27" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D27" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5549,28 +5549,28 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>872.4768911526128</v>
+        <v>916.1007357102434</v>
       </c>
       <c r="R27" t="n">
         <v>798</v>
       </c>
       <c r="S27" t="n">
-        <v>-74.47689115261278</v>
+        <v>-118.1007357102434</v>
       </c>
       <c r="T27" s="135" t="n">
         <v>354.8387096774193</v>
       </c>
       <c r="U27" s="135" t="n">
-        <v>7096.774193548386</v>
+        <v>7451.612903225806</v>
       </c>
       <c r="V27" s="135" t="n">
         <v>6422.6</v>
       </c>
       <c r="W27" s="135" t="n">
-        <v>-674.174193548386</v>
+        <v>-1029.012903225806</v>
       </c>
       <c r="X27" s="136" t="n">
-        <v>-0.0949972727272725</v>
+        <v>-0.1380926406926405</v>
       </c>
       <c r="Y27" s="135" t="n">
         <v>8.048370927318297</v>
@@ -5583,7 +5583,7 @@
       <c r="AD27" s="137" t="inlineStr"/>
       <c r="AE27" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>success;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5594,13 +5594,13 @@
         </is>
       </c>
       <c r="B28" s="134" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="C28" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D28" s="134" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5634,41 +5634,41 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>2055.305965326439</v>
+        <v>2158.071263592761</v>
       </c>
       <c r="R28" t="n">
         <v>2093</v>
       </c>
       <c r="S28" t="n">
-        <v>37.69403467356096</v>
+        <v>-65.07126359276072</v>
       </c>
       <c r="T28" s="135" t="n">
         <v>2032.258064516129</v>
       </c>
       <c r="U28" s="135" t="n">
-        <v>40645.16129032258</v>
+        <v>42677.41935483871</v>
       </c>
       <c r="V28" s="135" t="n">
-        <v>45627.168753</v>
+        <v>47454.958128</v>
       </c>
       <c r="W28" s="135" t="n">
-        <v>4982.007462677422</v>
+        <v>4777.538773161286</v>
       </c>
       <c r="X28" s="136" t="n">
-        <v>0.1225731994785715</v>
+        <v>0.1119453529614511</v>
       </c>
       <c r="Y28" s="135" t="n">
-        <v>21.7998895140946</v>
+        <v>22.67317636311515</v>
       </c>
       <c r="Z28" s="135" t="n">
-        <v>2.024166592049262</v>
+        <v>2.897453441069807</v>
       </c>
       <c r="AB28" s="137" t="inlineStr"/>
       <c r="AC28" s="137" t="inlineStr"/>
       <c r="AD28" s="137" t="inlineStr"/>
       <c r="AE28" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5764,7 +5764,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5804,7 +5804,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5824,7 +5824,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46224.50673611111</v>
+        <v>46225.29189814815</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Use a single Area Clienti lead total
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 21/07/2026  |  Ultimo aggiornamento: 22/07/2026 07:00</t>
+          <t>Periodo: 01/07/2026 - 17/07/2026  |  Ultimo aggiornamento: 22/07/2026 11:38</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1053,28 +1053,24 @@
       <c r="K5" s="119" t="n"/>
       <c r="L5" s="119" t="n"/>
       <c r="M5" s="119" t="n"/>
-      <c r="N5" s="119" t="n">
-        <v>66</v>
-      </c>
+      <c r="N5" s="119" t="n"/>
       <c r="O5" s="119" t="n"/>
       <c r="P5" s="117" t="n">
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>6435.483870967741</v>
+        <v>5209.677419354838</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>6924.614962</v>
+        <v>5794.215866</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>489.1310910322582</v>
+        <v>584.5384466451615</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0760053324411027</v>
-      </c>
-      <c r="U5" s="117" t="n">
-        <v>104.9184085151515</v>
-      </c>
+        <v>0.1122024262910217</v>
+      </c>
+      <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
       <c r="W5" s="120" t="inlineStr">
         <is>
@@ -1116,9 +1112,7 @@
       <c r="K6" s="119" t="n"/>
       <c r="L6" s="119" t="n"/>
       <c r="M6" s="119" t="n"/>
-      <c r="N6" s="119" t="n">
-        <v>66</v>
-      </c>
+      <c r="N6" s="119" t="n"/>
       <c r="O6" s="119" t="n"/>
       <c r="P6" s="117" t="n"/>
       <c r="Q6" s="117" t="n"/>
@@ -1167,28 +1161,24 @@
       <c r="K7" s="119" t="n"/>
       <c r="L7" s="119" t="n"/>
       <c r="M7" s="119" t="n"/>
-      <c r="N7" s="119" t="n">
-        <v>66</v>
-      </c>
+      <c r="N7" s="119" t="n"/>
       <c r="O7" s="119" t="n"/>
       <c r="P7" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>1016.129032258065</v>
+        <v>822.5806451612904</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>1236.075099</v>
+        <v>1074.27638</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>219.9460667419353</v>
+        <v>251.6957348387096</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>0.2164548593333331</v>
-      </c>
-      <c r="U7" s="117" t="n">
-        <v>18.72841059090909</v>
-      </c>
+        <v>0.3059830501960784</v>
+      </c>
+      <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
       <c r="W7" s="120" t="inlineStr">
         <is>
@@ -1230,9 +1220,7 @@
       <c r="K8" s="119" t="n"/>
       <c r="L8" s="119" t="n"/>
       <c r="M8" s="119" t="n"/>
-      <c r="N8" s="119" t="n">
-        <v>65</v>
-      </c>
+      <c r="N8" s="119" t="n"/>
       <c r="O8" s="119" t="n"/>
       <c r="P8" s="117" t="n"/>
       <c r="Q8" s="117" t="n"/>
@@ -1281,28 +1269,24 @@
       <c r="K9" s="119" t="n"/>
       <c r="L9" s="119" t="n"/>
       <c r="M9" s="119" t="n"/>
-      <c r="N9" s="119" t="n">
-        <v>65</v>
-      </c>
+      <c r="N9" s="119" t="n"/>
       <c r="O9" s="119" t="n"/>
       <c r="P9" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>6774.193548387097</v>
+        <v>5483.870967741936</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>6483.86</v>
+        <v>5657.94</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-290.3335483870969</v>
+        <v>174.069032258064</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.0428587619047619</v>
-      </c>
-      <c r="U9" s="117" t="n">
-        <v>99.75169230769232</v>
-      </c>
+        <v>0.0317419999999999</v>
+      </c>
+      <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
       <c r="W9" s="120" t="inlineStr">
         <is>
@@ -1338,34 +1322,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>316.1290322580645</v>
+        <v>255.9139784946237</v>
       </c>
       <c r="N10" s="125" t="n">
-        <v>328</v>
+        <v>291</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>11.87096774193549</v>
+        <v>35.08602150537632</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>14225.8064516129</v>
+        <v>11516.12903225806</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>14644.550061</v>
+        <v>12526.432246</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>418.7436093870965</v>
+        <v>1010.303213741934</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>0.0294354918163265</v>
+        <v>0.0877294107170867</v>
       </c>
       <c r="U10" s="123" t="n">
-        <v>44.64801847865854</v>
+        <v>43.04615892096219</v>
       </c>
       <c r="V10" s="123" t="n">
-        <v>-0.3519815213414645</v>
+        <v>-1.953841079037808</v>
       </c>
       <c r="W10" s="126" t="n"/>
     </row>
@@ -1417,34 +1401,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>158.357771260997</v>
+        <v>128.1943862589024</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>61</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-97.35777126099704</v>
+        <v>-67.19438625890237</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>6096.774193548387</v>
+        <v>4935.483870967741</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>6653.326913999999</v>
+        <v>5490.756616000001</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>556.552720451612</v>
+        <v>555.2727450322591</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0912864250476189</v>
+        <v>0.1125062424575165</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>109.0709330163934</v>
+        <v>90.01240354098361</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>70.57093301639343</v>
+        <v>51.51240354098361</v>
       </c>
       <c r="W11" s="120" t="inlineStr">
         <is>
@@ -1487,7 +1471,7 @@
       <c r="L12" s="119" t="n"/>
       <c r="M12" s="119" t="n"/>
       <c r="N12" s="119" t="n">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="O12" s="119" t="n"/>
       <c r="P12" s="117" t="n"/>
@@ -1547,34 +1531,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>79.69639468690701</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="N13" s="119" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>31.30360531309299</v>
+        <v>33.48387096774194</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>2709.677419354839</v>
+        <v>2193.548387096774</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>3552.685198</v>
+        <v>3069.617174</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>843.0077786451616</v>
+        <v>876.0687869032258</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.3111100135476192</v>
+        <v>0.3993842999117647</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>32.00617295495496</v>
+        <v>31.3226242244898</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>-1.993827045045045</v>
+        <v>-2.677375775510203</v>
       </c>
       <c r="W13" s="120" t="inlineStr">
         <is>
@@ -1630,34 +1614,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>17.82682512733446</v>
+        <v>14.43123938879457</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>5</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-12.82682512733446</v>
+        <v>-9.431239388794566</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>677.4193548387096</v>
+        <v>548.3870967741935</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>667.311784</v>
+        <v>510.988722</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-10.10757083870965</v>
+        <v>-37.39837477419354</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.0149206998095237</v>
+        <v>-0.0681970363529411</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>133.4623568</v>
+        <v>102.1977444</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>95.46235679999999</v>
+        <v>64.1977444</v>
       </c>
       <c r="W14" s="120" t="inlineStr">
         <is>
@@ -1713,34 +1697,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>2.709677419354839</v>
+        <v>2.193548387096774</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-0.7096774193548385</v>
+        <v>-0.193548387096774</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>677.4193548387096</v>
+        <v>548.3870967741935</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>704.740261</v>
+        <v>630.160373</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>27.3209061612904</v>
+        <v>81.77327622580651</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>0.0403308614761905</v>
+        <v>0.1491159742941177</v>
       </c>
       <c r="U15" s="117" t="n">
-        <v>352.3701305</v>
+        <v>315.0801865</v>
       </c>
       <c r="V15" s="117" t="n">
-        <v>102.3701305</v>
+        <v>65.08018650000002</v>
       </c>
       <c r="W15" s="120" t="inlineStr">
         <is>
@@ -1830,7 +1814,7 @@
       <c r="L17" s="119" t="n"/>
       <c r="M17" s="119" t="n"/>
       <c r="N17" s="119" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O17" s="119" t="n"/>
       <c r="P17" s="117" t="n"/>
@@ -1890,34 +1874,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>2.822580645161291</v>
+        <v>2.28494623655914</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>4</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>1.177419354838709</v>
+        <v>1.71505376344086</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>338.7096774193548</v>
+        <v>274.1935483870968</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>323.59</v>
+        <v>283.27</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>-15.11967741935484</v>
+        <v>9.076451612903211</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>-0.0446390476190476</v>
+        <v>0.0331023529411764</v>
       </c>
       <c r="U18" s="117" t="n">
-        <v>80.89749999999999</v>
+        <v>70.8175</v>
       </c>
       <c r="V18" s="117" t="n">
-        <v>-39.10250000000001</v>
+        <v>-49.1825</v>
       </c>
       <c r="W18" s="120" t="inlineStr"/>
     </row>
@@ -1969,34 +1953,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>8.46774193548387</v>
+        <v>6.854838709677419</v>
       </c>
       <c r="N19" s="119" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>23.53225806451613</v>
+        <v>24.14516129032258</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>338.7096774193548</v>
+        <v>274.1935483870968</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>365.93</v>
+        <v>322.95</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>27.22032258064519</v>
+        <v>48.75645161290322</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>0.08036476190476199</v>
+        <v>0.1778176470588235</v>
       </c>
       <c r="U19" s="117" t="n">
-        <v>11.4353125</v>
+        <v>10.41774193548387</v>
       </c>
       <c r="V19" s="117" t="n">
-        <v>-28.5646875</v>
+        <v>-29.58225806451613</v>
       </c>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
@@ -2048,34 +2032,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>7.526881720430107</v>
+        <v>6.093189964157706</v>
       </c>
       <c r="N20" s="119" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>11.47311827956989</v>
+        <v>10.9068100358423</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>677.4193548387096</v>
+        <v>548.3870967741935</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>660.22</v>
+        <v>581.76</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-17.19935483870961</v>
+        <v>33.37290322580645</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.0253895238095237</v>
+        <v>0.0608564705882353</v>
       </c>
       <c r="U20" s="117" t="n">
-        <v>34.74842105263158</v>
+        <v>34.22117647058823</v>
       </c>
       <c r="V20" s="117" t="n">
-        <v>-55.25157894736842</v>
+        <v>-55.77882352941177</v>
       </c>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
@@ -2127,34 +2111,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>529.233870967742</v>
+        <v>428.4274193548387</v>
       </c>
       <c r="N21" s="119" t="n">
-        <v>417</v>
+        <v>367</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-112.233870967742</v>
+        <v>-61.42741935483872</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>6774.193548387097</v>
+        <v>5483.870967741936</v>
       </c>
       <c r="R21" s="117" t="n">
-        <v>9220.65</v>
+        <v>7444.1</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>2446.456451612903</v>
+        <v>1960.229032258065</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>0.3611435714285714</v>
+        <v>0.3574535294117647</v>
       </c>
       <c r="U21" s="117" t="n">
-        <v>22.11187050359712</v>
+        <v>20.28365122615804</v>
       </c>
       <c r="V21" s="117" t="n">
-        <v>9.31187050359712</v>
+        <v>7.483651226158038</v>
       </c>
       <c r="W21" s="120" t="inlineStr">
         <is>
@@ -2210,34 +2194,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>25.40322580645161</v>
+        <v>20.56451612903226</v>
       </c>
       <c r="N22" s="119" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-3.403225806451612</v>
+        <v>0.4354838709677402</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>1016.129032258065</v>
+        <v>822.5806451612904</v>
       </c>
       <c r="R22" s="117" t="n">
-        <v>1239.425384</v>
+        <v>1057.013242</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>223.2963517419353</v>
+        <v>234.4325968387096</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>0.2197519652063489</v>
+        <v>0.2849964902745097</v>
       </c>
       <c r="U22" s="117" t="n">
-        <v>56.33751745454545</v>
+        <v>50.3339639047619</v>
       </c>
       <c r="V22" s="117" t="n">
-        <v>16.33751745454545</v>
+        <v>10.3339639047619</v>
       </c>
       <c r="W22" s="120" t="inlineStr"/>
     </row>
@@ -2289,34 +2273,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>67.74193548387096</v>
+        <v>54.83870967741935</v>
       </c>
       <c r="N23" s="119" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>46.25806451612904</v>
+        <v>47.16129032258065</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>1016.129032258065</v>
+        <v>822.5806451612904</v>
       </c>
       <c r="R23" s="117" t="n">
-        <v>1455.378526</v>
+        <v>1241.033961</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>439.2494937419353</v>
+        <v>418.4533158387097</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.4322772795555554</v>
+        <v>0.5087079525882353</v>
       </c>
       <c r="U23" s="117" t="n">
-        <v>12.76647829824561</v>
+        <v>12.16699961764706</v>
       </c>
       <c r="V23" s="117" t="n">
-        <v>-2.233521701754386</v>
+        <v>-2.833000382352941</v>
       </c>
       <c r="W23" s="120" t="inlineStr">
         <is>
@@ -2372,34 +2356,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>26.0545905707196</v>
+        <v>21.09181141439206</v>
       </c>
       <c r="N24" s="119" t="n">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>40.9454094292804</v>
+        <v>37.90818858560795</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>677.4193548387096</v>
+        <v>548.3870967741935</v>
       </c>
       <c r="R24" s="117" t="n">
-        <v>1144.15</v>
+        <v>1016.68</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>466.7306451612905</v>
+        <v>468.2929032258064</v>
       </c>
       <c r="T24" s="118" t="n">
-        <v>0.6889833333333336</v>
+        <v>0.8539458823529411</v>
       </c>
       <c r="U24" s="117" t="n">
-        <v>17.07686567164179</v>
+        <v>17.23186440677966</v>
       </c>
       <c r="V24" s="117" t="n">
-        <v>-8.923134328358209</v>
+        <v>-8.76813559322034</v>
       </c>
       <c r="W24" s="120" t="inlineStr"/>
     </row>
@@ -2440,19 +2424,17 @@
       <c r="L25" s="119" t="n"/>
       <c r="M25" s="119" t="n"/>
       <c r="N25" s="119" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O25" s="119" t="n"/>
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>400.4</v>
+        <v>144.47</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
-      <c r="U25" s="117" t="n">
-        <v>400.4</v>
-      </c>
+      <c r="U25" s="117" t="n"/>
       <c r="V25" s="117" t="n"/>
       <c r="W25" s="120" t="inlineStr"/>
     </row>
@@ -2488,34 +2470,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>925.8414956244528</v>
+        <v>749.4907345531284</v>
       </c>
       <c r="N26" s="125" t="n">
-        <v>967</v>
+        <v>863</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>41.1585043755473</v>
+        <v>113.5092654468716</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>21000</v>
+        <v>17000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>26387.808067</v>
+        <v>21792.800088</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>5387.808066999998</v>
+        <v>4792.800088</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>0.2565622889047618</v>
+        <v>0.2819294169411764</v>
       </c>
       <c r="U26" s="123" t="n">
-        <v>27.28832271664943</v>
+        <v>25.25237553650058</v>
       </c>
       <c r="V26" s="123" t="n">
-        <v>4.606254458479473</v>
+        <v>2.570307278330624</v>
       </c>
       <c r="W26" s="126" t="n"/>
     </row>
@@ -2563,28 +2545,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>301.0752688172043</v>
+        <v>243.7275985663082</v>
       </c>
       <c r="N27" s="119" t="n">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-114.0752688172043</v>
+        <v>-68.72759856630825</v>
       </c>
       <c r="P27" s="117" t="n">
-        <v>129.0322580645161</v>
+        <v>173.9130434782609</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>2709.677419354839</v>
+        <v>2260.869565217391</v>
       </c>
       <c r="R27" s="117" t="n">
-        <v>1683</v>
+        <v>1575</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-1026.677419354838</v>
+        <v>-685.8695652173915</v>
       </c>
       <c r="T27" s="118" t="n">
-        <v>-0.3788928571428571</v>
+        <v>-0.3033653846153846</v>
       </c>
       <c r="U27" s="117" t="n">
         <v>9</v>
@@ -2638,28 +2620,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>445.6706281833617</v>
+        <v>360.7809847198643</v>
       </c>
       <c r="N28" s="119" t="n">
-        <v>371</v>
+        <v>360</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-74.67062818336171</v>
+        <v>-0.7809847198642501</v>
       </c>
       <c r="P28" s="117" t="n">
-        <v>161.2903225806452</v>
+        <v>217.3913043478261</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>3387.096774193548</v>
+        <v>2826.086956521739</v>
       </c>
       <c r="R28" s="117" t="n">
-        <v>2819.6</v>
+        <v>2736</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-567.4967741935484</v>
+        <v>-90.086956521739</v>
       </c>
       <c r="T28" s="118" t="n">
-        <v>-0.1675466666666666</v>
+        <v>-0.031876923076923</v>
       </c>
       <c r="U28" s="117" t="n">
         <v>7.6</v>
@@ -2713,28 +2695,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>169.3548387096774</v>
+        <v>137.0967741935484</v>
       </c>
       <c r="N29" s="119" t="n">
-        <v>240</v>
+        <v>223</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>70.64516129032259</v>
+        <v>85.90322580645162</v>
       </c>
       <c r="P29" s="117" t="n">
-        <v>64.51612903225806</v>
+        <v>86.95652173913044</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>1354.838709677419</v>
+        <v>1130.434782608696</v>
       </c>
       <c r="R29" s="117" t="n">
-        <v>1920</v>
+        <v>1784</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>565.1612903225807</v>
+        <v>653.5652173913043</v>
       </c>
       <c r="T29" s="118" t="n">
-        <v>0.4171428571428572</v>
+        <v>0.578153846153846</v>
       </c>
       <c r="U29" s="117" t="n">
         <v>8</v>
@@ -2776,34 +2758,34 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>916.1007357102434</v>
+        <v>741.6053574797209</v>
       </c>
       <c r="N30" s="125" t="n">
-        <v>798</v>
+        <v>758</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-118.1007357102434</v>
+        <v>16.39464252027915</v>
       </c>
       <c r="P30" s="123" t="n">
-        <v>354.8387096774193</v>
+        <v>478.2608695652174</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>7451.612903225806</v>
+        <v>6217.391304347826</v>
       </c>
       <c r="R30" s="123" t="n">
-        <v>6422.6</v>
+        <v>6095</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>-1029.012903225806</v>
+        <v>-122.391304347826</v>
       </c>
       <c r="T30" s="124" t="n">
-        <v>-0.1380926406926405</v>
+        <v>-0.0196853146853146</v>
       </c>
       <c r="U30" s="123" t="n">
-        <v>8.048370927318297</v>
+        <v>8.040897097625329</v>
       </c>
       <c r="V30" s="123" t="n">
-        <v>-0.0856831267357574</v>
+        <v>-0.0931569564287251</v>
       </c>
       <c r="W30" s="126" t="n"/>
     </row>
@@ -2839,34 +2821,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="131" t="n">
-        <v>2158.071263592761</v>
+        <v>1747.010070527473</v>
       </c>
       <c r="N31" s="131" t="n">
-        <v>2093</v>
+        <v>1912</v>
       </c>
       <c r="O31" s="131" t="n">
-        <v>-65.07126359276072</v>
+        <v>164.9899294725271</v>
       </c>
       <c r="P31" s="129" t="n">
-        <v>2032.258064516129</v>
+        <v>2155.680224403927</v>
       </c>
       <c r="Q31" s="129" t="n">
-        <v>42677.41935483871</v>
+        <v>34733.52033660589</v>
       </c>
       <c r="R31" s="129" t="n">
-        <v>47454.958128</v>
+        <v>40414.232334</v>
       </c>
       <c r="S31" s="129" t="n">
-        <v>4777.538773161286</v>
+        <v>5680.711997394108</v>
       </c>
       <c r="T31" s="130" t="n">
-        <v>0.1119453529614511</v>
+        <v>0.1635512882754693</v>
       </c>
       <c r="U31" s="129" t="n">
-        <v>22.67317636311515</v>
+        <v>21.13715080230126</v>
       </c>
       <c r="V31" s="129" t="n">
-        <v>2.897453441069807</v>
+        <v>1.361427880255917</v>
       </c>
       <c r="W31" s="132" t="n"/>
     </row>
@@ -3129,13 +3111,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3168,27 +3150,22 @@
       </c>
       <c r="L2" s="135" t="n"/>
       <c r="N2" s="135" t="n"/>
-      <c r="R2" t="n">
-        <v>66</v>
-      </c>
       <c r="T2" s="135" t="n">
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>6435.483870967741</v>
+        <v>5209.677419354838</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>6924.614962</v>
+        <v>5794.215866</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>489.1310910322582</v>
+        <v>584.5384466451615</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0760053324411027</v>
-      </c>
-      <c r="Y2" s="135" t="n">
-        <v>104.9184085151515</v>
-      </c>
+        <v>0.1122024262910217</v>
+      </c>
+      <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
       <c r="AA2" t="inlineStr">
         <is>
@@ -3204,12 +3181,12 @@
       <c r="AD2" s="137" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_3;crm:stale</t>
+          <t>google:ok;google:includes_excel_row_3</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>area_clienti_uniform</t>
+          <t>area_clienti_total</t>
         </is>
       </c>
     </row>
@@ -3220,13 +3197,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3255,9 +3232,6 @@
       <c r="K3" s="136" t="n"/>
       <c r="L3" s="135" t="n"/>
       <c r="N3" s="135" t="n"/>
-      <c r="R3" t="n">
-        <v>66</v>
-      </c>
       <c r="T3" s="135" t="n"/>
       <c r="U3" s="135" t="n"/>
       <c r="V3" s="135" t="n"/>
@@ -3274,12 +3248,12 @@
       <c r="AD3" s="137" t="inlineStr"/>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_2;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_2</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>area_clienti_uniform</t>
+          <t>area_clienti_total</t>
         </is>
       </c>
     </row>
@@ -3290,13 +3264,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3329,27 +3303,22 @@
       </c>
       <c r="L4" s="135" t="n"/>
       <c r="N4" s="135" t="n"/>
-      <c r="R4" t="n">
-        <v>66</v>
-      </c>
       <c r="T4" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>1016.129032258065</v>
+        <v>822.5806451612904</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>1236.075099</v>
+        <v>1074.27638</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>219.9460667419353</v>
+        <v>251.6957348387096</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>0.2164548593333331</v>
-      </c>
-      <c r="Y4" s="135" t="n">
-        <v>18.72841059090909</v>
-      </c>
+        <v>0.3059830501960784</v>
+      </c>
+      <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
       <c r="AA4" t="inlineStr">
         <is>
@@ -3365,12 +3334,12 @@
       <c r="AD4" s="137" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_5;crm:stale</t>
+          <t>google:ok;google:includes_excel_row_5</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>area_clienti_uniform</t>
+          <t>area_clienti_total</t>
         </is>
       </c>
     </row>
@@ -3381,13 +3350,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3416,9 +3385,6 @@
       <c r="K5" s="136" t="n"/>
       <c r="L5" s="135" t="n"/>
       <c r="N5" s="135" t="n"/>
-      <c r="R5" t="n">
-        <v>65</v>
-      </c>
       <c r="T5" s="135" t="n"/>
       <c r="U5" s="135" t="n"/>
       <c r="V5" s="135" t="n"/>
@@ -3435,12 +3401,12 @@
       <c r="AD5" s="137" t="inlineStr"/>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_4;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_4</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>area_clienti_uniform</t>
+          <t>area_clienti_total</t>
         </is>
       </c>
     </row>
@@ -3451,13 +3417,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3490,27 +3456,22 @@
       </c>
       <c r="L6" s="135" t="n"/>
       <c r="N6" s="135" t="n"/>
-      <c r="R6" t="n">
-        <v>65</v>
-      </c>
       <c r="T6" s="135" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>6774.193548387097</v>
+        <v>5483.870967741936</v>
       </c>
       <c r="V6" s="135" t="n">
-        <v>6483.86</v>
+        <v>5657.94</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-290.3335483870969</v>
+        <v>174.069032258064</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.0428587619047619</v>
-      </c>
-      <c r="Y6" s="135" t="n">
-        <v>99.75169230769232</v>
-      </c>
+        <v>0.0317419999999999</v>
+      </c>
+      <c r="Y6" s="135" t="n"/>
       <c r="Z6" s="135" t="n"/>
       <c r="AA6" t="inlineStr">
         <is>
@@ -3526,12 +3487,12 @@
       <c r="AD6" s="137" t="inlineStr"/>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>area_clienti_uniform</t>
+          <t>area_clienti_total</t>
         </is>
       </c>
     </row>
@@ -3542,13 +3503,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E7" t="n">
         <v>26</v>
@@ -3595,28 +3556,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q7" t="n">
-        <v>301.0752688172043</v>
+        <v>243.7275985663082</v>
       </c>
       <c r="R7" t="n">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="S7" t="n">
-        <v>-114.0752688172043</v>
+        <v>-68.72759856630825</v>
       </c>
       <c r="T7" s="135" t="n">
-        <v>129.0322580645161</v>
+        <v>173.9130434782609</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>2709.677419354839</v>
+        <v>2260.869565217391</v>
       </c>
       <c r="V7" s="135" t="n">
-        <v>1683</v>
+        <v>1575</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>-1026.677419354838</v>
+        <v>-685.8695652173915</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>-0.3788928571428571</v>
+        <v>-0.3033653846153846</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>9</v>
@@ -3629,7 +3590,7 @@
       <c r="AD7" s="137" t="inlineStr"/>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>manual:no_ads_source;crm:stale</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -3645,13 +3606,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E8" t="n">
         <v>25</v>
@@ -3698,28 +3659,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q8" t="n">
-        <v>445.6706281833617</v>
+        <v>360.7809847198643</v>
       </c>
       <c r="R8" t="n">
-        <v>371</v>
+        <v>360</v>
       </c>
       <c r="S8" t="n">
-        <v>-74.67062818336171</v>
+        <v>-0.7809847198642501</v>
       </c>
       <c r="T8" s="135" t="n">
-        <v>161.2903225806452</v>
+        <v>217.3913043478261</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>3387.096774193548</v>
+        <v>2826.086956521739</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>2819.6</v>
+        <v>2736</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>-567.4967741935484</v>
+        <v>-90.086956521739</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>-0.1675466666666666</v>
+        <v>-0.031876923076923</v>
       </c>
       <c r="Y8" s="135" t="n">
         <v>7.6</v>
@@ -3732,7 +3693,7 @@
       <c r="AD8" s="137" t="inlineStr"/>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>manual:no_ads_source;crm:stale</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -3748,13 +3709,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3801,28 +3762,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>169.3548387096774</v>
+        <v>137.0967741935484</v>
       </c>
       <c r="R9" t="n">
-        <v>240</v>
+        <v>223</v>
       </c>
       <c r="S9" t="n">
-        <v>70.64516129032259</v>
+        <v>85.90322580645162</v>
       </c>
       <c r="T9" s="135" t="n">
-        <v>64.51612903225806</v>
+        <v>86.95652173913044</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>1354.838709677419</v>
+        <v>1130.434782608696</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>1920</v>
+        <v>1784</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>565.1612903225807</v>
+        <v>653.5652173913043</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.4171428571428572</v>
+        <v>0.578153846153846</v>
       </c>
       <c r="Y9" s="135" t="n">
         <v>8</v>
@@ -3835,7 +3796,7 @@
       <c r="AD9" s="137" t="inlineStr"/>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>manual:no_ads_source;crm:stale</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -3851,13 +3812,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E10" t="n">
         <v>9</v>
@@ -3904,34 +3865,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q10" t="n">
-        <v>158.357771260997</v>
+        <v>128.1943862589024</v>
       </c>
       <c r="R10" t="n">
         <v>61</v>
       </c>
       <c r="S10" t="n">
-        <v>-97.35777126099704</v>
+        <v>-67.19438625890237</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>6096.774193548387</v>
+        <v>4935.483870967741</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>6653.326913999999</v>
+        <v>5490.756616000001</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>556.552720451612</v>
+        <v>555.2727450322591</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0912864250476189</v>
+        <v>0.1125062424575165</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>109.0709330163934</v>
+        <v>90.01240354098361</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>70.57093301639343</v>
+        <v>51.51240354098361</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -3947,7 +3908,7 @@
       <c r="AD10" s="137" t="inlineStr"/>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_10;crm:stale</t>
+          <t>google:ok;google:includes_excel_row_10</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -3963,13 +3924,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E11" t="n">
         <v>10</v>
@@ -3999,7 +3960,7 @@
       <c r="L11" s="135" t="n"/>
       <c r="N11" s="135" t="n"/>
       <c r="R11" t="n">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="T11" s="135" t="n"/>
       <c r="U11" s="135" t="n"/>
@@ -4017,7 +3978,7 @@
       <c r="AD11" s="137" t="inlineStr"/>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_9;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_9</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -4033,13 +3994,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E12" t="n">
         <v>8</v>
@@ -4086,34 +4047,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q12" t="n">
-        <v>79.69639468690701</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="R12" t="n">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="S12" t="n">
-        <v>31.30360531309299</v>
+        <v>33.48387096774194</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>2709.677419354839</v>
+        <v>2193.548387096774</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>3552.685198</v>
+        <v>3069.617174</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>843.0077786451616</v>
+        <v>876.0687869032258</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.3111100135476192</v>
+        <v>0.3993842999117647</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>32.00617295495496</v>
+        <v>31.3226242244898</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>-1.993827045045045</v>
+        <v>-2.677375775510203</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
@@ -4129,7 +4090,7 @@
       <c r="AD12" s="137" t="inlineStr"/>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:ok</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -4145,13 +4106,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4198,34 +4159,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>17.82682512733446</v>
+        <v>14.43123938879457</v>
       </c>
       <c r="R13" t="n">
         <v>5</v>
       </c>
       <c r="S13" t="n">
-        <v>-12.82682512733446</v>
+        <v>-9.431239388794566</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>677.4193548387096</v>
+        <v>548.3870967741935</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>667.311784</v>
+        <v>510.988722</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-10.10757083870965</v>
+        <v>-37.39837477419354</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.0149206998095237</v>
+        <v>-0.0681970363529411</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>133.4623568</v>
+        <v>102.1977444</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>95.46235679999999</v>
+        <v>64.1977444</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -4241,7 +4202,7 @@
       <c r="AD13" s="137" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_12;crm:stale</t>
+          <t>google:ok;google:includes_excel_row_12</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -4257,13 +4218,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -4310,34 +4271,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q14" t="n">
-        <v>2.709677419354839</v>
+        <v>2.193548387096774</v>
       </c>
       <c r="R14" t="n">
         <v>2</v>
       </c>
       <c r="S14" t="n">
-        <v>-0.7096774193548385</v>
+        <v>-0.193548387096774</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>677.4193548387096</v>
+        <v>548.3870967741935</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>704.740261</v>
+        <v>630.160373</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>27.3209061612904</v>
+        <v>81.77327622580651</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>0.0403308614761905</v>
+        <v>0.1491159742941177</v>
       </c>
       <c r="Y14" s="135" t="n">
-        <v>352.3701305</v>
+        <v>315.0801865</v>
       </c>
       <c r="Z14" s="135" t="n">
-        <v>102.3701305</v>
+        <v>65.08018650000002</v>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
@@ -4353,7 +4314,7 @@
       <c r="AD14" s="137" t="inlineStr"/>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_14;crm:stale</t>
+          <t>google:ok;google:includes_excel_row_14</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -4369,13 +4330,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E15" t="n">
         <v>14</v>
@@ -4423,7 +4384,7 @@
       <c r="AD15" s="137" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_13;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_13</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -4439,13 +4400,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E16" t="n">
         <v>12</v>
@@ -4475,7 +4436,7 @@
       <c r="L16" s="135" t="n"/>
       <c r="N16" s="135" t="n"/>
       <c r="R16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T16" s="135" t="n"/>
       <c r="U16" s="135" t="n"/>
@@ -4493,7 +4454,7 @@
       <c r="AD16" s="137" t="inlineStr"/>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_11;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_11</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -4509,13 +4470,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E17" t="n">
         <v>21</v>
@@ -4562,34 +4523,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q17" t="n">
-        <v>2.822580645161291</v>
+        <v>2.28494623655914</v>
       </c>
       <c r="R17" t="n">
         <v>4</v>
       </c>
       <c r="S17" t="n">
-        <v>1.177419354838709</v>
+        <v>1.71505376344086</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>338.7096774193548</v>
+        <v>274.1935483870968</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>323.59</v>
+        <v>283.27</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-15.11967741935484</v>
+        <v>9.076451612903211</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0446390476190476</v>
+        <v>0.0331023529411764</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>80.89749999999999</v>
+        <v>70.8175</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>-39.10250000000001</v>
+        <v>-49.1825</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr">
@@ -4600,7 +4561,7 @@
       <c r="AD17" s="137" t="inlineStr"/>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
@@ -4616,13 +4577,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4669,34 +4630,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>8.46774193548387</v>
+        <v>6.854838709677419</v>
       </c>
       <c r="R18" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="S18" t="n">
-        <v>23.53225806451613</v>
+        <v>24.14516129032258</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>338.7096774193548</v>
+        <v>274.1935483870968</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>365.93</v>
+        <v>322.95</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>27.22032258064519</v>
+        <v>48.75645161290322</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>0.08036476190476199</v>
+        <v>0.1778176470588235</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>11.4353125</v>
+        <v>10.41774193548387</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>-28.5646875</v>
+        <v>-29.58225806451613</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr">
@@ -4707,7 +4668,7 @@
       <c r="AD18" s="137" t="inlineStr"/>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
@@ -4723,13 +4684,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4776,34 +4737,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>7.526881720430107</v>
+        <v>6.093189964157706</v>
       </c>
       <c r="R19" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="S19" t="n">
-        <v>11.47311827956989</v>
+        <v>10.9068100358423</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>677.4193548387096</v>
+        <v>548.3870967741935</v>
       </c>
       <c r="V19" s="135" t="n">
-        <v>660.22</v>
+        <v>581.76</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-17.19935483870961</v>
+        <v>33.37290322580645</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.0253895238095237</v>
+        <v>0.0608564705882353</v>
       </c>
       <c r="Y19" s="135" t="n">
-        <v>34.74842105263158</v>
+        <v>34.22117647058823</v>
       </c>
       <c r="Z19" s="135" t="n">
-        <v>-55.25157894736842</v>
+        <v>-55.77882352941177</v>
       </c>
       <c r="AB19" s="137" t="inlineStr"/>
       <c r="AC19" s="137" t="inlineStr">
@@ -4814,7 +4775,7 @@
       <c r="AD19" s="137" t="inlineStr"/>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
@@ -4830,13 +4791,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E20" t="n">
         <v>17</v>
@@ -4883,34 +4844,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q20" t="n">
-        <v>529.233870967742</v>
+        <v>428.4274193548387</v>
       </c>
       <c r="R20" t="n">
-        <v>417</v>
+        <v>367</v>
       </c>
       <c r="S20" t="n">
-        <v>-112.233870967742</v>
+        <v>-61.42741935483872</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>6774.193548387097</v>
+        <v>5483.870967741936</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>9220.65</v>
+        <v>7444.1</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>2446.456451612903</v>
+        <v>1960.229032258065</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>0.3611435714285714</v>
+        <v>0.3574535294117647</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>22.11187050359712</v>
+        <v>20.28365122615804</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>9.31187050359712</v>
+        <v>7.483651226158038</v>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
@@ -4926,7 +4887,7 @@
       <c r="AD20" s="137" t="inlineStr"/>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr">
@@ -4942,13 +4903,13 @@
         </is>
       </c>
       <c r="B21" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C21" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D21" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4995,34 +4956,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>25.40322580645161</v>
+        <v>20.56451612903226</v>
       </c>
       <c r="R21" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S21" t="n">
-        <v>-3.403225806451612</v>
+        <v>0.4354838709677402</v>
       </c>
       <c r="T21" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="135" t="n">
-        <v>1016.129032258065</v>
+        <v>822.5806451612904</v>
       </c>
       <c r="V21" s="135" t="n">
-        <v>1239.425384</v>
+        <v>1057.013242</v>
       </c>
       <c r="W21" s="135" t="n">
-        <v>223.2963517419353</v>
+        <v>234.4325968387096</v>
       </c>
       <c r="X21" s="136" t="n">
-        <v>0.2197519652063489</v>
+        <v>0.2849964902745097</v>
       </c>
       <c r="Y21" s="135" t="n">
-        <v>56.33751745454545</v>
+        <v>50.3339639047619</v>
       </c>
       <c r="Z21" s="135" t="n">
-        <v>16.33751745454545</v>
+        <v>10.3339639047619</v>
       </c>
       <c r="AB21" s="137" t="inlineStr">
         <is>
@@ -5033,7 +4994,7 @@
       <c r="AD21" s="137" t="inlineStr"/>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:ok</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
@@ -5049,13 +5010,13 @@
         </is>
       </c>
       <c r="B22" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C22" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D22" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -5102,34 +5063,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>67.74193548387096</v>
+        <v>54.83870967741935</v>
       </c>
       <c r="R22" t="n">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="S22" t="n">
-        <v>46.25806451612904</v>
+        <v>47.16129032258065</v>
       </c>
       <c r="T22" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="135" t="n">
-        <v>1016.129032258065</v>
+        <v>822.5806451612904</v>
       </c>
       <c r="V22" s="135" t="n">
-        <v>1455.378526</v>
+        <v>1241.033961</v>
       </c>
       <c r="W22" s="135" t="n">
-        <v>439.2494937419353</v>
+        <v>418.4533158387097</v>
       </c>
       <c r="X22" s="136" t="n">
-        <v>0.4322772795555554</v>
+        <v>0.5087079525882353</v>
       </c>
       <c r="Y22" s="135" t="n">
-        <v>12.76647829824561</v>
+        <v>12.16699961764706</v>
       </c>
       <c r="Z22" s="135" t="n">
-        <v>-2.233521701754386</v>
+        <v>-2.833000382352941</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -5145,7 +5106,7 @@
       <c r="AD22" s="137" t="inlineStr"/>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:ok</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
@@ -5161,13 +5122,13 @@
         </is>
       </c>
       <c r="B23" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C23" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D23" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5214,34 +5175,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>26.0545905707196</v>
+        <v>21.09181141439206</v>
       </c>
       <c r="R23" t="n">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="S23" t="n">
-        <v>40.9454094292804</v>
+        <v>37.90818858560795</v>
       </c>
       <c r="T23" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="135" t="n">
-        <v>677.4193548387096</v>
+        <v>548.3870967741935</v>
       </c>
       <c r="V23" s="135" t="n">
-        <v>1144.15</v>
+        <v>1016.68</v>
       </c>
       <c r="W23" s="135" t="n">
-        <v>466.7306451612905</v>
+        <v>468.2929032258064</v>
       </c>
       <c r="X23" s="136" t="n">
-        <v>0.6889833333333336</v>
+        <v>0.8539458823529411</v>
       </c>
       <c r="Y23" s="135" t="n">
-        <v>17.07686567164179</v>
+        <v>17.23186440677966</v>
       </c>
       <c r="Z23" s="135" t="n">
-        <v>-8.923134328358209</v>
+        <v>-8.76813559322034</v>
       </c>
       <c r="AB23" s="137" t="inlineStr"/>
       <c r="AC23" s="137" t="inlineStr">
@@ -5252,7 +5213,7 @@
       <c r="AD23" s="137" t="inlineStr"/>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -5268,13 +5229,13 @@
         </is>
       </c>
       <c r="B24" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C24" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D24" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5306,18 +5267,16 @@
       <c r="L24" s="135" t="n"/>
       <c r="N24" s="135" t="n"/>
       <c r="R24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T24" s="135" t="n"/>
       <c r="U24" s="135" t="n"/>
       <c r="V24" s="135" t="n">
-        <v>400.4</v>
+        <v>144.47</v>
       </c>
       <c r="W24" s="135" t="n"/>
       <c r="X24" s="136" t="n"/>
-      <c r="Y24" s="135" t="n">
-        <v>400.4</v>
-      </c>
+      <c r="Y24" s="135" t="n"/>
       <c r="Z24" s="135" t="n"/>
       <c r="AB24" s="137" t="inlineStr"/>
       <c r="AC24" s="137" t="inlineStr">
@@ -5328,7 +5287,7 @@
       <c r="AD24" s="137" t="inlineStr"/>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
@@ -5344,13 +5303,13 @@
         </is>
       </c>
       <c r="B25" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C25" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D25" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5379,41 +5338,41 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>316.1290322580645</v>
+        <v>255.9139784946237</v>
       </c>
       <c r="R25" t="n">
-        <v>328</v>
+        <v>291</v>
       </c>
       <c r="S25" t="n">
-        <v>11.87096774193549</v>
+        <v>35.08602150537632</v>
       </c>
       <c r="T25" s="135" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="135" t="n">
-        <v>14225.8064516129</v>
+        <v>11516.12903225806</v>
       </c>
       <c r="V25" s="135" t="n">
-        <v>14644.550061</v>
+        <v>12526.432246</v>
       </c>
       <c r="W25" s="135" t="n">
-        <v>418.7436093870965</v>
+        <v>1010.303213741934</v>
       </c>
       <c r="X25" s="136" t="n">
-        <v>0.0294354918163265</v>
+        <v>0.0877294107170867</v>
       </c>
       <c r="Y25" s="135" t="n">
-        <v>44.64801847865854</v>
+        <v>43.04615892096219</v>
       </c>
       <c r="Z25" s="135" t="n">
-        <v>-0.3519815213414645</v>
+        <v>-1.953841079037808</v>
       </c>
       <c r="AB25" s="137" t="inlineStr"/>
       <c r="AC25" s="137" t="inlineStr"/>
       <c r="AD25" s="137" t="inlineStr"/>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>partial;crm:stale</t>
+          <t>partial</t>
         </is>
       </c>
     </row>
@@ -5424,13 +5383,13 @@
         </is>
       </c>
       <c r="B26" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C26" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D26" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5464,41 +5423,41 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>925.8414956244528</v>
+        <v>749.4907345531284</v>
       </c>
       <c r="R26" t="n">
-        <v>967</v>
+        <v>863</v>
       </c>
       <c r="S26" t="n">
-        <v>41.1585043755473</v>
+        <v>113.5092654468716</v>
       </c>
       <c r="T26" s="135" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="135" t="n">
-        <v>21000</v>
+        <v>17000</v>
       </c>
       <c r="V26" s="135" t="n">
-        <v>26387.808067</v>
+        <v>21792.800088</v>
       </c>
       <c r="W26" s="135" t="n">
-        <v>5387.808066999998</v>
+        <v>4792.800088</v>
       </c>
       <c r="X26" s="136" t="n">
-        <v>0.2565622889047618</v>
+        <v>0.2819294169411764</v>
       </c>
       <c r="Y26" s="135" t="n">
-        <v>27.28832271664943</v>
+        <v>25.25237553650058</v>
       </c>
       <c r="Z26" s="135" t="n">
-        <v>4.606254458479473</v>
+        <v>2.570307278330624</v>
       </c>
       <c r="AB26" s="137" t="inlineStr"/>
       <c r="AC26" s="137" t="inlineStr"/>
       <c r="AD26" s="137" t="inlineStr"/>
       <c r="AE26" t="inlineStr">
         <is>
-          <t>partial;crm:stale</t>
+          <t>partial</t>
         </is>
       </c>
     </row>
@@ -5509,13 +5468,13 @@
         </is>
       </c>
       <c r="B27" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C27" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D27" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5549,41 +5508,41 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>916.1007357102434</v>
+        <v>741.6053574797209</v>
       </c>
       <c r="R27" t="n">
-        <v>798</v>
+        <v>758</v>
       </c>
       <c r="S27" t="n">
-        <v>-118.1007357102434</v>
+        <v>16.39464252027915</v>
       </c>
       <c r="T27" s="135" t="n">
-        <v>354.8387096774193</v>
+        <v>478.2608695652174</v>
       </c>
       <c r="U27" s="135" t="n">
-        <v>7451.612903225806</v>
+        <v>6217.391304347826</v>
       </c>
       <c r="V27" s="135" t="n">
-        <v>6422.6</v>
+        <v>6095</v>
       </c>
       <c r="W27" s="135" t="n">
-        <v>-1029.012903225806</v>
+        <v>-122.391304347826</v>
       </c>
       <c r="X27" s="136" t="n">
-        <v>-0.1380926406926405</v>
+        <v>-0.0196853146853146</v>
       </c>
       <c r="Y27" s="135" t="n">
-        <v>8.048370927318297</v>
+        <v>8.040897097625329</v>
       </c>
       <c r="Z27" s="135" t="n">
-        <v>-0.0856831267357574</v>
+        <v>-0.0931569564287251</v>
       </c>
       <c r="AB27" s="137" t="inlineStr"/>
       <c r="AC27" s="137" t="inlineStr"/>
       <c r="AD27" s="137" t="inlineStr"/>
       <c r="AE27" t="inlineStr">
         <is>
-          <t>success;crm:stale</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -5594,13 +5553,13 @@
         </is>
       </c>
       <c r="B28" s="134" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="C28" s="134" t="n">
         <v>46204</v>
       </c>
       <c r="D28" s="134" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5634,41 +5593,41 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>2158.071263592761</v>
+        <v>1747.010070527473</v>
       </c>
       <c r="R28" t="n">
-        <v>2093</v>
+        <v>1912</v>
       </c>
       <c r="S28" t="n">
-        <v>-65.07126359276072</v>
+        <v>164.9899294725271</v>
       </c>
       <c r="T28" s="135" t="n">
-        <v>2032.258064516129</v>
+        <v>2155.680224403927</v>
       </c>
       <c r="U28" s="135" t="n">
-        <v>42677.41935483871</v>
+        <v>34733.52033660589</v>
       </c>
       <c r="V28" s="135" t="n">
-        <v>47454.958128</v>
+        <v>40414.232334</v>
       </c>
       <c r="W28" s="135" t="n">
-        <v>4777.538773161286</v>
+        <v>5680.711997394108</v>
       </c>
       <c r="X28" s="136" t="n">
-        <v>0.1119453529614511</v>
+        <v>0.1635512882754693</v>
       </c>
       <c r="Y28" s="135" t="n">
-        <v>22.67317636311515</v>
+        <v>21.13715080230126</v>
       </c>
       <c r="Z28" s="135" t="n">
-        <v>2.897453441069807</v>
+        <v>1.361427880255917</v>
       </c>
       <c r="AB28" s="137" t="inlineStr"/>
       <c r="AC28" s="137" t="inlineStr"/>
       <c r="AD28" s="137" t="inlineStr"/>
       <c r="AE28" t="inlineStr">
         <is>
-          <t>partial;crm:stale</t>
+          <t>partial</t>
         </is>
       </c>
     </row>
@@ -5764,7 +5723,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5804,7 +5763,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5824,7 +5783,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46225.29189814815</v>
+        <v>46225.48482638889</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Unify legacy and new CRM campaign metrics
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -152,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="142">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -443,6 +443,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -872,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 17/07/2026  |  Ultimo aggiornamento: 22/07/2026 11:38</t>
+          <t>Periodo: 01/07/2026 - 17/07/2026  |  Ultimo aggiornamento: 22/07/2026 12:05</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1353,7 +1359,7 @@
       </c>
       <c r="W10" s="126" t="n"/>
     </row>
-    <row r="11" ht="36" customHeight="1" s="74">
+    <row r="11" ht="66" customHeight="1" s="74">
       <c r="A11" s="93" t="inlineStr">
         <is>
           <t>Lead Veloce</t>
@@ -1371,68 +1377,68 @@
       </c>
       <c r="D11" s="115" t="inlineStr">
         <is>
-          <t>22822606735</t>
+          <t>23968989759</t>
         </is>
       </c>
       <c r="E11" s="116" t="inlineStr">
         <is>
-          <t>DYN_VELOCE Cessione del Quinto [Esatta]</t>
+          <t>DYN_VELOCE Cessione del Quinto QUINTO DIGITALE</t>
         </is>
       </c>
       <c r="F11" s="117" t="n">
-        <v>9000</v>
+        <v>4000</v>
       </c>
       <c r="G11" s="118" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.06349206349206341</v>
       </c>
       <c r="H11" s="117" t="n">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="I11" s="119" t="n">
-        <v>15</v>
+        <v>5.714285714285714</v>
       </c>
       <c r="J11" s="117" t="n">
-        <v>38.5</v>
+        <v>34</v>
       </c>
       <c r="K11" s="119" t="n">
-        <v>233.7662337662338</v>
+        <v>117.6470588235294</v>
       </c>
       <c r="L11" s="119" t="n">
-        <v>7.540846250523669</v>
+        <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>128.1943862589024</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="N11" s="119" t="n">
-        <v>61</v>
+        <v>98</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-67.19438625890237</v>
+        <v>33.48387096774194</v>
       </c>
       <c r="P11" s="117" t="n">
-        <v>290.3225806451613</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>4935.483870967741</v>
+        <v>2193.548387096774</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>5490.756616000001</v>
+        <v>3069.617174</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>555.2727450322591</v>
+        <v>876.0687869032258</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.1125062424575165</v>
+        <v>0.3993842999117647</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>90.01240354098361</v>
+        <v>31.3226242244898</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>51.51240354098361</v>
+        <v>-2.677375775510203</v>
       </c>
       <c r="W11" s="120" t="inlineStr">
         <is>
-          <t>SWITCH fatto</t>
+          <t>diminuito cpa target - alzato a giugno per dare più dati alla campagna che è stata rilanciata da zero</t>
         </is>
       </c>
     </row>
@@ -1454,117 +1460,117 @@
       </c>
       <c r="D12" s="115" t="inlineStr">
         <is>
+          <t>22822606735</t>
+        </is>
+      </c>
+      <c r="E12" s="116" t="inlineStr">
+        <is>
+          <t>DYN_VELOCE Cessione del Quinto [Esatta]</t>
+        </is>
+      </c>
+      <c r="F12" s="117" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G12" s="118" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="H12" s="117" t="n">
+        <v>600</v>
+      </c>
+      <c r="I12" s="119" t="n">
+        <v>15</v>
+      </c>
+      <c r="J12" s="117" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="K12" s="127" t="n">
+        <v>233.7662337662338</v>
+      </c>
+      <c r="L12" s="127" t="n">
+        <v>7.540846250523669</v>
+      </c>
+      <c r="M12" s="127" t="n">
+        <v>128.1943862589024</v>
+      </c>
+      <c r="N12" s="119" t="n">
+        <v>61</v>
+      </c>
+      <c r="O12" s="127" t="n">
+        <v>24.80561374109763</v>
+      </c>
+      <c r="P12" s="117" t="n">
+        <v>290.3225806451613</v>
+      </c>
+      <c r="Q12" s="117" t="n">
+        <v>4935.483870967741</v>
+      </c>
+      <c r="R12" s="117" t="n">
+        <v>5490.756616000001</v>
+      </c>
+      <c r="S12" s="117" t="n">
+        <v>555.2727450322591</v>
+      </c>
+      <c r="T12" s="118" t="n">
+        <v>0.1125062424575165</v>
+      </c>
+      <c r="U12" s="128" t="n">
+        <v>35.88729814379085</v>
+      </c>
+      <c r="V12" s="128" t="n">
+        <v>-2.612701856209149</v>
+      </c>
+      <c r="W12" s="120" t="inlineStr">
+        <is>
+          <t>SWITCH fatto</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1" s="74">
+      <c r="A13" s="93" t="inlineStr">
+        <is>
+          <t>Lead Veloce</t>
+        </is>
+      </c>
+      <c r="B13" s="94" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C13" s="94" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="D13" s="115" t="inlineStr">
+        <is>
           <t>23990314506</t>
         </is>
       </c>
-      <c r="E12" s="116" t="inlineStr">
+      <c r="E13" s="116" t="inlineStr">
         <is>
           <t>DYN_VELOCE Cessione del Quinto [Esatta] QUINTO DIGITALE</t>
         </is>
       </c>
-      <c r="F12" s="117" t="n"/>
-      <c r="G12" s="118" t="n"/>
-      <c r="H12" s="117" t="n"/>
-      <c r="I12" s="119" t="n"/>
-      <c r="J12" s="117" t="n"/>
-      <c r="K12" s="119" t="n"/>
-      <c r="L12" s="119" t="n"/>
-      <c r="M12" s="119" t="n"/>
-      <c r="N12" s="119" t="n">
+      <c r="F13" s="117" t="n"/>
+      <c r="G13" s="118" t="n"/>
+      <c r="H13" s="117" t="n"/>
+      <c r="I13" s="119" t="n"/>
+      <c r="J13" s="117" t="n"/>
+      <c r="K13" s="113" t="n"/>
+      <c r="L13" s="113" t="n"/>
+      <c r="M13" s="113" t="n"/>
+      <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
-      <c r="O12" s="119" t="n"/>
-      <c r="P12" s="117" t="n"/>
-      <c r="Q12" s="117" t="n"/>
-      <c r="R12" s="117" t="n"/>
-      <c r="S12" s="117" t="n"/>
-      <c r="T12" s="118" t="n"/>
-      <c r="U12" s="117" t="n"/>
-      <c r="V12" s="117" t="n"/>
-      <c r="W12" s="120" t="inlineStr"/>
-    </row>
-    <row r="13" ht="66" customHeight="1" s="74">
-      <c r="A13" s="93" t="inlineStr">
-        <is>
-          <t>Lead Veloce</t>
-        </is>
-      </c>
-      <c r="B13" s="94" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="C13" s="94" t="inlineStr">
-        <is>
-          <t>Search</t>
-        </is>
-      </c>
-      <c r="D13" s="115" t="inlineStr">
-        <is>
-          <t>23968989759</t>
-        </is>
-      </c>
-      <c r="E13" s="116" t="inlineStr">
-        <is>
-          <t>DYN_VELOCE Cessione del Quinto QUINTO DIGITALE</t>
-        </is>
-      </c>
-      <c r="F13" s="117" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G13" s="118" t="n">
-        <v>0.06349206349206341</v>
-      </c>
-      <c r="H13" s="117" t="n">
-        <v>700</v>
-      </c>
-      <c r="I13" s="119" t="n">
-        <v>5.714285714285714</v>
-      </c>
-      <c r="J13" s="117" t="n">
-        <v>34</v>
-      </c>
-      <c r="K13" s="119" t="n">
-        <v>117.6470588235294</v>
-      </c>
-      <c r="L13" s="119" t="n">
-        <v>3.795066413662239</v>
-      </c>
-      <c r="M13" s="119" t="n">
-        <v>64.51612903225806</v>
-      </c>
-      <c r="N13" s="119" t="n">
-        <v>98</v>
-      </c>
-      <c r="O13" s="119" t="n">
-        <v>33.48387096774194</v>
-      </c>
-      <c r="P13" s="117" t="n">
-        <v>129.0322580645161</v>
-      </c>
-      <c r="Q13" s="117" t="n">
-        <v>2193.548387096774</v>
-      </c>
-      <c r="R13" s="117" t="n">
-        <v>3069.617174</v>
-      </c>
-      <c r="S13" s="117" t="n">
-        <v>876.0687869032258</v>
-      </c>
-      <c r="T13" s="118" t="n">
-        <v>0.3993842999117647</v>
-      </c>
-      <c r="U13" s="117" t="n">
-        <v>31.3226242244898</v>
-      </c>
-      <c r="V13" s="117" t="n">
-        <v>-2.677375775510203</v>
-      </c>
-      <c r="W13" s="120" t="inlineStr">
-        <is>
-          <t>diminuito cpa target - alzato a giugno per dare più dati alla campagna che è stata rilanciata da zero</t>
-        </is>
-      </c>
+      <c r="O13" s="113" t="n"/>
+      <c r="P13" s="117" t="n"/>
+      <c r="Q13" s="117" t="n"/>
+      <c r="R13" s="117" t="n"/>
+      <c r="S13" s="117" t="n"/>
+      <c r="T13" s="118" t="n"/>
+      <c r="U13" s="113" t="n"/>
+      <c r="V13" s="113" t="n"/>
+      <c r="W13" s="120" t="inlineStr"/>
     </row>
     <row r="14" ht="51" customHeight="1" s="74">
       <c r="A14" s="93" t="inlineStr">
@@ -1607,20 +1613,20 @@
       <c r="J14" s="117" t="n">
         <v>38</v>
       </c>
-      <c r="K14" s="119" t="n">
+      <c r="K14" s="127" t="n">
         <v>26.31578947368421</v>
       </c>
-      <c r="L14" s="119" t="n">
+      <c r="L14" s="127" t="n">
         <v>0.8488964346349744</v>
       </c>
-      <c r="M14" s="119" t="n">
+      <c r="M14" s="127" t="n">
         <v>14.43123938879457</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>5</v>
       </c>
-      <c r="O14" s="119" t="n">
-        <v>-9.431239388794566</v>
+      <c r="O14" s="127" t="n">
+        <v>-5.431239388794566</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
@@ -1637,11 +1643,11 @@
       <c r="T14" s="118" t="n">
         <v>-0.0681970363529411</v>
       </c>
-      <c r="U14" s="117" t="n">
-        <v>102.1977444</v>
-      </c>
-      <c r="V14" s="117" t="n">
-        <v>64.1977444</v>
+      <c r="U14" s="128" t="n">
+        <v>56.77652466666667</v>
+      </c>
+      <c r="V14" s="128" t="n">
+        <v>18.77652466666667</v>
       </c>
       <c r="W14" s="120" t="inlineStr">
         <is>
@@ -1649,7 +1655,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="51" customHeight="1" s="74">
+    <row r="15" ht="36" customHeight="1" s="74">
       <c r="A15" s="93" t="inlineStr">
         <is>
           <t>Lead Veloce</t>
@@ -1667,117 +1673,117 @@
       </c>
       <c r="D15" s="115" t="inlineStr">
         <is>
+          <t>23993375943</t>
+        </is>
+      </c>
+      <c r="E15" s="116" t="inlineStr">
+        <is>
+          <t>DYN_VELOCE CQ Pensionati QUINTO DIGITALE</t>
+        </is>
+      </c>
+      <c r="F15" s="117" t="n"/>
+      <c r="G15" s="118" t="n"/>
+      <c r="H15" s="117" t="n"/>
+      <c r="I15" s="119" t="n"/>
+      <c r="J15" s="117" t="n"/>
+      <c r="K15" s="113" t="n"/>
+      <c r="L15" s="113" t="n"/>
+      <c r="M15" s="113" t="n"/>
+      <c r="N15" s="119" t="n">
+        <v>4</v>
+      </c>
+      <c r="O15" s="113" t="n"/>
+      <c r="P15" s="117" t="n"/>
+      <c r="Q15" s="117" t="n"/>
+      <c r="R15" s="117" t="n"/>
+      <c r="S15" s="117" t="n"/>
+      <c r="T15" s="118" t="n"/>
+      <c r="U15" s="113" t="n"/>
+      <c r="V15" s="113" t="n"/>
+      <c r="W15" s="120" t="inlineStr"/>
+    </row>
+    <row r="16" ht="51" customHeight="1" s="74">
+      <c r="A16" s="93" t="inlineStr">
+        <is>
+          <t>Lead Veloce</t>
+        </is>
+      </c>
+      <c r="B16" s="94" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C16" s="94" t="inlineStr">
+        <is>
+          <t>Search</t>
+        </is>
+      </c>
+      <c r="D16" s="115" t="inlineStr">
+        <is>
           <t>23267957688</t>
         </is>
       </c>
-      <c r="E15" s="116" t="inlineStr">
+      <c r="E16" s="116" t="inlineStr">
         <is>
           <t>DYN_VELOCE CQ Pensionati ESTERO - Paesi Prioritari</t>
         </is>
       </c>
-      <c r="F15" s="117" t="n">
+      <c r="F16" s="117" t="n">
         <v>1000</v>
       </c>
-      <c r="G15" s="118" t="n">
+      <c r="G16" s="118" t="n">
         <v>0.0158730158730158</v>
       </c>
-      <c r="H15" s="117" t="n">
+      <c r="H16" s="117" t="n">
         <v>1000</v>
       </c>
-      <c r="I15" s="119" t="n">
+      <c r="I16" s="119" t="n">
         <v>1</v>
       </c>
-      <c r="J15" s="117" t="n">
+      <c r="J16" s="117" t="n">
         <v>250</v>
       </c>
-      <c r="K15" s="119" t="n">
+      <c r="K16" s="127" t="n">
         <v>4</v>
       </c>
-      <c r="L15" s="119" t="n">
+      <c r="L16" s="127" t="n">
         <v>0.1290322580645161</v>
       </c>
-      <c r="M15" s="119" t="n">
+      <c r="M16" s="127" t="n">
         <v>2.193548387096774</v>
       </c>
-      <c r="N15" s="119" t="n">
+      <c r="N16" s="119" t="n">
         <v>2</v>
       </c>
-      <c r="O15" s="119" t="n">
+      <c r="O16" s="127" t="n">
         <v>-0.193548387096774</v>
       </c>
-      <c r="P15" s="117" t="n">
+      <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
-      <c r="Q15" s="117" t="n">
+      <c r="Q16" s="117" t="n">
         <v>548.3870967741935</v>
       </c>
-      <c r="R15" s="117" t="n">
+      <c r="R16" s="117" t="n">
         <v>630.160373</v>
       </c>
-      <c r="S15" s="117" t="n">
+      <c r="S16" s="117" t="n">
         <v>81.77327622580651</v>
       </c>
-      <c r="T15" s="118" t="n">
+      <c r="T16" s="118" t="n">
         <v>0.1491159742941177</v>
       </c>
-      <c r="U15" s="117" t="n">
+      <c r="U16" s="128" t="n">
         <v>315.0801865</v>
       </c>
-      <c r="V15" s="117" t="n">
+      <c r="V16" s="128" t="n">
         <v>65.08018650000002</v>
       </c>
-      <c r="W15" s="120" t="inlineStr">
+      <c r="W16" s="120" t="inlineStr">
         <is>
           <t>ATTIVATA nuova campagna - quando esce da apprendimento abbassare cpa target</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="36" customHeight="1" s="74">
-      <c r="A16" s="93" t="inlineStr">
-        <is>
-          <t>Lead Veloce</t>
-        </is>
-      </c>
-      <c r="B16" s="94" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="C16" s="94" t="inlineStr">
-        <is>
-          <t>Search</t>
-        </is>
-      </c>
-      <c r="D16" s="115" t="inlineStr">
-        <is>
-          <t>23993437149</t>
-        </is>
-      </c>
-      <c r="E16" s="116" t="inlineStr">
-        <is>
-          <t>DYN_VELOCE CQ Pensionati ESTERO - Paesi Prioritari QUINTO DIGITALE</t>
-        </is>
-      </c>
-      <c r="F16" s="117" t="n"/>
-      <c r="G16" s="118" t="n"/>
-      <c r="H16" s="117" t="n"/>
-      <c r="I16" s="119" t="n"/>
-      <c r="J16" s="117" t="n"/>
-      <c r="K16" s="119" t="n"/>
-      <c r="L16" s="119" t="n"/>
-      <c r="M16" s="119" t="n"/>
-      <c r="N16" s="119" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="119" t="n"/>
-      <c r="P16" s="117" t="n"/>
-      <c r="Q16" s="117" t="n"/>
-      <c r="R16" s="117" t="n"/>
-      <c r="S16" s="117" t="n"/>
-      <c r="T16" s="118" t="n"/>
-      <c r="U16" s="117" t="n"/>
-      <c r="V16" s="117" t="n"/>
-      <c r="W16" s="120" t="inlineStr"/>
     </row>
     <row r="17" ht="36" customHeight="1" s="74">
       <c r="A17" s="93" t="inlineStr">
@@ -1797,12 +1803,12 @@
       </c>
       <c r="D17" s="115" t="inlineStr">
         <is>
-          <t>23993375943</t>
+          <t>23993437149</t>
         </is>
       </c>
       <c r="E17" s="116" t="inlineStr">
         <is>
-          <t>DYN_VELOCE CQ Pensionati QUINTO DIGITALE</t>
+          <t>DYN_VELOCE CQ Pensionati ESTERO - Paesi Prioritari QUINTO DIGITALE</t>
         </is>
       </c>
       <c r="F17" s="117" t="n"/>
@@ -1810,23 +1816,23 @@
       <c r="H17" s="117" t="n"/>
       <c r="I17" s="119" t="n"/>
       <c r="J17" s="117" t="n"/>
-      <c r="K17" s="119" t="n"/>
-      <c r="L17" s="119" t="n"/>
-      <c r="M17" s="119" t="n"/>
+      <c r="K17" s="113" t="n"/>
+      <c r="L17" s="113" t="n"/>
+      <c r="M17" s="113" t="n"/>
       <c r="N17" s="119" t="n">
-        <v>4</v>
-      </c>
-      <c r="O17" s="119" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="O17" s="113" t="n"/>
       <c r="P17" s="117" t="n"/>
       <c r="Q17" s="117" t="n"/>
       <c r="R17" s="117" t="n"/>
       <c r="S17" s="117" t="n"/>
       <c r="T17" s="118" t="n"/>
-      <c r="U17" s="117" t="n"/>
-      <c r="V17" s="117" t="n"/>
+      <c r="U17" s="113" t="n"/>
+      <c r="V17" s="113" t="n"/>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
-    <row r="18" ht="36" customHeight="1" s="74">
+    <row r="18" ht="51" customHeight="1" s="74">
       <c r="A18" s="93" t="inlineStr">
         <is>
           <t>Lead Veloce</t>
@@ -1844,66 +1850,70 @@
       </c>
       <c r="D18" s="115" t="inlineStr">
         <is>
-          <t>6666147663775</t>
+          <t>6944411197975</t>
         </is>
       </c>
       <c r="E18" s="116" t="inlineStr">
         <is>
-          <t>[BMK 2025] LeadGen CQD PEN [Albania]</t>
+          <t>DYN_VELOCE New Creative Apr26</t>
         </is>
       </c>
       <c r="F18" s="117" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G18" s="118" t="n">
+        <v>0.1587301587301587</v>
+      </c>
+      <c r="H18" s="117" t="n">
         <v>500</v>
       </c>
-      <c r="G18" s="118" t="n">
-        <v>0.0079365079365079</v>
-      </c>
-      <c r="H18" s="117" t="n">
-        <v>540</v>
-      </c>
       <c r="I18" s="119" t="n">
-        <v>0.925925925925926</v>
+        <v>20</v>
       </c>
       <c r="J18" s="117" t="n">
-        <v>120</v>
+        <v>12.8</v>
       </c>
       <c r="K18" s="119" t="n">
-        <v>4.166666666666667</v>
+        <v>781.25</v>
       </c>
       <c r="L18" s="119" t="n">
-        <v>0.1344086021505376</v>
+        <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>2.28494623655914</v>
+        <v>428.4274193548387</v>
       </c>
       <c r="N18" s="119" t="n">
-        <v>4</v>
+        <v>367</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>1.71505376344086</v>
+        <v>-61.42741935483872</v>
       </c>
       <c r="P18" s="117" t="n">
-        <v>16.12903225806452</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>274.1935483870968</v>
+        <v>5483.870967741936</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>283.27</v>
+        <v>7444.1</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>9.076451612903211</v>
+        <v>1960.229032258065</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>0.0331023529411764</v>
+        <v>0.3574535294117647</v>
       </c>
       <c r="U18" s="117" t="n">
-        <v>70.8175</v>
+        <v>20.28365122615804</v>
       </c>
       <c r="V18" s="117" t="n">
-        <v>-49.1825</v>
-      </c>
-      <c r="W18" s="120" t="inlineStr"/>
+        <v>7.483651226158038</v>
+      </c>
+      <c r="W18" s="120" t="inlineStr">
+        <is>
+          <t>diminuito cpa target che era stato alzato per aiutare la campagna ad uscire dalla fase di apprendimento</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="36" customHeight="1" s="74">
       <c r="A19" s="93" t="inlineStr">
@@ -2063,7 +2073,7 @@
       </c>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
-    <row r="21" ht="51" customHeight="1" s="74">
+    <row r="21" ht="36" customHeight="1" s="74">
       <c r="A21" s="93" t="inlineStr">
         <is>
           <t>Lead Veloce</t>
@@ -2081,70 +2091,66 @@
       </c>
       <c r="D21" s="115" t="inlineStr">
         <is>
-          <t>6944411197975</t>
+          <t>6666147663775</t>
         </is>
       </c>
       <c r="E21" s="116" t="inlineStr">
         <is>
-          <t>DYN_VELOCE New Creative Apr26</t>
+          <t>[BMK 2025] LeadGen CQD PEN [Albania]</t>
         </is>
       </c>
       <c r="F21" s="117" t="n">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="G21" s="118" t="n">
-        <v>0.1587301587301587</v>
+        <v>0.0079365079365079</v>
       </c>
       <c r="H21" s="117" t="n">
-        <v>500</v>
+        <v>540</v>
       </c>
       <c r="I21" s="119" t="n">
-        <v>20</v>
+        <v>0.925925925925926</v>
       </c>
       <c r="J21" s="117" t="n">
-        <v>12.8</v>
+        <v>120</v>
       </c>
       <c r="K21" s="119" t="n">
-        <v>781.25</v>
+        <v>4.166666666666667</v>
       </c>
       <c r="L21" s="119" t="n">
-        <v>25.20161290322581</v>
+        <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>428.4274193548387</v>
+        <v>2.28494623655914</v>
       </c>
       <c r="N21" s="119" t="n">
-        <v>367</v>
+        <v>4</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-61.42741935483872</v>
+        <v>1.71505376344086</v>
       </c>
       <c r="P21" s="117" t="n">
-        <v>322.5806451612903</v>
+        <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>5483.870967741936</v>
+        <v>274.1935483870968</v>
       </c>
       <c r="R21" s="117" t="n">
-        <v>7444.1</v>
+        <v>283.27</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>1960.229032258065</v>
+        <v>9.076451612903211</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>0.3574535294117647</v>
+        <v>0.0331023529411764</v>
       </c>
       <c r="U21" s="117" t="n">
-        <v>20.28365122615804</v>
+        <v>70.8175</v>
       </c>
       <c r="V21" s="117" t="n">
-        <v>7.483651226158038</v>
-      </c>
-      <c r="W21" s="120" t="inlineStr">
-        <is>
-          <t>diminuito cpa target che era stato alzato per aiutare la campagna ad uscire dalla fase di apprendimento</t>
-        </is>
-      </c>
+        <v>-49.1825</v>
+      </c>
+      <c r="W21" s="120" t="inlineStr"/>
     </row>
     <row r="22" ht="21" customHeight="1" s="74">
       <c r="A22" s="93" t="inlineStr">
@@ -2520,56 +2526,56 @@
       <c r="D27" s="115" t="inlineStr"/>
       <c r="E27" s="116" t="inlineStr">
         <is>
-          <t>DEM DIGITOO</t>
+          <t>DEM DYNAMICS ADVICE ME</t>
         </is>
       </c>
       <c r="F27" s="117" t="n">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="G27" s="118" t="n">
-        <v>0.06349206349206341</v>
+        <v>0.07936507936507931</v>
       </c>
       <c r="H27" s="117" t="n">
-        <v>350</v>
+        <v>450</v>
       </c>
       <c r="I27" s="119" t="n">
-        <v>11.42857142857143</v>
+        <v>11.11111111111111</v>
       </c>
       <c r="J27" s="117" t="n">
-        <v>9</v>
+        <v>7.6</v>
       </c>
       <c r="K27" s="119" t="n">
-        <v>444.4444444444445</v>
+        <v>657.8947368421053</v>
       </c>
       <c r="L27" s="119" t="n">
-        <v>14.33691756272402</v>
+        <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>243.7275985663082</v>
+        <v>360.7809847198643</v>
       </c>
       <c r="N27" s="119" t="n">
-        <v>175</v>
+        <v>360</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-68.72759856630825</v>
+        <v>-0.7809847198642501</v>
       </c>
       <c r="P27" s="117" t="n">
-        <v>173.9130434782609</v>
+        <v>217.3913043478261</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>2260.869565217391</v>
+        <v>2826.086956521739</v>
       </c>
       <c r="R27" s="117" t="n">
-        <v>1575</v>
+        <v>2736</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-685.8695652173915</v>
+        <v>-90.086956521739</v>
       </c>
       <c r="T27" s="118" t="n">
-        <v>-0.3033653846153846</v>
+        <v>-0.031876923076923</v>
       </c>
       <c r="U27" s="117" t="n">
-        <v>9</v>
+        <v>7.6</v>
       </c>
       <c r="V27" s="117" t="n">
         <v>0</v>
@@ -2595,56 +2601,56 @@
       <c r="D28" s="115" t="inlineStr"/>
       <c r="E28" s="116" t="inlineStr">
         <is>
-          <t>DEM DYNAMICS ADVICE ME</t>
+          <t>DEM DIGITOO</t>
         </is>
       </c>
       <c r="F28" s="117" t="n">
-        <v>5000</v>
+        <v>4000</v>
       </c>
       <c r="G28" s="118" t="n">
-        <v>0.07936507936507931</v>
+        <v>0.06349206349206341</v>
       </c>
       <c r="H28" s="117" t="n">
-        <v>450</v>
+        <v>350</v>
       </c>
       <c r="I28" s="119" t="n">
-        <v>11.11111111111111</v>
+        <v>11.42857142857143</v>
       </c>
       <c r="J28" s="117" t="n">
-        <v>7.6</v>
+        <v>9</v>
       </c>
       <c r="K28" s="119" t="n">
-        <v>657.8947368421053</v>
+        <v>444.4444444444445</v>
       </c>
       <c r="L28" s="119" t="n">
-        <v>21.22241086587437</v>
+        <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>360.7809847198643</v>
+        <v>243.7275985663082</v>
       </c>
       <c r="N28" s="119" t="n">
-        <v>360</v>
+        <v>175</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-0.7809847198642501</v>
+        <v>-68.72759856630825</v>
       </c>
       <c r="P28" s="117" t="n">
-        <v>217.3913043478261</v>
+        <v>173.9130434782609</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>2826.086956521739</v>
+        <v>2260.869565217391</v>
       </c>
       <c r="R28" s="117" t="n">
-        <v>2736</v>
+        <v>1575</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-90.086956521739</v>
+        <v>-685.8695652173915</v>
       </c>
       <c r="T28" s="118" t="n">
-        <v>-0.031876923076923</v>
+        <v>-0.3033653846153846</v>
       </c>
       <c r="U28" s="117" t="n">
-        <v>7.6</v>
+        <v>9</v>
       </c>
       <c r="V28" s="117" t="n">
         <v>0</v>
@@ -2790,80 +2796,98 @@
       <c r="W30" s="126" t="n"/>
     </row>
     <row r="31" ht="21" customHeight="1" s="74">
-      <c r="A31" s="127" t="inlineStr">
+      <c r="A31" s="129" t="inlineStr">
         <is>
           <t>TOTALE GENERALE</t>
         </is>
       </c>
-      <c r="B31" s="128" t="n"/>
-      <c r="C31" s="128" t="n"/>
-      <c r="D31" s="128" t="n"/>
-      <c r="E31" s="128" t="n"/>
-      <c r="F31" s="129" t="n">
+      <c r="B31" s="130" t="n"/>
+      <c r="C31" s="130" t="n"/>
+      <c r="D31" s="130" t="n"/>
+      <c r="E31" s="130" t="n"/>
+      <c r="F31" s="131" t="n">
         <v>63000</v>
       </c>
-      <c r="G31" s="130" t="n">
+      <c r="G31" s="132" t="n">
         <v>1</v>
       </c>
-      <c r="H31" s="129" t="n">
+      <c r="H31" s="131" t="n">
         <v>745.0169133605773</v>
       </c>
-      <c r="I31" s="131" t="n">
+      <c r="I31" s="133" t="n">
         <v>84.56183862433862</v>
       </c>
-      <c r="J31" s="129" t="n">
+      <c r="J31" s="131" t="n">
         <v>19.77572292204534</v>
       </c>
-      <c r="K31" s="131" t="n">
+      <c r="K31" s="133" t="n">
         <v>3185.72424625598</v>
       </c>
-      <c r="L31" s="131" t="n">
+      <c r="L31" s="133" t="n">
         <v>102.7652982663219</v>
       </c>
-      <c r="M31" s="131" t="n">
+      <c r="M31" s="133" t="n">
         <v>1747.010070527473</v>
       </c>
-      <c r="N31" s="131" t="n">
+      <c r="N31" s="133" t="n">
         <v>1912</v>
       </c>
-      <c r="O31" s="131" t="n">
+      <c r="O31" s="133" t="n">
         <v>164.9899294725271</v>
       </c>
-      <c r="P31" s="129" t="n">
+      <c r="P31" s="131" t="n">
         <v>2155.680224403927</v>
       </c>
-      <c r="Q31" s="129" t="n">
+      <c r="Q31" s="131" t="n">
         <v>34733.52033660589</v>
       </c>
-      <c r="R31" s="129" t="n">
+      <c r="R31" s="131" t="n">
         <v>40414.232334</v>
       </c>
-      <c r="S31" s="129" t="n">
+      <c r="S31" s="131" t="n">
         <v>5680.711997394108</v>
       </c>
-      <c r="T31" s="130" t="n">
+      <c r="T31" s="132" t="n">
         <v>0.1635512882754693</v>
       </c>
-      <c r="U31" s="129" t="n">
+      <c r="U31" s="131" t="n">
         <v>21.13715080230126</v>
       </c>
-      <c r="V31" s="129" t="n">
+      <c r="V31" s="131" t="n">
         <v>1.361427880255917</v>
       </c>
-      <c r="W31" s="132" t="n"/>
+      <c r="W31" s="134" t="n"/>
     </row>
     <row r="32" ht="21" customHeight="1" s="74"/>
     <row r="33" ht="21" customHeight="1" s="74"/>
     <row r="34" ht="21" customHeight="1" s="74"/>
     <row r="35" ht="24" customHeight="1" s="74"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="24">
     <mergeCell ref="A30:E30"/>
+    <mergeCell ref="L12:L13"/>
+    <mergeCell ref="O16:O17"/>
+    <mergeCell ref="U16:U17"/>
+    <mergeCell ref="L14:L15"/>
     <mergeCell ref="A1:W1"/>
+    <mergeCell ref="M16:M17"/>
+    <mergeCell ref="K12:K13"/>
+    <mergeCell ref="M12:M13"/>
+    <mergeCell ref="O12:O13"/>
+    <mergeCell ref="U12:U13"/>
+    <mergeCell ref="K14:K15"/>
     <mergeCell ref="A26:E26"/>
+    <mergeCell ref="M14:M15"/>
+    <mergeCell ref="U14:U15"/>
+    <mergeCell ref="V16:V17"/>
+    <mergeCell ref="V12:V13"/>
+    <mergeCell ref="A2:W2"/>
+    <mergeCell ref="O14:O15"/>
     <mergeCell ref="A10:E10"/>
+    <mergeCell ref="K16:K17"/>
+    <mergeCell ref="L16:L17"/>
     <mergeCell ref="A31:E31"/>
-    <mergeCell ref="A2:W2"/>
+    <mergeCell ref="V14:V15"/>
   </mergeCells>
   <conditionalFormatting sqref="O5:O31">
     <cfRule type="cellIs" priority="10" operator="greaterThan" dxfId="9">
@@ -2943,162 +2967,162 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1" s="74">
-      <c r="A1" s="133" t="inlineStr">
+      <c r="A1" s="135" t="inlineStr">
         <is>
           <t>row_type</t>
         </is>
       </c>
-      <c r="B1" s="133" t="inlineStr">
+      <c r="B1" s="135" t="inlineStr">
         <is>
           <t>report_date</t>
         </is>
       </c>
-      <c r="C1" s="133" t="inlineStr">
+      <c r="C1" s="135" t="inlineStr">
         <is>
           <t>start_date</t>
         </is>
       </c>
-      <c r="D1" s="133" t="inlineStr">
+      <c r="D1" s="135" t="inlineStr">
         <is>
           <t>end_date</t>
         </is>
       </c>
-      <c r="E1" s="133" t="inlineStr">
+      <c r="E1" s="135" t="inlineStr">
         <is>
           <t>excel_row</t>
         </is>
       </c>
-      <c r="F1" s="133" t="inlineStr">
+      <c r="F1" s="135" t="inlineStr">
         <is>
           <t>funnel</t>
         </is>
       </c>
-      <c r="G1" s="133" t="inlineStr">
+      <c r="G1" s="135" t="inlineStr">
         <is>
           <t>platform</t>
         </is>
       </c>
-      <c r="H1" s="133" t="inlineStr">
+      <c r="H1" s="135" t="inlineStr">
         <is>
           <t>channel</t>
         </is>
       </c>
-      <c r="I1" s="133" t="inlineStr">
+      <c r="I1" s="135" t="inlineStr">
         <is>
           <t>campaign_name</t>
         </is>
       </c>
-      <c r="J1" s="133" t="inlineStr">
+      <c r="J1" s="135" t="inlineStr">
         <is>
           <t>investimento_media</t>
         </is>
       </c>
-      <c r="K1" s="133" t="inlineStr">
+      <c r="K1" s="135" t="inlineStr">
         <is>
           <t>percentuale_investimento</t>
         </is>
       </c>
-      <c r="L1" s="133" t="inlineStr">
+      <c r="L1" s="135" t="inlineStr">
         <is>
           <t>cpp_medio</t>
         </is>
       </c>
-      <c r="M1" s="133" t="inlineStr">
+      <c r="M1" s="135" t="inlineStr">
         <is>
           <t>stima_pratiche</t>
         </is>
       </c>
-      <c r="N1" s="133" t="inlineStr">
+      <c r="N1" s="135" t="inlineStr">
         <is>
           <t>cpl_target</t>
         </is>
       </c>
-      <c r="O1" s="133" t="inlineStr">
+      <c r="O1" s="135" t="inlineStr">
         <is>
           <t>stima_lead</t>
         </is>
       </c>
-      <c r="P1" s="133" t="inlineStr">
+      <c r="P1" s="135" t="inlineStr">
         <is>
           <t>stima_lead_giornaliere</t>
         </is>
       </c>
-      <c r="Q1" s="133" t="inlineStr">
+      <c r="Q1" s="135" t="inlineStr">
         <is>
           <t>stima_lead_progressiva</t>
         </is>
       </c>
-      <c r="R1" s="133" t="inlineStr">
+      <c r="R1" s="135" t="inlineStr">
         <is>
           <t>lead_effettive</t>
         </is>
       </c>
-      <c r="S1" s="133" t="inlineStr">
+      <c r="S1" s="135" t="inlineStr">
         <is>
           <t>delta_lead</t>
         </is>
       </c>
-      <c r="T1" s="133" t="inlineStr">
+      <c r="T1" s="135" t="inlineStr">
         <is>
           <t>stima_spending_giornaliera</t>
         </is>
       </c>
-      <c r="U1" s="133" t="inlineStr">
+      <c r="U1" s="135" t="inlineStr">
         <is>
           <t>stima_spending_progressiva</t>
         </is>
       </c>
-      <c r="V1" s="133" t="inlineStr">
+      <c r="V1" s="135" t="inlineStr">
         <is>
           <t>speso_effettivo</t>
         </is>
       </c>
-      <c r="W1" s="133" t="inlineStr">
+      <c r="W1" s="135" t="inlineStr">
         <is>
           <t>delta_speso</t>
         </is>
       </c>
-      <c r="X1" s="133" t="inlineStr">
+      <c r="X1" s="135" t="inlineStr">
         <is>
           <t>delta_delivery_pct</t>
         </is>
       </c>
-      <c r="Y1" s="133" t="inlineStr">
+      <c r="Y1" s="135" t="inlineStr">
         <is>
           <t>cpl_effettivo</t>
         </is>
       </c>
-      <c r="Z1" s="133" t="inlineStr">
+      <c r="Z1" s="135" t="inlineStr">
         <is>
           <t>delta_cpl</t>
         </is>
       </c>
-      <c r="AA1" s="133" t="inlineStr">
+      <c r="AA1" s="135" t="inlineStr">
         <is>
           <t>action</t>
         </is>
       </c>
-      <c r="AB1" s="133" t="inlineStr">
+      <c r="AB1" s="135" t="inlineStr">
         <is>
           <t>google_campaign_id</t>
         </is>
       </c>
-      <c r="AC1" s="133" t="inlineStr">
+      <c r="AC1" s="135" t="inlineStr">
         <is>
           <t>meta_campaign_id</t>
         </is>
       </c>
-      <c r="AD1" s="133" t="inlineStr">
+      <c r="AD1" s="135" t="inlineStr">
         <is>
           <t>dynamics_campaign_key</t>
         </is>
       </c>
-      <c r="AE1" s="133" t="inlineStr">
+      <c r="AE1" s="135" t="inlineStr">
         <is>
           <t>source_status</t>
         </is>
       </c>
-      <c r="AF1" s="133" t="inlineStr">
+      <c r="AF1" s="135" t="inlineStr">
         <is>
           <t>lead_allocation_method</t>
         </is>
@@ -3110,13 +3134,13 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B2" s="134" t="n">
+      <c r="B2" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C2" s="134" t="n">
+      <c r="C2" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D2" s="134" t="n">
+      <c r="D2" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E2" t="n">
@@ -3142,43 +3166,43 @@
           <t>CQ e CQP | Calcola Preventivo - Area Clienti</t>
         </is>
       </c>
-      <c r="J2" s="135" t="n">
+      <c r="J2" s="137" t="n">
         <v>9500</v>
       </c>
-      <c r="K2" s="136" t="n">
+      <c r="K2" s="138" t="n">
         <v>0.1507936507936507</v>
       </c>
-      <c r="L2" s="135" t="n"/>
-      <c r="N2" s="135" t="n"/>
-      <c r="T2" s="135" t="n">
+      <c r="L2" s="137" t="n"/>
+      <c r="N2" s="137" t="n"/>
+      <c r="T2" s="137" t="n">
         <v>306.4516129032258</v>
       </c>
-      <c r="U2" s="135" t="n">
+      <c r="U2" s="137" t="n">
         <v>5209.677419354838</v>
       </c>
-      <c r="V2" s="135" t="n">
+      <c r="V2" s="137" t="n">
         <v>5794.215866</v>
       </c>
-      <c r="W2" s="135" t="n">
+      <c r="W2" s="137" t="n">
         <v>584.5384466451615</v>
       </c>
-      <c r="X2" s="136" t="n">
+      <c r="X2" s="138" t="n">
         <v>0.1122024262910217</v>
       </c>
-      <c r="Y2" s="135" t="n"/>
-      <c r="Z2" s="135" t="n"/>
+      <c r="Y2" s="137" t="n"/>
+      <c r="Z2" s="137" t="n"/>
       <c r="AA2" t="inlineStr">
         <is>
           <t>SWITCH fatto</t>
         </is>
       </c>
-      <c r="AB2" s="137" t="inlineStr">
+      <c r="AB2" s="139" t="inlineStr">
         <is>
           <t>17559294673</t>
         </is>
       </c>
-      <c r="AC2" s="137" t="inlineStr"/>
-      <c r="AD2" s="137" t="inlineStr"/>
+      <c r="AC2" s="139" t="inlineStr"/>
+      <c r="AD2" s="139" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
           <t>google:ok;google:includes_excel_row_3</t>
@@ -3196,13 +3220,13 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B3" s="134" t="n">
+      <c r="B3" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C3" s="134" t="n">
+      <c r="C3" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D3" s="134" t="n">
+      <c r="D3" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E3" t="n">
@@ -3228,24 +3252,24 @@
           <t>DYN_AREACL CQ e CQP | Calcola Preventivo - QUINTO DIGITALE</t>
         </is>
       </c>
-      <c r="J3" s="135" t="n"/>
-      <c r="K3" s="136" t="n"/>
-      <c r="L3" s="135" t="n"/>
-      <c r="N3" s="135" t="n"/>
-      <c r="T3" s="135" t="n"/>
-      <c r="U3" s="135" t="n"/>
-      <c r="V3" s="135" t="n"/>
-      <c r="W3" s="135" t="n"/>
-      <c r="X3" s="136" t="n"/>
-      <c r="Y3" s="135" t="n"/>
-      <c r="Z3" s="135" t="n"/>
-      <c r="AB3" s="137" t="inlineStr">
+      <c r="J3" s="137" t="n"/>
+      <c r="K3" s="138" t="n"/>
+      <c r="L3" s="137" t="n"/>
+      <c r="N3" s="137" t="n"/>
+      <c r="T3" s="137" t="n"/>
+      <c r="U3" s="137" t="n"/>
+      <c r="V3" s="137" t="n"/>
+      <c r="W3" s="137" t="n"/>
+      <c r="X3" s="138" t="n"/>
+      <c r="Y3" s="137" t="n"/>
+      <c r="Z3" s="137" t="n"/>
+      <c r="AB3" s="139" t="inlineStr">
         <is>
           <t>23993507424</t>
         </is>
       </c>
-      <c r="AC3" s="137" t="inlineStr"/>
-      <c r="AD3" s="137" t="inlineStr"/>
+      <c r="AC3" s="139" t="inlineStr"/>
+      <c r="AD3" s="139" t="inlineStr"/>
       <c r="AE3" t="inlineStr">
         <is>
           <t>google:rolled_up_to_excel_row_2</t>
@@ -3263,13 +3287,13 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B4" s="134" t="n">
+      <c r="B4" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C4" s="134" t="n">
+      <c r="C4" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D4" s="134" t="n">
+      <c r="D4" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E4" t="n">
@@ -3295,43 +3319,43 @@
           <t>DYN_AREACL Delega di Pagamento - Area Clienti</t>
         </is>
       </c>
-      <c r="J4" s="135" t="n">
+      <c r="J4" s="137" t="n">
         <v>1500</v>
       </c>
-      <c r="K4" s="136" t="n">
+      <c r="K4" s="138" t="n">
         <v>0.0238095238095238</v>
       </c>
-      <c r="L4" s="135" t="n"/>
-      <c r="N4" s="135" t="n"/>
-      <c r="T4" s="135" t="n">
+      <c r="L4" s="137" t="n"/>
+      <c r="N4" s="137" t="n"/>
+      <c r="T4" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
-      <c r="U4" s="135" t="n">
+      <c r="U4" s="137" t="n">
         <v>822.5806451612904</v>
       </c>
-      <c r="V4" s="135" t="n">
+      <c r="V4" s="137" t="n">
         <v>1074.27638</v>
       </c>
-      <c r="W4" s="135" t="n">
+      <c r="W4" s="137" t="n">
         <v>251.6957348387096</v>
       </c>
-      <c r="X4" s="136" t="n">
+      <c r="X4" s="138" t="n">
         <v>0.3059830501960784</v>
       </c>
-      <c r="Y4" s="135" t="n"/>
-      <c r="Z4" s="135" t="n"/>
+      <c r="Y4" s="137" t="n"/>
+      <c r="Z4" s="137" t="n"/>
       <c r="AA4" t="inlineStr">
         <is>
           <t>SWITCH fatto</t>
         </is>
       </c>
-      <c r="AB4" s="137" t="inlineStr">
+      <c r="AB4" s="139" t="inlineStr">
         <is>
           <t>17559324373</t>
         </is>
       </c>
-      <c r="AC4" s="137" t="inlineStr"/>
-      <c r="AD4" s="137" t="inlineStr"/>
+      <c r="AC4" s="139" t="inlineStr"/>
+      <c r="AD4" s="139" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
           <t>google:ok;google:includes_excel_row_5</t>
@@ -3349,13 +3373,13 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B5" s="134" t="n">
+      <c r="B5" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C5" s="134" t="n">
+      <c r="C5" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D5" s="134" t="n">
+      <c r="D5" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E5" t="n">
@@ -3381,24 +3405,24 @@
           <t>DYN_AREACL Delega di Pagamento - QUINTO DIGITALE</t>
         </is>
       </c>
-      <c r="J5" s="135" t="n"/>
-      <c r="K5" s="136" t="n"/>
-      <c r="L5" s="135" t="n"/>
-      <c r="N5" s="135" t="n"/>
-      <c r="T5" s="135" t="n"/>
-      <c r="U5" s="135" t="n"/>
-      <c r="V5" s="135" t="n"/>
-      <c r="W5" s="135" t="n"/>
-      <c r="X5" s="136" t="n"/>
-      <c r="Y5" s="135" t="n"/>
-      <c r="Z5" s="135" t="n"/>
-      <c r="AB5" s="137" t="inlineStr">
+      <c r="J5" s="137" t="n"/>
+      <c r="K5" s="138" t="n"/>
+      <c r="L5" s="137" t="n"/>
+      <c r="N5" s="137" t="n"/>
+      <c r="T5" s="137" t="n"/>
+      <c r="U5" s="137" t="n"/>
+      <c r="V5" s="137" t="n"/>
+      <c r="W5" s="137" t="n"/>
+      <c r="X5" s="138" t="n"/>
+      <c r="Y5" s="137" t="n"/>
+      <c r="Z5" s="137" t="n"/>
+      <c r="AB5" s="139" t="inlineStr">
         <is>
           <t>23998450448</t>
         </is>
       </c>
-      <c r="AC5" s="137" t="inlineStr"/>
-      <c r="AD5" s="137" t="inlineStr"/>
+      <c r="AC5" s="139" t="inlineStr"/>
+      <c r="AD5" s="139" t="inlineStr"/>
       <c r="AE5" t="inlineStr">
         <is>
           <t>google:rolled_up_to_excel_row_4</t>
@@ -3416,13 +3440,13 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B6" s="134" t="n">
+      <c r="B6" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C6" s="134" t="n">
+      <c r="C6" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D6" s="134" t="n">
+      <c r="D6" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E6" t="n">
@@ -3448,43 +3472,43 @@
           <t>DYN_AREACL 2.0 - PURCHASE</t>
         </is>
       </c>
-      <c r="J6" s="135" t="n">
+      <c r="J6" s="137" t="n">
         <v>10000</v>
       </c>
-      <c r="K6" s="136" t="n">
+      <c r="K6" s="138" t="n">
         <v>0.1587301587301587</v>
       </c>
-      <c r="L6" s="135" t="n"/>
-      <c r="N6" s="135" t="n"/>
-      <c r="T6" s="135" t="n">
+      <c r="L6" s="137" t="n"/>
+      <c r="N6" s="137" t="n"/>
+      <c r="T6" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
-      <c r="U6" s="135" t="n">
+      <c r="U6" s="137" t="n">
         <v>5483.870967741936</v>
       </c>
-      <c r="V6" s="135" t="n">
+      <c r="V6" s="137" t="n">
         <v>5657.94</v>
       </c>
-      <c r="W6" s="135" t="n">
+      <c r="W6" s="137" t="n">
         <v>174.069032258064</v>
       </c>
-      <c r="X6" s="136" t="n">
+      <c r="X6" s="138" t="n">
         <v>0.0317419999999999</v>
       </c>
-      <c r="Y6" s="135" t="n"/>
-      <c r="Z6" s="135" t="n"/>
+      <c r="Y6" s="137" t="n"/>
+      <c r="Z6" s="137" t="n"/>
       <c r="AA6" t="inlineStr">
         <is>
           <t>abbassato leggermente lo spending giornaliero</t>
         </is>
       </c>
-      <c r="AB6" s="137" t="inlineStr"/>
-      <c r="AC6" s="137" t="inlineStr">
+      <c r="AB6" s="139" t="inlineStr"/>
+      <c r="AC6" s="139" t="inlineStr">
         <is>
           <t>6905931065575</t>
         </is>
       </c>
-      <c r="AD6" s="137" t="inlineStr"/>
+      <c r="AD6" s="139" t="inlineStr"/>
       <c r="AE6" t="inlineStr">
         <is>
           <t>meta:ok</t>
@@ -3502,17 +3526,17 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B7" s="134" t="n">
+      <c r="B7" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C7" s="134" t="n">
+      <c r="C7" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D7" s="134" t="n">
+      <c r="D7" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E7" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -3531,63 +3555,63 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>DEM DIGITOO</t>
-        </is>
-      </c>
-      <c r="J7" s="135" t="n">
-        <v>4000</v>
-      </c>
-      <c r="K7" s="136" t="n">
-        <v>0.06349206349206341</v>
-      </c>
-      <c r="L7" s="135" t="n">
-        <v>350</v>
+          <t>DEM DYNAMICS ADVICE ME</t>
+        </is>
+      </c>
+      <c r="J7" s="137" t="n">
+        <v>5000</v>
+      </c>
+      <c r="K7" s="138" t="n">
+        <v>0.07936507936507931</v>
+      </c>
+      <c r="L7" s="137" t="n">
+        <v>450</v>
       </c>
       <c r="M7" t="n">
-        <v>11.42857142857143</v>
-      </c>
-      <c r="N7" s="135" t="n">
-        <v>9</v>
+        <v>11.11111111111111</v>
+      </c>
+      <c r="N7" s="137" t="n">
+        <v>7.6</v>
       </c>
       <c r="O7" t="n">
-        <v>444.4444444444445</v>
+        <v>657.8947368421053</v>
       </c>
       <c r="P7" t="n">
-        <v>14.33691756272402</v>
+        <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>243.7275985663082</v>
+        <v>360.7809847198643</v>
       </c>
       <c r="R7" t="n">
-        <v>175</v>
+        <v>360</v>
       </c>
       <c r="S7" t="n">
-        <v>-68.72759856630825</v>
-      </c>
-      <c r="T7" s="135" t="n">
-        <v>173.9130434782609</v>
-      </c>
-      <c r="U7" s="135" t="n">
-        <v>2260.869565217391</v>
-      </c>
-      <c r="V7" s="135" t="n">
-        <v>1575</v>
-      </c>
-      <c r="W7" s="135" t="n">
-        <v>-685.8695652173915</v>
-      </c>
-      <c r="X7" s="136" t="n">
-        <v>-0.3033653846153846</v>
-      </c>
-      <c r="Y7" s="135" t="n">
-        <v>9</v>
-      </c>
-      <c r="Z7" s="135" t="n">
+        <v>-0.7809847198642501</v>
+      </c>
+      <c r="T7" s="137" t="n">
+        <v>217.3913043478261</v>
+      </c>
+      <c r="U7" s="137" t="n">
+        <v>2826.086956521739</v>
+      </c>
+      <c r="V7" s="137" t="n">
+        <v>2736</v>
+      </c>
+      <c r="W7" s="137" t="n">
+        <v>-90.086956521739</v>
+      </c>
+      <c r="X7" s="138" t="n">
+        <v>-0.031876923076923</v>
+      </c>
+      <c r="Y7" s="137" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="Z7" s="137" t="n">
         <v>0</v>
       </c>
-      <c r="AB7" s="137" t="inlineStr"/>
-      <c r="AC7" s="137" t="inlineStr"/>
-      <c r="AD7" s="137" t="inlineStr"/>
+      <c r="AB7" s="139" t="inlineStr"/>
+      <c r="AC7" s="139" t="inlineStr"/>
+      <c r="AD7" s="139" t="inlineStr"/>
       <c r="AE7" t="inlineStr">
         <is>
           <t>manual:no_ads_source</t>
@@ -3605,17 +3629,17 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B8" s="134" t="n">
+      <c r="B8" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C8" s="134" t="n">
+      <c r="C8" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D8" s="134" t="n">
+      <c r="D8" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E8" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -3634,63 +3658,63 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>DEM DYNAMICS ADVICE ME</t>
-        </is>
-      </c>
-      <c r="J8" s="135" t="n">
-        <v>5000</v>
-      </c>
-      <c r="K8" s="136" t="n">
-        <v>0.07936507936507931</v>
-      </c>
-      <c r="L8" s="135" t="n">
-        <v>450</v>
+          <t>DEM DIGITOO</t>
+        </is>
+      </c>
+      <c r="J8" s="137" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K8" s="138" t="n">
+        <v>0.06349206349206341</v>
+      </c>
+      <c r="L8" s="137" t="n">
+        <v>350</v>
       </c>
       <c r="M8" t="n">
-        <v>11.11111111111111</v>
-      </c>
-      <c r="N8" s="135" t="n">
-        <v>7.6</v>
+        <v>11.42857142857143</v>
+      </c>
+      <c r="N8" s="137" t="n">
+        <v>9</v>
       </c>
       <c r="O8" t="n">
-        <v>657.8947368421053</v>
+        <v>444.4444444444445</v>
       </c>
       <c r="P8" t="n">
-        <v>21.22241086587437</v>
+        <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>360.7809847198643</v>
+        <v>243.7275985663082</v>
       </c>
       <c r="R8" t="n">
-        <v>360</v>
+        <v>175</v>
       </c>
       <c r="S8" t="n">
-        <v>-0.7809847198642501</v>
-      </c>
-      <c r="T8" s="135" t="n">
-        <v>217.3913043478261</v>
-      </c>
-      <c r="U8" s="135" t="n">
-        <v>2826.086956521739</v>
-      </c>
-      <c r="V8" s="135" t="n">
-        <v>2736</v>
-      </c>
-      <c r="W8" s="135" t="n">
-        <v>-90.086956521739</v>
-      </c>
-      <c r="X8" s="136" t="n">
-        <v>-0.031876923076923</v>
-      </c>
-      <c r="Y8" s="135" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="Z8" s="135" t="n">
+        <v>-68.72759856630825</v>
+      </c>
+      <c r="T8" s="137" t="n">
+        <v>173.9130434782609</v>
+      </c>
+      <c r="U8" s="137" t="n">
+        <v>2260.869565217391</v>
+      </c>
+      <c r="V8" s="137" t="n">
+        <v>1575</v>
+      </c>
+      <c r="W8" s="137" t="n">
+        <v>-685.8695652173915</v>
+      </c>
+      <c r="X8" s="138" t="n">
+        <v>-0.3033653846153846</v>
+      </c>
+      <c r="Y8" s="137" t="n">
+        <v>9</v>
+      </c>
+      <c r="Z8" s="137" t="n">
         <v>0</v>
       </c>
-      <c r="AB8" s="137" t="inlineStr"/>
-      <c r="AC8" s="137" t="inlineStr"/>
-      <c r="AD8" s="137" t="inlineStr"/>
+      <c r="AB8" s="139" t="inlineStr"/>
+      <c r="AC8" s="139" t="inlineStr"/>
+      <c r="AD8" s="139" t="inlineStr"/>
       <c r="AE8" t="inlineStr">
         <is>
           <t>manual:no_ads_source</t>
@@ -3708,13 +3732,13 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B9" s="134" t="n">
+      <c r="B9" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C9" s="134" t="n">
+      <c r="C9" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D9" s="134" t="n">
+      <c r="D9" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E9" t="n">
@@ -3740,19 +3764,19 @@
           <t>DEM TIG</t>
         </is>
       </c>
-      <c r="J9" s="135" t="n">
+      <c r="J9" s="137" t="n">
         <v>2000</v>
       </c>
-      <c r="K9" s="136" t="n">
+      <c r="K9" s="138" t="n">
         <v>0.0317460317460317</v>
       </c>
-      <c r="L9" s="135" t="n">
+      <c r="L9" s="137" t="n">
         <v>300</v>
       </c>
       <c r="M9" t="n">
         <v>6.666666666666667</v>
       </c>
-      <c r="N9" s="135" t="n">
+      <c r="N9" s="137" t="n">
         <v>8</v>
       </c>
       <c r="O9" t="n">
@@ -3770,30 +3794,30 @@
       <c r="S9" t="n">
         <v>85.90322580645162</v>
       </c>
-      <c r="T9" s="135" t="n">
+      <c r="T9" s="137" t="n">
         <v>86.95652173913044</v>
       </c>
-      <c r="U9" s="135" t="n">
+      <c r="U9" s="137" t="n">
         <v>1130.434782608696</v>
       </c>
-      <c r="V9" s="135" t="n">
+      <c r="V9" s="137" t="n">
         <v>1784</v>
       </c>
-      <c r="W9" s="135" t="n">
+      <c r="W9" s="137" t="n">
         <v>653.5652173913043</v>
       </c>
-      <c r="X9" s="136" t="n">
+      <c r="X9" s="138" t="n">
         <v>0.578153846153846</v>
       </c>
-      <c r="Y9" s="135" t="n">
+      <c r="Y9" s="137" t="n">
         <v>8</v>
       </c>
-      <c r="Z9" s="135" t="n">
+      <c r="Z9" s="137" t="n">
         <v>0</v>
       </c>
-      <c r="AB9" s="137" t="inlineStr"/>
-      <c r="AC9" s="137" t="inlineStr"/>
-      <c r="AD9" s="137" t="inlineStr"/>
+      <c r="AB9" s="139" t="inlineStr"/>
+      <c r="AC9" s="139" t="inlineStr"/>
+      <c r="AD9" s="139" t="inlineStr"/>
       <c r="AE9" t="inlineStr">
         <is>
           <t>manual:no_ads_source</t>
@@ -3811,17 +3835,17 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B10" s="134" t="n">
+      <c r="B10" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C10" s="134" t="n">
+      <c r="C10" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D10" s="134" t="n">
+      <c r="D10" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -3840,75 +3864,75 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>DYN_VELOCE Cessione del Quinto [Esatta]</t>
-        </is>
-      </c>
-      <c r="J10" s="135" t="n">
-        <v>9000</v>
-      </c>
-      <c r="K10" s="136" t="n">
-        <v>0.1428571428571428</v>
-      </c>
-      <c r="L10" s="135" t="n">
-        <v>600</v>
+          <t>DYN_VELOCE Cessione del Quinto QUINTO DIGITALE</t>
+        </is>
+      </c>
+      <c r="J10" s="137" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K10" s="138" t="n">
+        <v>0.06349206349206341</v>
+      </c>
+      <c r="L10" s="137" t="n">
+        <v>700</v>
       </c>
       <c r="M10" t="n">
-        <v>15</v>
-      </c>
-      <c r="N10" s="135" t="n">
-        <v>38.5</v>
+        <v>5.714285714285714</v>
+      </c>
+      <c r="N10" s="137" t="n">
+        <v>34</v>
       </c>
       <c r="O10" t="n">
-        <v>233.7662337662338</v>
+        <v>117.6470588235294</v>
       </c>
       <c r="P10" t="n">
-        <v>7.540846250523669</v>
+        <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>128.1943862589024</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="R10" t="n">
-        <v>61</v>
+        <v>98</v>
       </c>
       <c r="S10" t="n">
-        <v>-67.19438625890237</v>
-      </c>
-      <c r="T10" s="135" t="n">
-        <v>290.3225806451613</v>
-      </c>
-      <c r="U10" s="135" t="n">
-        <v>4935.483870967741</v>
-      </c>
-      <c r="V10" s="135" t="n">
-        <v>5490.756616000001</v>
-      </c>
-      <c r="W10" s="135" t="n">
-        <v>555.2727450322591</v>
-      </c>
-      <c r="X10" s="136" t="n">
-        <v>0.1125062424575165</v>
-      </c>
-      <c r="Y10" s="135" t="n">
-        <v>90.01240354098361</v>
-      </c>
-      <c r="Z10" s="135" t="n">
-        <v>51.51240354098361</v>
+        <v>33.48387096774194</v>
+      </c>
+      <c r="T10" s="137" t="n">
+        <v>129.0322580645161</v>
+      </c>
+      <c r="U10" s="137" t="n">
+        <v>2193.548387096774</v>
+      </c>
+      <c r="V10" s="137" t="n">
+        <v>3069.617174</v>
+      </c>
+      <c r="W10" s="137" t="n">
+        <v>876.0687869032258</v>
+      </c>
+      <c r="X10" s="138" t="n">
+        <v>0.3993842999117647</v>
+      </c>
+      <c r="Y10" s="137" t="n">
+        <v>31.3226242244898</v>
+      </c>
+      <c r="Z10" s="137" t="n">
+        <v>-2.677375775510203</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>SWITCH fatto</t>
-        </is>
-      </c>
-      <c r="AB10" s="137" t="inlineStr">
-        <is>
-          <t>22822606735</t>
-        </is>
-      </c>
-      <c r="AC10" s="137" t="inlineStr"/>
-      <c r="AD10" s="137" t="inlineStr"/>
+          <t>diminuito cpa target - alzato a giugno per dare più dati alla campagna che è stata rilanciata da zero</t>
+        </is>
+      </c>
+      <c r="AB10" s="139" t="inlineStr">
+        <is>
+          <t>23968989759</t>
+        </is>
+      </c>
+      <c r="AC10" s="139" t="inlineStr"/>
+      <c r="AD10" s="139" t="inlineStr"/>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_10</t>
+          <t>google:ok</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -3923,17 +3947,17 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B11" s="134" t="n">
+      <c r="B11" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C11" s="134" t="n">
+      <c r="C11" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D11" s="134" t="n">
+      <c r="D11" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -3952,33 +3976,75 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>DYN_VELOCE Cessione del Quinto [Esatta] QUINTO DIGITALE</t>
-        </is>
-      </c>
-      <c r="J11" s="135" t="n"/>
-      <c r="K11" s="136" t="n"/>
-      <c r="L11" s="135" t="n"/>
-      <c r="N11" s="135" t="n"/>
+          <t>DYN_VELOCE Cessione del Quinto [Esatta]</t>
+        </is>
+      </c>
+      <c r="J11" s="137" t="n">
+        <v>9000</v>
+      </c>
+      <c r="K11" s="138" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="L11" s="137" t="n">
+        <v>600</v>
+      </c>
+      <c r="M11" t="n">
+        <v>15</v>
+      </c>
+      <c r="N11" s="137" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="O11" t="n">
+        <v>233.7662337662338</v>
+      </c>
+      <c r="P11" t="n">
+        <v>7.540846250523669</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>128.1943862589024</v>
+      </c>
       <c r="R11" t="n">
-        <v>92</v>
-      </c>
-      <c r="T11" s="135" t="n"/>
-      <c r="U11" s="135" t="n"/>
-      <c r="V11" s="135" t="n"/>
-      <c r="W11" s="135" t="n"/>
-      <c r="X11" s="136" t="n"/>
-      <c r="Y11" s="135" t="n"/>
-      <c r="Z11" s="135" t="n"/>
-      <c r="AB11" s="137" t="inlineStr">
-        <is>
-          <t>23990314506</t>
-        </is>
-      </c>
-      <c r="AC11" s="137" t="inlineStr"/>
-      <c r="AD11" s="137" t="inlineStr"/>
+        <v>61</v>
+      </c>
+      <c r="S11" t="n">
+        <v>24.80561374109763</v>
+      </c>
+      <c r="T11" s="137" t="n">
+        <v>290.3225806451613</v>
+      </c>
+      <c r="U11" s="137" t="n">
+        <v>4935.483870967741</v>
+      </c>
+      <c r="V11" s="137" t="n">
+        <v>5490.756616000001</v>
+      </c>
+      <c r="W11" s="137" t="n">
+        <v>555.2727450322591</v>
+      </c>
+      <c r="X11" s="138" t="n">
+        <v>0.1125062424575165</v>
+      </c>
+      <c r="Y11" s="137" t="n">
+        <v>35.88729814379085</v>
+      </c>
+      <c r="Z11" s="137" t="n">
+        <v>-2.612701856209149</v>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>SWITCH fatto</t>
+        </is>
+      </c>
+      <c r="AB11" s="139" t="inlineStr">
+        <is>
+          <t>22822606735</t>
+        </is>
+      </c>
+      <c r="AC11" s="139" t="inlineStr"/>
+      <c r="AD11" s="139" t="inlineStr"/>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_9</t>
+          <t>google:ok;google:includes_excel_row_10;crm_metrics_combined_with_excel_row_10</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -3993,17 +4059,17 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B12" s="134" t="n">
+      <c r="B12" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C12" s="134" t="n">
+      <c r="C12" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D12" s="134" t="n">
+      <c r="D12" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E12" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -4022,75 +4088,33 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>DYN_VELOCE Cessione del Quinto QUINTO DIGITALE</t>
-        </is>
-      </c>
-      <c r="J12" s="135" t="n">
-        <v>4000</v>
-      </c>
-      <c r="K12" s="136" t="n">
-        <v>0.06349206349206341</v>
-      </c>
-      <c r="L12" s="135" t="n">
-        <v>700</v>
-      </c>
-      <c r="M12" t="n">
-        <v>5.714285714285714</v>
-      </c>
-      <c r="N12" s="135" t="n">
-        <v>34</v>
-      </c>
-      <c r="O12" t="n">
-        <v>117.6470588235294</v>
-      </c>
-      <c r="P12" t="n">
-        <v>3.795066413662239</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>64.51612903225806</v>
-      </c>
+          <t>DYN_VELOCE Cessione del Quinto [Esatta] QUINTO DIGITALE</t>
+        </is>
+      </c>
+      <c r="J12" s="137" t="n"/>
+      <c r="K12" s="138" t="n"/>
+      <c r="L12" s="137" t="n"/>
+      <c r="N12" s="137" t="n"/>
       <c r="R12" t="n">
-        <v>98</v>
-      </c>
-      <c r="S12" t="n">
-        <v>33.48387096774194</v>
-      </c>
-      <c r="T12" s="135" t="n">
-        <v>129.0322580645161</v>
-      </c>
-      <c r="U12" s="135" t="n">
-        <v>2193.548387096774</v>
-      </c>
-      <c r="V12" s="135" t="n">
-        <v>3069.617174</v>
-      </c>
-      <c r="W12" s="135" t="n">
-        <v>876.0687869032258</v>
-      </c>
-      <c r="X12" s="136" t="n">
-        <v>0.3993842999117647</v>
-      </c>
-      <c r="Y12" s="135" t="n">
-        <v>31.3226242244898</v>
-      </c>
-      <c r="Z12" s="135" t="n">
-        <v>-2.677375775510203</v>
-      </c>
-      <c r="AA12" t="inlineStr">
-        <is>
-          <t>diminuito cpa target - alzato a giugno per dare più dati alla campagna che è stata rilanciata da zero</t>
-        </is>
-      </c>
-      <c r="AB12" s="137" t="inlineStr">
-        <is>
-          <t>23968989759</t>
-        </is>
-      </c>
-      <c r="AC12" s="137" t="inlineStr"/>
-      <c r="AD12" s="137" t="inlineStr"/>
+        <v>92</v>
+      </c>
+      <c r="T12" s="137" t="n"/>
+      <c r="U12" s="137" t="n"/>
+      <c r="V12" s="137" t="n"/>
+      <c r="W12" s="137" t="n"/>
+      <c r="X12" s="138" t="n"/>
+      <c r="Y12" s="137" t="n"/>
+      <c r="Z12" s="137" t="n"/>
+      <c r="AB12" s="139" t="inlineStr">
+        <is>
+          <t>23990314506</t>
+        </is>
+      </c>
+      <c r="AC12" s="139" t="inlineStr"/>
+      <c r="AD12" s="139" t="inlineStr"/>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:rolled_up_to_excel_row_9</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -4105,13 +4129,13 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B13" s="134" t="n">
+      <c r="B13" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C13" s="134" t="n">
+      <c r="C13" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D13" s="134" t="n">
+      <c r="D13" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E13" t="n">
@@ -4137,19 +4161,19 @@
           <t>DYN_VELOCE CQ Pensionati [Esatta]</t>
         </is>
       </c>
-      <c r="J13" s="135" t="n">
+      <c r="J13" s="137" t="n">
         <v>1000</v>
       </c>
-      <c r="K13" s="136" t="n">
+      <c r="K13" s="138" t="n">
         <v>0.0158730158730158</v>
       </c>
-      <c r="L13" s="135" t="n">
+      <c r="L13" s="137" t="n">
         <v>800</v>
       </c>
       <c r="M13" t="n">
         <v>1.25</v>
       </c>
-      <c r="N13" s="135" t="n">
+      <c r="N13" s="137" t="n">
         <v>38</v>
       </c>
       <c r="O13" t="n">
@@ -4165,44 +4189,44 @@
         <v>5</v>
       </c>
       <c r="S13" t="n">
-        <v>-9.431239388794566</v>
-      </c>
-      <c r="T13" s="135" t="n">
+        <v>-5.431239388794566</v>
+      </c>
+      <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
-      <c r="U13" s="135" t="n">
+      <c r="U13" s="137" t="n">
         <v>548.3870967741935</v>
       </c>
-      <c r="V13" s="135" t="n">
+      <c r="V13" s="137" t="n">
         <v>510.988722</v>
       </c>
-      <c r="W13" s="135" t="n">
+      <c r="W13" s="137" t="n">
         <v>-37.39837477419354</v>
       </c>
-      <c r="X13" s="136" t="n">
+      <c r="X13" s="138" t="n">
         <v>-0.0681970363529411</v>
       </c>
-      <c r="Y13" s="135" t="n">
-        <v>102.1977444</v>
-      </c>
-      <c r="Z13" s="135" t="n">
-        <v>64.1977444</v>
+      <c r="Y13" s="137" t="n">
+        <v>56.77652466666667</v>
+      </c>
+      <c r="Z13" s="137" t="n">
+        <v>18.77652466666667</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
           <t>ATTIVATA nuova campagna - quando esce da apprendimento abbassare cpa target</t>
         </is>
       </c>
-      <c r="AB13" s="137" t="inlineStr">
+      <c r="AB13" s="139" t="inlineStr">
         <is>
           <t>23061435070</t>
         </is>
       </c>
-      <c r="AC13" s="137" t="inlineStr"/>
-      <c r="AD13" s="137" t="inlineStr"/>
+      <c r="AC13" s="139" t="inlineStr"/>
+      <c r="AD13" s="139" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_12</t>
+          <t>google:ok;google:includes_excel_row_12;crm_metrics_combined_with_excel_row_12</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -4217,17 +4241,17 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B14" s="134" t="n">
+      <c r="B14" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C14" s="134" t="n">
+      <c r="C14" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D14" s="134" t="n">
+      <c r="D14" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -4246,75 +4270,33 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>DYN_VELOCE CQ Pensionati ESTERO - Paesi Prioritari</t>
-        </is>
-      </c>
-      <c r="J14" s="135" t="n">
-        <v>1000</v>
-      </c>
-      <c r="K14" s="136" t="n">
-        <v>0.0158730158730158</v>
-      </c>
-      <c r="L14" s="135" t="n">
-        <v>1000</v>
-      </c>
-      <c r="M14" t="n">
-        <v>1</v>
-      </c>
-      <c r="N14" s="135" t="n">
-        <v>250</v>
-      </c>
-      <c r="O14" t="n">
+          <t>DYN_VELOCE CQ Pensionati QUINTO DIGITALE</t>
+        </is>
+      </c>
+      <c r="J14" s="137" t="n"/>
+      <c r="K14" s="138" t="n"/>
+      <c r="L14" s="137" t="n"/>
+      <c r="N14" s="137" t="n"/>
+      <c r="R14" t="n">
         <v>4</v>
       </c>
-      <c r="P14" t="n">
-        <v>0.1290322580645161</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>2.193548387096774</v>
-      </c>
-      <c r="R14" t="n">
-        <v>2</v>
-      </c>
-      <c r="S14" t="n">
-        <v>-0.193548387096774</v>
-      </c>
-      <c r="T14" s="135" t="n">
-        <v>32.25806451612903</v>
-      </c>
-      <c r="U14" s="135" t="n">
-        <v>548.3870967741935</v>
-      </c>
-      <c r="V14" s="135" t="n">
-        <v>630.160373</v>
-      </c>
-      <c r="W14" s="135" t="n">
-        <v>81.77327622580651</v>
-      </c>
-      <c r="X14" s="136" t="n">
-        <v>0.1491159742941177</v>
-      </c>
-      <c r="Y14" s="135" t="n">
-        <v>315.0801865</v>
-      </c>
-      <c r="Z14" s="135" t="n">
-        <v>65.08018650000002</v>
-      </c>
-      <c r="AA14" t="inlineStr">
-        <is>
-          <t>ATTIVATA nuova campagna - quando esce da apprendimento abbassare cpa target</t>
-        </is>
-      </c>
-      <c r="AB14" s="137" t="inlineStr">
-        <is>
-          <t>23267957688</t>
-        </is>
-      </c>
-      <c r="AC14" s="137" t="inlineStr"/>
-      <c r="AD14" s="137" t="inlineStr"/>
+      <c r="T14" s="137" t="n"/>
+      <c r="U14" s="137" t="n"/>
+      <c r="V14" s="137" t="n"/>
+      <c r="W14" s="137" t="n"/>
+      <c r="X14" s="138" t="n"/>
+      <c r="Y14" s="137" t="n"/>
+      <c r="Z14" s="137" t="n"/>
+      <c r="AB14" s="139" t="inlineStr">
+        <is>
+          <t>23993375943</t>
+        </is>
+      </c>
+      <c r="AC14" s="139" t="inlineStr"/>
+      <c r="AD14" s="139" t="inlineStr"/>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_14</t>
+          <t>google:rolled_up_to_excel_row_11</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -4329,17 +4311,17 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B15" s="134" t="n">
+      <c r="B15" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C15" s="134" t="n">
+      <c r="C15" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D15" s="134" t="n">
+      <c r="D15" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -4358,33 +4340,75 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>DYN_VELOCE CQ Pensionati ESTERO - Paesi Prioritari QUINTO DIGITALE</t>
-        </is>
-      </c>
-      <c r="J15" s="135" t="n"/>
-      <c r="K15" s="136" t="n"/>
-      <c r="L15" s="135" t="n"/>
-      <c r="N15" s="135" t="n"/>
+          <t>DYN_VELOCE CQ Pensionati ESTERO - Paesi Prioritari</t>
+        </is>
+      </c>
+      <c r="J15" s="137" t="n">
+        <v>1000</v>
+      </c>
+      <c r="K15" s="138" t="n">
+        <v>0.0158730158730158</v>
+      </c>
+      <c r="L15" s="137" t="n">
+        <v>1000</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" s="137" t="n">
+        <v>250</v>
+      </c>
+      <c r="O15" t="n">
+        <v>4</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0.1290322580645161</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>2.193548387096774</v>
+      </c>
       <c r="R15" t="n">
-        <v>0</v>
-      </c>
-      <c r="T15" s="135" t="n"/>
-      <c r="U15" s="135" t="n"/>
-      <c r="V15" s="135" t="n"/>
-      <c r="W15" s="135" t="n"/>
-      <c r="X15" s="136" t="n"/>
-      <c r="Y15" s="135" t="n"/>
-      <c r="Z15" s="135" t="n"/>
-      <c r="AB15" s="137" t="inlineStr">
-        <is>
-          <t>23993437149</t>
-        </is>
-      </c>
-      <c r="AC15" s="137" t="inlineStr"/>
-      <c r="AD15" s="137" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="S15" t="n">
+        <v>-0.193548387096774</v>
+      </c>
+      <c r="T15" s="137" t="n">
+        <v>32.25806451612903</v>
+      </c>
+      <c r="U15" s="137" t="n">
+        <v>548.3870967741935</v>
+      </c>
+      <c r="V15" s="137" t="n">
+        <v>630.160373</v>
+      </c>
+      <c r="W15" s="137" t="n">
+        <v>81.77327622580651</v>
+      </c>
+      <c r="X15" s="138" t="n">
+        <v>0.1491159742941177</v>
+      </c>
+      <c r="Y15" s="137" t="n">
+        <v>315.0801865</v>
+      </c>
+      <c r="Z15" s="137" t="n">
+        <v>65.08018650000002</v>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>ATTIVATA nuova campagna - quando esce da apprendimento abbassare cpa target</t>
+        </is>
+      </c>
+      <c r="AB15" s="139" t="inlineStr">
+        <is>
+          <t>23267957688</t>
+        </is>
+      </c>
+      <c r="AC15" s="139" t="inlineStr"/>
+      <c r="AD15" s="139" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_13</t>
+          <t>google:ok;google:includes_excel_row_14;crm_metrics_combined_with_excel_row_14</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -4399,17 +4423,17 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B16" s="134" t="n">
+      <c r="B16" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C16" s="134" t="n">
+      <c r="C16" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D16" s="134" t="n">
+      <c r="D16" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E16" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -4428,33 +4452,33 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>DYN_VELOCE CQ Pensionati QUINTO DIGITALE</t>
-        </is>
-      </c>
-      <c r="J16" s="135" t="n"/>
-      <c r="K16" s="136" t="n"/>
-      <c r="L16" s="135" t="n"/>
-      <c r="N16" s="135" t="n"/>
+          <t>DYN_VELOCE CQ Pensionati ESTERO - Paesi Prioritari QUINTO DIGITALE</t>
+        </is>
+      </c>
+      <c r="J16" s="137" t="n"/>
+      <c r="K16" s="138" t="n"/>
+      <c r="L16" s="137" t="n"/>
+      <c r="N16" s="137" t="n"/>
       <c r="R16" t="n">
-        <v>4</v>
-      </c>
-      <c r="T16" s="135" t="n"/>
-      <c r="U16" s="135" t="n"/>
-      <c r="V16" s="135" t="n"/>
-      <c r="W16" s="135" t="n"/>
-      <c r="X16" s="136" t="n"/>
-      <c r="Y16" s="135" t="n"/>
-      <c r="Z16" s="135" t="n"/>
-      <c r="AB16" s="137" t="inlineStr">
-        <is>
-          <t>23993375943</t>
-        </is>
-      </c>
-      <c r="AC16" s="137" t="inlineStr"/>
-      <c r="AD16" s="137" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="T16" s="137" t="n"/>
+      <c r="U16" s="137" t="n"/>
+      <c r="V16" s="137" t="n"/>
+      <c r="W16" s="137" t="n"/>
+      <c r="X16" s="138" t="n"/>
+      <c r="Y16" s="137" t="n"/>
+      <c r="Z16" s="137" t="n"/>
+      <c r="AB16" s="139" t="inlineStr">
+        <is>
+          <t>23993437149</t>
+        </is>
+      </c>
+      <c r="AC16" s="139" t="inlineStr"/>
+      <c r="AD16" s="139" t="inlineStr"/>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_11</t>
+          <t>google:rolled_up_to_excel_row_13</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -4469,17 +4493,17 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B17" s="134" t="n">
+      <c r="B17" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C17" s="134" t="n">
+      <c r="C17" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D17" s="134" t="n">
+      <c r="D17" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E17" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4498,67 +4522,72 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>[BMK 2025] LeadGen CQD PEN [Albania]</t>
-        </is>
-      </c>
-      <c r="J17" s="135" t="n">
+          <t>DYN_VELOCE New Creative Apr26</t>
+        </is>
+      </c>
+      <c r="J17" s="137" t="n">
+        <v>10000</v>
+      </c>
+      <c r="K17" s="138" t="n">
+        <v>0.1587301587301587</v>
+      </c>
+      <c r="L17" s="137" t="n">
         <v>500</v>
       </c>
-      <c r="K17" s="136" t="n">
-        <v>0.0079365079365079</v>
-      </c>
-      <c r="L17" s="135" t="n">
-        <v>540</v>
-      </c>
       <c r="M17" t="n">
-        <v>0.925925925925926</v>
-      </c>
-      <c r="N17" s="135" t="n">
-        <v>120</v>
+        <v>20</v>
+      </c>
+      <c r="N17" s="137" t="n">
+        <v>12.8</v>
       </c>
       <c r="O17" t="n">
-        <v>4.166666666666667</v>
+        <v>781.25</v>
       </c>
       <c r="P17" t="n">
-        <v>0.1344086021505376</v>
+        <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>2.28494623655914</v>
+        <v>428.4274193548387</v>
       </c>
       <c r="R17" t="n">
-        <v>4</v>
+        <v>367</v>
       </c>
       <c r="S17" t="n">
-        <v>1.71505376344086</v>
-      </c>
-      <c r="T17" s="135" t="n">
-        <v>16.12903225806452</v>
-      </c>
-      <c r="U17" s="135" t="n">
-        <v>274.1935483870968</v>
-      </c>
-      <c r="V17" s="135" t="n">
-        <v>283.27</v>
-      </c>
-      <c r="W17" s="135" t="n">
-        <v>9.076451612903211</v>
-      </c>
-      <c r="X17" s="136" t="n">
-        <v>0.0331023529411764</v>
-      </c>
-      <c r="Y17" s="135" t="n">
-        <v>70.8175</v>
-      </c>
-      <c r="Z17" s="135" t="n">
-        <v>-49.1825</v>
-      </c>
-      <c r="AB17" s="137" t="inlineStr"/>
-      <c r="AC17" s="137" t="inlineStr">
-        <is>
-          <t>6666147663775</t>
-        </is>
-      </c>
-      <c r="AD17" s="137" t="inlineStr"/>
+        <v>-61.42741935483872</v>
+      </c>
+      <c r="T17" s="137" t="n">
+        <v>322.5806451612903</v>
+      </c>
+      <c r="U17" s="137" t="n">
+        <v>5483.870967741936</v>
+      </c>
+      <c r="V17" s="137" t="n">
+        <v>7444.1</v>
+      </c>
+      <c r="W17" s="137" t="n">
+        <v>1960.229032258065</v>
+      </c>
+      <c r="X17" s="138" t="n">
+        <v>0.3574535294117647</v>
+      </c>
+      <c r="Y17" s="137" t="n">
+        <v>20.28365122615804</v>
+      </c>
+      <c r="Z17" s="137" t="n">
+        <v>7.483651226158038</v>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>diminuito cpa target che era stato alzato per aiutare la campagna ad uscire dalla fase di apprendimento</t>
+        </is>
+      </c>
+      <c r="AB17" s="139" t="inlineStr"/>
+      <c r="AC17" s="139" t="inlineStr">
+        <is>
+          <t>6944411197975</t>
+        </is>
+      </c>
+      <c r="AD17" s="139" t="inlineStr"/>
       <c r="AE17" t="inlineStr">
         <is>
           <t>meta:ok</t>
@@ -4576,13 +4605,13 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B18" s="134" t="n">
+      <c r="B18" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C18" s="134" t="n">
+      <c r="C18" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D18" s="134" t="n">
+      <c r="D18" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E18" t="n">
@@ -4608,19 +4637,19 @@
           <t>[BMK 2025] LeadGen CQD PEN [Romania]</t>
         </is>
       </c>
-      <c r="J18" s="135" t="n">
+      <c r="J18" s="137" t="n">
         <v>500</v>
       </c>
-      <c r="K18" s="136" t="n">
+      <c r="K18" s="138" t="n">
         <v>0.0079365079365079</v>
       </c>
-      <c r="L18" s="135" t="n">
+      <c r="L18" s="137" t="n">
         <v>540</v>
       </c>
       <c r="M18" t="n">
         <v>0.925925925925926</v>
       </c>
-      <c r="N18" s="135" t="n">
+      <c r="N18" s="137" t="n">
         <v>40</v>
       </c>
       <c r="O18" t="n">
@@ -4638,34 +4667,34 @@
       <c r="S18" t="n">
         <v>24.14516129032258</v>
       </c>
-      <c r="T18" s="135" t="n">
+      <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
-      <c r="U18" s="135" t="n">
+      <c r="U18" s="137" t="n">
         <v>274.1935483870968</v>
       </c>
-      <c r="V18" s="135" t="n">
+      <c r="V18" s="137" t="n">
         <v>322.95</v>
       </c>
-      <c r="W18" s="135" t="n">
+      <c r="W18" s="137" t="n">
         <v>48.75645161290322</v>
       </c>
-      <c r="X18" s="136" t="n">
+      <c r="X18" s="138" t="n">
         <v>0.1778176470588235</v>
       </c>
-      <c r="Y18" s="135" t="n">
+      <c r="Y18" s="137" t="n">
         <v>10.41774193548387</v>
       </c>
-      <c r="Z18" s="135" t="n">
+      <c r="Z18" s="137" t="n">
         <v>-29.58225806451613</v>
       </c>
-      <c r="AB18" s="137" t="inlineStr"/>
-      <c r="AC18" s="137" t="inlineStr">
+      <c r="AB18" s="139" t="inlineStr"/>
+      <c r="AC18" s="139" t="inlineStr">
         <is>
           <t>6970690462575</t>
         </is>
       </c>
-      <c r="AD18" s="137" t="inlineStr"/>
+      <c r="AD18" s="139" t="inlineStr"/>
       <c r="AE18" t="inlineStr">
         <is>
           <t>meta:ok</t>
@@ -4683,13 +4712,13 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B19" s="134" t="n">
+      <c r="B19" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C19" s="134" t="n">
+      <c r="C19" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D19" s="134" t="n">
+      <c r="D19" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E19" t="n">
@@ -4715,19 +4744,19 @@
           <t>[BMK 2025] LeadGen CQD PEN [Tunisia]</t>
         </is>
       </c>
-      <c r="J19" s="135" t="n">
+      <c r="J19" s="137" t="n">
         <v>1000</v>
       </c>
-      <c r="K19" s="136" t="n">
+      <c r="K19" s="138" t="n">
         <v>0.0158730158730158</v>
       </c>
-      <c r="L19" s="135" t="n">
+      <c r="L19" s="137" t="n">
         <v>540</v>
       </c>
       <c r="M19" t="n">
         <v>1.851851851851852</v>
       </c>
-      <c r="N19" s="135" t="n">
+      <c r="N19" s="137" t="n">
         <v>90</v>
       </c>
       <c r="O19" t="n">
@@ -4745,34 +4774,34 @@
       <c r="S19" t="n">
         <v>10.9068100358423</v>
       </c>
-      <c r="T19" s="135" t="n">
+      <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
-      <c r="U19" s="135" t="n">
+      <c r="U19" s="137" t="n">
         <v>548.3870967741935</v>
       </c>
-      <c r="V19" s="135" t="n">
+      <c r="V19" s="137" t="n">
         <v>581.76</v>
       </c>
-      <c r="W19" s="135" t="n">
+      <c r="W19" s="137" t="n">
         <v>33.37290322580645</v>
       </c>
-      <c r="X19" s="136" t="n">
+      <c r="X19" s="138" t="n">
         <v>0.0608564705882353</v>
       </c>
-      <c r="Y19" s="135" t="n">
+      <c r="Y19" s="137" t="n">
         <v>34.22117647058823</v>
       </c>
-      <c r="Z19" s="135" t="n">
+      <c r="Z19" s="137" t="n">
         <v>-55.77882352941177</v>
       </c>
-      <c r="AB19" s="137" t="inlineStr"/>
-      <c r="AC19" s="137" t="inlineStr">
+      <c r="AB19" s="139" t="inlineStr"/>
+      <c r="AC19" s="139" t="inlineStr">
         <is>
           <t>6634088776775</t>
         </is>
       </c>
-      <c r="AD19" s="137" t="inlineStr"/>
+      <c r="AD19" s="139" t="inlineStr"/>
       <c r="AE19" t="inlineStr">
         <is>
           <t>meta:ok</t>
@@ -4790,17 +4819,17 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B20" s="134" t="n">
+      <c r="B20" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C20" s="134" t="n">
+      <c r="C20" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D20" s="134" t="n">
+      <c r="D20" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E20" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4819,72 +4848,67 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>DYN_VELOCE New Creative Apr26</t>
-        </is>
-      </c>
-      <c r="J20" s="135" t="n">
-        <v>10000</v>
-      </c>
-      <c r="K20" s="136" t="n">
-        <v>0.1587301587301587</v>
-      </c>
-      <c r="L20" s="135" t="n">
+          <t>[BMK 2025] LeadGen CQD PEN [Albania]</t>
+        </is>
+      </c>
+      <c r="J20" s="137" t="n">
         <v>500</v>
       </c>
+      <c r="K20" s="138" t="n">
+        <v>0.0079365079365079</v>
+      </c>
+      <c r="L20" s="137" t="n">
+        <v>540</v>
+      </c>
       <c r="M20" t="n">
-        <v>20</v>
-      </c>
-      <c r="N20" s="135" t="n">
-        <v>12.8</v>
+        <v>0.925925925925926</v>
+      </c>
+      <c r="N20" s="137" t="n">
+        <v>120</v>
       </c>
       <c r="O20" t="n">
-        <v>781.25</v>
+        <v>4.166666666666667</v>
       </c>
       <c r="P20" t="n">
-        <v>25.20161290322581</v>
+        <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>428.4274193548387</v>
+        <v>2.28494623655914</v>
       </c>
       <c r="R20" t="n">
-        <v>367</v>
+        <v>4</v>
       </c>
       <c r="S20" t="n">
-        <v>-61.42741935483872</v>
-      </c>
-      <c r="T20" s="135" t="n">
-        <v>322.5806451612903</v>
-      </c>
-      <c r="U20" s="135" t="n">
-        <v>5483.870967741936</v>
-      </c>
-      <c r="V20" s="135" t="n">
-        <v>7444.1</v>
-      </c>
-      <c r="W20" s="135" t="n">
-        <v>1960.229032258065</v>
-      </c>
-      <c r="X20" s="136" t="n">
-        <v>0.3574535294117647</v>
-      </c>
-      <c r="Y20" s="135" t="n">
-        <v>20.28365122615804</v>
-      </c>
-      <c r="Z20" s="135" t="n">
-        <v>7.483651226158038</v>
-      </c>
-      <c r="AA20" t="inlineStr">
-        <is>
-          <t>diminuito cpa target che era stato alzato per aiutare la campagna ad uscire dalla fase di apprendimento</t>
-        </is>
-      </c>
-      <c r="AB20" s="137" t="inlineStr"/>
-      <c r="AC20" s="137" t="inlineStr">
-        <is>
-          <t>6944411197975</t>
-        </is>
-      </c>
-      <c r="AD20" s="137" t="inlineStr"/>
+        <v>1.71505376344086</v>
+      </c>
+      <c r="T20" s="137" t="n">
+        <v>16.12903225806452</v>
+      </c>
+      <c r="U20" s="137" t="n">
+        <v>274.1935483870968</v>
+      </c>
+      <c r="V20" s="137" t="n">
+        <v>283.27</v>
+      </c>
+      <c r="W20" s="137" t="n">
+        <v>9.076451612903211</v>
+      </c>
+      <c r="X20" s="138" t="n">
+        <v>0.0331023529411764</v>
+      </c>
+      <c r="Y20" s="137" t="n">
+        <v>70.8175</v>
+      </c>
+      <c r="Z20" s="137" t="n">
+        <v>-49.1825</v>
+      </c>
+      <c r="AB20" s="139" t="inlineStr"/>
+      <c r="AC20" s="139" t="inlineStr">
+        <is>
+          <t>6666147663775</t>
+        </is>
+      </c>
+      <c r="AD20" s="139" t="inlineStr"/>
       <c r="AE20" t="inlineStr">
         <is>
           <t>meta:ok</t>
@@ -4902,13 +4926,13 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B21" s="134" t="n">
+      <c r="B21" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C21" s="134" t="n">
+      <c r="C21" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D21" s="134" t="n">
+      <c r="D21" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E21" t="n">
@@ -4934,19 +4958,19 @@
           <t>DYN_PUL Landing a pulsanti</t>
         </is>
       </c>
-      <c r="J21" s="135" t="n">
+      <c r="J21" s="137" t="n">
         <v>1500</v>
       </c>
-      <c r="K21" s="136" t="n">
+      <c r="K21" s="138" t="n">
         <v>0.0238095238095238</v>
       </c>
-      <c r="L21" s="135" t="n">
+      <c r="L21" s="137" t="n">
         <v>320</v>
       </c>
       <c r="M21" t="n">
         <v>4.6875</v>
       </c>
-      <c r="N21" s="135" t="n">
+      <c r="N21" s="137" t="n">
         <v>40</v>
       </c>
       <c r="O21" t="n">
@@ -4964,34 +4988,34 @@
       <c r="S21" t="n">
         <v>0.4354838709677402</v>
       </c>
-      <c r="T21" s="135" t="n">
+      <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
-      <c r="U21" s="135" t="n">
+      <c r="U21" s="137" t="n">
         <v>822.5806451612904</v>
       </c>
-      <c r="V21" s="135" t="n">
+      <c r="V21" s="137" t="n">
         <v>1057.013242</v>
       </c>
-      <c r="W21" s="135" t="n">
+      <c r="W21" s="137" t="n">
         <v>234.4325968387096</v>
       </c>
-      <c r="X21" s="136" t="n">
+      <c r="X21" s="138" t="n">
         <v>0.2849964902745097</v>
       </c>
-      <c r="Y21" s="135" t="n">
+      <c r="Y21" s="137" t="n">
         <v>50.3339639047619</v>
       </c>
-      <c r="Z21" s="135" t="n">
+      <c r="Z21" s="137" t="n">
         <v>10.3339639047619</v>
       </c>
-      <c r="AB21" s="137" t="inlineStr">
+      <c r="AB21" s="139" t="inlineStr">
         <is>
           <t>22660883424</t>
         </is>
       </c>
-      <c r="AC21" s="137" t="inlineStr"/>
-      <c r="AD21" s="137" t="inlineStr"/>
+      <c r="AC21" s="139" t="inlineStr"/>
+      <c r="AD21" s="139" t="inlineStr"/>
       <c r="AE21" t="inlineStr">
         <is>
           <t>google:ok</t>
@@ -5009,13 +5033,13 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B22" s="134" t="n">
+      <c r="B22" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C22" s="134" t="n">
+      <c r="C22" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D22" s="134" t="n">
+      <c r="D22" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E22" t="n">
@@ -5041,19 +5065,19 @@
           <t>DYN_PUL Leads-Pmax</t>
         </is>
       </c>
-      <c r="J22" s="135" t="n">
+      <c r="J22" s="137" t="n">
         <v>1500</v>
       </c>
-      <c r="K22" s="136" t="n">
+      <c r="K22" s="138" t="n">
         <v>0.0238095238095238</v>
       </c>
-      <c r="L22" s="135" t="n">
+      <c r="L22" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="M22" t="n">
         <v>1.5</v>
       </c>
-      <c r="N22" s="135" t="n">
+      <c r="N22" s="137" t="n">
         <v>15</v>
       </c>
       <c r="O22" t="n">
@@ -5071,25 +5095,25 @@
       <c r="S22" t="n">
         <v>47.16129032258065</v>
       </c>
-      <c r="T22" s="135" t="n">
+      <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
-      <c r="U22" s="135" t="n">
+      <c r="U22" s="137" t="n">
         <v>822.5806451612904</v>
       </c>
-      <c r="V22" s="135" t="n">
+      <c r="V22" s="137" t="n">
         <v>1241.033961</v>
       </c>
-      <c r="W22" s="135" t="n">
+      <c r="W22" s="137" t="n">
         <v>418.4533158387097</v>
       </c>
-      <c r="X22" s="136" t="n">
+      <c r="X22" s="138" t="n">
         <v>0.5087079525882353</v>
       </c>
-      <c r="Y22" s="135" t="n">
+      <c r="Y22" s="137" t="n">
         <v>12.16699961764706</v>
       </c>
-      <c r="Z22" s="135" t="n">
+      <c r="Z22" s="137" t="n">
         <v>-2.833000382352941</v>
       </c>
       <c r="AA22" t="inlineStr">
@@ -5097,13 +5121,13 @@
           <t>abbassato leggermente lo spending giornaliero</t>
         </is>
       </c>
-      <c r="AB22" s="137" t="inlineStr">
+      <c r="AB22" s="139" t="inlineStr">
         <is>
           <t>21905808840</t>
         </is>
       </c>
-      <c r="AC22" s="137" t="inlineStr"/>
-      <c r="AD22" s="137" t="inlineStr"/>
+      <c r="AC22" s="139" t="inlineStr"/>
+      <c r="AD22" s="139" t="inlineStr"/>
       <c r="AE22" t="inlineStr">
         <is>
           <t>google:ok</t>
@@ -5121,13 +5145,13 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B23" s="134" t="n">
+      <c r="B23" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C23" s="134" t="n">
+      <c r="C23" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D23" s="134" t="n">
+      <c r="D23" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E23" t="n">
@@ -5153,19 +5177,19 @@
           <t>DYN_PUL NEW Meta</t>
         </is>
       </c>
-      <c r="J23" s="135" t="n">
+      <c r="J23" s="137" t="n">
         <v>1000</v>
       </c>
-      <c r="K23" s="136" t="n">
+      <c r="K23" s="138" t="n">
         <v>0.0158730158730158</v>
       </c>
-      <c r="L23" s="135" t="n">
+      <c r="L23" s="137" t="n">
         <v>400</v>
       </c>
       <c r="M23" t="n">
         <v>2.5</v>
       </c>
-      <c r="N23" s="135" t="n">
+      <c r="N23" s="137" t="n">
         <v>26</v>
       </c>
       <c r="O23" t="n">
@@ -5183,34 +5207,34 @@
       <c r="S23" t="n">
         <v>37.90818858560795</v>
       </c>
-      <c r="T23" s="135" t="n">
+      <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
-      <c r="U23" s="135" t="n">
+      <c r="U23" s="137" t="n">
         <v>548.3870967741935</v>
       </c>
-      <c r="V23" s="135" t="n">
+      <c r="V23" s="137" t="n">
         <v>1016.68</v>
       </c>
-      <c r="W23" s="135" t="n">
+      <c r="W23" s="137" t="n">
         <v>468.2929032258064</v>
       </c>
-      <c r="X23" s="136" t="n">
+      <c r="X23" s="138" t="n">
         <v>0.8539458823529411</v>
       </c>
-      <c r="Y23" s="135" t="n">
+      <c r="Y23" s="137" t="n">
         <v>17.23186440677966</v>
       </c>
-      <c r="Z23" s="135" t="n">
+      <c r="Z23" s="137" t="n">
         <v>-8.76813559322034</v>
       </c>
-      <c r="AB23" s="137" t="inlineStr"/>
-      <c r="AC23" s="137" t="inlineStr">
+      <c r="AB23" s="139" t="inlineStr"/>
+      <c r="AC23" s="139" t="inlineStr">
         <is>
           <t>6901683340975</t>
         </is>
       </c>
-      <c r="AD23" s="137" t="inlineStr"/>
+      <c r="AD23" s="139" t="inlineStr"/>
       <c r="AE23" t="inlineStr">
         <is>
           <t>meta:ok</t>
@@ -5228,13 +5252,13 @@
           <t>campaign</t>
         </is>
       </c>
-      <c r="B24" s="134" t="n">
+      <c r="B24" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C24" s="134" t="n">
+      <c r="C24" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D24" s="134" t="n">
+      <c r="D24" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="E24" t="n">
@@ -5260,31 +5284,31 @@
           <t>DYN_Landing_Whatsapp</t>
         </is>
       </c>
-      <c r="J24" s="135" t="n"/>
-      <c r="K24" s="136" t="n">
+      <c r="J24" s="137" t="n"/>
+      <c r="K24" s="138" t="n">
         <v>0</v>
       </c>
-      <c r="L24" s="135" t="n"/>
-      <c r="N24" s="135" t="n"/>
+      <c r="L24" s="137" t="n"/>
+      <c r="N24" s="137" t="n"/>
       <c r="R24" t="n">
         <v>0</v>
       </c>
-      <c r="T24" s="135" t="n"/>
-      <c r="U24" s="135" t="n"/>
-      <c r="V24" s="135" t="n">
+      <c r="T24" s="137" t="n"/>
+      <c r="U24" s="137" t="n"/>
+      <c r="V24" s="137" t="n">
         <v>144.47</v>
       </c>
-      <c r="W24" s="135" t="n"/>
-      <c r="X24" s="136" t="n"/>
-      <c r="Y24" s="135" t="n"/>
-      <c r="Z24" s="135" t="n"/>
-      <c r="AB24" s="137" t="inlineStr"/>
-      <c r="AC24" s="137" t="inlineStr">
+      <c r="W24" s="137" t="n"/>
+      <c r="X24" s="138" t="n"/>
+      <c r="Y24" s="137" t="n"/>
+      <c r="Z24" s="137" t="n"/>
+      <c r="AB24" s="139" t="inlineStr"/>
+      <c r="AC24" s="139" t="inlineStr">
         <is>
           <t>52533122877779</t>
         </is>
       </c>
-      <c r="AD24" s="137" t="inlineStr"/>
+      <c r="AD24" s="139" t="inlineStr"/>
       <c r="AE24" t="inlineStr">
         <is>
           <t>meta:ok</t>
@@ -5302,13 +5326,13 @@
           <t>subtotal</t>
         </is>
       </c>
-      <c r="B25" s="134" t="n">
+      <c r="B25" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C25" s="134" t="n">
+      <c r="C25" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D25" s="134" t="n">
+      <c r="D25" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -5321,14 +5345,14 @@
           <t>TOT Area Clienti</t>
         </is>
       </c>
-      <c r="J25" s="135" t="n">
+      <c r="J25" s="137" t="n">
         <v>21000</v>
       </c>
-      <c r="K25" s="136" t="n">
+      <c r="K25" s="138" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="L25" s="135" t="n"/>
-      <c r="N25" s="135" t="n">
+      <c r="L25" s="137" t="n"/>
+      <c r="N25" s="137" t="n">
         <v>45</v>
       </c>
       <c r="O25" t="n">
@@ -5346,30 +5370,30 @@
       <c r="S25" t="n">
         <v>35.08602150537632</v>
       </c>
-      <c r="T25" s="135" t="n">
+      <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
-      <c r="U25" s="135" t="n">
+      <c r="U25" s="137" t="n">
         <v>11516.12903225806</v>
       </c>
-      <c r="V25" s="135" t="n">
+      <c r="V25" s="137" t="n">
         <v>12526.432246</v>
       </c>
-      <c r="W25" s="135" t="n">
+      <c r="W25" s="137" t="n">
         <v>1010.303213741934</v>
       </c>
-      <c r="X25" s="136" t="n">
+      <c r="X25" s="138" t="n">
         <v>0.0877294107170867</v>
       </c>
-      <c r="Y25" s="135" t="n">
+      <c r="Y25" s="137" t="n">
         <v>43.04615892096219</v>
       </c>
-      <c r="Z25" s="135" t="n">
+      <c r="Z25" s="137" t="n">
         <v>-1.953841079037808</v>
       </c>
-      <c r="AB25" s="137" t="inlineStr"/>
-      <c r="AC25" s="137" t="inlineStr"/>
-      <c r="AD25" s="137" t="inlineStr"/>
+      <c r="AB25" s="139" t="inlineStr"/>
+      <c r="AC25" s="139" t="inlineStr"/>
+      <c r="AD25" s="139" t="inlineStr"/>
       <c r="AE25" t="inlineStr">
         <is>
           <t>partial</t>
@@ -5382,13 +5406,13 @@
           <t>subtotal</t>
         </is>
       </c>
-      <c r="B26" s="134" t="n">
+      <c r="B26" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C26" s="134" t="n">
+      <c r="C26" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D26" s="134" t="n">
+      <c r="D26" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -5401,19 +5425,19 @@
           <t>TOT Lead Veloce</t>
         </is>
       </c>
-      <c r="J26" s="135" t="n">
+      <c r="J26" s="137" t="n">
         <v>31000</v>
       </c>
-      <c r="K26" s="136" t="n">
+      <c r="K26" s="138" t="n">
         <v>0.492063492063492</v>
       </c>
-      <c r="L26" s="135" t="n">
+      <c r="L26" s="137" t="n">
         <v>560.016726903432</v>
       </c>
       <c r="M26" t="n">
         <v>55.35548941798942</v>
       </c>
-      <c r="N26" s="135" t="n">
+      <c r="N26" s="137" t="n">
         <v>22.68206825816996</v>
       </c>
       <c r="O26" t="n">
@@ -5431,30 +5455,30 @@
       <c r="S26" t="n">
         <v>113.5092654468716</v>
       </c>
-      <c r="T26" s="135" t="n">
+      <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
-      <c r="U26" s="135" t="n">
+      <c r="U26" s="137" t="n">
         <v>17000</v>
       </c>
-      <c r="V26" s="135" t="n">
+      <c r="V26" s="137" t="n">
         <v>21792.800088</v>
       </c>
-      <c r="W26" s="135" t="n">
+      <c r="W26" s="137" t="n">
         <v>4792.800088</v>
       </c>
-      <c r="X26" s="136" t="n">
+      <c r="X26" s="138" t="n">
         <v>0.2819294169411764</v>
       </c>
-      <c r="Y26" s="135" t="n">
+      <c r="Y26" s="137" t="n">
         <v>25.25237553650058</v>
       </c>
-      <c r="Z26" s="135" t="n">
+      <c r="Z26" s="137" t="n">
         <v>2.570307278330624</v>
       </c>
-      <c r="AB26" s="137" t="inlineStr"/>
-      <c r="AC26" s="137" t="inlineStr"/>
-      <c r="AD26" s="137" t="inlineStr"/>
+      <c r="AB26" s="139" t="inlineStr"/>
+      <c r="AC26" s="139" t="inlineStr"/>
+      <c r="AD26" s="139" t="inlineStr"/>
       <c r="AE26" t="inlineStr">
         <is>
           <t>partial</t>
@@ -5467,13 +5491,13 @@
           <t>subtotal</t>
         </is>
       </c>
-      <c r="B27" s="134" t="n">
+      <c r="B27" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C27" s="134" t="n">
+      <c r="C27" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D27" s="134" t="n">
+      <c r="D27" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -5486,19 +5510,19 @@
           <t>TOT DEM</t>
         </is>
       </c>
-      <c r="J27" s="135" t="n">
+      <c r="J27" s="137" t="n">
         <v>11000</v>
       </c>
-      <c r="K27" s="136" t="n">
+      <c r="K27" s="138" t="n">
         <v>0.1746031746031746</v>
       </c>
-      <c r="L27" s="135" t="n">
+      <c r="L27" s="137" t="n">
         <v>376.6304347826087</v>
       </c>
       <c r="M27" t="n">
         <v>29.20634920634921</v>
       </c>
-      <c r="N27" s="135" t="n">
+      <c r="N27" s="137" t="n">
         <v>8.134054054054054</v>
       </c>
       <c r="O27" t="n">
@@ -5516,30 +5540,30 @@
       <c r="S27" t="n">
         <v>16.39464252027915</v>
       </c>
-      <c r="T27" s="135" t="n">
+      <c r="T27" s="137" t="n">
         <v>478.2608695652174</v>
       </c>
-      <c r="U27" s="135" t="n">
+      <c r="U27" s="137" t="n">
         <v>6217.391304347826</v>
       </c>
-      <c r="V27" s="135" t="n">
+      <c r="V27" s="137" t="n">
         <v>6095</v>
       </c>
-      <c r="W27" s="135" t="n">
+      <c r="W27" s="137" t="n">
         <v>-122.391304347826</v>
       </c>
-      <c r="X27" s="136" t="n">
+      <c r="X27" s="138" t="n">
         <v>-0.0196853146853146</v>
       </c>
-      <c r="Y27" s="135" t="n">
+      <c r="Y27" s="137" t="n">
         <v>8.040897097625329</v>
       </c>
-      <c r="Z27" s="135" t="n">
+      <c r="Z27" s="137" t="n">
         <v>-0.0931569564287251</v>
       </c>
-      <c r="AB27" s="137" t="inlineStr"/>
-      <c r="AC27" s="137" t="inlineStr"/>
-      <c r="AD27" s="137" t="inlineStr"/>
+      <c r="AB27" s="139" t="inlineStr"/>
+      <c r="AC27" s="139" t="inlineStr"/>
+      <c r="AD27" s="139" t="inlineStr"/>
       <c r="AE27" t="inlineStr">
         <is>
           <t>success</t>
@@ -5552,13 +5576,13 @@
           <t>total</t>
         </is>
       </c>
-      <c r="B28" s="134" t="n">
+      <c r="B28" s="136" t="n">
         <v>46221</v>
       </c>
-      <c r="C28" s="134" t="n">
+      <c r="C28" s="136" t="n">
         <v>46204</v>
       </c>
-      <c r="D28" s="134" t="n">
+      <c r="D28" s="136" t="n">
         <v>46220</v>
       </c>
       <c r="F28" t="inlineStr">
@@ -5571,19 +5595,19 @@
           <t>TOTALE GENERALE</t>
         </is>
       </c>
-      <c r="J28" s="135" t="n">
+      <c r="J28" s="137" t="n">
         <v>63000</v>
       </c>
-      <c r="K28" s="136" t="n">
+      <c r="K28" s="138" t="n">
         <v>1</v>
       </c>
-      <c r="L28" s="135" t="n">
+      <c r="L28" s="137" t="n">
         <v>745.0169133605773</v>
       </c>
       <c r="M28" t="n">
         <v>84.56183862433862</v>
       </c>
-      <c r="N28" s="135" t="n">
+      <c r="N28" s="137" t="n">
         <v>19.77572292204534</v>
       </c>
       <c r="O28" t="n">
@@ -5601,30 +5625,30 @@
       <c r="S28" t="n">
         <v>164.9899294725271</v>
       </c>
-      <c r="T28" s="135" t="n">
+      <c r="T28" s="137" t="n">
         <v>2155.680224403927</v>
       </c>
-      <c r="U28" s="135" t="n">
+      <c r="U28" s="137" t="n">
         <v>34733.52033660589</v>
       </c>
-      <c r="V28" s="135" t="n">
+      <c r="V28" s="137" t="n">
         <v>40414.232334</v>
       </c>
-      <c r="W28" s="135" t="n">
+      <c r="W28" s="137" t="n">
         <v>5680.711997394108</v>
       </c>
-      <c r="X28" s="136" t="n">
+      <c r="X28" s="138" t="n">
         <v>0.1635512882754693</v>
       </c>
-      <c r="Y28" s="135" t="n">
+      <c r="Y28" s="137" t="n">
         <v>21.13715080230126</v>
       </c>
-      <c r="Z28" s="135" t="n">
+      <c r="Z28" s="137" t="n">
         <v>1.361427880255917</v>
       </c>
-      <c r="AB28" s="137" t="inlineStr"/>
-      <c r="AC28" s="137" t="inlineStr"/>
-      <c r="AD28" s="137" t="inlineStr"/>
+      <c r="AB28" s="139" t="inlineStr"/>
+      <c r="AC28" s="139" t="inlineStr"/>
+      <c r="AD28" s="139" t="inlineStr"/>
       <c r="AE28" t="inlineStr">
         <is>
           <t>partial</t>
@@ -5702,7 +5726,7 @@
           <t>start_date</t>
         </is>
       </c>
-      <c r="B3" s="138" t="n">
+      <c r="B3" s="140" t="n">
         <v>46204</v>
       </c>
       <c r="D3" s="33" t="inlineStr">
@@ -5722,7 +5746,7 @@
           <t>end_date</t>
         </is>
       </c>
-      <c r="B4" s="138" t="n">
+      <c r="B4" s="140" t="n">
         <v>46220</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
@@ -5782,8 +5806,8 @@
           <t>updated_at</t>
         </is>
       </c>
-      <c r="B7" s="139" t="n">
-        <v>46225.48482638889</v>
+      <c r="B7" s="141" t="n">
+        <v>46225.5041550926</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-07-23
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 17/07/2026  |  Ultimo aggiornamento: 22/07/2026 12:05</t>
+          <t>Periodo: 01/07/2026 - 22/07/2026  |  Ultimo aggiornamento: 23/07/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1065,16 +1065,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>5209.677419354838</v>
+        <v>6741.935483870968</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>5794.215866</v>
+        <v>7194.217537</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>584.5384466451615</v>
+        <v>452.2820531290327</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.1122024262910217</v>
+        <v>0.06708489783253591</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1173,16 +1173,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>822.5806451612904</v>
+        <v>1064.516129032258</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>1074.27638</v>
+        <v>1257.348004</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>251.6957348387096</v>
+        <v>192.8318749677419</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>0.3059830501960784</v>
+        <v>0.1811450946666666</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1281,16 +1281,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>5483.870967741936</v>
+        <v>7096.774193548386</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>5657.94</v>
+        <v>6645.12</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>174.069032258064</v>
+        <v>-451.6541935483865</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.0317419999999999</v>
+        <v>-0.0636421818181817</v>
       </c>
       <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
@@ -1328,34 +1328,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>255.9139784946237</v>
+        <v>331.1827956989247</v>
       </c>
       <c r="N10" s="125" t="n">
-        <v>291</v>
+        <v>328</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>35.08602150537632</v>
+        <v>-3.182795698924735</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>11516.12903225806</v>
+        <v>14903.22580645161</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>12526.432246</v>
+        <v>15096.685541</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>1010.303213741934</v>
+        <v>193.4597345483889</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>0.0877294107170867</v>
+        <v>0.012981064439394</v>
       </c>
       <c r="U10" s="123" t="n">
-        <v>43.04615892096219</v>
+        <v>46.02648030792683</v>
       </c>
       <c r="V10" s="123" t="n">
-        <v>-1.953841079037808</v>
+        <v>1.026480307926832</v>
       </c>
       <c r="W10" s="126" t="n"/>
     </row>
@@ -1407,34 +1407,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>64.51612903225806</v>
+        <v>83.49146110056925</v>
       </c>
       <c r="N11" s="119" t="n">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>33.48387096774194</v>
+        <v>27.50853889943074</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>2193.548387096774</v>
+        <v>2838.709677419354</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>3069.617174</v>
+        <v>3637.892963</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>876.0687869032258</v>
+        <v>799.1832855806451</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.3993842999117647</v>
+        <v>0.2815304756022727</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>31.3226242244898</v>
+        <v>32.77381047747748</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>-2.677375775510203</v>
+        <v>-1.226189522522525</v>
       </c>
       <c r="W11" s="120" t="inlineStr">
         <is>
@@ -1490,34 +1490,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M12" s="127" t="n">
-        <v>128.1943862589024</v>
+        <v>165.8986175115207</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>61</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>24.80561374109763</v>
+        <v>2.10138248847926</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>4935.483870967741</v>
+        <v>6387.096774193548</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>5490.756616000001</v>
+        <v>6906.593127</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>555.2727450322591</v>
+        <v>519.4963528064518</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>0.1125062424575165</v>
+        <v>0.0813352875606061</v>
       </c>
       <c r="U12" s="128" t="n">
-        <v>35.88729814379085</v>
+        <v>41.110673375</v>
       </c>
       <c r="V12" s="128" t="n">
-        <v>-2.612701856209149</v>
+        <v>2.610673374999997</v>
       </c>
       <c r="W12" s="120" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="L13" s="113" t="n"/>
       <c r="M13" s="113" t="n"/>
       <c r="N13" s="119" t="n">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="O13" s="113" t="n"/>
       <c r="P13" s="117" t="n"/>
@@ -1620,34 +1620,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="127" t="n">
-        <v>14.43123938879457</v>
+        <v>18.67572156196944</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>5</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-5.431239388794566</v>
+        <v>-8.675721561969439</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>548.3870967741935</v>
+        <v>709.6774193548387</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>510.988722</v>
+        <v>702.1896790000001</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-37.39837477419354</v>
+        <v>-7.487740354838593</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.0681970363529411</v>
+        <v>-0.0105509068636362</v>
       </c>
       <c r="U14" s="128" t="n">
-        <v>56.77652466666667</v>
+        <v>70.21896790000001</v>
       </c>
       <c r="V14" s="128" t="n">
-        <v>18.77652466666667</v>
+        <v>32.21896790000001</v>
       </c>
       <c r="W14" s="120" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
       <c r="L15" s="113" t="n"/>
       <c r="M15" s="113" t="n"/>
       <c r="N15" s="119" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O15" s="113" t="n"/>
       <c r="P15" s="117" t="n"/>
@@ -1750,34 +1750,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M16" s="127" t="n">
-        <v>2.193548387096774</v>
+        <v>2.838709677419355</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>-0.193548387096774</v>
+        <v>-0.838709677419355</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>548.3870967741935</v>
+        <v>709.6774193548387</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>630.160373</v>
+        <v>748.7606519999999</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>81.77327622580651</v>
+        <v>39.08323264516128</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.1491159742941177</v>
+        <v>0.0550718278181818</v>
       </c>
       <c r="U16" s="128" t="n">
-        <v>315.0801865</v>
+        <v>374.380326</v>
       </c>
       <c r="V16" s="128" t="n">
-        <v>65.08018650000002</v>
+        <v>124.380326</v>
       </c>
       <c r="W16" s="120" t="inlineStr">
         <is>
@@ -1880,34 +1880,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>428.4274193548387</v>
+        <v>554.4354838709678</v>
       </c>
       <c r="N18" s="119" t="n">
-        <v>367</v>
+        <v>417</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-61.42741935483872</v>
+        <v>-137.4354838709678</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>5483.870967741936</v>
+        <v>7096.774193548386</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>7444.1</v>
+        <v>9676.860000000001</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>1960.229032258065</v>
+        <v>2580.085806451614</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>0.3574535294117647</v>
+        <v>0.3635575454545456</v>
       </c>
       <c r="U18" s="117" t="n">
-        <v>20.28365122615804</v>
+        <v>23.20589928057554</v>
       </c>
       <c r="V18" s="117" t="n">
-        <v>7.483651226158038</v>
+        <v>10.40589928057554</v>
       </c>
       <c r="W18" s="120" t="inlineStr">
         <is>
@@ -1963,34 +1963,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>6.854838709677419</v>
+        <v>8.870967741935484</v>
       </c>
       <c r="N19" s="119" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>24.14516129032258</v>
+        <v>23.12903225806452</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>274.1935483870968</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>322.95</v>
+        <v>376.46</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>48.75645161290322</v>
+        <v>21.62129032258065</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>0.1778176470588235</v>
+        <v>0.0609327272727272</v>
       </c>
       <c r="U19" s="117" t="n">
-        <v>10.41774193548387</v>
+        <v>11.764375</v>
       </c>
       <c r="V19" s="117" t="n">
-        <v>-29.58225806451613</v>
+        <v>-28.235625</v>
       </c>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
@@ -2042,34 +2042,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>6.093189964157706</v>
+        <v>7.885304659498208</v>
       </c>
       <c r="N20" s="119" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>10.9068100358423</v>
+        <v>11.11469534050179</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>548.3870967741935</v>
+        <v>709.6774193548387</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>581.76</v>
+        <v>679.27</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>33.37290322580645</v>
+        <v>-30.40741935483868</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>0.0608564705882353</v>
+        <v>-0.0428468181818181</v>
       </c>
       <c r="U20" s="117" t="n">
-        <v>34.22117647058823</v>
+        <v>35.75105263157894</v>
       </c>
       <c r="V20" s="117" t="n">
-        <v>-55.77882352941177</v>
+        <v>-54.24894736842106</v>
       </c>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
@@ -2121,34 +2121,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>2.28494623655914</v>
+        <v>2.956989247311828</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>4</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>1.71505376344086</v>
+        <v>1.043010752688172</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>274.1935483870968</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="R21" s="117" t="n">
-        <v>283.27</v>
+        <v>335.9</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>9.076451612903211</v>
+        <v>-18.93870967741936</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>0.0331023529411764</v>
+        <v>-0.0533727272727272</v>
       </c>
       <c r="U21" s="117" t="n">
-        <v>70.8175</v>
+        <v>83.97499999999999</v>
       </c>
       <c r="V21" s="117" t="n">
-        <v>-49.1825</v>
+        <v>-36.02500000000001</v>
       </c>
       <c r="W21" s="120" t="inlineStr"/>
     </row>
@@ -2200,34 +2200,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>20.56451612903226</v>
+        <v>26.61290322580645</v>
       </c>
       <c r="N22" s="119" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>0.4354838709677402</v>
+        <v>-4.612903225806452</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>822.5806451612904</v>
+        <v>1064.516129032258</v>
       </c>
       <c r="R22" s="117" t="n">
-        <v>1057.013242</v>
+        <v>1277.522538</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>234.4325968387096</v>
+        <v>213.0064089677419</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>0.2849964902745097</v>
+        <v>0.2000969296363636</v>
       </c>
       <c r="U22" s="117" t="n">
-        <v>50.3339639047619</v>
+        <v>58.06920627272727</v>
       </c>
       <c r="V22" s="117" t="n">
-        <v>10.3339639047619</v>
+        <v>18.06920627272727</v>
       </c>
       <c r="W22" s="120" t="inlineStr"/>
     </row>
@@ -2279,34 +2279,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>54.83870967741935</v>
+        <v>70.96774193548387</v>
       </c>
       <c r="N23" s="119" t="n">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>47.16129032258065</v>
+        <v>43.03225806451613</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>822.5806451612904</v>
+        <v>1064.516129032258</v>
       </c>
       <c r="R23" s="117" t="n">
-        <v>1241.033961</v>
+        <v>1551.287959</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>418.4533158387097</v>
+        <v>486.771829967742</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.5087079525882353</v>
+        <v>0.457270506939394</v>
       </c>
       <c r="U23" s="117" t="n">
-        <v>12.16699961764706</v>
+        <v>13.60778911403509</v>
       </c>
       <c r="V23" s="117" t="n">
-        <v>-2.833000382352941</v>
+        <v>-1.392210885964912</v>
       </c>
       <c r="W23" s="120" t="inlineStr">
         <is>
@@ -2362,34 +2362,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>21.09181141439206</v>
+        <v>27.29528535980149</v>
       </c>
       <c r="N24" s="119" t="n">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>37.90818858560795</v>
+        <v>39.70471464019852</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>548.3870967741935</v>
+        <v>709.6774193548387</v>
       </c>
       <c r="R24" s="117" t="n">
-        <v>1016.68</v>
+        <v>1173.01</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>468.2929032258064</v>
+        <v>463.3325806451613</v>
       </c>
       <c r="T24" s="118" t="n">
-        <v>0.8539458823529411</v>
+        <v>0.6528777272727274</v>
       </c>
       <c r="U24" s="117" t="n">
-        <v>17.23186440677966</v>
+        <v>17.50761194029851</v>
       </c>
       <c r="V24" s="117" t="n">
-        <v>-8.76813559322034</v>
+        <v>-8.492388059701494</v>
       </c>
       <c r="W24" s="120" t="inlineStr"/>
     </row>
@@ -2430,17 +2430,19 @@
       <c r="L25" s="119" t="n"/>
       <c r="M25" s="119" t="n"/>
       <c r="N25" s="119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O25" s="119" t="n"/>
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>144.47</v>
+        <v>466.69</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
-      <c r="U25" s="117" t="n"/>
+      <c r="U25" s="117" t="n">
+        <v>466.69</v>
+      </c>
       <c r="V25" s="117" t="n"/>
       <c r="W25" s="120" t="inlineStr"/>
     </row>
@@ -2476,34 +2478,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>749.4907345531284</v>
+        <v>969.929185892284</v>
       </c>
       <c r="N26" s="125" t="n">
-        <v>863</v>
+        <v>967</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>113.5092654468716</v>
+        <v>-2.929185892283954</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>17000</v>
+        <v>22000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>21792.800088</v>
+        <v>27532.436918</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>4792.800088</v>
+        <v>5532.436917999999</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>0.2819294169411764</v>
+        <v>0.2514744053636363</v>
       </c>
       <c r="U26" s="123" t="n">
-        <v>25.25237553650058</v>
+        <v>28.47201335884177</v>
       </c>
       <c r="V26" s="123" t="n">
-        <v>2.570307278330624</v>
+        <v>5.789945100671822</v>
       </c>
       <c r="W26" s="126" t="n"/>
     </row>
@@ -2551,28 +2553,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>360.7809847198643</v>
+        <v>466.8930390492361</v>
       </c>
       <c r="N27" s="119" t="n">
-        <v>360</v>
+        <v>371</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-0.7809847198642501</v>
+        <v>-95.89303904923604</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>2826.086956521739</v>
+        <v>3478.260869565217</v>
       </c>
       <c r="R27" s="117" t="n">
-        <v>2736</v>
+        <v>2819.6</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-90.086956521739</v>
+        <v>-658.6608695652176</v>
       </c>
       <c r="T27" s="118" t="n">
-        <v>-0.031876923076923</v>
+        <v>-0.189365</v>
       </c>
       <c r="U27" s="117" t="n">
         <v>7.6</v>
@@ -2626,28 +2628,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>243.7275985663082</v>
+        <v>315.4121863799283</v>
       </c>
       <c r="N28" s="119" t="n">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-68.72759856630825</v>
+        <v>-128.4121863799283</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>2260.869565217391</v>
+        <v>2782.608695652174</v>
       </c>
       <c r="R28" s="117" t="n">
-        <v>1575</v>
+        <v>1683</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-685.8695652173915</v>
+        <v>-1099.608695652174</v>
       </c>
       <c r="T28" s="118" t="n">
-        <v>-0.3033653846153846</v>
+        <v>-0.395171875</v>
       </c>
       <c r="U28" s="117" t="n">
         <v>9</v>
@@ -2701,28 +2703,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>137.0967741935484</v>
+        <v>177.4193548387097</v>
       </c>
       <c r="N29" s="119" t="n">
-        <v>223</v>
+        <v>240</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>85.90322580645162</v>
+        <v>62.58064516129033</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>1130.434782608696</v>
+        <v>1391.304347826087</v>
       </c>
       <c r="R29" s="117" t="n">
-        <v>1784</v>
+        <v>1920</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>653.5652173913043</v>
+        <v>528.695652173913</v>
       </c>
       <c r="T29" s="118" t="n">
-        <v>0.578153846153846</v>
+        <v>0.3799999999999999</v>
       </c>
       <c r="U29" s="117" t="n">
         <v>8</v>
@@ -2764,34 +2766,34 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>741.6053574797209</v>
+        <v>959.724580267874</v>
       </c>
       <c r="N30" s="125" t="n">
-        <v>758</v>
+        <v>798</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>16.39464252027915</v>
+        <v>-161.724580267874</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>6217.391304347826</v>
+        <v>7652.173913043478</v>
       </c>
       <c r="R30" s="123" t="n">
-        <v>6095</v>
+        <v>6422.6</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>-122.391304347826</v>
+        <v>-1229.573913043478</v>
       </c>
       <c r="T30" s="124" t="n">
-        <v>-0.0196853146853146</v>
+        <v>-0.1606829545454544</v>
       </c>
       <c r="U30" s="123" t="n">
-        <v>8.040897097625329</v>
+        <v>8.048370927318297</v>
       </c>
       <c r="V30" s="123" t="n">
-        <v>-0.0931569564287251</v>
+        <v>-0.0856831267357574</v>
       </c>
       <c r="W30" s="126" t="n"/>
     </row>
@@ -2827,34 +2829,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="133" t="n">
-        <v>1747.010070527473</v>
+        <v>2260.836561859083</v>
       </c>
       <c r="N31" s="133" t="n">
-        <v>1912</v>
+        <v>2093</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>164.9899294725271</v>
+        <v>-167.8365618590828</v>
       </c>
       <c r="P31" s="131" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="Q31" s="131" t="n">
-        <v>34733.52033660589</v>
+        <v>44555.39971949509</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>40414.232334</v>
+        <v>49051.722459</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>5680.711997394108</v>
+        <v>4496.322739504911</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>0.1635512882754693</v>
+        <v>0.1009153271615147</v>
       </c>
       <c r="U31" s="131" t="n">
-        <v>21.13715080230126</v>
+        <v>23.43608335355948</v>
       </c>
       <c r="V31" s="131" t="n">
-        <v>1.361427880255917</v>
+        <v>3.660360431514143</v>
       </c>
       <c r="W31" s="134" t="n"/>
     </row>
@@ -3135,13 +3137,13 @@
         </is>
       </c>
       <c r="B2" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C2" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D2" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3178,16 +3180,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="137" t="n">
-        <v>5209.677419354838</v>
+        <v>6741.935483870968</v>
       </c>
       <c r="V2" s="137" t="n">
-        <v>5794.215866</v>
+        <v>7194.217537</v>
       </c>
       <c r="W2" s="137" t="n">
-        <v>584.5384466451615</v>
+        <v>452.2820531290327</v>
       </c>
       <c r="X2" s="138" t="n">
-        <v>0.1122024262910217</v>
+        <v>0.06708489783253591</v>
       </c>
       <c r="Y2" s="137" t="n"/>
       <c r="Z2" s="137" t="n"/>
@@ -3205,7 +3207,7 @@
       <c r="AD2" s="139" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_3</t>
+          <t>google:ok;google:includes_excel_row_3;crm:stale</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -3221,13 +3223,13 @@
         </is>
       </c>
       <c r="B3" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C3" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D3" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3272,7 +3274,7 @@
       <c r="AD3" s="139" t="inlineStr"/>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_2</t>
+          <t>google:rolled_up_to_excel_row_2;crm:stale</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -3288,13 +3290,13 @@
         </is>
       </c>
       <c r="B4" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C4" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D4" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3331,16 +3333,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="137" t="n">
-        <v>822.5806451612904</v>
+        <v>1064.516129032258</v>
       </c>
       <c r="V4" s="137" t="n">
-        <v>1074.27638</v>
+        <v>1257.348004</v>
       </c>
       <c r="W4" s="137" t="n">
-        <v>251.6957348387096</v>
+        <v>192.8318749677419</v>
       </c>
       <c r="X4" s="138" t="n">
-        <v>0.3059830501960784</v>
+        <v>0.1811450946666666</v>
       </c>
       <c r="Y4" s="137" t="n"/>
       <c r="Z4" s="137" t="n"/>
@@ -3358,7 +3360,7 @@
       <c r="AD4" s="139" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_5</t>
+          <t>google:ok;google:includes_excel_row_5;crm:stale</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -3374,13 +3376,13 @@
         </is>
       </c>
       <c r="B5" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C5" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D5" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3425,7 +3427,7 @@
       <c r="AD5" s="139" t="inlineStr"/>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_4</t>
+          <t>google:rolled_up_to_excel_row_4;crm:stale</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -3441,13 +3443,13 @@
         </is>
       </c>
       <c r="B6" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C6" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D6" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3484,16 +3486,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="137" t="n">
-        <v>5483.870967741936</v>
+        <v>7096.774193548386</v>
       </c>
       <c r="V6" s="137" t="n">
-        <v>5657.94</v>
+        <v>6645.12</v>
       </c>
       <c r="W6" s="137" t="n">
-        <v>174.069032258064</v>
+        <v>-451.6541935483865</v>
       </c>
       <c r="X6" s="138" t="n">
-        <v>0.0317419999999999</v>
+        <v>-0.0636421818181817</v>
       </c>
       <c r="Y6" s="137" t="n"/>
       <c r="Z6" s="137" t="n"/>
@@ -3511,7 +3513,7 @@
       <c r="AD6" s="139" t="inlineStr"/>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -3527,13 +3529,13 @@
         </is>
       </c>
       <c r="B7" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C7" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D7" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -3580,28 +3582,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>360.7809847198643</v>
+        <v>466.8930390492361</v>
       </c>
       <c r="R7" t="n">
-        <v>360</v>
+        <v>371</v>
       </c>
       <c r="S7" t="n">
-        <v>-0.7809847198642501</v>
+        <v>-95.89303904923604</v>
       </c>
       <c r="T7" s="137" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="U7" s="137" t="n">
-        <v>2826.086956521739</v>
+        <v>3478.260869565217</v>
       </c>
       <c r="V7" s="137" t="n">
-        <v>2736</v>
+        <v>2819.6</v>
       </c>
       <c r="W7" s="137" t="n">
-        <v>-90.086956521739</v>
+        <v>-658.6608695652176</v>
       </c>
       <c r="X7" s="138" t="n">
-        <v>-0.031876923076923</v>
+        <v>-0.189365</v>
       </c>
       <c r="Y7" s="137" t="n">
         <v>7.6</v>
@@ -3614,7 +3616,7 @@
       <c r="AD7" s="139" t="inlineStr"/>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -3630,13 +3632,13 @@
         </is>
       </c>
       <c r="B8" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C8" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D8" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E8" t="n">
         <v>26</v>
@@ -3683,28 +3685,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>243.7275985663082</v>
+        <v>315.4121863799283</v>
       </c>
       <c r="R8" t="n">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="S8" t="n">
-        <v>-68.72759856630825</v>
+        <v>-128.4121863799283</v>
       </c>
       <c r="T8" s="137" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="U8" s="137" t="n">
-        <v>2260.869565217391</v>
+        <v>2782.608695652174</v>
       </c>
       <c r="V8" s="137" t="n">
-        <v>1575</v>
+        <v>1683</v>
       </c>
       <c r="W8" s="137" t="n">
-        <v>-685.8695652173915</v>
+        <v>-1099.608695652174</v>
       </c>
       <c r="X8" s="138" t="n">
-        <v>-0.3033653846153846</v>
+        <v>-0.395171875</v>
       </c>
       <c r="Y8" s="137" t="n">
         <v>9</v>
@@ -3717,7 +3719,7 @@
       <c r="AD8" s="139" t="inlineStr"/>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -3733,13 +3735,13 @@
         </is>
       </c>
       <c r="B9" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C9" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D9" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3786,28 +3788,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>137.0967741935484</v>
+        <v>177.4193548387097</v>
       </c>
       <c r="R9" t="n">
-        <v>223</v>
+        <v>240</v>
       </c>
       <c r="S9" t="n">
-        <v>85.90322580645162</v>
+        <v>62.58064516129033</v>
       </c>
       <c r="T9" s="137" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="U9" s="137" t="n">
-        <v>1130.434782608696</v>
+        <v>1391.304347826087</v>
       </c>
       <c r="V9" s="137" t="n">
-        <v>1784</v>
+        <v>1920</v>
       </c>
       <c r="W9" s="137" t="n">
-        <v>653.5652173913043</v>
+        <v>528.695652173913</v>
       </c>
       <c r="X9" s="138" t="n">
-        <v>0.578153846153846</v>
+        <v>0.3799999999999999</v>
       </c>
       <c r="Y9" s="137" t="n">
         <v>8</v>
@@ -3820,7 +3822,7 @@
       <c r="AD9" s="139" t="inlineStr"/>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -3836,13 +3838,13 @@
         </is>
       </c>
       <c r="B10" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C10" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D10" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3889,34 +3891,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>64.51612903225806</v>
+        <v>83.49146110056925</v>
       </c>
       <c r="R10" t="n">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="S10" t="n">
-        <v>33.48387096774194</v>
+        <v>27.50853889943074</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U10" s="137" t="n">
-        <v>2193.548387096774</v>
+        <v>2838.709677419354</v>
       </c>
       <c r="V10" s="137" t="n">
-        <v>3069.617174</v>
+        <v>3637.892963</v>
       </c>
       <c r="W10" s="137" t="n">
-        <v>876.0687869032258</v>
+        <v>799.1832855806451</v>
       </c>
       <c r="X10" s="138" t="n">
-        <v>0.3993842999117647</v>
+        <v>0.2815304756022727</v>
       </c>
       <c r="Y10" s="137" t="n">
-        <v>31.3226242244898</v>
+        <v>32.77381047747748</v>
       </c>
       <c r="Z10" s="137" t="n">
-        <v>-2.677375775510203</v>
+        <v>-1.226189522522525</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -3932,7 +3934,7 @@
       <c r="AD10" s="139" t="inlineStr"/>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -3948,13 +3950,13 @@
         </is>
       </c>
       <c r="B11" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C11" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D11" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -4001,34 +4003,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q11" t="n">
-        <v>128.1943862589024</v>
+        <v>165.8986175115207</v>
       </c>
       <c r="R11" t="n">
         <v>61</v>
       </c>
       <c r="S11" t="n">
-        <v>24.80561374109763</v>
+        <v>2.10138248847926</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U11" s="137" t="n">
-        <v>4935.483870967741</v>
+        <v>6387.096774193548</v>
       </c>
       <c r="V11" s="137" t="n">
-        <v>5490.756616000001</v>
+        <v>6906.593127</v>
       </c>
       <c r="W11" s="137" t="n">
-        <v>555.2727450322591</v>
+        <v>519.4963528064518</v>
       </c>
       <c r="X11" s="138" t="n">
-        <v>0.1125062424575165</v>
+        <v>0.0813352875606061</v>
       </c>
       <c r="Y11" s="137" t="n">
-        <v>35.88729814379085</v>
+        <v>41.110673375</v>
       </c>
       <c r="Z11" s="137" t="n">
-        <v>-2.612701856209149</v>
+        <v>2.610673374999997</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -4044,7 +4046,7 @@
       <c r="AD11" s="139" t="inlineStr"/>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_10;crm_metrics_combined_with_excel_row_10</t>
+          <t>google:ok;google:includes_excel_row_10;crm_metrics_combined_with_excel_row_10;crm:stale</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -4060,13 +4062,13 @@
         </is>
       </c>
       <c r="B12" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C12" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D12" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -4096,7 +4098,7 @@
       <c r="L12" s="137" t="n"/>
       <c r="N12" s="137" t="n"/>
       <c r="R12" t="n">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="T12" s="137" t="n"/>
       <c r="U12" s="137" t="n"/>
@@ -4114,7 +4116,7 @@
       <c r="AD12" s="139" t="inlineStr"/>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_9</t>
+          <t>google:rolled_up_to_excel_row_9;crm:stale</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -4130,13 +4132,13 @@
         </is>
       </c>
       <c r="B13" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C13" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D13" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4183,34 +4185,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>14.43123938879457</v>
+        <v>18.67572156196944</v>
       </c>
       <c r="R13" t="n">
         <v>5</v>
       </c>
       <c r="S13" t="n">
-        <v>-5.431239388794566</v>
+        <v>-8.675721561969439</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="137" t="n">
-        <v>548.3870967741935</v>
+        <v>709.6774193548387</v>
       </c>
       <c r="V13" s="137" t="n">
-        <v>510.988722</v>
+        <v>702.1896790000001</v>
       </c>
       <c r="W13" s="137" t="n">
-        <v>-37.39837477419354</v>
+        <v>-7.487740354838593</v>
       </c>
       <c r="X13" s="138" t="n">
-        <v>-0.0681970363529411</v>
+        <v>-0.0105509068636362</v>
       </c>
       <c r="Y13" s="137" t="n">
-        <v>56.77652466666667</v>
+        <v>70.21896790000001</v>
       </c>
       <c r="Z13" s="137" t="n">
-        <v>18.77652466666667</v>
+        <v>32.21896790000001</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -4226,7 +4228,7 @@
       <c r="AD13" s="139" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_12;crm_metrics_combined_with_excel_row_12</t>
+          <t>google:ok;google:includes_excel_row_12;crm_metrics_combined_with_excel_row_12;crm:stale</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -4242,13 +4244,13 @@
         </is>
       </c>
       <c r="B14" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C14" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D14" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
@@ -4278,7 +4280,7 @@
       <c r="L14" s="137" t="n"/>
       <c r="N14" s="137" t="n"/>
       <c r="R14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T14" s="137" t="n"/>
       <c r="U14" s="137" t="n"/>
@@ -4296,7 +4298,7 @@
       <c r="AD14" s="139" t="inlineStr"/>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_11</t>
+          <t>google:rolled_up_to_excel_row_11;crm:stale</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -4312,13 +4314,13 @@
         </is>
       </c>
       <c r="B15" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C15" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D15" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -4365,34 +4367,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q15" t="n">
-        <v>2.193548387096774</v>
+        <v>2.838709677419355</v>
       </c>
       <c r="R15" t="n">
         <v>2</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.193548387096774</v>
+        <v>-0.838709677419355</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U15" s="137" t="n">
-        <v>548.3870967741935</v>
+        <v>709.6774193548387</v>
       </c>
       <c r="V15" s="137" t="n">
-        <v>630.160373</v>
+        <v>748.7606519999999</v>
       </c>
       <c r="W15" s="137" t="n">
-        <v>81.77327622580651</v>
+        <v>39.08323264516128</v>
       </c>
       <c r="X15" s="138" t="n">
-        <v>0.1491159742941177</v>
+        <v>0.0550718278181818</v>
       </c>
       <c r="Y15" s="137" t="n">
-        <v>315.0801865</v>
+        <v>374.380326</v>
       </c>
       <c r="Z15" s="137" t="n">
-        <v>65.08018650000002</v>
+        <v>124.380326</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -4408,7 +4410,7 @@
       <c r="AD15" s="139" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_14;crm_metrics_combined_with_excel_row_14</t>
+          <t>google:ok;google:includes_excel_row_14;crm_metrics_combined_with_excel_row_14;crm:stale</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -4424,13 +4426,13 @@
         </is>
       </c>
       <c r="B16" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C16" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D16" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4478,7 +4480,7 @@
       <c r="AD16" s="139" t="inlineStr"/>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_13</t>
+          <t>google:rolled_up_to_excel_row_13;crm:stale</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -4494,13 +4496,13 @@
         </is>
       </c>
       <c r="B17" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C17" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D17" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E17" t="n">
         <v>17</v>
@@ -4547,34 +4549,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>428.4274193548387</v>
+        <v>554.4354838709678</v>
       </c>
       <c r="R17" t="n">
-        <v>367</v>
+        <v>417</v>
       </c>
       <c r="S17" t="n">
-        <v>-61.42741935483872</v>
+        <v>-137.4354838709678</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U17" s="137" t="n">
-        <v>5483.870967741936</v>
+        <v>7096.774193548386</v>
       </c>
       <c r="V17" s="137" t="n">
-        <v>7444.1</v>
+        <v>9676.860000000001</v>
       </c>
       <c r="W17" s="137" t="n">
-        <v>1960.229032258065</v>
+        <v>2580.085806451614</v>
       </c>
       <c r="X17" s="138" t="n">
-        <v>0.3574535294117647</v>
+        <v>0.3635575454545456</v>
       </c>
       <c r="Y17" s="137" t="n">
-        <v>20.28365122615804</v>
+        <v>23.20589928057554</v>
       </c>
       <c r="Z17" s="137" t="n">
-        <v>7.483651226158038</v>
+        <v>10.40589928057554</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -4590,7 +4592,7 @@
       <c r="AD17" s="139" t="inlineStr"/>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
@@ -4606,13 +4608,13 @@
         </is>
       </c>
       <c r="B18" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C18" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D18" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4659,34 +4661,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>6.854838709677419</v>
+        <v>8.870967741935484</v>
       </c>
       <c r="R18" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S18" t="n">
-        <v>24.14516129032258</v>
+        <v>23.12903225806452</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="137" t="n">
-        <v>274.1935483870968</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="V18" s="137" t="n">
-        <v>322.95</v>
+        <v>376.46</v>
       </c>
       <c r="W18" s="137" t="n">
-        <v>48.75645161290322</v>
+        <v>21.62129032258065</v>
       </c>
       <c r="X18" s="138" t="n">
-        <v>0.1778176470588235</v>
+        <v>0.0609327272727272</v>
       </c>
       <c r="Y18" s="137" t="n">
-        <v>10.41774193548387</v>
+        <v>11.764375</v>
       </c>
       <c r="Z18" s="137" t="n">
-        <v>-29.58225806451613</v>
+        <v>-28.235625</v>
       </c>
       <c r="AB18" s="139" t="inlineStr"/>
       <c r="AC18" s="139" t="inlineStr">
@@ -4697,7 +4699,7 @@
       <c r="AD18" s="139" t="inlineStr"/>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
@@ -4713,13 +4715,13 @@
         </is>
       </c>
       <c r="B19" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C19" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D19" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4766,34 +4768,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>6.093189964157706</v>
+        <v>7.885304659498208</v>
       </c>
       <c r="R19" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="S19" t="n">
-        <v>10.9068100358423</v>
+        <v>11.11469534050179</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="137" t="n">
-        <v>548.3870967741935</v>
+        <v>709.6774193548387</v>
       </c>
       <c r="V19" s="137" t="n">
-        <v>581.76</v>
+        <v>679.27</v>
       </c>
       <c r="W19" s="137" t="n">
-        <v>33.37290322580645</v>
+        <v>-30.40741935483868</v>
       </c>
       <c r="X19" s="138" t="n">
-        <v>0.0608564705882353</v>
+        <v>-0.0428468181818181</v>
       </c>
       <c r="Y19" s="137" t="n">
-        <v>34.22117647058823</v>
+        <v>35.75105263157894</v>
       </c>
       <c r="Z19" s="137" t="n">
-        <v>-55.77882352941177</v>
+        <v>-54.24894736842106</v>
       </c>
       <c r="AB19" s="139" t="inlineStr"/>
       <c r="AC19" s="139" t="inlineStr">
@@ -4804,7 +4806,7 @@
       <c r="AD19" s="139" t="inlineStr"/>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
@@ -4820,13 +4822,13 @@
         </is>
       </c>
       <c r="B20" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C20" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D20" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
@@ -4873,34 +4875,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>2.28494623655914</v>
+        <v>2.956989247311828</v>
       </c>
       <c r="R20" t="n">
         <v>4</v>
       </c>
       <c r="S20" t="n">
-        <v>1.71505376344086</v>
+        <v>1.043010752688172</v>
       </c>
       <c r="T20" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U20" s="137" t="n">
-        <v>274.1935483870968</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="V20" s="137" t="n">
-        <v>283.27</v>
+        <v>335.9</v>
       </c>
       <c r="W20" s="137" t="n">
-        <v>9.076451612903211</v>
+        <v>-18.93870967741936</v>
       </c>
       <c r="X20" s="138" t="n">
-        <v>0.0331023529411764</v>
+        <v>-0.0533727272727272</v>
       </c>
       <c r="Y20" s="137" t="n">
-        <v>70.8175</v>
+        <v>83.97499999999999</v>
       </c>
       <c r="Z20" s="137" t="n">
-        <v>-49.1825</v>
+        <v>-36.02500000000001</v>
       </c>
       <c r="AB20" s="139" t="inlineStr"/>
       <c r="AC20" s="139" t="inlineStr">
@@ -4911,7 +4913,7 @@
       <c r="AD20" s="139" t="inlineStr"/>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr">
@@ -4927,13 +4929,13 @@
         </is>
       </c>
       <c r="B21" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C21" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D21" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4980,34 +4982,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>20.56451612903226</v>
+        <v>26.61290322580645</v>
       </c>
       <c r="R21" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S21" t="n">
-        <v>0.4354838709677402</v>
+        <v>-4.612903225806452</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="137" t="n">
-        <v>822.5806451612904</v>
+        <v>1064.516129032258</v>
       </c>
       <c r="V21" s="137" t="n">
-        <v>1057.013242</v>
+        <v>1277.522538</v>
       </c>
       <c r="W21" s="137" t="n">
-        <v>234.4325968387096</v>
+        <v>213.0064089677419</v>
       </c>
       <c r="X21" s="138" t="n">
-        <v>0.2849964902745097</v>
+        <v>0.2000969296363636</v>
       </c>
       <c r="Y21" s="137" t="n">
-        <v>50.3339639047619</v>
+        <v>58.06920627272727</v>
       </c>
       <c r="Z21" s="137" t="n">
-        <v>10.3339639047619</v>
+        <v>18.06920627272727</v>
       </c>
       <c r="AB21" s="139" t="inlineStr">
         <is>
@@ -5018,7 +5020,7 @@
       <c r="AD21" s="139" t="inlineStr"/>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
@@ -5034,13 +5036,13 @@
         </is>
       </c>
       <c r="B22" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C22" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D22" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -5087,34 +5089,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>54.83870967741935</v>
+        <v>70.96774193548387</v>
       </c>
       <c r="R22" t="n">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="S22" t="n">
-        <v>47.16129032258065</v>
+        <v>43.03225806451613</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="137" t="n">
-        <v>822.5806451612904</v>
+        <v>1064.516129032258</v>
       </c>
       <c r="V22" s="137" t="n">
-        <v>1241.033961</v>
+        <v>1551.287959</v>
       </c>
       <c r="W22" s="137" t="n">
-        <v>418.4533158387097</v>
+        <v>486.771829967742</v>
       </c>
       <c r="X22" s="138" t="n">
-        <v>0.5087079525882353</v>
+        <v>0.457270506939394</v>
       </c>
       <c r="Y22" s="137" t="n">
-        <v>12.16699961764706</v>
+        <v>13.60778911403509</v>
       </c>
       <c r="Z22" s="137" t="n">
-        <v>-2.833000382352941</v>
+        <v>-1.392210885964912</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -5130,7 +5132,7 @@
       <c r="AD22" s="139" t="inlineStr"/>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
@@ -5146,13 +5148,13 @@
         </is>
       </c>
       <c r="B23" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C23" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D23" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5199,34 +5201,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>21.09181141439206</v>
+        <v>27.29528535980149</v>
       </c>
       <c r="R23" t="n">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="S23" t="n">
-        <v>37.90818858560795</v>
+        <v>39.70471464019852</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="137" t="n">
-        <v>548.3870967741935</v>
+        <v>709.6774193548387</v>
       </c>
       <c r="V23" s="137" t="n">
-        <v>1016.68</v>
+        <v>1173.01</v>
       </c>
       <c r="W23" s="137" t="n">
-        <v>468.2929032258064</v>
+        <v>463.3325806451613</v>
       </c>
       <c r="X23" s="138" t="n">
-        <v>0.8539458823529411</v>
+        <v>0.6528777272727274</v>
       </c>
       <c r="Y23" s="137" t="n">
-        <v>17.23186440677966</v>
+        <v>17.50761194029851</v>
       </c>
       <c r="Z23" s="137" t="n">
-        <v>-8.76813559322034</v>
+        <v>-8.492388059701494</v>
       </c>
       <c r="AB23" s="139" t="inlineStr"/>
       <c r="AC23" s="139" t="inlineStr">
@@ -5237,7 +5239,7 @@
       <c r="AD23" s="139" t="inlineStr"/>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -5253,13 +5255,13 @@
         </is>
       </c>
       <c r="B24" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C24" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D24" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5291,16 +5293,18 @@
       <c r="L24" s="137" t="n"/>
       <c r="N24" s="137" t="n"/>
       <c r="R24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T24" s="137" t="n"/>
       <c r="U24" s="137" t="n"/>
       <c r="V24" s="137" t="n">
-        <v>144.47</v>
+        <v>466.69</v>
       </c>
       <c r="W24" s="137" t="n"/>
       <c r="X24" s="138" t="n"/>
-      <c r="Y24" s="137" t="n"/>
+      <c r="Y24" s="137" t="n">
+        <v>466.69</v>
+      </c>
       <c r="Z24" s="137" t="n"/>
       <c r="AB24" s="139" t="inlineStr"/>
       <c r="AC24" s="139" t="inlineStr">
@@ -5311,7 +5315,7 @@
       <c r="AD24" s="139" t="inlineStr"/>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
@@ -5327,13 +5331,13 @@
         </is>
       </c>
       <c r="B25" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C25" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D25" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5362,41 +5366,41 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>255.9139784946237</v>
+        <v>331.1827956989247</v>
       </c>
       <c r="R25" t="n">
-        <v>291</v>
+        <v>328</v>
       </c>
       <c r="S25" t="n">
-        <v>35.08602150537632</v>
+        <v>-3.182795698924735</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="137" t="n">
-        <v>11516.12903225806</v>
+        <v>14903.22580645161</v>
       </c>
       <c r="V25" s="137" t="n">
-        <v>12526.432246</v>
+        <v>15096.685541</v>
       </c>
       <c r="W25" s="137" t="n">
-        <v>1010.303213741934</v>
+        <v>193.4597345483889</v>
       </c>
       <c r="X25" s="138" t="n">
-        <v>0.0877294107170867</v>
+        <v>0.012981064439394</v>
       </c>
       <c r="Y25" s="137" t="n">
-        <v>43.04615892096219</v>
+        <v>46.02648030792683</v>
       </c>
       <c r="Z25" s="137" t="n">
-        <v>-1.953841079037808</v>
+        <v>1.026480307926832</v>
       </c>
       <c r="AB25" s="139" t="inlineStr"/>
       <c r="AC25" s="139" t="inlineStr"/>
       <c r="AD25" s="139" t="inlineStr"/>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5407,13 +5411,13 @@
         </is>
       </c>
       <c r="B26" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C26" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D26" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5447,41 +5451,41 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>749.4907345531284</v>
+        <v>969.929185892284</v>
       </c>
       <c r="R26" t="n">
-        <v>863</v>
+        <v>967</v>
       </c>
       <c r="S26" t="n">
-        <v>113.5092654468716</v>
+        <v>-2.929185892283954</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="137" t="n">
-        <v>17000</v>
+        <v>22000</v>
       </c>
       <c r="V26" s="137" t="n">
-        <v>21792.800088</v>
+        <v>27532.436918</v>
       </c>
       <c r="W26" s="137" t="n">
-        <v>4792.800088</v>
+        <v>5532.436917999999</v>
       </c>
       <c r="X26" s="138" t="n">
-        <v>0.2819294169411764</v>
+        <v>0.2514744053636363</v>
       </c>
       <c r="Y26" s="137" t="n">
-        <v>25.25237553650058</v>
+        <v>28.47201335884177</v>
       </c>
       <c r="Z26" s="137" t="n">
-        <v>2.570307278330624</v>
+        <v>5.789945100671822</v>
       </c>
       <c r="AB26" s="139" t="inlineStr"/>
       <c r="AC26" s="139" t="inlineStr"/>
       <c r="AD26" s="139" t="inlineStr"/>
       <c r="AE26" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5492,13 +5496,13 @@
         </is>
       </c>
       <c r="B27" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C27" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D27" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5532,41 +5536,41 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>741.6053574797209</v>
+        <v>959.724580267874</v>
       </c>
       <c r="R27" t="n">
-        <v>758</v>
+        <v>798</v>
       </c>
       <c r="S27" t="n">
-        <v>16.39464252027915</v>
+        <v>-161.724580267874</v>
       </c>
       <c r="T27" s="137" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="U27" s="137" t="n">
-        <v>6217.391304347826</v>
+        <v>7652.173913043478</v>
       </c>
       <c r="V27" s="137" t="n">
-        <v>6095</v>
+        <v>6422.6</v>
       </c>
       <c r="W27" s="137" t="n">
-        <v>-122.391304347826</v>
+        <v>-1229.573913043478</v>
       </c>
       <c r="X27" s="138" t="n">
-        <v>-0.0196853146853146</v>
+        <v>-0.1606829545454544</v>
       </c>
       <c r="Y27" s="137" t="n">
-        <v>8.040897097625329</v>
+        <v>8.048370927318297</v>
       </c>
       <c r="Z27" s="137" t="n">
-        <v>-0.0931569564287251</v>
+        <v>-0.0856831267357574</v>
       </c>
       <c r="AB27" s="139" t="inlineStr"/>
       <c r="AC27" s="139" t="inlineStr"/>
       <c r="AD27" s="139" t="inlineStr"/>
       <c r="AE27" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>success;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5577,13 +5581,13 @@
         </is>
       </c>
       <c r="B28" s="136" t="n">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C28" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D28" s="136" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5617,41 +5621,41 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>1747.010070527473</v>
+        <v>2260.836561859083</v>
       </c>
       <c r="R28" t="n">
-        <v>1912</v>
+        <v>2093</v>
       </c>
       <c r="S28" t="n">
-        <v>164.9899294725271</v>
+        <v>-167.8365618590828</v>
       </c>
       <c r="T28" s="137" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="U28" s="137" t="n">
-        <v>34733.52033660589</v>
+        <v>44555.39971949509</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>40414.232334</v>
+        <v>49051.722459</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>5680.711997394108</v>
+        <v>4496.322739504911</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>0.1635512882754693</v>
+        <v>0.1009153271615147</v>
       </c>
       <c r="Y28" s="137" t="n">
-        <v>21.13715080230126</v>
+        <v>23.43608335355948</v>
       </c>
       <c r="Z28" s="137" t="n">
-        <v>1.361427880255917</v>
+        <v>3.660360431514143</v>
       </c>
       <c r="AB28" s="139" t="inlineStr"/>
       <c r="AC28" s="139" t="inlineStr"/>
       <c r="AD28" s="139" t="inlineStr"/>
       <c r="AE28" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5747,7 +5751,7 @@
         </is>
       </c>
       <c r="B4" s="140" t="n">
-        <v>46220</v>
+        <v>46225</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5787,7 +5791,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5807,7 +5811,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46225.5041550926</v>
+        <v>46226.29195601852</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-07-24
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 22/07/2026  |  Ultimo aggiornamento: 23/07/2026 07:00</t>
+          <t>Periodo: 01/07/2026 - 23/07/2026  |  Ultimo aggiornamento: 24/07/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1065,16 +1065,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>6741.935483870968</v>
+        <v>7048.387096774193</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>7194.217537</v>
+        <v>7475.593311999999</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>452.2820531290327</v>
+        <v>427.2062152258059</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.06708489783253591</v>
+        <v>0.0606104927780319</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1173,16 +1173,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>1064.516129032258</v>
+        <v>1112.903225806452</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>1257.348004</v>
+        <v>1281.92283</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>192.8318749677419</v>
+        <v>169.0196041935483</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>0.1811450946666666</v>
+        <v>0.1518726878260868</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1281,16 +1281,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>7096.774193548386</v>
+        <v>7419.354838709677</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>6645.12</v>
+        <v>6749.32</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-451.6541935483865</v>
+        <v>-670.0348387096774</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.0636421818181817</v>
+        <v>-0.0903090434782608</v>
       </c>
       <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
@@ -1328,34 +1328,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>331.1827956989247</v>
+        <v>346.236559139785</v>
       </c>
       <c r="N10" s="125" t="n">
         <v>328</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>-3.182795698924735</v>
+        <v>-18.23655913978496</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>14903.22580645161</v>
+        <v>15580.64516129032</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>15096.685541</v>
+        <v>15506.836142</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>193.4597345483889</v>
+        <v>-73.8090192903237</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>0.012981064439394</v>
+        <v>-0.0047372248405797</v>
       </c>
       <c r="U10" s="123" t="n">
-        <v>46.02648030792683</v>
+        <v>47.27693945731707</v>
       </c>
       <c r="V10" s="123" t="n">
-        <v>1.026480307926832</v>
+        <v>2.27693945731707</v>
       </c>
       <c r="W10" s="126" t="n"/>
     </row>
@@ -1407,34 +1407,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>83.49146110056925</v>
+        <v>87.28652751423149</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>111</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>27.50853889943074</v>
+        <v>23.71347248576851</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>2838.709677419354</v>
+        <v>2967.741935483871</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>3637.892963</v>
+        <v>3718.643776</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>799.1832855806451</v>
+        <v>750.9018405161291</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.2815304756022727</v>
+        <v>0.2530212723478261</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>32.77381047747748</v>
+        <v>33.50129527927928</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>-1.226189522522525</v>
+        <v>-0.498704720720724</v>
       </c>
       <c r="W11" s="120" t="inlineStr">
         <is>
@@ -1490,34 +1490,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M12" s="127" t="n">
-        <v>165.8986175115207</v>
+        <v>173.4394637620444</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>61</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>2.10138248847926</v>
+        <v>-5.439463762044397</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>6387.096774193548</v>
+        <v>6677.419354838709</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>6906.593127</v>
+        <v>7130.470476</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>519.4963528064518</v>
+        <v>453.0511211612911</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>0.0813352875606061</v>
+        <v>0.067848235536232</v>
       </c>
       <c r="U12" s="128" t="n">
-        <v>41.110673375</v>
+        <v>42.44327664285714</v>
       </c>
       <c r="V12" s="128" t="n">
-        <v>2.610673374999997</v>
+        <v>3.943276642857143</v>
       </c>
       <c r="W12" s="120" t="inlineStr">
         <is>
@@ -1620,34 +1620,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="127" t="n">
-        <v>18.67572156196944</v>
+        <v>19.52461799660441</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>5</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-8.675721561969439</v>
+        <v>-9.524617996604412</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>709.6774193548387</v>
+        <v>741.9354838709677</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>702.1896790000001</v>
+        <v>732.8096790000001</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-7.487740354838593</v>
+        <v>-9.125804870967611</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.0105509068636362</v>
+        <v>-0.012299997869565</v>
       </c>
       <c r="U14" s="128" t="n">
-        <v>70.21896790000001</v>
+        <v>73.28096790000001</v>
       </c>
       <c r="V14" s="128" t="n">
-        <v>32.21896790000001</v>
+        <v>35.28096790000001</v>
       </c>
       <c r="W14" s="120" t="inlineStr">
         <is>
@@ -1750,34 +1750,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M16" s="127" t="n">
-        <v>2.838709677419355</v>
+        <v>2.967741935483871</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>-0.838709677419355</v>
+        <v>-0.967741935483871</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>709.6774193548387</v>
+        <v>741.9354838709677</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>748.7606519999999</v>
+        <v>778.320652</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>39.08323264516128</v>
+        <v>36.38516812903231</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.0550718278181818</v>
+        <v>0.0490408787826087</v>
       </c>
       <c r="U16" s="128" t="n">
-        <v>374.380326</v>
+        <v>389.160326</v>
       </c>
       <c r="V16" s="128" t="n">
-        <v>124.380326</v>
+        <v>139.160326</v>
       </c>
       <c r="W16" s="120" t="inlineStr">
         <is>
@@ -1880,34 +1880,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>554.4354838709678</v>
+        <v>579.6370967741935</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>417</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-137.4354838709678</v>
+        <v>-162.6370967741935</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>7096.774193548386</v>
+        <v>7419.354838709677</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>9676.860000000001</v>
+        <v>10090.15</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>2580.085806451614</v>
+        <v>2670.795161290323</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>0.3635575454545456</v>
+        <v>0.3599767391304348</v>
       </c>
       <c r="U18" s="117" t="n">
-        <v>23.20589928057554</v>
+        <v>24.19700239808153</v>
       </c>
       <c r="V18" s="117" t="n">
-        <v>10.40589928057554</v>
+        <v>11.39700239808153</v>
       </c>
       <c r="W18" s="120" t="inlineStr">
         <is>
@@ -1963,34 +1963,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>8.870967741935484</v>
+        <v>9.274193548387096</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>32</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>23.12903225806452</v>
+        <v>22.7258064516129</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>354.8387096774193</v>
+        <v>370.9677419354838</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>376.46</v>
+        <v>384.99</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>21.62129032258065</v>
+        <v>14.02225806451617</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>0.0609327272727272</v>
+        <v>0.0377991304347827</v>
       </c>
       <c r="U19" s="117" t="n">
-        <v>11.764375</v>
+        <v>12.0309375</v>
       </c>
       <c r="V19" s="117" t="n">
-        <v>-28.235625</v>
+        <v>-27.9690625</v>
       </c>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
@@ -2042,34 +2042,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>7.885304659498208</v>
+        <v>8.243727598566307</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>11.11469534050179</v>
+        <v>10.75627240143369</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>709.6774193548387</v>
+        <v>741.9354838709677</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>679.27</v>
+        <v>697.0700000000001</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-30.40741935483868</v>
+        <v>-44.86548387096764</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.0428468181818181</v>
+        <v>-0.0604708695652172</v>
       </c>
       <c r="U20" s="117" t="n">
-        <v>35.75105263157894</v>
+        <v>36.68789473684211</v>
       </c>
       <c r="V20" s="117" t="n">
-        <v>-54.24894736842106</v>
+        <v>-53.31210526315789</v>
       </c>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
@@ -2121,34 +2121,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>2.956989247311828</v>
+        <v>3.091397849462366</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>4</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>1.043010752688172</v>
+        <v>0.908602150537634</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>354.8387096774193</v>
+        <v>370.9677419354838</v>
       </c>
       <c r="R21" s="117" t="n">
-        <v>335.9</v>
+        <v>344.39</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-18.93870967741936</v>
+        <v>-26.57774193548386</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.0533727272727272</v>
+        <v>-0.0716443478260869</v>
       </c>
       <c r="U21" s="117" t="n">
-        <v>83.97499999999999</v>
+        <v>86.0975</v>
       </c>
       <c r="V21" s="117" t="n">
-        <v>-36.02500000000001</v>
+        <v>-33.9025</v>
       </c>
       <c r="W21" s="120" t="inlineStr"/>
     </row>
@@ -2200,34 +2200,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>26.61290322580645</v>
+        <v>27.82258064516129</v>
       </c>
       <c r="N22" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-4.612903225806452</v>
+        <v>-5.822580645161292</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>1064.516129032258</v>
+        <v>1112.903225806452</v>
       </c>
       <c r="R22" s="117" t="n">
-        <v>1277.522538</v>
+        <v>1312.096658</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>213.0064089677419</v>
+        <v>199.1934321935482</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>0.2000969296363636</v>
+        <v>0.1789854028405795</v>
       </c>
       <c r="U22" s="117" t="n">
-        <v>58.06920627272727</v>
+        <v>59.64075718181818</v>
       </c>
       <c r="V22" s="117" t="n">
-        <v>18.06920627272727</v>
+        <v>19.64075718181818</v>
       </c>
       <c r="W22" s="120" t="inlineStr"/>
     </row>
@@ -2279,34 +2279,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>70.96774193548387</v>
+        <v>74.19354838709677</v>
       </c>
       <c r="N23" s="119" t="n">
         <v>114</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>43.03225806451613</v>
+        <v>39.80645161290323</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>1064.516129032258</v>
+        <v>1112.903225806452</v>
       </c>
       <c r="R23" s="117" t="n">
-        <v>1551.287959</v>
+        <v>1637.830756</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>486.771829967742</v>
+        <v>524.9275301935484</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.457270506939394</v>
+        <v>0.4716740126376811</v>
       </c>
       <c r="U23" s="117" t="n">
-        <v>13.60778911403509</v>
+        <v>14.36693645614035</v>
       </c>
       <c r="V23" s="117" t="n">
-        <v>-1.392210885964912</v>
+        <v>-0.6330635438596488</v>
       </c>
       <c r="W23" s="120" t="inlineStr">
         <is>
@@ -2362,34 +2362,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>27.29528535980149</v>
+        <v>28.53598014888337</v>
       </c>
       <c r="N24" s="119" t="n">
         <v>67</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>39.70471464019852</v>
+        <v>38.46401985111663</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>709.6774193548387</v>
+        <v>741.9354838709677</v>
       </c>
       <c r="R24" s="117" t="n">
-        <v>1173.01</v>
+        <v>1195.66</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>463.3325806451613</v>
+        <v>453.7245161290324</v>
       </c>
       <c r="T24" s="118" t="n">
-        <v>0.6528777272727274</v>
+        <v>0.611541739130435</v>
       </c>
       <c r="U24" s="117" t="n">
-        <v>17.50761194029851</v>
+        <v>17.84567164179105</v>
       </c>
       <c r="V24" s="117" t="n">
-        <v>-8.492388059701494</v>
+        <v>-8.154328358208954</v>
       </c>
       <c r="W24" s="120" t="inlineStr"/>
     </row>
@@ -2436,12 +2436,12 @@
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>466.69</v>
+        <v>510.42</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
       <c r="U25" s="117" t="n">
-        <v>466.69</v>
+        <v>510.42</v>
       </c>
       <c r="V25" s="117" t="n"/>
       <c r="W25" s="120" t="inlineStr"/>
@@ -2478,34 +2478,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>969.929185892284</v>
+        <v>1014.016876160115</v>
       </c>
       <c r="N26" s="125" t="n">
         <v>967</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>-2.929185892283954</v>
+        <v>-47.01687616011486</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>22000</v>
+        <v>23000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>27532.436918</v>
+        <v>28532.851997</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>5532.436917999999</v>
+        <v>5532.851997000002</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>0.2514744053636363</v>
+        <v>0.2405587824782609</v>
       </c>
       <c r="U26" s="123" t="n">
-        <v>28.47201335884177</v>
+        <v>29.50656876628749</v>
       </c>
       <c r="V26" s="123" t="n">
-        <v>5.789945100671822</v>
+        <v>6.824500508117534</v>
       </c>
       <c r="W26" s="126" t="n"/>
     </row>
@@ -2553,28 +2553,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>466.8930390492361</v>
+        <v>488.1154499151104</v>
       </c>
       <c r="N27" s="119" t="n">
         <v>371</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-95.89303904923604</v>
+        <v>-117.1154499151104</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>3478.260869565217</v>
+        <v>3695.652173913044</v>
       </c>
       <c r="R27" s="117" t="n">
         <v>2819.6</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-658.6608695652176</v>
+        <v>-876.0521739130436</v>
       </c>
       <c r="T27" s="118" t="n">
-        <v>-0.189365</v>
+        <v>-0.2370494117647059</v>
       </c>
       <c r="U27" s="117" t="n">
         <v>7.6</v>
@@ -2628,28 +2628,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>315.4121863799283</v>
+        <v>329.7491039426523</v>
       </c>
       <c r="N28" s="119" t="n">
         <v>187</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-128.4121863799283</v>
+        <v>-142.7491039426523</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>2782.608695652174</v>
+        <v>2956.521739130435</v>
       </c>
       <c r="R28" s="117" t="n">
         <v>1683</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-1099.608695652174</v>
+        <v>-1273.521739130435</v>
       </c>
       <c r="T28" s="118" t="n">
-        <v>-0.395171875</v>
+        <v>-0.43075</v>
       </c>
       <c r="U28" s="117" t="n">
         <v>9</v>
@@ -2703,28 +2703,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>177.4193548387097</v>
+        <v>185.4838709677419</v>
       </c>
       <c r="N29" s="119" t="n">
         <v>240</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>62.58064516129033</v>
+        <v>54.51612903225808</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>1391.304347826087</v>
+        <v>1478.260869565217</v>
       </c>
       <c r="R29" s="117" t="n">
         <v>1920</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>528.695652173913</v>
+        <v>441.7391304347825</v>
       </c>
       <c r="T29" s="118" t="n">
-        <v>0.3799999999999999</v>
+        <v>0.2988235294117646</v>
       </c>
       <c r="U29" s="117" t="n">
         <v>8</v>
@@ -2766,28 +2766,28 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>959.724580267874</v>
+        <v>1003.348424825505</v>
       </c>
       <c r="N30" s="125" t="n">
         <v>798</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-161.724580267874</v>
+        <v>-205.3484248255046</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>7652.173913043478</v>
+        <v>8130.434782608696</v>
       </c>
       <c r="R30" s="123" t="n">
         <v>6422.6</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>-1229.573913043478</v>
+        <v>-1707.834782608696</v>
       </c>
       <c r="T30" s="124" t="n">
-        <v>-0.1606829545454544</v>
+        <v>-0.2100545454545454</v>
       </c>
       <c r="U30" s="123" t="n">
         <v>8.048370927318297</v>
@@ -2829,34 +2829,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="133" t="n">
-        <v>2260.836561859083</v>
+        <v>2363.601860125405</v>
       </c>
       <c r="N31" s="133" t="n">
         <v>2093</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>-167.8365618590828</v>
+        <v>-270.6018601254045</v>
       </c>
       <c r="P31" s="131" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="Q31" s="131" t="n">
-        <v>44555.39971949509</v>
+        <v>46711.07994389901</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>49051.722459</v>
+        <v>50462.288139</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>4496.322739504911</v>
+        <v>3751.208195100982</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>0.1009153271615147</v>
+        <v>0.08030660390653049</v>
       </c>
       <c r="U31" s="131" t="n">
-        <v>23.43608335355948</v>
+        <v>24.11002777783086</v>
       </c>
       <c r="V31" s="131" t="n">
-        <v>3.660360431514143</v>
+        <v>4.334304855785522</v>
       </c>
       <c r="W31" s="134" t="n"/>
     </row>
@@ -3137,13 +3137,13 @@
         </is>
       </c>
       <c r="B2" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C2" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D2" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3180,16 +3180,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="137" t="n">
-        <v>6741.935483870968</v>
+        <v>7048.387096774193</v>
       </c>
       <c r="V2" s="137" t="n">
-        <v>7194.217537</v>
+        <v>7475.593311999999</v>
       </c>
       <c r="W2" s="137" t="n">
-        <v>452.2820531290327</v>
+        <v>427.2062152258059</v>
       </c>
       <c r="X2" s="138" t="n">
-        <v>0.06708489783253591</v>
+        <v>0.0606104927780319</v>
       </c>
       <c r="Y2" s="137" t="n"/>
       <c r="Z2" s="137" t="n"/>
@@ -3223,13 +3223,13 @@
         </is>
       </c>
       <c r="B3" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C3" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D3" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3290,13 +3290,13 @@
         </is>
       </c>
       <c r="B4" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C4" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D4" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3333,16 +3333,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="137" t="n">
-        <v>1064.516129032258</v>
+        <v>1112.903225806452</v>
       </c>
       <c r="V4" s="137" t="n">
-        <v>1257.348004</v>
+        <v>1281.92283</v>
       </c>
       <c r="W4" s="137" t="n">
-        <v>192.8318749677419</v>
+        <v>169.0196041935483</v>
       </c>
       <c r="X4" s="138" t="n">
-        <v>0.1811450946666666</v>
+        <v>0.1518726878260868</v>
       </c>
       <c r="Y4" s="137" t="n"/>
       <c r="Z4" s="137" t="n"/>
@@ -3376,13 +3376,13 @@
         </is>
       </c>
       <c r="B5" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C5" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D5" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3443,13 +3443,13 @@
         </is>
       </c>
       <c r="B6" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C6" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D6" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3486,16 +3486,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="137" t="n">
-        <v>7096.774193548386</v>
+        <v>7419.354838709677</v>
       </c>
       <c r="V6" s="137" t="n">
-        <v>6645.12</v>
+        <v>6749.32</v>
       </c>
       <c r="W6" s="137" t="n">
-        <v>-451.6541935483865</v>
+        <v>-670.0348387096774</v>
       </c>
       <c r="X6" s="138" t="n">
-        <v>-0.0636421818181817</v>
+        <v>-0.0903090434782608</v>
       </c>
       <c r="Y6" s="137" t="n"/>
       <c r="Z6" s="137" t="n"/>
@@ -3529,13 +3529,13 @@
         </is>
       </c>
       <c r="B7" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C7" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D7" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -3582,28 +3582,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>466.8930390492361</v>
+        <v>488.1154499151104</v>
       </c>
       <c r="R7" t="n">
         <v>371</v>
       </c>
       <c r="S7" t="n">
-        <v>-95.89303904923604</v>
+        <v>-117.1154499151104</v>
       </c>
       <c r="T7" s="137" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="U7" s="137" t="n">
-        <v>3478.260869565217</v>
+        <v>3695.652173913044</v>
       </c>
       <c r="V7" s="137" t="n">
         <v>2819.6</v>
       </c>
       <c r="W7" s="137" t="n">
-        <v>-658.6608695652176</v>
+        <v>-876.0521739130436</v>
       </c>
       <c r="X7" s="138" t="n">
-        <v>-0.189365</v>
+        <v>-0.2370494117647059</v>
       </c>
       <c r="Y7" s="137" t="n">
         <v>7.6</v>
@@ -3632,13 +3632,13 @@
         </is>
       </c>
       <c r="B8" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C8" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D8" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E8" t="n">
         <v>26</v>
@@ -3685,28 +3685,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>315.4121863799283</v>
+        <v>329.7491039426523</v>
       </c>
       <c r="R8" t="n">
         <v>187</v>
       </c>
       <c r="S8" t="n">
-        <v>-128.4121863799283</v>
+        <v>-142.7491039426523</v>
       </c>
       <c r="T8" s="137" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="U8" s="137" t="n">
-        <v>2782.608695652174</v>
+        <v>2956.521739130435</v>
       </c>
       <c r="V8" s="137" t="n">
         <v>1683</v>
       </c>
       <c r="W8" s="137" t="n">
-        <v>-1099.608695652174</v>
+        <v>-1273.521739130435</v>
       </c>
       <c r="X8" s="138" t="n">
-        <v>-0.395171875</v>
+        <v>-0.43075</v>
       </c>
       <c r="Y8" s="137" t="n">
         <v>9</v>
@@ -3735,13 +3735,13 @@
         </is>
       </c>
       <c r="B9" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C9" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D9" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3788,28 +3788,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>177.4193548387097</v>
+        <v>185.4838709677419</v>
       </c>
       <c r="R9" t="n">
         <v>240</v>
       </c>
       <c r="S9" t="n">
-        <v>62.58064516129033</v>
+        <v>54.51612903225808</v>
       </c>
       <c r="T9" s="137" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="U9" s="137" t="n">
-        <v>1391.304347826087</v>
+        <v>1478.260869565217</v>
       </c>
       <c r="V9" s="137" t="n">
         <v>1920</v>
       </c>
       <c r="W9" s="137" t="n">
-        <v>528.695652173913</v>
+        <v>441.7391304347825</v>
       </c>
       <c r="X9" s="138" t="n">
-        <v>0.3799999999999999</v>
+        <v>0.2988235294117646</v>
       </c>
       <c r="Y9" s="137" t="n">
         <v>8</v>
@@ -3838,13 +3838,13 @@
         </is>
       </c>
       <c r="B10" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C10" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D10" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3891,34 +3891,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>83.49146110056925</v>
+        <v>87.28652751423149</v>
       </c>
       <c r="R10" t="n">
         <v>111</v>
       </c>
       <c r="S10" t="n">
-        <v>27.50853889943074</v>
+        <v>23.71347248576851</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U10" s="137" t="n">
-        <v>2838.709677419354</v>
+        <v>2967.741935483871</v>
       </c>
       <c r="V10" s="137" t="n">
-        <v>3637.892963</v>
+        <v>3718.643776</v>
       </c>
       <c r="W10" s="137" t="n">
-        <v>799.1832855806451</v>
+        <v>750.9018405161291</v>
       </c>
       <c r="X10" s="138" t="n">
-        <v>0.2815304756022727</v>
+        <v>0.2530212723478261</v>
       </c>
       <c r="Y10" s="137" t="n">
-        <v>32.77381047747748</v>
+        <v>33.50129527927928</v>
       </c>
       <c r="Z10" s="137" t="n">
-        <v>-1.226189522522525</v>
+        <v>-0.498704720720724</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -3950,13 +3950,13 @@
         </is>
       </c>
       <c r="B11" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C11" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D11" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -4003,34 +4003,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q11" t="n">
-        <v>165.8986175115207</v>
+        <v>173.4394637620444</v>
       </c>
       <c r="R11" t="n">
         <v>61</v>
       </c>
       <c r="S11" t="n">
-        <v>2.10138248847926</v>
+        <v>-5.439463762044397</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U11" s="137" t="n">
-        <v>6387.096774193548</v>
+        <v>6677.419354838709</v>
       </c>
       <c r="V11" s="137" t="n">
-        <v>6906.593127</v>
+        <v>7130.470476</v>
       </c>
       <c r="W11" s="137" t="n">
-        <v>519.4963528064518</v>
+        <v>453.0511211612911</v>
       </c>
       <c r="X11" s="138" t="n">
-        <v>0.0813352875606061</v>
+        <v>0.067848235536232</v>
       </c>
       <c r="Y11" s="137" t="n">
-        <v>41.110673375</v>
+        <v>42.44327664285714</v>
       </c>
       <c r="Z11" s="137" t="n">
-        <v>2.610673374999997</v>
+        <v>3.943276642857143</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -4062,13 +4062,13 @@
         </is>
       </c>
       <c r="B12" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C12" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D12" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -4132,13 +4132,13 @@
         </is>
       </c>
       <c r="B13" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C13" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D13" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4185,34 +4185,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>18.67572156196944</v>
+        <v>19.52461799660441</v>
       </c>
       <c r="R13" t="n">
         <v>5</v>
       </c>
       <c r="S13" t="n">
-        <v>-8.675721561969439</v>
+        <v>-9.524617996604412</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="137" t="n">
-        <v>709.6774193548387</v>
+        <v>741.9354838709677</v>
       </c>
       <c r="V13" s="137" t="n">
-        <v>702.1896790000001</v>
+        <v>732.8096790000001</v>
       </c>
       <c r="W13" s="137" t="n">
-        <v>-7.487740354838593</v>
+        <v>-9.125804870967611</v>
       </c>
       <c r="X13" s="138" t="n">
-        <v>-0.0105509068636362</v>
+        <v>-0.012299997869565</v>
       </c>
       <c r="Y13" s="137" t="n">
-        <v>70.21896790000001</v>
+        <v>73.28096790000001</v>
       </c>
       <c r="Z13" s="137" t="n">
-        <v>32.21896790000001</v>
+        <v>35.28096790000001</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -4244,13 +4244,13 @@
         </is>
       </c>
       <c r="B14" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C14" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D14" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
@@ -4314,13 +4314,13 @@
         </is>
       </c>
       <c r="B15" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C15" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D15" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -4367,34 +4367,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q15" t="n">
-        <v>2.838709677419355</v>
+        <v>2.967741935483871</v>
       </c>
       <c r="R15" t="n">
         <v>2</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.838709677419355</v>
+        <v>-0.967741935483871</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U15" s="137" t="n">
-        <v>709.6774193548387</v>
+        <v>741.9354838709677</v>
       </c>
       <c r="V15" s="137" t="n">
-        <v>748.7606519999999</v>
+        <v>778.320652</v>
       </c>
       <c r="W15" s="137" t="n">
-        <v>39.08323264516128</v>
+        <v>36.38516812903231</v>
       </c>
       <c r="X15" s="138" t="n">
-        <v>0.0550718278181818</v>
+        <v>0.0490408787826087</v>
       </c>
       <c r="Y15" s="137" t="n">
-        <v>374.380326</v>
+        <v>389.160326</v>
       </c>
       <c r="Z15" s="137" t="n">
-        <v>124.380326</v>
+        <v>139.160326</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -4426,13 +4426,13 @@
         </is>
       </c>
       <c r="B16" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C16" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D16" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4496,13 +4496,13 @@
         </is>
       </c>
       <c r="B17" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C17" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D17" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E17" t="n">
         <v>17</v>
@@ -4549,34 +4549,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>554.4354838709678</v>
+        <v>579.6370967741935</v>
       </c>
       <c r="R17" t="n">
         <v>417</v>
       </c>
       <c r="S17" t="n">
-        <v>-137.4354838709678</v>
+        <v>-162.6370967741935</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U17" s="137" t="n">
-        <v>7096.774193548386</v>
+        <v>7419.354838709677</v>
       </c>
       <c r="V17" s="137" t="n">
-        <v>9676.860000000001</v>
+        <v>10090.15</v>
       </c>
       <c r="W17" s="137" t="n">
-        <v>2580.085806451614</v>
+        <v>2670.795161290323</v>
       </c>
       <c r="X17" s="138" t="n">
-        <v>0.3635575454545456</v>
+        <v>0.3599767391304348</v>
       </c>
       <c r="Y17" s="137" t="n">
-        <v>23.20589928057554</v>
+        <v>24.19700239808153</v>
       </c>
       <c r="Z17" s="137" t="n">
-        <v>10.40589928057554</v>
+        <v>11.39700239808153</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -4608,13 +4608,13 @@
         </is>
       </c>
       <c r="B18" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C18" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D18" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4661,34 +4661,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>8.870967741935484</v>
+        <v>9.274193548387096</v>
       </c>
       <c r="R18" t="n">
         <v>32</v>
       </c>
       <c r="S18" t="n">
-        <v>23.12903225806452</v>
+        <v>22.7258064516129</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="137" t="n">
-        <v>354.8387096774193</v>
+        <v>370.9677419354838</v>
       </c>
       <c r="V18" s="137" t="n">
-        <v>376.46</v>
+        <v>384.99</v>
       </c>
       <c r="W18" s="137" t="n">
-        <v>21.62129032258065</v>
+        <v>14.02225806451617</v>
       </c>
       <c r="X18" s="138" t="n">
-        <v>0.0609327272727272</v>
+        <v>0.0377991304347827</v>
       </c>
       <c r="Y18" s="137" t="n">
-        <v>11.764375</v>
+        <v>12.0309375</v>
       </c>
       <c r="Z18" s="137" t="n">
-        <v>-28.235625</v>
+        <v>-27.9690625</v>
       </c>
       <c r="AB18" s="139" t="inlineStr"/>
       <c r="AC18" s="139" t="inlineStr">
@@ -4715,13 +4715,13 @@
         </is>
       </c>
       <c r="B19" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C19" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D19" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4768,34 +4768,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>7.885304659498208</v>
+        <v>8.243727598566307</v>
       </c>
       <c r="R19" t="n">
         <v>19</v>
       </c>
       <c r="S19" t="n">
-        <v>11.11469534050179</v>
+        <v>10.75627240143369</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="137" t="n">
-        <v>709.6774193548387</v>
+        <v>741.9354838709677</v>
       </c>
       <c r="V19" s="137" t="n">
-        <v>679.27</v>
+        <v>697.0700000000001</v>
       </c>
       <c r="W19" s="137" t="n">
-        <v>-30.40741935483868</v>
+        <v>-44.86548387096764</v>
       </c>
       <c r="X19" s="138" t="n">
-        <v>-0.0428468181818181</v>
+        <v>-0.0604708695652172</v>
       </c>
       <c r="Y19" s="137" t="n">
-        <v>35.75105263157894</v>
+        <v>36.68789473684211</v>
       </c>
       <c r="Z19" s="137" t="n">
-        <v>-54.24894736842106</v>
+        <v>-53.31210526315789</v>
       </c>
       <c r="AB19" s="139" t="inlineStr"/>
       <c r="AC19" s="139" t="inlineStr">
@@ -4822,13 +4822,13 @@
         </is>
       </c>
       <c r="B20" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C20" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D20" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
@@ -4875,34 +4875,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>2.956989247311828</v>
+        <v>3.091397849462366</v>
       </c>
       <c r="R20" t="n">
         <v>4</v>
       </c>
       <c r="S20" t="n">
-        <v>1.043010752688172</v>
+        <v>0.908602150537634</v>
       </c>
       <c r="T20" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U20" s="137" t="n">
-        <v>354.8387096774193</v>
+        <v>370.9677419354838</v>
       </c>
       <c r="V20" s="137" t="n">
-        <v>335.9</v>
+        <v>344.39</v>
       </c>
       <c r="W20" s="137" t="n">
-        <v>-18.93870967741936</v>
+        <v>-26.57774193548386</v>
       </c>
       <c r="X20" s="138" t="n">
-        <v>-0.0533727272727272</v>
+        <v>-0.0716443478260869</v>
       </c>
       <c r="Y20" s="137" t="n">
-        <v>83.97499999999999</v>
+        <v>86.0975</v>
       </c>
       <c r="Z20" s="137" t="n">
-        <v>-36.02500000000001</v>
+        <v>-33.9025</v>
       </c>
       <c r="AB20" s="139" t="inlineStr"/>
       <c r="AC20" s="139" t="inlineStr">
@@ -4929,13 +4929,13 @@
         </is>
       </c>
       <c r="B21" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C21" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D21" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4982,34 +4982,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>26.61290322580645</v>
+        <v>27.82258064516129</v>
       </c>
       <c r="R21" t="n">
         <v>22</v>
       </c>
       <c r="S21" t="n">
-        <v>-4.612903225806452</v>
+        <v>-5.822580645161292</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="137" t="n">
-        <v>1064.516129032258</v>
+        <v>1112.903225806452</v>
       </c>
       <c r="V21" s="137" t="n">
-        <v>1277.522538</v>
+        <v>1312.096658</v>
       </c>
       <c r="W21" s="137" t="n">
-        <v>213.0064089677419</v>
+        <v>199.1934321935482</v>
       </c>
       <c r="X21" s="138" t="n">
-        <v>0.2000969296363636</v>
+        <v>0.1789854028405795</v>
       </c>
       <c r="Y21" s="137" t="n">
-        <v>58.06920627272727</v>
+        <v>59.64075718181818</v>
       </c>
       <c r="Z21" s="137" t="n">
-        <v>18.06920627272727</v>
+        <v>19.64075718181818</v>
       </c>
       <c r="AB21" s="139" t="inlineStr">
         <is>
@@ -5036,13 +5036,13 @@
         </is>
       </c>
       <c r="B22" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C22" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D22" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -5089,34 +5089,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>70.96774193548387</v>
+        <v>74.19354838709677</v>
       </c>
       <c r="R22" t="n">
         <v>114</v>
       </c>
       <c r="S22" t="n">
-        <v>43.03225806451613</v>
+        <v>39.80645161290323</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="137" t="n">
-        <v>1064.516129032258</v>
+        <v>1112.903225806452</v>
       </c>
       <c r="V22" s="137" t="n">
-        <v>1551.287959</v>
+        <v>1637.830756</v>
       </c>
       <c r="W22" s="137" t="n">
-        <v>486.771829967742</v>
+        <v>524.9275301935484</v>
       </c>
       <c r="X22" s="138" t="n">
-        <v>0.457270506939394</v>
+        <v>0.4716740126376811</v>
       </c>
       <c r="Y22" s="137" t="n">
-        <v>13.60778911403509</v>
+        <v>14.36693645614035</v>
       </c>
       <c r="Z22" s="137" t="n">
-        <v>-1.392210885964912</v>
+        <v>-0.6330635438596488</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -5148,13 +5148,13 @@
         </is>
       </c>
       <c r="B23" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C23" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D23" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5201,34 +5201,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>27.29528535980149</v>
+        <v>28.53598014888337</v>
       </c>
       <c r="R23" t="n">
         <v>67</v>
       </c>
       <c r="S23" t="n">
-        <v>39.70471464019852</v>
+        <v>38.46401985111663</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="137" t="n">
-        <v>709.6774193548387</v>
+        <v>741.9354838709677</v>
       </c>
       <c r="V23" s="137" t="n">
-        <v>1173.01</v>
+        <v>1195.66</v>
       </c>
       <c r="W23" s="137" t="n">
-        <v>463.3325806451613</v>
+        <v>453.7245161290324</v>
       </c>
       <c r="X23" s="138" t="n">
-        <v>0.6528777272727274</v>
+        <v>0.611541739130435</v>
       </c>
       <c r="Y23" s="137" t="n">
-        <v>17.50761194029851</v>
+        <v>17.84567164179105</v>
       </c>
       <c r="Z23" s="137" t="n">
-        <v>-8.492388059701494</v>
+        <v>-8.154328358208954</v>
       </c>
       <c r="AB23" s="139" t="inlineStr"/>
       <c r="AC23" s="139" t="inlineStr">
@@ -5255,13 +5255,13 @@
         </is>
       </c>
       <c r="B24" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C24" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D24" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5298,12 +5298,12 @@
       <c r="T24" s="137" t="n"/>
       <c r="U24" s="137" t="n"/>
       <c r="V24" s="137" t="n">
-        <v>466.69</v>
+        <v>510.42</v>
       </c>
       <c r="W24" s="137" t="n"/>
       <c r="X24" s="138" t="n"/>
       <c r="Y24" s="137" t="n">
-        <v>466.69</v>
+        <v>510.42</v>
       </c>
       <c r="Z24" s="137" t="n"/>
       <c r="AB24" s="139" t="inlineStr"/>
@@ -5331,13 +5331,13 @@
         </is>
       </c>
       <c r="B25" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C25" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D25" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5366,34 +5366,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>331.1827956989247</v>
+        <v>346.236559139785</v>
       </c>
       <c r="R25" t="n">
         <v>328</v>
       </c>
       <c r="S25" t="n">
-        <v>-3.182795698924735</v>
+        <v>-18.23655913978496</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="137" t="n">
-        <v>14903.22580645161</v>
+        <v>15580.64516129032</v>
       </c>
       <c r="V25" s="137" t="n">
-        <v>15096.685541</v>
+        <v>15506.836142</v>
       </c>
       <c r="W25" s="137" t="n">
-        <v>193.4597345483889</v>
+        <v>-73.8090192903237</v>
       </c>
       <c r="X25" s="138" t="n">
-        <v>0.012981064439394</v>
+        <v>-0.0047372248405797</v>
       </c>
       <c r="Y25" s="137" t="n">
-        <v>46.02648030792683</v>
+        <v>47.27693945731707</v>
       </c>
       <c r="Z25" s="137" t="n">
-        <v>1.026480307926832</v>
+        <v>2.27693945731707</v>
       </c>
       <c r="AB25" s="139" t="inlineStr"/>
       <c r="AC25" s="139" t="inlineStr"/>
@@ -5411,13 +5411,13 @@
         </is>
       </c>
       <c r="B26" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C26" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D26" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5451,34 +5451,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>969.929185892284</v>
+        <v>1014.016876160115</v>
       </c>
       <c r="R26" t="n">
         <v>967</v>
       </c>
       <c r="S26" t="n">
-        <v>-2.929185892283954</v>
+        <v>-47.01687616011486</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="137" t="n">
-        <v>22000</v>
+        <v>23000</v>
       </c>
       <c r="V26" s="137" t="n">
-        <v>27532.436918</v>
+        <v>28532.851997</v>
       </c>
       <c r="W26" s="137" t="n">
-        <v>5532.436917999999</v>
+        <v>5532.851997000002</v>
       </c>
       <c r="X26" s="138" t="n">
-        <v>0.2514744053636363</v>
+        <v>0.2405587824782609</v>
       </c>
       <c r="Y26" s="137" t="n">
-        <v>28.47201335884177</v>
+        <v>29.50656876628749</v>
       </c>
       <c r="Z26" s="137" t="n">
-        <v>5.789945100671822</v>
+        <v>6.824500508117534</v>
       </c>
       <c r="AB26" s="139" t="inlineStr"/>
       <c r="AC26" s="139" t="inlineStr"/>
@@ -5496,13 +5496,13 @@
         </is>
       </c>
       <c r="B27" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C27" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D27" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5536,28 +5536,28 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>959.724580267874</v>
+        <v>1003.348424825505</v>
       </c>
       <c r="R27" t="n">
         <v>798</v>
       </c>
       <c r="S27" t="n">
-        <v>-161.724580267874</v>
+        <v>-205.3484248255046</v>
       </c>
       <c r="T27" s="137" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="U27" s="137" t="n">
-        <v>7652.173913043478</v>
+        <v>8130.434782608696</v>
       </c>
       <c r="V27" s="137" t="n">
         <v>6422.6</v>
       </c>
       <c r="W27" s="137" t="n">
-        <v>-1229.573913043478</v>
+        <v>-1707.834782608696</v>
       </c>
       <c r="X27" s="138" t="n">
-        <v>-0.1606829545454544</v>
+        <v>-0.2100545454545454</v>
       </c>
       <c r="Y27" s="137" t="n">
         <v>8.048370927318297</v>
@@ -5581,13 +5581,13 @@
         </is>
       </c>
       <c r="B28" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="C28" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D28" s="136" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5621,34 +5621,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>2260.836561859083</v>
+        <v>2363.601860125405</v>
       </c>
       <c r="R28" t="n">
         <v>2093</v>
       </c>
       <c r="S28" t="n">
-        <v>-167.8365618590828</v>
+        <v>-270.6018601254045</v>
       </c>
       <c r="T28" s="137" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="U28" s="137" t="n">
-        <v>44555.39971949509</v>
+        <v>46711.07994389901</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>49051.722459</v>
+        <v>50462.288139</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>4496.322739504911</v>
+        <v>3751.208195100982</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>0.1009153271615147</v>
+        <v>0.08030660390653049</v>
       </c>
       <c r="Y28" s="137" t="n">
-        <v>23.43608335355948</v>
+        <v>24.11002777783086</v>
       </c>
       <c r="Z28" s="137" t="n">
-        <v>3.660360431514143</v>
+        <v>4.334304855785522</v>
       </c>
       <c r="AB28" s="139" t="inlineStr"/>
       <c r="AC28" s="139" t="inlineStr"/>
@@ -5751,7 +5751,7 @@
         </is>
       </c>
       <c r="B4" s="140" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5791,7 +5791,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5811,7 +5811,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46226.29195601852</v>
+        <v>46227.2918287037</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-07-25
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 23/07/2026  |  Ultimo aggiornamento: 24/07/2026 07:00</t>
+          <t>Periodo: 01/07/2026 - 24/07/2026  |  Ultimo aggiornamento: 25/07/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1065,16 +1065,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>7048.387096774193</v>
+        <v>7354.838709677419</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>7475.593311999999</v>
+        <v>7640.583312000001</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>427.2062152258059</v>
+        <v>285.7446023225821</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0606104927780319</v>
+        <v>0.0388512397894738</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1173,16 +1173,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>1112.903225806452</v>
+        <v>1161.290322580645</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>1281.92283</v>
+        <v>1302.88283</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>169.0196041935483</v>
+        <v>141.5925074193547</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>0.1518726878260868</v>
+        <v>0.1219268813888887</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1281,16 +1281,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>7419.354838709677</v>
+        <v>7741.935483870968</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>6749.32</v>
+        <v>6832.92</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-670.0348387096774</v>
+        <v>-909.0154838709676</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.0903090434782608</v>
+        <v>-0.1174144999999999</v>
       </c>
       <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
@@ -1328,34 +1328,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>346.236559139785</v>
+        <v>361.2903225806452</v>
       </c>
       <c r="N10" s="125" t="n">
         <v>328</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>-18.23655913978496</v>
+        <v>-33.29032258064518</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>15580.64516129032</v>
+        <v>16258.06451612903</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>15506.836142</v>
+        <v>15776.386142</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>-73.8090192903237</v>
+        <v>-481.678374129031</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>-0.0047372248405797</v>
+        <v>-0.0296270428531745</v>
       </c>
       <c r="U10" s="123" t="n">
-        <v>47.27693945731707</v>
+        <v>48.09873823780488</v>
       </c>
       <c r="V10" s="123" t="n">
-        <v>2.27693945731707</v>
+        <v>3.098738237804881</v>
       </c>
       <c r="W10" s="126" t="n"/>
     </row>
@@ -1407,34 +1407,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>87.28652751423149</v>
+        <v>91.08159392789372</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>111</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>23.71347248576851</v>
+        <v>19.91840607210627</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>2967.741935483871</v>
+        <v>3096.774193548388</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>3718.643776</v>
+        <v>3799.368604</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>750.9018405161291</v>
+        <v>702.5944104516125</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.2530212723478261</v>
+        <v>0.2268794450416665</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>33.50129527927928</v>
+        <v>34.22854598198198</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>-0.498704720720724</v>
+        <v>0.2285459819819806</v>
       </c>
       <c r="W11" s="120" t="inlineStr">
         <is>
@@ -1490,34 +1490,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M12" s="127" t="n">
-        <v>173.4394637620444</v>
+        <v>180.980310012568</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>61</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>-5.439463762044397</v>
+        <v>-12.98031001256805</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>6677.419354838709</v>
+        <v>6967.741935483871</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>7130.470476</v>
+        <v>7388.488579000001</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>453.0511211612911</v>
+        <v>420.7466435161296</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>0.067848235536232</v>
+        <v>0.0603849349490741</v>
       </c>
       <c r="U12" s="128" t="n">
-        <v>42.44327664285714</v>
+        <v>43.97909868452381</v>
       </c>
       <c r="V12" s="128" t="n">
-        <v>3.943276642857143</v>
+        <v>5.479098684523812</v>
       </c>
       <c r="W12" s="120" t="inlineStr">
         <is>
@@ -1620,34 +1620,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="127" t="n">
-        <v>19.52461799660441</v>
+        <v>20.37351443123939</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>5</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-9.524617996604412</v>
+        <v>-10.37351443123939</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>741.9354838709677</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>732.8096790000001</v>
+        <v>764.399679</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-9.125804870967611</v>
+        <v>-9.793869387096834</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.012299997869565</v>
+        <v>-0.012650414625</v>
       </c>
       <c r="U14" s="128" t="n">
-        <v>73.28096790000001</v>
+        <v>76.4399679</v>
       </c>
       <c r="V14" s="128" t="n">
-        <v>35.28096790000001</v>
+        <v>38.4399679</v>
       </c>
       <c r="W14" s="120" t="inlineStr">
         <is>
@@ -1750,34 +1750,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M16" s="127" t="n">
-        <v>2.967741935483871</v>
+        <v>3.096774193548387</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>-0.967741935483871</v>
+        <v>-1.096774193548387</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>741.9354838709677</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>778.320652</v>
+        <v>801.563374</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>36.38516812903231</v>
+        <v>27.36982561290313</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.0490408787826087</v>
+        <v>0.0353526914166665</v>
       </c>
       <c r="U16" s="128" t="n">
-        <v>389.160326</v>
+        <v>400.781687</v>
       </c>
       <c r="V16" s="128" t="n">
-        <v>139.160326</v>
+        <v>150.781687</v>
       </c>
       <c r="W16" s="120" t="inlineStr">
         <is>
@@ -1880,34 +1880,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>579.6370967741935</v>
+        <v>604.8387096774194</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>417</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-162.6370967741935</v>
+        <v>-187.8387096774194</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>7419.354838709677</v>
+        <v>7741.935483870968</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>10090.15</v>
+        <v>10351.47</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>2670.795161290323</v>
+        <v>2609.534516129032</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>0.3599767391304348</v>
+        <v>0.3370648749999999</v>
       </c>
       <c r="U18" s="117" t="n">
-        <v>24.19700239808153</v>
+        <v>24.8236690647482</v>
       </c>
       <c r="V18" s="117" t="n">
-        <v>11.39700239808153</v>
+        <v>12.0236690647482</v>
       </c>
       <c r="W18" s="120" t="inlineStr">
         <is>
@@ -1963,34 +1963,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>9.274193548387096</v>
+        <v>9.677419354838708</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>32</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>22.7258064516129</v>
+        <v>22.32258064516129</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>370.9677419354838</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>384.99</v>
+        <v>393.57</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>14.02225806451617</v>
+        <v>6.47322580645158</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>0.0377991304347827</v>
+        <v>0.0167224999999999</v>
       </c>
       <c r="U19" s="117" t="n">
-        <v>12.0309375</v>
+        <v>12.2990625</v>
       </c>
       <c r="V19" s="117" t="n">
-        <v>-27.9690625</v>
+        <v>-27.7009375</v>
       </c>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
@@ -2042,34 +2042,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>8.243727598566307</v>
+        <v>8.602150537634408</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>10.75627240143369</v>
+        <v>10.39784946236559</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>741.9354838709677</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>697.0700000000001</v>
+        <v>707</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-44.86548387096764</v>
+        <v>-67.19354838709683</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.0604708695652172</v>
+        <v>-0.0867916666666667</v>
       </c>
       <c r="U20" s="117" t="n">
-        <v>36.68789473684211</v>
+        <v>37.21052631578947</v>
       </c>
       <c r="V20" s="117" t="n">
-        <v>-53.31210526315789</v>
+        <v>-52.78947368421053</v>
       </c>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
@@ -2121,34 +2121,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>3.091397849462366</v>
+        <v>3.225806451612904</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>4</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>0.908602150537634</v>
+        <v>0.7741935483870961</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>370.9677419354838</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="R21" s="117" t="n">
-        <v>344.39</v>
+        <v>353.43</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-26.57774193548386</v>
+        <v>-33.66677419354841</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.0716443478260869</v>
+        <v>-0.08697249999999999</v>
       </c>
       <c r="U21" s="117" t="n">
-        <v>86.0975</v>
+        <v>88.3575</v>
       </c>
       <c r="V21" s="117" t="n">
-        <v>-33.9025</v>
+        <v>-31.6425</v>
       </c>
       <c r="W21" s="120" t="inlineStr"/>
     </row>
@@ -2200,34 +2200,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>27.82258064516129</v>
+        <v>29.03225806451613</v>
       </c>
       <c r="N22" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-5.822580645161292</v>
+        <v>-7.032258064516128</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>1112.903225806452</v>
+        <v>1161.290322580645</v>
       </c>
       <c r="R22" s="117" t="n">
-        <v>1312.096658</v>
+        <v>1335.846658</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>199.1934321935482</v>
+        <v>174.5563354193546</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>0.1789854028405795</v>
+        <v>0.1503123999444442</v>
       </c>
       <c r="U22" s="117" t="n">
-        <v>59.64075718181818</v>
+        <v>60.72030263636363</v>
       </c>
       <c r="V22" s="117" t="n">
-        <v>19.64075718181818</v>
+        <v>20.72030263636364</v>
       </c>
       <c r="W22" s="120" t="inlineStr"/>
     </row>
@@ -2279,34 +2279,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>74.19354838709677</v>
+        <v>77.41935483870967</v>
       </c>
       <c r="N23" s="119" t="n">
         <v>114</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>39.80645161290323</v>
+        <v>36.58064516129033</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>1112.903225806452</v>
+        <v>1161.290322580645</v>
       </c>
       <c r="R23" s="117" t="n">
-        <v>1637.830756</v>
+        <v>1728.505387</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>524.9275301935484</v>
+        <v>567.2150644193546</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.4716740126376811</v>
+        <v>0.4884351943611108</v>
       </c>
       <c r="U23" s="117" t="n">
-        <v>14.36693645614035</v>
+        <v>15.16232795614035</v>
       </c>
       <c r="V23" s="117" t="n">
-        <v>-0.6330635438596488</v>
+        <v>0.1623279561403503</v>
       </c>
       <c r="W23" s="120" t="inlineStr">
         <is>
@@ -2362,34 +2362,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>28.53598014888337</v>
+        <v>29.77667493796526</v>
       </c>
       <c r="N24" s="119" t="n">
         <v>67</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>38.46401985111663</v>
+        <v>37.22332506203474</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>741.9354838709677</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="R24" s="117" t="n">
-        <v>1195.66</v>
+        <v>1215.59</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>453.7245161290324</v>
+        <v>441.3964516129031</v>
       </c>
       <c r="T24" s="118" t="n">
-        <v>0.611541739130435</v>
+        <v>0.5701370833333331</v>
       </c>
       <c r="U24" s="117" t="n">
-        <v>17.84567164179105</v>
+        <v>18.14313432835821</v>
       </c>
       <c r="V24" s="117" t="n">
-        <v>-8.154328358208954</v>
+        <v>-7.856865671641792</v>
       </c>
       <c r="W24" s="120" t="inlineStr"/>
     </row>
@@ -2436,12 +2436,12 @@
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>510.42</v>
+        <v>551.6</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
       <c r="U25" s="117" t="n">
-        <v>510.42</v>
+        <v>551.6</v>
       </c>
       <c r="V25" s="117" t="n"/>
       <c r="W25" s="120" t="inlineStr"/>
@@ -2478,34 +2478,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>1014.016876160115</v>
+        <v>1058.104566427946</v>
       </c>
       <c r="N26" s="125" t="n">
         <v>967</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>-47.01687616011486</v>
+        <v>-91.10456642794612</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>23000</v>
+        <v>24000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>28532.851997</v>
+        <v>29390.832281</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>5532.851997000002</v>
+        <v>5390.832280999999</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>0.2405587824782609</v>
+        <v>0.2246180117083333</v>
       </c>
       <c r="U26" s="123" t="n">
-        <v>29.50656876628749</v>
+        <v>30.39382862564633</v>
       </c>
       <c r="V26" s="123" t="n">
-        <v>6.824500508117534</v>
+        <v>7.711760367476373</v>
       </c>
       <c r="W26" s="126" t="n"/>
     </row>
@@ -2553,28 +2553,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>488.1154499151104</v>
+        <v>509.3378607809848</v>
       </c>
       <c r="N27" s="119" t="n">
         <v>371</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-117.1154499151104</v>
+        <v>-138.3378607809848</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>3695.652173913044</v>
+        <v>3913.04347826087</v>
       </c>
       <c r="R27" s="117" t="n">
         <v>2819.6</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-876.0521739130436</v>
+        <v>-1093.44347826087</v>
       </c>
       <c r="T27" s="118" t="n">
-        <v>-0.2370494117647059</v>
+        <v>-0.2794355555555555</v>
       </c>
       <c r="U27" s="117" t="n">
         <v>7.6</v>
@@ -2628,28 +2628,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>329.7491039426523</v>
+        <v>344.0860215053764</v>
       </c>
       <c r="N28" s="119" t="n">
         <v>187</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-142.7491039426523</v>
+        <v>-157.0860215053764</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>2956.521739130435</v>
+        <v>3130.434782608696</v>
       </c>
       <c r="R28" s="117" t="n">
         <v>1683</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-1273.521739130435</v>
+        <v>-1447.434782608696</v>
       </c>
       <c r="T28" s="118" t="n">
-        <v>-0.43075</v>
+        <v>-0.462375</v>
       </c>
       <c r="U28" s="117" t="n">
         <v>9</v>
@@ -2703,28 +2703,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>185.4838709677419</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="N29" s="119" t="n">
         <v>240</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>54.51612903225808</v>
+        <v>46.45161290322579</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>1478.260869565217</v>
+        <v>1565.217391304348</v>
       </c>
       <c r="R29" s="117" t="n">
         <v>1920</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>441.7391304347825</v>
+        <v>354.782608695652</v>
       </c>
       <c r="T29" s="118" t="n">
-        <v>0.2988235294117646</v>
+        <v>0.2266666666666665</v>
       </c>
       <c r="U29" s="117" t="n">
         <v>8</v>
@@ -2766,28 +2766,28 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>1003.348424825505</v>
+        <v>1046.972269383135</v>
       </c>
       <c r="N30" s="125" t="n">
         <v>798</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-205.3484248255046</v>
+        <v>-248.9722693831354</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>8130.434782608696</v>
+        <v>8608.695652173914</v>
       </c>
       <c r="R30" s="123" t="n">
         <v>6422.6</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>-1707.834782608696</v>
+        <v>-2186.095652173913</v>
       </c>
       <c r="T30" s="124" t="n">
-        <v>-0.2100545454545454</v>
+        <v>-0.2539404040404041</v>
       </c>
       <c r="U30" s="123" t="n">
         <v>8.048370927318297</v>
@@ -2829,34 +2829,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="133" t="n">
-        <v>2363.601860125405</v>
+        <v>2466.367158391727</v>
       </c>
       <c r="N31" s="133" t="n">
         <v>2093</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>-270.6018601254045</v>
+        <v>-373.3671583917267</v>
       </c>
       <c r="P31" s="131" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="Q31" s="131" t="n">
-        <v>46711.07994389901</v>
+        <v>48866.76016830295</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>50462.288139</v>
+        <v>51589.818423</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>3751.208195100982</v>
+        <v>2723.058254697047</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>0.08030660390653049</v>
+        <v>0.0557241414269845</v>
       </c>
       <c r="U31" s="131" t="n">
-        <v>24.11002777783086</v>
+        <v>24.64874267701863</v>
       </c>
       <c r="V31" s="131" t="n">
-        <v>4.334304855785522</v>
+        <v>4.873019754973292</v>
       </c>
       <c r="W31" s="134" t="n"/>
     </row>
@@ -3137,13 +3137,13 @@
         </is>
       </c>
       <c r="B2" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C2" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D2" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3180,16 +3180,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="137" t="n">
-        <v>7048.387096774193</v>
+        <v>7354.838709677419</v>
       </c>
       <c r="V2" s="137" t="n">
-        <v>7475.593311999999</v>
+        <v>7640.583312000001</v>
       </c>
       <c r="W2" s="137" t="n">
-        <v>427.2062152258059</v>
+        <v>285.7446023225821</v>
       </c>
       <c r="X2" s="138" t="n">
-        <v>0.0606104927780319</v>
+        <v>0.0388512397894738</v>
       </c>
       <c r="Y2" s="137" t="n"/>
       <c r="Z2" s="137" t="n"/>
@@ -3223,13 +3223,13 @@
         </is>
       </c>
       <c r="B3" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C3" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D3" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3290,13 +3290,13 @@
         </is>
       </c>
       <c r="B4" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C4" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D4" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3333,16 +3333,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="137" t="n">
-        <v>1112.903225806452</v>
+        <v>1161.290322580645</v>
       </c>
       <c r="V4" s="137" t="n">
-        <v>1281.92283</v>
+        <v>1302.88283</v>
       </c>
       <c r="W4" s="137" t="n">
-        <v>169.0196041935483</v>
+        <v>141.5925074193547</v>
       </c>
       <c r="X4" s="138" t="n">
-        <v>0.1518726878260868</v>
+        <v>0.1219268813888887</v>
       </c>
       <c r="Y4" s="137" t="n"/>
       <c r="Z4" s="137" t="n"/>
@@ -3376,13 +3376,13 @@
         </is>
       </c>
       <c r="B5" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C5" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D5" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3443,13 +3443,13 @@
         </is>
       </c>
       <c r="B6" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C6" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D6" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3486,16 +3486,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="137" t="n">
-        <v>7419.354838709677</v>
+        <v>7741.935483870968</v>
       </c>
       <c r="V6" s="137" t="n">
-        <v>6749.32</v>
+        <v>6832.92</v>
       </c>
       <c r="W6" s="137" t="n">
-        <v>-670.0348387096774</v>
+        <v>-909.0154838709676</v>
       </c>
       <c r="X6" s="138" t="n">
-        <v>-0.0903090434782608</v>
+        <v>-0.1174144999999999</v>
       </c>
       <c r="Y6" s="137" t="n"/>
       <c r="Z6" s="137" t="n"/>
@@ -3529,13 +3529,13 @@
         </is>
       </c>
       <c r="B7" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C7" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D7" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -3582,28 +3582,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>488.1154499151104</v>
+        <v>509.3378607809848</v>
       </c>
       <c r="R7" t="n">
         <v>371</v>
       </c>
       <c r="S7" t="n">
-        <v>-117.1154499151104</v>
+        <v>-138.3378607809848</v>
       </c>
       <c r="T7" s="137" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="U7" s="137" t="n">
-        <v>3695.652173913044</v>
+        <v>3913.04347826087</v>
       </c>
       <c r="V7" s="137" t="n">
         <v>2819.6</v>
       </c>
       <c r="W7" s="137" t="n">
-        <v>-876.0521739130436</v>
+        <v>-1093.44347826087</v>
       </c>
       <c r="X7" s="138" t="n">
-        <v>-0.2370494117647059</v>
+        <v>-0.2794355555555555</v>
       </c>
       <c r="Y7" s="137" t="n">
         <v>7.6</v>
@@ -3632,13 +3632,13 @@
         </is>
       </c>
       <c r="B8" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C8" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D8" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E8" t="n">
         <v>26</v>
@@ -3685,28 +3685,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>329.7491039426523</v>
+        <v>344.0860215053764</v>
       </c>
       <c r="R8" t="n">
         <v>187</v>
       </c>
       <c r="S8" t="n">
-        <v>-142.7491039426523</v>
+        <v>-157.0860215053764</v>
       </c>
       <c r="T8" s="137" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="U8" s="137" t="n">
-        <v>2956.521739130435</v>
+        <v>3130.434782608696</v>
       </c>
       <c r="V8" s="137" t="n">
         <v>1683</v>
       </c>
       <c r="W8" s="137" t="n">
-        <v>-1273.521739130435</v>
+        <v>-1447.434782608696</v>
       </c>
       <c r="X8" s="138" t="n">
-        <v>-0.43075</v>
+        <v>-0.462375</v>
       </c>
       <c r="Y8" s="137" t="n">
         <v>9</v>
@@ -3735,13 +3735,13 @@
         </is>
       </c>
       <c r="B9" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C9" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D9" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3788,28 +3788,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>185.4838709677419</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="R9" t="n">
         <v>240</v>
       </c>
       <c r="S9" t="n">
-        <v>54.51612903225808</v>
+        <v>46.45161290322579</v>
       </c>
       <c r="T9" s="137" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="U9" s="137" t="n">
-        <v>1478.260869565217</v>
+        <v>1565.217391304348</v>
       </c>
       <c r="V9" s="137" t="n">
         <v>1920</v>
       </c>
       <c r="W9" s="137" t="n">
-        <v>441.7391304347825</v>
+        <v>354.782608695652</v>
       </c>
       <c r="X9" s="138" t="n">
-        <v>0.2988235294117646</v>
+        <v>0.2266666666666665</v>
       </c>
       <c r="Y9" s="137" t="n">
         <v>8</v>
@@ -3838,13 +3838,13 @@
         </is>
       </c>
       <c r="B10" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C10" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D10" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3891,34 +3891,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>87.28652751423149</v>
+        <v>91.08159392789372</v>
       </c>
       <c r="R10" t="n">
         <v>111</v>
       </c>
       <c r="S10" t="n">
-        <v>23.71347248576851</v>
+        <v>19.91840607210627</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U10" s="137" t="n">
-        <v>2967.741935483871</v>
+        <v>3096.774193548388</v>
       </c>
       <c r="V10" s="137" t="n">
-        <v>3718.643776</v>
+        <v>3799.368604</v>
       </c>
       <c r="W10" s="137" t="n">
-        <v>750.9018405161291</v>
+        <v>702.5944104516125</v>
       </c>
       <c r="X10" s="138" t="n">
-        <v>0.2530212723478261</v>
+        <v>0.2268794450416665</v>
       </c>
       <c r="Y10" s="137" t="n">
-        <v>33.50129527927928</v>
+        <v>34.22854598198198</v>
       </c>
       <c r="Z10" s="137" t="n">
-        <v>-0.498704720720724</v>
+        <v>0.2285459819819806</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -3950,13 +3950,13 @@
         </is>
       </c>
       <c r="B11" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C11" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D11" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -4003,34 +4003,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q11" t="n">
-        <v>173.4394637620444</v>
+        <v>180.980310012568</v>
       </c>
       <c r="R11" t="n">
         <v>61</v>
       </c>
       <c r="S11" t="n">
-        <v>-5.439463762044397</v>
+        <v>-12.98031001256805</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U11" s="137" t="n">
-        <v>6677.419354838709</v>
+        <v>6967.741935483871</v>
       </c>
       <c r="V11" s="137" t="n">
-        <v>7130.470476</v>
+        <v>7388.488579000001</v>
       </c>
       <c r="W11" s="137" t="n">
-        <v>453.0511211612911</v>
+        <v>420.7466435161296</v>
       </c>
       <c r="X11" s="138" t="n">
-        <v>0.067848235536232</v>
+        <v>0.0603849349490741</v>
       </c>
       <c r="Y11" s="137" t="n">
-        <v>42.44327664285714</v>
+        <v>43.97909868452381</v>
       </c>
       <c r="Z11" s="137" t="n">
-        <v>3.943276642857143</v>
+        <v>5.479098684523812</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -4062,13 +4062,13 @@
         </is>
       </c>
       <c r="B12" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C12" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D12" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -4132,13 +4132,13 @@
         </is>
       </c>
       <c r="B13" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C13" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D13" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4185,34 +4185,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>19.52461799660441</v>
+        <v>20.37351443123939</v>
       </c>
       <c r="R13" t="n">
         <v>5</v>
       </c>
       <c r="S13" t="n">
-        <v>-9.524617996604412</v>
+        <v>-10.37351443123939</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="137" t="n">
-        <v>741.9354838709677</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="V13" s="137" t="n">
-        <v>732.8096790000001</v>
+        <v>764.399679</v>
       </c>
       <c r="W13" s="137" t="n">
-        <v>-9.125804870967611</v>
+        <v>-9.793869387096834</v>
       </c>
       <c r="X13" s="138" t="n">
-        <v>-0.012299997869565</v>
+        <v>-0.012650414625</v>
       </c>
       <c r="Y13" s="137" t="n">
-        <v>73.28096790000001</v>
+        <v>76.4399679</v>
       </c>
       <c r="Z13" s="137" t="n">
-        <v>35.28096790000001</v>
+        <v>38.4399679</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -4244,13 +4244,13 @@
         </is>
       </c>
       <c r="B14" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C14" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D14" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
@@ -4314,13 +4314,13 @@
         </is>
       </c>
       <c r="B15" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C15" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D15" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -4367,34 +4367,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q15" t="n">
-        <v>2.967741935483871</v>
+        <v>3.096774193548387</v>
       </c>
       <c r="R15" t="n">
         <v>2</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.967741935483871</v>
+        <v>-1.096774193548387</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U15" s="137" t="n">
-        <v>741.9354838709677</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="V15" s="137" t="n">
-        <v>778.320652</v>
+        <v>801.563374</v>
       </c>
       <c r="W15" s="137" t="n">
-        <v>36.38516812903231</v>
+        <v>27.36982561290313</v>
       </c>
       <c r="X15" s="138" t="n">
-        <v>0.0490408787826087</v>
+        <v>0.0353526914166665</v>
       </c>
       <c r="Y15" s="137" t="n">
-        <v>389.160326</v>
+        <v>400.781687</v>
       </c>
       <c r="Z15" s="137" t="n">
-        <v>139.160326</v>
+        <v>150.781687</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -4426,13 +4426,13 @@
         </is>
       </c>
       <c r="B16" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C16" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D16" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4496,13 +4496,13 @@
         </is>
       </c>
       <c r="B17" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C17" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D17" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E17" t="n">
         <v>17</v>
@@ -4549,34 +4549,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>579.6370967741935</v>
+        <v>604.8387096774194</v>
       </c>
       <c r="R17" t="n">
         <v>417</v>
       </c>
       <c r="S17" t="n">
-        <v>-162.6370967741935</v>
+        <v>-187.8387096774194</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U17" s="137" t="n">
-        <v>7419.354838709677</v>
+        <v>7741.935483870968</v>
       </c>
       <c r="V17" s="137" t="n">
-        <v>10090.15</v>
+        <v>10351.47</v>
       </c>
       <c r="W17" s="137" t="n">
-        <v>2670.795161290323</v>
+        <v>2609.534516129032</v>
       </c>
       <c r="X17" s="138" t="n">
-        <v>0.3599767391304348</v>
+        <v>0.3370648749999999</v>
       </c>
       <c r="Y17" s="137" t="n">
-        <v>24.19700239808153</v>
+        <v>24.8236690647482</v>
       </c>
       <c r="Z17" s="137" t="n">
-        <v>11.39700239808153</v>
+        <v>12.0236690647482</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -4608,13 +4608,13 @@
         </is>
       </c>
       <c r="B18" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C18" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D18" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4661,34 +4661,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>9.274193548387096</v>
+        <v>9.677419354838708</v>
       </c>
       <c r="R18" t="n">
         <v>32</v>
       </c>
       <c r="S18" t="n">
-        <v>22.7258064516129</v>
+        <v>22.32258064516129</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="137" t="n">
-        <v>370.9677419354838</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="V18" s="137" t="n">
-        <v>384.99</v>
+        <v>393.57</v>
       </c>
       <c r="W18" s="137" t="n">
-        <v>14.02225806451617</v>
+        <v>6.47322580645158</v>
       </c>
       <c r="X18" s="138" t="n">
-        <v>0.0377991304347827</v>
+        <v>0.0167224999999999</v>
       </c>
       <c r="Y18" s="137" t="n">
-        <v>12.0309375</v>
+        <v>12.2990625</v>
       </c>
       <c r="Z18" s="137" t="n">
-        <v>-27.9690625</v>
+        <v>-27.7009375</v>
       </c>
       <c r="AB18" s="139" t="inlineStr"/>
       <c r="AC18" s="139" t="inlineStr">
@@ -4715,13 +4715,13 @@
         </is>
       </c>
       <c r="B19" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C19" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D19" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4768,34 +4768,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>8.243727598566307</v>
+        <v>8.602150537634408</v>
       </c>
       <c r="R19" t="n">
         <v>19</v>
       </c>
       <c r="S19" t="n">
-        <v>10.75627240143369</v>
+        <v>10.39784946236559</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="137" t="n">
-        <v>741.9354838709677</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="V19" s="137" t="n">
-        <v>697.0700000000001</v>
+        <v>707</v>
       </c>
       <c r="W19" s="137" t="n">
-        <v>-44.86548387096764</v>
+        <v>-67.19354838709683</v>
       </c>
       <c r="X19" s="138" t="n">
-        <v>-0.0604708695652172</v>
+        <v>-0.0867916666666667</v>
       </c>
       <c r="Y19" s="137" t="n">
-        <v>36.68789473684211</v>
+        <v>37.21052631578947</v>
       </c>
       <c r="Z19" s="137" t="n">
-        <v>-53.31210526315789</v>
+        <v>-52.78947368421053</v>
       </c>
       <c r="AB19" s="139" t="inlineStr"/>
       <c r="AC19" s="139" t="inlineStr">
@@ -4822,13 +4822,13 @@
         </is>
       </c>
       <c r="B20" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C20" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D20" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
@@ -4875,34 +4875,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>3.091397849462366</v>
+        <v>3.225806451612904</v>
       </c>
       <c r="R20" t="n">
         <v>4</v>
       </c>
       <c r="S20" t="n">
-        <v>0.908602150537634</v>
+        <v>0.7741935483870961</v>
       </c>
       <c r="T20" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U20" s="137" t="n">
-        <v>370.9677419354838</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="V20" s="137" t="n">
-        <v>344.39</v>
+        <v>353.43</v>
       </c>
       <c r="W20" s="137" t="n">
-        <v>-26.57774193548386</v>
+        <v>-33.66677419354841</v>
       </c>
       <c r="X20" s="138" t="n">
-        <v>-0.0716443478260869</v>
+        <v>-0.08697249999999999</v>
       </c>
       <c r="Y20" s="137" t="n">
-        <v>86.0975</v>
+        <v>88.3575</v>
       </c>
       <c r="Z20" s="137" t="n">
-        <v>-33.9025</v>
+        <v>-31.6425</v>
       </c>
       <c r="AB20" s="139" t="inlineStr"/>
       <c r="AC20" s="139" t="inlineStr">
@@ -4929,13 +4929,13 @@
         </is>
       </c>
       <c r="B21" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C21" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D21" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4982,34 +4982,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>27.82258064516129</v>
+        <v>29.03225806451613</v>
       </c>
       <c r="R21" t="n">
         <v>22</v>
       </c>
       <c r="S21" t="n">
-        <v>-5.822580645161292</v>
+        <v>-7.032258064516128</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="137" t="n">
-        <v>1112.903225806452</v>
+        <v>1161.290322580645</v>
       </c>
       <c r="V21" s="137" t="n">
-        <v>1312.096658</v>
+        <v>1335.846658</v>
       </c>
       <c r="W21" s="137" t="n">
-        <v>199.1934321935482</v>
+        <v>174.5563354193546</v>
       </c>
       <c r="X21" s="138" t="n">
-        <v>0.1789854028405795</v>
+        <v>0.1503123999444442</v>
       </c>
       <c r="Y21" s="137" t="n">
-        <v>59.64075718181818</v>
+        <v>60.72030263636363</v>
       </c>
       <c r="Z21" s="137" t="n">
-        <v>19.64075718181818</v>
+        <v>20.72030263636364</v>
       </c>
       <c r="AB21" s="139" t="inlineStr">
         <is>
@@ -5036,13 +5036,13 @@
         </is>
       </c>
       <c r="B22" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C22" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D22" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -5089,34 +5089,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>74.19354838709677</v>
+        <v>77.41935483870967</v>
       </c>
       <c r="R22" t="n">
         <v>114</v>
       </c>
       <c r="S22" t="n">
-        <v>39.80645161290323</v>
+        <v>36.58064516129033</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="137" t="n">
-        <v>1112.903225806452</v>
+        <v>1161.290322580645</v>
       </c>
       <c r="V22" s="137" t="n">
-        <v>1637.830756</v>
+        <v>1728.505387</v>
       </c>
       <c r="W22" s="137" t="n">
-        <v>524.9275301935484</v>
+        <v>567.2150644193546</v>
       </c>
       <c r="X22" s="138" t="n">
-        <v>0.4716740126376811</v>
+        <v>0.4884351943611108</v>
       </c>
       <c r="Y22" s="137" t="n">
-        <v>14.36693645614035</v>
+        <v>15.16232795614035</v>
       </c>
       <c r="Z22" s="137" t="n">
-        <v>-0.6330635438596488</v>
+        <v>0.1623279561403503</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -5148,13 +5148,13 @@
         </is>
       </c>
       <c r="B23" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C23" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D23" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5201,34 +5201,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>28.53598014888337</v>
+        <v>29.77667493796526</v>
       </c>
       <c r="R23" t="n">
         <v>67</v>
       </c>
       <c r="S23" t="n">
-        <v>38.46401985111663</v>
+        <v>37.22332506203474</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="137" t="n">
-        <v>741.9354838709677</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="V23" s="137" t="n">
-        <v>1195.66</v>
+        <v>1215.59</v>
       </c>
       <c r="W23" s="137" t="n">
-        <v>453.7245161290324</v>
+        <v>441.3964516129031</v>
       </c>
       <c r="X23" s="138" t="n">
-        <v>0.611541739130435</v>
+        <v>0.5701370833333331</v>
       </c>
       <c r="Y23" s="137" t="n">
-        <v>17.84567164179105</v>
+        <v>18.14313432835821</v>
       </c>
       <c r="Z23" s="137" t="n">
-        <v>-8.154328358208954</v>
+        <v>-7.856865671641792</v>
       </c>
       <c r="AB23" s="139" t="inlineStr"/>
       <c r="AC23" s="139" t="inlineStr">
@@ -5255,13 +5255,13 @@
         </is>
       </c>
       <c r="B24" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C24" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D24" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5298,12 +5298,12 @@
       <c r="T24" s="137" t="n"/>
       <c r="U24" s="137" t="n"/>
       <c r="V24" s="137" t="n">
-        <v>510.42</v>
+        <v>551.6</v>
       </c>
       <c r="W24" s="137" t="n"/>
       <c r="X24" s="138" t="n"/>
       <c r="Y24" s="137" t="n">
-        <v>510.42</v>
+        <v>551.6</v>
       </c>
       <c r="Z24" s="137" t="n"/>
       <c r="AB24" s="139" t="inlineStr"/>
@@ -5331,13 +5331,13 @@
         </is>
       </c>
       <c r="B25" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C25" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D25" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5366,34 +5366,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>346.236559139785</v>
+        <v>361.2903225806452</v>
       </c>
       <c r="R25" t="n">
         <v>328</v>
       </c>
       <c r="S25" t="n">
-        <v>-18.23655913978496</v>
+        <v>-33.29032258064518</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="137" t="n">
-        <v>15580.64516129032</v>
+        <v>16258.06451612903</v>
       </c>
       <c r="V25" s="137" t="n">
-        <v>15506.836142</v>
+        <v>15776.386142</v>
       </c>
       <c r="W25" s="137" t="n">
-        <v>-73.8090192903237</v>
+        <v>-481.678374129031</v>
       </c>
       <c r="X25" s="138" t="n">
-        <v>-0.0047372248405797</v>
+        <v>-0.0296270428531745</v>
       </c>
       <c r="Y25" s="137" t="n">
-        <v>47.27693945731707</v>
+        <v>48.09873823780488</v>
       </c>
       <c r="Z25" s="137" t="n">
-        <v>2.27693945731707</v>
+        <v>3.098738237804881</v>
       </c>
       <c r="AB25" s="139" t="inlineStr"/>
       <c r="AC25" s="139" t="inlineStr"/>
@@ -5411,13 +5411,13 @@
         </is>
       </c>
       <c r="B26" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C26" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D26" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5451,34 +5451,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>1014.016876160115</v>
+        <v>1058.104566427946</v>
       </c>
       <c r="R26" t="n">
         <v>967</v>
       </c>
       <c r="S26" t="n">
-        <v>-47.01687616011486</v>
+        <v>-91.10456642794612</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="137" t="n">
-        <v>23000</v>
+        <v>24000</v>
       </c>
       <c r="V26" s="137" t="n">
-        <v>28532.851997</v>
+        <v>29390.832281</v>
       </c>
       <c r="W26" s="137" t="n">
-        <v>5532.851997000002</v>
+        <v>5390.832280999999</v>
       </c>
       <c r="X26" s="138" t="n">
-        <v>0.2405587824782609</v>
+        <v>0.2246180117083333</v>
       </c>
       <c r="Y26" s="137" t="n">
-        <v>29.50656876628749</v>
+        <v>30.39382862564633</v>
       </c>
       <c r="Z26" s="137" t="n">
-        <v>6.824500508117534</v>
+        <v>7.711760367476373</v>
       </c>
       <c r="AB26" s="139" t="inlineStr"/>
       <c r="AC26" s="139" t="inlineStr"/>
@@ -5496,13 +5496,13 @@
         </is>
       </c>
       <c r="B27" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C27" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D27" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5536,28 +5536,28 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>1003.348424825505</v>
+        <v>1046.972269383135</v>
       </c>
       <c r="R27" t="n">
         <v>798</v>
       </c>
       <c r="S27" t="n">
-        <v>-205.3484248255046</v>
+        <v>-248.9722693831354</v>
       </c>
       <c r="T27" s="137" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="U27" s="137" t="n">
-        <v>8130.434782608696</v>
+        <v>8608.695652173914</v>
       </c>
       <c r="V27" s="137" t="n">
         <v>6422.6</v>
       </c>
       <c r="W27" s="137" t="n">
-        <v>-1707.834782608696</v>
+        <v>-2186.095652173913</v>
       </c>
       <c r="X27" s="138" t="n">
-        <v>-0.2100545454545454</v>
+        <v>-0.2539404040404041</v>
       </c>
       <c r="Y27" s="137" t="n">
         <v>8.048370927318297</v>
@@ -5581,13 +5581,13 @@
         </is>
       </c>
       <c r="B28" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="C28" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D28" s="136" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5621,34 +5621,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>2363.601860125405</v>
+        <v>2466.367158391727</v>
       </c>
       <c r="R28" t="n">
         <v>2093</v>
       </c>
       <c r="S28" t="n">
-        <v>-270.6018601254045</v>
+        <v>-373.3671583917267</v>
       </c>
       <c r="T28" s="137" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="U28" s="137" t="n">
-        <v>46711.07994389901</v>
+        <v>48866.76016830295</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>50462.288139</v>
+        <v>51589.818423</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>3751.208195100982</v>
+        <v>2723.058254697047</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>0.08030660390653049</v>
+        <v>0.0557241414269845</v>
       </c>
       <c r="Y28" s="137" t="n">
-        <v>24.11002777783086</v>
+        <v>24.64874267701863</v>
       </c>
       <c r="Z28" s="137" t="n">
-        <v>4.334304855785522</v>
+        <v>4.873019754973292</v>
       </c>
       <c r="AB28" s="139" t="inlineStr"/>
       <c r="AC28" s="139" t="inlineStr"/>
@@ -5751,7 +5751,7 @@
         </is>
       </c>
       <c r="B4" s="140" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5791,7 +5791,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5811,7 +5811,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46227.2918287037</v>
+        <v>46228.29190972223</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-07-26
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 24/07/2026  |  Ultimo aggiornamento: 25/07/2026 07:00</t>
+          <t>Periodo: 01/07/2026 - 25/07/2026  |  Ultimo aggiornamento: 26/07/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1065,16 +1065,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>7354.838709677419</v>
+        <v>7661.290322580645</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>7640.583312000001</v>
+        <v>7807.164287</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>285.7446023225821</v>
+        <v>145.8739644193547</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0388512397894738</v>
+        <v>0.0190403911452631</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1173,16 +1173,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>1161.290322580645</v>
+        <v>1209.677419354839</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>1302.88283</v>
+        <v>1327.24283</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>141.5925074193547</v>
+        <v>117.5654106451611</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>0.1219268813888887</v>
+        <v>0.0971874061333332</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1281,16 +1281,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>7741.935483870968</v>
+        <v>8064.516129032258</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>6832.92</v>
+        <v>6905.08</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-909.0154838709676</v>
+        <v>-1159.436129032258</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.1174144999999999</v>
+        <v>-0.1437700799999999</v>
       </c>
       <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
@@ -1328,34 +1328,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>361.2903225806452</v>
+        <v>376.3440860215054</v>
       </c>
       <c r="N10" s="125" t="n">
         <v>328</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>-33.29032258064518</v>
+        <v>-48.3440860215054</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>16258.06451612903</v>
+        <v>16935.48387096774</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>15776.386142</v>
+        <v>16039.487117</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>-481.678374129031</v>
+        <v>-895.9967539677436</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>-0.0296270428531745</v>
+        <v>-0.0529064749961905</v>
       </c>
       <c r="U10" s="123" t="n">
-        <v>48.09873823780488</v>
+        <v>48.90087535670731</v>
       </c>
       <c r="V10" s="123" t="n">
-        <v>3.098738237804881</v>
+        <v>3.90087535670731</v>
       </c>
       <c r="W10" s="126" t="n"/>
     </row>
@@ -1407,34 +1407,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>91.08159392789372</v>
+        <v>94.87666034155598</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>111</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>19.91840607210627</v>
+        <v>16.12333965844402</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>3096.774193548388</v>
+        <v>3225.806451612903</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>3799.368604</v>
+        <v>3881.173415</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>702.5944104516125</v>
+        <v>655.3669633870968</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.2268794450416665</v>
+        <v>0.20316375865</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>34.22854598198198</v>
+        <v>34.96552626126126</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>0.2285459819819806</v>
+        <v>0.9655262612612604</v>
       </c>
       <c r="W11" s="120" t="inlineStr">
         <is>
@@ -1490,34 +1490,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M12" s="127" t="n">
-        <v>180.980310012568</v>
+        <v>188.5211562630917</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>61</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>-12.98031001256805</v>
+        <v>-20.52115626309174</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>6967.741935483871</v>
+        <v>7258.064516129032</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>7388.488579000001</v>
+        <v>7595.101119000001</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>420.7466435161296</v>
+        <v>337.0366028709686</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>0.0603849349490741</v>
+        <v>0.0464361541733334</v>
       </c>
       <c r="U12" s="128" t="n">
-        <v>43.97909868452381</v>
+        <v>45.20893523214286</v>
       </c>
       <c r="V12" s="128" t="n">
-        <v>5.479098684523812</v>
+        <v>6.708935232142864</v>
       </c>
       <c r="W12" s="120" t="inlineStr">
         <is>
@@ -1620,34 +1620,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="127" t="n">
-        <v>20.37351443123939</v>
+        <v>21.22241086587436</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>5</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-10.37351443123939</v>
+        <v>-11.22241086587436</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>774.1935483870968</v>
+        <v>806.4516129032259</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>764.399679</v>
+        <v>790.9651590000001</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-9.793869387096834</v>
+        <v>-15.48645390322576</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.012650414625</v>
+        <v>-0.0192032028399999</v>
       </c>
       <c r="U14" s="128" t="n">
-        <v>76.4399679</v>
+        <v>79.09651590000001</v>
       </c>
       <c r="V14" s="128" t="n">
-        <v>38.4399679</v>
+        <v>41.09651590000001</v>
       </c>
       <c r="W14" s="120" t="inlineStr">
         <is>
@@ -1750,34 +1750,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M16" s="127" t="n">
-        <v>3.096774193548387</v>
+        <v>3.225806451612903</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>-1.096774193548387</v>
+        <v>-1.225806451612903</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>774.1935483870968</v>
+        <v>806.4516129032259</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>801.563374</v>
+        <v>823.103314</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>27.36982561290313</v>
+        <v>16.6517010967741</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.0353526914166665</v>
+        <v>0.0206481093599998</v>
       </c>
       <c r="U16" s="128" t="n">
-        <v>400.781687</v>
+        <v>411.551657</v>
       </c>
       <c r="V16" s="128" t="n">
-        <v>150.781687</v>
+        <v>161.551657</v>
       </c>
       <c r="W16" s="120" t="inlineStr">
         <is>
@@ -1880,34 +1880,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>604.8387096774194</v>
+        <v>630.0403225806452</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>417</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-187.8387096774194</v>
+        <v>-213.0403225806452</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>7741.935483870968</v>
+        <v>8064.516129032258</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>10351.47</v>
+        <v>10569.57</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>2609.534516129032</v>
+        <v>2505.053870967742</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>0.3370648749999999</v>
+        <v>0.31062668</v>
       </c>
       <c r="U18" s="117" t="n">
-        <v>24.8236690647482</v>
+        <v>25.34669064748201</v>
       </c>
       <c r="V18" s="117" t="n">
-        <v>12.0236690647482</v>
+        <v>12.54669064748201</v>
       </c>
       <c r="W18" s="120" t="inlineStr">
         <is>
@@ -1963,34 +1963,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>9.677419354838708</v>
+        <v>10.08064516129032</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>32</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>22.32258064516129</v>
+        <v>21.91935483870968</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>387.0967741935484</v>
+        <v>403.2258064516129</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>393.57</v>
+        <v>401.82</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>6.47322580645158</v>
+        <v>-1.405806451612932</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>0.0167224999999999</v>
+        <v>-0.0034864</v>
       </c>
       <c r="U19" s="117" t="n">
-        <v>12.2990625</v>
+        <v>12.556875</v>
       </c>
       <c r="V19" s="117" t="n">
-        <v>-27.7009375</v>
+        <v>-27.443125</v>
       </c>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
@@ -2042,34 +2042,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>8.602150537634408</v>
+        <v>8.960573476702509</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>10.39784946236559</v>
+        <v>10.03942652329749</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>774.1935483870968</v>
+        <v>806.4516129032259</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>707</v>
+        <v>716.45</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-67.19354838709683</v>
+        <v>-90.0016129032258</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.0867916666666667</v>
+        <v>-0.1116019999999999</v>
       </c>
       <c r="U20" s="117" t="n">
-        <v>37.21052631578947</v>
+        <v>37.70789473684211</v>
       </c>
       <c r="V20" s="117" t="n">
-        <v>-52.78947368421053</v>
+        <v>-52.29210526315789</v>
       </c>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
@@ -2121,34 +2121,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>3.225806451612904</v>
+        <v>3.360215053763441</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>4</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>0.7741935483870961</v>
+        <v>0.6397849462365586</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>387.0967741935484</v>
+        <v>403.2258064516129</v>
       </c>
       <c r="R21" s="117" t="n">
-        <v>353.43</v>
+        <v>360.69</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-33.66677419354841</v>
+        <v>-42.53580645161293</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.08697249999999999</v>
+        <v>-0.1054888</v>
       </c>
       <c r="U21" s="117" t="n">
-        <v>88.3575</v>
+        <v>90.1725</v>
       </c>
       <c r="V21" s="117" t="n">
-        <v>-31.6425</v>
+        <v>-29.8275</v>
       </c>
       <c r="W21" s="120" t="inlineStr"/>
     </row>
@@ -2200,34 +2200,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>29.03225806451613</v>
+        <v>30.24193548387097</v>
       </c>
       <c r="N22" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-7.032258064516128</v>
+        <v>-8.241935483870968</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>1161.290322580645</v>
+        <v>1209.677419354839</v>
       </c>
       <c r="R22" s="117" t="n">
-        <v>1335.846658</v>
+        <v>1357.706658</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>174.5563354193546</v>
+        <v>148.0292386451613</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>0.1503123999444442</v>
+        <v>0.1223708372799999</v>
       </c>
       <c r="U22" s="117" t="n">
-        <v>60.72030263636363</v>
+        <v>61.713939</v>
       </c>
       <c r="V22" s="117" t="n">
-        <v>20.72030263636364</v>
+        <v>21.713939</v>
       </c>
       <c r="W22" s="120" t="inlineStr"/>
     </row>
@@ -2279,34 +2279,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>77.41935483870967</v>
+        <v>80.64516129032258</v>
       </c>
       <c r="N23" s="119" t="n">
         <v>114</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>36.58064516129033</v>
+        <v>33.35483870967742</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>1161.290322580645</v>
+        <v>1209.677419354839</v>
       </c>
       <c r="R23" s="117" t="n">
-        <v>1728.505387</v>
+        <v>1816.561969</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>567.2150644193546</v>
+        <v>606.8845496451613</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.4884351943611108</v>
+        <v>0.5016912277066666</v>
       </c>
       <c r="U23" s="117" t="n">
-        <v>15.16232795614035</v>
+        <v>15.93475411403509</v>
       </c>
       <c r="V23" s="117" t="n">
-        <v>0.1623279561403503</v>
+        <v>0.9347541140350888</v>
       </c>
       <c r="W23" s="120" t="inlineStr">
         <is>
@@ -2362,34 +2362,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>29.77667493796526</v>
+        <v>31.01736972704714</v>
       </c>
       <c r="N24" s="119" t="n">
         <v>67</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>37.22332506203474</v>
+        <v>35.98263027295285</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>774.1935483870968</v>
+        <v>806.4516129032259</v>
       </c>
       <c r="R24" s="117" t="n">
-        <v>1215.59</v>
+        <v>1224.02</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>441.3964516129031</v>
+        <v>417.5683870967741</v>
       </c>
       <c r="T24" s="118" t="n">
-        <v>0.5701370833333331</v>
+        <v>0.5177847999999999</v>
       </c>
       <c r="U24" s="117" t="n">
-        <v>18.14313432835821</v>
+        <v>18.2689552238806</v>
       </c>
       <c r="V24" s="117" t="n">
-        <v>-7.856865671641792</v>
+        <v>-7.731044776119404</v>
       </c>
       <c r="W24" s="120" t="inlineStr"/>
     </row>
@@ -2436,12 +2436,12 @@
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>551.6</v>
+        <v>581.75</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
       <c r="U25" s="117" t="n">
-        <v>551.6</v>
+        <v>581.75</v>
       </c>
       <c r="V25" s="117" t="n"/>
       <c r="W25" s="120" t="inlineStr"/>
@@ -2478,34 +2478,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>1058.104566427946</v>
+        <v>1102.192256695777</v>
       </c>
       <c r="N26" s="125" t="n">
         <v>967</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>-91.10456642794612</v>
+        <v>-135.1922566957771</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>24000</v>
+        <v>25000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>29390.832281</v>
+        <v>30118.911634</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>5390.832280999999</v>
+        <v>5118.911634</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>0.2246180117083333</v>
+        <v>0.20475646536</v>
       </c>
       <c r="U26" s="123" t="n">
-        <v>30.39382862564633</v>
+        <v>31.1467545336091</v>
       </c>
       <c r="V26" s="123" t="n">
-        <v>7.711760367476373</v>
+        <v>8.464686275439146</v>
       </c>
       <c r="W26" s="126" t="n"/>
     </row>
@@ -2553,13 +2553,13 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>509.3378607809848</v>
+        <v>530.5602716468592</v>
       </c>
       <c r="N27" s="119" t="n">
         <v>371</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-138.3378607809848</v>
+        <v>-159.5602716468592</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>217.3913043478261</v>
@@ -2628,13 +2628,13 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>344.0860215053764</v>
+        <v>358.4229390681004</v>
       </c>
       <c r="N28" s="119" t="n">
         <v>187</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-157.0860215053764</v>
+        <v>-171.4229390681004</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>173.9130434782609</v>
@@ -2703,13 +2703,13 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>193.5483870967742</v>
+        <v>201.6129032258065</v>
       </c>
       <c r="N29" s="119" t="n">
         <v>240</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>46.45161290322579</v>
+        <v>38.38709677419354</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>86.95652173913044</v>
@@ -2766,13 +2766,13 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>1046.972269383135</v>
+        <v>1090.596113940766</v>
       </c>
       <c r="N30" s="125" t="n">
         <v>798</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-248.9722693831354</v>
+        <v>-292.5961139407659</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>478.2608695652174</v>
@@ -2829,34 +2829,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="133" t="n">
-        <v>2466.367158391727</v>
+        <v>2569.132456658048</v>
       </c>
       <c r="N31" s="133" t="n">
         <v>2093</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>-373.3671583917267</v>
+        <v>-476.1324566580483</v>
       </c>
       <c r="P31" s="131" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="Q31" s="131" t="n">
-        <v>48866.76016830295</v>
+        <v>50544.17952314165</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>51589.818423</v>
+        <v>52580.998751</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>2723.058254697047</v>
+        <v>2036.819227858345</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>0.0557241414269845</v>
+        <v>0.0402977998075087</v>
       </c>
       <c r="U31" s="131" t="n">
-        <v>24.64874267701863</v>
+        <v>25.12231187338748</v>
       </c>
       <c r="V31" s="131" t="n">
-        <v>4.873019754973292</v>
+        <v>5.346588951342142</v>
       </c>
       <c r="W31" s="134" t="n"/>
     </row>
@@ -3137,13 +3137,13 @@
         </is>
       </c>
       <c r="B2" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C2" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D2" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3180,16 +3180,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="137" t="n">
-        <v>7354.838709677419</v>
+        <v>7661.290322580645</v>
       </c>
       <c r="V2" s="137" t="n">
-        <v>7640.583312000001</v>
+        <v>7807.164287</v>
       </c>
       <c r="W2" s="137" t="n">
-        <v>285.7446023225821</v>
+        <v>145.8739644193547</v>
       </c>
       <c r="X2" s="138" t="n">
-        <v>0.0388512397894738</v>
+        <v>0.0190403911452631</v>
       </c>
       <c r="Y2" s="137" t="n"/>
       <c r="Z2" s="137" t="n"/>
@@ -3223,13 +3223,13 @@
         </is>
       </c>
       <c r="B3" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C3" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D3" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3290,13 +3290,13 @@
         </is>
       </c>
       <c r="B4" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C4" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D4" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3333,16 +3333,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="137" t="n">
-        <v>1161.290322580645</v>
+        <v>1209.677419354839</v>
       </c>
       <c r="V4" s="137" t="n">
-        <v>1302.88283</v>
+        <v>1327.24283</v>
       </c>
       <c r="W4" s="137" t="n">
-        <v>141.5925074193547</v>
+        <v>117.5654106451611</v>
       </c>
       <c r="X4" s="138" t="n">
-        <v>0.1219268813888887</v>
+        <v>0.0971874061333332</v>
       </c>
       <c r="Y4" s="137" t="n"/>
       <c r="Z4" s="137" t="n"/>
@@ -3376,13 +3376,13 @@
         </is>
       </c>
       <c r="B5" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C5" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D5" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3443,13 +3443,13 @@
         </is>
       </c>
       <c r="B6" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C6" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D6" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3486,16 +3486,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="137" t="n">
-        <v>7741.935483870968</v>
+        <v>8064.516129032258</v>
       </c>
       <c r="V6" s="137" t="n">
-        <v>6832.92</v>
+        <v>6905.08</v>
       </c>
       <c r="W6" s="137" t="n">
-        <v>-909.0154838709676</v>
+        <v>-1159.436129032258</v>
       </c>
       <c r="X6" s="138" t="n">
-        <v>-0.1174144999999999</v>
+        <v>-0.1437700799999999</v>
       </c>
       <c r="Y6" s="137" t="n"/>
       <c r="Z6" s="137" t="n"/>
@@ -3529,13 +3529,13 @@
         </is>
       </c>
       <c r="B7" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C7" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D7" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -3582,13 +3582,13 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>509.3378607809848</v>
+        <v>530.5602716468592</v>
       </c>
       <c r="R7" t="n">
         <v>371</v>
       </c>
       <c r="S7" t="n">
-        <v>-138.3378607809848</v>
+        <v>-159.5602716468592</v>
       </c>
       <c r="T7" s="137" t="n">
         <v>217.3913043478261</v>
@@ -3632,13 +3632,13 @@
         </is>
       </c>
       <c r="B8" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C8" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D8" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E8" t="n">
         <v>26</v>
@@ -3685,13 +3685,13 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>344.0860215053764</v>
+        <v>358.4229390681004</v>
       </c>
       <c r="R8" t="n">
         <v>187</v>
       </c>
       <c r="S8" t="n">
-        <v>-157.0860215053764</v>
+        <v>-171.4229390681004</v>
       </c>
       <c r="T8" s="137" t="n">
         <v>173.9130434782609</v>
@@ -3735,13 +3735,13 @@
         </is>
       </c>
       <c r="B9" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C9" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D9" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3788,13 +3788,13 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>193.5483870967742</v>
+        <v>201.6129032258065</v>
       </c>
       <c r="R9" t="n">
         <v>240</v>
       </c>
       <c r="S9" t="n">
-        <v>46.45161290322579</v>
+        <v>38.38709677419354</v>
       </c>
       <c r="T9" s="137" t="n">
         <v>86.95652173913044</v>
@@ -3838,13 +3838,13 @@
         </is>
       </c>
       <c r="B10" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C10" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D10" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3891,34 +3891,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>91.08159392789372</v>
+        <v>94.87666034155598</v>
       </c>
       <c r="R10" t="n">
         <v>111</v>
       </c>
       <c r="S10" t="n">
-        <v>19.91840607210627</v>
+        <v>16.12333965844402</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U10" s="137" t="n">
-        <v>3096.774193548388</v>
+        <v>3225.806451612903</v>
       </c>
       <c r="V10" s="137" t="n">
-        <v>3799.368604</v>
+        <v>3881.173415</v>
       </c>
       <c r="W10" s="137" t="n">
-        <v>702.5944104516125</v>
+        <v>655.3669633870968</v>
       </c>
       <c r="X10" s="138" t="n">
-        <v>0.2268794450416665</v>
+        <v>0.20316375865</v>
       </c>
       <c r="Y10" s="137" t="n">
-        <v>34.22854598198198</v>
+        <v>34.96552626126126</v>
       </c>
       <c r="Z10" s="137" t="n">
-        <v>0.2285459819819806</v>
+        <v>0.9655262612612604</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -3950,13 +3950,13 @@
         </is>
       </c>
       <c r="B11" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C11" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D11" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -4003,34 +4003,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q11" t="n">
-        <v>180.980310012568</v>
+        <v>188.5211562630917</v>
       </c>
       <c r="R11" t="n">
         <v>61</v>
       </c>
       <c r="S11" t="n">
-        <v>-12.98031001256805</v>
+        <v>-20.52115626309174</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U11" s="137" t="n">
-        <v>6967.741935483871</v>
+        <v>7258.064516129032</v>
       </c>
       <c r="V11" s="137" t="n">
-        <v>7388.488579000001</v>
+        <v>7595.101119000001</v>
       </c>
       <c r="W11" s="137" t="n">
-        <v>420.7466435161296</v>
+        <v>337.0366028709686</v>
       </c>
       <c r="X11" s="138" t="n">
-        <v>0.0603849349490741</v>
+        <v>0.0464361541733334</v>
       </c>
       <c r="Y11" s="137" t="n">
-        <v>43.97909868452381</v>
+        <v>45.20893523214286</v>
       </c>
       <c r="Z11" s="137" t="n">
-        <v>5.479098684523812</v>
+        <v>6.708935232142864</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -4062,13 +4062,13 @@
         </is>
       </c>
       <c r="B12" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C12" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D12" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -4132,13 +4132,13 @@
         </is>
       </c>
       <c r="B13" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C13" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D13" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4185,34 +4185,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>20.37351443123939</v>
+        <v>21.22241086587436</v>
       </c>
       <c r="R13" t="n">
         <v>5</v>
       </c>
       <c r="S13" t="n">
-        <v>-10.37351443123939</v>
+        <v>-11.22241086587436</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="137" t="n">
-        <v>774.1935483870968</v>
+        <v>806.4516129032259</v>
       </c>
       <c r="V13" s="137" t="n">
-        <v>764.399679</v>
+        <v>790.9651590000001</v>
       </c>
       <c r="W13" s="137" t="n">
-        <v>-9.793869387096834</v>
+        <v>-15.48645390322576</v>
       </c>
       <c r="X13" s="138" t="n">
-        <v>-0.012650414625</v>
+        <v>-0.0192032028399999</v>
       </c>
       <c r="Y13" s="137" t="n">
-        <v>76.4399679</v>
+        <v>79.09651590000001</v>
       </c>
       <c r="Z13" s="137" t="n">
-        <v>38.4399679</v>
+        <v>41.09651590000001</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -4244,13 +4244,13 @@
         </is>
       </c>
       <c r="B14" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C14" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D14" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
@@ -4314,13 +4314,13 @@
         </is>
       </c>
       <c r="B15" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C15" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D15" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -4367,34 +4367,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q15" t="n">
-        <v>3.096774193548387</v>
+        <v>3.225806451612903</v>
       </c>
       <c r="R15" t="n">
         <v>2</v>
       </c>
       <c r="S15" t="n">
-        <v>-1.096774193548387</v>
+        <v>-1.225806451612903</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U15" s="137" t="n">
-        <v>774.1935483870968</v>
+        <v>806.4516129032259</v>
       </c>
       <c r="V15" s="137" t="n">
-        <v>801.563374</v>
+        <v>823.103314</v>
       </c>
       <c r="W15" s="137" t="n">
-        <v>27.36982561290313</v>
+        <v>16.6517010967741</v>
       </c>
       <c r="X15" s="138" t="n">
-        <v>0.0353526914166665</v>
+        <v>0.0206481093599998</v>
       </c>
       <c r="Y15" s="137" t="n">
-        <v>400.781687</v>
+        <v>411.551657</v>
       </c>
       <c r="Z15" s="137" t="n">
-        <v>150.781687</v>
+        <v>161.551657</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -4426,13 +4426,13 @@
         </is>
       </c>
       <c r="B16" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C16" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D16" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4496,13 +4496,13 @@
         </is>
       </c>
       <c r="B17" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C17" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D17" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E17" t="n">
         <v>17</v>
@@ -4549,34 +4549,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>604.8387096774194</v>
+        <v>630.0403225806452</v>
       </c>
       <c r="R17" t="n">
         <v>417</v>
       </c>
       <c r="S17" t="n">
-        <v>-187.8387096774194</v>
+        <v>-213.0403225806452</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U17" s="137" t="n">
-        <v>7741.935483870968</v>
+        <v>8064.516129032258</v>
       </c>
       <c r="V17" s="137" t="n">
-        <v>10351.47</v>
+        <v>10569.57</v>
       </c>
       <c r="W17" s="137" t="n">
-        <v>2609.534516129032</v>
+        <v>2505.053870967742</v>
       </c>
       <c r="X17" s="138" t="n">
-        <v>0.3370648749999999</v>
+        <v>0.31062668</v>
       </c>
       <c r="Y17" s="137" t="n">
-        <v>24.8236690647482</v>
+        <v>25.34669064748201</v>
       </c>
       <c r="Z17" s="137" t="n">
-        <v>12.0236690647482</v>
+        <v>12.54669064748201</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -4608,13 +4608,13 @@
         </is>
       </c>
       <c r="B18" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C18" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D18" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4661,34 +4661,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>9.677419354838708</v>
+        <v>10.08064516129032</v>
       </c>
       <c r="R18" t="n">
         <v>32</v>
       </c>
       <c r="S18" t="n">
-        <v>22.32258064516129</v>
+        <v>21.91935483870968</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="137" t="n">
-        <v>387.0967741935484</v>
+        <v>403.2258064516129</v>
       </c>
       <c r="V18" s="137" t="n">
-        <v>393.57</v>
+        <v>401.82</v>
       </c>
       <c r="W18" s="137" t="n">
-        <v>6.47322580645158</v>
+        <v>-1.405806451612932</v>
       </c>
       <c r="X18" s="138" t="n">
-        <v>0.0167224999999999</v>
+        <v>-0.0034864</v>
       </c>
       <c r="Y18" s="137" t="n">
-        <v>12.2990625</v>
+        <v>12.556875</v>
       </c>
       <c r="Z18" s="137" t="n">
-        <v>-27.7009375</v>
+        <v>-27.443125</v>
       </c>
       <c r="AB18" s="139" t="inlineStr"/>
       <c r="AC18" s="139" t="inlineStr">
@@ -4715,13 +4715,13 @@
         </is>
       </c>
       <c r="B19" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C19" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D19" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4768,34 +4768,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>8.602150537634408</v>
+        <v>8.960573476702509</v>
       </c>
       <c r="R19" t="n">
         <v>19</v>
       </c>
       <c r="S19" t="n">
-        <v>10.39784946236559</v>
+        <v>10.03942652329749</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="137" t="n">
-        <v>774.1935483870968</v>
+        <v>806.4516129032259</v>
       </c>
       <c r="V19" s="137" t="n">
-        <v>707</v>
+        <v>716.45</v>
       </c>
       <c r="W19" s="137" t="n">
-        <v>-67.19354838709683</v>
+        <v>-90.0016129032258</v>
       </c>
       <c r="X19" s="138" t="n">
-        <v>-0.0867916666666667</v>
+        <v>-0.1116019999999999</v>
       </c>
       <c r="Y19" s="137" t="n">
-        <v>37.21052631578947</v>
+        <v>37.70789473684211</v>
       </c>
       <c r="Z19" s="137" t="n">
-        <v>-52.78947368421053</v>
+        <v>-52.29210526315789</v>
       </c>
       <c r="AB19" s="139" t="inlineStr"/>
       <c r="AC19" s="139" t="inlineStr">
@@ -4822,13 +4822,13 @@
         </is>
       </c>
       <c r="B20" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C20" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D20" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
@@ -4875,34 +4875,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>3.225806451612904</v>
+        <v>3.360215053763441</v>
       </c>
       <c r="R20" t="n">
         <v>4</v>
       </c>
       <c r="S20" t="n">
-        <v>0.7741935483870961</v>
+        <v>0.6397849462365586</v>
       </c>
       <c r="T20" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U20" s="137" t="n">
-        <v>387.0967741935484</v>
+        <v>403.2258064516129</v>
       </c>
       <c r="V20" s="137" t="n">
-        <v>353.43</v>
+        <v>360.69</v>
       </c>
       <c r="W20" s="137" t="n">
-        <v>-33.66677419354841</v>
+        <v>-42.53580645161293</v>
       </c>
       <c r="X20" s="138" t="n">
-        <v>-0.08697249999999999</v>
+        <v>-0.1054888</v>
       </c>
       <c r="Y20" s="137" t="n">
-        <v>88.3575</v>
+        <v>90.1725</v>
       </c>
       <c r="Z20" s="137" t="n">
-        <v>-31.6425</v>
+        <v>-29.8275</v>
       </c>
       <c r="AB20" s="139" t="inlineStr"/>
       <c r="AC20" s="139" t="inlineStr">
@@ -4929,13 +4929,13 @@
         </is>
       </c>
       <c r="B21" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C21" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D21" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4982,34 +4982,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>29.03225806451613</v>
+        <v>30.24193548387097</v>
       </c>
       <c r="R21" t="n">
         <v>22</v>
       </c>
       <c r="S21" t="n">
-        <v>-7.032258064516128</v>
+        <v>-8.241935483870968</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="137" t="n">
-        <v>1161.290322580645</v>
+        <v>1209.677419354839</v>
       </c>
       <c r="V21" s="137" t="n">
-        <v>1335.846658</v>
+        <v>1357.706658</v>
       </c>
       <c r="W21" s="137" t="n">
-        <v>174.5563354193546</v>
+        <v>148.0292386451613</v>
       </c>
       <c r="X21" s="138" t="n">
-        <v>0.1503123999444442</v>
+        <v>0.1223708372799999</v>
       </c>
       <c r="Y21" s="137" t="n">
-        <v>60.72030263636363</v>
+        <v>61.713939</v>
       </c>
       <c r="Z21" s="137" t="n">
-        <v>20.72030263636364</v>
+        <v>21.713939</v>
       </c>
       <c r="AB21" s="139" t="inlineStr">
         <is>
@@ -5036,13 +5036,13 @@
         </is>
       </c>
       <c r="B22" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C22" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D22" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -5089,34 +5089,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>77.41935483870967</v>
+        <v>80.64516129032258</v>
       </c>
       <c r="R22" t="n">
         <v>114</v>
       </c>
       <c r="S22" t="n">
-        <v>36.58064516129033</v>
+        <v>33.35483870967742</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="137" t="n">
-        <v>1161.290322580645</v>
+        <v>1209.677419354839</v>
       </c>
       <c r="V22" s="137" t="n">
-        <v>1728.505387</v>
+        <v>1816.561969</v>
       </c>
       <c r="W22" s="137" t="n">
-        <v>567.2150644193546</v>
+        <v>606.8845496451613</v>
       </c>
       <c r="X22" s="138" t="n">
-        <v>0.4884351943611108</v>
+        <v>0.5016912277066666</v>
       </c>
       <c r="Y22" s="137" t="n">
-        <v>15.16232795614035</v>
+        <v>15.93475411403509</v>
       </c>
       <c r="Z22" s="137" t="n">
-        <v>0.1623279561403503</v>
+        <v>0.9347541140350888</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -5148,13 +5148,13 @@
         </is>
       </c>
       <c r="B23" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C23" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D23" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5201,34 +5201,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>29.77667493796526</v>
+        <v>31.01736972704714</v>
       </c>
       <c r="R23" t="n">
         <v>67</v>
       </c>
       <c r="S23" t="n">
-        <v>37.22332506203474</v>
+        <v>35.98263027295285</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="137" t="n">
-        <v>774.1935483870968</v>
+        <v>806.4516129032259</v>
       </c>
       <c r="V23" s="137" t="n">
-        <v>1215.59</v>
+        <v>1224.02</v>
       </c>
       <c r="W23" s="137" t="n">
-        <v>441.3964516129031</v>
+        <v>417.5683870967741</v>
       </c>
       <c r="X23" s="138" t="n">
-        <v>0.5701370833333331</v>
+        <v>0.5177847999999999</v>
       </c>
       <c r="Y23" s="137" t="n">
-        <v>18.14313432835821</v>
+        <v>18.2689552238806</v>
       </c>
       <c r="Z23" s="137" t="n">
-        <v>-7.856865671641792</v>
+        <v>-7.731044776119404</v>
       </c>
       <c r="AB23" s="139" t="inlineStr"/>
       <c r="AC23" s="139" t="inlineStr">
@@ -5255,13 +5255,13 @@
         </is>
       </c>
       <c r="B24" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C24" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D24" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5298,12 +5298,12 @@
       <c r="T24" s="137" t="n"/>
       <c r="U24" s="137" t="n"/>
       <c r="V24" s="137" t="n">
-        <v>551.6</v>
+        <v>581.75</v>
       </c>
       <c r="W24" s="137" t="n"/>
       <c r="X24" s="138" t="n"/>
       <c r="Y24" s="137" t="n">
-        <v>551.6</v>
+        <v>581.75</v>
       </c>
       <c r="Z24" s="137" t="n"/>
       <c r="AB24" s="139" t="inlineStr"/>
@@ -5331,13 +5331,13 @@
         </is>
       </c>
       <c r="B25" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C25" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D25" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5366,34 +5366,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>361.2903225806452</v>
+        <v>376.3440860215054</v>
       </c>
       <c r="R25" t="n">
         <v>328</v>
       </c>
       <c r="S25" t="n">
-        <v>-33.29032258064518</v>
+        <v>-48.3440860215054</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="137" t="n">
-        <v>16258.06451612903</v>
+        <v>16935.48387096774</v>
       </c>
       <c r="V25" s="137" t="n">
-        <v>15776.386142</v>
+        <v>16039.487117</v>
       </c>
       <c r="W25" s="137" t="n">
-        <v>-481.678374129031</v>
+        <v>-895.9967539677436</v>
       </c>
       <c r="X25" s="138" t="n">
-        <v>-0.0296270428531745</v>
+        <v>-0.0529064749961905</v>
       </c>
       <c r="Y25" s="137" t="n">
-        <v>48.09873823780488</v>
+        <v>48.90087535670731</v>
       </c>
       <c r="Z25" s="137" t="n">
-        <v>3.098738237804881</v>
+        <v>3.90087535670731</v>
       </c>
       <c r="AB25" s="139" t="inlineStr"/>
       <c r="AC25" s="139" t="inlineStr"/>
@@ -5411,13 +5411,13 @@
         </is>
       </c>
       <c r="B26" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C26" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D26" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5451,34 +5451,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>1058.104566427946</v>
+        <v>1102.192256695777</v>
       </c>
       <c r="R26" t="n">
         <v>967</v>
       </c>
       <c r="S26" t="n">
-        <v>-91.10456642794612</v>
+        <v>-135.1922566957771</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="137" t="n">
-        <v>24000</v>
+        <v>25000</v>
       </c>
       <c r="V26" s="137" t="n">
-        <v>29390.832281</v>
+        <v>30118.911634</v>
       </c>
       <c r="W26" s="137" t="n">
-        <v>5390.832280999999</v>
+        <v>5118.911634</v>
       </c>
       <c r="X26" s="138" t="n">
-        <v>0.2246180117083333</v>
+        <v>0.20475646536</v>
       </c>
       <c r="Y26" s="137" t="n">
-        <v>30.39382862564633</v>
+        <v>31.1467545336091</v>
       </c>
       <c r="Z26" s="137" t="n">
-        <v>7.711760367476373</v>
+        <v>8.464686275439146</v>
       </c>
       <c r="AB26" s="139" t="inlineStr"/>
       <c r="AC26" s="139" t="inlineStr"/>
@@ -5496,13 +5496,13 @@
         </is>
       </c>
       <c r="B27" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C27" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D27" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5536,13 +5536,13 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>1046.972269383135</v>
+        <v>1090.596113940766</v>
       </c>
       <c r="R27" t="n">
         <v>798</v>
       </c>
       <c r="S27" t="n">
-        <v>-248.9722693831354</v>
+        <v>-292.5961139407659</v>
       </c>
       <c r="T27" s="137" t="n">
         <v>478.2608695652174</v>
@@ -5581,13 +5581,13 @@
         </is>
       </c>
       <c r="B28" s="136" t="n">
-        <v>46228</v>
+        <v>46229</v>
       </c>
       <c r="C28" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D28" s="136" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5621,34 +5621,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>2466.367158391727</v>
+        <v>2569.132456658048</v>
       </c>
       <c r="R28" t="n">
         <v>2093</v>
       </c>
       <c r="S28" t="n">
-        <v>-373.3671583917267</v>
+        <v>-476.1324566580483</v>
       </c>
       <c r="T28" s="137" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="U28" s="137" t="n">
-        <v>48866.76016830295</v>
+        <v>50544.17952314165</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>51589.818423</v>
+        <v>52580.998751</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>2723.058254697047</v>
+        <v>2036.819227858345</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>0.0557241414269845</v>
+        <v>0.0402977998075087</v>
       </c>
       <c r="Y28" s="137" t="n">
-        <v>24.64874267701863</v>
+        <v>25.12231187338748</v>
       </c>
       <c r="Z28" s="137" t="n">
-        <v>4.873019754973292</v>
+        <v>5.346588951342142</v>
       </c>
       <c r="AB28" s="139" t="inlineStr"/>
       <c r="AC28" s="139" t="inlineStr"/>
@@ -5751,7 +5751,7 @@
         </is>
       </c>
       <c r="B4" s="140" t="n">
-        <v>46227</v>
+        <v>46228</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5791,7 +5791,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5811,7 +5811,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46228.29190972223</v>
+        <v>46229.29190972223</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-07-28
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 25/07/2026  |  Ultimo aggiornamento: 26/07/2026 07:00</t>
+          <t>Periodo: 01/07/2026 - 27/07/2026  |  Ultimo aggiornamento: 28/07/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1065,16 +1065,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>7661.290322580645</v>
+        <v>8274.193548387097</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>7807.164287</v>
+        <v>8077.867025</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>145.8739644193547</v>
+        <v>-196.326523387097</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0190403911452631</v>
+        <v>-0.0237275720272904</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1173,16 +1173,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>1209.677419354839</v>
+        <v>1306.451612903226</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>1327.24283</v>
+        <v>1368.086458</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>117.5654106451611</v>
+        <v>61.63484509677414</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>0.0971874061333332</v>
+        <v>0.0471772888395061</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1281,16 +1281,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>8064.516129032258</v>
+        <v>8709.677419354839</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>6905.08</v>
+        <v>7066.69</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-1159.436129032258</v>
+        <v>-1642.987419354839</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.1437700799999999</v>
+        <v>-0.1886392962962963</v>
       </c>
       <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
@@ -1328,34 +1328,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>376.3440860215054</v>
+        <v>406.4516129032259</v>
       </c>
       <c r="N10" s="125" t="n">
         <v>328</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>-48.3440860215054</v>
+        <v>-78.45161290322585</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>16935.48387096774</v>
+        <v>18290.32258064516</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>16039.487117</v>
+        <v>16512.643483</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>-895.9967539677436</v>
+        <v>-1777.679097645163</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>-0.0529064749961905</v>
+        <v>-0.09719233161728399</v>
       </c>
       <c r="U10" s="123" t="n">
-        <v>48.90087535670731</v>
+        <v>50.34342525304878</v>
       </c>
       <c r="V10" s="123" t="n">
-        <v>3.90087535670731</v>
+        <v>5.343425253048778</v>
       </c>
       <c r="W10" s="126" t="n"/>
     </row>
@@ -1407,34 +1407,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>94.87666034155598</v>
+        <v>102.4667931688805</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>111</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>16.12333965844402</v>
+        <v>8.533206831119543</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>3225.806451612903</v>
+        <v>3483.870967741936</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>3881.173415</v>
+        <v>4033.470302</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>655.3669633870968</v>
+        <v>549.5993342580646</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.20316375865</v>
+        <v>0.1577553644629629</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>34.96552626126126</v>
+        <v>36.33757028828829</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>0.9655262612612604</v>
+        <v>2.33757028828829</v>
       </c>
       <c r="W11" s="120" t="inlineStr">
         <is>
@@ -1490,34 +1490,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M12" s="127" t="n">
-        <v>188.5211562630917</v>
+        <v>203.6028487641391</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>61</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>-20.52115626309174</v>
+        <v>-35.60284876413908</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>7258.064516129032</v>
+        <v>7838.709677419354</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>7595.101119000001</v>
+        <v>7997.154267</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>337.0366028709686</v>
+        <v>158.4445895806457</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>0.0464361541733334</v>
+        <v>0.0202130957901235</v>
       </c>
       <c r="U12" s="128" t="n">
-        <v>45.20893523214286</v>
+        <v>47.60210873214286</v>
       </c>
       <c r="V12" s="128" t="n">
-        <v>6.708935232142864</v>
+        <v>9.10210873214286</v>
       </c>
       <c r="W12" s="120" t="inlineStr">
         <is>
@@ -1620,34 +1620,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="127" t="n">
-        <v>21.22241086587436</v>
+        <v>22.92020373514431</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>5</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-11.22241086587436</v>
+        <v>-12.92020373514431</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>806.4516129032259</v>
+        <v>870.9677419354839</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>790.9651590000001</v>
+        <v>853.4385040000001</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-15.48645390322576</v>
+        <v>-17.52923793548382</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.0192032028399999</v>
+        <v>-0.020126162074074</v>
       </c>
       <c r="U14" s="128" t="n">
-        <v>79.09651590000001</v>
+        <v>85.34385040000001</v>
       </c>
       <c r="V14" s="128" t="n">
-        <v>41.09651590000001</v>
+        <v>47.34385040000001</v>
       </c>
       <c r="W14" s="120" t="inlineStr">
         <is>
@@ -1750,34 +1750,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M16" s="127" t="n">
-        <v>3.225806451612903</v>
+        <v>3.483870967741935</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>-1.225806451612903</v>
+        <v>-1.483870967741935</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>806.4516129032259</v>
+        <v>870.9677419354839</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>823.103314</v>
+        <v>875.3623249999999</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>16.6517010967741</v>
+        <v>4.394583064516041</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.0206481093599998</v>
+        <v>0.0050456324074073</v>
       </c>
       <c r="U16" s="128" t="n">
-        <v>411.551657</v>
+        <v>437.6811625</v>
       </c>
       <c r="V16" s="128" t="n">
-        <v>161.551657</v>
+        <v>187.6811625</v>
       </c>
       <c r="W16" s="120" t="inlineStr">
         <is>
@@ -1880,34 +1880,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>630.0403225806452</v>
+        <v>680.4435483870968</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>417</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-213.0403225806452</v>
+        <v>-263.4435483870968</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>8064.516129032258</v>
+        <v>8709.677419354839</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>10569.57</v>
+        <v>11088.19</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>2505.053870967742</v>
+        <v>2378.512580645161</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>0.31062668</v>
+        <v>0.2730884814814815</v>
       </c>
       <c r="U18" s="117" t="n">
-        <v>25.34669064748201</v>
+        <v>26.59038369304556</v>
       </c>
       <c r="V18" s="117" t="n">
-        <v>12.54669064748201</v>
+        <v>13.79038369304556</v>
       </c>
       <c r="W18" s="120" t="inlineStr">
         <is>
@@ -1963,34 +1963,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>10.08064516129032</v>
+        <v>10.88709677419355</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>32</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>21.91935483870968</v>
+        <v>21.11290322580645</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>403.2258064516129</v>
+        <v>435.483870967742</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>401.82</v>
+        <v>426.16</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-1.405806451612932</v>
+        <v>-9.323870967741923</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.0034864</v>
+        <v>-0.0214103703703703</v>
       </c>
       <c r="U19" s="117" t="n">
-        <v>12.556875</v>
+        <v>13.3175</v>
       </c>
       <c r="V19" s="117" t="n">
-        <v>-27.443125</v>
+        <v>-26.6825</v>
       </c>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
@@ -2042,34 +2042,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>8.960573476702509</v>
+        <v>9.67741935483871</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>10.03942652329749</v>
+        <v>9.32258064516129</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>806.4516129032259</v>
+        <v>870.9677419354839</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>716.45</v>
+        <v>736.39</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-90.0016129032258</v>
+        <v>-134.5777419354839</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.1116019999999999</v>
+        <v>-0.1545151851851852</v>
       </c>
       <c r="U20" s="117" t="n">
-        <v>37.70789473684211</v>
+        <v>38.75736842105263</v>
       </c>
       <c r="V20" s="117" t="n">
-        <v>-52.29210526315789</v>
+        <v>-51.24263157894737</v>
       </c>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
@@ -2121,34 +2121,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>3.360215053763441</v>
+        <v>3.629032258064517</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>4</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>0.6397849462365586</v>
+        <v>0.3709677419354835</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>403.2258064516129</v>
+        <v>435.483870967742</v>
       </c>
       <c r="R21" s="117" t="n">
-        <v>360.69</v>
+        <v>382.04</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-42.53580645161293</v>
+        <v>-53.44387096774193</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.1054888</v>
+        <v>-0.1227229629629629</v>
       </c>
       <c r="U21" s="117" t="n">
-        <v>90.1725</v>
+        <v>95.51000000000001</v>
       </c>
       <c r="V21" s="117" t="n">
-        <v>-29.8275</v>
+        <v>-24.48999999999999</v>
       </c>
       <c r="W21" s="120" t="inlineStr"/>
     </row>
@@ -2200,34 +2200,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>30.24193548387097</v>
+        <v>32.66129032258065</v>
       </c>
       <c r="N22" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-8.241935483870968</v>
+        <v>-10.66129032258065</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>1209.677419354839</v>
+        <v>1306.451612903226</v>
       </c>
       <c r="R22" s="117" t="n">
-        <v>1357.706658</v>
+        <v>1414.698441</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>148.0292386451613</v>
+        <v>108.2468280967742</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>0.1223708372799999</v>
+        <v>0.08285559681481471</v>
       </c>
       <c r="U22" s="117" t="n">
-        <v>61.713939</v>
+        <v>64.30447459090909</v>
       </c>
       <c r="V22" s="117" t="n">
-        <v>21.713939</v>
+        <v>24.30447459090909</v>
       </c>
       <c r="W22" s="120" t="inlineStr"/>
     </row>
@@ -2279,34 +2279,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>80.64516129032258</v>
+        <v>87.09677419354838</v>
       </c>
       <c r="N23" s="119" t="n">
         <v>114</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>33.35483870967742</v>
+        <v>26.90322580645162</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>1209.677419354839</v>
+        <v>1306.451612903226</v>
       </c>
       <c r="R23" s="117" t="n">
-        <v>1816.561969</v>
+        <v>1928.318895</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>606.8845496451613</v>
+        <v>621.8672820967743</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.5016912277066666</v>
+        <v>0.4759971788888889</v>
       </c>
       <c r="U23" s="117" t="n">
-        <v>15.93475411403509</v>
+        <v>16.91507802631579</v>
       </c>
       <c r="V23" s="117" t="n">
-        <v>0.9347541140350888</v>
+        <v>1.91507802631579</v>
       </c>
       <c r="W23" s="120" t="inlineStr">
         <is>
@@ -2362,34 +2362,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>31.01736972704714</v>
+        <v>33.49875930521092</v>
       </c>
       <c r="N24" s="119" t="n">
         <v>67</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>35.98263027295285</v>
+        <v>33.50124069478908</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>806.4516129032259</v>
+        <v>870.9677419354839</v>
       </c>
       <c r="R24" s="117" t="n">
-        <v>1224.02</v>
+        <v>1252.69</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>417.5683870967741</v>
+        <v>381.7222580645162</v>
       </c>
       <c r="T24" s="118" t="n">
-        <v>0.5177847999999999</v>
+        <v>0.4382737037037037</v>
       </c>
       <c r="U24" s="117" t="n">
-        <v>18.2689552238806</v>
+        <v>18.69686567164179</v>
       </c>
       <c r="V24" s="117" t="n">
-        <v>-7.731044776119404</v>
+        <v>-7.303134328358208</v>
       </c>
       <c r="W24" s="120" t="inlineStr"/>
     </row>
@@ -2436,12 +2436,12 @@
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>581.75</v>
+        <v>669.92</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
       <c r="U25" s="117" t="n">
-        <v>581.75</v>
+        <v>669.92</v>
       </c>
       <c r="V25" s="117" t="n"/>
       <c r="W25" s="120" t="inlineStr"/>
@@ -2478,34 +2478,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>1102.192256695777</v>
+        <v>1190.367637231439</v>
       </c>
       <c r="N26" s="125" t="n">
         <v>967</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>-135.1922566957771</v>
+        <v>-223.3676372314394</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>25000</v>
+        <v>27000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>30118.911634</v>
+        <v>31657.832734</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>5118.911634</v>
+        <v>4657.832734</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>0.20475646536</v>
+        <v>0.1725123234814814</v>
       </c>
       <c r="U26" s="123" t="n">
-        <v>31.1467545336091</v>
+        <v>32.73819310651499</v>
       </c>
       <c r="V26" s="123" t="n">
-        <v>8.464686275439146</v>
+        <v>10.05612484834504</v>
       </c>
       <c r="W26" s="126" t="n"/>
     </row>
@@ -2553,28 +2553,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>530.5602716468592</v>
+        <v>573.0050933786079</v>
       </c>
       <c r="N27" s="119" t="n">
         <v>371</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-159.5602716468592</v>
+        <v>-202.0050933786079</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>3913.04347826087</v>
+        <v>4130.434782608696</v>
       </c>
       <c r="R27" s="117" t="n">
         <v>2819.6</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-1093.44347826087</v>
+        <v>-1310.834782608696</v>
       </c>
       <c r="T27" s="118" t="n">
-        <v>-0.2794355555555555</v>
+        <v>-0.3173600000000001</v>
       </c>
       <c r="U27" s="117" t="n">
         <v>7.6</v>
@@ -2628,28 +2628,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>358.4229390681004</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="N28" s="119" t="n">
         <v>187</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-171.4229390681004</v>
+        <v>-200.0967741935484</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>3130.434782608696</v>
+        <v>3304.347826086957</v>
       </c>
       <c r="R28" s="117" t="n">
         <v>1683</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-1447.434782608696</v>
+        <v>-1621.347826086957</v>
       </c>
       <c r="T28" s="118" t="n">
-        <v>-0.462375</v>
+        <v>-0.4906710526315789</v>
       </c>
       <c r="U28" s="117" t="n">
         <v>9</v>
@@ -2703,28 +2703,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>201.6129032258065</v>
+        <v>217.7419354838709</v>
       </c>
       <c r="N29" s="119" t="n">
         <v>240</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>38.38709677419354</v>
+        <v>22.25806451612902</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>1565.217391304348</v>
+        <v>1652.173913043478</v>
       </c>
       <c r="R29" s="117" t="n">
         <v>1920</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>354.782608695652</v>
+        <v>267.8260869565217</v>
       </c>
       <c r="T29" s="118" t="n">
-        <v>0.2266666666666665</v>
+        <v>0.1621052631578947</v>
       </c>
       <c r="U29" s="117" t="n">
         <v>8</v>
@@ -2766,28 +2766,28 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>1090.596113940766</v>
+        <v>1177.843803056027</v>
       </c>
       <c r="N30" s="125" t="n">
         <v>798</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-292.5961139407659</v>
+        <v>-379.8438030560274</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>8608.695652173914</v>
+        <v>9086.95652173913</v>
       </c>
       <c r="R30" s="123" t="n">
         <v>6422.6</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>-2186.095652173913</v>
+        <v>-2664.35652173913</v>
       </c>
       <c r="T30" s="124" t="n">
-        <v>-0.2539404040404041</v>
+        <v>-0.2932066985645932</v>
       </c>
       <c r="U30" s="123" t="n">
         <v>8.048370927318297</v>
@@ -2829,34 +2829,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="133" t="n">
-        <v>2569.132456658048</v>
+        <v>2774.663053190693</v>
       </c>
       <c r="N31" s="133" t="n">
         <v>2093</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>-476.1324566580483</v>
+        <v>-681.6630531906926</v>
       </c>
       <c r="P31" s="131" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="Q31" s="131" t="n">
-        <v>50544.17952314165</v>
+        <v>54377.27910238429</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>52580.998751</v>
+        <v>54593.076217</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>2036.819227858345</v>
+        <v>215.797114615707</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>0.0402977998075087</v>
+        <v>0.0039685162291661</v>
       </c>
       <c r="U31" s="131" t="n">
-        <v>25.12231187338748</v>
+        <v>26.08364845532728</v>
       </c>
       <c r="V31" s="131" t="n">
-        <v>5.346588951342142</v>
+        <v>6.307925533281942</v>
       </c>
       <c r="W31" s="134" t="n"/>
     </row>
@@ -3137,13 +3137,13 @@
         </is>
       </c>
       <c r="B2" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C2" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D2" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3180,16 +3180,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="137" t="n">
-        <v>7661.290322580645</v>
+        <v>8274.193548387097</v>
       </c>
       <c r="V2" s="137" t="n">
-        <v>7807.164287</v>
+        <v>8077.867025</v>
       </c>
       <c r="W2" s="137" t="n">
-        <v>145.8739644193547</v>
+        <v>-196.326523387097</v>
       </c>
       <c r="X2" s="138" t="n">
-        <v>0.0190403911452631</v>
+        <v>-0.0237275720272904</v>
       </c>
       <c r="Y2" s="137" t="n"/>
       <c r="Z2" s="137" t="n"/>
@@ -3223,13 +3223,13 @@
         </is>
       </c>
       <c r="B3" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C3" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D3" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3290,13 +3290,13 @@
         </is>
       </c>
       <c r="B4" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C4" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D4" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3333,16 +3333,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="137" t="n">
-        <v>1209.677419354839</v>
+        <v>1306.451612903226</v>
       </c>
       <c r="V4" s="137" t="n">
-        <v>1327.24283</v>
+        <v>1368.086458</v>
       </c>
       <c r="W4" s="137" t="n">
-        <v>117.5654106451611</v>
+        <v>61.63484509677414</v>
       </c>
       <c r="X4" s="138" t="n">
-        <v>0.0971874061333332</v>
+        <v>0.0471772888395061</v>
       </c>
       <c r="Y4" s="137" t="n"/>
       <c r="Z4" s="137" t="n"/>
@@ -3376,13 +3376,13 @@
         </is>
       </c>
       <c r="B5" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C5" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D5" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3443,13 +3443,13 @@
         </is>
       </c>
       <c r="B6" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C6" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D6" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3486,16 +3486,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="137" t="n">
-        <v>8064.516129032258</v>
+        <v>8709.677419354839</v>
       </c>
       <c r="V6" s="137" t="n">
-        <v>6905.08</v>
+        <v>7066.69</v>
       </c>
       <c r="W6" s="137" t="n">
-        <v>-1159.436129032258</v>
+        <v>-1642.987419354839</v>
       </c>
       <c r="X6" s="138" t="n">
-        <v>-0.1437700799999999</v>
+        <v>-0.1886392962962963</v>
       </c>
       <c r="Y6" s="137" t="n"/>
       <c r="Z6" s="137" t="n"/>
@@ -3529,13 +3529,13 @@
         </is>
       </c>
       <c r="B7" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C7" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D7" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -3582,28 +3582,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>530.5602716468592</v>
+        <v>573.0050933786079</v>
       </c>
       <c r="R7" t="n">
         <v>371</v>
       </c>
       <c r="S7" t="n">
-        <v>-159.5602716468592</v>
+        <v>-202.0050933786079</v>
       </c>
       <c r="T7" s="137" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="U7" s="137" t="n">
-        <v>3913.04347826087</v>
+        <v>4130.434782608696</v>
       </c>
       <c r="V7" s="137" t="n">
         <v>2819.6</v>
       </c>
       <c r="W7" s="137" t="n">
-        <v>-1093.44347826087</v>
+        <v>-1310.834782608696</v>
       </c>
       <c r="X7" s="138" t="n">
-        <v>-0.2794355555555555</v>
+        <v>-0.3173600000000001</v>
       </c>
       <c r="Y7" s="137" t="n">
         <v>7.6</v>
@@ -3632,13 +3632,13 @@
         </is>
       </c>
       <c r="B8" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C8" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D8" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E8" t="n">
         <v>26</v>
@@ -3685,28 +3685,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>358.4229390681004</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="R8" t="n">
         <v>187</v>
       </c>
       <c r="S8" t="n">
-        <v>-171.4229390681004</v>
+        <v>-200.0967741935484</v>
       </c>
       <c r="T8" s="137" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="U8" s="137" t="n">
-        <v>3130.434782608696</v>
+        <v>3304.347826086957</v>
       </c>
       <c r="V8" s="137" t="n">
         <v>1683</v>
       </c>
       <c r="W8" s="137" t="n">
-        <v>-1447.434782608696</v>
+        <v>-1621.347826086957</v>
       </c>
       <c r="X8" s="138" t="n">
-        <v>-0.462375</v>
+        <v>-0.4906710526315789</v>
       </c>
       <c r="Y8" s="137" t="n">
         <v>9</v>
@@ -3735,13 +3735,13 @@
         </is>
       </c>
       <c r="B9" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C9" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D9" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3788,28 +3788,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>201.6129032258065</v>
+        <v>217.7419354838709</v>
       </c>
       <c r="R9" t="n">
         <v>240</v>
       </c>
       <c r="S9" t="n">
-        <v>38.38709677419354</v>
+        <v>22.25806451612902</v>
       </c>
       <c r="T9" s="137" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="U9" s="137" t="n">
-        <v>1565.217391304348</v>
+        <v>1652.173913043478</v>
       </c>
       <c r="V9" s="137" t="n">
         <v>1920</v>
       </c>
       <c r="W9" s="137" t="n">
-        <v>354.782608695652</v>
+        <v>267.8260869565217</v>
       </c>
       <c r="X9" s="138" t="n">
-        <v>0.2266666666666665</v>
+        <v>0.1621052631578947</v>
       </c>
       <c r="Y9" s="137" t="n">
         <v>8</v>
@@ -3838,13 +3838,13 @@
         </is>
       </c>
       <c r="B10" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C10" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D10" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3891,34 +3891,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>94.87666034155598</v>
+        <v>102.4667931688805</v>
       </c>
       <c r="R10" t="n">
         <v>111</v>
       </c>
       <c r="S10" t="n">
-        <v>16.12333965844402</v>
+        <v>8.533206831119543</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U10" s="137" t="n">
-        <v>3225.806451612903</v>
+        <v>3483.870967741936</v>
       </c>
       <c r="V10" s="137" t="n">
-        <v>3881.173415</v>
+        <v>4033.470302</v>
       </c>
       <c r="W10" s="137" t="n">
-        <v>655.3669633870968</v>
+        <v>549.5993342580646</v>
       </c>
       <c r="X10" s="138" t="n">
-        <v>0.20316375865</v>
+        <v>0.1577553644629629</v>
       </c>
       <c r="Y10" s="137" t="n">
-        <v>34.96552626126126</v>
+        <v>36.33757028828829</v>
       </c>
       <c r="Z10" s="137" t="n">
-        <v>0.9655262612612604</v>
+        <v>2.33757028828829</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -3950,13 +3950,13 @@
         </is>
       </c>
       <c r="B11" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C11" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D11" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -4003,34 +4003,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q11" t="n">
-        <v>188.5211562630917</v>
+        <v>203.6028487641391</v>
       </c>
       <c r="R11" t="n">
         <v>61</v>
       </c>
       <c r="S11" t="n">
-        <v>-20.52115626309174</v>
+        <v>-35.60284876413908</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U11" s="137" t="n">
-        <v>7258.064516129032</v>
+        <v>7838.709677419354</v>
       </c>
       <c r="V11" s="137" t="n">
-        <v>7595.101119000001</v>
+        <v>7997.154267</v>
       </c>
       <c r="W11" s="137" t="n">
-        <v>337.0366028709686</v>
+        <v>158.4445895806457</v>
       </c>
       <c r="X11" s="138" t="n">
-        <v>0.0464361541733334</v>
+        <v>0.0202130957901235</v>
       </c>
       <c r="Y11" s="137" t="n">
-        <v>45.20893523214286</v>
+        <v>47.60210873214286</v>
       </c>
       <c r="Z11" s="137" t="n">
-        <v>6.708935232142864</v>
+        <v>9.10210873214286</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -4062,13 +4062,13 @@
         </is>
       </c>
       <c r="B12" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C12" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D12" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -4132,13 +4132,13 @@
         </is>
       </c>
       <c r="B13" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C13" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D13" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4185,34 +4185,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>21.22241086587436</v>
+        <v>22.92020373514431</v>
       </c>
       <c r="R13" t="n">
         <v>5</v>
       </c>
       <c r="S13" t="n">
-        <v>-11.22241086587436</v>
+        <v>-12.92020373514431</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="137" t="n">
-        <v>806.4516129032259</v>
+        <v>870.9677419354839</v>
       </c>
       <c r="V13" s="137" t="n">
-        <v>790.9651590000001</v>
+        <v>853.4385040000001</v>
       </c>
       <c r="W13" s="137" t="n">
-        <v>-15.48645390322576</v>
+        <v>-17.52923793548382</v>
       </c>
       <c r="X13" s="138" t="n">
-        <v>-0.0192032028399999</v>
+        <v>-0.020126162074074</v>
       </c>
       <c r="Y13" s="137" t="n">
-        <v>79.09651590000001</v>
+        <v>85.34385040000001</v>
       </c>
       <c r="Z13" s="137" t="n">
-        <v>41.09651590000001</v>
+        <v>47.34385040000001</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -4244,13 +4244,13 @@
         </is>
       </c>
       <c r="B14" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C14" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D14" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
@@ -4314,13 +4314,13 @@
         </is>
       </c>
       <c r="B15" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C15" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D15" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -4367,34 +4367,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q15" t="n">
-        <v>3.225806451612903</v>
+        <v>3.483870967741935</v>
       </c>
       <c r="R15" t="n">
         <v>2</v>
       </c>
       <c r="S15" t="n">
-        <v>-1.225806451612903</v>
+        <v>-1.483870967741935</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U15" s="137" t="n">
-        <v>806.4516129032259</v>
+        <v>870.9677419354839</v>
       </c>
       <c r="V15" s="137" t="n">
-        <v>823.103314</v>
+        <v>875.3623249999999</v>
       </c>
       <c r="W15" s="137" t="n">
-        <v>16.6517010967741</v>
+        <v>4.394583064516041</v>
       </c>
       <c r="X15" s="138" t="n">
-        <v>0.0206481093599998</v>
+        <v>0.0050456324074073</v>
       </c>
       <c r="Y15" s="137" t="n">
-        <v>411.551657</v>
+        <v>437.6811625</v>
       </c>
       <c r="Z15" s="137" t="n">
-        <v>161.551657</v>
+        <v>187.6811625</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -4426,13 +4426,13 @@
         </is>
       </c>
       <c r="B16" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C16" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D16" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4496,13 +4496,13 @@
         </is>
       </c>
       <c r="B17" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C17" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D17" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E17" t="n">
         <v>17</v>
@@ -4549,34 +4549,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>630.0403225806452</v>
+        <v>680.4435483870968</v>
       </c>
       <c r="R17" t="n">
         <v>417</v>
       </c>
       <c r="S17" t="n">
-        <v>-213.0403225806452</v>
+        <v>-263.4435483870968</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U17" s="137" t="n">
-        <v>8064.516129032258</v>
+        <v>8709.677419354839</v>
       </c>
       <c r="V17" s="137" t="n">
-        <v>10569.57</v>
+        <v>11088.19</v>
       </c>
       <c r="W17" s="137" t="n">
-        <v>2505.053870967742</v>
+        <v>2378.512580645161</v>
       </c>
       <c r="X17" s="138" t="n">
-        <v>0.31062668</v>
+        <v>0.2730884814814815</v>
       </c>
       <c r="Y17" s="137" t="n">
-        <v>25.34669064748201</v>
+        <v>26.59038369304556</v>
       </c>
       <c r="Z17" s="137" t="n">
-        <v>12.54669064748201</v>
+        <v>13.79038369304556</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -4608,13 +4608,13 @@
         </is>
       </c>
       <c r="B18" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C18" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D18" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4661,34 +4661,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>10.08064516129032</v>
+        <v>10.88709677419355</v>
       </c>
       <c r="R18" t="n">
         <v>32</v>
       </c>
       <c r="S18" t="n">
-        <v>21.91935483870968</v>
+        <v>21.11290322580645</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="137" t="n">
-        <v>403.2258064516129</v>
+        <v>435.483870967742</v>
       </c>
       <c r="V18" s="137" t="n">
-        <v>401.82</v>
+        <v>426.16</v>
       </c>
       <c r="W18" s="137" t="n">
-        <v>-1.405806451612932</v>
+        <v>-9.323870967741923</v>
       </c>
       <c r="X18" s="138" t="n">
-        <v>-0.0034864</v>
+        <v>-0.0214103703703703</v>
       </c>
       <c r="Y18" s="137" t="n">
-        <v>12.556875</v>
+        <v>13.3175</v>
       </c>
       <c r="Z18" s="137" t="n">
-        <v>-27.443125</v>
+        <v>-26.6825</v>
       </c>
       <c r="AB18" s="139" t="inlineStr"/>
       <c r="AC18" s="139" t="inlineStr">
@@ -4715,13 +4715,13 @@
         </is>
       </c>
       <c r="B19" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C19" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D19" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4768,34 +4768,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>8.960573476702509</v>
+        <v>9.67741935483871</v>
       </c>
       <c r="R19" t="n">
         <v>19</v>
       </c>
       <c r="S19" t="n">
-        <v>10.03942652329749</v>
+        <v>9.32258064516129</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="137" t="n">
-        <v>806.4516129032259</v>
+        <v>870.9677419354839</v>
       </c>
       <c r="V19" s="137" t="n">
-        <v>716.45</v>
+        <v>736.39</v>
       </c>
       <c r="W19" s="137" t="n">
-        <v>-90.0016129032258</v>
+        <v>-134.5777419354839</v>
       </c>
       <c r="X19" s="138" t="n">
-        <v>-0.1116019999999999</v>
+        <v>-0.1545151851851852</v>
       </c>
       <c r="Y19" s="137" t="n">
-        <v>37.70789473684211</v>
+        <v>38.75736842105263</v>
       </c>
       <c r="Z19" s="137" t="n">
-        <v>-52.29210526315789</v>
+        <v>-51.24263157894737</v>
       </c>
       <c r="AB19" s="139" t="inlineStr"/>
       <c r="AC19" s="139" t="inlineStr">
@@ -4822,13 +4822,13 @@
         </is>
       </c>
       <c r="B20" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C20" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D20" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
@@ -4875,34 +4875,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>3.360215053763441</v>
+        <v>3.629032258064517</v>
       </c>
       <c r="R20" t="n">
         <v>4</v>
       </c>
       <c r="S20" t="n">
-        <v>0.6397849462365586</v>
+        <v>0.3709677419354835</v>
       </c>
       <c r="T20" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U20" s="137" t="n">
-        <v>403.2258064516129</v>
+        <v>435.483870967742</v>
       </c>
       <c r="V20" s="137" t="n">
-        <v>360.69</v>
+        <v>382.04</v>
       </c>
       <c r="W20" s="137" t="n">
-        <v>-42.53580645161293</v>
+        <v>-53.44387096774193</v>
       </c>
       <c r="X20" s="138" t="n">
-        <v>-0.1054888</v>
+        <v>-0.1227229629629629</v>
       </c>
       <c r="Y20" s="137" t="n">
-        <v>90.1725</v>
+        <v>95.51000000000001</v>
       </c>
       <c r="Z20" s="137" t="n">
-        <v>-29.8275</v>
+        <v>-24.48999999999999</v>
       </c>
       <c r="AB20" s="139" t="inlineStr"/>
       <c r="AC20" s="139" t="inlineStr">
@@ -4929,13 +4929,13 @@
         </is>
       </c>
       <c r="B21" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C21" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D21" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4982,34 +4982,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>30.24193548387097</v>
+        <v>32.66129032258065</v>
       </c>
       <c r="R21" t="n">
         <v>22</v>
       </c>
       <c r="S21" t="n">
-        <v>-8.241935483870968</v>
+        <v>-10.66129032258065</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="137" t="n">
-        <v>1209.677419354839</v>
+        <v>1306.451612903226</v>
       </c>
       <c r="V21" s="137" t="n">
-        <v>1357.706658</v>
+        <v>1414.698441</v>
       </c>
       <c r="W21" s="137" t="n">
-        <v>148.0292386451613</v>
+        <v>108.2468280967742</v>
       </c>
       <c r="X21" s="138" t="n">
-        <v>0.1223708372799999</v>
+        <v>0.08285559681481471</v>
       </c>
       <c r="Y21" s="137" t="n">
-        <v>61.713939</v>
+        <v>64.30447459090909</v>
       </c>
       <c r="Z21" s="137" t="n">
-        <v>21.713939</v>
+        <v>24.30447459090909</v>
       </c>
       <c r="AB21" s="139" t="inlineStr">
         <is>
@@ -5036,13 +5036,13 @@
         </is>
       </c>
       <c r="B22" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C22" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D22" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -5089,34 +5089,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>80.64516129032258</v>
+        <v>87.09677419354838</v>
       </c>
       <c r="R22" t="n">
         <v>114</v>
       </c>
       <c r="S22" t="n">
-        <v>33.35483870967742</v>
+        <v>26.90322580645162</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="137" t="n">
-        <v>1209.677419354839</v>
+        <v>1306.451612903226</v>
       </c>
       <c r="V22" s="137" t="n">
-        <v>1816.561969</v>
+        <v>1928.318895</v>
       </c>
       <c r="W22" s="137" t="n">
-        <v>606.8845496451613</v>
+        <v>621.8672820967743</v>
       </c>
       <c r="X22" s="138" t="n">
-        <v>0.5016912277066666</v>
+        <v>0.4759971788888889</v>
       </c>
       <c r="Y22" s="137" t="n">
-        <v>15.93475411403509</v>
+        <v>16.91507802631579</v>
       </c>
       <c r="Z22" s="137" t="n">
-        <v>0.9347541140350888</v>
+        <v>1.91507802631579</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -5148,13 +5148,13 @@
         </is>
       </c>
       <c r="B23" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C23" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D23" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5201,34 +5201,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>31.01736972704714</v>
+        <v>33.49875930521092</v>
       </c>
       <c r="R23" t="n">
         <v>67</v>
       </c>
       <c r="S23" t="n">
-        <v>35.98263027295285</v>
+        <v>33.50124069478908</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="137" t="n">
-        <v>806.4516129032259</v>
+        <v>870.9677419354839</v>
       </c>
       <c r="V23" s="137" t="n">
-        <v>1224.02</v>
+        <v>1252.69</v>
       </c>
       <c r="W23" s="137" t="n">
-        <v>417.5683870967741</v>
+        <v>381.7222580645162</v>
       </c>
       <c r="X23" s="138" t="n">
-        <v>0.5177847999999999</v>
+        <v>0.4382737037037037</v>
       </c>
       <c r="Y23" s="137" t="n">
-        <v>18.2689552238806</v>
+        <v>18.69686567164179</v>
       </c>
       <c r="Z23" s="137" t="n">
-        <v>-7.731044776119404</v>
+        <v>-7.303134328358208</v>
       </c>
       <c r="AB23" s="139" t="inlineStr"/>
       <c r="AC23" s="139" t="inlineStr">
@@ -5255,13 +5255,13 @@
         </is>
       </c>
       <c r="B24" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C24" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D24" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5298,12 +5298,12 @@
       <c r="T24" s="137" t="n"/>
       <c r="U24" s="137" t="n"/>
       <c r="V24" s="137" t="n">
-        <v>581.75</v>
+        <v>669.92</v>
       </c>
       <c r="W24" s="137" t="n"/>
       <c r="X24" s="138" t="n"/>
       <c r="Y24" s="137" t="n">
-        <v>581.75</v>
+        <v>669.92</v>
       </c>
       <c r="Z24" s="137" t="n"/>
       <c r="AB24" s="139" t="inlineStr"/>
@@ -5331,13 +5331,13 @@
         </is>
       </c>
       <c r="B25" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C25" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D25" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5366,34 +5366,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>376.3440860215054</v>
+        <v>406.4516129032259</v>
       </c>
       <c r="R25" t="n">
         <v>328</v>
       </c>
       <c r="S25" t="n">
-        <v>-48.3440860215054</v>
+        <v>-78.45161290322585</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="137" t="n">
-        <v>16935.48387096774</v>
+        <v>18290.32258064516</v>
       </c>
       <c r="V25" s="137" t="n">
-        <v>16039.487117</v>
+        <v>16512.643483</v>
       </c>
       <c r="W25" s="137" t="n">
-        <v>-895.9967539677436</v>
+        <v>-1777.679097645163</v>
       </c>
       <c r="X25" s="138" t="n">
-        <v>-0.0529064749961905</v>
+        <v>-0.09719233161728399</v>
       </c>
       <c r="Y25" s="137" t="n">
-        <v>48.90087535670731</v>
+        <v>50.34342525304878</v>
       </c>
       <c r="Z25" s="137" t="n">
-        <v>3.90087535670731</v>
+        <v>5.343425253048778</v>
       </c>
       <c r="AB25" s="139" t="inlineStr"/>
       <c r="AC25" s="139" t="inlineStr"/>
@@ -5411,13 +5411,13 @@
         </is>
       </c>
       <c r="B26" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C26" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D26" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5451,34 +5451,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>1102.192256695777</v>
+        <v>1190.367637231439</v>
       </c>
       <c r="R26" t="n">
         <v>967</v>
       </c>
       <c r="S26" t="n">
-        <v>-135.1922566957771</v>
+        <v>-223.3676372314394</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="137" t="n">
-        <v>25000</v>
+        <v>27000</v>
       </c>
       <c r="V26" s="137" t="n">
-        <v>30118.911634</v>
+        <v>31657.832734</v>
       </c>
       <c r="W26" s="137" t="n">
-        <v>5118.911634</v>
+        <v>4657.832734</v>
       </c>
       <c r="X26" s="138" t="n">
-        <v>0.20475646536</v>
+        <v>0.1725123234814814</v>
       </c>
       <c r="Y26" s="137" t="n">
-        <v>31.1467545336091</v>
+        <v>32.73819310651499</v>
       </c>
       <c r="Z26" s="137" t="n">
-        <v>8.464686275439146</v>
+        <v>10.05612484834504</v>
       </c>
       <c r="AB26" s="139" t="inlineStr"/>
       <c r="AC26" s="139" t="inlineStr"/>
@@ -5496,13 +5496,13 @@
         </is>
       </c>
       <c r="B27" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C27" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D27" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5536,28 +5536,28 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>1090.596113940766</v>
+        <v>1177.843803056027</v>
       </c>
       <c r="R27" t="n">
         <v>798</v>
       </c>
       <c r="S27" t="n">
-        <v>-292.5961139407659</v>
+        <v>-379.8438030560274</v>
       </c>
       <c r="T27" s="137" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="U27" s="137" t="n">
-        <v>8608.695652173914</v>
+        <v>9086.95652173913</v>
       </c>
       <c r="V27" s="137" t="n">
         <v>6422.6</v>
       </c>
       <c r="W27" s="137" t="n">
-        <v>-2186.095652173913</v>
+        <v>-2664.35652173913</v>
       </c>
       <c r="X27" s="138" t="n">
-        <v>-0.2539404040404041</v>
+        <v>-0.2932066985645932</v>
       </c>
       <c r="Y27" s="137" t="n">
         <v>8.048370927318297</v>
@@ -5581,13 +5581,13 @@
         </is>
       </c>
       <c r="B28" s="136" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="C28" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D28" s="136" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5621,34 +5621,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>2569.132456658048</v>
+        <v>2774.663053190693</v>
       </c>
       <c r="R28" t="n">
         <v>2093</v>
       </c>
       <c r="S28" t="n">
-        <v>-476.1324566580483</v>
+        <v>-681.6630531906926</v>
       </c>
       <c r="T28" s="137" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="U28" s="137" t="n">
-        <v>50544.17952314165</v>
+        <v>54377.27910238429</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>52580.998751</v>
+        <v>54593.076217</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>2036.819227858345</v>
+        <v>215.797114615707</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>0.0402977998075087</v>
+        <v>0.0039685162291661</v>
       </c>
       <c r="Y28" s="137" t="n">
-        <v>25.12231187338748</v>
+        <v>26.08364845532728</v>
       </c>
       <c r="Z28" s="137" t="n">
-        <v>5.346588951342142</v>
+        <v>6.307925533281942</v>
       </c>
       <c r="AB28" s="139" t="inlineStr"/>
       <c r="AC28" s="139" t="inlineStr"/>
@@ -5751,7 +5751,7 @@
         </is>
       </c>
       <c r="B4" s="140" t="n">
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5791,7 +5791,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5811,7 +5811,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46229.29190972223</v>
+        <v>46231.29190972223</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-07-29
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 27/07/2026  |  Ultimo aggiornamento: 28/07/2026 07:00</t>
+          <t>Periodo: 01/07/2026 - 28/07/2026  |  Ultimo aggiornamento: 29/07/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1065,16 +1065,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>8274.193548387097</v>
+        <v>8580.645161290322</v>
       </c>
       <c r="R5" s="117" t="n">
         <v>8077.867025</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>-196.326523387097</v>
+        <v>-502.7781362903224</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>-0.0237275720272904</v>
+        <v>-0.0585944444548872</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1173,16 +1173,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>1306.451612903226</v>
+        <v>1354.83870967742</v>
       </c>
       <c r="R7" s="117" t="n">
         <v>1368.086458</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>61.63484509677414</v>
+        <v>13.24774832258049</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>0.0471772888395061</v>
+        <v>0.009778099952380799</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1281,16 +1281,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>8709.677419354839</v>
+        <v>9032.258064516129</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>7066.69</v>
+        <v>7185.39</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-1642.987419354839</v>
+        <v>-1846.868064516128</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.1886392962962963</v>
+        <v>-0.2044746785714285</v>
       </c>
       <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
@@ -1328,34 +1328,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>406.4516129032259</v>
+        <v>421.505376344086</v>
       </c>
       <c r="N10" s="125" t="n">
         <v>328</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>-78.45161290322585</v>
+        <v>-93.50537634408602</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>18290.32258064516</v>
+        <v>18967.74193548387</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>16512.643483</v>
+        <v>16631.343483</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>-1777.679097645163</v>
+        <v>-2336.39845248387</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>-0.09719233161728399</v>
+        <v>-0.1231774694336734</v>
       </c>
       <c r="U10" s="123" t="n">
-        <v>50.34342525304878</v>
+        <v>50.70531549695122</v>
       </c>
       <c r="V10" s="123" t="n">
-        <v>5.343425253048778</v>
+        <v>5.705315496951222</v>
       </c>
       <c r="W10" s="126" t="n"/>
     </row>
@@ -1407,28 +1407,28 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>102.4667931688805</v>
+        <v>106.2618595825427</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>111</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>8.533206831119543</v>
+        <v>4.738140417457316</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>3483.870967741936</v>
+        <v>3612.903225806452</v>
       </c>
       <c r="R11" s="117" t="n">
         <v>4033.470302</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>549.5993342580646</v>
+        <v>420.5670761935485</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.1577553644629629</v>
+        <v>0.1164069585892857</v>
       </c>
       <c r="U11" s="117" t="n">
         <v>36.33757028828829</v>
@@ -1490,28 +1490,28 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M12" s="127" t="n">
-        <v>203.6028487641391</v>
+        <v>211.1436950146628</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>61</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>-35.60284876413908</v>
+        <v>-43.14369501466274</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>7838.709677419354</v>
+        <v>8129.032258064516</v>
       </c>
       <c r="R12" s="117" t="n">
         <v>7997.154267</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>158.4445895806457</v>
+        <v>-131.8779910645162</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>0.0202130957901235</v>
+        <v>-0.0162230862023809</v>
       </c>
       <c r="U12" s="128" t="n">
         <v>47.60210873214286</v>
@@ -1620,28 +1620,28 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="127" t="n">
-        <v>22.92020373514431</v>
+        <v>23.76910016977929</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>5</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-12.92020373514431</v>
+        <v>-13.76910016977929</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>870.9677419354839</v>
+        <v>903.2258064516128</v>
       </c>
       <c r="R14" s="117" t="n">
         <v>853.4385040000001</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-17.52923793548382</v>
+        <v>-49.78730245161285</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.020126162074074</v>
+        <v>-0.0551216562857142</v>
       </c>
       <c r="U14" s="128" t="n">
         <v>85.34385040000001</v>
@@ -1750,28 +1750,28 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M16" s="127" t="n">
-        <v>3.483870967741935</v>
+        <v>3.612903225806452</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>-1.483870967741935</v>
+        <v>-1.612903225806452</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>870.9677419354839</v>
+        <v>903.2258064516128</v>
       </c>
       <c r="R16" s="117" t="n">
         <v>875.3623249999999</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>4.394583064516041</v>
+        <v>-27.86348145161298</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.0050456324074073</v>
+        <v>-0.0308488544642858</v>
       </c>
       <c r="U16" s="128" t="n">
         <v>437.6811625</v>
@@ -1880,34 +1880,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>680.4435483870968</v>
+        <v>705.6451612903227</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>417</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-263.4435483870968</v>
+        <v>-288.6451612903227</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>8709.677419354839</v>
+        <v>9032.258064516129</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>11088.19</v>
+        <v>11267.67</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>2378.512580645161</v>
+        <v>2235.411935483872</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>0.2730884814814815</v>
+        <v>0.2474920357142857</v>
       </c>
       <c r="U18" s="117" t="n">
-        <v>26.59038369304556</v>
+        <v>27.02079136690648</v>
       </c>
       <c r="V18" s="117" t="n">
-        <v>13.79038369304556</v>
+        <v>14.22079136690648</v>
       </c>
       <c r="W18" s="120" t="inlineStr">
         <is>
@@ -1963,34 +1963,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>10.88709677419355</v>
+        <v>11.29032258064516</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>32</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>21.11290322580645</v>
+        <v>20.70967741935484</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>435.483870967742</v>
+        <v>451.6129032258065</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>426.16</v>
+        <v>431.64</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-9.323870967741923</v>
+        <v>-19.97290322580648</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.0214103703703703</v>
+        <v>-0.0442257142857143</v>
       </c>
       <c r="U19" s="117" t="n">
-        <v>13.3175</v>
+        <v>13.48875</v>
       </c>
       <c r="V19" s="117" t="n">
-        <v>-26.6825</v>
+        <v>-26.51125</v>
       </c>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
@@ -2042,34 +2042,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>9.67741935483871</v>
+        <v>10.03584229390681</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>9.32258064516129</v>
+        <v>8.964157706093189</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>870.9677419354839</v>
+        <v>903.2258064516128</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>736.39</v>
+        <v>742.34</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-134.5777419354839</v>
+        <v>-160.8858064516129</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.1545151851851852</v>
+        <v>-0.1781235714285714</v>
       </c>
       <c r="U20" s="117" t="n">
-        <v>38.75736842105263</v>
+        <v>39.07052631578947</v>
       </c>
       <c r="V20" s="117" t="n">
-        <v>-51.24263157894737</v>
+        <v>-50.92947368421053</v>
       </c>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
@@ -2121,34 +2121,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>3.629032258064517</v>
+        <v>3.763440860215054</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>4</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>0.3709677419354835</v>
+        <v>0.2365591397849455</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>435.483870967742</v>
+        <v>451.6129032258065</v>
       </c>
       <c r="R21" s="117" t="n">
-        <v>382.04</v>
+        <v>387.91</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-53.44387096774193</v>
+        <v>-63.70290322580644</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.1227229629629629</v>
+        <v>-0.1410564285714285</v>
       </c>
       <c r="U21" s="117" t="n">
-        <v>95.51000000000001</v>
+        <v>96.97750000000001</v>
       </c>
       <c r="V21" s="117" t="n">
-        <v>-24.48999999999999</v>
+        <v>-23.0225</v>
       </c>
       <c r="W21" s="120" t="inlineStr"/>
     </row>
@@ -2200,28 +2200,28 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>32.66129032258065</v>
+        <v>33.87096774193549</v>
       </c>
       <c r="N22" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-10.66129032258065</v>
+        <v>-11.87096774193549</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>1306.451612903226</v>
+        <v>1354.83870967742</v>
       </c>
       <c r="R22" s="117" t="n">
         <v>1414.698441</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>108.2468280967742</v>
+        <v>59.8597313225805</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>0.08285559681481471</v>
+        <v>0.044182182642857</v>
       </c>
       <c r="U22" s="117" t="n">
         <v>64.30447459090909</v>
@@ -2279,28 +2279,28 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>87.09677419354838</v>
+        <v>90.32258064516128</v>
       </c>
       <c r="N23" s="119" t="n">
         <v>114</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>26.90322580645162</v>
+        <v>23.67741935483872</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>1306.451612903226</v>
+        <v>1354.83870967742</v>
       </c>
       <c r="R23" s="117" t="n">
         <v>1928.318895</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>621.8672820967743</v>
+        <v>573.4801853225806</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.4759971788888889</v>
+        <v>0.4232829939285714</v>
       </c>
       <c r="U23" s="117" t="n">
         <v>16.91507802631579</v>
@@ -2362,34 +2362,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>33.49875930521092</v>
+        <v>34.7394540942928</v>
       </c>
       <c r="N24" s="119" t="n">
         <v>67</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>33.50124069478908</v>
+        <v>32.2605459057072</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>870.9677419354839</v>
+        <v>903.2258064516128</v>
       </c>
       <c r="R24" s="117" t="n">
-        <v>1252.69</v>
+        <v>1282.1</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>381.7222580645162</v>
+        <v>378.874193548387</v>
       </c>
       <c r="T24" s="118" t="n">
-        <v>0.4382737037037037</v>
+        <v>0.419467857142857</v>
       </c>
       <c r="U24" s="117" t="n">
-        <v>18.69686567164179</v>
+        <v>19.13582089552238</v>
       </c>
       <c r="V24" s="117" t="n">
-        <v>-7.303134328358208</v>
+        <v>-6.864179104477614</v>
       </c>
       <c r="W24" s="120" t="inlineStr"/>
     </row>
@@ -2436,12 +2436,12 @@
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>669.92</v>
+        <v>705.61</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
       <c r="U25" s="117" t="n">
-        <v>669.92</v>
+        <v>705.61</v>
       </c>
       <c r="V25" s="117" t="n"/>
       <c r="W25" s="120" t="inlineStr"/>
@@ -2478,34 +2478,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>1190.367637231439</v>
+        <v>1234.45532749927</v>
       </c>
       <c r="N26" s="125" t="n">
         <v>967</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>-223.3676372314394</v>
+        <v>-267.4553274992704</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>27000</v>
+        <v>28000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>31657.832734</v>
+        <v>31919.712734</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>4657.832734</v>
+        <v>3919.712734000001</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>0.1725123234814814</v>
+        <v>0.1399897405</v>
       </c>
       <c r="U26" s="123" t="n">
-        <v>32.73819310651499</v>
+        <v>33.00901006618408</v>
       </c>
       <c r="V26" s="123" t="n">
-        <v>10.05612484834504</v>
+        <v>10.32694180801412</v>
       </c>
       <c r="W26" s="126" t="n"/>
     </row>
@@ -2553,28 +2553,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>573.0050933786079</v>
+        <v>594.2275042444822</v>
       </c>
       <c r="N27" s="119" t="n">
         <v>371</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-202.0050933786079</v>
+        <v>-223.2275042444822</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>4130.434782608696</v>
+        <v>4347.826086956522</v>
       </c>
       <c r="R27" s="117" t="n">
         <v>2819.6</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-1310.834782608696</v>
+        <v>-1528.226086956522</v>
       </c>
       <c r="T27" s="118" t="n">
-        <v>-0.3173600000000001</v>
+        <v>-0.3514920000000001</v>
       </c>
       <c r="U27" s="117" t="n">
         <v>7.6</v>
@@ -2628,28 +2628,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>387.0967741935484</v>
+        <v>401.4336917562724</v>
       </c>
       <c r="N28" s="119" t="n">
         <v>187</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-200.0967741935484</v>
+        <v>-214.4336917562724</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>3304.347826086957</v>
+        <v>3478.260869565217</v>
       </c>
       <c r="R28" s="117" t="n">
         <v>1683</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-1621.347826086957</v>
+        <v>-1795.260869565217</v>
       </c>
       <c r="T28" s="118" t="n">
-        <v>-0.4906710526315789</v>
+        <v>-0.5161375</v>
       </c>
       <c r="U28" s="117" t="n">
         <v>9</v>
@@ -2703,28 +2703,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>217.7419354838709</v>
+        <v>225.8064516129032</v>
       </c>
       <c r="N29" s="119" t="n">
         <v>240</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>22.25806451612902</v>
+        <v>14.19354838709677</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>1652.173913043478</v>
+        <v>1739.130434782609</v>
       </c>
       <c r="R29" s="117" t="n">
         <v>1920</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>267.8260869565217</v>
+        <v>180.8695652173912</v>
       </c>
       <c r="T29" s="118" t="n">
-        <v>0.1621052631578947</v>
+        <v>0.1039999999999999</v>
       </c>
       <c r="U29" s="117" t="n">
         <v>8</v>
@@ -2766,28 +2766,28 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>1177.843803056027</v>
+        <v>1221.467647613658</v>
       </c>
       <c r="N30" s="125" t="n">
         <v>798</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-379.8438030560274</v>
+        <v>-423.4676476136578</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>9086.95652173913</v>
+        <v>9565.217391304348</v>
       </c>
       <c r="R30" s="123" t="n">
         <v>6422.6</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>-2664.35652173913</v>
+        <v>-3142.617391304348</v>
       </c>
       <c r="T30" s="124" t="n">
-        <v>-0.2932066985645932</v>
+        <v>-0.3285463636363636</v>
       </c>
       <c r="U30" s="123" t="n">
         <v>8.048370927318297</v>
@@ -2829,34 +2829,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="133" t="n">
-        <v>2774.663053190693</v>
+        <v>2877.428351457014</v>
       </c>
       <c r="N31" s="133" t="n">
         <v>2093</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>-681.6630531906926</v>
+        <v>-784.4283514570143</v>
       </c>
       <c r="P31" s="131" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="Q31" s="131" t="n">
-        <v>54377.27910238429</v>
+        <v>56532.95932678822</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>54593.076217</v>
+        <v>54973.656217</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>215.797114615707</v>
+        <v>-1559.303109788212</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>0.0039685162291661</v>
+        <v>-0.027582195030242</v>
       </c>
       <c r="U31" s="131" t="n">
-        <v>26.08364845532728</v>
+        <v>26.26548314237936</v>
       </c>
       <c r="V31" s="131" t="n">
-        <v>6.307925533281942</v>
+        <v>6.489760220334023</v>
       </c>
       <c r="W31" s="134" t="n"/>
     </row>
@@ -3137,13 +3137,13 @@
         </is>
       </c>
       <c r="B2" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C2" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D2" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3180,16 +3180,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="137" t="n">
-        <v>8274.193548387097</v>
+        <v>8580.645161290322</v>
       </c>
       <c r="V2" s="137" t="n">
         <v>8077.867025</v>
       </c>
       <c r="W2" s="137" t="n">
-        <v>-196.326523387097</v>
+        <v>-502.7781362903224</v>
       </c>
       <c r="X2" s="138" t="n">
-        <v>-0.0237275720272904</v>
+        <v>-0.0585944444548872</v>
       </c>
       <c r="Y2" s="137" t="n"/>
       <c r="Z2" s="137" t="n"/>
@@ -3207,7 +3207,7 @@
       <c r="AD2" s="139" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_3;crm:stale</t>
+          <t>google:stale;google:includes_excel_row_3;crm:stale</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -3223,13 +3223,13 @@
         </is>
       </c>
       <c r="B3" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C3" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D3" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3290,13 +3290,13 @@
         </is>
       </c>
       <c r="B4" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C4" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D4" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3333,16 +3333,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="137" t="n">
-        <v>1306.451612903226</v>
+        <v>1354.83870967742</v>
       </c>
       <c r="V4" s="137" t="n">
         <v>1368.086458</v>
       </c>
       <c r="W4" s="137" t="n">
-        <v>61.63484509677414</v>
+        <v>13.24774832258049</v>
       </c>
       <c r="X4" s="138" t="n">
-        <v>0.0471772888395061</v>
+        <v>0.009778099952380799</v>
       </c>
       <c r="Y4" s="137" t="n"/>
       <c r="Z4" s="137" t="n"/>
@@ -3360,7 +3360,7 @@
       <c r="AD4" s="139" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_5;crm:stale</t>
+          <t>google:stale;google:includes_excel_row_5;crm:stale</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -3376,13 +3376,13 @@
         </is>
       </c>
       <c r="B5" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C5" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D5" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3443,13 +3443,13 @@
         </is>
       </c>
       <c r="B6" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C6" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D6" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3486,16 +3486,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="137" t="n">
-        <v>8709.677419354839</v>
+        <v>9032.258064516129</v>
       </c>
       <c r="V6" s="137" t="n">
-        <v>7066.69</v>
+        <v>7185.39</v>
       </c>
       <c r="W6" s="137" t="n">
-        <v>-1642.987419354839</v>
+        <v>-1846.868064516128</v>
       </c>
       <c r="X6" s="138" t="n">
-        <v>-0.1886392962962963</v>
+        <v>-0.2044746785714285</v>
       </c>
       <c r="Y6" s="137" t="n"/>
       <c r="Z6" s="137" t="n"/>
@@ -3529,13 +3529,13 @@
         </is>
       </c>
       <c r="B7" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C7" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D7" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -3582,28 +3582,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>573.0050933786079</v>
+        <v>594.2275042444822</v>
       </c>
       <c r="R7" t="n">
         <v>371</v>
       </c>
       <c r="S7" t="n">
-        <v>-202.0050933786079</v>
+        <v>-223.2275042444822</v>
       </c>
       <c r="T7" s="137" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="U7" s="137" t="n">
-        <v>4130.434782608696</v>
+        <v>4347.826086956522</v>
       </c>
       <c r="V7" s="137" t="n">
         <v>2819.6</v>
       </c>
       <c r="W7" s="137" t="n">
-        <v>-1310.834782608696</v>
+        <v>-1528.226086956522</v>
       </c>
       <c r="X7" s="138" t="n">
-        <v>-0.3173600000000001</v>
+        <v>-0.3514920000000001</v>
       </c>
       <c r="Y7" s="137" t="n">
         <v>7.6</v>
@@ -3632,13 +3632,13 @@
         </is>
       </c>
       <c r="B8" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C8" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D8" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E8" t="n">
         <v>26</v>
@@ -3685,28 +3685,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>387.0967741935484</v>
+        <v>401.4336917562724</v>
       </c>
       <c r="R8" t="n">
         <v>187</v>
       </c>
       <c r="S8" t="n">
-        <v>-200.0967741935484</v>
+        <v>-214.4336917562724</v>
       </c>
       <c r="T8" s="137" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="U8" s="137" t="n">
-        <v>3304.347826086957</v>
+        <v>3478.260869565217</v>
       </c>
       <c r="V8" s="137" t="n">
         <v>1683</v>
       </c>
       <c r="W8" s="137" t="n">
-        <v>-1621.347826086957</v>
+        <v>-1795.260869565217</v>
       </c>
       <c r="X8" s="138" t="n">
-        <v>-0.4906710526315789</v>
+        <v>-0.5161375</v>
       </c>
       <c r="Y8" s="137" t="n">
         <v>9</v>
@@ -3735,13 +3735,13 @@
         </is>
       </c>
       <c r="B9" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C9" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D9" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3788,28 +3788,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>217.7419354838709</v>
+        <v>225.8064516129032</v>
       </c>
       <c r="R9" t="n">
         <v>240</v>
       </c>
       <c r="S9" t="n">
-        <v>22.25806451612902</v>
+        <v>14.19354838709677</v>
       </c>
       <c r="T9" s="137" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="U9" s="137" t="n">
-        <v>1652.173913043478</v>
+        <v>1739.130434782609</v>
       </c>
       <c r="V9" s="137" t="n">
         <v>1920</v>
       </c>
       <c r="W9" s="137" t="n">
-        <v>267.8260869565217</v>
+        <v>180.8695652173912</v>
       </c>
       <c r="X9" s="138" t="n">
-        <v>0.1621052631578947</v>
+        <v>0.1039999999999999</v>
       </c>
       <c r="Y9" s="137" t="n">
         <v>8</v>
@@ -3838,13 +3838,13 @@
         </is>
       </c>
       <c r="B10" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C10" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D10" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3891,28 +3891,28 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>102.4667931688805</v>
+        <v>106.2618595825427</v>
       </c>
       <c r="R10" t="n">
         <v>111</v>
       </c>
       <c r="S10" t="n">
-        <v>8.533206831119543</v>
+        <v>4.738140417457316</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U10" s="137" t="n">
-        <v>3483.870967741936</v>
+        <v>3612.903225806452</v>
       </c>
       <c r="V10" s="137" t="n">
         <v>4033.470302</v>
       </c>
       <c r="W10" s="137" t="n">
-        <v>549.5993342580646</v>
+        <v>420.5670761935485</v>
       </c>
       <c r="X10" s="138" t="n">
-        <v>0.1577553644629629</v>
+        <v>0.1164069585892857</v>
       </c>
       <c r="Y10" s="137" t="n">
         <v>36.33757028828829</v>
@@ -3934,7 +3934,7 @@
       <c r="AD10" s="139" t="inlineStr"/>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:stale;crm:stale</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -3950,13 +3950,13 @@
         </is>
       </c>
       <c r="B11" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C11" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D11" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -4003,28 +4003,28 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q11" t="n">
-        <v>203.6028487641391</v>
+        <v>211.1436950146628</v>
       </c>
       <c r="R11" t="n">
         <v>61</v>
       </c>
       <c r="S11" t="n">
-        <v>-35.60284876413908</v>
+        <v>-43.14369501466274</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U11" s="137" t="n">
-        <v>7838.709677419354</v>
+        <v>8129.032258064516</v>
       </c>
       <c r="V11" s="137" t="n">
         <v>7997.154267</v>
       </c>
       <c r="W11" s="137" t="n">
-        <v>158.4445895806457</v>
+        <v>-131.8779910645162</v>
       </c>
       <c r="X11" s="138" t="n">
-        <v>0.0202130957901235</v>
+        <v>-0.0162230862023809</v>
       </c>
       <c r="Y11" s="137" t="n">
         <v>47.60210873214286</v>
@@ -4046,7 +4046,7 @@
       <c r="AD11" s="139" t="inlineStr"/>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_10;crm_metrics_combined_with_excel_row_10;crm:stale</t>
+          <t>google:stale;google:includes_excel_row_10;crm_metrics_combined_with_excel_row_10;crm:stale</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -4062,13 +4062,13 @@
         </is>
       </c>
       <c r="B12" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C12" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D12" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -4132,13 +4132,13 @@
         </is>
       </c>
       <c r="B13" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C13" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D13" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4185,28 +4185,28 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>22.92020373514431</v>
+        <v>23.76910016977929</v>
       </c>
       <c r="R13" t="n">
         <v>5</v>
       </c>
       <c r="S13" t="n">
-        <v>-12.92020373514431</v>
+        <v>-13.76910016977929</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="137" t="n">
-        <v>870.9677419354839</v>
+        <v>903.2258064516128</v>
       </c>
       <c r="V13" s="137" t="n">
         <v>853.4385040000001</v>
       </c>
       <c r="W13" s="137" t="n">
-        <v>-17.52923793548382</v>
+        <v>-49.78730245161285</v>
       </c>
       <c r="X13" s="138" t="n">
-        <v>-0.020126162074074</v>
+        <v>-0.0551216562857142</v>
       </c>
       <c r="Y13" s="137" t="n">
         <v>85.34385040000001</v>
@@ -4228,7 +4228,7 @@
       <c r="AD13" s="139" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_12;crm_metrics_combined_with_excel_row_12;crm:stale</t>
+          <t>google:stale;google:includes_excel_row_12;crm_metrics_combined_with_excel_row_12;crm:stale</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -4244,13 +4244,13 @@
         </is>
       </c>
       <c r="B14" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C14" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D14" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
@@ -4314,13 +4314,13 @@
         </is>
       </c>
       <c r="B15" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C15" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D15" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -4367,28 +4367,28 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q15" t="n">
-        <v>3.483870967741935</v>
+        <v>3.612903225806452</v>
       </c>
       <c r="R15" t="n">
         <v>2</v>
       </c>
       <c r="S15" t="n">
-        <v>-1.483870967741935</v>
+        <v>-1.612903225806452</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U15" s="137" t="n">
-        <v>870.9677419354839</v>
+        <v>903.2258064516128</v>
       </c>
       <c r="V15" s="137" t="n">
         <v>875.3623249999999</v>
       </c>
       <c r="W15" s="137" t="n">
-        <v>4.394583064516041</v>
+        <v>-27.86348145161298</v>
       </c>
       <c r="X15" s="138" t="n">
-        <v>0.0050456324074073</v>
+        <v>-0.0308488544642858</v>
       </c>
       <c r="Y15" s="137" t="n">
         <v>437.6811625</v>
@@ -4410,7 +4410,7 @@
       <c r="AD15" s="139" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_14;crm_metrics_combined_with_excel_row_14;crm:stale</t>
+          <t>google:stale;google:includes_excel_row_14;crm_metrics_combined_with_excel_row_14;crm:stale</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -4426,13 +4426,13 @@
         </is>
       </c>
       <c r="B16" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C16" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D16" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4496,13 +4496,13 @@
         </is>
       </c>
       <c r="B17" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C17" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D17" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E17" t="n">
         <v>17</v>
@@ -4549,34 +4549,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>680.4435483870968</v>
+        <v>705.6451612903227</v>
       </c>
       <c r="R17" t="n">
         <v>417</v>
       </c>
       <c r="S17" t="n">
-        <v>-263.4435483870968</v>
+        <v>-288.6451612903227</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U17" s="137" t="n">
-        <v>8709.677419354839</v>
+        <v>9032.258064516129</v>
       </c>
       <c r="V17" s="137" t="n">
-        <v>11088.19</v>
+        <v>11267.67</v>
       </c>
       <c r="W17" s="137" t="n">
-        <v>2378.512580645161</v>
+        <v>2235.411935483872</v>
       </c>
       <c r="X17" s="138" t="n">
-        <v>0.2730884814814815</v>
+        <v>0.2474920357142857</v>
       </c>
       <c r="Y17" s="137" t="n">
-        <v>26.59038369304556</v>
+        <v>27.02079136690648</v>
       </c>
       <c r="Z17" s="137" t="n">
-        <v>13.79038369304556</v>
+        <v>14.22079136690648</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -4608,13 +4608,13 @@
         </is>
       </c>
       <c r="B18" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C18" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D18" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4661,34 +4661,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>10.88709677419355</v>
+        <v>11.29032258064516</v>
       </c>
       <c r="R18" t="n">
         <v>32</v>
       </c>
       <c r="S18" t="n">
-        <v>21.11290322580645</v>
+        <v>20.70967741935484</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="137" t="n">
-        <v>435.483870967742</v>
+        <v>451.6129032258065</v>
       </c>
       <c r="V18" s="137" t="n">
-        <v>426.16</v>
+        <v>431.64</v>
       </c>
       <c r="W18" s="137" t="n">
-        <v>-9.323870967741923</v>
+        <v>-19.97290322580648</v>
       </c>
       <c r="X18" s="138" t="n">
-        <v>-0.0214103703703703</v>
+        <v>-0.0442257142857143</v>
       </c>
       <c r="Y18" s="137" t="n">
-        <v>13.3175</v>
+        <v>13.48875</v>
       </c>
       <c r="Z18" s="137" t="n">
-        <v>-26.6825</v>
+        <v>-26.51125</v>
       </c>
       <c r="AB18" s="139" t="inlineStr"/>
       <c r="AC18" s="139" t="inlineStr">
@@ -4715,13 +4715,13 @@
         </is>
       </c>
       <c r="B19" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C19" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D19" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4768,34 +4768,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>9.67741935483871</v>
+        <v>10.03584229390681</v>
       </c>
       <c r="R19" t="n">
         <v>19</v>
       </c>
       <c r="S19" t="n">
-        <v>9.32258064516129</v>
+        <v>8.964157706093189</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="137" t="n">
-        <v>870.9677419354839</v>
+        <v>903.2258064516128</v>
       </c>
       <c r="V19" s="137" t="n">
-        <v>736.39</v>
+        <v>742.34</v>
       </c>
       <c r="W19" s="137" t="n">
-        <v>-134.5777419354839</v>
+        <v>-160.8858064516129</v>
       </c>
       <c r="X19" s="138" t="n">
-        <v>-0.1545151851851852</v>
+        <v>-0.1781235714285714</v>
       </c>
       <c r="Y19" s="137" t="n">
-        <v>38.75736842105263</v>
+        <v>39.07052631578947</v>
       </c>
       <c r="Z19" s="137" t="n">
-        <v>-51.24263157894737</v>
+        <v>-50.92947368421053</v>
       </c>
       <c r="AB19" s="139" t="inlineStr"/>
       <c r="AC19" s="139" t="inlineStr">
@@ -4822,13 +4822,13 @@
         </is>
       </c>
       <c r="B20" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C20" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D20" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
@@ -4875,34 +4875,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>3.629032258064517</v>
+        <v>3.763440860215054</v>
       </c>
       <c r="R20" t="n">
         <v>4</v>
       </c>
       <c r="S20" t="n">
-        <v>0.3709677419354835</v>
+        <v>0.2365591397849455</v>
       </c>
       <c r="T20" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U20" s="137" t="n">
-        <v>435.483870967742</v>
+        <v>451.6129032258065</v>
       </c>
       <c r="V20" s="137" t="n">
-        <v>382.04</v>
+        <v>387.91</v>
       </c>
       <c r="W20" s="137" t="n">
-        <v>-53.44387096774193</v>
+        <v>-63.70290322580644</v>
       </c>
       <c r="X20" s="138" t="n">
-        <v>-0.1227229629629629</v>
+        <v>-0.1410564285714285</v>
       </c>
       <c r="Y20" s="137" t="n">
-        <v>95.51000000000001</v>
+        <v>96.97750000000001</v>
       </c>
       <c r="Z20" s="137" t="n">
-        <v>-24.48999999999999</v>
+        <v>-23.0225</v>
       </c>
       <c r="AB20" s="139" t="inlineStr"/>
       <c r="AC20" s="139" t="inlineStr">
@@ -4929,13 +4929,13 @@
         </is>
       </c>
       <c r="B21" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C21" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D21" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4982,28 +4982,28 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>32.66129032258065</v>
+        <v>33.87096774193549</v>
       </c>
       <c r="R21" t="n">
         <v>22</v>
       </c>
       <c r="S21" t="n">
-        <v>-10.66129032258065</v>
+        <v>-11.87096774193549</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="137" t="n">
-        <v>1306.451612903226</v>
+        <v>1354.83870967742</v>
       </c>
       <c r="V21" s="137" t="n">
         <v>1414.698441</v>
       </c>
       <c r="W21" s="137" t="n">
-        <v>108.2468280967742</v>
+        <v>59.8597313225805</v>
       </c>
       <c r="X21" s="138" t="n">
-        <v>0.08285559681481471</v>
+        <v>0.044182182642857</v>
       </c>
       <c r="Y21" s="137" t="n">
         <v>64.30447459090909</v>
@@ -5020,7 +5020,7 @@
       <c r="AD21" s="139" t="inlineStr"/>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:stale;crm:stale</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
@@ -5036,13 +5036,13 @@
         </is>
       </c>
       <c r="B22" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C22" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D22" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -5089,28 +5089,28 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>87.09677419354838</v>
+        <v>90.32258064516128</v>
       </c>
       <c r="R22" t="n">
         <v>114</v>
       </c>
       <c r="S22" t="n">
-        <v>26.90322580645162</v>
+        <v>23.67741935483872</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="137" t="n">
-        <v>1306.451612903226</v>
+        <v>1354.83870967742</v>
       </c>
       <c r="V22" s="137" t="n">
         <v>1928.318895</v>
       </c>
       <c r="W22" s="137" t="n">
-        <v>621.8672820967743</v>
+        <v>573.4801853225806</v>
       </c>
       <c r="X22" s="138" t="n">
-        <v>0.4759971788888889</v>
+        <v>0.4232829939285714</v>
       </c>
       <c r="Y22" s="137" t="n">
         <v>16.91507802631579</v>
@@ -5132,7 +5132,7 @@
       <c r="AD22" s="139" t="inlineStr"/>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:stale;crm:stale</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
@@ -5148,13 +5148,13 @@
         </is>
       </c>
       <c r="B23" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C23" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D23" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5201,34 +5201,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>33.49875930521092</v>
+        <v>34.7394540942928</v>
       </c>
       <c r="R23" t="n">
         <v>67</v>
       </c>
       <c r="S23" t="n">
-        <v>33.50124069478908</v>
+        <v>32.2605459057072</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="137" t="n">
-        <v>870.9677419354839</v>
+        <v>903.2258064516128</v>
       </c>
       <c r="V23" s="137" t="n">
-        <v>1252.69</v>
+        <v>1282.1</v>
       </c>
       <c r="W23" s="137" t="n">
-        <v>381.7222580645162</v>
+        <v>378.874193548387</v>
       </c>
       <c r="X23" s="138" t="n">
-        <v>0.4382737037037037</v>
+        <v>0.419467857142857</v>
       </c>
       <c r="Y23" s="137" t="n">
-        <v>18.69686567164179</v>
+        <v>19.13582089552238</v>
       </c>
       <c r="Z23" s="137" t="n">
-        <v>-7.303134328358208</v>
+        <v>-6.864179104477614</v>
       </c>
       <c r="AB23" s="139" t="inlineStr"/>
       <c r="AC23" s="139" t="inlineStr">
@@ -5255,13 +5255,13 @@
         </is>
       </c>
       <c r="B24" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C24" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D24" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5298,12 +5298,12 @@
       <c r="T24" s="137" t="n"/>
       <c r="U24" s="137" t="n"/>
       <c r="V24" s="137" t="n">
-        <v>669.92</v>
+        <v>705.61</v>
       </c>
       <c r="W24" s="137" t="n"/>
       <c r="X24" s="138" t="n"/>
       <c r="Y24" s="137" t="n">
-        <v>669.92</v>
+        <v>705.61</v>
       </c>
       <c r="Z24" s="137" t="n"/>
       <c r="AB24" s="139" t="inlineStr"/>
@@ -5331,13 +5331,13 @@
         </is>
       </c>
       <c r="B25" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C25" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D25" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5366,34 +5366,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>406.4516129032259</v>
+        <v>421.505376344086</v>
       </c>
       <c r="R25" t="n">
         <v>328</v>
       </c>
       <c r="S25" t="n">
-        <v>-78.45161290322585</v>
+        <v>-93.50537634408602</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="137" t="n">
-        <v>18290.32258064516</v>
+        <v>18967.74193548387</v>
       </c>
       <c r="V25" s="137" t="n">
-        <v>16512.643483</v>
+        <v>16631.343483</v>
       </c>
       <c r="W25" s="137" t="n">
-        <v>-1777.679097645163</v>
+        <v>-2336.39845248387</v>
       </c>
       <c r="X25" s="138" t="n">
-        <v>-0.09719233161728399</v>
+        <v>-0.1231774694336734</v>
       </c>
       <c r="Y25" s="137" t="n">
-        <v>50.34342525304878</v>
+        <v>50.70531549695122</v>
       </c>
       <c r="Z25" s="137" t="n">
-        <v>5.343425253048778</v>
+        <v>5.705315496951222</v>
       </c>
       <c r="AB25" s="139" t="inlineStr"/>
       <c r="AC25" s="139" t="inlineStr"/>
@@ -5411,13 +5411,13 @@
         </is>
       </c>
       <c r="B26" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C26" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D26" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5451,34 +5451,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>1190.367637231439</v>
+        <v>1234.45532749927</v>
       </c>
       <c r="R26" t="n">
         <v>967</v>
       </c>
       <c r="S26" t="n">
-        <v>-223.3676372314394</v>
+        <v>-267.4553274992704</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="137" t="n">
-        <v>27000</v>
+        <v>28000</v>
       </c>
       <c r="V26" s="137" t="n">
-        <v>31657.832734</v>
+        <v>31919.712734</v>
       </c>
       <c r="W26" s="137" t="n">
-        <v>4657.832734</v>
+        <v>3919.712734000001</v>
       </c>
       <c r="X26" s="138" t="n">
-        <v>0.1725123234814814</v>
+        <v>0.1399897405</v>
       </c>
       <c r="Y26" s="137" t="n">
-        <v>32.73819310651499</v>
+        <v>33.00901006618408</v>
       </c>
       <c r="Z26" s="137" t="n">
-        <v>10.05612484834504</v>
+        <v>10.32694180801412</v>
       </c>
       <c r="AB26" s="139" t="inlineStr"/>
       <c r="AC26" s="139" t="inlineStr"/>
@@ -5496,13 +5496,13 @@
         </is>
       </c>
       <c r="B27" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C27" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D27" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5536,28 +5536,28 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>1177.843803056027</v>
+        <v>1221.467647613658</v>
       </c>
       <c r="R27" t="n">
         <v>798</v>
       </c>
       <c r="S27" t="n">
-        <v>-379.8438030560274</v>
+        <v>-423.4676476136578</v>
       </c>
       <c r="T27" s="137" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="U27" s="137" t="n">
-        <v>9086.95652173913</v>
+        <v>9565.217391304348</v>
       </c>
       <c r="V27" s="137" t="n">
         <v>6422.6</v>
       </c>
       <c r="W27" s="137" t="n">
-        <v>-2664.35652173913</v>
+        <v>-3142.617391304348</v>
       </c>
       <c r="X27" s="138" t="n">
-        <v>-0.2932066985645932</v>
+        <v>-0.3285463636363636</v>
       </c>
       <c r="Y27" s="137" t="n">
         <v>8.048370927318297</v>
@@ -5581,13 +5581,13 @@
         </is>
       </c>
       <c r="B28" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C28" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D28" s="136" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5621,34 +5621,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>2774.663053190693</v>
+        <v>2877.428351457014</v>
       </c>
       <c r="R28" t="n">
         <v>2093</v>
       </c>
       <c r="S28" t="n">
-        <v>-681.6630531906926</v>
+        <v>-784.4283514570143</v>
       </c>
       <c r="T28" s="137" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="U28" s="137" t="n">
-        <v>54377.27910238429</v>
+        <v>56532.95932678822</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>54593.076217</v>
+        <v>54973.656217</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>215.797114615707</v>
+        <v>-1559.303109788212</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>0.0039685162291661</v>
+        <v>-0.027582195030242</v>
       </c>
       <c r="Y28" s="137" t="n">
-        <v>26.08364845532728</v>
+        <v>26.26548314237936</v>
       </c>
       <c r="Z28" s="137" t="n">
-        <v>6.307925533281942</v>
+        <v>6.489760220334023</v>
       </c>
       <c r="AB28" s="139" t="inlineStr"/>
       <c r="AC28" s="139" t="inlineStr"/>
@@ -5751,7 +5751,7 @@
         </is>
       </c>
       <c r="B4" s="140" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5791,7 +5791,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5811,7 +5811,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46231.29190972223</v>
+        <v>46232.29190972223</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-07-30
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 28/07/2026  |  Ultimo aggiornamento: 29/07/2026 07:00</t>
+          <t>Periodo: 01/07/2026 - 29/07/2026  |  Ultimo aggiornamento: 30/07/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1065,16 +1065,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>8580.645161290322</v>
+        <v>8887.096774193547</v>
       </c>
       <c r="R5" s="117" t="n">
         <v>8077.867025</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>-502.7781362903224</v>
+        <v>-809.2297491935478</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>-0.0585944444548872</v>
+        <v>-0.0910567049909255</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1173,16 +1173,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>1354.83870967742</v>
+        <v>1403.225806451613</v>
       </c>
       <c r="R7" s="117" t="n">
         <v>1368.086458</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>13.24774832258049</v>
+        <v>-35.13934845161293</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>0.009778099952380799</v>
+        <v>-0.0250418345287356</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1281,16 +1281,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>9032.258064516129</v>
+        <v>9354.83870967742</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>7185.39</v>
+        <v>7318.73</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-1846.868064516128</v>
+        <v>-2036.108709677419</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.2044746785714285</v>
+        <v>-0.2176529999999999</v>
       </c>
       <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
@@ -1328,34 +1328,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>421.505376344086</v>
+        <v>436.5591397849462</v>
       </c>
       <c r="N10" s="125" t="n">
         <v>328</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>-93.50537634408602</v>
+        <v>-108.5591397849462</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>18967.74193548387</v>
+        <v>19645.16129032258</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>16631.343483</v>
+        <v>16764.683483</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>-2336.39845248387</v>
+        <v>-2880.477807322579</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>-0.1231774694336734</v>
+        <v>-0.1466253071050902</v>
       </c>
       <c r="U10" s="123" t="n">
-        <v>50.70531549695122</v>
+        <v>51.11183988719512</v>
       </c>
       <c r="V10" s="123" t="n">
-        <v>5.705315496951222</v>
+        <v>6.111839887195124</v>
       </c>
       <c r="W10" s="126" t="n"/>
     </row>
@@ -1407,28 +1407,28 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>106.2618595825427</v>
+        <v>110.0569259962049</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>111</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>4.738140417457316</v>
+        <v>0.9430740037950756</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>3612.903225806452</v>
+        <v>3741.935483870968</v>
       </c>
       <c r="R11" s="117" t="n">
         <v>4033.470302</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>420.5670761935485</v>
+        <v>291.5348181290324</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.1164069585892857</v>
+        <v>0.0779101669137931</v>
       </c>
       <c r="U11" s="117" t="n">
         <v>36.33757028828829</v>
@@ -1490,28 +1490,28 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M12" s="127" t="n">
-        <v>211.1436950146628</v>
+        <v>218.6845412651865</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>61</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>-43.14369501466274</v>
+        <v>-50.68454126518643</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>8129.032258064516</v>
+        <v>8419.354838709678</v>
       </c>
       <c r="R12" s="117" t="n">
         <v>7997.154267</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-131.8779910645162</v>
+        <v>-422.2005717096781</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.0162230862023809</v>
+        <v>-0.0501464280574713</v>
       </c>
       <c r="U12" s="128" t="n">
         <v>47.60210873214286</v>
@@ -1620,28 +1620,28 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="127" t="n">
-        <v>23.76910016977929</v>
+        <v>24.61799660441426</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>5</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-13.76910016977929</v>
+        <v>-14.61799660441426</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>903.2258064516128</v>
+        <v>935.483870967742</v>
       </c>
       <c r="R14" s="117" t="n">
         <v>853.4385040000001</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-49.78730245161285</v>
+        <v>-82.04536696774187</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.0551216562857142</v>
+        <v>-0.0877036681379309</v>
       </c>
       <c r="U14" s="128" t="n">
         <v>85.34385040000001</v>
@@ -1750,28 +1750,28 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M16" s="127" t="n">
-        <v>3.612903225806452</v>
+        <v>3.741935483870968</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>-1.612903225806452</v>
+        <v>-1.741935483870968</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>903.2258064516128</v>
+        <v>935.483870967742</v>
       </c>
       <c r="R16" s="117" t="n">
         <v>875.3623249999999</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>-27.86348145161298</v>
+        <v>-60.12154596774201</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>-0.0308488544642858</v>
+        <v>-0.0642678594827587</v>
       </c>
       <c r="U16" s="128" t="n">
         <v>437.6811625</v>
@@ -1880,34 +1880,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>705.6451612903227</v>
+        <v>730.8467741935484</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>417</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-288.6451612903227</v>
+        <v>-313.8467741935484</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>9032.258064516129</v>
+        <v>9354.83870967742</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>11267.67</v>
+        <v>11396.21</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>2235.411935483872</v>
+        <v>2041.37129032258</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>0.2474920357142857</v>
+        <v>0.2182155517241379</v>
       </c>
       <c r="U18" s="117" t="n">
-        <v>27.02079136690648</v>
+        <v>27.32904076738609</v>
       </c>
       <c r="V18" s="117" t="n">
-        <v>14.22079136690648</v>
+        <v>14.52904076738609</v>
       </c>
       <c r="W18" s="120" t="inlineStr">
         <is>
@@ -1963,34 +1963,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>11.29032258064516</v>
+        <v>11.69354838709677</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>32</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>20.70967741935484</v>
+        <v>20.30645161290322</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>451.6129032258065</v>
+        <v>467.741935483871</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>431.64</v>
+        <v>436.05</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-19.97290322580648</v>
+        <v>-31.69193548387096</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.0442257142857143</v>
+        <v>-0.0677551724137931</v>
       </c>
       <c r="U19" s="117" t="n">
-        <v>13.48875</v>
+        <v>13.6265625</v>
       </c>
       <c r="V19" s="117" t="n">
-        <v>-26.51125</v>
+        <v>-26.3734375</v>
       </c>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
@@ -2042,34 +2042,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>10.03584229390681</v>
+        <v>10.39426523297491</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>8.964157706093189</v>
+        <v>8.605734767025091</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>903.2258064516128</v>
+        <v>935.483870967742</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>742.34</v>
+        <v>747.83</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-160.8858064516129</v>
+        <v>-187.6538709677419</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.1781235714285714</v>
+        <v>-0.2005955172413792</v>
       </c>
       <c r="U20" s="117" t="n">
-        <v>39.07052631578947</v>
+        <v>39.35947368421053</v>
       </c>
       <c r="V20" s="117" t="n">
-        <v>-50.92947368421053</v>
+        <v>-50.64052631578947</v>
       </c>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
@@ -2121,34 +2121,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>3.763440860215054</v>
+        <v>3.897849462365592</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>4</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>0.2365591397849455</v>
+        <v>0.102150537634408</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>451.6129032258065</v>
+        <v>467.741935483871</v>
       </c>
       <c r="R21" s="117" t="n">
-        <v>387.91</v>
+        <v>393.09</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-63.70290322580644</v>
+        <v>-74.651935483871</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.1410564285714285</v>
+        <v>-0.1596006896551725</v>
       </c>
       <c r="U21" s="117" t="n">
-        <v>96.97750000000001</v>
+        <v>98.27249999999999</v>
       </c>
       <c r="V21" s="117" t="n">
-        <v>-23.0225</v>
+        <v>-21.72750000000001</v>
       </c>
       <c r="W21" s="120" t="inlineStr"/>
     </row>
@@ -2200,28 +2200,28 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>33.87096774193549</v>
+        <v>35.08064516129032</v>
       </c>
       <c r="N22" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-11.87096774193549</v>
+        <v>-13.08064516129032</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>1354.83870967742</v>
+        <v>1403.225806451613</v>
       </c>
       <c r="R22" s="117" t="n">
         <v>1414.698441</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>59.8597313225805</v>
+        <v>11.47263454838708</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>0.044182182642857</v>
+        <v>0.0081759004827586</v>
       </c>
       <c r="U22" s="117" t="n">
         <v>64.30447459090909</v>
@@ -2279,28 +2279,28 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>90.32258064516128</v>
+        <v>93.54838709677421</v>
       </c>
       <c r="N23" s="119" t="n">
         <v>114</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>23.67741935483872</v>
+        <v>20.45161290322581</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>1354.83870967742</v>
+        <v>1403.225806451613</v>
       </c>
       <c r="R23" s="117" t="n">
         <v>1928.318895</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>573.4801853225806</v>
+        <v>525.0930885483872</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.4232829939285714</v>
+        <v>0.37420427</v>
       </c>
       <c r="U23" s="117" t="n">
         <v>16.91507802631579</v>
@@ -2362,34 +2362,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>34.7394540942928</v>
+        <v>35.98014888337469</v>
       </c>
       <c r="N24" s="119" t="n">
         <v>67</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>32.2605459057072</v>
+        <v>31.01985111662531</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>903.2258064516128</v>
+        <v>935.483870967742</v>
       </c>
       <c r="R24" s="117" t="n">
-        <v>1282.1</v>
+        <v>1308.82</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>378.874193548387</v>
+        <v>373.336129032258</v>
       </c>
       <c r="T24" s="118" t="n">
-        <v>0.419467857142857</v>
+        <v>0.3990834482758619</v>
       </c>
       <c r="U24" s="117" t="n">
-        <v>19.13582089552238</v>
+        <v>19.53462686567164</v>
       </c>
       <c r="V24" s="117" t="n">
-        <v>-6.864179104477614</v>
+        <v>-6.46537313432836</v>
       </c>
       <c r="W24" s="120" t="inlineStr"/>
     </row>
@@ -2436,12 +2436,12 @@
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>705.61</v>
+        <v>732.3</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
       <c r="U25" s="117" t="n">
-        <v>705.61</v>
+        <v>732.3</v>
       </c>
       <c r="V25" s="117" t="n"/>
       <c r="W25" s="120" t="inlineStr"/>
@@ -2478,34 +2478,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>1234.45532749927</v>
+        <v>1278.543017767101</v>
       </c>
       <c r="N26" s="125" t="n">
         <v>967</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>-267.4553274992704</v>
+        <v>-311.5430177671014</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>28000</v>
+        <v>29000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>31919.712734</v>
+        <v>32116.742734</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>3919.712734000001</v>
+        <v>3116.742733999999</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>0.1399897405</v>
+        <v>0.1074738873793103</v>
       </c>
       <c r="U26" s="123" t="n">
-        <v>33.00901006618408</v>
+        <v>33.21276394415719</v>
       </c>
       <c r="V26" s="123" t="n">
-        <v>10.32694180801412</v>
+        <v>10.53069568598723</v>
       </c>
       <c r="W26" s="126" t="n"/>
     </row>
@@ -2553,28 +2553,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>594.2275042444822</v>
+        <v>615.4499151103566</v>
       </c>
       <c r="N27" s="119" t="n">
         <v>371</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-223.2275042444822</v>
+        <v>-244.4499151103566</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>4347.826086956522</v>
+        <v>4565.217391304348</v>
       </c>
       <c r="R27" s="117" t="n">
         <v>2819.6</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-1528.226086956522</v>
+        <v>-1745.617391304348</v>
       </c>
       <c r="T27" s="118" t="n">
-        <v>-0.3514920000000001</v>
+        <v>-0.3823733333333334</v>
       </c>
       <c r="U27" s="117" t="n">
         <v>7.6</v>
@@ -2628,28 +2628,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>401.4336917562724</v>
+        <v>415.7706093189964</v>
       </c>
       <c r="N28" s="119" t="n">
         <v>187</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-214.4336917562724</v>
+        <v>-228.7706093189964</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>3478.260869565217</v>
+        <v>3652.173913043479</v>
       </c>
       <c r="R28" s="117" t="n">
         <v>1683</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-1795.260869565217</v>
+        <v>-1969.173913043478</v>
       </c>
       <c r="T28" s="118" t="n">
-        <v>-0.5161375</v>
+        <v>-0.5391785714285715</v>
       </c>
       <c r="U28" s="117" t="n">
         <v>9</v>
@@ -2703,28 +2703,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>225.8064516129032</v>
+        <v>233.8709677419355</v>
       </c>
       <c r="N29" s="119" t="n">
         <v>240</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>14.19354838709677</v>
+        <v>6.129032258064512</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>1739.130434782609</v>
+        <v>1826.086956521739</v>
       </c>
       <c r="R29" s="117" t="n">
         <v>1920</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>180.8695652173912</v>
+        <v>93.91304347826076</v>
       </c>
       <c r="T29" s="118" t="n">
-        <v>0.1039999999999999</v>
+        <v>0.0514285714285713</v>
       </c>
       <c r="U29" s="117" t="n">
         <v>8</v>
@@ -2766,28 +2766,28 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>1221.467647613658</v>
+        <v>1265.091492171289</v>
       </c>
       <c r="N30" s="125" t="n">
         <v>798</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-423.4676476136578</v>
+        <v>-467.0914921712886</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>9565.217391304348</v>
+        <v>10043.47826086957</v>
       </c>
       <c r="R30" s="123" t="n">
         <v>6422.6</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>-3142.617391304348</v>
+        <v>-3620.878260869566</v>
       </c>
       <c r="T30" s="124" t="n">
-        <v>-0.3285463636363636</v>
+        <v>-0.3605203463203463</v>
       </c>
       <c r="U30" s="123" t="n">
         <v>8.048370927318297</v>
@@ -2829,34 +2829,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="133" t="n">
-        <v>2877.428351457014</v>
+        <v>2980.193649723336</v>
       </c>
       <c r="N31" s="133" t="n">
         <v>2093</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>-784.4283514570143</v>
+        <v>-887.1936497233364</v>
       </c>
       <c r="P31" s="131" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="Q31" s="131" t="n">
-        <v>56532.95932678822</v>
+        <v>58688.63955119214</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>54973.656217</v>
+        <v>55304.026217</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>-1559.303109788212</v>
+        <v>-3384.613334192145</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>-0.027582195030242</v>
+        <v>-0.0576706728947066</v>
       </c>
       <c r="U31" s="131" t="n">
-        <v>26.26548314237936</v>
+        <v>26.42332834065934</v>
       </c>
       <c r="V31" s="131" t="n">
-        <v>6.489760220334023</v>
+        <v>6.647605418613999</v>
       </c>
       <c r="W31" s="134" t="n"/>
     </row>
@@ -3137,13 +3137,13 @@
         </is>
       </c>
       <c r="B2" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C2" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D2" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3180,16 +3180,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="137" t="n">
-        <v>8580.645161290322</v>
+        <v>8887.096774193547</v>
       </c>
       <c r="V2" s="137" t="n">
         <v>8077.867025</v>
       </c>
       <c r="W2" s="137" t="n">
-        <v>-502.7781362903224</v>
+        <v>-809.2297491935478</v>
       </c>
       <c r="X2" s="138" t="n">
-        <v>-0.0585944444548872</v>
+        <v>-0.0910567049909255</v>
       </c>
       <c r="Y2" s="137" t="n"/>
       <c r="Z2" s="137" t="n"/>
@@ -3223,13 +3223,13 @@
         </is>
       </c>
       <c r="B3" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C3" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D3" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3290,13 +3290,13 @@
         </is>
       </c>
       <c r="B4" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C4" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D4" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3333,16 +3333,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="137" t="n">
-        <v>1354.83870967742</v>
+        <v>1403.225806451613</v>
       </c>
       <c r="V4" s="137" t="n">
         <v>1368.086458</v>
       </c>
       <c r="W4" s="137" t="n">
-        <v>13.24774832258049</v>
+        <v>-35.13934845161293</v>
       </c>
       <c r="X4" s="138" t="n">
-        <v>0.009778099952380799</v>
+        <v>-0.0250418345287356</v>
       </c>
       <c r="Y4" s="137" t="n"/>
       <c r="Z4" s="137" t="n"/>
@@ -3376,13 +3376,13 @@
         </is>
       </c>
       <c r="B5" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C5" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D5" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3443,13 +3443,13 @@
         </is>
       </c>
       <c r="B6" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C6" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D6" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3486,16 +3486,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="137" t="n">
-        <v>9032.258064516129</v>
+        <v>9354.83870967742</v>
       </c>
       <c r="V6" s="137" t="n">
-        <v>7185.39</v>
+        <v>7318.73</v>
       </c>
       <c r="W6" s="137" t="n">
-        <v>-1846.868064516128</v>
+        <v>-2036.108709677419</v>
       </c>
       <c r="X6" s="138" t="n">
-        <v>-0.2044746785714285</v>
+        <v>-0.2176529999999999</v>
       </c>
       <c r="Y6" s="137" t="n"/>
       <c r="Z6" s="137" t="n"/>
@@ -3529,13 +3529,13 @@
         </is>
       </c>
       <c r="B7" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C7" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D7" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -3582,28 +3582,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>594.2275042444822</v>
+        <v>615.4499151103566</v>
       </c>
       <c r="R7" t="n">
         <v>371</v>
       </c>
       <c r="S7" t="n">
-        <v>-223.2275042444822</v>
+        <v>-244.4499151103566</v>
       </c>
       <c r="T7" s="137" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="U7" s="137" t="n">
-        <v>4347.826086956522</v>
+        <v>4565.217391304348</v>
       </c>
       <c r="V7" s="137" t="n">
         <v>2819.6</v>
       </c>
       <c r="W7" s="137" t="n">
-        <v>-1528.226086956522</v>
+        <v>-1745.617391304348</v>
       </c>
       <c r="X7" s="138" t="n">
-        <v>-0.3514920000000001</v>
+        <v>-0.3823733333333334</v>
       </c>
       <c r="Y7" s="137" t="n">
         <v>7.6</v>
@@ -3632,13 +3632,13 @@
         </is>
       </c>
       <c r="B8" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C8" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D8" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E8" t="n">
         <v>26</v>
@@ -3685,28 +3685,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>401.4336917562724</v>
+        <v>415.7706093189964</v>
       </c>
       <c r="R8" t="n">
         <v>187</v>
       </c>
       <c r="S8" t="n">
-        <v>-214.4336917562724</v>
+        <v>-228.7706093189964</v>
       </c>
       <c r="T8" s="137" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="U8" s="137" t="n">
-        <v>3478.260869565217</v>
+        <v>3652.173913043479</v>
       </c>
       <c r="V8" s="137" t="n">
         <v>1683</v>
       </c>
       <c r="W8" s="137" t="n">
-        <v>-1795.260869565217</v>
+        <v>-1969.173913043478</v>
       </c>
       <c r="X8" s="138" t="n">
-        <v>-0.5161375</v>
+        <v>-0.5391785714285715</v>
       </c>
       <c r="Y8" s="137" t="n">
         <v>9</v>
@@ -3735,13 +3735,13 @@
         </is>
       </c>
       <c r="B9" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C9" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D9" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3788,28 +3788,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>225.8064516129032</v>
+        <v>233.8709677419355</v>
       </c>
       <c r="R9" t="n">
         <v>240</v>
       </c>
       <c r="S9" t="n">
-        <v>14.19354838709677</v>
+        <v>6.129032258064512</v>
       </c>
       <c r="T9" s="137" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="U9" s="137" t="n">
-        <v>1739.130434782609</v>
+        <v>1826.086956521739</v>
       </c>
       <c r="V9" s="137" t="n">
         <v>1920</v>
       </c>
       <c r="W9" s="137" t="n">
-        <v>180.8695652173912</v>
+        <v>93.91304347826076</v>
       </c>
       <c r="X9" s="138" t="n">
-        <v>0.1039999999999999</v>
+        <v>0.0514285714285713</v>
       </c>
       <c r="Y9" s="137" t="n">
         <v>8</v>
@@ -3838,13 +3838,13 @@
         </is>
       </c>
       <c r="B10" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C10" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D10" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3891,28 +3891,28 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>106.2618595825427</v>
+        <v>110.0569259962049</v>
       </c>
       <c r="R10" t="n">
         <v>111</v>
       </c>
       <c r="S10" t="n">
-        <v>4.738140417457316</v>
+        <v>0.9430740037950756</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U10" s="137" t="n">
-        <v>3612.903225806452</v>
+        <v>3741.935483870968</v>
       </c>
       <c r="V10" s="137" t="n">
         <v>4033.470302</v>
       </c>
       <c r="W10" s="137" t="n">
-        <v>420.5670761935485</v>
+        <v>291.5348181290324</v>
       </c>
       <c r="X10" s="138" t="n">
-        <v>0.1164069585892857</v>
+        <v>0.0779101669137931</v>
       </c>
       <c r="Y10" s="137" t="n">
         <v>36.33757028828829</v>
@@ -3950,13 +3950,13 @@
         </is>
       </c>
       <c r="B11" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C11" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D11" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -4003,28 +4003,28 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q11" t="n">
-        <v>211.1436950146628</v>
+        <v>218.6845412651865</v>
       </c>
       <c r="R11" t="n">
         <v>61</v>
       </c>
       <c r="S11" t="n">
-        <v>-43.14369501466274</v>
+        <v>-50.68454126518643</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U11" s="137" t="n">
-        <v>8129.032258064516</v>
+        <v>8419.354838709678</v>
       </c>
       <c r="V11" s="137" t="n">
         <v>7997.154267</v>
       </c>
       <c r="W11" s="137" t="n">
-        <v>-131.8779910645162</v>
+        <v>-422.2005717096781</v>
       </c>
       <c r="X11" s="138" t="n">
-        <v>-0.0162230862023809</v>
+        <v>-0.0501464280574713</v>
       </c>
       <c r="Y11" s="137" t="n">
         <v>47.60210873214286</v>
@@ -4062,13 +4062,13 @@
         </is>
       </c>
       <c r="B12" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C12" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D12" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -4132,13 +4132,13 @@
         </is>
       </c>
       <c r="B13" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C13" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D13" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4185,28 +4185,28 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>23.76910016977929</v>
+        <v>24.61799660441426</v>
       </c>
       <c r="R13" t="n">
         <v>5</v>
       </c>
       <c r="S13" t="n">
-        <v>-13.76910016977929</v>
+        <v>-14.61799660441426</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="137" t="n">
-        <v>903.2258064516128</v>
+        <v>935.483870967742</v>
       </c>
       <c r="V13" s="137" t="n">
         <v>853.4385040000001</v>
       </c>
       <c r="W13" s="137" t="n">
-        <v>-49.78730245161285</v>
+        <v>-82.04536696774187</v>
       </c>
       <c r="X13" s="138" t="n">
-        <v>-0.0551216562857142</v>
+        <v>-0.0877036681379309</v>
       </c>
       <c r="Y13" s="137" t="n">
         <v>85.34385040000001</v>
@@ -4244,13 +4244,13 @@
         </is>
       </c>
       <c r="B14" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C14" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D14" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
@@ -4314,13 +4314,13 @@
         </is>
       </c>
       <c r="B15" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C15" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D15" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -4367,28 +4367,28 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q15" t="n">
-        <v>3.612903225806452</v>
+        <v>3.741935483870968</v>
       </c>
       <c r="R15" t="n">
         <v>2</v>
       </c>
       <c r="S15" t="n">
-        <v>-1.612903225806452</v>
+        <v>-1.741935483870968</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U15" s="137" t="n">
-        <v>903.2258064516128</v>
+        <v>935.483870967742</v>
       </c>
       <c r="V15" s="137" t="n">
         <v>875.3623249999999</v>
       </c>
       <c r="W15" s="137" t="n">
-        <v>-27.86348145161298</v>
+        <v>-60.12154596774201</v>
       </c>
       <c r="X15" s="138" t="n">
-        <v>-0.0308488544642858</v>
+        <v>-0.0642678594827587</v>
       </c>
       <c r="Y15" s="137" t="n">
         <v>437.6811625</v>
@@ -4426,13 +4426,13 @@
         </is>
       </c>
       <c r="B16" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C16" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D16" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4496,13 +4496,13 @@
         </is>
       </c>
       <c r="B17" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C17" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D17" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E17" t="n">
         <v>17</v>
@@ -4549,34 +4549,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>705.6451612903227</v>
+        <v>730.8467741935484</v>
       </c>
       <c r="R17" t="n">
         <v>417</v>
       </c>
       <c r="S17" t="n">
-        <v>-288.6451612903227</v>
+        <v>-313.8467741935484</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U17" s="137" t="n">
-        <v>9032.258064516129</v>
+        <v>9354.83870967742</v>
       </c>
       <c r="V17" s="137" t="n">
-        <v>11267.67</v>
+        <v>11396.21</v>
       </c>
       <c r="W17" s="137" t="n">
-        <v>2235.411935483872</v>
+        <v>2041.37129032258</v>
       </c>
       <c r="X17" s="138" t="n">
-        <v>0.2474920357142857</v>
+        <v>0.2182155517241379</v>
       </c>
       <c r="Y17" s="137" t="n">
-        <v>27.02079136690648</v>
+        <v>27.32904076738609</v>
       </c>
       <c r="Z17" s="137" t="n">
-        <v>14.22079136690648</v>
+        <v>14.52904076738609</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -4608,13 +4608,13 @@
         </is>
       </c>
       <c r="B18" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C18" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D18" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4661,34 +4661,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.29032258064516</v>
+        <v>11.69354838709677</v>
       </c>
       <c r="R18" t="n">
         <v>32</v>
       </c>
       <c r="S18" t="n">
-        <v>20.70967741935484</v>
+        <v>20.30645161290322</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="137" t="n">
-        <v>451.6129032258065</v>
+        <v>467.741935483871</v>
       </c>
       <c r="V18" s="137" t="n">
-        <v>431.64</v>
+        <v>436.05</v>
       </c>
       <c r="W18" s="137" t="n">
-        <v>-19.97290322580648</v>
+        <v>-31.69193548387096</v>
       </c>
       <c r="X18" s="138" t="n">
-        <v>-0.0442257142857143</v>
+        <v>-0.0677551724137931</v>
       </c>
       <c r="Y18" s="137" t="n">
-        <v>13.48875</v>
+        <v>13.6265625</v>
       </c>
       <c r="Z18" s="137" t="n">
-        <v>-26.51125</v>
+        <v>-26.3734375</v>
       </c>
       <c r="AB18" s="139" t="inlineStr"/>
       <c r="AC18" s="139" t="inlineStr">
@@ -4715,13 +4715,13 @@
         </is>
       </c>
       <c r="B19" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C19" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D19" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4768,34 +4768,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>10.03584229390681</v>
+        <v>10.39426523297491</v>
       </c>
       <c r="R19" t="n">
         <v>19</v>
       </c>
       <c r="S19" t="n">
-        <v>8.964157706093189</v>
+        <v>8.605734767025091</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="137" t="n">
-        <v>903.2258064516128</v>
+        <v>935.483870967742</v>
       </c>
       <c r="V19" s="137" t="n">
-        <v>742.34</v>
+        <v>747.83</v>
       </c>
       <c r="W19" s="137" t="n">
-        <v>-160.8858064516129</v>
+        <v>-187.6538709677419</v>
       </c>
       <c r="X19" s="138" t="n">
-        <v>-0.1781235714285714</v>
+        <v>-0.2005955172413792</v>
       </c>
       <c r="Y19" s="137" t="n">
-        <v>39.07052631578947</v>
+        <v>39.35947368421053</v>
       </c>
       <c r="Z19" s="137" t="n">
-        <v>-50.92947368421053</v>
+        <v>-50.64052631578947</v>
       </c>
       <c r="AB19" s="139" t="inlineStr"/>
       <c r="AC19" s="139" t="inlineStr">
@@ -4822,13 +4822,13 @@
         </is>
       </c>
       <c r="B20" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C20" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D20" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
@@ -4875,34 +4875,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>3.763440860215054</v>
+        <v>3.897849462365592</v>
       </c>
       <c r="R20" t="n">
         <v>4</v>
       </c>
       <c r="S20" t="n">
-        <v>0.2365591397849455</v>
+        <v>0.102150537634408</v>
       </c>
       <c r="T20" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U20" s="137" t="n">
-        <v>451.6129032258065</v>
+        <v>467.741935483871</v>
       </c>
       <c r="V20" s="137" t="n">
-        <v>387.91</v>
+        <v>393.09</v>
       </c>
       <c r="W20" s="137" t="n">
-        <v>-63.70290322580644</v>
+        <v>-74.651935483871</v>
       </c>
       <c r="X20" s="138" t="n">
-        <v>-0.1410564285714285</v>
+        <v>-0.1596006896551725</v>
       </c>
       <c r="Y20" s="137" t="n">
-        <v>96.97750000000001</v>
+        <v>98.27249999999999</v>
       </c>
       <c r="Z20" s="137" t="n">
-        <v>-23.0225</v>
+        <v>-21.72750000000001</v>
       </c>
       <c r="AB20" s="139" t="inlineStr"/>
       <c r="AC20" s="139" t="inlineStr">
@@ -4929,13 +4929,13 @@
         </is>
       </c>
       <c r="B21" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C21" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D21" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4982,28 +4982,28 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>33.87096774193549</v>
+        <v>35.08064516129032</v>
       </c>
       <c r="R21" t="n">
         <v>22</v>
       </c>
       <c r="S21" t="n">
-        <v>-11.87096774193549</v>
+        <v>-13.08064516129032</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="137" t="n">
-        <v>1354.83870967742</v>
+        <v>1403.225806451613</v>
       </c>
       <c r="V21" s="137" t="n">
         <v>1414.698441</v>
       </c>
       <c r="W21" s="137" t="n">
-        <v>59.8597313225805</v>
+        <v>11.47263454838708</v>
       </c>
       <c r="X21" s="138" t="n">
-        <v>0.044182182642857</v>
+        <v>0.0081759004827586</v>
       </c>
       <c r="Y21" s="137" t="n">
         <v>64.30447459090909</v>
@@ -5036,13 +5036,13 @@
         </is>
       </c>
       <c r="B22" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C22" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D22" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -5089,28 +5089,28 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>90.32258064516128</v>
+        <v>93.54838709677421</v>
       </c>
       <c r="R22" t="n">
         <v>114</v>
       </c>
       <c r="S22" t="n">
-        <v>23.67741935483872</v>
+        <v>20.45161290322581</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="137" t="n">
-        <v>1354.83870967742</v>
+        <v>1403.225806451613</v>
       </c>
       <c r="V22" s="137" t="n">
         <v>1928.318895</v>
       </c>
       <c r="W22" s="137" t="n">
-        <v>573.4801853225806</v>
+        <v>525.0930885483872</v>
       </c>
       <c r="X22" s="138" t="n">
-        <v>0.4232829939285714</v>
+        <v>0.37420427</v>
       </c>
       <c r="Y22" s="137" t="n">
         <v>16.91507802631579</v>
@@ -5148,13 +5148,13 @@
         </is>
       </c>
       <c r="B23" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C23" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D23" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5201,34 +5201,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>34.7394540942928</v>
+        <v>35.98014888337469</v>
       </c>
       <c r="R23" t="n">
         <v>67</v>
       </c>
       <c r="S23" t="n">
-        <v>32.2605459057072</v>
+        <v>31.01985111662531</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="137" t="n">
-        <v>903.2258064516128</v>
+        <v>935.483870967742</v>
       </c>
       <c r="V23" s="137" t="n">
-        <v>1282.1</v>
+        <v>1308.82</v>
       </c>
       <c r="W23" s="137" t="n">
-        <v>378.874193548387</v>
+        <v>373.336129032258</v>
       </c>
       <c r="X23" s="138" t="n">
-        <v>0.419467857142857</v>
+        <v>0.3990834482758619</v>
       </c>
       <c r="Y23" s="137" t="n">
-        <v>19.13582089552238</v>
+        <v>19.53462686567164</v>
       </c>
       <c r="Z23" s="137" t="n">
-        <v>-6.864179104477614</v>
+        <v>-6.46537313432836</v>
       </c>
       <c r="AB23" s="139" t="inlineStr"/>
       <c r="AC23" s="139" t="inlineStr">
@@ -5255,13 +5255,13 @@
         </is>
       </c>
       <c r="B24" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C24" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D24" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5298,12 +5298,12 @@
       <c r="T24" s="137" t="n"/>
       <c r="U24" s="137" t="n"/>
       <c r="V24" s="137" t="n">
-        <v>705.61</v>
+        <v>732.3</v>
       </c>
       <c r="W24" s="137" t="n"/>
       <c r="X24" s="138" t="n"/>
       <c r="Y24" s="137" t="n">
-        <v>705.61</v>
+        <v>732.3</v>
       </c>
       <c r="Z24" s="137" t="n"/>
       <c r="AB24" s="139" t="inlineStr"/>
@@ -5331,13 +5331,13 @@
         </is>
       </c>
       <c r="B25" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C25" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D25" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5366,34 +5366,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>421.505376344086</v>
+        <v>436.5591397849462</v>
       </c>
       <c r="R25" t="n">
         <v>328</v>
       </c>
       <c r="S25" t="n">
-        <v>-93.50537634408602</v>
+        <v>-108.5591397849462</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="137" t="n">
-        <v>18967.74193548387</v>
+        <v>19645.16129032258</v>
       </c>
       <c r="V25" s="137" t="n">
-        <v>16631.343483</v>
+        <v>16764.683483</v>
       </c>
       <c r="W25" s="137" t="n">
-        <v>-2336.39845248387</v>
+        <v>-2880.477807322579</v>
       </c>
       <c r="X25" s="138" t="n">
-        <v>-0.1231774694336734</v>
+        <v>-0.1466253071050902</v>
       </c>
       <c r="Y25" s="137" t="n">
-        <v>50.70531549695122</v>
+        <v>51.11183988719512</v>
       </c>
       <c r="Z25" s="137" t="n">
-        <v>5.705315496951222</v>
+        <v>6.111839887195124</v>
       </c>
       <c r="AB25" s="139" t="inlineStr"/>
       <c r="AC25" s="139" t="inlineStr"/>
@@ -5411,13 +5411,13 @@
         </is>
       </c>
       <c r="B26" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C26" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D26" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5451,34 +5451,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>1234.45532749927</v>
+        <v>1278.543017767101</v>
       </c>
       <c r="R26" t="n">
         <v>967</v>
       </c>
       <c r="S26" t="n">
-        <v>-267.4553274992704</v>
+        <v>-311.5430177671014</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="137" t="n">
-        <v>28000</v>
+        <v>29000</v>
       </c>
       <c r="V26" s="137" t="n">
-        <v>31919.712734</v>
+        <v>32116.742734</v>
       </c>
       <c r="W26" s="137" t="n">
-        <v>3919.712734000001</v>
+        <v>3116.742733999999</v>
       </c>
       <c r="X26" s="138" t="n">
-        <v>0.1399897405</v>
+        <v>0.1074738873793103</v>
       </c>
       <c r="Y26" s="137" t="n">
-        <v>33.00901006618408</v>
+        <v>33.21276394415719</v>
       </c>
       <c r="Z26" s="137" t="n">
-        <v>10.32694180801412</v>
+        <v>10.53069568598723</v>
       </c>
       <c r="AB26" s="139" t="inlineStr"/>
       <c r="AC26" s="139" t="inlineStr"/>
@@ -5496,13 +5496,13 @@
         </is>
       </c>
       <c r="B27" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C27" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D27" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5536,28 +5536,28 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>1221.467647613658</v>
+        <v>1265.091492171289</v>
       </c>
       <c r="R27" t="n">
         <v>798</v>
       </c>
       <c r="S27" t="n">
-        <v>-423.4676476136578</v>
+        <v>-467.0914921712886</v>
       </c>
       <c r="T27" s="137" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="U27" s="137" t="n">
-        <v>9565.217391304348</v>
+        <v>10043.47826086957</v>
       </c>
       <c r="V27" s="137" t="n">
         <v>6422.6</v>
       </c>
       <c r="W27" s="137" t="n">
-        <v>-3142.617391304348</v>
+        <v>-3620.878260869566</v>
       </c>
       <c r="X27" s="138" t="n">
-        <v>-0.3285463636363636</v>
+        <v>-0.3605203463203463</v>
       </c>
       <c r="Y27" s="137" t="n">
         <v>8.048370927318297</v>
@@ -5581,13 +5581,13 @@
         </is>
       </c>
       <c r="B28" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C28" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D28" s="136" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5621,34 +5621,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>2877.428351457014</v>
+        <v>2980.193649723336</v>
       </c>
       <c r="R28" t="n">
         <v>2093</v>
       </c>
       <c r="S28" t="n">
-        <v>-784.4283514570143</v>
+        <v>-887.1936497233364</v>
       </c>
       <c r="T28" s="137" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="U28" s="137" t="n">
-        <v>56532.95932678822</v>
+        <v>58688.63955119214</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>54973.656217</v>
+        <v>55304.026217</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>-1559.303109788212</v>
+        <v>-3384.613334192145</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>-0.027582195030242</v>
+        <v>-0.0576706728947066</v>
       </c>
       <c r="Y28" s="137" t="n">
-        <v>26.26548314237936</v>
+        <v>26.42332834065934</v>
       </c>
       <c r="Z28" s="137" t="n">
-        <v>6.489760220334023</v>
+        <v>6.647605418613999</v>
       </c>
       <c r="AB28" s="139" t="inlineStr"/>
       <c r="AC28" s="139" t="inlineStr"/>
@@ -5751,7 +5751,7 @@
         </is>
       </c>
       <c r="B4" s="140" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5791,7 +5791,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5811,7 +5811,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46232.29190972223</v>
+        <v>46233.291875</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento lead CRM al 2026-07-29
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 29/07/2026  |  Ultimo aggiornamento: 30/07/2026 07:00</t>
+          <t>Periodo: 01/07/2026 - 29/07/2026  |  Ultimo aggiornamento: 30/07/2026 12:11</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1331,10 +1331,10 @@
         <v>436.5591397849462</v>
       </c>
       <c r="N10" s="125" t="n">
-        <v>328</v>
+        <v>451</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>-108.5591397849462</v>
+        <v>14.44086021505376</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
@@ -1352,10 +1352,10 @@
         <v>-0.1466253071050902</v>
       </c>
       <c r="U10" s="123" t="n">
-        <v>51.11183988719512</v>
+        <v>37.17224719068737</v>
       </c>
       <c r="V10" s="123" t="n">
-        <v>6.111839887195124</v>
+        <v>-7.827752809312635</v>
       </c>
       <c r="W10" s="126" t="n"/>
     </row>
@@ -1410,10 +1410,10 @@
         <v>110.0569259962049</v>
       </c>
       <c r="N11" s="119" t="n">
-        <v>111</v>
+        <v>138</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>0.9430740037950756</v>
+        <v>27.94307400379508</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
@@ -1431,10 +1431,10 @@
         <v>0.0779101669137931</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>36.33757028828829</v>
+        <v>29.22804566666667</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>2.33757028828829</v>
+        <v>-4.771954333333333</v>
       </c>
       <c r="W11" s="120" t="inlineStr">
         <is>
@@ -1493,10 +1493,10 @@
         <v>218.6845412651865</v>
       </c>
       <c r="N12" s="119" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>-50.68454126518643</v>
+        <v>20.31545873481357</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
@@ -1514,10 +1514,10 @@
         <v>-0.0501464280574713</v>
       </c>
       <c r="U12" s="128" t="n">
-        <v>47.60210873214286</v>
+        <v>33.46089651464435</v>
       </c>
       <c r="V12" s="128" t="n">
-        <v>9.10210873214286</v>
+        <v>-5.039103485355646</v>
       </c>
       <c r="W12" s="120" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="L13" s="113" t="n"/>
       <c r="M13" s="113" t="n"/>
       <c r="N13" s="119" t="n">
-        <v>107</v>
+        <v>177</v>
       </c>
       <c r="O13" s="113" t="n"/>
       <c r="P13" s="117" t="n"/>
@@ -1626,7 +1626,7 @@
         <v>5</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-14.61799660441426</v>
+        <v>-8.617996604414259</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
@@ -1644,10 +1644,10 @@
         <v>-0.0877036681379309</v>
       </c>
       <c r="U14" s="128" t="n">
-        <v>85.34385040000001</v>
+        <v>53.3399065</v>
       </c>
       <c r="V14" s="128" t="n">
-        <v>47.34385040000001</v>
+        <v>15.3399065</v>
       </c>
       <c r="W14" s="120" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
       <c r="L15" s="113" t="n"/>
       <c r="M15" s="113" t="n"/>
       <c r="N15" s="119" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="O15" s="113" t="n"/>
       <c r="P15" s="117" t="n"/>
@@ -1753,10 +1753,10 @@
         <v>3.741935483870968</v>
       </c>
       <c r="N16" s="119" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>-1.741935483870968</v>
+        <v>1.258064516129032</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
@@ -1774,10 +1774,10 @@
         <v>-0.0642678594827587</v>
       </c>
       <c r="U16" s="128" t="n">
-        <v>437.6811625</v>
+        <v>175.072465</v>
       </c>
       <c r="V16" s="128" t="n">
-        <v>187.6811625</v>
+        <v>-74.92753500000001</v>
       </c>
       <c r="W16" s="120" t="inlineStr">
         <is>
@@ -1820,7 +1820,7 @@
       <c r="L17" s="113" t="n"/>
       <c r="M17" s="113" t="n"/>
       <c r="N17" s="119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O17" s="113" t="n"/>
       <c r="P17" s="117" t="n"/>
@@ -1883,10 +1883,10 @@
         <v>730.8467741935484</v>
       </c>
       <c r="N18" s="119" t="n">
-        <v>417</v>
+        <v>600</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-313.8467741935484</v>
+        <v>-130.8467741935484</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
@@ -1904,10 +1904,10 @@
         <v>0.2182155517241379</v>
       </c>
       <c r="U18" s="117" t="n">
-        <v>27.32904076738609</v>
+        <v>18.99368333333333</v>
       </c>
       <c r="V18" s="117" t="n">
-        <v>14.52904076738609</v>
+        <v>6.193683333333333</v>
       </c>
       <c r="W18" s="120" t="inlineStr">
         <is>
@@ -1966,10 +1966,10 @@
         <v>11.69354838709677</v>
       </c>
       <c r="N19" s="119" t="n">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>20.30645161290322</v>
+        <v>34.30645161290322</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
@@ -1987,10 +1987,10 @@
         <v>-0.0677551724137931</v>
       </c>
       <c r="U19" s="117" t="n">
-        <v>13.6265625</v>
+        <v>9.479347826086956</v>
       </c>
       <c r="V19" s="117" t="n">
-        <v>-26.3734375</v>
+        <v>-30.52065217391304</v>
       </c>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
@@ -2045,10 +2045,10 @@
         <v>10.39426523297491</v>
       </c>
       <c r="N20" s="119" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>8.605734767025091</v>
+        <v>13.60573476702509</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
@@ -2066,10 +2066,10 @@
         <v>-0.2005955172413792</v>
       </c>
       <c r="U20" s="117" t="n">
-        <v>39.35947368421053</v>
+        <v>31.15958333333333</v>
       </c>
       <c r="V20" s="117" t="n">
-        <v>-50.64052631578947</v>
+        <v>-58.84041666666667</v>
       </c>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
@@ -2203,10 +2203,10 @@
         <v>35.08064516129032</v>
       </c>
       <c r="N22" s="119" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-13.08064516129032</v>
+        <v>-3.08064516129032</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
@@ -2224,10 +2224,10 @@
         <v>0.0081759004827586</v>
       </c>
       <c r="U22" s="117" t="n">
-        <v>64.30447459090909</v>
+        <v>44.20932628125</v>
       </c>
       <c r="V22" s="117" t="n">
-        <v>24.30447459090909</v>
+        <v>4.20932628125</v>
       </c>
       <c r="W22" s="120" t="inlineStr"/>
     </row>
@@ -2282,10 +2282,10 @@
         <v>93.54838709677421</v>
       </c>
       <c r="N23" s="119" t="n">
-        <v>114</v>
+        <v>169</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>20.45161290322581</v>
+        <v>75.45161290322581</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
@@ -2303,10 +2303,10 @@
         <v>0.37420427</v>
       </c>
       <c r="U23" s="117" t="n">
-        <v>16.91507802631579</v>
+        <v>11.41017097633136</v>
       </c>
       <c r="V23" s="117" t="n">
-        <v>1.91507802631579</v>
+        <v>-3.589829023668639</v>
       </c>
       <c r="W23" s="120" t="inlineStr">
         <is>
@@ -2365,10 +2365,10 @@
         <v>35.98014888337469</v>
       </c>
       <c r="N24" s="119" t="n">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>31.01985111662531</v>
+        <v>49.01985111662531</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
@@ -2386,10 +2386,10 @@
         <v>0.3990834482758619</v>
       </c>
       <c r="U24" s="117" t="n">
-        <v>19.53462686567164</v>
+        <v>15.39788235294118</v>
       </c>
       <c r="V24" s="117" t="n">
-        <v>-6.46537313432836</v>
+        <v>-10.60211764705882</v>
       </c>
       <c r="W24" s="120" t="inlineStr"/>
     </row>
@@ -2430,7 +2430,7 @@
       <c r="L25" s="119" t="n"/>
       <c r="M25" s="119" t="n"/>
       <c r="N25" s="119" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="O25" s="119" t="n"/>
       <c r="P25" s="117" t="n"/>
@@ -2441,7 +2441,7 @@
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
       <c r="U25" s="117" t="n">
-        <v>732.3</v>
+        <v>45.76875</v>
       </c>
       <c r="V25" s="117" t="n"/>
       <c r="W25" s="120" t="inlineStr"/>
@@ -2481,10 +2481,10 @@
         <v>1278.543017767101</v>
       </c>
       <c r="N26" s="125" t="n">
-        <v>967</v>
+        <v>1374</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>-311.5430177671014</v>
+        <v>95.45698223289855</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
@@ -2502,10 +2502,10 @@
         <v>0.1074738873793103</v>
       </c>
       <c r="U26" s="123" t="n">
-        <v>33.21276394415719</v>
+        <v>23.37463081077147</v>
       </c>
       <c r="V26" s="123" t="n">
-        <v>10.53069568598723</v>
+        <v>0.6925625526015153</v>
       </c>
       <c r="W26" s="126" t="n"/>
     </row>
@@ -2556,10 +2556,10 @@
         <v>615.4499151103566</v>
       </c>
       <c r="N27" s="119" t="n">
-        <v>371</v>
+        <v>472</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-244.4499151103566</v>
+        <v>-143.4499151103566</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>217.3913043478261</v>
@@ -2568,13 +2568,13 @@
         <v>4565.217391304348</v>
       </c>
       <c r="R27" s="117" t="n">
-        <v>2819.6</v>
+        <v>3587.2</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-1745.617391304348</v>
+        <v>-978.0173913043482</v>
       </c>
       <c r="T27" s="118" t="n">
-        <v>-0.3823733333333334</v>
+        <v>-0.214232380952381</v>
       </c>
       <c r="U27" s="117" t="n">
         <v>7.6</v>
@@ -2631,10 +2631,10 @@
         <v>415.7706093189964</v>
       </c>
       <c r="N28" s="119" t="n">
-        <v>187</v>
+        <v>281</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-228.7706093189964</v>
+        <v>-134.7706093189964</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>173.9130434782609</v>
@@ -2643,13 +2643,13 @@
         <v>3652.173913043479</v>
       </c>
       <c r="R28" s="117" t="n">
-        <v>1683</v>
+        <v>2529</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-1969.173913043478</v>
+        <v>-1123.173913043478</v>
       </c>
       <c r="T28" s="118" t="n">
-        <v>-0.5391785714285715</v>
+        <v>-0.3075357142857143</v>
       </c>
       <c r="U28" s="117" t="n">
         <v>9</v>
@@ -2706,10 +2706,10 @@
         <v>233.8709677419355</v>
       </c>
       <c r="N29" s="119" t="n">
-        <v>240</v>
+        <v>281</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>6.129032258064512</v>
+        <v>47.12903225806451</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>86.95652173913044</v>
@@ -2718,13 +2718,13 @@
         <v>1826.086956521739</v>
       </c>
       <c r="R29" s="117" t="n">
-        <v>1920</v>
+        <v>2248</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>93.91304347826076</v>
+        <v>421.9130434782608</v>
       </c>
       <c r="T29" s="118" t="n">
-        <v>0.0514285714285713</v>
+        <v>0.2310476190476189</v>
       </c>
       <c r="U29" s="117" t="n">
         <v>8</v>
@@ -2769,10 +2769,10 @@
         <v>1265.091492171289</v>
       </c>
       <c r="N30" s="125" t="n">
-        <v>798</v>
+        <v>1034</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-467.0914921712886</v>
+        <v>-231.0914921712886</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>478.2608695652174</v>
@@ -2781,19 +2781,19 @@
         <v>10043.47826086957</v>
       </c>
       <c r="R30" s="123" t="n">
-        <v>6422.6</v>
+        <v>8364.200000000001</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>-3620.878260869566</v>
+        <v>-1679.278260869565</v>
       </c>
       <c r="T30" s="124" t="n">
-        <v>-0.3605203463203463</v>
+        <v>-0.1672008658008658</v>
       </c>
       <c r="U30" s="123" t="n">
-        <v>8.048370927318297</v>
+        <v>8.089168278529982</v>
       </c>
       <c r="V30" s="123" t="n">
-        <v>-0.0856831267357574</v>
+        <v>-0.0448857755240723</v>
       </c>
       <c r="W30" s="126" t="n"/>
     </row>
@@ -2832,10 +2832,10 @@
         <v>2980.193649723336</v>
       </c>
       <c r="N31" s="133" t="n">
-        <v>2093</v>
+        <v>2859</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>-887.1936497233364</v>
+        <v>-121.1936497233364</v>
       </c>
       <c r="P31" s="131" t="n">
         <v>2155.680224403927</v>
@@ -2844,19 +2844,19 @@
         <v>58688.63955119214</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>55304.026217</v>
+        <v>57245.626217</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>-3384.613334192145</v>
+        <v>-1443.013334192146</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>-0.0576706728947066</v>
+        <v>-0.0245876092072888</v>
       </c>
       <c r="U31" s="131" t="n">
-        <v>26.42332834065934</v>
+        <v>20.0229542556838</v>
       </c>
       <c r="V31" s="131" t="n">
-        <v>6.647605418613999</v>
+        <v>0.2472313336384637</v>
       </c>
       <c r="W31" s="134" t="n"/>
     </row>
@@ -3207,7 +3207,7 @@
       <c r="AD2" s="139" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>google:stale;google:includes_excel_row_3;crm:stale</t>
+          <t>google:stale;google:includes_excel_row_3</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -3274,7 +3274,7 @@
       <c r="AD3" s="139" t="inlineStr"/>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_2;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_2</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -3360,7 +3360,7 @@
       <c r="AD4" s="139" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>google:stale;google:includes_excel_row_5;crm:stale</t>
+          <t>google:stale;google:includes_excel_row_5</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -3427,7 +3427,7 @@
       <c r="AD5" s="139" t="inlineStr"/>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_4;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_4</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -3513,7 +3513,7 @@
       <c r="AD6" s="139" t="inlineStr"/>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -3585,10 +3585,10 @@
         <v>615.4499151103566</v>
       </c>
       <c r="R7" t="n">
-        <v>371</v>
+        <v>472</v>
       </c>
       <c r="S7" t="n">
-        <v>-244.4499151103566</v>
+        <v>-143.4499151103566</v>
       </c>
       <c r="T7" s="137" t="n">
         <v>217.3913043478261</v>
@@ -3597,13 +3597,13 @@
         <v>4565.217391304348</v>
       </c>
       <c r="V7" s="137" t="n">
-        <v>2819.6</v>
+        <v>3587.2</v>
       </c>
       <c r="W7" s="137" t="n">
-        <v>-1745.617391304348</v>
+        <v>-978.0173913043482</v>
       </c>
       <c r="X7" s="138" t="n">
-        <v>-0.3823733333333334</v>
+        <v>-0.214232380952381</v>
       </c>
       <c r="Y7" s="137" t="n">
         <v>7.6</v>
@@ -3616,7 +3616,7 @@
       <c r="AD7" s="139" t="inlineStr"/>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>manual:no_ads_source;crm:stale</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -3688,10 +3688,10 @@
         <v>415.7706093189964</v>
       </c>
       <c r="R8" t="n">
-        <v>187</v>
+        <v>281</v>
       </c>
       <c r="S8" t="n">
-        <v>-228.7706093189964</v>
+        <v>-134.7706093189964</v>
       </c>
       <c r="T8" s="137" t="n">
         <v>173.9130434782609</v>
@@ -3700,13 +3700,13 @@
         <v>3652.173913043479</v>
       </c>
       <c r="V8" s="137" t="n">
-        <v>1683</v>
+        <v>2529</v>
       </c>
       <c r="W8" s="137" t="n">
-        <v>-1969.173913043478</v>
+        <v>-1123.173913043478</v>
       </c>
       <c r="X8" s="138" t="n">
-        <v>-0.5391785714285715</v>
+        <v>-0.3075357142857143</v>
       </c>
       <c r="Y8" s="137" t="n">
         <v>9</v>
@@ -3719,7 +3719,7 @@
       <c r="AD8" s="139" t="inlineStr"/>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>manual:no_ads_source;crm:stale</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -3791,10 +3791,10 @@
         <v>233.8709677419355</v>
       </c>
       <c r="R9" t="n">
-        <v>240</v>
+        <v>281</v>
       </c>
       <c r="S9" t="n">
-        <v>6.129032258064512</v>
+        <v>47.12903225806451</v>
       </c>
       <c r="T9" s="137" t="n">
         <v>86.95652173913044</v>
@@ -3803,13 +3803,13 @@
         <v>1826.086956521739</v>
       </c>
       <c r="V9" s="137" t="n">
-        <v>1920</v>
+        <v>2248</v>
       </c>
       <c r="W9" s="137" t="n">
-        <v>93.91304347826076</v>
+        <v>421.9130434782608</v>
       </c>
       <c r="X9" s="138" t="n">
-        <v>0.0514285714285713</v>
+        <v>0.2310476190476189</v>
       </c>
       <c r="Y9" s="137" t="n">
         <v>8</v>
@@ -3822,7 +3822,7 @@
       <c r="AD9" s="139" t="inlineStr"/>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>manual:no_ads_source;crm:stale</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -3894,10 +3894,10 @@
         <v>110.0569259962049</v>
       </c>
       <c r="R10" t="n">
-        <v>111</v>
+        <v>138</v>
       </c>
       <c r="S10" t="n">
-        <v>0.9430740037950756</v>
+        <v>27.94307400379508</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
@@ -3915,10 +3915,10 @@
         <v>0.0779101669137931</v>
       </c>
       <c r="Y10" s="137" t="n">
-        <v>36.33757028828829</v>
+        <v>29.22804566666667</v>
       </c>
       <c r="Z10" s="137" t="n">
-        <v>2.33757028828829</v>
+        <v>-4.771954333333333</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -3934,7 +3934,7 @@
       <c r="AD10" s="139" t="inlineStr"/>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>google:stale;crm:stale</t>
+          <t>google:stale</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -4006,10 +4006,10 @@
         <v>218.6845412651865</v>
       </c>
       <c r="R11" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="S11" t="n">
-        <v>-50.68454126518643</v>
+        <v>20.31545873481357</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
@@ -4027,10 +4027,10 @@
         <v>-0.0501464280574713</v>
       </c>
       <c r="Y11" s="137" t="n">
-        <v>47.60210873214286</v>
+        <v>33.46089651464435</v>
       </c>
       <c r="Z11" s="137" t="n">
-        <v>9.10210873214286</v>
+        <v>-5.039103485355646</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -4046,7 +4046,7 @@
       <c r="AD11" s="139" t="inlineStr"/>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>google:stale;google:includes_excel_row_10;crm_metrics_combined_with_excel_row_10;crm:stale</t>
+          <t>google:stale;google:includes_excel_row_10;crm_metrics_combined_with_excel_row_10</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -4098,7 +4098,7 @@
       <c r="L12" s="137" t="n"/>
       <c r="N12" s="137" t="n"/>
       <c r="R12" t="n">
-        <v>107</v>
+        <v>177</v>
       </c>
       <c r="T12" s="137" t="n"/>
       <c r="U12" s="137" t="n"/>
@@ -4116,7 +4116,7 @@
       <c r="AD12" s="139" t="inlineStr"/>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_9;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_9</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -4191,7 +4191,7 @@
         <v>5</v>
       </c>
       <c r="S13" t="n">
-        <v>-14.61799660441426</v>
+        <v>-8.617996604414259</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
@@ -4209,10 +4209,10 @@
         <v>-0.0877036681379309</v>
       </c>
       <c r="Y13" s="137" t="n">
-        <v>85.34385040000001</v>
+        <v>53.3399065</v>
       </c>
       <c r="Z13" s="137" t="n">
-        <v>47.34385040000001</v>
+        <v>15.3399065</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -4228,7 +4228,7 @@
       <c r="AD13" s="139" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>google:stale;google:includes_excel_row_12;crm_metrics_combined_with_excel_row_12;crm:stale</t>
+          <t>google:stale;google:includes_excel_row_12;crm_metrics_combined_with_excel_row_12</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -4280,7 +4280,7 @@
       <c r="L14" s="137" t="n"/>
       <c r="N14" s="137" t="n"/>
       <c r="R14" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="T14" s="137" t="n"/>
       <c r="U14" s="137" t="n"/>
@@ -4298,7 +4298,7 @@
       <c r="AD14" s="139" t="inlineStr"/>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_11;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_11</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -4370,10 +4370,10 @@
         <v>3.741935483870968</v>
       </c>
       <c r="R15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S15" t="n">
-        <v>-1.741935483870968</v>
+        <v>1.258064516129032</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
@@ -4391,10 +4391,10 @@
         <v>-0.0642678594827587</v>
       </c>
       <c r="Y15" s="137" t="n">
-        <v>437.6811625</v>
+        <v>175.072465</v>
       </c>
       <c r="Z15" s="137" t="n">
-        <v>187.6811625</v>
+        <v>-74.92753500000001</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -4410,7 +4410,7 @@
       <c r="AD15" s="139" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>google:stale;google:includes_excel_row_14;crm_metrics_combined_with_excel_row_14;crm:stale</t>
+          <t>google:stale;google:includes_excel_row_14;crm_metrics_combined_with_excel_row_14</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -4462,7 +4462,7 @@
       <c r="L16" s="137" t="n"/>
       <c r="N16" s="137" t="n"/>
       <c r="R16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T16" s="137" t="n"/>
       <c r="U16" s="137" t="n"/>
@@ -4480,7 +4480,7 @@
       <c r="AD16" s="139" t="inlineStr"/>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_13;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_13</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -4552,10 +4552,10 @@
         <v>730.8467741935484</v>
       </c>
       <c r="R17" t="n">
-        <v>417</v>
+        <v>600</v>
       </c>
       <c r="S17" t="n">
-        <v>-313.8467741935484</v>
+        <v>-130.8467741935484</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
@@ -4573,10 +4573,10 @@
         <v>0.2182155517241379</v>
       </c>
       <c r="Y17" s="137" t="n">
-        <v>27.32904076738609</v>
+        <v>18.99368333333333</v>
       </c>
       <c r="Z17" s="137" t="n">
-        <v>14.52904076738609</v>
+        <v>6.193683333333333</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -4592,7 +4592,7 @@
       <c r="AD17" s="139" t="inlineStr"/>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
@@ -4664,10 +4664,10 @@
         <v>11.69354838709677</v>
       </c>
       <c r="R18" t="n">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="S18" t="n">
-        <v>20.30645161290322</v>
+        <v>34.30645161290322</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
@@ -4685,10 +4685,10 @@
         <v>-0.0677551724137931</v>
       </c>
       <c r="Y18" s="137" t="n">
-        <v>13.6265625</v>
+        <v>9.479347826086956</v>
       </c>
       <c r="Z18" s="137" t="n">
-        <v>-26.3734375</v>
+        <v>-30.52065217391304</v>
       </c>
       <c r="AB18" s="139" t="inlineStr"/>
       <c r="AC18" s="139" t="inlineStr">
@@ -4699,7 +4699,7 @@
       <c r="AD18" s="139" t="inlineStr"/>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
@@ -4771,10 +4771,10 @@
         <v>10.39426523297491</v>
       </c>
       <c r="R19" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="S19" t="n">
-        <v>8.605734767025091</v>
+        <v>13.60573476702509</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
@@ -4792,10 +4792,10 @@
         <v>-0.2005955172413792</v>
       </c>
       <c r="Y19" s="137" t="n">
-        <v>39.35947368421053</v>
+        <v>31.15958333333333</v>
       </c>
       <c r="Z19" s="137" t="n">
-        <v>-50.64052631578947</v>
+        <v>-58.84041666666667</v>
       </c>
       <c r="AB19" s="139" t="inlineStr"/>
       <c r="AC19" s="139" t="inlineStr">
@@ -4806,7 +4806,7 @@
       <c r="AD19" s="139" t="inlineStr"/>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
@@ -4913,7 +4913,7 @@
       <c r="AD20" s="139" t="inlineStr"/>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr">
@@ -4985,10 +4985,10 @@
         <v>35.08064516129032</v>
       </c>
       <c r="R21" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="S21" t="n">
-        <v>-13.08064516129032</v>
+        <v>-3.08064516129032</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
@@ -5006,10 +5006,10 @@
         <v>0.0081759004827586</v>
       </c>
       <c r="Y21" s="137" t="n">
-        <v>64.30447459090909</v>
+        <v>44.20932628125</v>
       </c>
       <c r="Z21" s="137" t="n">
-        <v>24.30447459090909</v>
+        <v>4.20932628125</v>
       </c>
       <c r="AB21" s="139" t="inlineStr">
         <is>
@@ -5020,7 +5020,7 @@
       <c r="AD21" s="139" t="inlineStr"/>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>google:stale;crm:stale</t>
+          <t>google:stale</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
@@ -5092,10 +5092,10 @@
         <v>93.54838709677421</v>
       </c>
       <c r="R22" t="n">
-        <v>114</v>
+        <v>169</v>
       </c>
       <c r="S22" t="n">
-        <v>20.45161290322581</v>
+        <v>75.45161290322581</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
@@ -5113,10 +5113,10 @@
         <v>0.37420427</v>
       </c>
       <c r="Y22" s="137" t="n">
-        <v>16.91507802631579</v>
+        <v>11.41017097633136</v>
       </c>
       <c r="Z22" s="137" t="n">
-        <v>1.91507802631579</v>
+        <v>-3.589829023668639</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       <c r="AD22" s="139" t="inlineStr"/>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>google:stale;crm:stale</t>
+          <t>google:stale</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
@@ -5204,10 +5204,10 @@
         <v>35.98014888337469</v>
       </c>
       <c r="R23" t="n">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="S23" t="n">
-        <v>31.01985111662531</v>
+        <v>49.01985111662531</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
@@ -5225,10 +5225,10 @@
         <v>0.3990834482758619</v>
       </c>
       <c r="Y23" s="137" t="n">
-        <v>19.53462686567164</v>
+        <v>15.39788235294118</v>
       </c>
       <c r="Z23" s="137" t="n">
-        <v>-6.46537313432836</v>
+        <v>-10.60211764705882</v>
       </c>
       <c r="AB23" s="139" t="inlineStr"/>
       <c r="AC23" s="139" t="inlineStr">
@@ -5239,7 +5239,7 @@
       <c r="AD23" s="139" t="inlineStr"/>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -5293,7 +5293,7 @@
       <c r="L24" s="137" t="n"/>
       <c r="N24" s="137" t="n"/>
       <c r="R24" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="T24" s="137" t="n"/>
       <c r="U24" s="137" t="n"/>
@@ -5303,7 +5303,7 @@
       <c r="W24" s="137" t="n"/>
       <c r="X24" s="138" t="n"/>
       <c r="Y24" s="137" t="n">
-        <v>732.3</v>
+        <v>45.76875</v>
       </c>
       <c r="Z24" s="137" t="n"/>
       <c r="AB24" s="139" t="inlineStr"/>
@@ -5315,7 +5315,7 @@
       <c r="AD24" s="139" t="inlineStr"/>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
@@ -5369,10 +5369,10 @@
         <v>436.5591397849462</v>
       </c>
       <c r="R25" t="n">
-        <v>328</v>
+        <v>451</v>
       </c>
       <c r="S25" t="n">
-        <v>-108.5591397849462</v>
+        <v>14.44086021505376</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
@@ -5390,17 +5390,17 @@
         <v>-0.1466253071050902</v>
       </c>
       <c r="Y25" s="137" t="n">
-        <v>51.11183988719512</v>
+        <v>37.17224719068737</v>
       </c>
       <c r="Z25" s="137" t="n">
-        <v>6.111839887195124</v>
+        <v>-7.827752809312635</v>
       </c>
       <c r="AB25" s="139" t="inlineStr"/>
       <c r="AC25" s="139" t="inlineStr"/>
       <c r="AD25" s="139" t="inlineStr"/>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>partial;crm:stale</t>
+          <t>partial</t>
         </is>
       </c>
     </row>
@@ -5454,10 +5454,10 @@
         <v>1278.543017767101</v>
       </c>
       <c r="R26" t="n">
-        <v>967</v>
+        <v>1374</v>
       </c>
       <c r="S26" t="n">
-        <v>-311.5430177671014</v>
+        <v>95.45698223289855</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
@@ -5475,17 +5475,17 @@
         <v>0.1074738873793103</v>
       </c>
       <c r="Y26" s="137" t="n">
-        <v>33.21276394415719</v>
+        <v>23.37463081077147</v>
       </c>
       <c r="Z26" s="137" t="n">
-        <v>10.53069568598723</v>
+        <v>0.6925625526015153</v>
       </c>
       <c r="AB26" s="139" t="inlineStr"/>
       <c r="AC26" s="139" t="inlineStr"/>
       <c r="AD26" s="139" t="inlineStr"/>
       <c r="AE26" t="inlineStr">
         <is>
-          <t>partial;crm:stale</t>
+          <t>partial</t>
         </is>
       </c>
     </row>
@@ -5539,10 +5539,10 @@
         <v>1265.091492171289</v>
       </c>
       <c r="R27" t="n">
-        <v>798</v>
+        <v>1034</v>
       </c>
       <c r="S27" t="n">
-        <v>-467.0914921712886</v>
+        <v>-231.0914921712886</v>
       </c>
       <c r="T27" s="137" t="n">
         <v>478.2608695652174</v>
@@ -5551,26 +5551,26 @@
         <v>10043.47826086957</v>
       </c>
       <c r="V27" s="137" t="n">
-        <v>6422.6</v>
+        <v>8364.200000000001</v>
       </c>
       <c r="W27" s="137" t="n">
-        <v>-3620.878260869566</v>
+        <v>-1679.278260869565</v>
       </c>
       <c r="X27" s="138" t="n">
-        <v>-0.3605203463203463</v>
+        <v>-0.1672008658008658</v>
       </c>
       <c r="Y27" s="137" t="n">
-        <v>8.048370927318297</v>
+        <v>8.089168278529982</v>
       </c>
       <c r="Z27" s="137" t="n">
-        <v>-0.0856831267357574</v>
+        <v>-0.0448857755240723</v>
       </c>
       <c r="AB27" s="139" t="inlineStr"/>
       <c r="AC27" s="139" t="inlineStr"/>
       <c r="AD27" s="139" t="inlineStr"/>
       <c r="AE27" t="inlineStr">
         <is>
-          <t>success;crm:stale</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -5624,10 +5624,10 @@
         <v>2980.193649723336</v>
       </c>
       <c r="R28" t="n">
-        <v>2093</v>
+        <v>2859</v>
       </c>
       <c r="S28" t="n">
-        <v>-887.1936497233364</v>
+        <v>-121.1936497233364</v>
       </c>
       <c r="T28" s="137" t="n">
         <v>2155.680224403927</v>
@@ -5636,26 +5636,26 @@
         <v>58688.63955119214</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>55304.026217</v>
+        <v>57245.626217</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>-3384.613334192145</v>
+        <v>-1443.013334192146</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>-0.0576706728947066</v>
+        <v>-0.0245876092072888</v>
       </c>
       <c r="Y28" s="137" t="n">
-        <v>26.42332834065934</v>
+        <v>20.0229542556838</v>
       </c>
       <c r="Z28" s="137" t="n">
-        <v>6.647605418613999</v>
+        <v>0.2472313336384637</v>
       </c>
       <c r="AB28" s="139" t="inlineStr"/>
       <c r="AC28" s="139" t="inlineStr"/>
       <c r="AD28" s="139" t="inlineStr"/>
       <c r="AE28" t="inlineStr">
         <is>
-          <t>partial;crm:stale</t>
+          <t>partial</t>
         </is>
       </c>
     </row>
@@ -5811,7 +5811,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46233.291875</v>
+        <v>46233.50799768518</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-07-31
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 29/07/2026  |  Ultimo aggiornamento: 30/07/2026 12:56</t>
+          <t>Periodo: 01/07/2026 - 30/07/2026  |  Ultimo aggiornamento: 31/07/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1065,16 +1065,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>8887.096774193547</v>
+        <v>9193.548387096776</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>8291.347024999999</v>
+        <v>8398.713701000001</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>-595.7497491935483</v>
+        <v>-794.834686096774</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>-0.06703536197822139</v>
+        <v>-0.0864557026982456</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1173,16 +1173,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>1403.225806451613</v>
+        <v>1451.612903225807</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>1400.46155</v>
+        <v>1421.847963</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-2.764256451612937</v>
+        <v>-29.76494022580664</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0019699298850574</v>
+        <v>-0.0205047366000001</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1281,16 +1281,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>9354.83870967742</v>
+        <v>9677.419354838708</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>7318.88</v>
+        <v>7437.29</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-2035.958709677418</v>
+        <v>-2240.129354838708</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.2176369655172413</v>
+        <v>-0.2314800333333332</v>
       </c>
       <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
@@ -1328,34 +1328,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>436.5591397849462</v>
+        <v>451.6129032258065</v>
       </c>
       <c r="N10" s="125" t="n">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>14.44086021505376</v>
+        <v>1.387096774193537</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>19645.16129032258</v>
+        <v>20322.58064516129</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>17010.688575</v>
+        <v>17257.851664</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>-2634.472715322579</v>
+        <v>-3064.728981161286</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>-0.1341028804187191</v>
+        <v>-0.1508041244698411</v>
       </c>
       <c r="U10" s="123" t="n">
-        <v>37.71771302660754</v>
+        <v>38.09680279028698</v>
       </c>
       <c r="V10" s="123" t="n">
-        <v>-7.282286973392459</v>
+        <v>-6.903197209713021</v>
       </c>
       <c r="W10" s="126" t="n"/>
     </row>
@@ -1407,34 +1407,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>110.0569259962049</v>
+        <v>113.8519924098672</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>138</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>27.94307400379508</v>
+        <v>24.14800759013283</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>3741.935483870968</v>
+        <v>3870.967741935484</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>4178.169465</v>
+        <v>4284.185833</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>436.2339811290321</v>
+        <v>413.2180910645157</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.1165797708189654</v>
+        <v>0.1067480068583332</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>30.27659032608696</v>
+        <v>31.04482487681159</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>-3.723409673913043</v>
+        <v>-2.955175123188408</v>
       </c>
       <c r="W11" s="120" t="inlineStr">
         <is>
@@ -1490,34 +1490,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M12" s="127" t="n">
-        <v>218.6845412651865</v>
+        <v>226.2253875157101</v>
       </c>
       <c r="N12" s="119" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>20.31545873481357</v>
+        <v>14.77461248428992</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>8419.354838709678</v>
+        <v>8709.677419354839</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>8373.760593000001</v>
+        <v>8586.704412000001</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-45.59424570967712</v>
+        <v>-122.973007354838</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.0054154084942528</v>
+        <v>-0.0141191230666665</v>
       </c>
       <c r="U12" s="128" t="n">
-        <v>35.03665520083683</v>
+        <v>35.62947888796681</v>
       </c>
       <c r="V12" s="128" t="n">
-        <v>-3.463344799163174</v>
+        <v>-2.870521112033188</v>
       </c>
       <c r="W12" s="120" t="inlineStr">
         <is>
@@ -1560,7 +1560,7 @@
       <c r="L13" s="113" t="n"/>
       <c r="M13" s="113" t="n"/>
       <c r="N13" s="119" t="n">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="O13" s="113" t="n"/>
       <c r="P13" s="117" t="n"/>
@@ -1620,34 +1620,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="127" t="n">
-        <v>24.61799660441426</v>
+        <v>25.46689303904923</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>5</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-8.617996604414259</v>
+        <v>-9.466893039049232</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>935.483870967742</v>
+        <v>967.741935483871</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>881.2377</v>
+        <v>897.6755330000001</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-54.24617096774193</v>
+        <v>-70.06640248387089</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.0579872862068965</v>
+        <v>-0.07240194923333319</v>
       </c>
       <c r="U14" s="128" t="n">
-        <v>55.07735625</v>
+        <v>56.10472081250001</v>
       </c>
       <c r="V14" s="128" t="n">
-        <v>17.07735625</v>
+        <v>18.10472081250001</v>
       </c>
       <c r="W14" s="120" t="inlineStr">
         <is>
@@ -1750,34 +1750,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M16" s="127" t="n">
-        <v>3.741935483870968</v>
+        <v>3.870967741935484</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>4</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>1.258064516129032</v>
+        <v>1.129032258064516</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>935.483870967742</v>
+        <v>967.741935483871</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>921.802325</v>
+        <v>929.402325</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>-13.68154596774195</v>
+        <v>-38.33961048387096</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>-0.0146251008620689</v>
+        <v>-0.0396175974999999</v>
       </c>
       <c r="U16" s="128" t="n">
-        <v>184.360465</v>
+        <v>185.880465</v>
       </c>
       <c r="V16" s="128" t="n">
-        <v>-65.639535</v>
+        <v>-64.11953499999998</v>
       </c>
       <c r="W16" s="120" t="inlineStr">
         <is>
@@ -1880,34 +1880,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>730.8467741935484</v>
+        <v>756.0483870967743</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>600</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-130.8467741935484</v>
+        <v>-156.0483870967743</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>9354.83870967742</v>
+        <v>9677.419354838708</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>11396.45</v>
+        <v>11565.81</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>2041.611290322582</v>
+        <v>1888.390645161291</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>0.2182412068965519</v>
+        <v>0.1951337000000001</v>
       </c>
       <c r="U18" s="117" t="n">
-        <v>18.99408333333334</v>
+        <v>19.27635</v>
       </c>
       <c r="V18" s="117" t="n">
-        <v>6.194083333333335</v>
+        <v>6.47635</v>
       </c>
       <c r="W18" s="120" t="inlineStr">
         <is>
@@ -1963,34 +1963,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>11.69354838709677</v>
+        <v>12.09677419354839</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>46</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>34.30645161290322</v>
+        <v>33.90322580645162</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>467.741935483871</v>
+        <v>483.8709677419355</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>436.05</v>
+        <v>439.76</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-31.69193548387096</v>
+        <v>-44.1109677419355</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.0677551724137931</v>
+        <v>-0.0911626666666667</v>
       </c>
       <c r="U19" s="117" t="n">
-        <v>9.479347826086956</v>
+        <v>9.56</v>
       </c>
       <c r="V19" s="117" t="n">
-        <v>-30.52065217391304</v>
+        <v>-30.44</v>
       </c>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
@@ -2042,34 +2042,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>10.39426523297491</v>
+        <v>10.75268817204301</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>24</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>13.60573476702509</v>
+        <v>13.24731182795699</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>935.483870967742</v>
+        <v>967.741935483871</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>747.84</v>
+        <v>751.63</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-187.6438709677419</v>
+        <v>-216.111935483871</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.2005848275862068</v>
+        <v>-0.2233156666666667</v>
       </c>
       <c r="U20" s="117" t="n">
-        <v>31.16</v>
+        <v>31.31791666666667</v>
       </c>
       <c r="V20" s="117" t="n">
-        <v>-58.84</v>
+        <v>-58.68208333333334</v>
       </c>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
@@ -2121,34 +2121,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>3.897849462365592</v>
+        <v>4.03225806451613</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>4</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>0.102150537634408</v>
+        <v>-0.0322580645161298</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>467.741935483871</v>
+        <v>483.8709677419355</v>
       </c>
       <c r="R21" s="117" t="n">
-        <v>393.12</v>
+        <v>396.99</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-74.62193548387097</v>
+        <v>-86.88096774193548</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.1595365517241379</v>
+        <v>-0.179554</v>
       </c>
       <c r="U21" s="117" t="n">
-        <v>98.28</v>
+        <v>99.2475</v>
       </c>
       <c r="V21" s="117" t="n">
-        <v>-21.72</v>
+        <v>-20.7525</v>
       </c>
       <c r="W21" s="120" t="inlineStr"/>
     </row>
@@ -2200,34 +2200,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>35.08064516129032</v>
+        <v>36.29032258064516</v>
       </c>
       <c r="N22" s="119" t="n">
         <v>32</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-3.08064516129032</v>
+        <v>-4.29032258064516</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>1403.225806451613</v>
+        <v>1451.612903225807</v>
       </c>
       <c r="R22" s="117" t="n">
-        <v>1436.892291</v>
+        <v>1471.882129</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>33.66648454838696</v>
+        <v>20.2692257741935</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>0.0239922073793102</v>
+        <v>0.0139632444222221</v>
       </c>
       <c r="U22" s="117" t="n">
-        <v>44.90288409375</v>
+        <v>45.99631653125</v>
       </c>
       <c r="V22" s="117" t="n">
-        <v>4.902884093749996</v>
+        <v>5.996316531250002</v>
       </c>
       <c r="W22" s="120" t="inlineStr"/>
     </row>
@@ -2279,34 +2279,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>93.54838709677421</v>
+        <v>96.77419354838707</v>
       </c>
       <c r="N23" s="119" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>75.45161290322581</v>
+        <v>73.22580645161291</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>1403.225806451613</v>
+        <v>1451.612903225807</v>
       </c>
       <c r="R23" s="117" t="n">
-        <v>1995.797174</v>
+        <v>2098.751996</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>592.5713675483871</v>
+        <v>647.1390927741934</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.4222922389425287</v>
+        <v>0.4458069305777776</v>
       </c>
       <c r="U23" s="117" t="n">
-        <v>11.80945073372781</v>
+        <v>12.34559997647059</v>
       </c>
       <c r="V23" s="117" t="n">
-        <v>-3.190549266272189</v>
+        <v>-2.654400023529412</v>
       </c>
       <c r="W23" s="120" t="inlineStr">
         <is>
@@ -2362,34 +2362,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>35.98014888337469</v>
+        <v>37.22084367245657</v>
       </c>
       <c r="N24" s="119" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>49.01985111662531</v>
+        <v>49.77915632754343</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>935.483870967742</v>
+        <v>967.741935483871</v>
       </c>
       <c r="R24" s="117" t="n">
-        <v>1308.97</v>
+        <v>1327.37</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>373.4861290322581</v>
+        <v>359.6280645161289</v>
       </c>
       <c r="T24" s="118" t="n">
-        <v>0.3992437931034482</v>
+        <v>0.3716156666666665</v>
       </c>
       <c r="U24" s="117" t="n">
-        <v>15.39964705882353</v>
+        <v>15.25712643678161</v>
       </c>
       <c r="V24" s="117" t="n">
-        <v>-10.60035294117647</v>
+        <v>-10.74287356321839</v>
       </c>
       <c r="W24" s="120" t="inlineStr"/>
     </row>
@@ -2430,18 +2430,18 @@
       <c r="L25" s="119" t="n"/>
       <c r="M25" s="119" t="n"/>
       <c r="N25" s="119" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O25" s="119" t="n"/>
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>732.37</v>
+        <v>762.0599999999999</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
       <c r="U25" s="117" t="n">
-        <v>45.773125</v>
+        <v>44.82705882352941</v>
       </c>
       <c r="V25" s="117" t="n"/>
       <c r="W25" s="120" t="inlineStr"/>
@@ -2478,34 +2478,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>1278.543017767101</v>
+        <v>1322.630708034932</v>
       </c>
       <c r="N26" s="125" t="n">
-        <v>1374</v>
+        <v>1380</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>95.45698223289855</v>
+        <v>57.36929196506753</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>29000</v>
+        <v>30000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>32802.459548</v>
+        <v>33512.222228</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>3802.459547999999</v>
+        <v>3512.222227999999</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>0.1311192947586206</v>
+        <v>0.1170740742666666</v>
       </c>
       <c r="U26" s="123" t="n">
-        <v>23.87369690538573</v>
+        <v>24.2842190057971</v>
       </c>
       <c r="V26" s="123" t="n">
-        <v>1.191628647215779</v>
+        <v>1.602150747627146</v>
       </c>
       <c r="W26" s="126" t="n"/>
     </row>
@@ -2553,28 +2553,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>615.4499151103566</v>
+        <v>636.6723259762309</v>
       </c>
       <c r="N27" s="119" t="n">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-143.4499151103566</v>
+        <v>-162.6723259762309</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>4565.217391304348</v>
+        <v>4782.608695652174</v>
       </c>
       <c r="R27" s="117" t="n">
-        <v>3587.2</v>
+        <v>3602.4</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-978.0173913043482</v>
+        <v>-1180.208695652174</v>
       </c>
       <c r="T27" s="118" t="n">
-        <v>-0.214232380952381</v>
+        <v>-0.2467709090909091</v>
       </c>
       <c r="U27" s="117" t="n">
         <v>7.6</v>
@@ -2628,28 +2628,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>415.7706093189964</v>
+        <v>430.1075268817205</v>
       </c>
       <c r="N28" s="119" t="n">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-134.7706093189964</v>
+        <v>-146.1075268817204</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>3652.173913043479</v>
+        <v>3826.086956521739</v>
       </c>
       <c r="R28" s="117" t="n">
-        <v>2529</v>
+        <v>2556</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-1123.173913043478</v>
+        <v>-1270.086956521739</v>
       </c>
       <c r="T28" s="118" t="n">
-        <v>-0.3075357142857143</v>
+        <v>-0.3319545454545454</v>
       </c>
       <c r="U28" s="117" t="n">
         <v>9</v>
@@ -2703,28 +2703,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>233.8709677419355</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="N29" s="119" t="n">
         <v>281</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>47.12903225806451</v>
+        <v>39.06451612903226</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>1826.086956521739</v>
+        <v>1913.043478260869</v>
       </c>
       <c r="R29" s="117" t="n">
         <v>2248</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>421.9130434782608</v>
+        <v>334.9565217391305</v>
       </c>
       <c r="T29" s="118" t="n">
-        <v>0.2310476190476189</v>
+        <v>0.1750909090909091</v>
       </c>
       <c r="U29" s="117" t="n">
         <v>8</v>
@@ -2766,34 +2766,34 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>1265.091492171289</v>
+        <v>1308.715336728919</v>
       </c>
       <c r="N30" s="125" t="n">
-        <v>1034</v>
+        <v>1039</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-231.0914921712886</v>
+        <v>-269.7153367289191</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>10043.47826086957</v>
+        <v>10521.73913043478</v>
       </c>
       <c r="R30" s="123" t="n">
-        <v>8364.200000000001</v>
+        <v>8406.4</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>-1679.278260869565</v>
+        <v>-2115.339130434782</v>
       </c>
       <c r="T30" s="124" t="n">
-        <v>-0.1672008658008658</v>
+        <v>-0.2010446280991735</v>
       </c>
       <c r="U30" s="123" t="n">
-        <v>8.089168278529982</v>
+        <v>8.090856592877767</v>
       </c>
       <c r="V30" s="123" t="n">
-        <v>-0.0448857755240723</v>
+        <v>-0.0431974611762875</v>
       </c>
       <c r="W30" s="126" t="n"/>
     </row>
@@ -2829,34 +2829,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="133" t="n">
-        <v>2980.193649723336</v>
+        <v>3082.958947989658</v>
       </c>
       <c r="N31" s="133" t="n">
-        <v>2859</v>
+        <v>2872</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>-121.1936497233364</v>
+        <v>-210.9589479896581</v>
       </c>
       <c r="P31" s="131" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="Q31" s="131" t="n">
-        <v>58688.63955119214</v>
+        <v>60844.31977559607</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>58177.348123</v>
+        <v>59176.473892</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>-511.2914281921403</v>
+        <v>-1667.84588359607</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>-0.008711931850902001</v>
+        <v>-0.0274116941359088</v>
       </c>
       <c r="U31" s="131" t="n">
-        <v>20.34884509373907</v>
+        <v>20.60462182869081</v>
       </c>
       <c r="V31" s="131" t="n">
-        <v>0.5731221716937327</v>
+        <v>0.8288989066454704</v>
       </c>
       <c r="W31" s="134" t="n"/>
     </row>
@@ -3137,13 +3137,13 @@
         </is>
       </c>
       <c r="B2" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C2" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D2" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3180,16 +3180,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="137" t="n">
-        <v>8887.096774193547</v>
+        <v>9193.548387096776</v>
       </c>
       <c r="V2" s="137" t="n">
-        <v>8291.347024999999</v>
+        <v>8398.713701000001</v>
       </c>
       <c r="W2" s="137" t="n">
-        <v>-595.7497491935483</v>
+        <v>-794.834686096774</v>
       </c>
       <c r="X2" s="138" t="n">
-        <v>-0.06703536197822139</v>
+        <v>-0.0864557026982456</v>
       </c>
       <c r="Y2" s="137" t="n"/>
       <c r="Z2" s="137" t="n"/>
@@ -3223,13 +3223,13 @@
         </is>
       </c>
       <c r="B3" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C3" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D3" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3290,13 +3290,13 @@
         </is>
       </c>
       <c r="B4" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C4" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D4" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3333,16 +3333,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="137" t="n">
-        <v>1403.225806451613</v>
+        <v>1451.612903225807</v>
       </c>
       <c r="V4" s="137" t="n">
-        <v>1400.46155</v>
+        <v>1421.847963</v>
       </c>
       <c r="W4" s="137" t="n">
-        <v>-2.764256451612937</v>
+        <v>-29.76494022580664</v>
       </c>
       <c r="X4" s="138" t="n">
-        <v>-0.0019699298850574</v>
+        <v>-0.0205047366000001</v>
       </c>
       <c r="Y4" s="137" t="n"/>
       <c r="Z4" s="137" t="n"/>
@@ -3376,13 +3376,13 @@
         </is>
       </c>
       <c r="B5" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C5" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D5" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3443,13 +3443,13 @@
         </is>
       </c>
       <c r="B6" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C6" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D6" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3486,16 +3486,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="137" t="n">
-        <v>9354.83870967742</v>
+        <v>9677.419354838708</v>
       </c>
       <c r="V6" s="137" t="n">
-        <v>7318.88</v>
+        <v>7437.29</v>
       </c>
       <c r="W6" s="137" t="n">
-        <v>-2035.958709677418</v>
+        <v>-2240.129354838708</v>
       </c>
       <c r="X6" s="138" t="n">
-        <v>-0.2176369655172413</v>
+        <v>-0.2314800333333332</v>
       </c>
       <c r="Y6" s="137" t="n"/>
       <c r="Z6" s="137" t="n"/>
@@ -3529,13 +3529,13 @@
         </is>
       </c>
       <c r="B7" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C7" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D7" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -3582,28 +3582,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>615.4499151103566</v>
+        <v>636.6723259762309</v>
       </c>
       <c r="R7" t="n">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="S7" t="n">
-        <v>-143.4499151103566</v>
+        <v>-162.6723259762309</v>
       </c>
       <c r="T7" s="137" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="U7" s="137" t="n">
-        <v>4565.217391304348</v>
+        <v>4782.608695652174</v>
       </c>
       <c r="V7" s="137" t="n">
-        <v>3587.2</v>
+        <v>3602.4</v>
       </c>
       <c r="W7" s="137" t="n">
-        <v>-978.0173913043482</v>
+        <v>-1180.208695652174</v>
       </c>
       <c r="X7" s="138" t="n">
-        <v>-0.214232380952381</v>
+        <v>-0.2467709090909091</v>
       </c>
       <c r="Y7" s="137" t="n">
         <v>7.6</v>
@@ -3632,13 +3632,13 @@
         </is>
       </c>
       <c r="B8" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C8" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D8" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E8" t="n">
         <v>26</v>
@@ -3685,28 +3685,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>415.7706093189964</v>
+        <v>430.1075268817205</v>
       </c>
       <c r="R8" t="n">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="S8" t="n">
-        <v>-134.7706093189964</v>
+        <v>-146.1075268817204</v>
       </c>
       <c r="T8" s="137" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="U8" s="137" t="n">
-        <v>3652.173913043479</v>
+        <v>3826.086956521739</v>
       </c>
       <c r="V8" s="137" t="n">
-        <v>2529</v>
+        <v>2556</v>
       </c>
       <c r="W8" s="137" t="n">
-        <v>-1123.173913043478</v>
+        <v>-1270.086956521739</v>
       </c>
       <c r="X8" s="138" t="n">
-        <v>-0.3075357142857143</v>
+        <v>-0.3319545454545454</v>
       </c>
       <c r="Y8" s="137" t="n">
         <v>9</v>
@@ -3735,13 +3735,13 @@
         </is>
       </c>
       <c r="B9" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C9" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D9" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3788,28 +3788,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>233.8709677419355</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="R9" t="n">
         <v>281</v>
       </c>
       <c r="S9" t="n">
-        <v>47.12903225806451</v>
+        <v>39.06451612903226</v>
       </c>
       <c r="T9" s="137" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="U9" s="137" t="n">
-        <v>1826.086956521739</v>
+        <v>1913.043478260869</v>
       </c>
       <c r="V9" s="137" t="n">
         <v>2248</v>
       </c>
       <c r="W9" s="137" t="n">
-        <v>421.9130434782608</v>
+        <v>334.9565217391305</v>
       </c>
       <c r="X9" s="138" t="n">
-        <v>0.2310476190476189</v>
+        <v>0.1750909090909091</v>
       </c>
       <c r="Y9" s="137" t="n">
         <v>8</v>
@@ -3838,13 +3838,13 @@
         </is>
       </c>
       <c r="B10" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C10" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D10" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3891,34 +3891,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>110.0569259962049</v>
+        <v>113.8519924098672</v>
       </c>
       <c r="R10" t="n">
         <v>138</v>
       </c>
       <c r="S10" t="n">
-        <v>27.94307400379508</v>
+        <v>24.14800759013283</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U10" s="137" t="n">
-        <v>3741.935483870968</v>
+        <v>3870.967741935484</v>
       </c>
       <c r="V10" s="137" t="n">
-        <v>4178.169465</v>
+        <v>4284.185833</v>
       </c>
       <c r="W10" s="137" t="n">
-        <v>436.2339811290321</v>
+        <v>413.2180910645157</v>
       </c>
       <c r="X10" s="138" t="n">
-        <v>0.1165797708189654</v>
+        <v>0.1067480068583332</v>
       </c>
       <c r="Y10" s="137" t="n">
-        <v>30.27659032608696</v>
+        <v>31.04482487681159</v>
       </c>
       <c r="Z10" s="137" t="n">
-        <v>-3.723409673913043</v>
+        <v>-2.955175123188408</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -3950,13 +3950,13 @@
         </is>
       </c>
       <c r="B11" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C11" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D11" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -4003,34 +4003,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q11" t="n">
-        <v>218.6845412651865</v>
+        <v>226.2253875157101</v>
       </c>
       <c r="R11" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="S11" t="n">
-        <v>20.31545873481357</v>
+        <v>14.77461248428992</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U11" s="137" t="n">
-        <v>8419.354838709678</v>
+        <v>8709.677419354839</v>
       </c>
       <c r="V11" s="137" t="n">
-        <v>8373.760593000001</v>
+        <v>8586.704412000001</v>
       </c>
       <c r="W11" s="137" t="n">
-        <v>-45.59424570967712</v>
+        <v>-122.973007354838</v>
       </c>
       <c r="X11" s="138" t="n">
-        <v>-0.0054154084942528</v>
+        <v>-0.0141191230666665</v>
       </c>
       <c r="Y11" s="137" t="n">
-        <v>35.03665520083683</v>
+        <v>35.62947888796681</v>
       </c>
       <c r="Z11" s="137" t="n">
-        <v>-3.463344799163174</v>
+        <v>-2.870521112033188</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -4062,13 +4062,13 @@
         </is>
       </c>
       <c r="B12" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C12" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D12" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -4098,7 +4098,7 @@
       <c r="L12" s="137" t="n"/>
       <c r="N12" s="137" t="n"/>
       <c r="R12" t="n">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="T12" s="137" t="n"/>
       <c r="U12" s="137" t="n"/>
@@ -4132,13 +4132,13 @@
         </is>
       </c>
       <c r="B13" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C13" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D13" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4185,34 +4185,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>24.61799660441426</v>
+        <v>25.46689303904923</v>
       </c>
       <c r="R13" t="n">
         <v>5</v>
       </c>
       <c r="S13" t="n">
-        <v>-8.617996604414259</v>
+        <v>-9.466893039049232</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="137" t="n">
-        <v>935.483870967742</v>
+        <v>967.741935483871</v>
       </c>
       <c r="V13" s="137" t="n">
-        <v>881.2377</v>
+        <v>897.6755330000001</v>
       </c>
       <c r="W13" s="137" t="n">
-        <v>-54.24617096774193</v>
+        <v>-70.06640248387089</v>
       </c>
       <c r="X13" s="138" t="n">
-        <v>-0.0579872862068965</v>
+        <v>-0.07240194923333319</v>
       </c>
       <c r="Y13" s="137" t="n">
-        <v>55.07735625</v>
+        <v>56.10472081250001</v>
       </c>
       <c r="Z13" s="137" t="n">
-        <v>17.07735625</v>
+        <v>18.10472081250001</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -4244,13 +4244,13 @@
         </is>
       </c>
       <c r="B14" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C14" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D14" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
@@ -4314,13 +4314,13 @@
         </is>
       </c>
       <c r="B15" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C15" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D15" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -4367,34 +4367,34 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q15" t="n">
-        <v>3.741935483870968</v>
+        <v>3.870967741935484</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
       </c>
       <c r="S15" t="n">
-        <v>1.258064516129032</v>
+        <v>1.129032258064516</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U15" s="137" t="n">
-        <v>935.483870967742</v>
+        <v>967.741935483871</v>
       </c>
       <c r="V15" s="137" t="n">
-        <v>921.802325</v>
+        <v>929.402325</v>
       </c>
       <c r="W15" s="137" t="n">
-        <v>-13.68154596774195</v>
+        <v>-38.33961048387096</v>
       </c>
       <c r="X15" s="138" t="n">
-        <v>-0.0146251008620689</v>
+        <v>-0.0396175974999999</v>
       </c>
       <c r="Y15" s="137" t="n">
-        <v>184.360465</v>
+        <v>185.880465</v>
       </c>
       <c r="Z15" s="137" t="n">
-        <v>-65.639535</v>
+        <v>-64.11953499999998</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -4426,13 +4426,13 @@
         </is>
       </c>
       <c r="B16" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C16" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D16" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4496,13 +4496,13 @@
         </is>
       </c>
       <c r="B17" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C17" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D17" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E17" t="n">
         <v>17</v>
@@ -4549,34 +4549,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>730.8467741935484</v>
+        <v>756.0483870967743</v>
       </c>
       <c r="R17" t="n">
         <v>600</v>
       </c>
       <c r="S17" t="n">
-        <v>-130.8467741935484</v>
+        <v>-156.0483870967743</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U17" s="137" t="n">
-        <v>9354.83870967742</v>
+        <v>9677.419354838708</v>
       </c>
       <c r="V17" s="137" t="n">
-        <v>11396.45</v>
+        <v>11565.81</v>
       </c>
       <c r="W17" s="137" t="n">
-        <v>2041.611290322582</v>
+        <v>1888.390645161291</v>
       </c>
       <c r="X17" s="138" t="n">
-        <v>0.2182412068965519</v>
+        <v>0.1951337000000001</v>
       </c>
       <c r="Y17" s="137" t="n">
-        <v>18.99408333333334</v>
+        <v>19.27635</v>
       </c>
       <c r="Z17" s="137" t="n">
-        <v>6.194083333333335</v>
+        <v>6.47635</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -4608,13 +4608,13 @@
         </is>
       </c>
       <c r="B18" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C18" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D18" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4661,34 +4661,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.69354838709677</v>
+        <v>12.09677419354839</v>
       </c>
       <c r="R18" t="n">
         <v>46</v>
       </c>
       <c r="S18" t="n">
-        <v>34.30645161290322</v>
+        <v>33.90322580645162</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="137" t="n">
-        <v>467.741935483871</v>
+        <v>483.8709677419355</v>
       </c>
       <c r="V18" s="137" t="n">
-        <v>436.05</v>
+        <v>439.76</v>
       </c>
       <c r="W18" s="137" t="n">
-        <v>-31.69193548387096</v>
+        <v>-44.1109677419355</v>
       </c>
       <c r="X18" s="138" t="n">
-        <v>-0.0677551724137931</v>
+        <v>-0.0911626666666667</v>
       </c>
       <c r="Y18" s="137" t="n">
-        <v>9.479347826086956</v>
+        <v>9.56</v>
       </c>
       <c r="Z18" s="137" t="n">
-        <v>-30.52065217391304</v>
+        <v>-30.44</v>
       </c>
       <c r="AB18" s="139" t="inlineStr"/>
       <c r="AC18" s="139" t="inlineStr">
@@ -4715,13 +4715,13 @@
         </is>
       </c>
       <c r="B19" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C19" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D19" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4768,34 +4768,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>10.39426523297491</v>
+        <v>10.75268817204301</v>
       </c>
       <c r="R19" t="n">
         <v>24</v>
       </c>
       <c r="S19" t="n">
-        <v>13.60573476702509</v>
+        <v>13.24731182795699</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="137" t="n">
-        <v>935.483870967742</v>
+        <v>967.741935483871</v>
       </c>
       <c r="V19" s="137" t="n">
-        <v>747.84</v>
+        <v>751.63</v>
       </c>
       <c r="W19" s="137" t="n">
-        <v>-187.6438709677419</v>
+        <v>-216.111935483871</v>
       </c>
       <c r="X19" s="138" t="n">
-        <v>-0.2005848275862068</v>
+        <v>-0.2233156666666667</v>
       </c>
       <c r="Y19" s="137" t="n">
-        <v>31.16</v>
+        <v>31.31791666666667</v>
       </c>
       <c r="Z19" s="137" t="n">
-        <v>-58.84</v>
+        <v>-58.68208333333334</v>
       </c>
       <c r="AB19" s="139" t="inlineStr"/>
       <c r="AC19" s="139" t="inlineStr">
@@ -4822,13 +4822,13 @@
         </is>
       </c>
       <c r="B20" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C20" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D20" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
@@ -4875,34 +4875,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>3.897849462365592</v>
+        <v>4.03225806451613</v>
       </c>
       <c r="R20" t="n">
         <v>4</v>
       </c>
       <c r="S20" t="n">
-        <v>0.102150537634408</v>
+        <v>-0.0322580645161298</v>
       </c>
       <c r="T20" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U20" s="137" t="n">
-        <v>467.741935483871</v>
+        <v>483.8709677419355</v>
       </c>
       <c r="V20" s="137" t="n">
-        <v>393.12</v>
+        <v>396.99</v>
       </c>
       <c r="W20" s="137" t="n">
-        <v>-74.62193548387097</v>
+        <v>-86.88096774193548</v>
       </c>
       <c r="X20" s="138" t="n">
-        <v>-0.1595365517241379</v>
+        <v>-0.179554</v>
       </c>
       <c r="Y20" s="137" t="n">
-        <v>98.28</v>
+        <v>99.2475</v>
       </c>
       <c r="Z20" s="137" t="n">
-        <v>-21.72</v>
+        <v>-20.7525</v>
       </c>
       <c r="AB20" s="139" t="inlineStr"/>
       <c r="AC20" s="139" t="inlineStr">
@@ -4929,13 +4929,13 @@
         </is>
       </c>
       <c r="B21" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C21" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D21" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4982,34 +4982,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>35.08064516129032</v>
+        <v>36.29032258064516</v>
       </c>
       <c r="R21" t="n">
         <v>32</v>
       </c>
       <c r="S21" t="n">
-        <v>-3.08064516129032</v>
+        <v>-4.29032258064516</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="137" t="n">
-        <v>1403.225806451613</v>
+        <v>1451.612903225807</v>
       </c>
       <c r="V21" s="137" t="n">
-        <v>1436.892291</v>
+        <v>1471.882129</v>
       </c>
       <c r="W21" s="137" t="n">
-        <v>33.66648454838696</v>
+        <v>20.2692257741935</v>
       </c>
       <c r="X21" s="138" t="n">
-        <v>0.0239922073793102</v>
+        <v>0.0139632444222221</v>
       </c>
       <c r="Y21" s="137" t="n">
-        <v>44.90288409375</v>
+        <v>45.99631653125</v>
       </c>
       <c r="Z21" s="137" t="n">
-        <v>4.902884093749996</v>
+        <v>5.996316531250002</v>
       </c>
       <c r="AB21" s="139" t="inlineStr">
         <is>
@@ -5036,13 +5036,13 @@
         </is>
       </c>
       <c r="B22" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C22" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D22" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -5089,34 +5089,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>93.54838709677421</v>
+        <v>96.77419354838707</v>
       </c>
       <c r="R22" t="n">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="S22" t="n">
-        <v>75.45161290322581</v>
+        <v>73.22580645161291</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="137" t="n">
-        <v>1403.225806451613</v>
+        <v>1451.612903225807</v>
       </c>
       <c r="V22" s="137" t="n">
-        <v>1995.797174</v>
+        <v>2098.751996</v>
       </c>
       <c r="W22" s="137" t="n">
-        <v>592.5713675483871</v>
+        <v>647.1390927741934</v>
       </c>
       <c r="X22" s="138" t="n">
-        <v>0.4222922389425287</v>
+        <v>0.4458069305777776</v>
       </c>
       <c r="Y22" s="137" t="n">
-        <v>11.80945073372781</v>
+        <v>12.34559997647059</v>
       </c>
       <c r="Z22" s="137" t="n">
-        <v>-3.190549266272189</v>
+        <v>-2.654400023529412</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -5148,13 +5148,13 @@
         </is>
       </c>
       <c r="B23" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C23" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D23" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5201,34 +5201,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>35.98014888337469</v>
+        <v>37.22084367245657</v>
       </c>
       <c r="R23" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="S23" t="n">
-        <v>49.01985111662531</v>
+        <v>49.77915632754343</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="137" t="n">
-        <v>935.483870967742</v>
+        <v>967.741935483871</v>
       </c>
       <c r="V23" s="137" t="n">
-        <v>1308.97</v>
+        <v>1327.37</v>
       </c>
       <c r="W23" s="137" t="n">
-        <v>373.4861290322581</v>
+        <v>359.6280645161289</v>
       </c>
       <c r="X23" s="138" t="n">
-        <v>0.3992437931034482</v>
+        <v>0.3716156666666665</v>
       </c>
       <c r="Y23" s="137" t="n">
-        <v>15.39964705882353</v>
+        <v>15.25712643678161</v>
       </c>
       <c r="Z23" s="137" t="n">
-        <v>-10.60035294117647</v>
+        <v>-10.74287356321839</v>
       </c>
       <c r="AB23" s="139" t="inlineStr"/>
       <c r="AC23" s="139" t="inlineStr">
@@ -5255,13 +5255,13 @@
         </is>
       </c>
       <c r="B24" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C24" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D24" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5293,17 +5293,17 @@
       <c r="L24" s="137" t="n"/>
       <c r="N24" s="137" t="n"/>
       <c r="R24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="T24" s="137" t="n"/>
       <c r="U24" s="137" t="n"/>
       <c r="V24" s="137" t="n">
-        <v>732.37</v>
+        <v>762.0599999999999</v>
       </c>
       <c r="W24" s="137" t="n"/>
       <c r="X24" s="138" t="n"/>
       <c r="Y24" s="137" t="n">
-        <v>45.773125</v>
+        <v>44.82705882352941</v>
       </c>
       <c r="Z24" s="137" t="n"/>
       <c r="AB24" s="139" t="inlineStr"/>
@@ -5331,13 +5331,13 @@
         </is>
       </c>
       <c r="B25" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C25" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D25" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5366,34 +5366,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>436.5591397849462</v>
+        <v>451.6129032258065</v>
       </c>
       <c r="R25" t="n">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="S25" t="n">
-        <v>14.44086021505376</v>
+        <v>1.387096774193537</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="137" t="n">
-        <v>19645.16129032258</v>
+        <v>20322.58064516129</v>
       </c>
       <c r="V25" s="137" t="n">
-        <v>17010.688575</v>
+        <v>17257.851664</v>
       </c>
       <c r="W25" s="137" t="n">
-        <v>-2634.472715322579</v>
+        <v>-3064.728981161286</v>
       </c>
       <c r="X25" s="138" t="n">
-        <v>-0.1341028804187191</v>
+        <v>-0.1508041244698411</v>
       </c>
       <c r="Y25" s="137" t="n">
-        <v>37.71771302660754</v>
+        <v>38.09680279028698</v>
       </c>
       <c r="Z25" s="137" t="n">
-        <v>-7.282286973392459</v>
+        <v>-6.903197209713021</v>
       </c>
       <c r="AB25" s="139" t="inlineStr"/>
       <c r="AC25" s="139" t="inlineStr"/>
@@ -5411,13 +5411,13 @@
         </is>
       </c>
       <c r="B26" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C26" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D26" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5451,34 +5451,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>1278.543017767101</v>
+        <v>1322.630708034932</v>
       </c>
       <c r="R26" t="n">
-        <v>1374</v>
+        <v>1380</v>
       </c>
       <c r="S26" t="n">
-        <v>95.45698223289855</v>
+        <v>57.36929196506753</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="137" t="n">
-        <v>29000</v>
+        <v>30000</v>
       </c>
       <c r="V26" s="137" t="n">
-        <v>32802.459548</v>
+        <v>33512.222228</v>
       </c>
       <c r="W26" s="137" t="n">
-        <v>3802.459547999999</v>
+        <v>3512.222227999999</v>
       </c>
       <c r="X26" s="138" t="n">
-        <v>0.1311192947586206</v>
+        <v>0.1170740742666666</v>
       </c>
       <c r="Y26" s="137" t="n">
-        <v>23.87369690538573</v>
+        <v>24.2842190057971</v>
       </c>
       <c r="Z26" s="137" t="n">
-        <v>1.191628647215779</v>
+        <v>1.602150747627146</v>
       </c>
       <c r="AB26" s="139" t="inlineStr"/>
       <c r="AC26" s="139" t="inlineStr"/>
@@ -5496,13 +5496,13 @@
         </is>
       </c>
       <c r="B27" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C27" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D27" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5536,34 +5536,34 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>1265.091492171289</v>
+        <v>1308.715336728919</v>
       </c>
       <c r="R27" t="n">
-        <v>1034</v>
+        <v>1039</v>
       </c>
       <c r="S27" t="n">
-        <v>-231.0914921712886</v>
+        <v>-269.7153367289191</v>
       </c>
       <c r="T27" s="137" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="U27" s="137" t="n">
-        <v>10043.47826086957</v>
+        <v>10521.73913043478</v>
       </c>
       <c r="V27" s="137" t="n">
-        <v>8364.200000000001</v>
+        <v>8406.4</v>
       </c>
       <c r="W27" s="137" t="n">
-        <v>-1679.278260869565</v>
+        <v>-2115.339130434782</v>
       </c>
       <c r="X27" s="138" t="n">
-        <v>-0.1672008658008658</v>
+        <v>-0.2010446280991735</v>
       </c>
       <c r="Y27" s="137" t="n">
-        <v>8.089168278529982</v>
+        <v>8.090856592877767</v>
       </c>
       <c r="Z27" s="137" t="n">
-        <v>-0.0448857755240723</v>
+        <v>-0.0431974611762875</v>
       </c>
       <c r="AB27" s="139" t="inlineStr"/>
       <c r="AC27" s="139" t="inlineStr"/>
@@ -5581,13 +5581,13 @@
         </is>
       </c>
       <c r="B28" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="C28" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D28" s="136" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5621,34 +5621,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>2980.193649723336</v>
+        <v>3082.958947989658</v>
       </c>
       <c r="R28" t="n">
-        <v>2859</v>
+        <v>2872</v>
       </c>
       <c r="S28" t="n">
-        <v>-121.1936497233364</v>
+        <v>-210.9589479896581</v>
       </c>
       <c r="T28" s="137" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="U28" s="137" t="n">
-        <v>58688.63955119214</v>
+        <v>60844.31977559607</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>58177.348123</v>
+        <v>59176.473892</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>-511.2914281921403</v>
+        <v>-1667.84588359607</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>-0.008711931850902001</v>
+        <v>-0.0274116941359088</v>
       </c>
       <c r="Y28" s="137" t="n">
-        <v>20.34884509373907</v>
+        <v>20.60462182869081</v>
       </c>
       <c r="Z28" s="137" t="n">
-        <v>0.5731221716937327</v>
+        <v>0.8288989066454704</v>
       </c>
       <c r="AB28" s="139" t="inlineStr"/>
       <c r="AC28" s="139" t="inlineStr"/>
@@ -5751,7 +5751,7 @@
         </is>
       </c>
       <c r="B4" s="140" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5791,7 +5791,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5811,7 +5811,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46233.53930555555</v>
+        <v>46234.29199074074</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-01
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 30/07/2026  |  Ultimo aggiornamento: 31/07/2026 07:00</t>
+          <t>Periodo: 01/07/2026 - 31/07/2026  |  Ultimo aggiornamento: 01/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1065,16 +1065,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>9193.548387096776</v>
+        <v>9500</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>8398.713701000001</v>
+        <v>8612.152716999999</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>-794.834686096774</v>
+        <v>-887.847283000001</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>-0.0864557026982456</v>
+        <v>-0.0934576087368422</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1173,16 +1173,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>1451.612903225807</v>
+        <v>1500</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>1421.847963</v>
+        <v>1454.410187</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-29.76494022580664</v>
+        <v>-45.58981300000005</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0205047366000001</v>
+        <v>-0.0303932086666667</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1281,16 +1281,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>9677.419354838708</v>
+        <v>10000</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>7437.29</v>
+        <v>7603.16</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-2240.129354838708</v>
+        <v>-2396.84</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.2314800333333332</v>
+        <v>-0.239684</v>
       </c>
       <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
@@ -1328,34 +1328,34 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>451.6129032258065</v>
+        <v>466.6666666666667</v>
       </c>
       <c r="N10" s="125" t="n">
         <v>453</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>1.387096774193537</v>
+        <v>-13.66666666666669</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>20322.58064516129</v>
+        <v>21000</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>17257.851664</v>
+        <v>17669.722904</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>-3064.728981161286</v>
+        <v>-3330.277096000002</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>-0.1508041244698411</v>
+        <v>-0.1585846236190477</v>
       </c>
       <c r="U10" s="123" t="n">
-        <v>38.09680279028698</v>
+        <v>39.00601082560706</v>
       </c>
       <c r="V10" s="123" t="n">
-        <v>-6.903197209713021</v>
+        <v>-5.993989174392937</v>
       </c>
       <c r="W10" s="126" t="n"/>
     </row>
@@ -1407,34 +1407,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>113.8519924098672</v>
+        <v>117.6470588235294</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>138</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>24.14800759013283</v>
+        <v>20.3529411764706</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>3870.967741935484</v>
+        <v>4000</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>4284.185833</v>
+        <v>4381.027553</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>413.2180910645157</v>
+        <v>381.0275529999999</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.1067480068583332</v>
+        <v>0.09525688824999989</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>31.04482487681159</v>
+        <v>31.74657647101449</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>-2.955175123188408</v>
+        <v>-2.253423528985508</v>
       </c>
       <c r="W11" s="120" t="inlineStr">
         <is>
@@ -1490,34 +1490,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M12" s="127" t="n">
-        <v>226.2253875157101</v>
+        <v>233.7662337662338</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>63</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>14.77461248428992</v>
+        <v>7.233766233766232</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>8709.677419354839</v>
+        <v>9000</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>8586.704412000001</v>
+        <v>8808.234474999999</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-122.973007354838</v>
+        <v>-191.7655250000007</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.0141191230666665</v>
+        <v>-0.0213072805555556</v>
       </c>
       <c r="U12" s="128" t="n">
-        <v>35.62947888796681</v>
+        <v>36.54869076763485</v>
       </c>
       <c r="V12" s="128" t="n">
-        <v>-2.870521112033188</v>
+        <v>-1.951309232365148</v>
       </c>
       <c r="W12" s="120" t="inlineStr">
         <is>
@@ -1620,34 +1620,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="127" t="n">
-        <v>25.46689303904923</v>
+        <v>26.31578947368421</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>5</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-9.466893039049232</v>
+        <v>-10.31578947368421</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>967.741935483871</v>
+        <v>1000</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>897.6755330000001</v>
+        <v>912.600341</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-70.06640248387089</v>
+        <v>-87.39965899999993</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.07240194923333319</v>
+        <v>-0.08739965899999989</v>
       </c>
       <c r="U14" s="128" t="n">
-        <v>56.10472081250001</v>
+        <v>57.0375213125</v>
       </c>
       <c r="V14" s="128" t="n">
-        <v>18.10472081250001</v>
+        <v>19.0375213125</v>
       </c>
       <c r="W14" s="120" t="inlineStr">
         <is>
@@ -1750,28 +1750,28 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M16" s="127" t="n">
-        <v>3.870967741935484</v>
+        <v>4</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>4</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>1.129032258064516</v>
+        <v>1</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>967.741935483871</v>
+        <v>1000</v>
       </c>
       <c r="R16" s="117" t="n">
         <v>929.402325</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>-38.33961048387096</v>
+        <v>-70.59767499999998</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>-0.0396175974999999</v>
+        <v>-0.0705976749999999</v>
       </c>
       <c r="U16" s="128" t="n">
         <v>185.880465</v>
@@ -1880,34 +1880,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>756.0483870967743</v>
+        <v>781.25</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>600</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-156.0483870967743</v>
+        <v>-181.25</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>9677.419354838708</v>
+        <v>10000</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>11565.81</v>
+        <v>11780.04</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>1888.390645161291</v>
+        <v>1780.040000000001</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>0.1951337000000001</v>
+        <v>0.178004</v>
       </c>
       <c r="U18" s="117" t="n">
-        <v>19.27635</v>
+        <v>19.6334</v>
       </c>
       <c r="V18" s="117" t="n">
-        <v>6.47635</v>
+        <v>6.833400000000001</v>
       </c>
       <c r="W18" s="120" t="inlineStr">
         <is>
@@ -1963,34 +1963,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>12.09677419354839</v>
+        <v>12.5</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>46</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>33.90322580645162</v>
+        <v>33.5</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>483.8709677419355</v>
+        <v>500</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>439.76</v>
+        <v>445.27</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-44.1109677419355</v>
+        <v>-54.73000000000002</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.0911626666666667</v>
+        <v>-0.10946</v>
       </c>
       <c r="U19" s="117" t="n">
-        <v>9.56</v>
+        <v>9.679782608695652</v>
       </c>
       <c r="V19" s="117" t="n">
-        <v>-30.44</v>
+        <v>-30.32021739130435</v>
       </c>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
@@ -2042,34 +2042,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>10.75268817204301</v>
+        <v>11.11111111111111</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>24</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>13.24731182795699</v>
+        <v>12.88888888888889</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>967.741935483871</v>
+        <v>1000</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>751.63</v>
+        <v>756.8</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-216.111935483871</v>
+        <v>-243.2</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.2233156666666667</v>
+        <v>-0.2432</v>
       </c>
       <c r="U20" s="117" t="n">
-        <v>31.31791666666667</v>
+        <v>31.53333333333333</v>
       </c>
       <c r="V20" s="117" t="n">
-        <v>-58.68208333333334</v>
+        <v>-58.46666666666667</v>
       </c>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
@@ -2121,34 +2121,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>4.03225806451613</v>
+        <v>4.166666666666667</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>4</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-0.0322580645161298</v>
+        <v>-0.1666666666666669</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>483.8709677419355</v>
+        <v>500</v>
       </c>
       <c r="R21" s="117" t="n">
-        <v>396.99</v>
+        <v>397.7</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-86.88096774193548</v>
+        <v>-102.3</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.179554</v>
+        <v>-0.2046</v>
       </c>
       <c r="U21" s="117" t="n">
-        <v>99.2475</v>
+        <v>99.425</v>
       </c>
       <c r="V21" s="117" t="n">
-        <v>-20.7525</v>
+        <v>-20.575</v>
       </c>
       <c r="W21" s="120" t="inlineStr"/>
     </row>
@@ -2200,34 +2200,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>36.29032258064516</v>
+        <v>37.5</v>
       </c>
       <c r="N22" s="119" t="n">
         <v>32</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-4.29032258064516</v>
+        <v>-5.5</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>1451.612903225807</v>
+        <v>1500</v>
       </c>
       <c r="R22" s="117" t="n">
-        <v>1471.882129</v>
+        <v>1496.892129</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>20.2692257741935</v>
+        <v>-3.107870999999932</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>0.0139632444222221</v>
+        <v>-0.0020719139999999</v>
       </c>
       <c r="U22" s="117" t="n">
-        <v>45.99631653125</v>
+        <v>46.77787903125</v>
       </c>
       <c r="V22" s="117" t="n">
-        <v>5.996316531250002</v>
+        <v>6.777879031250002</v>
       </c>
       <c r="W22" s="120" t="inlineStr"/>
     </row>
@@ -2279,34 +2279,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>96.77419354838707</v>
+        <v>100</v>
       </c>
       <c r="N23" s="119" t="n">
         <v>170</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>73.22580645161291</v>
+        <v>70</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>1451.612903225807</v>
+        <v>1500</v>
       </c>
       <c r="R23" s="117" t="n">
-        <v>2098.751996</v>
+        <v>2248.803906</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>647.1390927741934</v>
+        <v>748.8039060000001</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.4458069305777776</v>
+        <v>0.499202604</v>
       </c>
       <c r="U23" s="117" t="n">
-        <v>12.34559997647059</v>
+        <v>13.22825827058824</v>
       </c>
       <c r="V23" s="117" t="n">
-        <v>-2.654400023529412</v>
+        <v>-1.771741729411763</v>
       </c>
       <c r="W23" s="120" t="inlineStr">
         <is>
@@ -2362,34 +2362,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>37.22084367245657</v>
+        <v>38.46153846153846</v>
       </c>
       <c r="N24" s="119" t="n">
         <v>87</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>49.77915632754343</v>
+        <v>48.53846153846154</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>967.741935483871</v>
+        <v>1000</v>
       </c>
       <c r="R24" s="117" t="n">
-        <v>1327.37</v>
+        <v>1339.66</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>359.6280645161289</v>
+        <v>339.6600000000001</v>
       </c>
       <c r="T24" s="118" t="n">
-        <v>0.3716156666666665</v>
+        <v>0.3396600000000001</v>
       </c>
       <c r="U24" s="117" t="n">
-        <v>15.25712643678161</v>
+        <v>15.3983908045977</v>
       </c>
       <c r="V24" s="117" t="n">
-        <v>-10.74287356321839</v>
+        <v>-10.6016091954023</v>
       </c>
       <c r="W24" s="120" t="inlineStr"/>
     </row>
@@ -2436,12 +2436,12 @@
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>762.0599999999999</v>
+        <v>785.66</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
       <c r="U25" s="117" t="n">
-        <v>44.82705882352941</v>
+        <v>46.21529411764705</v>
       </c>
       <c r="V25" s="117" t="n"/>
       <c r="W25" s="120" t="inlineStr"/>
@@ -2478,34 +2478,34 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>1322.630708034932</v>
+        <v>1366.718398302763</v>
       </c>
       <c r="N26" s="125" t="n">
         <v>1380</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>57.36929196506753</v>
+        <v>13.28160169723628</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>30000</v>
+        <v>31000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>33512.222228</v>
+        <v>34282.090729</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>3512.222227999999</v>
+        <v>3282.090729000003</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>0.1170740742666666</v>
+        <v>0.105873894483871</v>
       </c>
       <c r="U26" s="123" t="n">
-        <v>24.2842190057971</v>
+        <v>24.84209473115942</v>
       </c>
       <c r="V26" s="123" t="n">
-        <v>1.602150747627146</v>
+        <v>2.160026472989468</v>
       </c>
       <c r="W26" s="126" t="n"/>
     </row>
@@ -2553,28 +2553,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>636.6723259762309</v>
+        <v>657.8947368421053</v>
       </c>
       <c r="N27" s="119" t="n">
         <v>474</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-162.6723259762309</v>
+        <v>-183.8947368421053</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>4782.608695652174</v>
+        <v>5000</v>
       </c>
       <c r="R27" s="117" t="n">
         <v>3602.4</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-1180.208695652174</v>
+        <v>-1397.6</v>
       </c>
       <c r="T27" s="118" t="n">
-        <v>-0.2467709090909091</v>
+        <v>-0.27952</v>
       </c>
       <c r="U27" s="117" t="n">
         <v>7.6</v>
@@ -2628,28 +2628,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>430.1075268817205</v>
+        <v>444.4444444444445</v>
       </c>
       <c r="N28" s="119" t="n">
         <v>284</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-146.1075268817204</v>
+        <v>-160.4444444444445</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>3826.086956521739</v>
+        <v>4000</v>
       </c>
       <c r="R28" s="117" t="n">
         <v>2556</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-1270.086956521739</v>
+        <v>-1444</v>
       </c>
       <c r="T28" s="118" t="n">
-        <v>-0.3319545454545454</v>
+        <v>-0.361</v>
       </c>
       <c r="U28" s="117" t="n">
         <v>9</v>
@@ -2703,28 +2703,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>241.9354838709677</v>
+        <v>250</v>
       </c>
       <c r="N29" s="119" t="n">
         <v>281</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>39.06451612903226</v>
+        <v>31</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>1913.043478260869</v>
+        <v>2000</v>
       </c>
       <c r="R29" s="117" t="n">
         <v>2248</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>334.9565217391305</v>
+        <v>248</v>
       </c>
       <c r="T29" s="118" t="n">
-        <v>0.1750909090909091</v>
+        <v>0.124</v>
       </c>
       <c r="U29" s="117" t="n">
         <v>8</v>
@@ -2766,28 +2766,28 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>1308.715336728919</v>
+        <v>1352.33918128655</v>
       </c>
       <c r="N30" s="125" t="n">
         <v>1039</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-269.7153367289191</v>
+        <v>-313.3391812865498</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>10521.73913043478</v>
+        <v>11000</v>
       </c>
       <c r="R30" s="123" t="n">
         <v>8406.4</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>-2115.339130434782</v>
+        <v>-2593.6</v>
       </c>
       <c r="T30" s="124" t="n">
-        <v>-0.2010446280991735</v>
+        <v>-0.2357818181818182</v>
       </c>
       <c r="U30" s="123" t="n">
         <v>8.090856592877767</v>
@@ -2829,34 +2829,34 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="133" t="n">
-        <v>3082.958947989658</v>
+        <v>3185.72424625598</v>
       </c>
       <c r="N31" s="133" t="n">
         <v>2872</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>-210.9589479896581</v>
+        <v>-313.7242462559802</v>
       </c>
       <c r="P31" s="131" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="Q31" s="131" t="n">
-        <v>60844.31977559607</v>
+        <v>63000</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>59176.473892</v>
+        <v>60358.213633</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>-1667.84588359607</v>
+        <v>-2641.786367000001</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>-0.0274116941359088</v>
+        <v>-0.0419331169365079</v>
       </c>
       <c r="U31" s="131" t="n">
-        <v>20.60462182869081</v>
+        <v>21.01609109784122</v>
       </c>
       <c r="V31" s="131" t="n">
-        <v>0.8288989066454704</v>
+        <v>1.240368175795886</v>
       </c>
       <c r="W31" s="134" t="n"/>
     </row>
@@ -3137,13 +3137,13 @@
         </is>
       </c>
       <c r="B2" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C2" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D2" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3180,16 +3180,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="137" t="n">
-        <v>9193.548387096776</v>
+        <v>9500</v>
       </c>
       <c r="V2" s="137" t="n">
-        <v>8398.713701000001</v>
+        <v>8612.152716999999</v>
       </c>
       <c r="W2" s="137" t="n">
-        <v>-794.834686096774</v>
+        <v>-887.847283000001</v>
       </c>
       <c r="X2" s="138" t="n">
-        <v>-0.0864557026982456</v>
+        <v>-0.0934576087368422</v>
       </c>
       <c r="Y2" s="137" t="n"/>
       <c r="Z2" s="137" t="n"/>
@@ -3207,7 +3207,7 @@
       <c r="AD2" s="139" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_3</t>
+          <t>google:ok;google:includes_excel_row_3;crm:stale</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -3223,13 +3223,13 @@
         </is>
       </c>
       <c r="B3" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C3" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D3" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3274,7 +3274,7 @@
       <c r="AD3" s="139" t="inlineStr"/>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_2</t>
+          <t>google:rolled_up_to_excel_row_2;crm:stale</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -3290,13 +3290,13 @@
         </is>
       </c>
       <c r="B4" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C4" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D4" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3333,16 +3333,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="137" t="n">
-        <v>1451.612903225807</v>
+        <v>1500</v>
       </c>
       <c r="V4" s="137" t="n">
-        <v>1421.847963</v>
+        <v>1454.410187</v>
       </c>
       <c r="W4" s="137" t="n">
-        <v>-29.76494022580664</v>
+        <v>-45.58981300000005</v>
       </c>
       <c r="X4" s="138" t="n">
-        <v>-0.0205047366000001</v>
+        <v>-0.0303932086666667</v>
       </c>
       <c r="Y4" s="137" t="n"/>
       <c r="Z4" s="137" t="n"/>
@@ -3360,7 +3360,7 @@
       <c r="AD4" s="139" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_5</t>
+          <t>google:ok;google:includes_excel_row_5;crm:stale</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -3376,13 +3376,13 @@
         </is>
       </c>
       <c r="B5" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C5" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D5" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3427,7 +3427,7 @@
       <c r="AD5" s="139" t="inlineStr"/>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_4</t>
+          <t>google:rolled_up_to_excel_row_4;crm:stale</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -3443,13 +3443,13 @@
         </is>
       </c>
       <c r="B6" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C6" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D6" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3486,16 +3486,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="137" t="n">
-        <v>9677.419354838708</v>
+        <v>10000</v>
       </c>
       <c r="V6" s="137" t="n">
-        <v>7437.29</v>
+        <v>7603.16</v>
       </c>
       <c r="W6" s="137" t="n">
-        <v>-2240.129354838708</v>
+        <v>-2396.84</v>
       </c>
       <c r="X6" s="138" t="n">
-        <v>-0.2314800333333332</v>
+        <v>-0.239684</v>
       </c>
       <c r="Y6" s="137" t="n"/>
       <c r="Z6" s="137" t="n"/>
@@ -3513,7 +3513,7 @@
       <c r="AD6" s="139" t="inlineStr"/>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -3529,13 +3529,13 @@
         </is>
       </c>
       <c r="B7" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C7" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D7" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -3582,28 +3582,28 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>636.6723259762309</v>
+        <v>657.8947368421053</v>
       </c>
       <c r="R7" t="n">
         <v>474</v>
       </c>
       <c r="S7" t="n">
-        <v>-162.6723259762309</v>
+        <v>-183.8947368421053</v>
       </c>
       <c r="T7" s="137" t="n">
         <v>217.3913043478261</v>
       </c>
       <c r="U7" s="137" t="n">
-        <v>4782.608695652174</v>
+        <v>5000</v>
       </c>
       <c r="V7" s="137" t="n">
         <v>3602.4</v>
       </c>
       <c r="W7" s="137" t="n">
-        <v>-1180.208695652174</v>
+        <v>-1397.6</v>
       </c>
       <c r="X7" s="138" t="n">
-        <v>-0.2467709090909091</v>
+        <v>-0.27952</v>
       </c>
       <c r="Y7" s="137" t="n">
         <v>7.6</v>
@@ -3616,7 +3616,7 @@
       <c r="AD7" s="139" t="inlineStr"/>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -3632,13 +3632,13 @@
         </is>
       </c>
       <c r="B8" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C8" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D8" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E8" t="n">
         <v>26</v>
@@ -3685,28 +3685,28 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>430.1075268817205</v>
+        <v>444.4444444444445</v>
       </c>
       <c r="R8" t="n">
         <v>284</v>
       </c>
       <c r="S8" t="n">
-        <v>-146.1075268817204</v>
+        <v>-160.4444444444445</v>
       </c>
       <c r="T8" s="137" t="n">
         <v>173.9130434782609</v>
       </c>
       <c r="U8" s="137" t="n">
-        <v>3826.086956521739</v>
+        <v>4000</v>
       </c>
       <c r="V8" s="137" t="n">
         <v>2556</v>
       </c>
       <c r="W8" s="137" t="n">
-        <v>-1270.086956521739</v>
+        <v>-1444</v>
       </c>
       <c r="X8" s="138" t="n">
-        <v>-0.3319545454545454</v>
+        <v>-0.361</v>
       </c>
       <c r="Y8" s="137" t="n">
         <v>9</v>
@@ -3719,7 +3719,7 @@
       <c r="AD8" s="139" t="inlineStr"/>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -3735,13 +3735,13 @@
         </is>
       </c>
       <c r="B9" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C9" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D9" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3788,28 +3788,28 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>241.9354838709677</v>
+        <v>250</v>
       </c>
       <c r="R9" t="n">
         <v>281</v>
       </c>
       <c r="S9" t="n">
-        <v>39.06451612903226</v>
+        <v>31</v>
       </c>
       <c r="T9" s="137" t="n">
         <v>86.95652173913044</v>
       </c>
       <c r="U9" s="137" t="n">
-        <v>1913.043478260869</v>
+        <v>2000</v>
       </c>
       <c r="V9" s="137" t="n">
         <v>2248</v>
       </c>
       <c r="W9" s="137" t="n">
-        <v>334.9565217391305</v>
+        <v>248</v>
       </c>
       <c r="X9" s="138" t="n">
-        <v>0.1750909090909091</v>
+        <v>0.124</v>
       </c>
       <c r="Y9" s="137" t="n">
         <v>8</v>
@@ -3822,7 +3822,7 @@
       <c r="AD9" s="139" t="inlineStr"/>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -3838,13 +3838,13 @@
         </is>
       </c>
       <c r="B10" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C10" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D10" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3891,34 +3891,34 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>113.8519924098672</v>
+        <v>117.6470588235294</v>
       </c>
       <c r="R10" t="n">
         <v>138</v>
       </c>
       <c r="S10" t="n">
-        <v>24.14800759013283</v>
+        <v>20.3529411764706</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U10" s="137" t="n">
-        <v>3870.967741935484</v>
+        <v>4000</v>
       </c>
       <c r="V10" s="137" t="n">
-        <v>4284.185833</v>
+        <v>4381.027553</v>
       </c>
       <c r="W10" s="137" t="n">
-        <v>413.2180910645157</v>
+        <v>381.0275529999999</v>
       </c>
       <c r="X10" s="138" t="n">
-        <v>0.1067480068583332</v>
+        <v>0.09525688824999989</v>
       </c>
       <c r="Y10" s="137" t="n">
-        <v>31.04482487681159</v>
+        <v>31.74657647101449</v>
       </c>
       <c r="Z10" s="137" t="n">
-        <v>-2.955175123188408</v>
+        <v>-2.253423528985508</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -3934,7 +3934,7 @@
       <c r="AD10" s="139" t="inlineStr"/>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -3950,13 +3950,13 @@
         </is>
       </c>
       <c r="B11" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C11" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D11" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -4003,34 +4003,34 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q11" t="n">
-        <v>226.2253875157101</v>
+        <v>233.7662337662338</v>
       </c>
       <c r="R11" t="n">
         <v>63</v>
       </c>
       <c r="S11" t="n">
-        <v>14.77461248428992</v>
+        <v>7.233766233766232</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U11" s="137" t="n">
-        <v>8709.677419354839</v>
+        <v>9000</v>
       </c>
       <c r="V11" s="137" t="n">
-        <v>8586.704412000001</v>
+        <v>8808.234474999999</v>
       </c>
       <c r="W11" s="137" t="n">
-        <v>-122.973007354838</v>
+        <v>-191.7655250000007</v>
       </c>
       <c r="X11" s="138" t="n">
-        <v>-0.0141191230666665</v>
+        <v>-0.0213072805555556</v>
       </c>
       <c r="Y11" s="137" t="n">
-        <v>35.62947888796681</v>
+        <v>36.54869076763485</v>
       </c>
       <c r="Z11" s="137" t="n">
-        <v>-2.870521112033188</v>
+        <v>-1.951309232365148</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -4046,7 +4046,7 @@
       <c r="AD11" s="139" t="inlineStr"/>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_10;crm_metrics_combined_with_excel_row_10</t>
+          <t>google:ok;google:includes_excel_row_10;crm_metrics_combined_with_excel_row_10;crm:stale</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -4062,13 +4062,13 @@
         </is>
       </c>
       <c r="B12" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C12" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D12" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -4116,7 +4116,7 @@
       <c r="AD12" s="139" t="inlineStr"/>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_9</t>
+          <t>google:rolled_up_to_excel_row_9;crm:stale</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -4132,13 +4132,13 @@
         </is>
       </c>
       <c r="B13" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C13" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D13" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4185,34 +4185,34 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>25.46689303904923</v>
+        <v>26.31578947368421</v>
       </c>
       <c r="R13" t="n">
         <v>5</v>
       </c>
       <c r="S13" t="n">
-        <v>-9.466893039049232</v>
+        <v>-10.31578947368421</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="137" t="n">
-        <v>967.741935483871</v>
+        <v>1000</v>
       </c>
       <c r="V13" s="137" t="n">
-        <v>897.6755330000001</v>
+        <v>912.600341</v>
       </c>
       <c r="W13" s="137" t="n">
-        <v>-70.06640248387089</v>
+        <v>-87.39965899999993</v>
       </c>
       <c r="X13" s="138" t="n">
-        <v>-0.07240194923333319</v>
+        <v>-0.08739965899999989</v>
       </c>
       <c r="Y13" s="137" t="n">
-        <v>56.10472081250001</v>
+        <v>57.0375213125</v>
       </c>
       <c r="Z13" s="137" t="n">
-        <v>18.10472081250001</v>
+        <v>19.0375213125</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -4228,7 +4228,7 @@
       <c r="AD13" s="139" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_12;crm_metrics_combined_with_excel_row_12</t>
+          <t>google:ok;google:includes_excel_row_12;crm_metrics_combined_with_excel_row_12;crm:stale</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -4244,13 +4244,13 @@
         </is>
       </c>
       <c r="B14" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C14" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D14" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
@@ -4298,7 +4298,7 @@
       <c r="AD14" s="139" t="inlineStr"/>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_11</t>
+          <t>google:rolled_up_to_excel_row_11;crm:stale</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -4314,13 +4314,13 @@
         </is>
       </c>
       <c r="B15" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C15" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D15" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -4367,28 +4367,28 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q15" t="n">
-        <v>3.870967741935484</v>
+        <v>4</v>
       </c>
       <c r="R15" t="n">
         <v>4</v>
       </c>
       <c r="S15" t="n">
-        <v>1.129032258064516</v>
+        <v>1</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U15" s="137" t="n">
-        <v>967.741935483871</v>
+        <v>1000</v>
       </c>
       <c r="V15" s="137" t="n">
         <v>929.402325</v>
       </c>
       <c r="W15" s="137" t="n">
-        <v>-38.33961048387096</v>
+        <v>-70.59767499999998</v>
       </c>
       <c r="X15" s="138" t="n">
-        <v>-0.0396175974999999</v>
+        <v>-0.0705976749999999</v>
       </c>
       <c r="Y15" s="137" t="n">
         <v>185.880465</v>
@@ -4410,7 +4410,7 @@
       <c r="AD15" s="139" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_14;crm_metrics_combined_with_excel_row_14</t>
+          <t>google:ok;google:includes_excel_row_14;crm_metrics_combined_with_excel_row_14;crm:stale</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -4426,13 +4426,13 @@
         </is>
       </c>
       <c r="B16" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C16" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D16" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4480,7 +4480,7 @@
       <c r="AD16" s="139" t="inlineStr"/>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_13</t>
+          <t>google:rolled_up_to_excel_row_13;crm:stale</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -4496,13 +4496,13 @@
         </is>
       </c>
       <c r="B17" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C17" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D17" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E17" t="n">
         <v>17</v>
@@ -4549,34 +4549,34 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>756.0483870967743</v>
+        <v>781.25</v>
       </c>
       <c r="R17" t="n">
         <v>600</v>
       </c>
       <c r="S17" t="n">
-        <v>-156.0483870967743</v>
+        <v>-181.25</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U17" s="137" t="n">
-        <v>9677.419354838708</v>
+        <v>10000</v>
       </c>
       <c r="V17" s="137" t="n">
-        <v>11565.81</v>
+        <v>11780.04</v>
       </c>
       <c r="W17" s="137" t="n">
-        <v>1888.390645161291</v>
+        <v>1780.040000000001</v>
       </c>
       <c r="X17" s="138" t="n">
-        <v>0.1951337000000001</v>
+        <v>0.178004</v>
       </c>
       <c r="Y17" s="137" t="n">
-        <v>19.27635</v>
+        <v>19.6334</v>
       </c>
       <c r="Z17" s="137" t="n">
-        <v>6.47635</v>
+        <v>6.833400000000001</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -4592,7 +4592,7 @@
       <c r="AD17" s="139" t="inlineStr"/>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
@@ -4608,13 +4608,13 @@
         </is>
       </c>
       <c r="B18" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C18" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D18" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4661,34 +4661,34 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>12.09677419354839</v>
+        <v>12.5</v>
       </c>
       <c r="R18" t="n">
         <v>46</v>
       </c>
       <c r="S18" t="n">
-        <v>33.90322580645162</v>
+        <v>33.5</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="137" t="n">
-        <v>483.8709677419355</v>
+        <v>500</v>
       </c>
       <c r="V18" s="137" t="n">
-        <v>439.76</v>
+        <v>445.27</v>
       </c>
       <c r="W18" s="137" t="n">
-        <v>-44.1109677419355</v>
+        <v>-54.73000000000002</v>
       </c>
       <c r="X18" s="138" t="n">
-        <v>-0.0911626666666667</v>
+        <v>-0.10946</v>
       </c>
       <c r="Y18" s="137" t="n">
-        <v>9.56</v>
+        <v>9.679782608695652</v>
       </c>
       <c r="Z18" s="137" t="n">
-        <v>-30.44</v>
+        <v>-30.32021739130435</v>
       </c>
       <c r="AB18" s="139" t="inlineStr"/>
       <c r="AC18" s="139" t="inlineStr">
@@ -4699,7 +4699,7 @@
       <c r="AD18" s="139" t="inlineStr"/>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
@@ -4715,13 +4715,13 @@
         </is>
       </c>
       <c r="B19" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C19" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D19" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4768,34 +4768,34 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>10.75268817204301</v>
+        <v>11.11111111111111</v>
       </c>
       <c r="R19" t="n">
         <v>24</v>
       </c>
       <c r="S19" t="n">
-        <v>13.24731182795699</v>
+        <v>12.88888888888889</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="137" t="n">
-        <v>967.741935483871</v>
+        <v>1000</v>
       </c>
       <c r="V19" s="137" t="n">
-        <v>751.63</v>
+        <v>756.8</v>
       </c>
       <c r="W19" s="137" t="n">
-        <v>-216.111935483871</v>
+        <v>-243.2</v>
       </c>
       <c r="X19" s="138" t="n">
-        <v>-0.2233156666666667</v>
+        <v>-0.2432</v>
       </c>
       <c r="Y19" s="137" t="n">
-        <v>31.31791666666667</v>
+        <v>31.53333333333333</v>
       </c>
       <c r="Z19" s="137" t="n">
-        <v>-58.68208333333334</v>
+        <v>-58.46666666666667</v>
       </c>
       <c r="AB19" s="139" t="inlineStr"/>
       <c r="AC19" s="139" t="inlineStr">
@@ -4806,7 +4806,7 @@
       <c r="AD19" s="139" t="inlineStr"/>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
@@ -4822,13 +4822,13 @@
         </is>
       </c>
       <c r="B20" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C20" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D20" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
@@ -4875,34 +4875,34 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>4.03225806451613</v>
+        <v>4.166666666666667</v>
       </c>
       <c r="R20" t="n">
         <v>4</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.0322580645161298</v>
+        <v>-0.1666666666666669</v>
       </c>
       <c r="T20" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U20" s="137" t="n">
-        <v>483.8709677419355</v>
+        <v>500</v>
       </c>
       <c r="V20" s="137" t="n">
-        <v>396.99</v>
+        <v>397.7</v>
       </c>
       <c r="W20" s="137" t="n">
-        <v>-86.88096774193548</v>
+        <v>-102.3</v>
       </c>
       <c r="X20" s="138" t="n">
-        <v>-0.179554</v>
+        <v>-0.2046</v>
       </c>
       <c r="Y20" s="137" t="n">
-        <v>99.2475</v>
+        <v>99.425</v>
       </c>
       <c r="Z20" s="137" t="n">
-        <v>-20.7525</v>
+        <v>-20.575</v>
       </c>
       <c r="AB20" s="139" t="inlineStr"/>
       <c r="AC20" s="139" t="inlineStr">
@@ -4913,7 +4913,7 @@
       <c r="AD20" s="139" t="inlineStr"/>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr">
@@ -4929,13 +4929,13 @@
         </is>
       </c>
       <c r="B21" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C21" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D21" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4982,34 +4982,34 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>36.29032258064516</v>
+        <v>37.5</v>
       </c>
       <c r="R21" t="n">
         <v>32</v>
       </c>
       <c r="S21" t="n">
-        <v>-4.29032258064516</v>
+        <v>-5.5</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="137" t="n">
-        <v>1451.612903225807</v>
+        <v>1500</v>
       </c>
       <c r="V21" s="137" t="n">
-        <v>1471.882129</v>
+        <v>1496.892129</v>
       </c>
       <c r="W21" s="137" t="n">
-        <v>20.2692257741935</v>
+        <v>-3.107870999999932</v>
       </c>
       <c r="X21" s="138" t="n">
-        <v>0.0139632444222221</v>
+        <v>-0.0020719139999999</v>
       </c>
       <c r="Y21" s="137" t="n">
-        <v>45.99631653125</v>
+        <v>46.77787903125</v>
       </c>
       <c r="Z21" s="137" t="n">
-        <v>5.996316531250002</v>
+        <v>6.777879031250002</v>
       </c>
       <c r="AB21" s="139" t="inlineStr">
         <is>
@@ -5020,7 +5020,7 @@
       <c r="AD21" s="139" t="inlineStr"/>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
@@ -5036,13 +5036,13 @@
         </is>
       </c>
       <c r="B22" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C22" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D22" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -5089,34 +5089,34 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>96.77419354838707</v>
+        <v>100</v>
       </c>
       <c r="R22" t="n">
         <v>170</v>
       </c>
       <c r="S22" t="n">
-        <v>73.22580645161291</v>
+        <v>70</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="137" t="n">
-        <v>1451.612903225807</v>
+        <v>1500</v>
       </c>
       <c r="V22" s="137" t="n">
-        <v>2098.751996</v>
+        <v>2248.803906</v>
       </c>
       <c r="W22" s="137" t="n">
-        <v>647.1390927741934</v>
+        <v>748.8039060000001</v>
       </c>
       <c r="X22" s="138" t="n">
-        <v>0.4458069305777776</v>
+        <v>0.499202604</v>
       </c>
       <c r="Y22" s="137" t="n">
-        <v>12.34559997647059</v>
+        <v>13.22825827058824</v>
       </c>
       <c r="Z22" s="137" t="n">
-        <v>-2.654400023529412</v>
+        <v>-1.771741729411763</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -5132,7 +5132,7 @@
       <c r="AD22" s="139" t="inlineStr"/>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
@@ -5148,13 +5148,13 @@
         </is>
       </c>
       <c r="B23" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C23" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D23" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5201,34 +5201,34 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>37.22084367245657</v>
+        <v>38.46153846153846</v>
       </c>
       <c r="R23" t="n">
         <v>87</v>
       </c>
       <c r="S23" t="n">
-        <v>49.77915632754343</v>
+        <v>48.53846153846154</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="137" t="n">
-        <v>967.741935483871</v>
+        <v>1000</v>
       </c>
       <c r="V23" s="137" t="n">
-        <v>1327.37</v>
+        <v>1339.66</v>
       </c>
       <c r="W23" s="137" t="n">
-        <v>359.6280645161289</v>
+        <v>339.6600000000001</v>
       </c>
       <c r="X23" s="138" t="n">
-        <v>0.3716156666666665</v>
+        <v>0.3396600000000001</v>
       </c>
       <c r="Y23" s="137" t="n">
-        <v>15.25712643678161</v>
+        <v>15.3983908045977</v>
       </c>
       <c r="Z23" s="137" t="n">
-        <v>-10.74287356321839</v>
+        <v>-10.6016091954023</v>
       </c>
       <c r="AB23" s="139" t="inlineStr"/>
       <c r="AC23" s="139" t="inlineStr">
@@ -5239,7 +5239,7 @@
       <c r="AD23" s="139" t="inlineStr"/>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -5255,13 +5255,13 @@
         </is>
       </c>
       <c r="B24" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C24" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D24" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5298,12 +5298,12 @@
       <c r="T24" s="137" t="n"/>
       <c r="U24" s="137" t="n"/>
       <c r="V24" s="137" t="n">
-        <v>762.0599999999999</v>
+        <v>785.66</v>
       </c>
       <c r="W24" s="137" t="n"/>
       <c r="X24" s="138" t="n"/>
       <c r="Y24" s="137" t="n">
-        <v>44.82705882352941</v>
+        <v>46.21529411764705</v>
       </c>
       <c r="Z24" s="137" t="n"/>
       <c r="AB24" s="139" t="inlineStr"/>
@@ -5315,7 +5315,7 @@
       <c r="AD24" s="139" t="inlineStr"/>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
@@ -5331,13 +5331,13 @@
         </is>
       </c>
       <c r="B25" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C25" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D25" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5366,41 +5366,41 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>451.6129032258065</v>
+        <v>466.6666666666667</v>
       </c>
       <c r="R25" t="n">
         <v>453</v>
       </c>
       <c r="S25" t="n">
-        <v>1.387096774193537</v>
+        <v>-13.66666666666669</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="137" t="n">
-        <v>20322.58064516129</v>
+        <v>21000</v>
       </c>
       <c r="V25" s="137" t="n">
-        <v>17257.851664</v>
+        <v>17669.722904</v>
       </c>
       <c r="W25" s="137" t="n">
-        <v>-3064.728981161286</v>
+        <v>-3330.277096000002</v>
       </c>
       <c r="X25" s="138" t="n">
-        <v>-0.1508041244698411</v>
+        <v>-0.1585846236190477</v>
       </c>
       <c r="Y25" s="137" t="n">
-        <v>38.09680279028698</v>
+        <v>39.00601082560706</v>
       </c>
       <c r="Z25" s="137" t="n">
-        <v>-6.903197209713021</v>
+        <v>-5.993989174392937</v>
       </c>
       <c r="AB25" s="139" t="inlineStr"/>
       <c r="AC25" s="139" t="inlineStr"/>
       <c r="AD25" s="139" t="inlineStr"/>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5411,13 +5411,13 @@
         </is>
       </c>
       <c r="B26" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C26" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D26" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5451,41 +5451,41 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>1322.630708034932</v>
+        <v>1366.718398302763</v>
       </c>
       <c r="R26" t="n">
         <v>1380</v>
       </c>
       <c r="S26" t="n">
-        <v>57.36929196506753</v>
+        <v>13.28160169723628</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="137" t="n">
-        <v>30000</v>
+        <v>31000</v>
       </c>
       <c r="V26" s="137" t="n">
-        <v>33512.222228</v>
+        <v>34282.090729</v>
       </c>
       <c r="W26" s="137" t="n">
-        <v>3512.222227999999</v>
+        <v>3282.090729000003</v>
       </c>
       <c r="X26" s="138" t="n">
-        <v>0.1170740742666666</v>
+        <v>0.105873894483871</v>
       </c>
       <c r="Y26" s="137" t="n">
-        <v>24.2842190057971</v>
+        <v>24.84209473115942</v>
       </c>
       <c r="Z26" s="137" t="n">
-        <v>1.602150747627146</v>
+        <v>2.160026472989468</v>
       </c>
       <c r="AB26" s="139" t="inlineStr"/>
       <c r="AC26" s="139" t="inlineStr"/>
       <c r="AD26" s="139" t="inlineStr"/>
       <c r="AE26" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5496,13 +5496,13 @@
         </is>
       </c>
       <c r="B27" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C27" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D27" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5536,28 +5536,28 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>1308.715336728919</v>
+        <v>1352.33918128655</v>
       </c>
       <c r="R27" t="n">
         <v>1039</v>
       </c>
       <c r="S27" t="n">
-        <v>-269.7153367289191</v>
+        <v>-313.3391812865498</v>
       </c>
       <c r="T27" s="137" t="n">
         <v>478.2608695652174</v>
       </c>
       <c r="U27" s="137" t="n">
-        <v>10521.73913043478</v>
+        <v>11000</v>
       </c>
       <c r="V27" s="137" t="n">
         <v>8406.4</v>
       </c>
       <c r="W27" s="137" t="n">
-        <v>-2115.339130434782</v>
+        <v>-2593.6</v>
       </c>
       <c r="X27" s="138" t="n">
-        <v>-0.2010446280991735</v>
+        <v>-0.2357818181818182</v>
       </c>
       <c r="Y27" s="137" t="n">
         <v>8.090856592877767</v>
@@ -5570,7 +5570,7 @@
       <c r="AD27" s="139" t="inlineStr"/>
       <c r="AE27" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>success;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5581,13 +5581,13 @@
         </is>
       </c>
       <c r="B28" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="C28" s="136" t="n">
         <v>46204</v>
       </c>
       <c r="D28" s="136" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5621,41 +5621,41 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>3082.958947989658</v>
+        <v>3185.72424625598</v>
       </c>
       <c r="R28" t="n">
         <v>2872</v>
       </c>
       <c r="S28" t="n">
-        <v>-210.9589479896581</v>
+        <v>-313.7242462559802</v>
       </c>
       <c r="T28" s="137" t="n">
         <v>2155.680224403927</v>
       </c>
       <c r="U28" s="137" t="n">
-        <v>60844.31977559607</v>
+        <v>63000</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>59176.473892</v>
+        <v>60358.213633</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>-1667.84588359607</v>
+        <v>-2641.786367000001</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>-0.0274116941359088</v>
+        <v>-0.0419331169365079</v>
       </c>
       <c r="Y28" s="137" t="n">
-        <v>20.60462182869081</v>
+        <v>21.01609109784122</v>
       </c>
       <c r="Z28" s="137" t="n">
-        <v>0.8288989066454704</v>
+        <v>1.240368175795886</v>
       </c>
       <c r="AB28" s="139" t="inlineStr"/>
       <c r="AC28" s="139" t="inlineStr"/>
       <c r="AD28" s="139" t="inlineStr"/>
       <c r="AE28" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5751,7 +5751,7 @@
         </is>
       </c>
       <c r="B4" s="140" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5791,7 +5791,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5811,7 +5811,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46234.29199074074</v>
+        <v>46235.29208333333</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-02
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/07/2026 - 31/07/2026  |  Ultimo aggiornamento: 01/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 01/08/2026  |  Ultimo aggiornamento: 02/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1065,16 +1065,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>9500</v>
+        <v>306.4516129032258</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>8612.152716999999</v>
+        <v>258.514034</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>-887.847283000001</v>
+        <v>-47.93757890322581</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>-0.0934576087368422</v>
+        <v>-0.1564278890526316</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1173,16 +1173,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>1500</v>
+        <v>48.38709677419355</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>1454.410187</v>
+        <v>32.062678</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-45.58981300000005</v>
+        <v>-16.32441877419355</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0303932086666667</v>
+        <v>-0.3373713213333334</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1281,16 +1281,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>10000</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>7603.16</v>
+        <v>295.15</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-2396.84</v>
+        <v>-27.43064516129033</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.239684</v>
+        <v>-0.085035</v>
       </c>
       <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
@@ -1328,35 +1328,31 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>466.6666666666667</v>
+        <v>15.05376344086022</v>
       </c>
       <c r="N10" s="125" t="n">
-        <v>453</v>
+        <v>0</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>-13.66666666666669</v>
+        <v>-15.05376344086022</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>21000</v>
+        <v>677.4193548387096</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>17669.722904</v>
+        <v>585.7267119999999</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>-3330.277096000002</v>
+        <v>-91.69264283870972</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>-0.1585846236190477</v>
-      </c>
-      <c r="U10" s="123" t="n">
-        <v>39.00601082560706</v>
-      </c>
-      <c r="V10" s="123" t="n">
-        <v>-5.993989174392937</v>
-      </c>
+        <v>-0.1353558060952381</v>
+      </c>
+      <c r="U10" s="123" t="n"/>
+      <c r="V10" s="123" t="n"/>
       <c r="W10" s="126" t="n"/>
     </row>
     <row r="11" ht="66" customHeight="1" s="74">
@@ -1407,35 +1403,31 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>117.6470588235294</v>
+        <v>3.795066413662239</v>
       </c>
       <c r="N11" s="119" t="n">
-        <v>138</v>
+        <v>0</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>20.3529411764706</v>
+        <v>-3.795066413662239</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>4000</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>4381.027553</v>
+        <v>106.105276</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>381.0275529999999</v>
+        <v>-22.92698206451612</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.09525688824999989</v>
-      </c>
-      <c r="U11" s="117" t="n">
-        <v>31.74657647101449</v>
-      </c>
-      <c r="V11" s="117" t="n">
-        <v>-2.253423528985508</v>
-      </c>
+        <v>-0.1776841109999999</v>
+      </c>
+      <c r="U11" s="117" t="n"/>
+      <c r="V11" s="117" t="n"/>
       <c r="W11" s="120" t="inlineStr">
         <is>
           <t>diminuito cpa target - alzato a giugno per dare più dati alla campagna che è stata rilanciata da zero</t>
@@ -1490,35 +1482,31 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M12" s="127" t="n">
-        <v>233.7662337662338</v>
+        <v>7.540846250523669</v>
       </c>
       <c r="N12" s="119" t="n">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>7.233766233766232</v>
+        <v>-7.540846250523669</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>9000</v>
+        <v>290.3225806451613</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>8808.234474999999</v>
+        <v>139.48793</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-191.7655250000007</v>
+        <v>-150.8346506451613</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.0213072805555556</v>
-      </c>
-      <c r="U12" s="128" t="n">
-        <v>36.54869076763485</v>
-      </c>
-      <c r="V12" s="128" t="n">
-        <v>-1.951309232365148</v>
-      </c>
+        <v>-0.5195415744444444</v>
+      </c>
+      <c r="U12" s="128" t="n"/>
+      <c r="V12" s="128" t="n"/>
       <c r="W12" s="120" t="inlineStr">
         <is>
           <t>SWITCH fatto</t>
@@ -1560,7 +1548,7 @@
       <c r="L13" s="113" t="n"/>
       <c r="M13" s="113" t="n"/>
       <c r="N13" s="119" t="n">
-        <v>178</v>
+        <v>0</v>
       </c>
       <c r="O13" s="113" t="n"/>
       <c r="P13" s="117" t="n"/>
@@ -1620,35 +1608,31 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="127" t="n">
-        <v>26.31578947368421</v>
+        <v>0.8488964346349744</v>
       </c>
       <c r="N14" s="119" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-10.31578947368421</v>
+        <v>-0.8488964346349744</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>1000</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>912.600341</v>
+        <v>15.018146</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-87.39965899999993</v>
+        <v>-17.23991851612903</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.08739965899999989</v>
-      </c>
-      <c r="U14" s="128" t="n">
-        <v>57.0375213125</v>
-      </c>
-      <c r="V14" s="128" t="n">
-        <v>19.0375213125</v>
-      </c>
+        <v>-0.534437474</v>
+      </c>
+      <c r="U14" s="128" t="n"/>
+      <c r="V14" s="128" t="n"/>
       <c r="W14" s="120" t="inlineStr">
         <is>
           <t>ATTIVATA nuova campagna - quando esce da apprendimento abbassare cpa target</t>
@@ -1690,7 +1674,7 @@
       <c r="L15" s="113" t="n"/>
       <c r="M15" s="113" t="n"/>
       <c r="N15" s="119" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="O15" s="113" t="n"/>
       <c r="P15" s="117" t="n"/>
@@ -1750,35 +1734,31 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M16" s="127" t="n">
-        <v>4</v>
+        <v>0.1290322580645161</v>
       </c>
       <c r="N16" s="119" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>1</v>
+        <v>-0.1290322580645161</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>1000</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>929.402325</v>
+        <v>0</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>-70.59767499999998</v>
+        <v>-32.25806451612903</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>-0.0705976749999999</v>
-      </c>
-      <c r="U16" s="128" t="n">
-        <v>185.880465</v>
-      </c>
-      <c r="V16" s="128" t="n">
-        <v>-64.11953499999998</v>
-      </c>
+        <v>-1</v>
+      </c>
+      <c r="U16" s="128" t="n"/>
+      <c r="V16" s="128" t="n"/>
       <c r="W16" s="120" t="inlineStr">
         <is>
           <t>ATTIVATA nuova campagna - quando esce da apprendimento abbassare cpa target</t>
@@ -1820,7 +1800,7 @@
       <c r="L17" s="113" t="n"/>
       <c r="M17" s="113" t="n"/>
       <c r="N17" s="119" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O17" s="113" t="n"/>
       <c r="P17" s="117" t="n"/>
@@ -1880,35 +1860,31 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>781.25</v>
+        <v>25.20161290322581</v>
       </c>
       <c r="N18" s="119" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-181.25</v>
+        <v>-25.20161290322581</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>10000</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>11780.04</v>
+        <v>164.86</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>1780.040000000001</v>
+        <v>-157.7206451612903</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>0.178004</v>
-      </c>
-      <c r="U18" s="117" t="n">
-        <v>19.6334</v>
-      </c>
-      <c r="V18" s="117" t="n">
-        <v>6.833400000000001</v>
-      </c>
+        <v>-0.4889339999999999</v>
+      </c>
+      <c r="U18" s="117" t="n"/>
+      <c r="V18" s="117" t="n"/>
       <c r="W18" s="120" t="inlineStr">
         <is>
           <t>diminuito cpa target che era stato alzato per aiutare la campagna ad uscire dalla fase di apprendimento</t>
@@ -1963,35 +1939,31 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>12.5</v>
+        <v>0.4032258064516129</v>
       </c>
       <c r="N19" s="119" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>33.5</v>
+        <v>-0.4032258064516129</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>500</v>
+        <v>16.12903225806452</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>445.27</v>
+        <v>10.1</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-54.73000000000002</v>
+        <v>-6.029032258064516</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.10946</v>
-      </c>
-      <c r="U19" s="117" t="n">
-        <v>9.679782608695652</v>
-      </c>
-      <c r="V19" s="117" t="n">
-        <v>-30.32021739130435</v>
-      </c>
+        <v>-0.3738</v>
+      </c>
+      <c r="U19" s="117" t="n"/>
+      <c r="V19" s="117" t="n"/>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
     <row r="20" ht="36" customHeight="1" s="74">
@@ -2042,35 +2014,31 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>11.11111111111111</v>
+        <v>0.3584229390681003</v>
       </c>
       <c r="N20" s="119" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>12.88888888888889</v>
+        <v>-0.3584229390681003</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>1000</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>756.8</v>
+        <v>11.06</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-243.2</v>
+        <v>-21.19806451612903</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.2432</v>
-      </c>
-      <c r="U20" s="117" t="n">
-        <v>31.53333333333333</v>
-      </c>
-      <c r="V20" s="117" t="n">
-        <v>-58.46666666666667</v>
-      </c>
+        <v>-0.6571399999999999</v>
+      </c>
+      <c r="U20" s="117" t="n"/>
+      <c r="V20" s="117" t="n"/>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
     <row r="21" ht="36" customHeight="1" s="74">
@@ -2121,35 +2089,31 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>4.166666666666667</v>
+        <v>0.1344086021505376</v>
       </c>
       <c r="N21" s="119" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-0.1666666666666669</v>
+        <v>-0.1344086021505376</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>500</v>
+        <v>16.12903225806452</v>
       </c>
       <c r="R21" s="117" t="n">
-        <v>397.7</v>
+        <v>0</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-102.3</v>
+        <v>-16.12903225806452</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.2046</v>
-      </c>
-      <c r="U21" s="117" t="n">
-        <v>99.425</v>
-      </c>
-      <c r="V21" s="117" t="n">
-        <v>-20.575</v>
-      </c>
+        <v>-1</v>
+      </c>
+      <c r="U21" s="117" t="n"/>
+      <c r="V21" s="117" t="n"/>
       <c r="W21" s="120" t="inlineStr"/>
     </row>
     <row r="22" ht="21" customHeight="1" s="74">
@@ -2200,35 +2164,31 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>37.5</v>
+        <v>1.209677419354839</v>
       </c>
       <c r="N22" s="119" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-5.5</v>
+        <v>-1.209677419354839</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>1500</v>
+        <v>48.38709677419355</v>
       </c>
       <c r="R22" s="117" t="n">
-        <v>1496.892129</v>
+        <v>9.625539</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>-3.107870999999932</v>
+        <v>-38.76155777419355</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>-0.0020719139999999</v>
-      </c>
-      <c r="U22" s="117" t="n">
-        <v>46.77787903125</v>
-      </c>
-      <c r="V22" s="117" t="n">
-        <v>6.777879031250002</v>
-      </c>
+        <v>-0.801072194</v>
+      </c>
+      <c r="U22" s="117" t="n"/>
+      <c r="V22" s="117" t="n"/>
       <c r="W22" s="120" t="inlineStr"/>
     </row>
     <row r="23" ht="36" customHeight="1" s="74">
@@ -2279,35 +2239,31 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>100</v>
+        <v>3.225806451612903</v>
       </c>
       <c r="N23" s="119" t="n">
-        <v>170</v>
+        <v>0</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>70</v>
+        <v>-3.225806451612903</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>1500</v>
+        <v>48.38709677419355</v>
       </c>
       <c r="R23" s="117" t="n">
-        <v>2248.803906</v>
+        <v>107.355221</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>748.8039060000001</v>
+        <v>58.96812422580645</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.499202604</v>
-      </c>
-      <c r="U23" s="117" t="n">
-        <v>13.22825827058824</v>
-      </c>
-      <c r="V23" s="117" t="n">
-        <v>-1.771741729411763</v>
-      </c>
+        <v>1.218674567333333</v>
+      </c>
+      <c r="U23" s="117" t="n"/>
+      <c r="V23" s="117" t="n"/>
       <c r="W23" s="120" t="inlineStr">
         <is>
           <t>abbassato leggermente lo spending giornaliero</t>
@@ -2362,35 +2318,31 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>38.46153846153846</v>
+        <v>1.240694789081886</v>
       </c>
       <c r="N24" s="119" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>48.53846153846154</v>
+        <v>-1.240694789081886</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>1000</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="R24" s="117" t="n">
-        <v>1339.66</v>
+        <v>0</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>339.6600000000001</v>
+        <v>-32.25806451612903</v>
       </c>
       <c r="T24" s="118" t="n">
-        <v>0.3396600000000001</v>
-      </c>
-      <c r="U24" s="117" t="n">
-        <v>15.3983908045977</v>
-      </c>
-      <c r="V24" s="117" t="n">
-        <v>-10.6016091954023</v>
-      </c>
+        <v>-1</v>
+      </c>
+      <c r="U24" s="117" t="n"/>
+      <c r="V24" s="117" t="n"/>
       <c r="W24" s="120" t="inlineStr"/>
     </row>
     <row r="25" ht="21" customHeight="1" s="74">
@@ -2430,19 +2382,17 @@
       <c r="L25" s="119" t="n"/>
       <c r="M25" s="119" t="n"/>
       <c r="N25" s="119" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="O25" s="119" t="n"/>
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>785.66</v>
+        <v>0</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
-      <c r="U25" s="117" t="n">
-        <v>46.21529411764705</v>
-      </c>
+      <c r="U25" s="117" t="n"/>
       <c r="V25" s="117" t="n"/>
       <c r="W25" s="120" t="inlineStr"/>
     </row>
@@ -2478,35 +2428,31 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>1366.718398302763</v>
+        <v>44.08769026783109</v>
       </c>
       <c r="N26" s="125" t="n">
-        <v>1380</v>
+        <v>0</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>13.28160169723628</v>
+        <v>-44.08769026783109</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>31000</v>
+        <v>1000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>34282.090729</v>
+        <v>563.612112</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>3282.090729000003</v>
+        <v>-436.387888</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>0.105873894483871</v>
-      </c>
-      <c r="U26" s="123" t="n">
-        <v>24.84209473115942</v>
-      </c>
-      <c r="V26" s="123" t="n">
-        <v>2.160026472989468</v>
-      </c>
+        <v>-0.436387888</v>
+      </c>
+      <c r="U26" s="123" t="n"/>
+      <c r="V26" s="123" t="n"/>
       <c r="W26" s="126" t="n"/>
     </row>
     <row r="27" ht="21" customHeight="1" s="74">
@@ -2553,35 +2499,29 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>657.8947368421053</v>
+        <v>21.22241086587437</v>
       </c>
       <c r="N27" s="119" t="n">
-        <v>474</v>
+        <v>0</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-183.8947368421053</v>
+        <v>-21.22241086587437</v>
       </c>
       <c r="P27" s="117" t="n">
-        <v>217.3913043478261</v>
+        <v>238.0952380952381</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="R27" s="117" t="n">
-        <v>3602.4</v>
+        <v>0</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-1397.6</v>
-      </c>
-      <c r="T27" s="118" t="n">
-        <v>-0.27952</v>
-      </c>
-      <c r="U27" s="117" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="V27" s="117" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="T27" s="118" t="n"/>
+      <c r="U27" s="117" t="n"/>
+      <c r="V27" s="117" t="n"/>
       <c r="W27" s="120" t="inlineStr"/>
     </row>
     <row r="28" ht="21" customHeight="1" s="74">
@@ -2628,35 +2568,29 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>444.4444444444445</v>
+        <v>14.33691756272402</v>
       </c>
       <c r="N28" s="119" t="n">
-        <v>284</v>
+        <v>0</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-160.4444444444445</v>
+        <v>-14.33691756272402</v>
       </c>
       <c r="P28" s="117" t="n">
-        <v>173.9130434782609</v>
+        <v>190.4761904761905</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="R28" s="117" t="n">
-        <v>2556</v>
+        <v>0</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-1444</v>
-      </c>
-      <c r="T28" s="118" t="n">
-        <v>-0.361</v>
-      </c>
-      <c r="U28" s="117" t="n">
-        <v>9</v>
-      </c>
-      <c r="V28" s="117" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="T28" s="118" t="n"/>
+      <c r="U28" s="117" t="n"/>
+      <c r="V28" s="117" t="n"/>
       <c r="W28" s="120" t="inlineStr"/>
     </row>
     <row r="29" ht="21" customHeight="1" s="74">
@@ -2703,35 +2637,29 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>250</v>
+        <v>8.064516129032258</v>
       </c>
       <c r="N29" s="119" t="n">
-        <v>281</v>
+        <v>0</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>31</v>
+        <v>-8.064516129032258</v>
       </c>
       <c r="P29" s="117" t="n">
-        <v>86.95652173913044</v>
+        <v>95.23809523809524</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="R29" s="117" t="n">
-        <v>2248</v>
+        <v>0</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>248</v>
-      </c>
-      <c r="T29" s="118" t="n">
-        <v>0.124</v>
-      </c>
-      <c r="U29" s="117" t="n">
-        <v>8</v>
-      </c>
-      <c r="V29" s="117" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="T29" s="118" t="n"/>
+      <c r="U29" s="117" t="n"/>
+      <c r="V29" s="117" t="n"/>
       <c r="W29" s="120" t="inlineStr"/>
     </row>
     <row r="30" ht="21" customHeight="1" s="74">
@@ -2766,35 +2694,29 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>1352.33918128655</v>
+        <v>43.62384455763064</v>
       </c>
       <c r="N30" s="125" t="n">
-        <v>1039</v>
+        <v>0</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-313.3391812865498</v>
+        <v>-43.62384455763064</v>
       </c>
       <c r="P30" s="123" t="n">
-        <v>478.2608695652174</v>
+        <v>523.8095238095239</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>11000</v>
+        <v>0</v>
       </c>
       <c r="R30" s="123" t="n">
-        <v>8406.4</v>
+        <v>0</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>-2593.6</v>
-      </c>
-      <c r="T30" s="124" t="n">
-        <v>-0.2357818181818182</v>
-      </c>
-      <c r="U30" s="123" t="n">
-        <v>8.090856592877767</v>
-      </c>
-      <c r="V30" s="123" t="n">
-        <v>-0.0431974611762875</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="T30" s="124" t="n"/>
+      <c r="U30" s="123" t="n"/>
+      <c r="V30" s="123" t="n"/>
       <c r="W30" s="126" t="n"/>
     </row>
     <row r="31" ht="21" customHeight="1" s="74">
@@ -2829,35 +2751,31 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="133" t="n">
-        <v>3185.72424625598</v>
+        <v>102.7652982663219</v>
       </c>
       <c r="N31" s="133" t="n">
-        <v>2872</v>
+        <v>0</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>-313.7242462559802</v>
+        <v>-102.7652982663219</v>
       </c>
       <c r="P31" s="131" t="n">
-        <v>2155.680224403927</v>
+        <v>2201.228878648234</v>
       </c>
       <c r="Q31" s="131" t="n">
-        <v>63000</v>
+        <v>1677.41935483871</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>60358.213633</v>
+        <v>1149.338824</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>-2641.786367000001</v>
+        <v>-528.0805308387096</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>-0.0419331169365079</v>
-      </c>
-      <c r="U31" s="131" t="n">
-        <v>21.01609109784122</v>
-      </c>
-      <c r="V31" s="131" t="n">
-        <v>1.240368175795886</v>
-      </c>
+        <v>-0.3148172395384615</v>
+      </c>
+      <c r="U31" s="131" t="n"/>
+      <c r="V31" s="131" t="n"/>
       <c r="W31" s="134" t="n"/>
     </row>
     <row r="32" ht="21" customHeight="1" s="74"/>
@@ -3137,13 +3055,13 @@
         </is>
       </c>
       <c r="B2" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C2" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C2" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D2" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3180,16 +3098,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="137" t="n">
-        <v>9500</v>
+        <v>306.4516129032258</v>
       </c>
       <c r="V2" s="137" t="n">
-        <v>8612.152716999999</v>
+        <v>258.514034</v>
       </c>
       <c r="W2" s="137" t="n">
-        <v>-887.847283000001</v>
+        <v>-47.93757890322581</v>
       </c>
       <c r="X2" s="138" t="n">
-        <v>-0.0934576087368422</v>
+        <v>-0.1564278890526316</v>
       </c>
       <c r="Y2" s="137" t="n"/>
       <c r="Z2" s="137" t="n"/>
@@ -3223,13 +3141,13 @@
         </is>
       </c>
       <c r="B3" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C3" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C3" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D3" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3290,13 +3208,13 @@
         </is>
       </c>
       <c r="B4" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C4" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C4" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D4" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3333,16 +3251,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="137" t="n">
-        <v>1500</v>
+        <v>48.38709677419355</v>
       </c>
       <c r="V4" s="137" t="n">
-        <v>1454.410187</v>
+        <v>32.062678</v>
       </c>
       <c r="W4" s="137" t="n">
-        <v>-45.58981300000005</v>
+        <v>-16.32441877419355</v>
       </c>
       <c r="X4" s="138" t="n">
-        <v>-0.0303932086666667</v>
+        <v>-0.3373713213333334</v>
       </c>
       <c r="Y4" s="137" t="n"/>
       <c r="Z4" s="137" t="n"/>
@@ -3376,13 +3294,13 @@
         </is>
       </c>
       <c r="B5" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C5" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C5" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D5" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3443,13 +3361,13 @@
         </is>
       </c>
       <c r="B6" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C6" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C6" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D6" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3486,16 +3404,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="137" t="n">
-        <v>10000</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="V6" s="137" t="n">
-        <v>7603.16</v>
+        <v>295.15</v>
       </c>
       <c r="W6" s="137" t="n">
-        <v>-2396.84</v>
+        <v>-27.43064516129033</v>
       </c>
       <c r="X6" s="138" t="n">
-        <v>-0.239684</v>
+        <v>-0.085035</v>
       </c>
       <c r="Y6" s="137" t="n"/>
       <c r="Z6" s="137" t="n"/>
@@ -3529,13 +3447,13 @@
         </is>
       </c>
       <c r="B7" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C7" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C7" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D7" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -3582,35 +3500,29 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>657.8947368421053</v>
+        <v>21.22241086587437</v>
       </c>
       <c r="R7" t="n">
-        <v>474</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>-183.8947368421053</v>
+        <v>-21.22241086587437</v>
       </c>
       <c r="T7" s="137" t="n">
-        <v>217.3913043478261</v>
+        <v>238.0952380952381</v>
       </c>
       <c r="U7" s="137" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="V7" s="137" t="n">
-        <v>3602.4</v>
+        <v>0</v>
       </c>
       <c r="W7" s="137" t="n">
-        <v>-1397.6</v>
-      </c>
-      <c r="X7" s="138" t="n">
-        <v>-0.27952</v>
-      </c>
-      <c r="Y7" s="137" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="Z7" s="137" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="X7" s="138" t="n"/>
+      <c r="Y7" s="137" t="n"/>
+      <c r="Z7" s="137" t="n"/>
       <c r="AB7" s="139" t="inlineStr"/>
       <c r="AC7" s="139" t="inlineStr"/>
       <c r="AD7" s="139" t="inlineStr"/>
@@ -3632,13 +3544,13 @@
         </is>
       </c>
       <c r="B8" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C8" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C8" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D8" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E8" t="n">
         <v>26</v>
@@ -3685,35 +3597,29 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>444.4444444444445</v>
+        <v>14.33691756272402</v>
       </c>
       <c r="R8" t="n">
-        <v>284</v>
+        <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>-160.4444444444445</v>
+        <v>-14.33691756272402</v>
       </c>
       <c r="T8" s="137" t="n">
-        <v>173.9130434782609</v>
+        <v>190.4761904761905</v>
       </c>
       <c r="U8" s="137" t="n">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="V8" s="137" t="n">
-        <v>2556</v>
+        <v>0</v>
       </c>
       <c r="W8" s="137" t="n">
-        <v>-1444</v>
-      </c>
-      <c r="X8" s="138" t="n">
-        <v>-0.361</v>
-      </c>
-      <c r="Y8" s="137" t="n">
-        <v>9</v>
-      </c>
-      <c r="Z8" s="137" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="X8" s="138" t="n"/>
+      <c r="Y8" s="137" t="n"/>
+      <c r="Z8" s="137" t="n"/>
       <c r="AB8" s="139" t="inlineStr"/>
       <c r="AC8" s="139" t="inlineStr"/>
       <c r="AD8" s="139" t="inlineStr"/>
@@ -3735,13 +3641,13 @@
         </is>
       </c>
       <c r="B9" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C9" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C9" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D9" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3788,35 +3694,29 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>250</v>
+        <v>8.064516129032258</v>
       </c>
       <c r="R9" t="n">
-        <v>281</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>31</v>
+        <v>-8.064516129032258</v>
       </c>
       <c r="T9" s="137" t="n">
-        <v>86.95652173913044</v>
+        <v>95.23809523809524</v>
       </c>
       <c r="U9" s="137" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="V9" s="137" t="n">
-        <v>2248</v>
+        <v>0</v>
       </c>
       <c r="W9" s="137" t="n">
-        <v>248</v>
-      </c>
-      <c r="X9" s="138" t="n">
-        <v>0.124</v>
-      </c>
-      <c r="Y9" s="137" t="n">
-        <v>8</v>
-      </c>
-      <c r="Z9" s="137" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="X9" s="138" t="n"/>
+      <c r="Y9" s="137" t="n"/>
+      <c r="Z9" s="137" t="n"/>
       <c r="AB9" s="139" t="inlineStr"/>
       <c r="AC9" s="139" t="inlineStr"/>
       <c r="AD9" s="139" t="inlineStr"/>
@@ -3838,13 +3738,13 @@
         </is>
       </c>
       <c r="B10" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C10" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C10" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D10" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3891,35 +3791,31 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>117.6470588235294</v>
+        <v>3.795066413662239</v>
       </c>
       <c r="R10" t="n">
-        <v>138</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>20.3529411764706</v>
+        <v>-3.795066413662239</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U10" s="137" t="n">
-        <v>4000</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="V10" s="137" t="n">
-        <v>4381.027553</v>
+        <v>106.105276</v>
       </c>
       <c r="W10" s="137" t="n">
-        <v>381.0275529999999</v>
+        <v>-22.92698206451612</v>
       </c>
       <c r="X10" s="138" t="n">
-        <v>0.09525688824999989</v>
-      </c>
-      <c r="Y10" s="137" t="n">
-        <v>31.74657647101449</v>
-      </c>
-      <c r="Z10" s="137" t="n">
-        <v>-2.253423528985508</v>
-      </c>
+        <v>-0.1776841109999999</v>
+      </c>
+      <c r="Y10" s="137" t="n"/>
+      <c r="Z10" s="137" t="n"/>
       <c r="AA10" t="inlineStr">
         <is>
           <t>diminuito cpa target - alzato a giugno per dare più dati alla campagna che è stata rilanciata da zero</t>
@@ -3950,13 +3846,13 @@
         </is>
       </c>
       <c r="B11" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C11" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C11" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D11" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -4003,35 +3899,31 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q11" t="n">
-        <v>233.7662337662338</v>
+        <v>7.540846250523669</v>
       </c>
       <c r="R11" t="n">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>7.233766233766232</v>
+        <v>-7.540846250523669</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U11" s="137" t="n">
-        <v>9000</v>
+        <v>290.3225806451613</v>
       </c>
       <c r="V11" s="137" t="n">
-        <v>8808.234474999999</v>
+        <v>139.48793</v>
       </c>
       <c r="W11" s="137" t="n">
-        <v>-191.7655250000007</v>
+        <v>-150.8346506451613</v>
       </c>
       <c r="X11" s="138" t="n">
-        <v>-0.0213072805555556</v>
-      </c>
-      <c r="Y11" s="137" t="n">
-        <v>36.54869076763485</v>
-      </c>
-      <c r="Z11" s="137" t="n">
-        <v>-1.951309232365148</v>
-      </c>
+        <v>-0.5195415744444444</v>
+      </c>
+      <c r="Y11" s="137" t="n"/>
+      <c r="Z11" s="137" t="n"/>
       <c r="AA11" t="inlineStr">
         <is>
           <t>SWITCH fatto</t>
@@ -4062,13 +3954,13 @@
         </is>
       </c>
       <c r="B12" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C12" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C12" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D12" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -4098,7 +3990,7 @@
       <c r="L12" s="137" t="n"/>
       <c r="N12" s="137" t="n"/>
       <c r="R12" t="n">
-        <v>178</v>
+        <v>0</v>
       </c>
       <c r="T12" s="137" t="n"/>
       <c r="U12" s="137" t="n"/>
@@ -4132,13 +4024,13 @@
         </is>
       </c>
       <c r="B13" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C13" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C13" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D13" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4185,35 +4077,31 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>26.31578947368421</v>
+        <v>0.8488964346349744</v>
       </c>
       <c r="R13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>-10.31578947368421</v>
+        <v>-0.8488964346349744</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="137" t="n">
-        <v>1000</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="V13" s="137" t="n">
-        <v>912.600341</v>
+        <v>15.018146</v>
       </c>
       <c r="W13" s="137" t="n">
-        <v>-87.39965899999993</v>
+        <v>-17.23991851612903</v>
       </c>
       <c r="X13" s="138" t="n">
-        <v>-0.08739965899999989</v>
-      </c>
-      <c r="Y13" s="137" t="n">
-        <v>57.0375213125</v>
-      </c>
-      <c r="Z13" s="137" t="n">
-        <v>19.0375213125</v>
-      </c>
+        <v>-0.534437474</v>
+      </c>
+      <c r="Y13" s="137" t="n"/>
+      <c r="Z13" s="137" t="n"/>
       <c r="AA13" t="inlineStr">
         <is>
           <t>ATTIVATA nuova campagna - quando esce da apprendimento abbassare cpa target</t>
@@ -4244,13 +4132,13 @@
         </is>
       </c>
       <c r="B14" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C14" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C14" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D14" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
@@ -4280,7 +4168,7 @@
       <c r="L14" s="137" t="n"/>
       <c r="N14" s="137" t="n"/>
       <c r="R14" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="T14" s="137" t="n"/>
       <c r="U14" s="137" t="n"/>
@@ -4314,13 +4202,13 @@
         </is>
       </c>
       <c r="B15" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C15" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C15" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D15" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -4367,35 +4255,31 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q15" t="n">
-        <v>4</v>
+        <v>0.1290322580645161</v>
       </c>
       <c r="R15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>1</v>
+        <v>-0.1290322580645161</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U15" s="137" t="n">
-        <v>1000</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="V15" s="137" t="n">
-        <v>929.402325</v>
+        <v>0</v>
       </c>
       <c r="W15" s="137" t="n">
-        <v>-70.59767499999998</v>
+        <v>-32.25806451612903</v>
       </c>
       <c r="X15" s="138" t="n">
-        <v>-0.0705976749999999</v>
-      </c>
-      <c r="Y15" s="137" t="n">
-        <v>185.880465</v>
-      </c>
-      <c r="Z15" s="137" t="n">
-        <v>-64.11953499999998</v>
-      </c>
+        <v>-1</v>
+      </c>
+      <c r="Y15" s="137" t="n"/>
+      <c r="Z15" s="137" t="n"/>
       <c r="AA15" t="inlineStr">
         <is>
           <t>ATTIVATA nuova campagna - quando esce da apprendimento abbassare cpa target</t>
@@ -4426,13 +4310,13 @@
         </is>
       </c>
       <c r="B16" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C16" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C16" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D16" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4462,7 +4346,7 @@
       <c r="L16" s="137" t="n"/>
       <c r="N16" s="137" t="n"/>
       <c r="R16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T16" s="137" t="n"/>
       <c r="U16" s="137" t="n"/>
@@ -4496,13 +4380,13 @@
         </is>
       </c>
       <c r="B17" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C17" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C17" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D17" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E17" t="n">
         <v>17</v>
@@ -4549,35 +4433,31 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>781.25</v>
+        <v>25.20161290322581</v>
       </c>
       <c r="R17" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>-181.25</v>
+        <v>-25.20161290322581</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U17" s="137" t="n">
-        <v>10000</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="V17" s="137" t="n">
-        <v>11780.04</v>
+        <v>164.86</v>
       </c>
       <c r="W17" s="137" t="n">
-        <v>1780.040000000001</v>
+        <v>-157.7206451612903</v>
       </c>
       <c r="X17" s="138" t="n">
-        <v>0.178004</v>
-      </c>
-      <c r="Y17" s="137" t="n">
-        <v>19.6334</v>
-      </c>
-      <c r="Z17" s="137" t="n">
-        <v>6.833400000000001</v>
-      </c>
+        <v>-0.4889339999999999</v>
+      </c>
+      <c r="Y17" s="137" t="n"/>
+      <c r="Z17" s="137" t="n"/>
       <c r="AA17" t="inlineStr">
         <is>
           <t>diminuito cpa target che era stato alzato per aiutare la campagna ad uscire dalla fase di apprendimento</t>
@@ -4608,13 +4488,13 @@
         </is>
       </c>
       <c r="B18" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C18" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C18" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D18" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4661,35 +4541,31 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>12.5</v>
+        <v>0.4032258064516129</v>
       </c>
       <c r="R18" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>33.5</v>
+        <v>-0.4032258064516129</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="137" t="n">
-        <v>500</v>
+        <v>16.12903225806452</v>
       </c>
       <c r="V18" s="137" t="n">
-        <v>445.27</v>
+        <v>10.1</v>
       </c>
       <c r="W18" s="137" t="n">
-        <v>-54.73000000000002</v>
+        <v>-6.029032258064516</v>
       </c>
       <c r="X18" s="138" t="n">
-        <v>-0.10946</v>
-      </c>
-      <c r="Y18" s="137" t="n">
-        <v>9.679782608695652</v>
-      </c>
-      <c r="Z18" s="137" t="n">
-        <v>-30.32021739130435</v>
-      </c>
+        <v>-0.3738</v>
+      </c>
+      <c r="Y18" s="137" t="n"/>
+      <c r="Z18" s="137" t="n"/>
       <c r="AB18" s="139" t="inlineStr"/>
       <c r="AC18" s="139" t="inlineStr">
         <is>
@@ -4715,13 +4591,13 @@
         </is>
       </c>
       <c r="B19" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C19" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C19" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D19" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4768,35 +4644,31 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>11.11111111111111</v>
+        <v>0.3584229390681003</v>
       </c>
       <c r="R19" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>12.88888888888889</v>
+        <v>-0.3584229390681003</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="137" t="n">
-        <v>1000</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="V19" s="137" t="n">
-        <v>756.8</v>
+        <v>11.06</v>
       </c>
       <c r="W19" s="137" t="n">
-        <v>-243.2</v>
+        <v>-21.19806451612903</v>
       </c>
       <c r="X19" s="138" t="n">
-        <v>-0.2432</v>
-      </c>
-      <c r="Y19" s="137" t="n">
-        <v>31.53333333333333</v>
-      </c>
-      <c r="Z19" s="137" t="n">
-        <v>-58.46666666666667</v>
-      </c>
+        <v>-0.6571399999999999</v>
+      </c>
+      <c r="Y19" s="137" t="n"/>
+      <c r="Z19" s="137" t="n"/>
       <c r="AB19" s="139" t="inlineStr"/>
       <c r="AC19" s="139" t="inlineStr">
         <is>
@@ -4822,13 +4694,13 @@
         </is>
       </c>
       <c r="B20" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C20" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C20" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D20" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
@@ -4875,35 +4747,31 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>4.166666666666667</v>
+        <v>0.1344086021505376</v>
       </c>
       <c r="R20" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.1666666666666669</v>
+        <v>-0.1344086021505376</v>
       </c>
       <c r="T20" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U20" s="137" t="n">
-        <v>500</v>
+        <v>16.12903225806452</v>
       </c>
       <c r="V20" s="137" t="n">
-        <v>397.7</v>
+        <v>0</v>
       </c>
       <c r="W20" s="137" t="n">
-        <v>-102.3</v>
+        <v>-16.12903225806452</v>
       </c>
       <c r="X20" s="138" t="n">
-        <v>-0.2046</v>
-      </c>
-      <c r="Y20" s="137" t="n">
-        <v>99.425</v>
-      </c>
-      <c r="Z20" s="137" t="n">
-        <v>-20.575</v>
-      </c>
+        <v>-1</v>
+      </c>
+      <c r="Y20" s="137" t="n"/>
+      <c r="Z20" s="137" t="n"/>
       <c r="AB20" s="139" t="inlineStr"/>
       <c r="AC20" s="139" t="inlineStr">
         <is>
@@ -4913,7 +4781,7 @@
       <c r="AD20" s="139" t="inlineStr"/>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:no_delivery;crm:stale</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr">
@@ -4929,13 +4797,13 @@
         </is>
       </c>
       <c r="B21" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C21" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C21" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D21" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4982,35 +4850,31 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>37.5</v>
+        <v>1.209677419354839</v>
       </c>
       <c r="R21" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>-5.5</v>
+        <v>-1.209677419354839</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="137" t="n">
-        <v>1500</v>
+        <v>48.38709677419355</v>
       </c>
       <c r="V21" s="137" t="n">
-        <v>1496.892129</v>
+        <v>9.625539</v>
       </c>
       <c r="W21" s="137" t="n">
-        <v>-3.107870999999932</v>
+        <v>-38.76155777419355</v>
       </c>
       <c r="X21" s="138" t="n">
-        <v>-0.0020719139999999</v>
-      </c>
-      <c r="Y21" s="137" t="n">
-        <v>46.77787903125</v>
-      </c>
-      <c r="Z21" s="137" t="n">
-        <v>6.777879031250002</v>
-      </c>
+        <v>-0.801072194</v>
+      </c>
+      <c r="Y21" s="137" t="n"/>
+      <c r="Z21" s="137" t="n"/>
       <c r="AB21" s="139" t="inlineStr">
         <is>
           <t>22660883424</t>
@@ -5036,13 +4900,13 @@
         </is>
       </c>
       <c r="B22" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C22" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C22" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D22" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -5089,35 +4953,31 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>100</v>
+        <v>3.225806451612903</v>
       </c>
       <c r="R22" t="n">
-        <v>170</v>
+        <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>70</v>
+        <v>-3.225806451612903</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="137" t="n">
-        <v>1500</v>
+        <v>48.38709677419355</v>
       </c>
       <c r="V22" s="137" t="n">
-        <v>2248.803906</v>
+        <v>107.355221</v>
       </c>
       <c r="W22" s="137" t="n">
-        <v>748.8039060000001</v>
+        <v>58.96812422580645</v>
       </c>
       <c r="X22" s="138" t="n">
-        <v>0.499202604</v>
-      </c>
-      <c r="Y22" s="137" t="n">
-        <v>13.22825827058824</v>
-      </c>
-      <c r="Z22" s="137" t="n">
-        <v>-1.771741729411763</v>
-      </c>
+        <v>1.218674567333333</v>
+      </c>
+      <c r="Y22" s="137" t="n"/>
+      <c r="Z22" s="137" t="n"/>
       <c r="AA22" t="inlineStr">
         <is>
           <t>abbassato leggermente lo spending giornaliero</t>
@@ -5148,13 +5008,13 @@
         </is>
       </c>
       <c r="B23" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C23" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C23" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D23" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5201,35 +5061,31 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>38.46153846153846</v>
+        <v>1.240694789081886</v>
       </c>
       <c r="R23" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>48.53846153846154</v>
+        <v>-1.240694789081886</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="137" t="n">
-        <v>1000</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="V23" s="137" t="n">
-        <v>1339.66</v>
+        <v>0</v>
       </c>
       <c r="W23" s="137" t="n">
-        <v>339.6600000000001</v>
+        <v>-32.25806451612903</v>
       </c>
       <c r="X23" s="138" t="n">
-        <v>0.3396600000000001</v>
-      </c>
-      <c r="Y23" s="137" t="n">
-        <v>15.3983908045977</v>
-      </c>
-      <c r="Z23" s="137" t="n">
-        <v>-10.6016091954023</v>
-      </c>
+        <v>-1</v>
+      </c>
+      <c r="Y23" s="137" t="n"/>
+      <c r="Z23" s="137" t="n"/>
       <c r="AB23" s="139" t="inlineStr"/>
       <c r="AC23" s="139" t="inlineStr">
         <is>
@@ -5239,7 +5095,7 @@
       <c r="AD23" s="139" t="inlineStr"/>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:no_delivery;crm:stale</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -5255,13 +5111,13 @@
         </is>
       </c>
       <c r="B24" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C24" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C24" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D24" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5293,18 +5149,16 @@
       <c r="L24" s="137" t="n"/>
       <c r="N24" s="137" t="n"/>
       <c r="R24" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="T24" s="137" t="n"/>
       <c r="U24" s="137" t="n"/>
       <c r="V24" s="137" t="n">
-        <v>785.66</v>
+        <v>0</v>
       </c>
       <c r="W24" s="137" t="n"/>
       <c r="X24" s="138" t="n"/>
-      <c r="Y24" s="137" t="n">
-        <v>46.21529411764705</v>
-      </c>
+      <c r="Y24" s="137" t="n"/>
       <c r="Z24" s="137" t="n"/>
       <c r="AB24" s="139" t="inlineStr"/>
       <c r="AC24" s="139" t="inlineStr">
@@ -5315,7 +5169,7 @@
       <c r="AD24" s="139" t="inlineStr"/>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:no_delivery;crm:stale</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
@@ -5331,13 +5185,13 @@
         </is>
       </c>
       <c r="B25" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C25" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C25" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D25" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5366,35 +5220,31 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>466.6666666666667</v>
+        <v>15.05376344086022</v>
       </c>
       <c r="R25" t="n">
-        <v>453</v>
+        <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>-13.66666666666669</v>
+        <v>-15.05376344086022</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="137" t="n">
-        <v>21000</v>
+        <v>677.4193548387096</v>
       </c>
       <c r="V25" s="137" t="n">
-        <v>17669.722904</v>
+        <v>585.7267119999999</v>
       </c>
       <c r="W25" s="137" t="n">
-        <v>-3330.277096000002</v>
+        <v>-91.69264283870972</v>
       </c>
       <c r="X25" s="138" t="n">
-        <v>-0.1585846236190477</v>
-      </c>
-      <c r="Y25" s="137" t="n">
-        <v>39.00601082560706</v>
-      </c>
-      <c r="Z25" s="137" t="n">
-        <v>-5.993989174392937</v>
-      </c>
+        <v>-0.1353558060952381</v>
+      </c>
+      <c r="Y25" s="137" t="n"/>
+      <c r="Z25" s="137" t="n"/>
       <c r="AB25" s="139" t="inlineStr"/>
       <c r="AC25" s="139" t="inlineStr"/>
       <c r="AD25" s="139" t="inlineStr"/>
@@ -5411,13 +5261,13 @@
         </is>
       </c>
       <c r="B26" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C26" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C26" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D26" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5451,35 +5301,31 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>1366.718398302763</v>
+        <v>44.08769026783109</v>
       </c>
       <c r="R26" t="n">
-        <v>1380</v>
+        <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>13.28160169723628</v>
+        <v>-44.08769026783109</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="137" t="n">
-        <v>31000</v>
+        <v>1000</v>
       </c>
       <c r="V26" s="137" t="n">
-        <v>34282.090729</v>
+        <v>563.612112</v>
       </c>
       <c r="W26" s="137" t="n">
-        <v>3282.090729000003</v>
+        <v>-436.387888</v>
       </c>
       <c r="X26" s="138" t="n">
-        <v>0.105873894483871</v>
-      </c>
-      <c r="Y26" s="137" t="n">
-        <v>24.84209473115942</v>
-      </c>
-      <c r="Z26" s="137" t="n">
-        <v>2.160026472989468</v>
-      </c>
+        <v>-0.436387888</v>
+      </c>
+      <c r="Y26" s="137" t="n"/>
+      <c r="Z26" s="137" t="n"/>
       <c r="AB26" s="139" t="inlineStr"/>
       <c r="AC26" s="139" t="inlineStr"/>
       <c r="AD26" s="139" t="inlineStr"/>
@@ -5496,13 +5342,13 @@
         </is>
       </c>
       <c r="B27" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C27" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C27" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D27" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5536,35 +5382,29 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>1352.33918128655</v>
+        <v>43.62384455763064</v>
       </c>
       <c r="R27" t="n">
-        <v>1039</v>
+        <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>-313.3391812865498</v>
+        <v>-43.62384455763064</v>
       </c>
       <c r="T27" s="137" t="n">
-        <v>478.2608695652174</v>
+        <v>523.8095238095239</v>
       </c>
       <c r="U27" s="137" t="n">
-        <v>11000</v>
+        <v>0</v>
       </c>
       <c r="V27" s="137" t="n">
-        <v>8406.4</v>
+        <v>0</v>
       </c>
       <c r="W27" s="137" t="n">
-        <v>-2593.6</v>
-      </c>
-      <c r="X27" s="138" t="n">
-        <v>-0.2357818181818182</v>
-      </c>
-      <c r="Y27" s="137" t="n">
-        <v>8.090856592877767</v>
-      </c>
-      <c r="Z27" s="137" t="n">
-        <v>-0.0431974611762875</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="X27" s="138" t="n"/>
+      <c r="Y27" s="137" t="n"/>
+      <c r="Z27" s="137" t="n"/>
       <c r="AB27" s="139" t="inlineStr"/>
       <c r="AC27" s="139" t="inlineStr"/>
       <c r="AD27" s="139" t="inlineStr"/>
@@ -5581,13 +5421,13 @@
         </is>
       </c>
       <c r="B28" s="136" t="n">
+        <v>46236</v>
+      </c>
+      <c r="C28" s="136" t="n">
         <v>46235</v>
       </c>
-      <c r="C28" s="136" t="n">
-        <v>46204</v>
-      </c>
       <c r="D28" s="136" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5621,35 +5461,31 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>3185.72424625598</v>
+        <v>102.7652982663219</v>
       </c>
       <c r="R28" t="n">
-        <v>2872</v>
+        <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>-313.7242462559802</v>
+        <v>-102.7652982663219</v>
       </c>
       <c r="T28" s="137" t="n">
-        <v>2155.680224403927</v>
+        <v>2201.228878648234</v>
       </c>
       <c r="U28" s="137" t="n">
-        <v>63000</v>
+        <v>1677.41935483871</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>60358.213633</v>
+        <v>1149.338824</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>-2641.786367000001</v>
+        <v>-528.0805308387096</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>-0.0419331169365079</v>
-      </c>
-      <c r="Y28" s="137" t="n">
-        <v>21.01609109784122</v>
-      </c>
-      <c r="Z28" s="137" t="n">
-        <v>1.240368175795886</v>
-      </c>
+        <v>-0.3148172395384615</v>
+      </c>
+      <c r="Y28" s="137" t="n"/>
+      <c r="Z28" s="137" t="n"/>
       <c r="AB28" s="139" t="inlineStr"/>
       <c r="AC28" s="139" t="inlineStr"/>
       <c r="AD28" s="139" t="inlineStr"/>
@@ -5731,7 +5567,7 @@
         </is>
       </c>
       <c r="B3" s="140" t="n">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="D3" s="33" t="inlineStr">
         <is>
@@ -5751,7 +5587,7 @@
         </is>
       </c>
       <c r="B4" s="140" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5791,7 +5627,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5811,7 +5647,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46235.29208333333</v>
+        <v>46236.29188657407</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-03
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 01/08/2026  |  Ultimo aggiornamento: 02/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 02/08/2026  |  Ultimo aggiornamento: 03/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1065,16 +1065,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>306.4516129032258</v>
+        <v>612.9032258064516</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>258.514034</v>
+        <v>523.218704</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>-47.93757890322581</v>
+        <v>-89.68452180645158</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>-0.1564278890526316</v>
+        <v>-0.1463273776842104</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1173,16 +1173,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>48.38709677419355</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>32.062678</v>
+        <v>63.640853</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-16.32441877419355</v>
+        <v>-33.1333405483871</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.3373713213333334</v>
+        <v>-0.3423778523333334</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1281,16 +1281,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>322.5806451612903</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>295.15</v>
+        <v>565.75</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-27.43064516129033</v>
+        <v>-79.41129032258061</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.085035</v>
+        <v>-0.1230874999999999</v>
       </c>
       <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
@@ -1328,28 +1328,28 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>15.05376344086022</v>
+        <v>30.10752688172043</v>
       </c>
       <c r="N10" s="125" t="n">
         <v>0</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>-15.05376344086022</v>
+        <v>-30.10752688172043</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>677.4193548387096</v>
+        <v>1354.838709677419</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>585.7267119999999</v>
+        <v>1152.609557</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>-91.69264283870972</v>
+        <v>-202.2291526774193</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>-0.1353558060952381</v>
+        <v>-0.149264374595238</v>
       </c>
       <c r="U10" s="123" t="n"/>
       <c r="V10" s="123" t="n"/>
@@ -1403,28 +1403,28 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>3.795066413662239</v>
+        <v>7.590132827324478</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-3.795066413662239</v>
+        <v>-7.590132827324478</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>129.0322580645161</v>
+        <v>258.0645161290323</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>106.105276</v>
+        <v>210.361052</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>-22.92698206451612</v>
+        <v>-47.70346412903226</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>-0.1776841109999999</v>
+        <v>-0.1848509235</v>
       </c>
       <c r="U11" s="117" t="n"/>
       <c r="V11" s="117" t="n"/>
@@ -1482,28 +1482,28 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M12" s="127" t="n">
-        <v>7.540846250523669</v>
+        <v>15.08169250104734</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>-7.540846250523669</v>
+        <v>-15.08169250104734</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>290.3225806451613</v>
+        <v>580.6451612903226</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>139.48793</v>
+        <v>273.700389</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-150.8346506451613</v>
+        <v>-306.9447722903226</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.5195415744444444</v>
+        <v>-0.5286271078333333</v>
       </c>
       <c r="U12" s="128" t="n"/>
       <c r="V12" s="128" t="n"/>
@@ -1608,28 +1608,28 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="127" t="n">
-        <v>0.8488964346349744</v>
+        <v>1.697792869269949</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-0.8488964346349744</v>
+        <v>-1.697792869269949</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>32.25806451612903</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>15.018146</v>
+        <v>33.988146</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-17.23991851612903</v>
+        <v>-30.52798303225806</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.534437474</v>
+        <v>-0.473183737</v>
       </c>
       <c r="U14" s="128" t="n"/>
       <c r="V14" s="128" t="n"/>
@@ -1734,25 +1734,25 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M16" s="127" t="n">
-        <v>0.1290322580645161</v>
+        <v>0.2580645161290322</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>-0.1290322580645161</v>
+        <v>-0.2580645161290322</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>32.25806451612903</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="R16" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>-32.25806451612903</v>
+        <v>-64.51612903225806</v>
       </c>
       <c r="T16" s="118" t="n">
         <v>-1</v>
@@ -1860,28 +1860,28 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>25.20161290322581</v>
+        <v>50.40322580645162</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-25.20161290322581</v>
+        <v>-50.40322580645162</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>322.5806451612903</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>164.86</v>
+        <v>351.12</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>-157.7206451612903</v>
+        <v>-294.0412903225806</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>-0.4889339999999999</v>
+        <v>-0.4557639999999999</v>
       </c>
       <c r="U18" s="117" t="n"/>
       <c r="V18" s="117" t="n"/>
@@ -1939,28 +1939,28 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>0.4032258064516129</v>
+        <v>0.8064516129032258</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-0.4032258064516129</v>
+        <v>-0.8064516129032258</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>16.12903225806452</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>10.1</v>
+        <v>21.7</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-6.029032258064516</v>
+        <v>-10.55806451612903</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.3738</v>
+        <v>-0.3273</v>
       </c>
       <c r="U19" s="117" t="n"/>
       <c r="V19" s="117" t="n"/>
@@ -2014,28 +2014,28 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>0.3584229390681003</v>
+        <v>0.7168458781362007</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-0.3584229390681003</v>
+        <v>-0.7168458781362007</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>32.25806451612903</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>11.06</v>
+        <v>20.8</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-21.19806451612903</v>
+        <v>-43.71612903225807</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.6571399999999999</v>
+        <v>-0.6776000000000001</v>
       </c>
       <c r="U20" s="117" t="n"/>
       <c r="V20" s="117" t="n"/>
@@ -2089,25 +2089,25 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>0.1344086021505376</v>
+        <v>0.2688172043010753</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-0.1344086021505376</v>
+        <v>-0.2688172043010753</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>16.12903225806452</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-16.12903225806452</v>
+        <v>-32.25806451612903</v>
       </c>
       <c r="T21" s="118" t="n">
         <v>-1</v>
@@ -2164,28 +2164,28 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>1.209677419354839</v>
+        <v>2.419354838709677</v>
       </c>
       <c r="N22" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-1.209677419354839</v>
+        <v>-2.419354838709677</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>48.38709677419355</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="R22" s="117" t="n">
         <v>9.625539</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>-38.76155777419355</v>
+        <v>-87.1486545483871</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>-0.801072194</v>
+        <v>-0.9005360969999999</v>
       </c>
       <c r="U22" s="117" t="n"/>
       <c r="V22" s="117" t="n"/>
@@ -2239,28 +2239,28 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>3.225806451612903</v>
+        <v>6.451612903225806</v>
       </c>
       <c r="N23" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>-3.225806451612903</v>
+        <v>-6.451612903225806</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>48.38709677419355</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="R23" s="117" t="n">
-        <v>107.355221</v>
+        <v>189.306264</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>58.96812422580645</v>
+        <v>92.5320704516129</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>1.218674567333333</v>
+        <v>0.956164728</v>
       </c>
       <c r="U23" s="117" t="n"/>
       <c r="V23" s="117" t="n"/>
@@ -2318,25 +2318,25 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>1.240694789081886</v>
+        <v>2.481389578163772</v>
       </c>
       <c r="N24" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>-1.240694789081886</v>
+        <v>-2.481389578163772</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>32.25806451612903</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="R24" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>-32.25806451612903</v>
+        <v>-64.51612903225806</v>
       </c>
       <c r="T24" s="118" t="n">
         <v>-1</v>
@@ -2428,28 +2428,28 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>44.08769026783109</v>
+        <v>88.17538053566217</v>
       </c>
       <c r="N26" s="125" t="n">
         <v>0</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>-44.08769026783109</v>
+        <v>-88.17538053566217</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>563.612112</v>
+        <v>1110.60139</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>-436.387888</v>
+        <v>-889.39861</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>-0.436387888</v>
+        <v>-0.444699305</v>
       </c>
       <c r="U26" s="123" t="n"/>
       <c r="V26" s="123" t="n"/>
@@ -2499,13 +2499,13 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>21.22241086587437</v>
+        <v>42.44482173174873</v>
       </c>
       <c r="N27" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-21.22241086587437</v>
+        <v>-42.44482173174873</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>238.0952380952381</v>
@@ -2568,13 +2568,13 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>14.33691756272402</v>
+        <v>28.67383512544803</v>
       </c>
       <c r="N28" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-14.33691756272402</v>
+        <v>-28.67383512544803</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>190.4761904761905</v>
@@ -2637,13 +2637,13 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>8.064516129032258</v>
+        <v>16.12903225806452</v>
       </c>
       <c r="N29" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>-8.064516129032258</v>
+        <v>-16.12903225806452</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>95.23809523809524</v>
@@ -2694,13 +2694,13 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>43.62384455763064</v>
+        <v>87.24768911526128</v>
       </c>
       <c r="N30" s="125" t="n">
         <v>0</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-43.62384455763064</v>
+        <v>-87.24768911526128</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>523.8095238095239</v>
@@ -2751,28 +2751,28 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="133" t="n">
-        <v>102.7652982663219</v>
+        <v>205.5305965326439</v>
       </c>
       <c r="N31" s="133" t="n">
         <v>0</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>-102.7652982663219</v>
+        <v>-205.5305965326439</v>
       </c>
       <c r="P31" s="131" t="n">
         <v>2201.228878648234</v>
       </c>
       <c r="Q31" s="131" t="n">
-        <v>1677.41935483871</v>
+        <v>3354.838709677419</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>1149.338824</v>
+        <v>2263.210947</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>-528.0805308387096</v>
+        <v>-1091.627762677419</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>-0.3148172395384615</v>
+        <v>-0.3253890446442307</v>
       </c>
       <c r="U31" s="131" t="n"/>
       <c r="V31" s="131" t="n"/>
@@ -3055,13 +3055,13 @@
         </is>
       </c>
       <c r="B2" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C2" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3098,16 +3098,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="137" t="n">
-        <v>306.4516129032258</v>
+        <v>612.9032258064516</v>
       </c>
       <c r="V2" s="137" t="n">
-        <v>258.514034</v>
+        <v>523.218704</v>
       </c>
       <c r="W2" s="137" t="n">
-        <v>-47.93757890322581</v>
+        <v>-89.68452180645158</v>
       </c>
       <c r="X2" s="138" t="n">
-        <v>-0.1564278890526316</v>
+        <v>-0.1463273776842104</v>
       </c>
       <c r="Y2" s="137" t="n"/>
       <c r="Z2" s="137" t="n"/>
@@ -3141,13 +3141,13 @@
         </is>
       </c>
       <c r="B3" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C3" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3208,13 +3208,13 @@
         </is>
       </c>
       <c r="B4" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C4" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3251,16 +3251,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="137" t="n">
-        <v>48.38709677419355</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="V4" s="137" t="n">
-        <v>32.062678</v>
+        <v>63.640853</v>
       </c>
       <c r="W4" s="137" t="n">
-        <v>-16.32441877419355</v>
+        <v>-33.1333405483871</v>
       </c>
       <c r="X4" s="138" t="n">
-        <v>-0.3373713213333334</v>
+        <v>-0.3423778523333334</v>
       </c>
       <c r="Y4" s="137" t="n"/>
       <c r="Z4" s="137" t="n"/>
@@ -3294,13 +3294,13 @@
         </is>
       </c>
       <c r="B5" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C5" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3361,13 +3361,13 @@
         </is>
       </c>
       <c r="B6" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C6" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3404,16 +3404,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="137" t="n">
-        <v>322.5806451612903</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="V6" s="137" t="n">
-        <v>295.15</v>
+        <v>565.75</v>
       </c>
       <c r="W6" s="137" t="n">
-        <v>-27.43064516129033</v>
+        <v>-79.41129032258061</v>
       </c>
       <c r="X6" s="138" t="n">
-        <v>-0.085035</v>
+        <v>-0.1230874999999999</v>
       </c>
       <c r="Y6" s="137" t="n"/>
       <c r="Z6" s="137" t="n"/>
@@ -3447,13 +3447,13 @@
         </is>
       </c>
       <c r="B7" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C7" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -3500,13 +3500,13 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>21.22241086587437</v>
+        <v>42.44482173174873</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>-21.22241086587437</v>
+        <v>-42.44482173174873</v>
       </c>
       <c r="T7" s="137" t="n">
         <v>238.0952380952381</v>
@@ -3544,13 +3544,13 @@
         </is>
       </c>
       <c r="B8" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C8" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E8" t="n">
         <v>26</v>
@@ -3597,13 +3597,13 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>14.33691756272402</v>
+        <v>28.67383512544803</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>-14.33691756272402</v>
+        <v>-28.67383512544803</v>
       </c>
       <c r="T8" s="137" t="n">
         <v>190.4761904761905</v>
@@ -3641,13 +3641,13 @@
         </is>
       </c>
       <c r="B9" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C9" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3694,13 +3694,13 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>8.064516129032258</v>
+        <v>16.12903225806452</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>-8.064516129032258</v>
+        <v>-16.12903225806452</v>
       </c>
       <c r="T9" s="137" t="n">
         <v>95.23809523809524</v>
@@ -3738,13 +3738,13 @@
         </is>
       </c>
       <c r="B10" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C10" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3791,28 +3791,28 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>3.795066413662239</v>
+        <v>7.590132827324478</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>-3.795066413662239</v>
+        <v>-7.590132827324478</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U10" s="137" t="n">
-        <v>129.0322580645161</v>
+        <v>258.0645161290323</v>
       </c>
       <c r="V10" s="137" t="n">
-        <v>106.105276</v>
+        <v>210.361052</v>
       </c>
       <c r="W10" s="137" t="n">
-        <v>-22.92698206451612</v>
+        <v>-47.70346412903226</v>
       </c>
       <c r="X10" s="138" t="n">
-        <v>-0.1776841109999999</v>
+        <v>-0.1848509235</v>
       </c>
       <c r="Y10" s="137" t="n"/>
       <c r="Z10" s="137" t="n"/>
@@ -3846,13 +3846,13 @@
         </is>
       </c>
       <c r="B11" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C11" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3899,28 +3899,28 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q11" t="n">
-        <v>7.540846250523669</v>
+        <v>15.08169250104734</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>-7.540846250523669</v>
+        <v>-15.08169250104734</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U11" s="137" t="n">
-        <v>290.3225806451613</v>
+        <v>580.6451612903226</v>
       </c>
       <c r="V11" s="137" t="n">
-        <v>139.48793</v>
+        <v>273.700389</v>
       </c>
       <c r="W11" s="137" t="n">
-        <v>-150.8346506451613</v>
+        <v>-306.9447722903226</v>
       </c>
       <c r="X11" s="138" t="n">
-        <v>-0.5195415744444444</v>
+        <v>-0.5286271078333333</v>
       </c>
       <c r="Y11" s="137" t="n"/>
       <c r="Z11" s="137" t="n"/>
@@ -3954,13 +3954,13 @@
         </is>
       </c>
       <c r="B12" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C12" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -4024,13 +4024,13 @@
         </is>
       </c>
       <c r="B13" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C13" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4077,28 +4077,28 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.8488964346349744</v>
+        <v>1.697792869269949</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>-0.8488964346349744</v>
+        <v>-1.697792869269949</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="137" t="n">
-        <v>32.25806451612903</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="V13" s="137" t="n">
-        <v>15.018146</v>
+        <v>33.988146</v>
       </c>
       <c r="W13" s="137" t="n">
-        <v>-17.23991851612903</v>
+        <v>-30.52798303225806</v>
       </c>
       <c r="X13" s="138" t="n">
-        <v>-0.534437474</v>
+        <v>-0.473183737</v>
       </c>
       <c r="Y13" s="137" t="n"/>
       <c r="Z13" s="137" t="n"/>
@@ -4132,13 +4132,13 @@
         </is>
       </c>
       <c r="B14" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C14" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
@@ -4202,13 +4202,13 @@
         </is>
       </c>
       <c r="B15" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C15" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -4255,25 +4255,25 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.1290322580645161</v>
+        <v>0.2580645161290322</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.1290322580645161</v>
+        <v>-0.2580645161290322</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U15" s="137" t="n">
-        <v>32.25806451612903</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="V15" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W15" s="137" t="n">
-        <v>-32.25806451612903</v>
+        <v>-64.51612903225806</v>
       </c>
       <c r="X15" s="138" t="n">
         <v>-1</v>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B16" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C16" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4380,13 +4380,13 @@
         </is>
       </c>
       <c r="B17" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C17" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E17" t="n">
         <v>17</v>
@@ -4433,28 +4433,28 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>25.20161290322581</v>
+        <v>50.40322580645162</v>
       </c>
       <c r="R17" t="n">
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>-25.20161290322581</v>
+        <v>-50.40322580645162</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U17" s="137" t="n">
-        <v>322.5806451612903</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="V17" s="137" t="n">
-        <v>164.86</v>
+        <v>351.12</v>
       </c>
       <c r="W17" s="137" t="n">
-        <v>-157.7206451612903</v>
+        <v>-294.0412903225806</v>
       </c>
       <c r="X17" s="138" t="n">
-        <v>-0.4889339999999999</v>
+        <v>-0.4557639999999999</v>
       </c>
       <c r="Y17" s="137" t="n"/>
       <c r="Z17" s="137" t="n"/>
@@ -4488,13 +4488,13 @@
         </is>
       </c>
       <c r="B18" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C18" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4541,28 +4541,28 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.4032258064516129</v>
+        <v>0.8064516129032258</v>
       </c>
       <c r="R18" t="n">
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>-0.4032258064516129</v>
+        <v>-0.8064516129032258</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="137" t="n">
-        <v>16.12903225806452</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="V18" s="137" t="n">
-        <v>10.1</v>
+        <v>21.7</v>
       </c>
       <c r="W18" s="137" t="n">
-        <v>-6.029032258064516</v>
+        <v>-10.55806451612903</v>
       </c>
       <c r="X18" s="138" t="n">
-        <v>-0.3738</v>
+        <v>-0.3273</v>
       </c>
       <c r="Y18" s="137" t="n"/>
       <c r="Z18" s="137" t="n"/>
@@ -4591,13 +4591,13 @@
         </is>
       </c>
       <c r="B19" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C19" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4644,28 +4644,28 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.3584229390681003</v>
+        <v>0.7168458781362007</v>
       </c>
       <c r="R19" t="n">
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>-0.3584229390681003</v>
+        <v>-0.7168458781362007</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="137" t="n">
-        <v>32.25806451612903</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="V19" s="137" t="n">
-        <v>11.06</v>
+        <v>20.8</v>
       </c>
       <c r="W19" s="137" t="n">
-        <v>-21.19806451612903</v>
+        <v>-43.71612903225807</v>
       </c>
       <c r="X19" s="138" t="n">
-        <v>-0.6571399999999999</v>
+        <v>-0.6776000000000001</v>
       </c>
       <c r="Y19" s="137" t="n"/>
       <c r="Z19" s="137" t="n"/>
@@ -4694,13 +4694,13 @@
         </is>
       </c>
       <c r="B20" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C20" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
@@ -4747,25 +4747,25 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.1344086021505376</v>
+        <v>0.2688172043010753</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.1344086021505376</v>
+        <v>-0.2688172043010753</v>
       </c>
       <c r="T20" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U20" s="137" t="n">
-        <v>16.12903225806452</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="V20" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W20" s="137" t="n">
-        <v>-16.12903225806452</v>
+        <v>-32.25806451612903</v>
       </c>
       <c r="X20" s="138" t="n">
         <v>-1</v>
@@ -4797,13 +4797,13 @@
         </is>
       </c>
       <c r="B21" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C21" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D21" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4850,28 +4850,28 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>1.209677419354839</v>
+        <v>2.419354838709677</v>
       </c>
       <c r="R21" t="n">
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>-1.209677419354839</v>
+        <v>-2.419354838709677</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="137" t="n">
-        <v>48.38709677419355</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="V21" s="137" t="n">
         <v>9.625539</v>
       </c>
       <c r="W21" s="137" t="n">
-        <v>-38.76155777419355</v>
+        <v>-87.1486545483871</v>
       </c>
       <c r="X21" s="138" t="n">
-        <v>-0.801072194</v>
+        <v>-0.9005360969999999</v>
       </c>
       <c r="Y21" s="137" t="n"/>
       <c r="Z21" s="137" t="n"/>
@@ -4900,13 +4900,13 @@
         </is>
       </c>
       <c r="B22" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C22" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D22" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -4953,28 +4953,28 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>3.225806451612903</v>
+        <v>6.451612903225806</v>
       </c>
       <c r="R22" t="n">
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>-3.225806451612903</v>
+        <v>-6.451612903225806</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="137" t="n">
-        <v>48.38709677419355</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="V22" s="137" t="n">
-        <v>107.355221</v>
+        <v>189.306264</v>
       </c>
       <c r="W22" s="137" t="n">
-        <v>58.96812422580645</v>
+        <v>92.5320704516129</v>
       </c>
       <c r="X22" s="138" t="n">
-        <v>1.218674567333333</v>
+        <v>0.956164728</v>
       </c>
       <c r="Y22" s="137" t="n"/>
       <c r="Z22" s="137" t="n"/>
@@ -5008,13 +5008,13 @@
         </is>
       </c>
       <c r="B23" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C23" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D23" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5061,25 +5061,25 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>1.240694789081886</v>
+        <v>2.481389578163772</v>
       </c>
       <c r="R23" t="n">
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>-1.240694789081886</v>
+        <v>-2.481389578163772</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="137" t="n">
-        <v>32.25806451612903</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="V23" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W23" s="137" t="n">
-        <v>-32.25806451612903</v>
+        <v>-64.51612903225806</v>
       </c>
       <c r="X23" s="138" t="n">
         <v>-1</v>
@@ -5111,13 +5111,13 @@
         </is>
       </c>
       <c r="B24" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C24" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D24" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5185,13 +5185,13 @@
         </is>
       </c>
       <c r="B25" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C25" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D25" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5220,28 +5220,28 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>15.05376344086022</v>
+        <v>30.10752688172043</v>
       </c>
       <c r="R25" t="n">
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>-15.05376344086022</v>
+        <v>-30.10752688172043</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="137" t="n">
-        <v>677.4193548387096</v>
+        <v>1354.838709677419</v>
       </c>
       <c r="V25" s="137" t="n">
-        <v>585.7267119999999</v>
+        <v>1152.609557</v>
       </c>
       <c r="W25" s="137" t="n">
-        <v>-91.69264283870972</v>
+        <v>-202.2291526774193</v>
       </c>
       <c r="X25" s="138" t="n">
-        <v>-0.1353558060952381</v>
+        <v>-0.149264374595238</v>
       </c>
       <c r="Y25" s="137" t="n"/>
       <c r="Z25" s="137" t="n"/>
@@ -5261,13 +5261,13 @@
         </is>
       </c>
       <c r="B26" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C26" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D26" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5301,28 +5301,28 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>44.08769026783109</v>
+        <v>88.17538053566217</v>
       </c>
       <c r="R26" t="n">
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>-44.08769026783109</v>
+        <v>-88.17538053566217</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="137" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="V26" s="137" t="n">
-        <v>563.612112</v>
+        <v>1110.60139</v>
       </c>
       <c r="W26" s="137" t="n">
-        <v>-436.387888</v>
+        <v>-889.39861</v>
       </c>
       <c r="X26" s="138" t="n">
-        <v>-0.436387888</v>
+        <v>-0.444699305</v>
       </c>
       <c r="Y26" s="137" t="n"/>
       <c r="Z26" s="137" t="n"/>
@@ -5342,13 +5342,13 @@
         </is>
       </c>
       <c r="B27" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C27" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D27" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5382,13 +5382,13 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>43.62384455763064</v>
+        <v>87.24768911526128</v>
       </c>
       <c r="R27" t="n">
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>-43.62384455763064</v>
+        <v>-87.24768911526128</v>
       </c>
       <c r="T27" s="137" t="n">
         <v>523.8095238095239</v>
@@ -5421,13 +5421,13 @@
         </is>
       </c>
       <c r="B28" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="C28" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D28" s="136" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5461,28 +5461,28 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>102.7652982663219</v>
+        <v>205.5305965326439</v>
       </c>
       <c r="R28" t="n">
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>-102.7652982663219</v>
+        <v>-205.5305965326439</v>
       </c>
       <c r="T28" s="137" t="n">
         <v>2201.228878648234</v>
       </c>
       <c r="U28" s="137" t="n">
-        <v>1677.41935483871</v>
+        <v>3354.838709677419</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>1149.338824</v>
+        <v>2263.210947</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>-528.0805308387096</v>
+        <v>-1091.627762677419</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>-0.3148172395384615</v>
+        <v>-0.3253890446442307</v>
       </c>
       <c r="Y28" s="137" t="n"/>
       <c r="Z28" s="137" t="n"/>
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="B4" s="140" t="n">
-        <v>46235</v>
+        <v>46236</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5627,7 +5627,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5647,7 +5647,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46236.29188657407</v>
+        <v>46237.29186342593</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-04
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 02/08/2026  |  Ultimo aggiornamento: 03/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 03/08/2026  |  Ultimo aggiornamento: 04/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1065,16 +1065,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>612.9032258064516</v>
+        <v>919.3548387096772</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>523.218704</v>
+        <v>786.210618</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>-89.68452180645158</v>
+        <v>-133.1442207096774</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>-0.1463273776842104</v>
+        <v>-0.1448235383157894</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1173,16 +1173,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>96.7741935483871</v>
+        <v>145.1612903225807</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>63.640853</v>
+        <v>95.516713</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-33.1333405483871</v>
+        <v>-49.64457732258067</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.3423778523333334</v>
+        <v>-0.3419959771111112</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1281,16 +1281,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>645.1612903225806</v>
+        <v>967.741935483871</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>565.75</v>
+        <v>866.5700000000001</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-79.41129032258061</v>
+        <v>-101.1719354838709</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.1230874999999999</v>
+        <v>-0.1045443333333333</v>
       </c>
       <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
@@ -1328,28 +1328,28 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>30.10752688172043</v>
+        <v>45.16129032258065</v>
       </c>
       <c r="N10" s="125" t="n">
         <v>0</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>-30.10752688172043</v>
+        <v>-45.16129032258065</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>1354.838709677419</v>
+        <v>2032.258064516129</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>1152.609557</v>
+        <v>1748.297331</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>-202.2291526774193</v>
+        <v>-283.960733516129</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>-0.149264374595238</v>
+        <v>-0.1397267101428571</v>
       </c>
       <c r="U10" s="123" t="n"/>
       <c r="V10" s="123" t="n"/>
@@ -1403,28 +1403,28 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>7.590132827324478</v>
+        <v>11.38519924098672</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-7.590132827324478</v>
+        <v>-11.38519924098672</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>258.0645161290323</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>210.361052</v>
+        <v>313.871355</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>-47.70346412903226</v>
+        <v>-73.22541919354842</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>-0.1848509235</v>
+        <v>-0.18916566625</v>
       </c>
       <c r="U11" s="117" t="n"/>
       <c r="V11" s="117" t="n"/>
@@ -1482,28 +1482,28 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M12" s="127" t="n">
-        <v>15.08169250104734</v>
+        <v>22.62253875157101</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>-15.08169250104734</v>
+        <v>-22.62253875157101</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>580.6451612903226</v>
+        <v>870.9677419354839</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>273.700389</v>
+        <v>418.97482</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-306.9447722903226</v>
+        <v>-451.9929219354839</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.5286271078333333</v>
+        <v>-0.5189548362962962</v>
       </c>
       <c r="U12" s="128" t="n"/>
       <c r="V12" s="128" t="n"/>
@@ -1608,28 +1608,28 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="127" t="n">
-        <v>1.697792869269949</v>
+        <v>2.546689303904923</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-1.697792869269949</v>
+        <v>-2.546689303904923</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>64.51612903225806</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>33.988146</v>
+        <v>49.638146</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-30.52798303225806</v>
+        <v>-47.1360475483871</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.473183737</v>
+        <v>-0.4870724913333333</v>
       </c>
       <c r="U14" s="128" t="n"/>
       <c r="V14" s="128" t="n"/>
@@ -1734,25 +1734,25 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M16" s="127" t="n">
-        <v>0.2580645161290322</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>-0.2580645161290322</v>
+        <v>-0.3870967741935484</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>64.51612903225806</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="R16" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>-64.51612903225806</v>
+        <v>-96.7741935483871</v>
       </c>
       <c r="T16" s="118" t="n">
         <v>-1</v>
@@ -1860,28 +1860,28 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>50.40322580645162</v>
+        <v>75.60483870967742</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-50.40322580645162</v>
+        <v>-75.60483870967742</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>645.1612903225806</v>
+        <v>967.741935483871</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>351.12</v>
+        <v>548.63</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>-294.0412903225806</v>
+        <v>-419.111935483871</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>-0.4557639999999999</v>
+        <v>-0.4330823333333333</v>
       </c>
       <c r="U18" s="117" t="n"/>
       <c r="V18" s="117" t="n"/>
@@ -1939,28 +1939,28 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>0.8064516129032258</v>
+        <v>1.209677419354838</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-0.8064516129032258</v>
+        <v>-1.209677419354838</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>32.25806451612903</v>
+        <v>48.38709677419355</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>21.7</v>
+        <v>31.28</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-10.55806451612903</v>
+        <v>-17.10709677419355</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.3273</v>
+        <v>-0.3535466666666667</v>
       </c>
       <c r="U19" s="117" t="n"/>
       <c r="V19" s="117" t="n"/>
@@ -2014,28 +2014,28 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>0.7168458781362007</v>
+        <v>1.075268817204301</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-0.7168458781362007</v>
+        <v>-1.075268817204301</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>64.51612903225806</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>20.8</v>
+        <v>31.97</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-43.71612903225807</v>
+        <v>-64.8041935483871</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.6776000000000001</v>
+        <v>-0.6696433333333334</v>
       </c>
       <c r="U20" s="117" t="n"/>
       <c r="V20" s="117" t="n"/>
@@ -2089,25 +2089,25 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>0.2688172043010753</v>
+        <v>0.403225806451613</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-0.2688172043010753</v>
+        <v>-0.403225806451613</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>32.25806451612903</v>
+        <v>48.38709677419355</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-32.25806451612903</v>
+        <v>-48.38709677419355</v>
       </c>
       <c r="T21" s="118" t="n">
         <v>-1</v>
@@ -2164,28 +2164,28 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>2.419354838709677</v>
+        <v>3.629032258064516</v>
       </c>
       <c r="N22" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-2.419354838709677</v>
+        <v>-3.629032258064516</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>96.7741935483871</v>
+        <v>145.1612903225807</v>
       </c>
       <c r="R22" s="117" t="n">
         <v>9.625539</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>-87.1486545483871</v>
+        <v>-135.5357513225807</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>-0.9005360969999999</v>
+        <v>-0.9336907313333334</v>
       </c>
       <c r="U22" s="117" t="n"/>
       <c r="V22" s="117" t="n"/>
@@ -2239,28 +2239,28 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>6.451612903225806</v>
+        <v>9.677419354838708</v>
       </c>
       <c r="N23" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>-6.451612903225806</v>
+        <v>-9.677419354838708</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>96.7741935483871</v>
+        <v>145.1612903225807</v>
       </c>
       <c r="R23" s="117" t="n">
-        <v>189.306264</v>
+        <v>227.600087</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>92.5320704516129</v>
+        <v>82.43879667741933</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.956164728</v>
+        <v>0.5679117104444442</v>
       </c>
       <c r="U23" s="117" t="n"/>
       <c r="V23" s="117" t="n"/>
@@ -2318,25 +2318,25 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>2.481389578163772</v>
+        <v>3.722084367245658</v>
       </c>
       <c r="N24" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>-2.481389578163772</v>
+        <v>-3.722084367245658</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>64.51612903225806</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="R24" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>-64.51612903225806</v>
+        <v>-96.7741935483871</v>
       </c>
       <c r="T24" s="118" t="n">
         <v>-1</v>
@@ -2388,7 +2388,7 @@
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>0</v>
+        <v>60.68</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
@@ -2428,28 +2428,28 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>88.17538053566217</v>
+        <v>132.2630708034933</v>
       </c>
       <c r="N26" s="125" t="n">
         <v>0</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>-88.17538053566217</v>
+        <v>-132.2630708034933</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>1110.60139</v>
+        <v>1692.269947</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>-889.39861</v>
+        <v>-1307.730053</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>-0.444699305</v>
+        <v>-0.4359100176666666</v>
       </c>
       <c r="U26" s="123" t="n"/>
       <c r="V26" s="123" t="n"/>
@@ -2499,27 +2499,29 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>42.44482173174873</v>
+        <v>63.6672325976231</v>
       </c>
       <c r="N27" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-42.44482173174873</v>
+        <v>-63.6672325976231</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>238.0952380952381</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>0</v>
+        <v>238.0952380952381</v>
       </c>
       <c r="R27" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>0</v>
-      </c>
-      <c r="T27" s="118" t="n"/>
+        <v>-238.0952380952381</v>
+      </c>
+      <c r="T27" s="118" t="n">
+        <v>-1</v>
+      </c>
       <c r="U27" s="117" t="n"/>
       <c r="V27" s="117" t="n"/>
       <c r="W27" s="120" t="inlineStr"/>
@@ -2568,27 +2570,29 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>28.67383512544803</v>
+        <v>43.01075268817205</v>
       </c>
       <c r="N28" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-28.67383512544803</v>
+        <v>-43.01075268817205</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>190.4761904761905</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>0</v>
+        <v>190.4761904761905</v>
       </c>
       <c r="R28" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>0</v>
-      </c>
-      <c r="T28" s="118" t="n"/>
+        <v>-190.4761904761905</v>
+      </c>
+      <c r="T28" s="118" t="n">
+        <v>-1</v>
+      </c>
       <c r="U28" s="117" t="n"/>
       <c r="V28" s="117" t="n"/>
       <c r="W28" s="120" t="inlineStr"/>
@@ -2637,27 +2641,29 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>16.12903225806452</v>
+        <v>24.19354838709678</v>
       </c>
       <c r="N29" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>-16.12903225806452</v>
+        <v>-24.19354838709678</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>95.23809523809524</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>0</v>
+        <v>95.23809523809524</v>
       </c>
       <c r="R29" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>0</v>
-      </c>
-      <c r="T29" s="118" t="n"/>
+        <v>-95.23809523809524</v>
+      </c>
+      <c r="T29" s="118" t="n">
+        <v>-1</v>
+      </c>
       <c r="U29" s="117" t="n"/>
       <c r="V29" s="117" t="n"/>
       <c r="W29" s="120" t="inlineStr"/>
@@ -2694,27 +2700,29 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>87.24768911526128</v>
+        <v>130.8715336728919</v>
       </c>
       <c r="N30" s="125" t="n">
         <v>0</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-87.24768911526128</v>
+        <v>-130.8715336728919</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>523.8095238095239</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>0</v>
+        <v>523.8095238095239</v>
       </c>
       <c r="R30" s="123" t="n">
         <v>0</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>0</v>
-      </c>
-      <c r="T30" s="124" t="n"/>
+        <v>-523.8095238095239</v>
+      </c>
+      <c r="T30" s="124" t="n">
+        <v>-1</v>
+      </c>
       <c r="U30" s="123" t="n"/>
       <c r="V30" s="123" t="n"/>
       <c r="W30" s="126" t="n"/>
@@ -2751,28 +2759,28 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="133" t="n">
-        <v>205.5305965326439</v>
+        <v>308.2958947989658</v>
       </c>
       <c r="N31" s="133" t="n">
         <v>0</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>-205.5305965326439</v>
+        <v>-308.2958947989658</v>
       </c>
       <c r="P31" s="131" t="n">
         <v>2201.228878648234</v>
       </c>
       <c r="Q31" s="131" t="n">
-        <v>3354.838709677419</v>
+        <v>5556.067588325653</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>2263.210947</v>
+        <v>3440.567278</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>-1091.627762677419</v>
+        <v>-2115.500310325653</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>-0.3253890446442307</v>
+        <v>-0.3807549632352778</v>
       </c>
       <c r="U31" s="131" t="n"/>
       <c r="V31" s="131" t="n"/>
@@ -3055,13 +3063,13 @@
         </is>
       </c>
       <c r="B2" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C2" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3098,16 +3106,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="137" t="n">
-        <v>612.9032258064516</v>
+        <v>919.3548387096772</v>
       </c>
       <c r="V2" s="137" t="n">
-        <v>523.218704</v>
+        <v>786.210618</v>
       </c>
       <c r="W2" s="137" t="n">
-        <v>-89.68452180645158</v>
+        <v>-133.1442207096774</v>
       </c>
       <c r="X2" s="138" t="n">
-        <v>-0.1463273776842104</v>
+        <v>-0.1448235383157894</v>
       </c>
       <c r="Y2" s="137" t="n"/>
       <c r="Z2" s="137" t="n"/>
@@ -3125,7 +3133,7 @@
       <c r="AD2" s="139" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_3;crm:stale</t>
+          <t>google:ok;google:includes_excel_row_3</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -3141,13 +3149,13 @@
         </is>
       </c>
       <c r="B3" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C3" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3192,7 +3200,7 @@
       <c r="AD3" s="139" t="inlineStr"/>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_2;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_2</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -3208,13 +3216,13 @@
         </is>
       </c>
       <c r="B4" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C4" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3251,16 +3259,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="137" t="n">
-        <v>96.7741935483871</v>
+        <v>145.1612903225807</v>
       </c>
       <c r="V4" s="137" t="n">
-        <v>63.640853</v>
+        <v>95.516713</v>
       </c>
       <c r="W4" s="137" t="n">
-        <v>-33.1333405483871</v>
+        <v>-49.64457732258067</v>
       </c>
       <c r="X4" s="138" t="n">
-        <v>-0.3423778523333334</v>
+        <v>-0.3419959771111112</v>
       </c>
       <c r="Y4" s="137" t="n"/>
       <c r="Z4" s="137" t="n"/>
@@ -3278,7 +3286,7 @@
       <c r="AD4" s="139" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_5;crm:stale</t>
+          <t>google:ok;google:includes_excel_row_5</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -3294,13 +3302,13 @@
         </is>
       </c>
       <c r="B5" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C5" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3345,7 +3353,7 @@
       <c r="AD5" s="139" t="inlineStr"/>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_4;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_4</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -3361,13 +3369,13 @@
         </is>
       </c>
       <c r="B6" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C6" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3404,16 +3412,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="137" t="n">
-        <v>645.1612903225806</v>
+        <v>967.741935483871</v>
       </c>
       <c r="V6" s="137" t="n">
-        <v>565.75</v>
+        <v>866.5700000000001</v>
       </c>
       <c r="W6" s="137" t="n">
-        <v>-79.41129032258061</v>
+        <v>-101.1719354838709</v>
       </c>
       <c r="X6" s="138" t="n">
-        <v>-0.1230874999999999</v>
+        <v>-0.1045443333333333</v>
       </c>
       <c r="Y6" s="137" t="n"/>
       <c r="Z6" s="137" t="n"/>
@@ -3431,7 +3439,7 @@
       <c r="AD6" s="139" t="inlineStr"/>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -3447,13 +3455,13 @@
         </is>
       </c>
       <c r="B7" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C7" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -3500,27 +3508,29 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>42.44482173174873</v>
+        <v>63.6672325976231</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>-42.44482173174873</v>
+        <v>-63.6672325976231</v>
       </c>
       <c r="T7" s="137" t="n">
         <v>238.0952380952381</v>
       </c>
       <c r="U7" s="137" t="n">
-        <v>0</v>
+        <v>238.0952380952381</v>
       </c>
       <c r="V7" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W7" s="137" t="n">
-        <v>0</v>
-      </c>
-      <c r="X7" s="138" t="n"/>
+        <v>-238.0952380952381</v>
+      </c>
+      <c r="X7" s="138" t="n">
+        <v>-1</v>
+      </c>
       <c r="Y7" s="137" t="n"/>
       <c r="Z7" s="137" t="n"/>
       <c r="AB7" s="139" t="inlineStr"/>
@@ -3528,7 +3538,7 @@
       <c r="AD7" s="139" t="inlineStr"/>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>manual:no_ads_source;crm:stale</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -3544,13 +3554,13 @@
         </is>
       </c>
       <c r="B8" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C8" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E8" t="n">
         <v>26</v>
@@ -3597,27 +3607,29 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>28.67383512544803</v>
+        <v>43.01075268817205</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>-28.67383512544803</v>
+        <v>-43.01075268817205</v>
       </c>
       <c r="T8" s="137" t="n">
         <v>190.4761904761905</v>
       </c>
       <c r="U8" s="137" t="n">
-        <v>0</v>
+        <v>190.4761904761905</v>
       </c>
       <c r="V8" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W8" s="137" t="n">
-        <v>0</v>
-      </c>
-      <c r="X8" s="138" t="n"/>
+        <v>-190.4761904761905</v>
+      </c>
+      <c r="X8" s="138" t="n">
+        <v>-1</v>
+      </c>
       <c r="Y8" s="137" t="n"/>
       <c r="Z8" s="137" t="n"/>
       <c r="AB8" s="139" t="inlineStr"/>
@@ -3625,7 +3637,7 @@
       <c r="AD8" s="139" t="inlineStr"/>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>manual:no_ads_source;crm:stale</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -3641,13 +3653,13 @@
         </is>
       </c>
       <c r="B9" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C9" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3694,27 +3706,29 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>16.12903225806452</v>
+        <v>24.19354838709678</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>-16.12903225806452</v>
+        <v>-24.19354838709678</v>
       </c>
       <c r="T9" s="137" t="n">
         <v>95.23809523809524</v>
       </c>
       <c r="U9" s="137" t="n">
-        <v>0</v>
+        <v>95.23809523809524</v>
       </c>
       <c r="V9" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W9" s="137" t="n">
-        <v>0</v>
-      </c>
-      <c r="X9" s="138" t="n"/>
+        <v>-95.23809523809524</v>
+      </c>
+      <c r="X9" s="138" t="n">
+        <v>-1</v>
+      </c>
       <c r="Y9" s="137" t="n"/>
       <c r="Z9" s="137" t="n"/>
       <c r="AB9" s="139" t="inlineStr"/>
@@ -3722,7 +3736,7 @@
       <c r="AD9" s="139" t="inlineStr"/>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>manual:no_ads_source;crm:stale</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -3738,13 +3752,13 @@
         </is>
       </c>
       <c r="B10" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C10" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3791,28 +3805,28 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>7.590132827324478</v>
+        <v>11.38519924098672</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>-7.590132827324478</v>
+        <v>-11.38519924098672</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U10" s="137" t="n">
-        <v>258.0645161290323</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="V10" s="137" t="n">
-        <v>210.361052</v>
+        <v>313.871355</v>
       </c>
       <c r="W10" s="137" t="n">
-        <v>-47.70346412903226</v>
+        <v>-73.22541919354842</v>
       </c>
       <c r="X10" s="138" t="n">
-        <v>-0.1848509235</v>
+        <v>-0.18916566625</v>
       </c>
       <c r="Y10" s="137" t="n"/>
       <c r="Z10" s="137" t="n"/>
@@ -3830,7 +3844,7 @@
       <c r="AD10" s="139" t="inlineStr"/>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:ok</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -3846,13 +3860,13 @@
         </is>
       </c>
       <c r="B11" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C11" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3899,28 +3913,28 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q11" t="n">
-        <v>15.08169250104734</v>
+        <v>22.62253875157101</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>-15.08169250104734</v>
+        <v>-22.62253875157101</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U11" s="137" t="n">
-        <v>580.6451612903226</v>
+        <v>870.9677419354839</v>
       </c>
       <c r="V11" s="137" t="n">
-        <v>273.700389</v>
+        <v>418.97482</v>
       </c>
       <c r="W11" s="137" t="n">
-        <v>-306.9447722903226</v>
+        <v>-451.9929219354839</v>
       </c>
       <c r="X11" s="138" t="n">
-        <v>-0.5286271078333333</v>
+        <v>-0.5189548362962962</v>
       </c>
       <c r="Y11" s="137" t="n"/>
       <c r="Z11" s="137" t="n"/>
@@ -3938,7 +3952,7 @@
       <c r="AD11" s="139" t="inlineStr"/>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_10;crm_metrics_combined_with_excel_row_10;crm:stale</t>
+          <t>google:ok;google:includes_excel_row_10;crm_metrics_combined_with_excel_row_10</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -3954,13 +3968,13 @@
         </is>
       </c>
       <c r="B12" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C12" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -4008,7 +4022,7 @@
       <c r="AD12" s="139" t="inlineStr"/>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_9;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_9</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -4024,13 +4038,13 @@
         </is>
       </c>
       <c r="B13" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C13" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4077,28 +4091,28 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>1.697792869269949</v>
+        <v>2.546689303904923</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>-1.697792869269949</v>
+        <v>-2.546689303904923</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="137" t="n">
-        <v>64.51612903225806</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="V13" s="137" t="n">
-        <v>33.988146</v>
+        <v>49.638146</v>
       </c>
       <c r="W13" s="137" t="n">
-        <v>-30.52798303225806</v>
+        <v>-47.1360475483871</v>
       </c>
       <c r="X13" s="138" t="n">
-        <v>-0.473183737</v>
+        <v>-0.4870724913333333</v>
       </c>
       <c r="Y13" s="137" t="n"/>
       <c r="Z13" s="137" t="n"/>
@@ -4116,7 +4130,7 @@
       <c r="AD13" s="139" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_12;crm_metrics_combined_with_excel_row_12;crm:stale</t>
+          <t>google:ok;google:includes_excel_row_12;crm_metrics_combined_with_excel_row_12</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -4132,13 +4146,13 @@
         </is>
       </c>
       <c r="B14" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C14" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
@@ -4186,7 +4200,7 @@
       <c r="AD14" s="139" t="inlineStr"/>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_11;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_11</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -4202,13 +4216,13 @@
         </is>
       </c>
       <c r="B15" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C15" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -4255,25 +4269,25 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.2580645161290322</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.2580645161290322</v>
+        <v>-0.3870967741935484</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U15" s="137" t="n">
-        <v>64.51612903225806</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="V15" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W15" s="137" t="n">
-        <v>-64.51612903225806</v>
+        <v>-96.7741935483871</v>
       </c>
       <c r="X15" s="138" t="n">
         <v>-1</v>
@@ -4294,7 +4308,7 @@
       <c r="AD15" s="139" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_14;crm_metrics_combined_with_excel_row_14;crm:stale</t>
+          <t>google:ok;google:includes_excel_row_14;crm_metrics_combined_with_excel_row_14</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -4310,13 +4324,13 @@
         </is>
       </c>
       <c r="B16" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C16" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4364,7 +4378,7 @@
       <c r="AD16" s="139" t="inlineStr"/>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_13;crm:stale</t>
+          <t>google:rolled_up_to_excel_row_13</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -4380,13 +4394,13 @@
         </is>
       </c>
       <c r="B17" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C17" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E17" t="n">
         <v>17</v>
@@ -4433,28 +4447,28 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>50.40322580645162</v>
+        <v>75.60483870967742</v>
       </c>
       <c r="R17" t="n">
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>-50.40322580645162</v>
+        <v>-75.60483870967742</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U17" s="137" t="n">
-        <v>645.1612903225806</v>
+        <v>967.741935483871</v>
       </c>
       <c r="V17" s="137" t="n">
-        <v>351.12</v>
+        <v>548.63</v>
       </c>
       <c r="W17" s="137" t="n">
-        <v>-294.0412903225806</v>
+        <v>-419.111935483871</v>
       </c>
       <c r="X17" s="138" t="n">
-        <v>-0.4557639999999999</v>
+        <v>-0.4330823333333333</v>
       </c>
       <c r="Y17" s="137" t="n"/>
       <c r="Z17" s="137" t="n"/>
@@ -4472,7 +4486,7 @@
       <c r="AD17" s="139" t="inlineStr"/>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
@@ -4488,13 +4502,13 @@
         </is>
       </c>
       <c r="B18" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C18" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4541,28 +4555,28 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.8064516129032258</v>
+        <v>1.209677419354838</v>
       </c>
       <c r="R18" t="n">
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>-0.8064516129032258</v>
+        <v>-1.209677419354838</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="137" t="n">
-        <v>32.25806451612903</v>
+        <v>48.38709677419355</v>
       </c>
       <c r="V18" s="137" t="n">
-        <v>21.7</v>
+        <v>31.28</v>
       </c>
       <c r="W18" s="137" t="n">
-        <v>-10.55806451612903</v>
+        <v>-17.10709677419355</v>
       </c>
       <c r="X18" s="138" t="n">
-        <v>-0.3273</v>
+        <v>-0.3535466666666667</v>
       </c>
       <c r="Y18" s="137" t="n"/>
       <c r="Z18" s="137" t="n"/>
@@ -4575,7 +4589,7 @@
       <c r="AD18" s="139" t="inlineStr"/>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
@@ -4591,13 +4605,13 @@
         </is>
       </c>
       <c r="B19" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C19" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4644,28 +4658,28 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.7168458781362007</v>
+        <v>1.075268817204301</v>
       </c>
       <c r="R19" t="n">
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>-0.7168458781362007</v>
+        <v>-1.075268817204301</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="137" t="n">
-        <v>64.51612903225806</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="V19" s="137" t="n">
-        <v>20.8</v>
+        <v>31.97</v>
       </c>
       <c r="W19" s="137" t="n">
-        <v>-43.71612903225807</v>
+        <v>-64.8041935483871</v>
       </c>
       <c r="X19" s="138" t="n">
-        <v>-0.6776000000000001</v>
+        <v>-0.6696433333333334</v>
       </c>
       <c r="Y19" s="137" t="n"/>
       <c r="Z19" s="137" t="n"/>
@@ -4678,7 +4692,7 @@
       <c r="AD19" s="139" t="inlineStr"/>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
@@ -4694,13 +4708,13 @@
         </is>
       </c>
       <c r="B20" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C20" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
@@ -4747,25 +4761,25 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.2688172043010753</v>
+        <v>0.403225806451613</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.2688172043010753</v>
+        <v>-0.403225806451613</v>
       </c>
       <c r="T20" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U20" s="137" t="n">
-        <v>32.25806451612903</v>
+        <v>48.38709677419355</v>
       </c>
       <c r="V20" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W20" s="137" t="n">
-        <v>-32.25806451612903</v>
+        <v>-48.38709677419355</v>
       </c>
       <c r="X20" s="138" t="n">
         <v>-1</v>
@@ -4781,7 +4795,7 @@
       <c r="AD20" s="139" t="inlineStr"/>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>meta:no_delivery;crm:stale</t>
+          <t>meta:no_delivery</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr">
@@ -4797,13 +4811,13 @@
         </is>
       </c>
       <c r="B21" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C21" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D21" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4850,28 +4864,28 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>2.419354838709677</v>
+        <v>3.629032258064516</v>
       </c>
       <c r="R21" t="n">
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>-2.419354838709677</v>
+        <v>-3.629032258064516</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="137" t="n">
-        <v>96.7741935483871</v>
+        <v>145.1612903225807</v>
       </c>
       <c r="V21" s="137" t="n">
         <v>9.625539</v>
       </c>
       <c r="W21" s="137" t="n">
-        <v>-87.1486545483871</v>
+        <v>-135.5357513225807</v>
       </c>
       <c r="X21" s="138" t="n">
-        <v>-0.9005360969999999</v>
+        <v>-0.9336907313333334</v>
       </c>
       <c r="Y21" s="137" t="n"/>
       <c r="Z21" s="137" t="n"/>
@@ -4884,7 +4898,7 @@
       <c r="AD21" s="139" t="inlineStr"/>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:ok</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
@@ -4900,13 +4914,13 @@
         </is>
       </c>
       <c r="B22" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C22" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D22" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -4953,28 +4967,28 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>6.451612903225806</v>
+        <v>9.677419354838708</v>
       </c>
       <c r="R22" t="n">
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>-6.451612903225806</v>
+        <v>-9.677419354838708</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="137" t="n">
-        <v>96.7741935483871</v>
+        <v>145.1612903225807</v>
       </c>
       <c r="V22" s="137" t="n">
-        <v>189.306264</v>
+        <v>227.600087</v>
       </c>
       <c r="W22" s="137" t="n">
-        <v>92.5320704516129</v>
+        <v>82.43879667741933</v>
       </c>
       <c r="X22" s="138" t="n">
-        <v>0.956164728</v>
+        <v>0.5679117104444442</v>
       </c>
       <c r="Y22" s="137" t="n"/>
       <c r="Z22" s="137" t="n"/>
@@ -4992,7 +5006,7 @@
       <c r="AD22" s="139" t="inlineStr"/>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:ok</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
@@ -5008,13 +5022,13 @@
         </is>
       </c>
       <c r="B23" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C23" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D23" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5061,25 +5075,25 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>2.481389578163772</v>
+        <v>3.722084367245658</v>
       </c>
       <c r="R23" t="n">
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>-2.481389578163772</v>
+        <v>-3.722084367245658</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="137" t="n">
-        <v>64.51612903225806</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="V23" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W23" s="137" t="n">
-        <v>-64.51612903225806</v>
+        <v>-96.7741935483871</v>
       </c>
       <c r="X23" s="138" t="n">
         <v>-1</v>
@@ -5095,7 +5109,7 @@
       <c r="AD23" s="139" t="inlineStr"/>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>meta:no_delivery;crm:stale</t>
+          <t>meta:no_delivery</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -5111,13 +5125,13 @@
         </is>
       </c>
       <c r="B24" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C24" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D24" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5154,7 +5168,7 @@
       <c r="T24" s="137" t="n"/>
       <c r="U24" s="137" t="n"/>
       <c r="V24" s="137" t="n">
-        <v>0</v>
+        <v>60.68</v>
       </c>
       <c r="W24" s="137" t="n"/>
       <c r="X24" s="138" t="n"/>
@@ -5169,7 +5183,7 @@
       <c r="AD24" s="139" t="inlineStr"/>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>meta:no_delivery;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
@@ -5185,13 +5199,13 @@
         </is>
       </c>
       <c r="B25" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C25" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D25" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5220,28 +5234,28 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>30.10752688172043</v>
+        <v>45.16129032258065</v>
       </c>
       <c r="R25" t="n">
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>-30.10752688172043</v>
+        <v>-45.16129032258065</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="137" t="n">
-        <v>1354.838709677419</v>
+        <v>2032.258064516129</v>
       </c>
       <c r="V25" s="137" t="n">
-        <v>1152.609557</v>
+        <v>1748.297331</v>
       </c>
       <c r="W25" s="137" t="n">
-        <v>-202.2291526774193</v>
+        <v>-283.960733516129</v>
       </c>
       <c r="X25" s="138" t="n">
-        <v>-0.149264374595238</v>
+        <v>-0.1397267101428571</v>
       </c>
       <c r="Y25" s="137" t="n"/>
       <c r="Z25" s="137" t="n"/>
@@ -5250,7 +5264,7 @@
       <c r="AD25" s="139" t="inlineStr"/>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>partial;crm:stale</t>
+          <t>partial</t>
         </is>
       </c>
     </row>
@@ -5261,13 +5275,13 @@
         </is>
       </c>
       <c r="B26" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C26" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D26" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5301,28 +5315,28 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>88.17538053566217</v>
+        <v>132.2630708034933</v>
       </c>
       <c r="R26" t="n">
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>-88.17538053566217</v>
+        <v>-132.2630708034933</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="137" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="V26" s="137" t="n">
-        <v>1110.60139</v>
+        <v>1692.269947</v>
       </c>
       <c r="W26" s="137" t="n">
-        <v>-889.39861</v>
+        <v>-1307.730053</v>
       </c>
       <c r="X26" s="138" t="n">
-        <v>-0.444699305</v>
+        <v>-0.4359100176666666</v>
       </c>
       <c r="Y26" s="137" t="n"/>
       <c r="Z26" s="137" t="n"/>
@@ -5331,7 +5345,7 @@
       <c r="AD26" s="139" t="inlineStr"/>
       <c r="AE26" t="inlineStr">
         <is>
-          <t>partial;crm:stale</t>
+          <t>partial</t>
         </is>
       </c>
     </row>
@@ -5342,13 +5356,13 @@
         </is>
       </c>
       <c r="B27" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C27" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D27" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5382,27 +5396,29 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>87.24768911526128</v>
+        <v>130.8715336728919</v>
       </c>
       <c r="R27" t="n">
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>-87.24768911526128</v>
+        <v>-130.8715336728919</v>
       </c>
       <c r="T27" s="137" t="n">
         <v>523.8095238095239</v>
       </c>
       <c r="U27" s="137" t="n">
-        <v>0</v>
+        <v>523.8095238095239</v>
       </c>
       <c r="V27" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W27" s="137" t="n">
-        <v>0</v>
-      </c>
-      <c r="X27" s="138" t="n"/>
+        <v>-523.8095238095239</v>
+      </c>
+      <c r="X27" s="138" t="n">
+        <v>-1</v>
+      </c>
       <c r="Y27" s="137" t="n"/>
       <c r="Z27" s="137" t="n"/>
       <c r="AB27" s="139" t="inlineStr"/>
@@ -5410,7 +5426,7 @@
       <c r="AD27" s="139" t="inlineStr"/>
       <c r="AE27" t="inlineStr">
         <is>
-          <t>success;crm:stale</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -5421,13 +5437,13 @@
         </is>
       </c>
       <c r="B28" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="C28" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D28" s="136" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5461,28 +5477,28 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>205.5305965326439</v>
+        <v>308.2958947989658</v>
       </c>
       <c r="R28" t="n">
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>-205.5305965326439</v>
+        <v>-308.2958947989658</v>
       </c>
       <c r="T28" s="137" t="n">
         <v>2201.228878648234</v>
       </c>
       <c r="U28" s="137" t="n">
-        <v>3354.838709677419</v>
+        <v>5556.067588325653</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>2263.210947</v>
+        <v>3440.567278</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>-1091.627762677419</v>
+        <v>-2115.500310325653</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>-0.3253890446442307</v>
+        <v>-0.3807549632352778</v>
       </c>
       <c r="Y28" s="137" t="n"/>
       <c r="Z28" s="137" t="n"/>
@@ -5491,7 +5507,7 @@
       <c r="AD28" s="139" t="inlineStr"/>
       <c r="AE28" t="inlineStr">
         <is>
-          <t>partial;crm:stale</t>
+          <t>partial</t>
         </is>
       </c>
     </row>
@@ -5587,7 +5603,7 @@
         </is>
       </c>
       <c r="B4" s="140" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5627,7 +5643,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5647,7 +5663,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46237.29186342593</v>
+        <v>46238.29189814815</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-05
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 03/08/2026  |  Ultimo aggiornamento: 04/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 04/08/2026  |  Ultimo aggiornamento: 05/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1065,16 +1065,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>919.3548387096772</v>
+        <v>1225.806451612903</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>786.210618</v>
+        <v>1058.588747</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>-133.1442207096774</v>
+        <v>-167.2177046129032</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>-0.1448235383157894</v>
+        <v>-0.136414443236842</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1173,16 +1173,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>145.1612903225807</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>95.516713</v>
+        <v>127.524928</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-49.64457732258067</v>
+        <v>-66.0234590967742</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.3419959771111112</v>
+        <v>-0.3411212053333333</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1281,16 +1281,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>967.741935483871</v>
+        <v>1290.322580645161</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>866.5700000000001</v>
+        <v>1157.8</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-101.1719354838709</v>
+        <v>-132.5225806451613</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.1045443333333333</v>
+        <v>-0.1027049999999999</v>
       </c>
       <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
@@ -1328,28 +1328,28 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>45.16129032258065</v>
+        <v>60.21505376344086</v>
       </c>
       <c r="N10" s="125" t="n">
         <v>0</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>-45.16129032258065</v>
+        <v>-60.21505376344086</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>2032.258064516129</v>
+        <v>2709.677419354839</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>1748.297331</v>
+        <v>2343.913675</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>-283.960733516129</v>
+        <v>-365.7637443548388</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>-0.1397267101428571</v>
+        <v>-0.1349842389880952</v>
       </c>
       <c r="U10" s="123" t="n"/>
       <c r="V10" s="123" t="n"/>
@@ -1403,28 +1403,28 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>11.38519924098672</v>
+        <v>15.18026565464896</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-11.38519924098672</v>
+        <v>-15.18026565464896</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>387.0967741935484</v>
+        <v>516.1290322580645</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>313.871355</v>
+        <v>416.563481</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>-73.22541919354842</v>
+        <v>-99.56555125806447</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>-0.18916566625</v>
+        <v>-0.1929082555624999</v>
       </c>
       <c r="U11" s="117" t="n"/>
       <c r="V11" s="117" t="n"/>
@@ -1482,28 +1482,28 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M12" s="127" t="n">
-        <v>22.62253875157101</v>
+        <v>30.16338500209468</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>-22.62253875157101</v>
+        <v>-30.16338500209468</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>870.9677419354839</v>
+        <v>1161.290322580645</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>418.97482</v>
+        <v>556.533175</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-451.9929219354839</v>
+        <v>-604.7571475806451</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.5189548362962962</v>
+        <v>-0.5207630993055555</v>
       </c>
       <c r="U12" s="128" t="n"/>
       <c r="V12" s="128" t="n"/>
@@ -1608,28 +1608,28 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="127" t="n">
-        <v>2.546689303904923</v>
+        <v>3.395585738539898</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-2.546689303904923</v>
+        <v>-3.395585738539898</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>96.7741935483871</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>49.638146</v>
+        <v>68.008146</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-47.1360475483871</v>
+        <v>-61.02411206451613</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.4870724913333333</v>
+        <v>-0.4729368685</v>
       </c>
       <c r="U14" s="128" t="n"/>
       <c r="V14" s="128" t="n"/>
@@ -1734,25 +1734,25 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M16" s="127" t="n">
-        <v>0.3870967741935484</v>
+        <v>0.5161290322580645</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>-0.3870967741935484</v>
+        <v>-0.5161290322580645</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>96.7741935483871</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="R16" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>-96.7741935483871</v>
+        <v>-129.0322580645161</v>
       </c>
       <c r="T16" s="118" t="n">
         <v>-1</v>
@@ -1860,28 +1860,28 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>75.60483870967742</v>
+        <v>100.8064516129032</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-75.60483870967742</v>
+        <v>-100.8064516129032</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>967.741935483871</v>
+        <v>1290.322580645161</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>548.63</v>
+        <v>717.78</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>-419.111935483871</v>
+        <v>-572.5425806451613</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>-0.4330823333333333</v>
+        <v>-0.4437205</v>
       </c>
       <c r="U18" s="117" t="n"/>
       <c r="V18" s="117" t="n"/>
@@ -1939,28 +1939,28 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>1.209677419354838</v>
+        <v>1.612903225806452</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-1.209677419354838</v>
+        <v>-1.612903225806452</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>48.38709677419355</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>31.28</v>
+        <v>42.43</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-17.10709677419355</v>
+        <v>-22.08612903225806</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.3535466666666667</v>
+        <v>-0.342335</v>
       </c>
       <c r="U19" s="117" t="n"/>
       <c r="V19" s="117" t="n"/>
@@ -2014,28 +2014,28 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>1.075268817204301</v>
+        <v>1.433691756272401</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-1.075268817204301</v>
+        <v>-1.433691756272401</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>96.7741935483871</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>31.97</v>
+        <v>39.57</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-64.8041935483871</v>
+        <v>-89.46225806451613</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.6696433333333334</v>
+        <v>-0.6933325</v>
       </c>
       <c r="U20" s="117" t="n"/>
       <c r="V20" s="117" t="n"/>
@@ -2089,25 +2089,25 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>0.403225806451613</v>
+        <v>0.5376344086021506</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-0.403225806451613</v>
+        <v>-0.5376344086021506</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>48.38709677419355</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-48.38709677419355</v>
+        <v>-64.51612903225806</v>
       </c>
       <c r="T21" s="118" t="n">
         <v>-1</v>
@@ -2164,28 +2164,28 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>3.629032258064516</v>
+        <v>4.838709677419355</v>
       </c>
       <c r="N22" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-3.629032258064516</v>
+        <v>-4.838709677419355</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>145.1612903225807</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="R22" s="117" t="n">
         <v>9.625539</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>-135.5357513225807</v>
+        <v>-183.9228480967742</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>-0.9336907313333334</v>
+        <v>-0.9502680485</v>
       </c>
       <c r="U22" s="117" t="n"/>
       <c r="V22" s="117" t="n"/>
@@ -2239,28 +2239,28 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>9.677419354838708</v>
+        <v>12.90322580645161</v>
       </c>
       <c r="N23" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>-9.677419354838708</v>
+        <v>-12.90322580645161</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>145.1612903225807</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="R23" s="117" t="n">
-        <v>227.600087</v>
+        <v>282.294398</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>82.43879667741933</v>
+        <v>88.74601090322579</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.5679117104444442</v>
+        <v>0.4585210563333332</v>
       </c>
       <c r="U23" s="117" t="n"/>
       <c r="V23" s="117" t="n"/>
@@ -2318,25 +2318,25 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>3.722084367245658</v>
+        <v>4.962779156327543</v>
       </c>
       <c r="N24" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>-3.722084367245658</v>
+        <v>-4.962779156327543</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>96.7741935483871</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="R24" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>-96.7741935483871</v>
+        <v>-129.0322580645161</v>
       </c>
       <c r="T24" s="118" t="n">
         <v>-1</v>
@@ -2388,7 +2388,7 @@
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>60.68</v>
+        <v>97.5</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
@@ -2428,28 +2428,28 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>132.2630708034933</v>
+        <v>176.3507610713243</v>
       </c>
       <c r="N26" s="125" t="n">
         <v>0</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>-132.2630708034933</v>
+        <v>-176.3507610713243</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>1692.269947</v>
+        <v>2230.304739</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>-1307.730053</v>
+        <v>-1769.695261</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>-0.4359100176666666</v>
+        <v>-0.4424238152499999</v>
       </c>
       <c r="U26" s="123" t="n"/>
       <c r="V26" s="123" t="n"/>
@@ -2499,25 +2499,25 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>63.6672325976231</v>
+        <v>84.88964346349746</v>
       </c>
       <c r="N27" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-63.6672325976231</v>
+        <v>-84.88964346349746</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>238.0952380952381</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>238.0952380952381</v>
+        <v>476.1904761904762</v>
       </c>
       <c r="R27" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-238.0952380952381</v>
+        <v>-476.1904761904762</v>
       </c>
       <c r="T27" s="118" t="n">
         <v>-1</v>
@@ -2570,25 +2570,25 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>43.01075268817205</v>
+        <v>57.34767025089606</v>
       </c>
       <c r="N28" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-43.01075268817205</v>
+        <v>-57.34767025089606</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>190.4761904761905</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>190.4761904761905</v>
+        <v>380.952380952381</v>
       </c>
       <c r="R28" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-190.4761904761905</v>
+        <v>-380.952380952381</v>
       </c>
       <c r="T28" s="118" t="n">
         <v>-1</v>
@@ -2641,25 +2641,25 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>24.19354838709678</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="N29" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>-24.19354838709678</v>
+        <v>-32.25806451612903</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>95.23809523809524</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>95.23809523809524</v>
+        <v>190.4761904761905</v>
       </c>
       <c r="R29" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>-95.23809523809524</v>
+        <v>-190.4761904761905</v>
       </c>
       <c r="T29" s="118" t="n">
         <v>-1</v>
@@ -2700,25 +2700,25 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>130.8715336728919</v>
+        <v>174.4953782305226</v>
       </c>
       <c r="N30" s="125" t="n">
         <v>0</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-130.8715336728919</v>
+        <v>-174.4953782305226</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>523.8095238095239</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>523.8095238095239</v>
+        <v>1047.619047619048</v>
       </c>
       <c r="R30" s="123" t="n">
         <v>0</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>-523.8095238095239</v>
+        <v>-1047.619047619048</v>
       </c>
       <c r="T30" s="124" t="n">
         <v>-1</v>
@@ -2759,28 +2759,28 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="133" t="n">
-        <v>308.2958947989658</v>
+        <v>411.0611930652877</v>
       </c>
       <c r="N31" s="133" t="n">
         <v>0</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>-308.2958947989658</v>
+        <v>-411.0611930652877</v>
       </c>
       <c r="P31" s="131" t="n">
         <v>2201.228878648234</v>
       </c>
       <c r="Q31" s="131" t="n">
-        <v>5556.067588325653</v>
+        <v>7757.296466973886</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>3440.567278</v>
+        <v>4574.218414</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>-2115.500310325653</v>
+        <v>-3183.078052973886</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>-0.3807549632352778</v>
+        <v>-0.4103334282150495</v>
       </c>
       <c r="U31" s="131" t="n"/>
       <c r="V31" s="131" t="n"/>
@@ -3063,13 +3063,13 @@
         </is>
       </c>
       <c r="B2" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C2" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3106,16 +3106,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="137" t="n">
-        <v>919.3548387096772</v>
+        <v>1225.806451612903</v>
       </c>
       <c r="V2" s="137" t="n">
-        <v>786.210618</v>
+        <v>1058.588747</v>
       </c>
       <c r="W2" s="137" t="n">
-        <v>-133.1442207096774</v>
+        <v>-167.2177046129032</v>
       </c>
       <c r="X2" s="138" t="n">
-        <v>-0.1448235383157894</v>
+        <v>-0.136414443236842</v>
       </c>
       <c r="Y2" s="137" t="n"/>
       <c r="Z2" s="137" t="n"/>
@@ -3133,7 +3133,7 @@
       <c r="AD2" s="139" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_3</t>
+          <t>google:ok;google:includes_excel_row_3;crm:stale</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -3149,13 +3149,13 @@
         </is>
       </c>
       <c r="B3" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C3" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3200,7 +3200,7 @@
       <c r="AD3" s="139" t="inlineStr"/>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_2</t>
+          <t>google:rolled_up_to_excel_row_2;crm:stale</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -3216,13 +3216,13 @@
         </is>
       </c>
       <c r="B4" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C4" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3259,16 +3259,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="137" t="n">
-        <v>145.1612903225807</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="V4" s="137" t="n">
-        <v>95.516713</v>
+        <v>127.524928</v>
       </c>
       <c r="W4" s="137" t="n">
-        <v>-49.64457732258067</v>
+        <v>-66.0234590967742</v>
       </c>
       <c r="X4" s="138" t="n">
-        <v>-0.3419959771111112</v>
+        <v>-0.3411212053333333</v>
       </c>
       <c r="Y4" s="137" t="n"/>
       <c r="Z4" s="137" t="n"/>
@@ -3286,7 +3286,7 @@
       <c r="AD4" s="139" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_5</t>
+          <t>google:ok;google:includes_excel_row_5;crm:stale</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -3302,13 +3302,13 @@
         </is>
       </c>
       <c r="B5" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C5" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3353,7 +3353,7 @@
       <c r="AD5" s="139" t="inlineStr"/>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_4</t>
+          <t>google:rolled_up_to_excel_row_4;crm:stale</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -3369,13 +3369,13 @@
         </is>
       </c>
       <c r="B6" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C6" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3412,16 +3412,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="137" t="n">
-        <v>967.741935483871</v>
+        <v>1290.322580645161</v>
       </c>
       <c r="V6" s="137" t="n">
-        <v>866.5700000000001</v>
+        <v>1157.8</v>
       </c>
       <c r="W6" s="137" t="n">
-        <v>-101.1719354838709</v>
+        <v>-132.5225806451613</v>
       </c>
       <c r="X6" s="138" t="n">
-        <v>-0.1045443333333333</v>
+        <v>-0.1027049999999999</v>
       </c>
       <c r="Y6" s="137" t="n"/>
       <c r="Z6" s="137" t="n"/>
@@ -3439,7 +3439,7 @@
       <c r="AD6" s="139" t="inlineStr"/>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -3455,13 +3455,13 @@
         </is>
       </c>
       <c r="B7" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C7" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -3508,25 +3508,25 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>63.6672325976231</v>
+        <v>84.88964346349746</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>-63.6672325976231</v>
+        <v>-84.88964346349746</v>
       </c>
       <c r="T7" s="137" t="n">
         <v>238.0952380952381</v>
       </c>
       <c r="U7" s="137" t="n">
-        <v>238.0952380952381</v>
+        <v>476.1904761904762</v>
       </c>
       <c r="V7" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W7" s="137" t="n">
-        <v>-238.0952380952381</v>
+        <v>-476.1904761904762</v>
       </c>
       <c r="X7" s="138" t="n">
         <v>-1</v>
@@ -3538,7 +3538,7 @@
       <c r="AD7" s="139" t="inlineStr"/>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -3554,13 +3554,13 @@
         </is>
       </c>
       <c r="B8" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C8" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E8" t="n">
         <v>26</v>
@@ -3607,25 +3607,25 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>43.01075268817205</v>
+        <v>57.34767025089606</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>-43.01075268817205</v>
+        <v>-57.34767025089606</v>
       </c>
       <c r="T8" s="137" t="n">
         <v>190.4761904761905</v>
       </c>
       <c r="U8" s="137" t="n">
-        <v>190.4761904761905</v>
+        <v>380.952380952381</v>
       </c>
       <c r="V8" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W8" s="137" t="n">
-        <v>-190.4761904761905</v>
+        <v>-380.952380952381</v>
       </c>
       <c r="X8" s="138" t="n">
         <v>-1</v>
@@ -3637,7 +3637,7 @@
       <c r="AD8" s="139" t="inlineStr"/>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -3653,13 +3653,13 @@
         </is>
       </c>
       <c r="B9" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C9" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3706,25 +3706,25 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>24.19354838709678</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>-24.19354838709678</v>
+        <v>-32.25806451612903</v>
       </c>
       <c r="T9" s="137" t="n">
         <v>95.23809523809524</v>
       </c>
       <c r="U9" s="137" t="n">
-        <v>95.23809523809524</v>
+        <v>190.4761904761905</v>
       </c>
       <c r="V9" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W9" s="137" t="n">
-        <v>-95.23809523809524</v>
+        <v>-190.4761904761905</v>
       </c>
       <c r="X9" s="138" t="n">
         <v>-1</v>
@@ -3736,7 +3736,7 @@
       <c r="AD9" s="139" t="inlineStr"/>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -3752,13 +3752,13 @@
         </is>
       </c>
       <c r="B10" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C10" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3805,28 +3805,28 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>11.38519924098672</v>
+        <v>15.18026565464896</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>-11.38519924098672</v>
+        <v>-15.18026565464896</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U10" s="137" t="n">
-        <v>387.0967741935484</v>
+        <v>516.1290322580645</v>
       </c>
       <c r="V10" s="137" t="n">
-        <v>313.871355</v>
+        <v>416.563481</v>
       </c>
       <c r="W10" s="137" t="n">
-        <v>-73.22541919354842</v>
+        <v>-99.56555125806447</v>
       </c>
       <c r="X10" s="138" t="n">
-        <v>-0.18916566625</v>
+        <v>-0.1929082555624999</v>
       </c>
       <c r="Y10" s="137" t="n"/>
       <c r="Z10" s="137" t="n"/>
@@ -3844,7 +3844,7 @@
       <c r="AD10" s="139" t="inlineStr"/>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -3860,13 +3860,13 @@
         </is>
       </c>
       <c r="B11" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C11" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3913,28 +3913,28 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q11" t="n">
-        <v>22.62253875157101</v>
+        <v>30.16338500209468</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>-22.62253875157101</v>
+        <v>-30.16338500209468</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U11" s="137" t="n">
-        <v>870.9677419354839</v>
+        <v>1161.290322580645</v>
       </c>
       <c r="V11" s="137" t="n">
-        <v>418.97482</v>
+        <v>556.533175</v>
       </c>
       <c r="W11" s="137" t="n">
-        <v>-451.9929219354839</v>
+        <v>-604.7571475806451</v>
       </c>
       <c r="X11" s="138" t="n">
-        <v>-0.5189548362962962</v>
+        <v>-0.5207630993055555</v>
       </c>
       <c r="Y11" s="137" t="n"/>
       <c r="Z11" s="137" t="n"/>
@@ -3952,7 +3952,7 @@
       <c r="AD11" s="139" t="inlineStr"/>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_10;crm_metrics_combined_with_excel_row_10</t>
+          <t>google:ok;google:includes_excel_row_10;crm_metrics_combined_with_excel_row_10;crm:stale</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -3968,13 +3968,13 @@
         </is>
       </c>
       <c r="B12" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C12" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -4022,7 +4022,7 @@
       <c r="AD12" s="139" t="inlineStr"/>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_9</t>
+          <t>google:rolled_up_to_excel_row_9;crm:stale</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B13" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C13" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4091,28 +4091,28 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>2.546689303904923</v>
+        <v>3.395585738539898</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>-2.546689303904923</v>
+        <v>-3.395585738539898</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="137" t="n">
-        <v>96.7741935483871</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="V13" s="137" t="n">
-        <v>49.638146</v>
+        <v>68.008146</v>
       </c>
       <c r="W13" s="137" t="n">
-        <v>-47.1360475483871</v>
+        <v>-61.02411206451613</v>
       </c>
       <c r="X13" s="138" t="n">
-        <v>-0.4870724913333333</v>
+        <v>-0.4729368685</v>
       </c>
       <c r="Y13" s="137" t="n"/>
       <c r="Z13" s="137" t="n"/>
@@ -4130,7 +4130,7 @@
       <c r="AD13" s="139" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_12;crm_metrics_combined_with_excel_row_12</t>
+          <t>google:ok;google:includes_excel_row_12;crm_metrics_combined_with_excel_row_12;crm:stale</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -4146,13 +4146,13 @@
         </is>
       </c>
       <c r="B14" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C14" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
@@ -4200,7 +4200,7 @@
       <c r="AD14" s="139" t="inlineStr"/>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_11</t>
+          <t>google:rolled_up_to_excel_row_11;crm:stale</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -4216,13 +4216,13 @@
         </is>
       </c>
       <c r="B15" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C15" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -4269,25 +4269,25 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.3870967741935484</v>
+        <v>0.5161290322580645</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.3870967741935484</v>
+        <v>-0.5161290322580645</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U15" s="137" t="n">
-        <v>96.7741935483871</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="V15" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W15" s="137" t="n">
-        <v>-96.7741935483871</v>
+        <v>-129.0322580645161</v>
       </c>
       <c r="X15" s="138" t="n">
         <v>-1</v>
@@ -4308,7 +4308,7 @@
       <c r="AD15" s="139" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>google:ok;google:includes_excel_row_14;crm_metrics_combined_with_excel_row_14</t>
+          <t>google:ok;google:includes_excel_row_14;crm_metrics_combined_with_excel_row_14;crm:stale</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -4324,13 +4324,13 @@
         </is>
       </c>
       <c r="B16" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C16" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4378,7 +4378,7 @@
       <c r="AD16" s="139" t="inlineStr"/>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>google:rolled_up_to_excel_row_13</t>
+          <t>google:rolled_up_to_excel_row_13;crm:stale</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -4394,13 +4394,13 @@
         </is>
       </c>
       <c r="B17" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C17" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E17" t="n">
         <v>17</v>
@@ -4447,28 +4447,28 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>75.60483870967742</v>
+        <v>100.8064516129032</v>
       </c>
       <c r="R17" t="n">
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>-75.60483870967742</v>
+        <v>-100.8064516129032</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U17" s="137" t="n">
-        <v>967.741935483871</v>
+        <v>1290.322580645161</v>
       </c>
       <c r="V17" s="137" t="n">
-        <v>548.63</v>
+        <v>717.78</v>
       </c>
       <c r="W17" s="137" t="n">
-        <v>-419.111935483871</v>
+        <v>-572.5425806451613</v>
       </c>
       <c r="X17" s="138" t="n">
-        <v>-0.4330823333333333</v>
+        <v>-0.4437205</v>
       </c>
       <c r="Y17" s="137" t="n"/>
       <c r="Z17" s="137" t="n"/>
@@ -4486,7 +4486,7 @@
       <c r="AD17" s="139" t="inlineStr"/>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
@@ -4502,13 +4502,13 @@
         </is>
       </c>
       <c r="B18" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C18" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4555,28 +4555,28 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>1.209677419354838</v>
+        <v>1.612903225806452</v>
       </c>
       <c r="R18" t="n">
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>-1.209677419354838</v>
+        <v>-1.612903225806452</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="137" t="n">
-        <v>48.38709677419355</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="V18" s="137" t="n">
-        <v>31.28</v>
+        <v>42.43</v>
       </c>
       <c r="W18" s="137" t="n">
-        <v>-17.10709677419355</v>
+        <v>-22.08612903225806</v>
       </c>
       <c r="X18" s="138" t="n">
-        <v>-0.3535466666666667</v>
+        <v>-0.342335</v>
       </c>
       <c r="Y18" s="137" t="n"/>
       <c r="Z18" s="137" t="n"/>
@@ -4589,7 +4589,7 @@
       <c r="AD18" s="139" t="inlineStr"/>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
@@ -4605,13 +4605,13 @@
         </is>
       </c>
       <c r="B19" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C19" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4658,28 +4658,28 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>1.075268817204301</v>
+        <v>1.433691756272401</v>
       </c>
       <c r="R19" t="n">
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>-1.075268817204301</v>
+        <v>-1.433691756272401</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="137" t="n">
-        <v>96.7741935483871</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="V19" s="137" t="n">
-        <v>31.97</v>
+        <v>39.57</v>
       </c>
       <c r="W19" s="137" t="n">
-        <v>-64.8041935483871</v>
+        <v>-89.46225806451613</v>
       </c>
       <c r="X19" s="138" t="n">
-        <v>-0.6696433333333334</v>
+        <v>-0.6933325</v>
       </c>
       <c r="Y19" s="137" t="n"/>
       <c r="Z19" s="137" t="n"/>
@@ -4692,7 +4692,7 @@
       <c r="AD19" s="139" t="inlineStr"/>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
@@ -4708,13 +4708,13 @@
         </is>
       </c>
       <c r="B20" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C20" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
@@ -4761,25 +4761,25 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.403225806451613</v>
+        <v>0.5376344086021506</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.403225806451613</v>
+        <v>-0.5376344086021506</v>
       </c>
       <c r="T20" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U20" s="137" t="n">
-        <v>48.38709677419355</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="V20" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W20" s="137" t="n">
-        <v>-48.38709677419355</v>
+        <v>-64.51612903225806</v>
       </c>
       <c r="X20" s="138" t="n">
         <v>-1</v>
@@ -4795,7 +4795,7 @@
       <c r="AD20" s="139" t="inlineStr"/>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>meta:no_delivery</t>
+          <t>meta:no_delivery;crm:stale</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr">
@@ -4811,13 +4811,13 @@
         </is>
       </c>
       <c r="B21" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C21" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D21" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4864,28 +4864,28 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>3.629032258064516</v>
+        <v>4.838709677419355</v>
       </c>
       <c r="R21" t="n">
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>-3.629032258064516</v>
+        <v>-4.838709677419355</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="137" t="n">
-        <v>145.1612903225807</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="V21" s="137" t="n">
         <v>9.625539</v>
       </c>
       <c r="W21" s="137" t="n">
-        <v>-135.5357513225807</v>
+        <v>-183.9228480967742</v>
       </c>
       <c r="X21" s="138" t="n">
-        <v>-0.9336907313333334</v>
+        <v>-0.9502680485</v>
       </c>
       <c r="Y21" s="137" t="n"/>
       <c r="Z21" s="137" t="n"/>
@@ -4898,7 +4898,7 @@
       <c r="AD21" s="139" t="inlineStr"/>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
@@ -4914,13 +4914,13 @@
         </is>
       </c>
       <c r="B22" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C22" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D22" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -4967,28 +4967,28 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>9.677419354838708</v>
+        <v>12.90322580645161</v>
       </c>
       <c r="R22" t="n">
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>-9.677419354838708</v>
+        <v>-12.90322580645161</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="137" t="n">
-        <v>145.1612903225807</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="V22" s="137" t="n">
-        <v>227.600087</v>
+        <v>282.294398</v>
       </c>
       <c r="W22" s="137" t="n">
-        <v>82.43879667741933</v>
+        <v>88.74601090322579</v>
       </c>
       <c r="X22" s="138" t="n">
-        <v>0.5679117104444442</v>
+        <v>0.4585210563333332</v>
       </c>
       <c r="Y22" s="137" t="n"/>
       <c r="Z22" s="137" t="n"/>
@@ -5006,7 +5006,7 @@
       <c r="AD22" s="139" t="inlineStr"/>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
@@ -5022,13 +5022,13 @@
         </is>
       </c>
       <c r="B23" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C23" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D23" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5075,25 +5075,25 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.722084367245658</v>
+        <v>4.962779156327543</v>
       </c>
       <c r="R23" t="n">
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>-3.722084367245658</v>
+        <v>-4.962779156327543</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="137" t="n">
-        <v>96.7741935483871</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="V23" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W23" s="137" t="n">
-        <v>-96.7741935483871</v>
+        <v>-129.0322580645161</v>
       </c>
       <c r="X23" s="138" t="n">
         <v>-1</v>
@@ -5109,7 +5109,7 @@
       <c r="AD23" s="139" t="inlineStr"/>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>meta:no_delivery</t>
+          <t>meta:no_delivery;crm:stale</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -5125,13 +5125,13 @@
         </is>
       </c>
       <c r="B24" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C24" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D24" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5168,7 +5168,7 @@
       <c r="T24" s="137" t="n"/>
       <c r="U24" s="137" t="n"/>
       <c r="V24" s="137" t="n">
-        <v>60.68</v>
+        <v>97.5</v>
       </c>
       <c r="W24" s="137" t="n"/>
       <c r="X24" s="138" t="n"/>
@@ -5183,7 +5183,7 @@
       <c r="AD24" s="139" t="inlineStr"/>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
@@ -5199,13 +5199,13 @@
         </is>
       </c>
       <c r="B25" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C25" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D25" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5234,28 +5234,28 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>45.16129032258065</v>
+        <v>60.21505376344086</v>
       </c>
       <c r="R25" t="n">
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>-45.16129032258065</v>
+        <v>-60.21505376344086</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="137" t="n">
-        <v>2032.258064516129</v>
+        <v>2709.677419354839</v>
       </c>
       <c r="V25" s="137" t="n">
-        <v>1748.297331</v>
+        <v>2343.913675</v>
       </c>
       <c r="W25" s="137" t="n">
-        <v>-283.960733516129</v>
+        <v>-365.7637443548388</v>
       </c>
       <c r="X25" s="138" t="n">
-        <v>-0.1397267101428571</v>
+        <v>-0.1349842389880952</v>
       </c>
       <c r="Y25" s="137" t="n"/>
       <c r="Z25" s="137" t="n"/>
@@ -5264,7 +5264,7 @@
       <c r="AD25" s="139" t="inlineStr"/>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5275,13 +5275,13 @@
         </is>
       </c>
       <c r="B26" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C26" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D26" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5315,28 +5315,28 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>132.2630708034933</v>
+        <v>176.3507610713243</v>
       </c>
       <c r="R26" t="n">
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>-132.2630708034933</v>
+        <v>-176.3507610713243</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="137" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="V26" s="137" t="n">
-        <v>1692.269947</v>
+        <v>2230.304739</v>
       </c>
       <c r="W26" s="137" t="n">
-        <v>-1307.730053</v>
+        <v>-1769.695261</v>
       </c>
       <c r="X26" s="138" t="n">
-        <v>-0.4359100176666666</v>
+        <v>-0.4424238152499999</v>
       </c>
       <c r="Y26" s="137" t="n"/>
       <c r="Z26" s="137" t="n"/>
@@ -5345,7 +5345,7 @@
       <c r="AD26" s="139" t="inlineStr"/>
       <c r="AE26" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5356,13 +5356,13 @@
         </is>
       </c>
       <c r="B27" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C27" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D27" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5396,25 +5396,25 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>130.8715336728919</v>
+        <v>174.4953782305226</v>
       </c>
       <c r="R27" t="n">
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>-130.8715336728919</v>
+        <v>-174.4953782305226</v>
       </c>
       <c r="T27" s="137" t="n">
         <v>523.8095238095239</v>
       </c>
       <c r="U27" s="137" t="n">
-        <v>523.8095238095239</v>
+        <v>1047.619047619048</v>
       </c>
       <c r="V27" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W27" s="137" t="n">
-        <v>-523.8095238095239</v>
+        <v>-1047.619047619048</v>
       </c>
       <c r="X27" s="138" t="n">
         <v>-1</v>
@@ -5426,7 +5426,7 @@
       <c r="AD27" s="139" t="inlineStr"/>
       <c r="AE27" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>success;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5437,13 +5437,13 @@
         </is>
       </c>
       <c r="B28" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="C28" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D28" s="136" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5477,28 +5477,28 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>308.2958947989658</v>
+        <v>411.0611930652877</v>
       </c>
       <c r="R28" t="n">
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>-308.2958947989658</v>
+        <v>-411.0611930652877</v>
       </c>
       <c r="T28" s="137" t="n">
         <v>2201.228878648234</v>
       </c>
       <c r="U28" s="137" t="n">
-        <v>5556.067588325653</v>
+        <v>7757.296466973886</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>3440.567278</v>
+        <v>4574.218414</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>-2115.500310325653</v>
+        <v>-3183.078052973886</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>-0.3807549632352778</v>
+        <v>-0.4103334282150495</v>
       </c>
       <c r="Y28" s="137" t="n"/>
       <c r="Z28" s="137" t="n"/>
@@ -5507,7 +5507,7 @@
       <c r="AD28" s="139" t="inlineStr"/>
       <c r="AE28" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -5603,7 +5603,7 @@
         </is>
       </c>
       <c r="B4" s="140" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5643,7 +5643,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5663,7 +5663,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46238.29189814815</v>
+        <v>46239.29190972223</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-06
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -878,7 +878,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 04/08/2026  |  Ultimo aggiornamento: 05/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 05/08/2026  |  Ultimo aggiornamento: 06/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1065,16 +1065,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>1225.806451612903</v>
+        <v>1532.258064516129</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>1058.588747</v>
+        <v>1321.187786</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>-167.2177046129032</v>
+        <v>-211.070278516129</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>-0.136414443236842</v>
+        <v>-0.1377511291368421</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1173,16 +1173,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>193.5483870967742</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>127.524928</v>
+        <v>159.499719</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-66.0234590967742</v>
+        <v>-82.43576487096774</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.3411212053333333</v>
+        <v>-0.3407344948</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1281,16 +1281,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>1290.322580645161</v>
+        <v>1612.903225806452</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>1157.8</v>
+        <v>1498.17</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-132.5225806451613</v>
+        <v>-114.7332258064514</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.1027049999999999</v>
+        <v>-0.0711345999999998</v>
       </c>
       <c r="U9" s="117" t="n"/>
       <c r="V9" s="117" t="n"/>
@@ -1328,28 +1328,28 @@
         <v>15.05376344086022</v>
       </c>
       <c r="M10" s="125" t="n">
-        <v>60.21505376344086</v>
+        <v>75.26881720430109</v>
       </c>
       <c r="N10" s="125" t="n">
         <v>0</v>
       </c>
       <c r="O10" s="125" t="n">
-        <v>-60.21505376344086</v>
+        <v>-75.26881720430109</v>
       </c>
       <c r="P10" s="123" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="Q10" s="123" t="n">
-        <v>2709.677419354839</v>
+        <v>3387.096774193548</v>
       </c>
       <c r="R10" s="123" t="n">
-        <v>2343.913675</v>
+        <v>2978.857505</v>
       </c>
       <c r="S10" s="123" t="n">
-        <v>-365.7637443548388</v>
+        <v>-408.2392691935484</v>
       </c>
       <c r="T10" s="124" t="n">
-        <v>-0.1349842389880952</v>
+        <v>-0.1205277842380952</v>
       </c>
       <c r="U10" s="123" t="n"/>
       <c r="V10" s="123" t="n"/>
@@ -1403,28 +1403,28 @@
         <v>3.795066413662239</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>15.18026565464896</v>
+        <v>18.9753320683112</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-15.18026565464896</v>
+        <v>-18.9753320683112</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>516.1290322580645</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>416.563481</v>
+        <v>522.312827</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>-99.56555125806447</v>
+        <v>-122.8484633225806</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>-0.1929082555624999</v>
+        <v>-0.19041511815</v>
       </c>
       <c r="U11" s="117" t="n"/>
       <c r="V11" s="117" t="n"/>
@@ -1482,28 +1482,28 @@
         <v>7.540846250523669</v>
       </c>
       <c r="M12" s="127" t="n">
-        <v>30.16338500209468</v>
+        <v>37.70423125261835</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O12" s="127" t="n">
-        <v>-30.16338500209468</v>
+        <v>-37.70423125261835</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>1161.290322580645</v>
+        <v>1451.612903225806</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>556.533175</v>
+        <v>692.909006</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-604.7571475806451</v>
+        <v>-758.7038972258064</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.5207630993055555</v>
+        <v>-0.5226626847555556</v>
       </c>
       <c r="U12" s="128" t="n"/>
       <c r="V12" s="128" t="n"/>
@@ -1608,28 +1608,28 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="M14" s="127" t="n">
-        <v>3.395585738539898</v>
+        <v>4.244482173174872</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O14" s="127" t="n">
-        <v>-3.395585738539898</v>
+        <v>-4.244482173174872</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>129.0322580645161</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>68.008146</v>
+        <v>84.108146</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-61.02411206451613</v>
+        <v>-77.18217658064515</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.4729368685</v>
+        <v>-0.4785294947999999</v>
       </c>
       <c r="U14" s="128" t="n"/>
       <c r="V14" s="128" t="n"/>
@@ -1734,25 +1734,25 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="M16" s="127" t="n">
-        <v>0.5161290322580645</v>
+        <v>0.6451612903225806</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O16" s="127" t="n">
-        <v>-0.5161290322580645</v>
+        <v>-0.6451612903225806</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>129.0322580645161</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="R16" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>-129.0322580645161</v>
+        <v>-161.2903225806452</v>
       </c>
       <c r="T16" s="118" t="n">
         <v>-1</v>
@@ -1860,28 +1860,28 @@
         <v>25.20161290322581</v>
       </c>
       <c r="M18" s="119" t="n">
-        <v>100.8064516129032</v>
+        <v>126.008064516129</v>
       </c>
       <c r="N18" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O18" s="119" t="n">
-        <v>-100.8064516129032</v>
+        <v>-126.008064516129</v>
       </c>
       <c r="P18" s="117" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="Q18" s="117" t="n">
-        <v>1290.322580645161</v>
+        <v>1612.903225806452</v>
       </c>
       <c r="R18" s="117" t="n">
-        <v>717.78</v>
+        <v>906.47</v>
       </c>
       <c r="S18" s="117" t="n">
-        <v>-572.5425806451613</v>
+        <v>-706.4332258064514</v>
       </c>
       <c r="T18" s="118" t="n">
-        <v>-0.4437205</v>
+        <v>-0.4379885999999999</v>
       </c>
       <c r="U18" s="117" t="n"/>
       <c r="V18" s="117" t="n"/>
@@ -1939,28 +1939,28 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>1.612903225806452</v>
+        <v>2.016129032258065</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-1.612903225806452</v>
+        <v>-2.016129032258065</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>64.51612903225806</v>
+        <v>80.64516129032258</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>42.43</v>
+        <v>51.35</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-22.08612903225806</v>
+        <v>-29.29516129032257</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.342335</v>
+        <v>-0.3632599999999999</v>
       </c>
       <c r="U19" s="117" t="n"/>
       <c r="V19" s="117" t="n"/>
@@ -2014,28 +2014,28 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>1.433691756272401</v>
+        <v>1.792114695340502</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-1.433691756272401</v>
+        <v>-1.792114695340502</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>129.0322580645161</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>39.57</v>
+        <v>47.84</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-89.46225806451613</v>
+        <v>-113.4503225806452</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.6933325</v>
+        <v>-0.703392</v>
       </c>
       <c r="U20" s="117" t="n"/>
       <c r="V20" s="117" t="n"/>
@@ -2089,25 +2089,25 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>0.5376344086021506</v>
+        <v>0.6720430107526882</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-0.5376344086021506</v>
+        <v>-0.6720430107526882</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>64.51612903225806</v>
+        <v>80.64516129032258</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-64.51612903225806</v>
+        <v>-80.64516129032258</v>
       </c>
       <c r="T21" s="118" t="n">
         <v>-1</v>
@@ -2164,28 +2164,28 @@
         <v>1.209677419354839</v>
       </c>
       <c r="M22" s="119" t="n">
-        <v>4.838709677419355</v>
+        <v>6.048387096774194</v>
       </c>
       <c r="N22" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O22" s="119" t="n">
-        <v>-4.838709677419355</v>
+        <v>-6.048387096774194</v>
       </c>
       <c r="P22" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q22" s="117" t="n">
-        <v>193.5483870967742</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="R22" s="117" t="n">
         <v>9.625539</v>
       </c>
       <c r="S22" s="117" t="n">
-        <v>-183.9228480967742</v>
+        <v>-232.3099448709677</v>
       </c>
       <c r="T22" s="118" t="n">
-        <v>-0.9502680485</v>
+        <v>-0.9602144388</v>
       </c>
       <c r="U22" s="117" t="n"/>
       <c r="V22" s="117" t="n"/>
@@ -2239,28 +2239,28 @@
         <v>3.225806451612903</v>
       </c>
       <c r="M23" s="119" t="n">
-        <v>12.90322580645161</v>
+        <v>16.12903225806452</v>
       </c>
       <c r="N23" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O23" s="119" t="n">
-        <v>-12.90322580645161</v>
+        <v>-16.12903225806452</v>
       </c>
       <c r="P23" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q23" s="117" t="n">
-        <v>193.5483870967742</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="R23" s="117" t="n">
-        <v>282.294398</v>
+        <v>357.215867</v>
       </c>
       <c r="S23" s="117" t="n">
-        <v>88.74601090322579</v>
+        <v>115.2803831290323</v>
       </c>
       <c r="T23" s="118" t="n">
-        <v>0.4585210563333332</v>
+        <v>0.4764922502666667</v>
       </c>
       <c r="U23" s="117" t="n"/>
       <c r="V23" s="117" t="n"/>
@@ -2318,25 +2318,25 @@
         <v>1.240694789081886</v>
       </c>
       <c r="M24" s="119" t="n">
-        <v>4.962779156327543</v>
+        <v>6.203473945409429</v>
       </c>
       <c r="N24" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O24" s="119" t="n">
-        <v>-4.962779156327543</v>
+        <v>-6.203473945409429</v>
       </c>
       <c r="P24" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q24" s="117" t="n">
-        <v>129.0322580645161</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="R24" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S24" s="117" t="n">
-        <v>-129.0322580645161</v>
+        <v>-161.2903225806452</v>
       </c>
       <c r="T24" s="118" t="n">
         <v>-1</v>
@@ -2388,7 +2388,7 @@
       <c r="P25" s="117" t="n"/>
       <c r="Q25" s="117" t="n"/>
       <c r="R25" s="117" t="n">
-        <v>97.5</v>
+        <v>127.47</v>
       </c>
       <c r="S25" s="117" t="n"/>
       <c r="T25" s="118" t="n"/>
@@ -2428,28 +2428,28 @@
         <v>44.08769026783109</v>
       </c>
       <c r="M26" s="125" t="n">
-        <v>176.3507610713243</v>
+        <v>220.4384513391554</v>
       </c>
       <c r="N26" s="125" t="n">
         <v>0</v>
       </c>
       <c r="O26" s="125" t="n">
-        <v>-176.3507610713243</v>
+        <v>-220.4384513391554</v>
       </c>
       <c r="P26" s="123" t="n">
         <v>1000</v>
       </c>
       <c r="Q26" s="123" t="n">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="R26" s="123" t="n">
-        <v>2230.304739</v>
+        <v>2799.301385</v>
       </c>
       <c r="S26" s="123" t="n">
-        <v>-1769.695261</v>
+        <v>-2200.698615</v>
       </c>
       <c r="T26" s="124" t="n">
-        <v>-0.4424238152499999</v>
+        <v>-0.440139723</v>
       </c>
       <c r="U26" s="123" t="n"/>
       <c r="V26" s="123" t="n"/>
@@ -2499,25 +2499,25 @@
         <v>21.22241086587437</v>
       </c>
       <c r="M27" s="119" t="n">
-        <v>84.88964346349746</v>
+        <v>106.1120543293718</v>
       </c>
       <c r="N27" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O27" s="119" t="n">
-        <v>-84.88964346349746</v>
+        <v>-106.1120543293718</v>
       </c>
       <c r="P27" s="117" t="n">
         <v>238.0952380952381</v>
       </c>
       <c r="Q27" s="117" t="n">
-        <v>476.1904761904762</v>
+        <v>714.2857142857143</v>
       </c>
       <c r="R27" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S27" s="117" t="n">
-        <v>-476.1904761904762</v>
+        <v>-714.2857142857143</v>
       </c>
       <c r="T27" s="118" t="n">
         <v>-1</v>
@@ -2570,25 +2570,25 @@
         <v>14.33691756272402</v>
       </c>
       <c r="M28" s="119" t="n">
-        <v>57.34767025089606</v>
+        <v>71.68458781362007</v>
       </c>
       <c r="N28" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O28" s="119" t="n">
-        <v>-57.34767025089606</v>
+        <v>-71.68458781362007</v>
       </c>
       <c r="P28" s="117" t="n">
         <v>190.4761904761905</v>
       </c>
       <c r="Q28" s="117" t="n">
-        <v>380.952380952381</v>
+        <v>571.4285714285714</v>
       </c>
       <c r="R28" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S28" s="117" t="n">
-        <v>-380.952380952381</v>
+        <v>-571.4285714285714</v>
       </c>
       <c r="T28" s="118" t="n">
         <v>-1</v>
@@ -2641,25 +2641,25 @@
         <v>8.064516129032258</v>
       </c>
       <c r="M29" s="119" t="n">
-        <v>32.25806451612903</v>
+        <v>40.32258064516129</v>
       </c>
       <c r="N29" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O29" s="119" t="n">
-        <v>-32.25806451612903</v>
+        <v>-40.32258064516129</v>
       </c>
       <c r="P29" s="117" t="n">
         <v>95.23809523809524</v>
       </c>
       <c r="Q29" s="117" t="n">
-        <v>190.4761904761905</v>
+        <v>285.7142857142857</v>
       </c>
       <c r="R29" s="117" t="n">
         <v>0</v>
       </c>
       <c r="S29" s="117" t="n">
-        <v>-190.4761904761905</v>
+        <v>-285.7142857142857</v>
       </c>
       <c r="T29" s="118" t="n">
         <v>-1</v>
@@ -2700,25 +2700,25 @@
         <v>43.62384455763064</v>
       </c>
       <c r="M30" s="125" t="n">
-        <v>174.4953782305226</v>
+        <v>218.1192227881532</v>
       </c>
       <c r="N30" s="125" t="n">
         <v>0</v>
       </c>
       <c r="O30" s="125" t="n">
-        <v>-174.4953782305226</v>
+        <v>-218.1192227881532</v>
       </c>
       <c r="P30" s="123" t="n">
         <v>523.8095238095239</v>
       </c>
       <c r="Q30" s="123" t="n">
-        <v>1047.619047619048</v>
+        <v>1571.428571428572</v>
       </c>
       <c r="R30" s="123" t="n">
         <v>0</v>
       </c>
       <c r="S30" s="123" t="n">
-        <v>-1047.619047619048</v>
+        <v>-1571.428571428572</v>
       </c>
       <c r="T30" s="124" t="n">
         <v>-1</v>
@@ -2759,28 +2759,28 @@
         <v>102.7652982663219</v>
       </c>
       <c r="M31" s="133" t="n">
-        <v>411.0611930652877</v>
+        <v>513.8264913316098</v>
       </c>
       <c r="N31" s="133" t="n">
         <v>0</v>
       </c>
       <c r="O31" s="133" t="n">
-        <v>-411.0611930652877</v>
+        <v>-513.8264913316098</v>
       </c>
       <c r="P31" s="131" t="n">
         <v>2201.228878648234</v>
       </c>
       <c r="Q31" s="131" t="n">
-        <v>7757.296466973886</v>
+        <v>9958.52534562212</v>
       </c>
       <c r="R31" s="131" t="n">
-        <v>4574.218414</v>
+        <v>5778.15889</v>
       </c>
       <c r="S31" s="131" t="n">
-        <v>-3183.078052973886</v>
+        <v>-4180.36645562212</v>
       </c>
       <c r="T31" s="132" t="n">
-        <v>-0.4103334282150495</v>
+        <v>-0.4197776588940305</v>
       </c>
       <c r="U31" s="131" t="n"/>
       <c r="V31" s="131" t="n"/>
@@ -3063,13 +3063,13 @@
         </is>
       </c>
       <c r="B2" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C2" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -3106,16 +3106,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U2" s="137" t="n">
-        <v>1225.806451612903</v>
+        <v>1532.258064516129</v>
       </c>
       <c r="V2" s="137" t="n">
-        <v>1058.588747</v>
+        <v>1321.187786</v>
       </c>
       <c r="W2" s="137" t="n">
-        <v>-167.2177046129032</v>
+        <v>-211.070278516129</v>
       </c>
       <c r="X2" s="138" t="n">
-        <v>-0.136414443236842</v>
+        <v>-0.1377511291368421</v>
       </c>
       <c r="Y2" s="137" t="n"/>
       <c r="Z2" s="137" t="n"/>
@@ -3149,13 +3149,13 @@
         </is>
       </c>
       <c r="B3" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C3" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -3216,13 +3216,13 @@
         </is>
       </c>
       <c r="B4" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C4" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -3259,16 +3259,16 @@
         <v>48.38709677419355</v>
       </c>
       <c r="U4" s="137" t="n">
-        <v>193.5483870967742</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="V4" s="137" t="n">
-        <v>127.524928</v>
+        <v>159.499719</v>
       </c>
       <c r="W4" s="137" t="n">
-        <v>-66.0234590967742</v>
+        <v>-82.43576487096774</v>
       </c>
       <c r="X4" s="138" t="n">
-        <v>-0.3411212053333333</v>
+        <v>-0.3407344948</v>
       </c>
       <c r="Y4" s="137" t="n"/>
       <c r="Z4" s="137" t="n"/>
@@ -3302,13 +3302,13 @@
         </is>
       </c>
       <c r="B5" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C5" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -3369,13 +3369,13 @@
         </is>
       </c>
       <c r="B6" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C6" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
@@ -3412,16 +3412,16 @@
         <v>322.5806451612903</v>
       </c>
       <c r="U6" s="137" t="n">
-        <v>1290.322580645161</v>
+        <v>1612.903225806452</v>
       </c>
       <c r="V6" s="137" t="n">
-        <v>1157.8</v>
+        <v>1498.17</v>
       </c>
       <c r="W6" s="137" t="n">
-        <v>-132.5225806451613</v>
+        <v>-114.7332258064514</v>
       </c>
       <c r="X6" s="138" t="n">
-        <v>-0.1027049999999999</v>
+        <v>-0.0711345999999998</v>
       </c>
       <c r="Y6" s="137" t="n"/>
       <c r="Z6" s="137" t="n"/>
@@ -3455,13 +3455,13 @@
         </is>
       </c>
       <c r="B7" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C7" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E7" t="n">
         <v>25</v>
@@ -3508,25 +3508,25 @@
         <v>21.22241086587437</v>
       </c>
       <c r="Q7" t="n">
-        <v>84.88964346349746</v>
+        <v>106.1120543293718</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>-84.88964346349746</v>
+        <v>-106.1120543293718</v>
       </c>
       <c r="T7" s="137" t="n">
         <v>238.0952380952381</v>
       </c>
       <c r="U7" s="137" t="n">
-        <v>476.1904761904762</v>
+        <v>714.2857142857143</v>
       </c>
       <c r="V7" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W7" s="137" t="n">
-        <v>-476.1904761904762</v>
+        <v>-714.2857142857143</v>
       </c>
       <c r="X7" s="138" t="n">
         <v>-1</v>
@@ -3554,13 +3554,13 @@
         </is>
       </c>
       <c r="B8" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C8" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E8" t="n">
         <v>26</v>
@@ -3607,25 +3607,25 @@
         <v>14.33691756272402</v>
       </c>
       <c r="Q8" t="n">
-        <v>57.34767025089606</v>
+        <v>71.68458781362007</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>-57.34767025089606</v>
+        <v>-71.68458781362007</v>
       </c>
       <c r="T8" s="137" t="n">
         <v>190.4761904761905</v>
       </c>
       <c r="U8" s="137" t="n">
-        <v>380.952380952381</v>
+        <v>571.4285714285714</v>
       </c>
       <c r="V8" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W8" s="137" t="n">
-        <v>-380.952380952381</v>
+        <v>-571.4285714285714</v>
       </c>
       <c r="X8" s="138" t="n">
         <v>-1</v>
@@ -3653,13 +3653,13 @@
         </is>
       </c>
       <c r="B9" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C9" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E9" t="n">
         <v>27</v>
@@ -3706,25 +3706,25 @@
         <v>8.064516129032258</v>
       </c>
       <c r="Q9" t="n">
-        <v>32.25806451612903</v>
+        <v>40.32258064516129</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>-32.25806451612903</v>
+        <v>-40.32258064516129</v>
       </c>
       <c r="T9" s="137" t="n">
         <v>95.23809523809524</v>
       </c>
       <c r="U9" s="137" t="n">
-        <v>190.4761904761905</v>
+        <v>285.7142857142857</v>
       </c>
       <c r="V9" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W9" s="137" t="n">
-        <v>-190.4761904761905</v>
+        <v>-285.7142857142857</v>
       </c>
       <c r="X9" s="138" t="n">
         <v>-1</v>
@@ -3752,13 +3752,13 @@
         </is>
       </c>
       <c r="B10" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C10" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3805,28 +3805,28 @@
         <v>3.795066413662239</v>
       </c>
       <c r="Q10" t="n">
-        <v>15.18026565464896</v>
+        <v>18.9753320683112</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>-15.18026565464896</v>
+        <v>-18.9753320683112</v>
       </c>
       <c r="T10" s="137" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U10" s="137" t="n">
-        <v>516.1290322580645</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="V10" s="137" t="n">
-        <v>416.563481</v>
+        <v>522.312827</v>
       </c>
       <c r="W10" s="137" t="n">
-        <v>-99.56555125806447</v>
+        <v>-122.8484633225806</v>
       </c>
       <c r="X10" s="138" t="n">
-        <v>-0.1929082555624999</v>
+        <v>-0.19041511815</v>
       </c>
       <c r="Y10" s="137" t="n"/>
       <c r="Z10" s="137" t="n"/>
@@ -3860,13 +3860,13 @@
         </is>
       </c>
       <c r="B11" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C11" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3913,28 +3913,28 @@
         <v>7.540846250523669</v>
       </c>
       <c r="Q11" t="n">
-        <v>30.16338500209468</v>
+        <v>37.70423125261835</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>-30.16338500209468</v>
+        <v>-37.70423125261835</v>
       </c>
       <c r="T11" s="137" t="n">
         <v>290.3225806451613</v>
       </c>
       <c r="U11" s="137" t="n">
-        <v>1161.290322580645</v>
+        <v>1451.612903225806</v>
       </c>
       <c r="V11" s="137" t="n">
-        <v>556.533175</v>
+        <v>692.909006</v>
       </c>
       <c r="W11" s="137" t="n">
-        <v>-604.7571475806451</v>
+        <v>-758.7038972258064</v>
       </c>
       <c r="X11" s="138" t="n">
-        <v>-0.5207630993055555</v>
+        <v>-0.5226626847555556</v>
       </c>
       <c r="Y11" s="137" t="n"/>
       <c r="Z11" s="137" t="n"/>
@@ -3968,13 +3968,13 @@
         </is>
       </c>
       <c r="B12" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C12" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B13" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C13" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
@@ -4091,28 +4091,28 @@
         <v>0.8488964346349744</v>
       </c>
       <c r="Q13" t="n">
-        <v>3.395585738539898</v>
+        <v>4.244482173174872</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>-3.395585738539898</v>
+        <v>-4.244482173174872</v>
       </c>
       <c r="T13" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U13" s="137" t="n">
-        <v>129.0322580645161</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="V13" s="137" t="n">
-        <v>68.008146</v>
+        <v>84.108146</v>
       </c>
       <c r="W13" s="137" t="n">
-        <v>-61.02411206451613</v>
+        <v>-77.18217658064515</v>
       </c>
       <c r="X13" s="138" t="n">
-        <v>-0.4729368685</v>
+        <v>-0.4785294947999999</v>
       </c>
       <c r="Y13" s="137" t="n"/>
       <c r="Z13" s="137" t="n"/>
@@ -4146,13 +4146,13 @@
         </is>
       </c>
       <c r="B14" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C14" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
@@ -4216,13 +4216,13 @@
         </is>
       </c>
       <c r="B15" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C15" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E15" t="n">
         <v>13</v>
@@ -4269,25 +4269,25 @@
         <v>0.1290322580645161</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.5161290322580645</v>
+        <v>0.6451612903225806</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.5161290322580645</v>
+        <v>-0.6451612903225806</v>
       </c>
       <c r="T15" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U15" s="137" t="n">
-        <v>129.0322580645161</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="V15" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W15" s="137" t="n">
-        <v>-129.0322580645161</v>
+        <v>-161.2903225806452</v>
       </c>
       <c r="X15" s="138" t="n">
         <v>-1</v>
@@ -4324,13 +4324,13 @@
         </is>
       </c>
       <c r="B16" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C16" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4394,13 +4394,13 @@
         </is>
       </c>
       <c r="B17" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C17" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E17" t="n">
         <v>17</v>
@@ -4447,28 +4447,28 @@
         <v>25.20161290322581</v>
       </c>
       <c r="Q17" t="n">
-        <v>100.8064516129032</v>
+        <v>126.008064516129</v>
       </c>
       <c r="R17" t="n">
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>-100.8064516129032</v>
+        <v>-126.008064516129</v>
       </c>
       <c r="T17" s="137" t="n">
         <v>322.5806451612903</v>
       </c>
       <c r="U17" s="137" t="n">
-        <v>1290.322580645161</v>
+        <v>1612.903225806452</v>
       </c>
       <c r="V17" s="137" t="n">
-        <v>717.78</v>
+        <v>906.47</v>
       </c>
       <c r="W17" s="137" t="n">
-        <v>-572.5425806451613</v>
+        <v>-706.4332258064514</v>
       </c>
       <c r="X17" s="138" t="n">
-        <v>-0.4437205</v>
+        <v>-0.4379885999999999</v>
       </c>
       <c r="Y17" s="137" t="n"/>
       <c r="Z17" s="137" t="n"/>
@@ -4502,13 +4502,13 @@
         </is>
       </c>
       <c r="B18" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C18" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E18" t="n">
         <v>19</v>
@@ -4555,28 +4555,28 @@
         <v>0.4032258064516129</v>
       </c>
       <c r="Q18" t="n">
-        <v>1.612903225806452</v>
+        <v>2.016129032258065</v>
       </c>
       <c r="R18" t="n">
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>-1.612903225806452</v>
+        <v>-2.016129032258065</v>
       </c>
       <c r="T18" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U18" s="137" t="n">
-        <v>64.51612903225806</v>
+        <v>80.64516129032258</v>
       </c>
       <c r="V18" s="137" t="n">
-        <v>42.43</v>
+        <v>51.35</v>
       </c>
       <c r="W18" s="137" t="n">
-        <v>-22.08612903225806</v>
+        <v>-29.29516129032257</v>
       </c>
       <c r="X18" s="138" t="n">
-        <v>-0.342335</v>
+        <v>-0.3632599999999999</v>
       </c>
       <c r="Y18" s="137" t="n"/>
       <c r="Z18" s="137" t="n"/>
@@ -4605,13 +4605,13 @@
         </is>
       </c>
       <c r="B19" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C19" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E19" t="n">
         <v>20</v>
@@ -4658,28 +4658,28 @@
         <v>0.3584229390681003</v>
       </c>
       <c r="Q19" t="n">
-        <v>1.433691756272401</v>
+        <v>1.792114695340502</v>
       </c>
       <c r="R19" t="n">
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>-1.433691756272401</v>
+        <v>-1.792114695340502</v>
       </c>
       <c r="T19" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U19" s="137" t="n">
-        <v>129.0322580645161</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="V19" s="137" t="n">
-        <v>39.57</v>
+        <v>47.84</v>
       </c>
       <c r="W19" s="137" t="n">
-        <v>-89.46225806451613</v>
+        <v>-113.4503225806452</v>
       </c>
       <c r="X19" s="138" t="n">
-        <v>-0.6933325</v>
+        <v>-0.703392</v>
       </c>
       <c r="Y19" s="137" t="n"/>
       <c r="Z19" s="137" t="n"/>
@@ -4708,13 +4708,13 @@
         </is>
       </c>
       <c r="B20" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C20" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E20" t="n">
         <v>21</v>
@@ -4761,25 +4761,25 @@
         <v>0.1344086021505376</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.5376344086021506</v>
+        <v>0.6720430107526882</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.5376344086021506</v>
+        <v>-0.6720430107526882</v>
       </c>
       <c r="T20" s="137" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U20" s="137" t="n">
-        <v>64.51612903225806</v>
+        <v>80.64516129032258</v>
       </c>
       <c r="V20" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W20" s="137" t="n">
-        <v>-64.51612903225806</v>
+        <v>-80.64516129032258</v>
       </c>
       <c r="X20" s="138" t="n">
         <v>-1</v>
@@ -4811,13 +4811,13 @@
         </is>
       </c>
       <c r="B21" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C21" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D21" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E21" t="n">
         <v>15</v>
@@ -4864,28 +4864,28 @@
         <v>1.209677419354839</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.838709677419355</v>
+        <v>6.048387096774194</v>
       </c>
       <c r="R21" t="n">
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>-4.838709677419355</v>
+        <v>-6.048387096774194</v>
       </c>
       <c r="T21" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U21" s="137" t="n">
-        <v>193.5483870967742</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="V21" s="137" t="n">
         <v>9.625539</v>
       </c>
       <c r="W21" s="137" t="n">
-        <v>-183.9228480967742</v>
+        <v>-232.3099448709677</v>
       </c>
       <c r="X21" s="138" t="n">
-        <v>-0.9502680485</v>
+        <v>-0.9602144388</v>
       </c>
       <c r="Y21" s="137" t="n"/>
       <c r="Z21" s="137" t="n"/>
@@ -4914,13 +4914,13 @@
         </is>
       </c>
       <c r="B22" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C22" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D22" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E22" t="n">
         <v>16</v>
@@ -4967,28 +4967,28 @@
         <v>3.225806451612903</v>
       </c>
       <c r="Q22" t="n">
-        <v>12.90322580645161</v>
+        <v>16.12903225806452</v>
       </c>
       <c r="R22" t="n">
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>-12.90322580645161</v>
+        <v>-16.12903225806452</v>
       </c>
       <c r="T22" s="137" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U22" s="137" t="n">
-        <v>193.5483870967742</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="V22" s="137" t="n">
-        <v>282.294398</v>
+        <v>357.215867</v>
       </c>
       <c r="W22" s="137" t="n">
-        <v>88.74601090322579</v>
+        <v>115.2803831290323</v>
       </c>
       <c r="X22" s="138" t="n">
-        <v>0.4585210563333332</v>
+        <v>0.4764922502666667</v>
       </c>
       <c r="Y22" s="137" t="n"/>
       <c r="Z22" s="137" t="n"/>
@@ -5022,13 +5022,13 @@
         </is>
       </c>
       <c r="B23" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C23" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D23" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E23" t="n">
         <v>22</v>
@@ -5075,25 +5075,25 @@
         <v>1.240694789081886</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.962779156327543</v>
+        <v>6.203473945409429</v>
       </c>
       <c r="R23" t="n">
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>-4.962779156327543</v>
+        <v>-6.203473945409429</v>
       </c>
       <c r="T23" s="137" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U23" s="137" t="n">
-        <v>129.0322580645161</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="V23" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W23" s="137" t="n">
-        <v>-129.0322580645161</v>
+        <v>-161.2903225806452</v>
       </c>
       <c r="X23" s="138" t="n">
         <v>-1</v>
@@ -5125,13 +5125,13 @@
         </is>
       </c>
       <c r="B24" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C24" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D24" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="E24" t="n">
         <v>23</v>
@@ -5168,7 +5168,7 @@
       <c r="T24" s="137" t="n"/>
       <c r="U24" s="137" t="n"/>
       <c r="V24" s="137" t="n">
-        <v>97.5</v>
+        <v>127.47</v>
       </c>
       <c r="W24" s="137" t="n"/>
       <c r="X24" s="138" t="n"/>
@@ -5199,13 +5199,13 @@
         </is>
       </c>
       <c r="B25" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C25" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D25" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -5234,28 +5234,28 @@
         <v>15.05376344086022</v>
       </c>
       <c r="Q25" t="n">
-        <v>60.21505376344086</v>
+        <v>75.26881720430109</v>
       </c>
       <c r="R25" t="n">
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>-60.21505376344086</v>
+        <v>-75.26881720430109</v>
       </c>
       <c r="T25" s="137" t="n">
         <v>677.4193548387096</v>
       </c>
       <c r="U25" s="137" t="n">
-        <v>2709.677419354839</v>
+        <v>3387.096774193548</v>
       </c>
       <c r="V25" s="137" t="n">
-        <v>2343.913675</v>
+        <v>2978.857505</v>
       </c>
       <c r="W25" s="137" t="n">
-        <v>-365.7637443548388</v>
+        <v>-408.2392691935484</v>
       </c>
       <c r="X25" s="138" t="n">
-        <v>-0.1349842389880952</v>
+        <v>-0.1205277842380952</v>
       </c>
       <c r="Y25" s="137" t="n"/>
       <c r="Z25" s="137" t="n"/>
@@ -5275,13 +5275,13 @@
         </is>
       </c>
       <c r="B26" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C26" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D26" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -5315,28 +5315,28 @@
         <v>44.08769026783109</v>
       </c>
       <c r="Q26" t="n">
-        <v>176.3507610713243</v>
+        <v>220.4384513391554</v>
       </c>
       <c r="R26" t="n">
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>-176.3507610713243</v>
+        <v>-220.4384513391554</v>
       </c>
       <c r="T26" s="137" t="n">
         <v>1000</v>
       </c>
       <c r="U26" s="137" t="n">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="V26" s="137" t="n">
-        <v>2230.304739</v>
+        <v>2799.301385</v>
       </c>
       <c r="W26" s="137" t="n">
-        <v>-1769.695261</v>
+        <v>-2200.698615</v>
       </c>
       <c r="X26" s="138" t="n">
-        <v>-0.4424238152499999</v>
+        <v>-0.440139723</v>
       </c>
       <c r="Y26" s="137" t="n"/>
       <c r="Z26" s="137" t="n"/>
@@ -5356,13 +5356,13 @@
         </is>
       </c>
       <c r="B27" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C27" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D27" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -5396,25 +5396,25 @@
         <v>43.62384455763064</v>
       </c>
       <c r="Q27" t="n">
-        <v>174.4953782305226</v>
+        <v>218.1192227881532</v>
       </c>
       <c r="R27" t="n">
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>-174.4953782305226</v>
+        <v>-218.1192227881532</v>
       </c>
       <c r="T27" s="137" t="n">
         <v>523.8095238095239</v>
       </c>
       <c r="U27" s="137" t="n">
-        <v>1047.619047619048</v>
+        <v>1571.428571428572</v>
       </c>
       <c r="V27" s="137" t="n">
         <v>0</v>
       </c>
       <c r="W27" s="137" t="n">
-        <v>-1047.619047619048</v>
+        <v>-1571.428571428572</v>
       </c>
       <c r="X27" s="138" t="n">
         <v>-1</v>
@@ -5437,13 +5437,13 @@
         </is>
       </c>
       <c r="B28" s="136" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="C28" s="136" t="n">
         <v>46235</v>
       </c>
       <c r="D28" s="136" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -5477,28 +5477,28 @@
         <v>102.7652982663219</v>
       </c>
       <c r="Q28" t="n">
-        <v>411.0611930652877</v>
+        <v>513.8264913316098</v>
       </c>
       <c r="R28" t="n">
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>-411.0611930652877</v>
+        <v>-513.8264913316098</v>
       </c>
       <c r="T28" s="137" t="n">
         <v>2201.228878648234</v>
       </c>
       <c r="U28" s="137" t="n">
-        <v>7757.296466973886</v>
+        <v>9958.52534562212</v>
       </c>
       <c r="V28" s="137" t="n">
-        <v>4574.218414</v>
+        <v>5778.15889</v>
       </c>
       <c r="W28" s="137" t="n">
-        <v>-3183.078052973886</v>
+        <v>-4180.36645562212</v>
       </c>
       <c r="X28" s="138" t="n">
-        <v>-0.4103334282150495</v>
+        <v>-0.4197776588940305</v>
       </c>
       <c r="Y28" s="137" t="n"/>
       <c r="Z28" s="137" t="n"/>
@@ -5603,7 +5603,7 @@
         </is>
       </c>
       <c r="B4" s="140" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -5643,7 +5643,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -5663,7 +5663,7 @@
         </is>
       </c>
       <c r="B7" s="141" t="n">
-        <v>46239.29190972223</v>
+        <v>46240.29195601852</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Allinea metriche report agosto
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 06/08/2026  |  Ultimo aggiornamento: 07/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 06/08/2026  |  Ultimo aggiornamento: 07/08/2026 09:38</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1180,13 +1180,13 @@
         <v>1838.709677419354</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>1714.36</v>
+        <v>1714.59</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-124.3496774193548</v>
+        <v>-124.1196774193547</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0676287719298245</v>
+        <v>-0.0675036842105262</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1208,8 +1208,12 @@
       <c r="G8" s="124" t="n">
         <v>0.4302325581395348</v>
       </c>
-      <c r="H8" s="123" t="n"/>
-      <c r="I8" s="125" t="n"/>
+      <c r="H8" s="123" t="n">
+        <v>418</v>
+      </c>
+      <c r="I8" s="125" t="n">
+        <v>44</v>
+      </c>
       <c r="J8" s="123" t="n">
         <v>43</v>
       </c>
@@ -1235,13 +1239,13 @@
         <v>3580.645161290322</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>3476.533471</v>
+        <v>3476.763471</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-104.1116902903223</v>
+        <v>-103.8816902903222</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0290762378288287</v>
+        <v>-0.0290120035945945</v>
       </c>
       <c r="U8" s="123" t="n"/>
       <c r="V8" s="123" t="n"/>
@@ -1610,13 +1614,13 @@
         <v>1064.516129032258</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>1095.83</v>
+        <v>1095.97</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>31.31387096774188</v>
+        <v>31.45387096774198</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.0294160606060605</v>
+        <v>0.0295475757575757</v>
       </c>
       <c r="U13" s="117" t="n"/>
       <c r="V13" s="117" t="n"/>
@@ -1685,13 +1689,13 @@
         <v>96.7741935483871</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>60.08</v>
+        <v>60.15</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-36.69419354838711</v>
+        <v>-36.62419354838711</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3791733333333334</v>
+        <v>-0.37845</v>
       </c>
       <c r="U14" s="117" t="n"/>
       <c r="V14" s="117" t="n"/>
@@ -1758,13 +1762,13 @@
         <v>96.7741935483871</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>58.09</v>
+        <v>58.1</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-38.6841935483871</v>
+        <v>-38.6741935483871</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3997366666666667</v>
+        <v>-0.3996333333333333</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1904,13 +1908,13 @@
         <v>193.5483870967742</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>159.21</v>
+        <v>159.25</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-34.3383870967742</v>
+        <v>-34.29838709677421</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.177415</v>
+        <v>-0.1772083333333333</v>
       </c>
       <c r="U17" s="117" t="n"/>
       <c r="V17" s="117" t="n"/>
@@ -1933,7 +1937,7 @@
         <v>0.3720930232558139</v>
       </c>
       <c r="H18" s="123" t="n">
-        <v>679.4055201698513</v>
+        <v>850</v>
       </c>
       <c r="I18" s="125" t="n">
         <v>23.55</v>
@@ -1942,7 +1946,7 @@
         <v>24.0766566765155</v>
       </c>
       <c r="K18" s="125" t="n">
-        <v>664.5440940978523</v>
+        <v>664.5440940978524</v>
       </c>
       <c r="L18" s="125" t="n">
         <v>21.43690626122104</v>
@@ -1963,13 +1967,13 @@
         <v>3096.774193548388</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>3286.11938</v>
+        <v>3286.37938</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>189.3451864516128</v>
+        <v>189.6051864516125</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>0.0611427164583332</v>
+        <v>0.0612266747916665</v>
       </c>
       <c r="U18" s="123" t="n"/>
       <c r="V18" s="123" t="n"/>
@@ -2264,10 +2268,10 @@
         <v>1</v>
       </c>
       <c r="H23" s="129" t="n">
-        <v>1010.575793184489</v>
+        <v>496.8226458694397</v>
       </c>
       <c r="I23" s="131" t="n">
-        <v>42.55</v>
+        <v>86.55</v>
       </c>
       <c r="J23" s="129" t="n">
         <v>20.04460858903758</v>
@@ -2294,13 +2298,13 @@
         <v>8296.466973886329</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>6762.652851</v>
+        <v>6763.142851</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-1533.814122886329</v>
+        <v>-1533.324122886329</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1848755774854656</v>
+        <v>-0.1848165162005184</v>
       </c>
       <c r="U23" s="129" t="n"/>
       <c r="V23" s="129" t="n"/>
@@ -2781,13 +2785,13 @@
         <v>1838.709677419354</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>1714.36</v>
+        <v>1714.59</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-124.3496774193548</v>
+        <v>-124.1196774193547</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0676287719298245</v>
+        <v>-0.0675036842105262</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -3593,13 +3597,13 @@
         <v>1064.516129032258</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>1095.83</v>
+        <v>1095.97</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>31.31387096774188</v>
+        <v>31.45387096774198</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.0294160606060605</v>
+        <v>0.0295475757575757</v>
       </c>
       <c r="Y12" s="135" t="n"/>
       <c r="Z12" s="135" t="n"/>
@@ -3696,13 +3700,13 @@
         <v>96.7741935483871</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>60.08</v>
+        <v>60.15</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-36.69419354838711</v>
+        <v>-36.62419354838711</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3791733333333334</v>
+        <v>-0.37845</v>
       </c>
       <c r="Y13" s="135" t="n"/>
       <c r="Z13" s="135" t="n"/>
@@ -3796,13 +3800,13 @@
         <v>96.7741935483871</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>58.09</v>
+        <v>58.1</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-38.6841935483871</v>
+        <v>-38.6741935483871</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3997366666666667</v>
+        <v>-0.3996333333333333</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3997,13 +4001,13 @@
         <v>193.5483870967742</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>159.21</v>
+        <v>159.25</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-34.3383870967742</v>
+        <v>-34.29838709677421</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.177415</v>
+        <v>-0.1772083333333333</v>
       </c>
       <c r="Y16" s="135" t="n"/>
       <c r="Z16" s="135" t="n"/>
@@ -4056,7 +4060,12 @@
       <c r="K17" s="136" t="n">
         <v>0.4302325581395348</v>
       </c>
-      <c r="L17" s="135" t="n"/>
+      <c r="L17" s="135" t="n">
+        <v>418</v>
+      </c>
+      <c r="M17" t="n">
+        <v>44</v>
+      </c>
       <c r="N17" s="135" t="n">
         <v>43</v>
       </c>
@@ -4082,13 +4091,13 @@
         <v>3580.645161290322</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>3476.533471</v>
+        <v>3476.763471</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-104.1116902903223</v>
+        <v>-103.8816902903222</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0290762378288287</v>
+        <v>-0.0290120035945945</v>
       </c>
       <c r="Y17" s="135" t="n"/>
       <c r="Z17" s="135" t="n"/>
@@ -4133,7 +4142,7 @@
         <v>0.3720930232558139</v>
       </c>
       <c r="L18" s="135" t="n">
-        <v>679.4055201698513</v>
+        <v>850</v>
       </c>
       <c r="M18" t="n">
         <v>23.55</v>
@@ -4142,7 +4151,7 @@
         <v>24.0766566765155</v>
       </c>
       <c r="O18" t="n">
-        <v>664.5440940978523</v>
+        <v>664.5440940978524</v>
       </c>
       <c r="P18" t="n">
         <v>21.43690626122104</v>
@@ -4163,13 +4172,13 @@
         <v>3096.774193548388</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>3286.11938</v>
+        <v>3286.37938</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>189.3451864516128</v>
+        <v>189.6051864516125</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>0.0611427164583332</v>
+        <v>0.0612266747916665</v>
       </c>
       <c r="Y18" s="135" t="n"/>
       <c r="Z18" s="135" t="n"/>
@@ -4295,10 +4304,10 @@
         <v>1</v>
       </c>
       <c r="L20" s="135" t="n">
-        <v>1010.575793184489</v>
+        <v>496.8226458694397</v>
       </c>
       <c r="M20" t="n">
-        <v>42.55</v>
+        <v>86.55</v>
       </c>
       <c r="N20" s="135" t="n">
         <v>20.04460858903758</v>
@@ -4325,13 +4334,13 @@
         <v>8296.466973886329</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>6762.652851</v>
+        <v>6763.142851</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-1533.814122886329</v>
+        <v>-1533.324122886329</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1848755774854656</v>
+        <v>-0.1848165162005184</v>
       </c>
       <c r="Y20" s="135" t="n"/>
       <c r="Z20" s="135" t="n"/>
@@ -4496,7 +4505,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46241.29204861111</v>
+        <v>46241.40172453703</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Apply Italian holiday-aware DEM pacing
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 06/08/2026  |  Ultimo aggiornamento: 07/08/2026 09:38</t>
+          <t>Periodo: 01/08/2026 - 06/08/2026  |  Ultimo aggiornamento: 07/08/2026 10:31</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1180,13 +1180,13 @@
         <v>1838.709677419354</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>1714.59</v>
+        <v>1714.66</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-124.1196774193547</v>
+        <v>-124.0496774193546</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0675036842105262</v>
+        <v>-0.0674656140350875</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1239,13 +1239,13 @@
         <v>3580.645161290322</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>3476.763471</v>
+        <v>3476.833471</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-103.8816902903222</v>
+        <v>-103.8116902903221</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0290120035945945</v>
+        <v>-0.0289924540450449</v>
       </c>
       <c r="U8" s="123" t="n"/>
       <c r="V8" s="123" t="n"/>
@@ -1614,13 +1614,13 @@
         <v>1064.516129032258</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>1095.97</v>
+        <v>1096.05</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>31.45387096774198</v>
+        <v>31.5338709677419</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.0295475757575757</v>
+        <v>0.0296227272727272</v>
       </c>
       <c r="U13" s="117" t="n"/>
       <c r="V13" s="117" t="n"/>
@@ -1967,13 +1967,13 @@
         <v>3096.774193548388</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>3286.37938</v>
+        <v>3286.45938</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>189.6051864516125</v>
+        <v>189.6851864516125</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>0.0612266747916665</v>
+        <v>0.0612525081249998</v>
       </c>
       <c r="U18" s="123" t="n"/>
       <c r="V18" s="123" t="n"/>
@@ -2020,16 +2020,16 @@
         <v>592.1052631578948</v>
       </c>
       <c r="L19" s="119" t="n">
-        <v>19.10016977928693</v>
+        <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>114.6010186757216</v>
+        <v>112.7819548872181</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-114.6010186757216</v>
+        <v>-112.7819548872181</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
@@ -2091,16 +2091,16 @@
         <v>333.3333333333333</v>
       </c>
       <c r="L20" s="119" t="n">
-        <v>10.75268817204301</v>
+        <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>64.51612903225806</v>
+        <v>63.49206349206349</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-64.51612903225806</v>
+        <v>-63.49206349206349</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
@@ -2162,16 +2162,16 @@
         <v>125</v>
       </c>
       <c r="L21" s="119" t="n">
-        <v>4.032258064516129</v>
+        <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>24.19354838709678</v>
+        <v>23.80952380952381</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-24.19354838709678</v>
+        <v>-23.80952380952381</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
@@ -2221,16 +2221,16 @@
         <v>1050.438596491228</v>
       </c>
       <c r="L22" s="125" t="n">
-        <v>33.88511601584607</v>
+        <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>203.3106960950764</v>
+        <v>200.0835421888053</v>
       </c>
       <c r="N22" s="125" t="n">
         <v>0</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-203.3106960950764</v>
+        <v>-200.0835421888053</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
@@ -2280,16 +2280,16 @@
         <v>2145.215248728616</v>
       </c>
       <c r="L23" s="131" t="n">
-        <v>69.20049189447145</v>
+        <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>415.2029513668288</v>
+        <v>411.9757974605577</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>0</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-415.2029513668288</v>
+        <v>-411.9757974605577</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
@@ -2298,13 +2298,13 @@
         <v>8296.466973886329</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>6763.142851</v>
+        <v>6763.292851</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-1533.324122886329</v>
+        <v>-1533.174122886328</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1848165162005184</v>
+        <v>-0.1847984362153304</v>
       </c>
       <c r="U23" s="129" t="n"/>
       <c r="V23" s="129" t="n"/>
@@ -2785,13 +2785,13 @@
         <v>1838.709677419354</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>1714.59</v>
+        <v>1714.66</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-124.1196774193547</v>
+        <v>-124.0496774193546</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0675036842105262</v>
+        <v>-0.0674656140350875</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2870,16 +2870,16 @@
         <v>592.1052631578948</v>
       </c>
       <c r="P5" t="n">
-        <v>19.10016977928693</v>
+        <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>114.6010186757216</v>
+        <v>112.7819548872181</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>-114.6010186757216</v>
+        <v>-112.7819548872181</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
@@ -2969,16 +2969,16 @@
         <v>333.3333333333333</v>
       </c>
       <c r="P6" t="n">
-        <v>10.75268817204301</v>
+        <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>64.51612903225806</v>
+        <v>63.49206349206349</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>-64.51612903225806</v>
+        <v>-63.49206349206349</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
@@ -3068,16 +3068,16 @@
         <v>125</v>
       </c>
       <c r="P7" t="n">
-        <v>4.032258064516129</v>
+        <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>24.19354838709678</v>
+        <v>23.80952380952381</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>-24.19354838709678</v>
+        <v>-23.80952380952381</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
@@ -3597,13 +3597,13 @@
         <v>1064.516129032258</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>1095.97</v>
+        <v>1096.05</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>31.45387096774198</v>
+        <v>31.5338709677419</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.0295475757575757</v>
+        <v>0.0296227272727272</v>
       </c>
       <c r="Y12" s="135" t="n"/>
       <c r="Z12" s="135" t="n"/>
@@ -4091,13 +4091,13 @@
         <v>3580.645161290322</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>3476.763471</v>
+        <v>3476.833471</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-103.8816902903222</v>
+        <v>-103.8116902903221</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0290120035945945</v>
+        <v>-0.0289924540450449</v>
       </c>
       <c r="Y17" s="135" t="n"/>
       <c r="Z17" s="135" t="n"/>
@@ -4172,13 +4172,13 @@
         <v>3096.774193548388</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>3286.37938</v>
+        <v>3286.45938</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>189.6051864516125</v>
+        <v>189.6851864516125</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>0.0612266747916665</v>
+        <v>0.0612525081249998</v>
       </c>
       <c r="Y18" s="135" t="n"/>
       <c r="Z18" s="135" t="n"/>
@@ -4235,16 +4235,16 @@
         <v>1050.438596491228</v>
       </c>
       <c r="P19" t="n">
-        <v>33.88511601584607</v>
+        <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>203.3106960950764</v>
+        <v>200.0835421888053</v>
       </c>
       <c r="R19" t="n">
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>-203.3106960950764</v>
+        <v>-200.0835421888053</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
@@ -4316,16 +4316,16 @@
         <v>2145.215248728616</v>
       </c>
       <c r="P20" t="n">
-        <v>69.20049189447145</v>
+        <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>415.2029513668288</v>
+        <v>411.9757974605577</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>-415.2029513668288</v>
+        <v>-411.9757974605577</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
@@ -4334,13 +4334,13 @@
         <v>8296.466973886329</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>6763.142851</v>
+        <v>6763.292851</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-1533.324122886329</v>
+        <v>-1533.174122886328</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1848165162005184</v>
+        <v>-0.1847984362153304</v>
       </c>
       <c r="Y20" s="135" t="n"/>
       <c r="Z20" s="135" t="n"/>
@@ -4505,7 +4505,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46241.40172453703</v>
+        <v>46241.43869212963</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiorna lead CRM al 2026-08-06
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 06/08/2026  |  Ultimo aggiornamento: 07/08/2026 10:31</t>
+          <t>Periodo: 01/08/2026 - 06/08/2026  |  Ultimo aggiornamento: 07/08/2026 11:18</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1227,10 +1227,10 @@
         <v>83.27081770442611</v>
       </c>
       <c r="N8" s="125" t="n">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-83.27081770442611</v>
+        <v>28.72918229557389</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
@@ -1247,8 +1247,12 @@
       <c r="T8" s="124" t="n">
         <v>-0.0289924540450449</v>
       </c>
-      <c r="U8" s="123" t="n"/>
-      <c r="V8" s="123" t="n"/>
+      <c r="U8" s="123" t="n">
+        <v>31.04315599107144</v>
+      </c>
+      <c r="V8" s="123" t="n">
+        <v>-11.95684400892857</v>
+      </c>
       <c r="W8" s="126" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1" s="74">
@@ -1302,10 +1306,10 @@
         <v>12.48699271592091</v>
       </c>
       <c r="N9" s="119" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-12.48699271592091</v>
+        <v>9.513007284079086</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
@@ -1322,8 +1326,12 @@
       <c r="T9" s="118" t="n">
         <v>0.4844851812499998</v>
       </c>
-      <c r="U9" s="117" t="n"/>
-      <c r="V9" s="117" t="n"/>
+      <c r="U9" s="117" t="n">
+        <v>26.11997386363636</v>
+      </c>
+      <c r="V9" s="117" t="n">
+        <v>-4.88002613636364</v>
+      </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
     <row r="10" ht="36" customHeight="1" s="74">
@@ -1377,10 +1385,10 @@
         <v>20.92414995640802</v>
       </c>
       <c r="N10" s="119" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-20.92414995640802</v>
+        <v>-0.9241499564080228</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
@@ -1397,8 +1405,12 @@
       <c r="T10" s="118" t="n">
         <v>0.0556119638333332</v>
       </c>
-      <c r="U10" s="117" t="n"/>
-      <c r="V10" s="117" t="n"/>
+      <c r="U10" s="117" t="n">
+        <v>40.8623986</v>
+      </c>
+      <c r="V10" s="117" t="n">
+        <v>3.862398599999999</v>
+      </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
     <row r="11" ht="36" customHeight="1" s="74">
@@ -1452,10 +1464,10 @@
         <v>1.668520578420468</v>
       </c>
       <c r="N11" s="119" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-1.668520578420468</v>
+        <v>0.3314794215795325</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
@@ -1472,8 +1484,12 @@
       <c r="T11" s="118" t="n">
         <v>0.0528441753333333</v>
       </c>
-      <c r="U11" s="117" t="n"/>
-      <c r="V11" s="117" t="n"/>
+      <c r="U11" s="117" t="n">
+        <v>50.944073</v>
+      </c>
+      <c r="V11" s="117" t="n">
+        <v>-7.055926999999997</v>
+      </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
     <row r="12" ht="36" customHeight="1" s="74">
@@ -1527,10 +1543,10 @@
         <v>0.6048387096774193</v>
       </c>
       <c r="N12" s="119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-0.6048387096774193</v>
+        <v>0.3951612903225807</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
@@ -1547,8 +1563,12 @@
       <c r="T12" s="118" t="n">
         <v>-0.8009799999999999</v>
       </c>
-      <c r="U12" s="117" t="n"/>
-      <c r="V12" s="117" t="n"/>
+      <c r="U12" s="117" t="n">
+        <v>19.26</v>
+      </c>
+      <c r="V12" s="117" t="n">
+        <v>-140.74</v>
+      </c>
       <c r="W12" s="120" t="inlineStr"/>
     </row>
     <row r="13" ht="21" customHeight="1" s="74">
@@ -1602,10 +1622,10 @@
         <v>56.02716468590832</v>
       </c>
       <c r="N13" s="119" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-56.02716468590832</v>
+        <v>30.97283531409168</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
@@ -1622,8 +1642,12 @@
       <c r="T13" s="118" t="n">
         <v>0.0296227272727272</v>
       </c>
-      <c r="U13" s="117" t="n"/>
-      <c r="V13" s="117" t="n"/>
+      <c r="U13" s="117" t="n">
+        <v>12.59827586206896</v>
+      </c>
+      <c r="V13" s="117" t="n">
+        <v>-6.401724137931035</v>
+      </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
     <row r="14" ht="36" customHeight="1" s="74">
@@ -1677,10 +1701,10 @@
         <v>3.225806451612904</v>
       </c>
       <c r="N14" s="119" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-3.225806451612904</v>
+        <v>3.774193548387096</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
@@ -1697,8 +1721,12 @@
       <c r="T14" s="118" t="n">
         <v>-0.37845</v>
       </c>
-      <c r="U14" s="117" t="n"/>
-      <c r="V14" s="117" t="n"/>
+      <c r="U14" s="117" t="n">
+        <v>8.592857142857143</v>
+      </c>
+      <c r="V14" s="117" t="n">
+        <v>-21.40714285714286</v>
+      </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
     <row r="15" ht="36" customHeight="1" s="74">
@@ -1825,10 +1853,10 @@
         <v>24.19354838709678</v>
       </c>
       <c r="N16" s="119" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-24.19354838709678</v>
+        <v>-5.193548387096776</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
@@ -1845,8 +1873,12 @@
       <c r="T16" s="118" t="n">
         <v>0.377343216333333</v>
       </c>
-      <c r="U16" s="117" t="n"/>
-      <c r="V16" s="117" t="n"/>
+      <c r="U16" s="117" t="n">
+        <v>21.04599142105263</v>
+      </c>
+      <c r="V16" s="117" t="n">
+        <v>9.04599142105263</v>
+      </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
     <row r="17" ht="21" customHeight="1" s="74">
@@ -1896,10 +1928,10 @@
         <v>8.415147265077138</v>
       </c>
       <c r="N17" s="119" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-8.415147265077138</v>
+        <v>-5.415147265077138</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
@@ -1916,8 +1948,12 @@
       <c r="T17" s="118" t="n">
         <v>-0.1772083333333333</v>
       </c>
-      <c r="U17" s="117" t="n"/>
-      <c r="V17" s="117" t="n"/>
+      <c r="U17" s="117" t="n">
+        <v>53.08333333333334</v>
+      </c>
+      <c r="V17" s="117" t="n">
+        <v>30.08333333333334</v>
+      </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
     <row r="18" ht="21" customHeight="1" s="74">
@@ -1955,10 +1991,10 @@
         <v>128.6214375673263</v>
       </c>
       <c r="N18" s="125" t="n">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-128.6214375673263</v>
+        <v>32.37856243267373</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
@@ -1975,8 +2011,12 @@
       <c r="T18" s="124" t="n">
         <v>0.0612525081249998</v>
       </c>
-      <c r="U18" s="123" t="n"/>
-      <c r="V18" s="123" t="n"/>
+      <c r="U18" s="123" t="n">
+        <v>20.41279118012422</v>
+      </c>
+      <c r="V18" s="123" t="n">
+        <v>-3.663865496391278</v>
+      </c>
       <c r="W18" s="126" t="n"/>
     </row>
     <row r="19" ht="21" customHeight="1" s="74">
@@ -2026,10 +2066,10 @@
         <v>112.7819548872181</v>
       </c>
       <c r="N19" s="119" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-112.7819548872181</v>
+        <v>-25.78195488721806</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
@@ -2038,16 +2078,20 @@
         <v>857.1428571428571</v>
       </c>
       <c r="R19" s="117" t="n">
+        <v>661.1999999999999</v>
+      </c>
+      <c r="S19" s="117" t="n">
+        <v>-195.9428571428572</v>
+      </c>
+      <c r="T19" s="118" t="n">
+        <v>-0.2286</v>
+      </c>
+      <c r="U19" s="117" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="V19" s="117" t="n">
         <v>0</v>
       </c>
-      <c r="S19" s="117" t="n">
-        <v>-857.1428571428571</v>
-      </c>
-      <c r="T19" s="118" t="n">
-        <v>-1</v>
-      </c>
-      <c r="U19" s="117" t="n"/>
-      <c r="V19" s="117" t="n"/>
       <c r="W19" s="120" t="inlineStr"/>
     </row>
     <row r="20" ht="21" customHeight="1" s="74">
@@ -2097,10 +2141,10 @@
         <v>63.49206349206349</v>
       </c>
       <c r="N20" s="119" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-63.49206349206349</v>
+        <v>-6.492063492063487</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
@@ -2109,16 +2153,20 @@
         <v>571.4285714285714</v>
       </c>
       <c r="R20" s="117" t="n">
+        <v>513</v>
+      </c>
+      <c r="S20" s="117" t="n">
+        <v>-58.42857142857144</v>
+      </c>
+      <c r="T20" s="118" t="n">
+        <v>-0.10225</v>
+      </c>
+      <c r="U20" s="117" t="n">
+        <v>9</v>
+      </c>
+      <c r="V20" s="117" t="n">
         <v>0</v>
       </c>
-      <c r="S20" s="117" t="n">
-        <v>-571.4285714285714</v>
-      </c>
-      <c r="T20" s="118" t="n">
-        <v>-1</v>
-      </c>
-      <c r="U20" s="117" t="n"/>
-      <c r="V20" s="117" t="n"/>
       <c r="W20" s="120" t="inlineStr"/>
     </row>
     <row r="21" ht="21" customHeight="1" s="74">
@@ -2168,10 +2216,10 @@
         <v>23.80952380952381</v>
       </c>
       <c r="N21" s="119" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-23.80952380952381</v>
+        <v>21.19047619047619</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
@@ -2180,16 +2228,20 @@
         <v>190.4761904761905</v>
       </c>
       <c r="R21" s="117" t="n">
+        <v>360</v>
+      </c>
+      <c r="S21" s="117" t="n">
+        <v>169.5238095238095</v>
+      </c>
+      <c r="T21" s="118" t="n">
+        <v>0.8899999999999999</v>
+      </c>
+      <c r="U21" s="117" t="n">
+        <v>8</v>
+      </c>
+      <c r="V21" s="117" t="n">
         <v>0</v>
       </c>
-      <c r="S21" s="117" t="n">
-        <v>-190.4761904761905</v>
-      </c>
-      <c r="T21" s="118" t="n">
-        <v>-1</v>
-      </c>
-      <c r="U21" s="117" t="n"/>
-      <c r="V21" s="117" t="n"/>
       <c r="W21" s="120" t="inlineStr"/>
     </row>
     <row r="22" ht="21" customHeight="1" s="74">
@@ -2227,10 +2279,10 @@
         <v>200.0835421888053</v>
       </c>
       <c r="N22" s="125" t="n">
-        <v>0</v>
+        <v>189</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-200.0835421888053</v>
+        <v>-11.08354218880535</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
@@ -2239,16 +2291,20 @@
         <v>1619.047619047619</v>
       </c>
       <c r="R22" s="123" t="n">
-        <v>0</v>
+        <v>1534.2</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-1619.047619047619</v>
+        <v>-84.84761904761922</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-1</v>
-      </c>
-      <c r="U22" s="123" t="n"/>
-      <c r="V22" s="123" t="n"/>
+        <v>-0.0524058823529412</v>
+      </c>
+      <c r="U22" s="123" t="n">
+        <v>8.117460317460317</v>
+      </c>
+      <c r="V22" s="123" t="n">
+        <v>0.0256022798820296</v>
+      </c>
       <c r="W22" s="126" t="n"/>
     </row>
     <row r="23" ht="21" customHeight="1" s="74">
@@ -2286,10 +2342,10 @@
         <v>411.9757974605577</v>
       </c>
       <c r="N23" s="131" t="n">
-        <v>0</v>
+        <v>462</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-411.9757974605577</v>
+        <v>50.02420253944229</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
@@ -2298,16 +2354,20 @@
         <v>8296.466973886329</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>6763.292851</v>
+        <v>8297.492851000001</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-1533.174122886328</v>
+        <v>1.025877113672323</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1847984362153304</v>
-      </c>
-      <c r="U23" s="129" t="n"/>
-      <c r="V23" s="129" t="n"/>
+        <v>0.0001236522867988</v>
+      </c>
+      <c r="U23" s="129" t="n">
+        <v>17.95994123593074</v>
+      </c>
+      <c r="V23" s="129" t="n">
+        <v>-2.084667353106845</v>
+      </c>
       <c r="W23" s="132" t="n"/>
     </row>
     <row r="24" ht="21" customHeight="1" s="74"/>
@@ -2642,7 +2702,7 @@
       <c r="AD2" s="137" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:ok</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -2723,7 +2783,7 @@
       <c r="AD3" s="137" t="inlineStr"/>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:ok</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -2804,7 +2864,7 @@
       <c r="AD4" s="137" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -2876,10 +2936,10 @@
         <v>112.7819548872181</v>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="S5" t="n">
-        <v>-112.7819548872181</v>
+        <v>-25.78195488721806</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
@@ -2888,22 +2948,26 @@
         <v>857.1428571428571</v>
       </c>
       <c r="V5" s="135" t="n">
+        <v>661.1999999999999</v>
+      </c>
+      <c r="W5" s="135" t="n">
+        <v>-195.9428571428572</v>
+      </c>
+      <c r="X5" s="136" t="n">
+        <v>-0.2286</v>
+      </c>
+      <c r="Y5" s="135" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="Z5" s="135" t="n">
         <v>0</v>
       </c>
-      <c r="W5" s="135" t="n">
-        <v>-857.1428571428571</v>
-      </c>
-      <c r="X5" s="136" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Y5" s="135" t="n"/>
-      <c r="Z5" s="135" t="n"/>
       <c r="AB5" s="137" t="inlineStr"/>
       <c r="AC5" s="137" t="inlineStr"/>
       <c r="AD5" s="137" t="inlineStr"/>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>manual:no_ads_source;crm:stale</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -2975,10 +3039,10 @@
         <v>63.49206349206349</v>
       </c>
       <c r="R6" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="S6" t="n">
-        <v>-63.49206349206349</v>
+        <v>-6.492063492063487</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
@@ -2987,22 +3051,26 @@
         <v>571.4285714285714</v>
       </c>
       <c r="V6" s="135" t="n">
+        <v>513</v>
+      </c>
+      <c r="W6" s="135" t="n">
+        <v>-58.42857142857144</v>
+      </c>
+      <c r="X6" s="136" t="n">
+        <v>-0.10225</v>
+      </c>
+      <c r="Y6" s="135" t="n">
+        <v>9</v>
+      </c>
+      <c r="Z6" s="135" t="n">
         <v>0</v>
       </c>
-      <c r="W6" s="135" t="n">
-        <v>-571.4285714285714</v>
-      </c>
-      <c r="X6" s="136" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Y6" s="135" t="n"/>
-      <c r="Z6" s="135" t="n"/>
       <c r="AB6" s="137" t="inlineStr"/>
       <c r="AC6" s="137" t="inlineStr"/>
       <c r="AD6" s="137" t="inlineStr"/>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>manual:no_ads_source;crm:stale</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -3074,10 +3142,10 @@
         <v>23.80952380952381</v>
       </c>
       <c r="R7" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>-23.80952380952381</v>
+        <v>21.19047619047619</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
@@ -3086,22 +3154,26 @@
         <v>190.4761904761905</v>
       </c>
       <c r="V7" s="135" t="n">
+        <v>360</v>
+      </c>
+      <c r="W7" s="135" t="n">
+        <v>169.5238095238095</v>
+      </c>
+      <c r="X7" s="136" t="n">
+        <v>0.8899999999999999</v>
+      </c>
+      <c r="Y7" s="135" t="n">
+        <v>8</v>
+      </c>
+      <c r="Z7" s="135" t="n">
         <v>0</v>
       </c>
-      <c r="W7" s="135" t="n">
-        <v>-190.4761904761905</v>
-      </c>
-      <c r="X7" s="136" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Y7" s="135" t="n"/>
-      <c r="Z7" s="135" t="n"/>
       <c r="AB7" s="137" t="inlineStr"/>
       <c r="AC7" s="137" t="inlineStr"/>
       <c r="AD7" s="137" t="inlineStr"/>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>manual:no_ads_source;crm:stale</t>
+          <t>manual:no_ads_source</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -3173,10 +3245,10 @@
         <v>12.48699271592091</v>
       </c>
       <c r="R8" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-12.48699271592091</v>
+        <v>9.513007284079086</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
@@ -3193,8 +3265,12 @@
       <c r="X8" s="136" t="n">
         <v>0.4844851812499998</v>
       </c>
-      <c r="Y8" s="135" t="n"/>
-      <c r="Z8" s="135" t="n"/>
+      <c r="Y8" s="135" t="n">
+        <v>26.11997386363636</v>
+      </c>
+      <c r="Z8" s="135" t="n">
+        <v>-4.88002613636364</v>
+      </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
           <t>23968989759</t>
@@ -3204,7 +3280,7 @@
       <c r="AD8" s="137" t="inlineStr"/>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:ok</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -3276,10 +3352,10 @@
         <v>20.92414995640802</v>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-20.92414995640802</v>
+        <v>-0.9241499564080228</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
@@ -3296,8 +3372,12 @@
       <c r="X9" s="136" t="n">
         <v>0.0556119638333332</v>
       </c>
-      <c r="Y9" s="135" t="n"/>
-      <c r="Z9" s="135" t="n"/>
+      <c r="Y9" s="135" t="n">
+        <v>40.8623986</v>
+      </c>
+      <c r="Z9" s="135" t="n">
+        <v>3.862398599999999</v>
+      </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
           <t>23990314506</t>
@@ -3307,7 +3387,7 @@
       <c r="AD9" s="137" t="inlineStr"/>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:ok</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -3379,10 +3459,10 @@
         <v>1.668520578420468</v>
       </c>
       <c r="R10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-1.668520578420468</v>
+        <v>0.3314794215795325</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
@@ -3399,8 +3479,12 @@
       <c r="X10" s="136" t="n">
         <v>0.0528441753333333</v>
       </c>
-      <c r="Y10" s="135" t="n"/>
-      <c r="Z10" s="135" t="n"/>
+      <c r="Y10" s="135" t="n">
+        <v>50.944073</v>
+      </c>
+      <c r="Z10" s="135" t="n">
+        <v>-7.055926999999997</v>
+      </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
           <t>23993375943</t>
@@ -3410,7 +3494,7 @@
       <c r="AD10" s="137" t="inlineStr"/>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:ok</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -3482,10 +3566,10 @@
         <v>0.6048387096774193</v>
       </c>
       <c r="R11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.6048387096774193</v>
+        <v>0.3951612903225807</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
@@ -3502,8 +3586,12 @@
       <c r="X11" s="136" t="n">
         <v>-0.8009799999999999</v>
       </c>
-      <c r="Y11" s="135" t="n"/>
-      <c r="Z11" s="135" t="n"/>
+      <c r="Y11" s="135" t="n">
+        <v>19.26</v>
+      </c>
+      <c r="Z11" s="135" t="n">
+        <v>-140.74</v>
+      </c>
       <c r="AB11" s="137" t="inlineStr">
         <is>
           <t>23993437149</t>
@@ -3513,7 +3601,7 @@
       <c r="AD11" s="137" t="inlineStr"/>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:ok</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -3585,10 +3673,10 @@
         <v>56.02716468590832</v>
       </c>
       <c r="R12" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="S12" t="n">
-        <v>-56.02716468590832</v>
+        <v>30.97283531409168</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
@@ -3605,8 +3693,12 @@
       <c r="X12" s="136" t="n">
         <v>0.0296227272727272</v>
       </c>
-      <c r="Y12" s="135" t="n"/>
-      <c r="Z12" s="135" t="n"/>
+      <c r="Y12" s="135" t="n">
+        <v>12.59827586206896</v>
+      </c>
+      <c r="Z12" s="135" t="n">
+        <v>-6.401724137931035</v>
+      </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
         <is>
@@ -3616,7 +3708,7 @@
       <c r="AD12" s="137" t="inlineStr"/>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -3688,10 +3780,10 @@
         <v>3.225806451612904</v>
       </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>-3.225806451612904</v>
+        <v>3.774193548387096</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
@@ -3708,8 +3800,12 @@
       <c r="X13" s="136" t="n">
         <v>-0.37845</v>
       </c>
-      <c r="Y13" s="135" t="n"/>
-      <c r="Z13" s="135" t="n"/>
+      <c r="Y13" s="135" t="n">
+        <v>8.592857142857143</v>
+      </c>
+      <c r="Z13" s="135" t="n">
+        <v>-21.40714285714286</v>
+      </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
         <is>
@@ -3719,7 +3815,7 @@
       <c r="AD13" s="137" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -3819,7 +3915,7 @@
       <c r="AD14" s="137" t="inlineStr"/>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -3891,10 +3987,10 @@
         <v>24.19354838709678</v>
       </c>
       <c r="R15" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-24.19354838709678</v>
+        <v>-5.193548387096776</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
@@ -3911,8 +4007,12 @@
       <c r="X15" s="136" t="n">
         <v>0.377343216333333</v>
       </c>
-      <c r="Y15" s="135" t="n"/>
-      <c r="Z15" s="135" t="n"/>
+      <c r="Y15" s="135" t="n">
+        <v>21.04599142105263</v>
+      </c>
+      <c r="Z15" s="135" t="n">
+        <v>9.04599142105263</v>
+      </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
           <t>21905808840</t>
@@ -3922,7 +4022,7 @@
       <c r="AD15" s="137" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>google:ok;crm:stale</t>
+          <t>google:ok</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -3989,10 +4089,10 @@
         <v>8.415147265077138</v>
       </c>
       <c r="R16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-8.415147265077138</v>
+        <v>-5.415147265077138</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
@@ -4009,8 +4109,12 @@
       <c r="X16" s="136" t="n">
         <v>-0.1772083333333333</v>
       </c>
-      <c r="Y16" s="135" t="n"/>
-      <c r="Z16" s="135" t="n"/>
+      <c r="Y16" s="135" t="n">
+        <v>53.08333333333334</v>
+      </c>
+      <c r="Z16" s="135" t="n">
+        <v>30.08333333333334</v>
+      </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
         <is>
@@ -4020,7 +4124,7 @@
       <c r="AD16" s="137" t="inlineStr"/>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:ok</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -4079,10 +4183,10 @@
         <v>83.27081770442611</v>
       </c>
       <c r="R17" t="n">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="S17" t="n">
-        <v>-83.27081770442611</v>
+        <v>28.72918229557389</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
@@ -4099,14 +4203,18 @@
       <c r="X17" s="136" t="n">
         <v>-0.0289924540450449</v>
       </c>
-      <c r="Y17" s="135" t="n"/>
-      <c r="Z17" s="135" t="n"/>
+      <c r="Y17" s="135" t="n">
+        <v>31.04315599107144</v>
+      </c>
+      <c r="Z17" s="135" t="n">
+        <v>-11.95684400892857</v>
+      </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
       <c r="AD17" s="137" t="inlineStr"/>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>partial;crm:stale</t>
+          <t>partial</t>
         </is>
       </c>
     </row>
@@ -4160,10 +4268,10 @@
         <v>128.6214375673263</v>
       </c>
       <c r="R18" t="n">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="S18" t="n">
-        <v>-128.6214375673263</v>
+        <v>32.37856243267373</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
@@ -4180,14 +4288,18 @@
       <c r="X18" s="136" t="n">
         <v>0.0612525081249998</v>
       </c>
-      <c r="Y18" s="135" t="n"/>
-      <c r="Z18" s="135" t="n"/>
+      <c r="Y18" s="135" t="n">
+        <v>20.41279118012422</v>
+      </c>
+      <c r="Z18" s="135" t="n">
+        <v>-3.663865496391278</v>
+      </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
       <c r="AD18" s="137" t="inlineStr"/>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>partial;crm:stale</t>
+          <t>partial</t>
         </is>
       </c>
     </row>
@@ -4241,10 +4353,10 @@
         <v>200.0835421888053</v>
       </c>
       <c r="R19" t="n">
-        <v>0</v>
+        <v>189</v>
       </c>
       <c r="S19" t="n">
-        <v>-200.0835421888053</v>
+        <v>-11.08354218880535</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
@@ -4253,22 +4365,26 @@
         <v>1619.047619047619</v>
       </c>
       <c r="V19" s="135" t="n">
-        <v>0</v>
+        <v>1534.2</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-1619.047619047619</v>
+        <v>-84.84761904761922</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Y19" s="135" t="n"/>
-      <c r="Z19" s="135" t="n"/>
+        <v>-0.0524058823529412</v>
+      </c>
+      <c r="Y19" s="135" t="n">
+        <v>8.117460317460317</v>
+      </c>
+      <c r="Z19" s="135" t="n">
+        <v>0.0256022798820296</v>
+      </c>
       <c r="AB19" s="137" t="inlineStr"/>
       <c r="AC19" s="137" t="inlineStr"/>
       <c r="AD19" s="137" t="inlineStr"/>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>success;crm:stale</t>
+          <t>success</t>
         </is>
       </c>
     </row>
@@ -4322,10 +4438,10 @@
         <v>411.9757974605577</v>
       </c>
       <c r="R20" t="n">
-        <v>0</v>
+        <v>462</v>
       </c>
       <c r="S20" t="n">
-        <v>-411.9757974605577</v>
+        <v>50.02420253944229</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
@@ -4334,22 +4450,26 @@
         <v>8296.466973886329</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>6763.292851</v>
+        <v>8297.492851000001</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-1533.174122886328</v>
+        <v>1.025877113672323</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1847984362153304</v>
-      </c>
-      <c r="Y20" s="135" t="n"/>
-      <c r="Z20" s="135" t="n"/>
+        <v>0.0001236522867988</v>
+      </c>
+      <c r="Y20" s="135" t="n">
+        <v>17.95994123593074</v>
+      </c>
+      <c r="Z20" s="135" t="n">
+        <v>-2.084667353106845</v>
+      </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
       <c r="AD20" s="137" t="inlineStr"/>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>partial;crm:stale</t>
+          <t>partial</t>
         </is>
       </c>
     </row>
@@ -4505,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46241.43869212963</v>
+        <v>46241.47125</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-08
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 06/08/2026  |  Ultimo aggiornamento: 07/08/2026 11:18</t>
+          <t>Periodo: 01/08/2026 - 07/08/2026  |  Ultimo aggiornamento: 08/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>1548.387096774194</v>
+        <v>1806.451612903226</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>1569.826148</v>
+        <v>1843.382292</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>21.43905122580645</v>
+        <v>36.93067909677416</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0138460539166666</v>
+        <v>0.0204437687857142</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>193.5483870967742</v>
+        <v>225.8064516129032</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>192.347323</v>
+        <v>223.381471</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>-1.201064096774218</v>
+        <v>-2.424980612903227</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>-0.0062054978333334</v>
+        <v>-0.0107391998571428</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>1838.709677419354</v>
+        <v>2145.16129032258</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>1714.66</v>
+        <v>2021.36</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-124.0496774193546</v>
+        <v>-123.8012903225806</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0674656140350875</v>
+        <v>-0.0577118796992481</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>83.27081770442611</v>
+        <v>97.14928732183046</v>
       </c>
       <c r="N8" s="125" t="n">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>28.72918229557389</v>
+        <v>18.85071267816954</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>3580.645161290322</v>
+        <v>4177.419354838709</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>3476.833471</v>
+        <v>4088.123763</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-103.8116902903221</v>
+        <v>-89.29559183870924</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0289924540450449</v>
+        <v>-0.0213757787413126</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>31.04315599107144</v>
+        <v>35.24244623275862</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>-11.95684400892857</v>
+        <v>-7.757553767241376</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>12.48699271592091</v>
+        <v>14.5681581685744</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>9.513007284079086</v>
+        <v>7.431841831425601</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>387.0967741935484</v>
+        <v>451.6129032258065</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>574.639425</v>
+        <v>632.053009</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>187.5426508064515</v>
+        <v>180.4401057741935</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.4844851812499998</v>
+        <v>0.3995459484999999</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>26.11997386363636</v>
+        <v>28.72968222727273</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>-4.88002613636364</v>
+        <v>-2.270317772727275</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>20.92414995640802</v>
+        <v>24.41150828247602</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-0.9241499564080228</v>
+        <v>-4.411508282476024</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>774.1935483870968</v>
+        <v>903.2258064516128</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>817.247972</v>
+        <v>944.880274</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>43.05442361290318</v>
+        <v>41.65446754838706</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>0.0556119638333332</v>
+        <v>0.0461174462142856</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>40.8623986</v>
+        <v>47.2440137</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>3.862398599999999</v>
+        <v>10.2440137</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>1.668520578420468</v>
+        <v>1.946607341490545</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>0.3314794215795325</v>
+        <v>0.0533926585094546</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>96.7741935483871</v>
+        <v>112.9032258064516</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>101.888146</v>
+        <v>118.181522</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>5.113952451612903</v>
+        <v>5.278296193548385</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0528441753333333</v>
+        <v>0.0467506234285714</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>50.944073</v>
+        <v>59.090761</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>-7.055926999999997</v>
+        <v>1.090761</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,28 +1540,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>0.6048387096774193</v>
+        <v>0.7056451612903225</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>0.3951612903225807</v>
+        <v>0.2943548387096775</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>96.7741935483871</v>
+        <v>112.9032258064516</v>
       </c>
       <c r="R12" s="117" t="n">
         <v>19.26</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-77.5141935483871</v>
+        <v>-93.6432258064516</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.8009799999999999</v>
+        <v>-0.8294114285714286</v>
       </c>
       <c r="U12" s="117" t="n">
         <v>19.26</v>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>56.02716468590832</v>
+        <v>65.36502546689303</v>
       </c>
       <c r="N13" s="119" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>30.97283531409168</v>
+        <v>26.63497453310697</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>1064.516129032258</v>
+        <v>1241.935483870968</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>1096.05</v>
+        <v>1268</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>31.5338709677419</v>
+        <v>26.06451612903243</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.0296227272727272</v>
+        <v>0.0209870129870131</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>12.59827586206896</v>
+        <v>13.78260869565217</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>-6.401724137931035</v>
+        <v>-5.217391304347826</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>3.225806451612904</v>
+        <v>3.763440860215054</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>3.774193548387096</v>
+        <v>3.236559139784946</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>96.7741935483871</v>
+        <v>112.9032258064516</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>60.15</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-36.62419354838711</v>
+        <v>-43.83322580645162</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.37845</v>
+        <v>-0.3882371428571429</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>8.592857142857143</v>
+        <v>9.867142857142856</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-21.40714285714286</v>
+        <v>-20.13285714285714</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>1.075268817204301</v>
+        <v>1.254480286738351</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-1.075268817204301</v>
+        <v>-1.254480286738351</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>96.7741935483871</v>
+        <v>112.9032258064516</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>58.1</v>
+        <v>68.09</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-38.6741935483871</v>
+        <v>-44.81322580645161</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3996333333333333</v>
+        <v>-0.3969171428571428</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>24.19354838709678</v>
+        <v>28.2258064516129</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-5.193548387096776</v>
+        <v>-9.225806451612904</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>290.3225806451613</v>
+        <v>338.7096774193549</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>399.873837</v>
+        <v>444.285041</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>109.5512563548386</v>
+        <v>105.5753635806451</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.377343216333333</v>
+        <v>0.3116986924761902</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>21.04599142105263</v>
+        <v>23.38342321052632</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>9.04599142105263</v>
+        <v>11.38342321052631</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>8.415147265077138</v>
+        <v>9.817671809256662</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-5.415147265077138</v>
+        <v>-6.817671809256662</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>193.5483870967742</v>
+        <v>225.8064516129032</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>159.25</v>
+        <v>188.48</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-34.29838709677421</v>
+        <v>-37.32645161290324</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.1772083333333333</v>
+        <v>-0.1653028571428572</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>53.08333333333334</v>
+        <v>62.82666666666666</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>30.08333333333334</v>
+        <v>39.82666666666666</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>128.6214375673263</v>
+        <v>150.0583438285473</v>
       </c>
       <c r="N18" s="125" t="n">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>32.37856243267373</v>
+        <v>15.94165617145271</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>3096.774193548388</v>
+        <v>3612.903225806452</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>3286.45938</v>
+        <v>3752.299846</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>189.6851864516125</v>
+        <v>139.3966201935482</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>0.0612525081249998</v>
+        <v>0.0385829930892856</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>20.41279118012422</v>
+        <v>22.60421593975904</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>-3.663865496391278</v>
+        <v>-1.472440736756464</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2063,28 +2063,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>112.7819548872181</v>
+        <v>140.9774436090226</v>
       </c>
       <c r="N19" s="119" t="n">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-25.78195488721806</v>
+        <v>-47.97744360902257</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>857.1428571428571</v>
+        <v>1071.428571428571</v>
       </c>
       <c r="R19" s="117" t="n">
-        <v>661.1999999999999</v>
+        <v>706.8</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-195.9428571428572</v>
+        <v>-364.6285714285714</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.2286</v>
+        <v>-0.3403199999999999</v>
       </c>
       <c r="U19" s="117" t="n">
         <v>7.6</v>
@@ -2138,28 +2138,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>63.49206349206349</v>
+        <v>79.36507936507935</v>
       </c>
       <c r="N20" s="119" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-6.492063492063487</v>
+        <v>-19.36507936507936</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>571.4285714285714</v>
+        <v>714.2857142857143</v>
       </c>
       <c r="R20" s="117" t="n">
-        <v>513</v>
+        <v>540</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-58.42857142857144</v>
+        <v>-174.2857142857143</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.10225</v>
+        <v>-0.244</v>
       </c>
       <c r="U20" s="117" t="n">
         <v>9</v>
@@ -2213,28 +2213,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>23.80952380952381</v>
+        <v>29.76190476190476</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>21.19047619047619</v>
+        <v>15.23809523809524</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>190.4761904761905</v>
+        <v>238.0952380952381</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>360</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>169.5238095238095</v>
+        <v>121.9047619047619</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>0.8899999999999999</v>
+        <v>0.512</v>
       </c>
       <c r="U21" s="117" t="n">
         <v>8</v>
@@ -2276,34 +2276,34 @@
         <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>200.0835421888053</v>
+        <v>250.1044277360067</v>
       </c>
       <c r="N22" s="125" t="n">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-11.08354218880535</v>
+        <v>-52.1044277360067</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="Q22" s="123" t="n">
-        <v>1619.047619047619</v>
+        <v>2023.809523809524</v>
       </c>
       <c r="R22" s="123" t="n">
-        <v>1534.2</v>
+        <v>1606.8</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-84.84761904761922</v>
+        <v>-417.0095238095239</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-0.0524058823529412</v>
+        <v>-0.2060517647058823</v>
       </c>
       <c r="U22" s="123" t="n">
-        <v>8.117460317460317</v>
+        <v>8.115151515151515</v>
       </c>
       <c r="V22" s="123" t="n">
-        <v>0.0256022798820296</v>
+        <v>0.0232934775732278</v>
       </c>
       <c r="W22" s="126" t="n"/>
     </row>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>411.9757974605577</v>
+        <v>497.3120588863844</v>
       </c>
       <c r="N23" s="131" t="n">
-        <v>462</v>
+        <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>50.02420253944229</v>
+        <v>-17.31205888638442</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>8296.466973886329</v>
+        <v>9814.132104454686</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>8297.492851000001</v>
+        <v>9447.223609000001</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>1.025877113672323</v>
+        <v>-366.9084954546852</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>0.0001236522867988</v>
+        <v>-0.0373857302458913</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>17.95994123593074</v>
+        <v>19.68171585208334</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>-2.084667353106845</v>
+        <v>-0.3628927369542474</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>1548.387096774194</v>
+        <v>1806.451612903226</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>1569.826148</v>
+        <v>1843.382292</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>21.43905122580645</v>
+        <v>36.93067909677416</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0138460539166666</v>
+        <v>0.0204437687857142</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>193.5483870967742</v>
+        <v>225.8064516129032</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>192.347323</v>
+        <v>223.381471</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>-1.201064096774218</v>
+        <v>-2.424980612903227</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>-0.0062054978333334</v>
+        <v>-0.0107391998571428</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>1838.709677419354</v>
+        <v>2145.16129032258</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>1714.66</v>
+        <v>2021.36</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-124.0496774193546</v>
+        <v>-123.8012903225806</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0674656140350875</v>
+        <v>-0.0577118796992481</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2933,28 +2933,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>112.7819548872181</v>
+        <v>140.9774436090226</v>
       </c>
       <c r="R5" t="n">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="S5" t="n">
-        <v>-25.78195488721806</v>
+        <v>-47.97744360902257</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="U5" s="135" t="n">
-        <v>857.1428571428571</v>
+        <v>1071.428571428571</v>
       </c>
       <c r="V5" s="135" t="n">
-        <v>661.1999999999999</v>
+        <v>706.8</v>
       </c>
       <c r="W5" s="135" t="n">
-        <v>-195.9428571428572</v>
+        <v>-364.6285714285714</v>
       </c>
       <c r="X5" s="136" t="n">
-        <v>-0.2286</v>
+        <v>-0.3403199999999999</v>
       </c>
       <c r="Y5" s="135" t="n">
         <v>7.6</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3036,28 +3036,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>63.49206349206349</v>
+        <v>79.36507936507935</v>
       </c>
       <c r="R6" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="S6" t="n">
-        <v>-6.492063492063487</v>
+        <v>-19.36507936507936</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>571.4285714285714</v>
+        <v>714.2857142857143</v>
       </c>
       <c r="V6" s="135" t="n">
-        <v>513</v>
+        <v>540</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-58.42857142857144</v>
+        <v>-174.2857142857143</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.10225</v>
+        <v>-0.244</v>
       </c>
       <c r="Y6" s="135" t="n">
         <v>9</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3139,28 +3139,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>23.80952380952381</v>
+        <v>29.76190476190476</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>21.19047619047619</v>
+        <v>15.23809523809524</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>190.4761904761905</v>
+        <v>238.0952380952381</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>360</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>169.5238095238095</v>
+        <v>121.9047619047619</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>0.8899999999999999</v>
+        <v>0.512</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>8</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>12.48699271592091</v>
+        <v>14.5681581685744</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>9.513007284079086</v>
+        <v>7.431841831425601</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>387.0967741935484</v>
+        <v>451.6129032258065</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>574.639425</v>
+        <v>632.053009</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>187.5426508064515</v>
+        <v>180.4401057741935</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>0.4844851812499998</v>
+        <v>0.3995459484999999</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>26.11997386363636</v>
+        <v>28.72968222727273</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>-4.88002613636364</v>
+        <v>-2.270317772727275</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>20.92414995640802</v>
+        <v>24.41150828247602</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.9241499564080228</v>
+        <v>-4.411508282476024</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>774.1935483870968</v>
+        <v>903.2258064516128</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>817.247972</v>
+        <v>944.880274</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>43.05442361290318</v>
+        <v>41.65446754838706</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.0556119638333332</v>
+        <v>0.0461174462142856</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>40.8623986</v>
+        <v>47.2440137</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>3.862398599999999</v>
+        <v>10.2440137</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>1.668520578420468</v>
+        <v>1.946607341490545</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>0.3314794215795325</v>
+        <v>0.0533926585094546</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>96.7741935483871</v>
+        <v>112.9032258064516</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>101.888146</v>
+        <v>118.181522</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>5.113952451612903</v>
+        <v>5.278296193548385</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0528441753333333</v>
+        <v>0.0467506234285714</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>50.944073</v>
+        <v>59.090761</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>-7.055926999999997</v>
+        <v>1.090761</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,28 +3563,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.6048387096774193</v>
+        <v>0.7056451612903225</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>0.3951612903225807</v>
+        <v>0.2943548387096775</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>96.7741935483871</v>
+        <v>112.9032258064516</v>
       </c>
       <c r="V11" s="135" t="n">
         <v>19.26</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-77.5141935483871</v>
+        <v>-93.6432258064516</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.8009799999999999</v>
+        <v>-0.8294114285714286</v>
       </c>
       <c r="Y11" s="135" t="n">
         <v>19.26</v>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>56.02716468590832</v>
+        <v>65.36502546689303</v>
       </c>
       <c r="R12" t="n">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>30.97283531409168</v>
+        <v>26.63497453310697</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>1064.516129032258</v>
+        <v>1241.935483870968</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>1096.05</v>
+        <v>1268</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>31.5338709677419</v>
+        <v>26.06451612903243</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.0296227272727272</v>
+        <v>0.0209870129870131</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>12.59827586206896</v>
+        <v>13.78260869565217</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>-6.401724137931035</v>
+        <v>-5.217391304347826</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>3.225806451612904</v>
+        <v>3.763440860215054</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>3.774193548387096</v>
+        <v>3.236559139784946</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>96.7741935483871</v>
+        <v>112.9032258064516</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>60.15</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-36.62419354838711</v>
+        <v>-43.83322580645162</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.37845</v>
+        <v>-0.3882371428571429</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>8.592857142857143</v>
+        <v>9.867142857142856</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-21.40714285714286</v>
+        <v>-20.13285714285714</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.075268817204301</v>
+        <v>1.254480286738351</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-1.075268817204301</v>
+        <v>-1.254480286738351</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>96.7741935483871</v>
+        <v>112.9032258064516</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>58.1</v>
+        <v>68.09</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-38.6741935483871</v>
+        <v>-44.81322580645161</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3996333333333333</v>
+        <v>-0.3969171428571428</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>24.19354838709678</v>
+        <v>28.2258064516129</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-5.193548387096776</v>
+        <v>-9.225806451612904</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>290.3225806451613</v>
+        <v>338.7096774193549</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>399.873837</v>
+        <v>444.285041</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>109.5512563548386</v>
+        <v>105.5753635806451</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>0.377343216333333</v>
+        <v>0.3116986924761902</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>21.04599142105263</v>
+        <v>23.38342321052632</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>9.04599142105263</v>
+        <v>11.38342321052631</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>8.415147265077138</v>
+        <v>9.817671809256662</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-5.415147265077138</v>
+        <v>-6.817671809256662</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>193.5483870967742</v>
+        <v>225.8064516129032</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>159.25</v>
+        <v>188.48</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-34.29838709677421</v>
+        <v>-37.32645161290324</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.1772083333333333</v>
+        <v>-0.1653028571428572</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>53.08333333333334</v>
+        <v>62.82666666666666</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>30.08333333333334</v>
+        <v>39.82666666666666</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>83.27081770442611</v>
+        <v>97.14928732183046</v>
       </c>
       <c r="R17" t="n">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>28.72918229557389</v>
+        <v>18.85071267816954</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>3580.645161290322</v>
+        <v>4177.419354838709</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>3476.833471</v>
+        <v>4088.123763</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-103.8116902903221</v>
+        <v>-89.29559183870924</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0289924540450449</v>
+        <v>-0.0213757787413126</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>31.04315599107144</v>
+        <v>35.24244623275862</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>-11.95684400892857</v>
+        <v>-7.757553767241376</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>128.6214375673263</v>
+        <v>150.0583438285473</v>
       </c>
       <c r="R18" t="n">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>32.37856243267373</v>
+        <v>15.94165617145271</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>3096.774193548388</v>
+        <v>3612.903225806452</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>3286.45938</v>
+        <v>3752.299846</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>189.6851864516125</v>
+        <v>139.3966201935482</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>0.0612525081249998</v>
+        <v>0.0385829930892856</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>20.41279118012422</v>
+        <v>22.60421593975904</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>-3.663865496391278</v>
+        <v>-1.472440736756464</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4350,34 +4350,34 @@
         <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>200.0835421888053</v>
+        <v>250.1044277360067</v>
       </c>
       <c r="R19" t="n">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="S19" t="n">
-        <v>-11.08354218880535</v>
+        <v>-52.1044277360067</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>1619.047619047619</v>
+        <v>2023.809523809524</v>
       </c>
       <c r="V19" s="135" t="n">
-        <v>1534.2</v>
+        <v>1606.8</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-84.84761904761922</v>
+        <v>-417.0095238095239</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.0524058823529412</v>
+        <v>-0.2060517647058823</v>
       </c>
       <c r="Y19" s="135" t="n">
-        <v>8.117460317460317</v>
+        <v>8.115151515151515</v>
       </c>
       <c r="Z19" s="135" t="n">
-        <v>0.0256022798820296</v>
+        <v>0.0232934775732278</v>
       </c>
       <c r="AB19" s="137" t="inlineStr"/>
       <c r="AC19" s="137" t="inlineStr"/>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>411.9757974605577</v>
+        <v>497.3120588863844</v>
       </c>
       <c r="R20" t="n">
-        <v>462</v>
+        <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>50.02420253944229</v>
+        <v>-17.31205888638442</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>8296.466973886329</v>
+        <v>9814.132104454686</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>8297.492851000001</v>
+        <v>9447.223609000001</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>1.025877113672323</v>
+        <v>-366.9084954546852</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>0.0001236522867988</v>
+        <v>-0.0373857302458913</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>17.95994123593074</v>
+        <v>19.68171585208334</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>-2.084667353106845</v>
+        <v>-0.3628927369542474</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46241.47125</v>
+        <v>46242.29189814815</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-09
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 07/08/2026  |  Ultimo aggiornamento: 08/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 08/08/2026  |  Ultimo aggiornamento: 09/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>1806.451612903226</v>
+        <v>2064.516129032258</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>1843.382292</v>
+        <v>2099.164782</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>36.93067909677416</v>
+        <v>34.64865296774178</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0204437687857142</v>
+        <v>0.0167829412812499</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>225.8064516129032</v>
+        <v>258.0645161290323</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>223.381471</v>
+        <v>256.14504</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>-2.424980612903227</v>
+        <v>-1.919476129032262</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>-0.0107391998571428</v>
+        <v>-0.00743797</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>2145.16129032258</v>
+        <v>2451.612903225806</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>2021.36</v>
+        <v>2389.63</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-123.8012903225806</v>
+        <v>-61.98290322580624</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0577118796992481</v>
+        <v>-0.0252824999999999</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>97.14928732183046</v>
+        <v>111.0277569392348</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>18.85071267816954</v>
+        <v>4.972243060765194</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>4177.419354838709</v>
+        <v>4774.193548387097</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>4088.123763</v>
+        <v>4744.939822</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-89.29559183870924</v>
+        <v>-29.25372638709632</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0213757787413126</v>
+        <v>-0.0061274697162161</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>35.24244623275862</v>
+        <v>40.90465363793104</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>-7.757553767241376</v>
+        <v>-2.095346362068966</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>14.5681581685744</v>
+        <v>16.64932362122789</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>7.431841831425601</v>
+        <v>5.350676378772114</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>451.6129032258065</v>
+        <v>516.1290322580645</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>632.053009</v>
+        <v>684.37487</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>180.4401057741935</v>
+        <v>168.2458377419355</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.3995459484999999</v>
+        <v>0.325976310625</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>28.72968222727273</v>
+        <v>31.10794863636364</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>-2.270317772727275</v>
+        <v>0.1079486363636341</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>24.41150828247602</v>
+        <v>27.89886660854403</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-4.411508282476024</v>
+        <v>-7.898866608544029</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>903.2258064516128</v>
+        <v>1032.258064516129</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>944.880274</v>
+        <v>1071.079165</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>41.65446754838706</v>
+        <v>38.82110048387108</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>0.0461174462142856</v>
+        <v>0.0376079410937501</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>47.2440137</v>
+        <v>53.55395825000001</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>10.2440137</v>
+        <v>16.55395825000001</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>1.946607341490545</v>
+        <v>2.224694104560623</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>0.0533926585094546</v>
+        <v>-0.2246941045606232</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>112.9032258064516</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>118.181522</v>
+        <v>135.328689</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>5.278296193548385</v>
+        <v>6.296430935483869</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0467506234285714</v>
+        <v>0.0487973397499999</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>59.090761</v>
+        <v>67.6643445</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>1.090761</v>
+        <v>9.6643445</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,28 +1540,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>0.7056451612903225</v>
+        <v>0.8064516129032258</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>0.2943548387096775</v>
+        <v>0.1935483870967742</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>112.9032258064516</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="R12" s="117" t="n">
         <v>19.26</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-93.6432258064516</v>
+        <v>-109.7722580645161</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.8294114285714286</v>
+        <v>-0.8507349999999999</v>
       </c>
       <c r="U12" s="117" t="n">
         <v>19.26</v>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>65.36502546689303</v>
+        <v>74.70288624787776</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>26.63497453310697</v>
+        <v>17.29711375212224</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>1241.935483870968</v>
+        <v>1419.354838709677</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>1268</v>
+        <v>1425.51</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>26.06451612903243</v>
+        <v>6.155161290322667</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.0209870129870131</v>
+        <v>0.0043365909090909</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>13.78260869565217</v>
+        <v>15.49467391304348</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>-5.217391304347826</v>
+        <v>-3.505326086956522</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>3.763440860215054</v>
+        <v>4.301075268817205</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>3.236559139784946</v>
+        <v>2.698924731182795</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>112.9032258064516</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>69.06999999999999</v>
+        <v>79.87</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-43.83322580645162</v>
+        <v>-49.16225806451613</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3882371428571429</v>
+        <v>-0.3810074999999999</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>9.867142857142856</v>
+        <v>11.41</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-20.13285714285714</v>
+        <v>-18.59</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>1.254480286738351</v>
+        <v>1.433691756272401</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-1.254480286738351</v>
+        <v>-1.433691756272401</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>112.9032258064516</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>68.09</v>
+        <v>80.66</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-44.81322580645161</v>
+        <v>-48.37225806451613</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3969171428571428</v>
+        <v>-0.374885</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>28.2258064516129</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-9.225806451612904</v>
+        <v>-13.25806451612903</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>338.7096774193549</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>444.285041</v>
+        <v>490.919982</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>105.5753635806451</v>
+        <v>103.8232078064516</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.3116986924761902</v>
+        <v>0.2682099534999999</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>23.38342321052632</v>
+        <v>25.83789378947369</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>11.38342321052631</v>
+        <v>13.83789378947369</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>9.817671809256662</v>
+        <v>11.22019635343618</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-6.817671809256662</v>
+        <v>-8.220196353436185</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>225.8064516129032</v>
+        <v>258.0645161290323</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>188.48</v>
+        <v>213.81</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-37.32645161290324</v>
+        <v>-44.25451612903225</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.1653028571428572</v>
+        <v>-0.1714862499999999</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>62.82666666666666</v>
+        <v>71.27</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>39.82666666666666</v>
+        <v>48.27</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>150.0583438285473</v>
+        <v>171.4952500897683</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>15.94165617145271</v>
+        <v>-5.495250089768348</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>3612.903225806452</v>
+        <v>4129.032258064516</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>3752.299846</v>
+        <v>4200.812706</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>139.3966201935482</v>
+        <v>71.78044793548361</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>0.0385829930892856</v>
+        <v>0.0173843272343749</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>22.60421593975904</v>
+        <v>25.30610063855422</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>-1.472440736756464</v>
+        <v>1.229443962038715</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>497.3120588863844</v>
+        <v>532.6274347650099</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-17.31205888638442</v>
+        <v>-52.62743476500987</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>9814.132104454686</v>
+        <v>10927.03533026114</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>9447.223609000001</v>
+        <v>10552.552528</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-366.9084954546852</v>
+        <v>-374.4828022611364</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.0373857302458913</v>
+        <v>-0.0342712173011878</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>19.68171585208334</v>
+        <v>21.98448443333333</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>-0.3628927369542474</v>
+        <v>1.939875844295749</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>1806.451612903226</v>
+        <v>2064.516129032258</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>1843.382292</v>
+        <v>2099.164782</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>36.93067909677416</v>
+        <v>34.64865296774178</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0204437687857142</v>
+        <v>0.0167829412812499</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2702,7 +2702,7 @@
       <c r="AD2" s="137" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>225.8064516129032</v>
+        <v>258.0645161290323</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>223.381471</v>
+        <v>256.14504</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>-2.424980612903227</v>
+        <v>-1.919476129032262</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>-0.0107391998571428</v>
+        <v>-0.00743797</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2783,7 +2783,7 @@
       <c r="AD3" s="137" t="inlineStr"/>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>2145.16129032258</v>
+        <v>2451.612903225806</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>2021.36</v>
+        <v>2389.63</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-123.8012903225806</v>
+        <v>-61.98290322580624</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0577118796992481</v>
+        <v>-0.0252824999999999</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2864,7 +2864,7 @@
       <c r="AD4" s="137" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2967,7 +2967,7 @@
       <c r="AD5" s="137" t="inlineStr"/>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3070,7 +3070,7 @@
       <c r="AD6" s="137" t="inlineStr"/>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3173,7 +3173,7 @@
       <c r="AD7" s="137" t="inlineStr"/>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>manual:no_ads_source</t>
+          <t>manual:no_ads_source;crm:stale</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>14.5681581685744</v>
+        <v>16.64932362122789</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>7.431841831425601</v>
+        <v>5.350676378772114</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>451.6129032258065</v>
+        <v>516.1290322580645</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>632.053009</v>
+        <v>684.37487</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>180.4401057741935</v>
+        <v>168.2458377419355</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>0.3995459484999999</v>
+        <v>0.325976310625</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>28.72968222727273</v>
+        <v>31.10794863636364</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>-2.270317772727275</v>
+        <v>0.1079486363636341</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3280,7 +3280,7 @@
       <c r="AD8" s="137" t="inlineStr"/>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>24.41150828247602</v>
+        <v>27.89886660854403</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-4.411508282476024</v>
+        <v>-7.898866608544029</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>903.2258064516128</v>
+        <v>1032.258064516129</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>944.880274</v>
+        <v>1071.079165</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>41.65446754838706</v>
+        <v>38.82110048387108</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.0461174462142856</v>
+        <v>0.0376079410937501</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>47.2440137</v>
+        <v>53.55395825000001</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>10.2440137</v>
+        <v>16.55395825000001</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3387,7 +3387,7 @@
       <c r="AD9" s="137" t="inlineStr"/>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>1.946607341490545</v>
+        <v>2.224694104560623</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>0.0533926585094546</v>
+        <v>-0.2246941045606232</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>112.9032258064516</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>118.181522</v>
+        <v>135.328689</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>5.278296193548385</v>
+        <v>6.296430935483869</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0467506234285714</v>
+        <v>0.0487973397499999</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>59.090761</v>
+        <v>67.6643445</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>1.090761</v>
+        <v>9.6643445</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3494,7 +3494,7 @@
       <c r="AD10" s="137" t="inlineStr"/>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,28 +3563,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.7056451612903225</v>
+        <v>0.8064516129032258</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>0.2943548387096775</v>
+        <v>0.1935483870967742</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>112.9032258064516</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="V11" s="135" t="n">
         <v>19.26</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-93.6432258064516</v>
+        <v>-109.7722580645161</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.8294114285714286</v>
+        <v>-0.8507349999999999</v>
       </c>
       <c r="Y11" s="135" t="n">
         <v>19.26</v>
@@ -3601,7 +3601,7 @@
       <c r="AD11" s="137" t="inlineStr"/>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>65.36502546689303</v>
+        <v>74.70288624787776</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>26.63497453310697</v>
+        <v>17.29711375212224</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>1241.935483870968</v>
+        <v>1419.354838709677</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>1268</v>
+        <v>1425.51</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>26.06451612903243</v>
+        <v>6.155161290322667</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.0209870129870131</v>
+        <v>0.0043365909090909</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>13.78260869565217</v>
+        <v>15.49467391304348</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>-5.217391304347826</v>
+        <v>-3.505326086956522</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3708,7 +3708,7 @@
       <c r="AD12" s="137" t="inlineStr"/>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>3.763440860215054</v>
+        <v>4.301075268817205</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>3.236559139784946</v>
+        <v>2.698924731182795</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>112.9032258064516</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>69.06999999999999</v>
+        <v>79.87</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-43.83322580645162</v>
+        <v>-49.16225806451613</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3882371428571429</v>
+        <v>-0.3810074999999999</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>9.867142857142856</v>
+        <v>11.41</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-20.13285714285714</v>
+        <v>-18.59</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3815,7 +3815,7 @@
       <c r="AD13" s="137" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.254480286738351</v>
+        <v>1.433691756272401</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-1.254480286738351</v>
+        <v>-1.433691756272401</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>112.9032258064516</v>
+        <v>129.0322580645161</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>68.09</v>
+        <v>80.66</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-44.81322580645161</v>
+        <v>-48.37225806451613</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3969171428571428</v>
+        <v>-0.374885</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3915,7 +3915,7 @@
       <c r="AD14" s="137" t="inlineStr"/>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>28.2258064516129</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-9.225806451612904</v>
+        <v>-13.25806451612903</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>338.7096774193549</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>444.285041</v>
+        <v>490.919982</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>105.5753635806451</v>
+        <v>103.8232078064516</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>0.3116986924761902</v>
+        <v>0.2682099534999999</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>23.38342321052632</v>
+        <v>25.83789378947369</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>11.38342321052631</v>
+        <v>13.83789378947369</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4022,7 +4022,7 @@
       <c r="AD15" s="137" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>google:ok</t>
+          <t>google:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>9.817671809256662</v>
+        <v>11.22019635343618</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-6.817671809256662</v>
+        <v>-8.220196353436185</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>225.8064516129032</v>
+        <v>258.0645161290323</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>188.48</v>
+        <v>213.81</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-37.32645161290324</v>
+        <v>-44.25451612903225</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.1653028571428572</v>
+        <v>-0.1714862499999999</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>62.82666666666666</v>
+        <v>71.27</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>39.82666666666666</v>
+        <v>48.27</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4124,7 +4124,7 @@
       <c r="AD16" s="137" t="inlineStr"/>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>meta:ok</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,41 +4180,41 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>97.14928732183046</v>
+        <v>111.0277569392348</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>18.85071267816954</v>
+        <v>4.972243060765194</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>4177.419354838709</v>
+        <v>4774.193548387097</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>4088.123763</v>
+        <v>4744.939822</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-89.29559183870924</v>
+        <v>-29.25372638709632</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0213757787413126</v>
+        <v>-0.0061274697162161</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>35.24244623275862</v>
+        <v>40.90465363793104</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>-7.757553767241376</v>
+        <v>-2.095346362068966</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
       <c r="AD17" s="137" t="inlineStr"/>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,41 +4265,41 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>150.0583438285473</v>
+        <v>171.4952500897683</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>15.94165617145271</v>
+        <v>-5.495250089768348</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>3612.903225806452</v>
+        <v>4129.032258064516</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>3752.299846</v>
+        <v>4200.812706</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>139.3966201935482</v>
+        <v>71.78044793548361</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>0.0385829930892856</v>
+        <v>0.0173843272343749</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>22.60421593975904</v>
+        <v>25.30610063855422</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>-1.472440736756464</v>
+        <v>1.229443962038715</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
       <c r="AD18" s="137" t="inlineStr"/>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4384,7 +4384,7 @@
       <c r="AD19" s="137" t="inlineStr"/>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>success</t>
+          <t>success;crm:stale</t>
         </is>
       </c>
     </row>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,41 +4435,41 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>497.3120588863844</v>
+        <v>532.6274347650099</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-17.31205888638442</v>
+        <v>-52.62743476500987</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>9814.132104454686</v>
+        <v>10927.03533026114</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>9447.223609000001</v>
+        <v>10552.552528</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-366.9084954546852</v>
+        <v>-374.4828022611364</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.0373857302458913</v>
+        <v>-0.0342712173011878</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>19.68171585208334</v>
+        <v>21.98448443333333</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>-0.3628927369542474</v>
+        <v>1.939875844295749</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
       <c r="AD20" s="137" t="inlineStr"/>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>partial;crm:stale</t>
         </is>
       </c>
     </row>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46242.29189814815</v>
+        <v>46243.29188657407</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-10
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 08/08/2026  |  Ultimo aggiornamento: 09/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 09/08/2026  |  Ultimo aggiornamento: 10/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>2064.516129032258</v>
+        <v>2322.58064516129</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>2099.164782</v>
+        <v>2358.145757</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>34.64865296774178</v>
+        <v>35.56511183870953</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0167829412812499</v>
+        <v>0.015312756486111</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>258.0645161290323</v>
+        <v>290.3225806451613</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>256.14504</v>
+        <v>288.417943</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>-1.919476129032262</v>
+        <v>-1.904637645161301</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>-0.00743797</v>
+        <v>-0.0065604185555555</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>2451.612903225806</v>
+        <v>2758.064516129032</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>2389.63</v>
+        <v>2674.78</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-61.98290322580624</v>
+        <v>-83.284516129032</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0252824999999999</v>
+        <v>-0.0301967251461987</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>111.0277569392348</v>
+        <v>124.9062265566392</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>4.972243060765194</v>
+        <v>-8.906226556639155</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>4774.193548387097</v>
+        <v>5370.967741935484</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>4744.939822</v>
+        <v>5321.3437</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-29.25372638709632</v>
+        <v>-49.62404193548355</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0061274697162161</v>
+        <v>-0.009239311111111001</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>40.90465363793104</v>
+        <v>45.8736525862069</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>-2.095346362068966</v>
+        <v>2.873652586206902</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>16.64932362122789</v>
+        <v>18.73048907388137</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>5.350676378772114</v>
+        <v>3.269510926118627</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>516.1290322580645</v>
+        <v>580.6451612903226</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>684.37487</v>
+        <v>737.770342</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>168.2458377419355</v>
+        <v>157.1251807096775</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.325976310625</v>
+        <v>0.270604477888889</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>31.10794863636364</v>
+        <v>33.53501554545455</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>0.1079486363636341</v>
+        <v>2.535015545454549</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>27.89886660854403</v>
+        <v>31.38622493461203</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-7.898866608544029</v>
+        <v>-11.38622493461203</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>1032.258064516129</v>
+        <v>1161.290322580645</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>1071.079165</v>
+        <v>1203.648603</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>38.82110048387108</v>
+        <v>42.35828041935497</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>0.0376079410937501</v>
+        <v>0.0364751859166667</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>53.55395825000001</v>
+        <v>60.18243015</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>16.55395825000001</v>
+        <v>23.18243015</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>2.224694104560623</v>
+        <v>2.502780867630701</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-0.2246941045606232</v>
+        <v>-0.5027808676307011</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>129.0322580645161</v>
+        <v>145.1612903225806</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>135.328689</v>
+        <v>152.627791</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>6.296430935483869</v>
+        <v>7.466500677419361</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0487973397499999</v>
+        <v>0.0514358935555556</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>67.6643445</v>
+        <v>76.3138955</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>9.6643445</v>
+        <v>18.3138955</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,28 +1540,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>0.8064516129032258</v>
+        <v>0.907258064516129</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>0.1935483870967742</v>
+        <v>0.092741935483871</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>129.0322580645161</v>
+        <v>145.1612903225806</v>
       </c>
       <c r="R12" s="117" t="n">
         <v>19.26</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-109.7722580645161</v>
+        <v>-125.9012903225806</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.8507349999999999</v>
+        <v>-0.86732</v>
       </c>
       <c r="U12" s="117" t="n">
         <v>19.26</v>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>74.70288624787776</v>
+        <v>84.04074702886248</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>17.29711375212224</v>
+        <v>7.959252971137516</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>1419.354838709677</v>
+        <v>1596.774193548387</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>1425.51</v>
+        <v>1622.82</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>6.155161290322667</v>
+        <v>26.04580645161286</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.0043365909090909</v>
+        <v>0.0163115151515151</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>15.49467391304348</v>
+        <v>17.63934782608695</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>-3.505326086956522</v>
+        <v>-1.360652173913045</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>4.301075268817205</v>
+        <v>4.838709677419356</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>2.698924731182795</v>
+        <v>2.161290322580644</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>129.0322580645161</v>
+        <v>145.1612903225806</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>79.87</v>
+        <v>92.20999999999999</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-49.16225806451613</v>
+        <v>-52.95129032258065</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3810074999999999</v>
+        <v>-0.3647755555555556</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>11.41</v>
+        <v>13.17285714285714</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-18.59</v>
+        <v>-16.82714285714286</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>1.433691756272401</v>
+        <v>1.612903225806452</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-1.433691756272401</v>
+        <v>-1.612903225806452</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>129.0322580645161</v>
+        <v>145.1612903225806</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>80.66</v>
+        <v>93</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-48.37225806451613</v>
+        <v>-52.16129032258064</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.374885</v>
+        <v>-0.3593333333333333</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>32.25806451612903</v>
+        <v>36.29032258064516</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-13.25806451612903</v>
+        <v>-17.29032258064516</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>387.0967741935484</v>
+        <v>435.483870967742</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>490.919982</v>
+        <v>527.797274</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>103.8232078064516</v>
+        <v>92.31340303225808</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.2682099534999999</v>
+        <v>0.2119789254814814</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>25.83789378947369</v>
+        <v>27.77880389473684</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>13.83789378947369</v>
+        <v>15.77880389473684</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>11.22019635343618</v>
+        <v>12.62272089761571</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-8.220196353436185</v>
+        <v>-9.622720897615707</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>258.0645161290323</v>
+        <v>290.3225806451613</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>213.81</v>
+        <v>247.39</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-44.25451612903225</v>
+        <v>-42.93258064516129</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.1714862499999999</v>
+        <v>-0.1478788888888889</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>71.27</v>
+        <v>82.46333333333332</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>48.27</v>
+        <v>59.46333333333333</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>171.4952500897683</v>
+        <v>192.9321563509894</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-5.495250089768348</v>
+        <v>-26.9321563509894</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>4129.032258064516</v>
+        <v>4645.16129032258</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>4200.812706</v>
+        <v>4696.52401</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>71.78044793548361</v>
+        <v>51.36271967741959</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>0.0173843272343749</v>
+        <v>0.0110572521527778</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>25.30610063855422</v>
+        <v>28.29231331325301</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>1.229443962038715</v>
+        <v>4.21565663673751</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>532.6274347650099</v>
+        <v>567.9428106436353</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-52.62743476500987</v>
+        <v>-87.94281064363531</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>10927.03533026114</v>
+        <v>12039.93855606759</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>10552.552528</v>
+        <v>11624.66771</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-374.4828022611364</v>
+        <v>-415.2708460675876</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.0342712173011878</v>
+        <v>-0.0344911100778259</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>21.98448443333333</v>
+        <v>24.21805772916667</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>1.939875844295749</v>
+        <v>4.173449140129083</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>2064.516129032258</v>
+        <v>2322.58064516129</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>2099.164782</v>
+        <v>2358.145757</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>34.64865296774178</v>
+        <v>35.56511183870953</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0167829412812499</v>
+        <v>0.015312756486111</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>258.0645161290323</v>
+        <v>290.3225806451613</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>256.14504</v>
+        <v>288.417943</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>-1.919476129032262</v>
+        <v>-1.904637645161301</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>-0.00743797</v>
+        <v>-0.0065604185555555</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>2451.612903225806</v>
+        <v>2758.064516129032</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>2389.63</v>
+        <v>2674.78</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-61.98290322580624</v>
+        <v>-83.284516129032</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0252824999999999</v>
+        <v>-0.0301967251461987</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>16.64932362122789</v>
+        <v>18.73048907388137</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>5.350676378772114</v>
+        <v>3.269510926118627</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>516.1290322580645</v>
+        <v>580.6451612903226</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>684.37487</v>
+        <v>737.770342</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>168.2458377419355</v>
+        <v>157.1251807096775</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>0.325976310625</v>
+        <v>0.270604477888889</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>31.10794863636364</v>
+        <v>33.53501554545455</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>0.1079486363636341</v>
+        <v>2.535015545454549</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>27.89886660854403</v>
+        <v>31.38622493461203</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-7.898866608544029</v>
+        <v>-11.38622493461203</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>1032.258064516129</v>
+        <v>1161.290322580645</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>1071.079165</v>
+        <v>1203.648603</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>38.82110048387108</v>
+        <v>42.35828041935497</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.0376079410937501</v>
+        <v>0.0364751859166667</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>53.55395825000001</v>
+        <v>60.18243015</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>16.55395825000001</v>
+        <v>23.18243015</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>2.224694104560623</v>
+        <v>2.502780867630701</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-0.2246941045606232</v>
+        <v>-0.5027808676307011</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>129.0322580645161</v>
+        <v>145.1612903225806</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>135.328689</v>
+        <v>152.627791</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>6.296430935483869</v>
+        <v>7.466500677419361</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0487973397499999</v>
+        <v>0.0514358935555556</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>67.6643445</v>
+        <v>76.3138955</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>9.6643445</v>
+        <v>18.3138955</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,28 +3563,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.8064516129032258</v>
+        <v>0.907258064516129</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>0.1935483870967742</v>
+        <v>0.092741935483871</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>129.0322580645161</v>
+        <v>145.1612903225806</v>
       </c>
       <c r="V11" s="135" t="n">
         <v>19.26</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-109.7722580645161</v>
+        <v>-125.9012903225806</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.8507349999999999</v>
+        <v>-0.86732</v>
       </c>
       <c r="Y11" s="135" t="n">
         <v>19.26</v>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>74.70288624787776</v>
+        <v>84.04074702886248</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>17.29711375212224</v>
+        <v>7.959252971137516</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>1419.354838709677</v>
+        <v>1596.774193548387</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>1425.51</v>
+        <v>1622.82</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>6.155161290322667</v>
+        <v>26.04580645161286</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.0043365909090909</v>
+        <v>0.0163115151515151</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>15.49467391304348</v>
+        <v>17.63934782608695</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>-3.505326086956522</v>
+        <v>-1.360652173913045</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.301075268817205</v>
+        <v>4.838709677419356</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>2.698924731182795</v>
+        <v>2.161290322580644</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>129.0322580645161</v>
+        <v>145.1612903225806</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>79.87</v>
+        <v>92.20999999999999</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-49.16225806451613</v>
+        <v>-52.95129032258065</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3810074999999999</v>
+        <v>-0.3647755555555556</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>11.41</v>
+        <v>13.17285714285714</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-18.59</v>
+        <v>-16.82714285714286</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.433691756272401</v>
+        <v>1.612903225806452</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-1.433691756272401</v>
+        <v>-1.612903225806452</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>129.0322580645161</v>
+        <v>145.1612903225806</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>80.66</v>
+        <v>93</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-48.37225806451613</v>
+        <v>-52.16129032258064</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.374885</v>
+        <v>-0.3593333333333333</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>32.25806451612903</v>
+        <v>36.29032258064516</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-13.25806451612903</v>
+        <v>-17.29032258064516</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>387.0967741935484</v>
+        <v>435.483870967742</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>490.919982</v>
+        <v>527.797274</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>103.8232078064516</v>
+        <v>92.31340303225808</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>0.2682099534999999</v>
+        <v>0.2119789254814814</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>25.83789378947369</v>
+        <v>27.77880389473684</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>13.83789378947369</v>
+        <v>15.77880389473684</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>11.22019635343618</v>
+        <v>12.62272089761571</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-8.220196353436185</v>
+        <v>-9.622720897615707</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>258.0645161290323</v>
+        <v>290.3225806451613</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>213.81</v>
+        <v>247.39</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-44.25451612903225</v>
+        <v>-42.93258064516129</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.1714862499999999</v>
+        <v>-0.1478788888888889</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>71.27</v>
+        <v>82.46333333333332</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>48.27</v>
+        <v>59.46333333333333</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>111.0277569392348</v>
+        <v>124.9062265566392</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>4.972243060765194</v>
+        <v>-8.906226556639155</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>4774.193548387097</v>
+        <v>5370.967741935484</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>4744.939822</v>
+        <v>5321.3437</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-29.25372638709632</v>
+        <v>-49.62404193548355</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0061274697162161</v>
+        <v>-0.009239311111111001</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>40.90465363793104</v>
+        <v>45.8736525862069</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>-2.095346362068966</v>
+        <v>2.873652586206902</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>171.4952500897683</v>
+        <v>192.9321563509894</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-5.495250089768348</v>
+        <v>-26.9321563509894</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>4129.032258064516</v>
+        <v>4645.16129032258</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>4200.812706</v>
+        <v>4696.52401</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>71.78044793548361</v>
+        <v>51.36271967741959</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>0.0173843272343749</v>
+        <v>0.0110572521527778</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>25.30610063855422</v>
+        <v>28.29231331325301</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>1.229443962038715</v>
+        <v>4.21565663673751</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>532.6274347650099</v>
+        <v>567.9428106436353</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-52.62743476500987</v>
+        <v>-87.94281064363531</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>10927.03533026114</v>
+        <v>12039.93855606759</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>10552.552528</v>
+        <v>11624.66771</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-374.4828022611364</v>
+        <v>-415.2708460675876</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.0342712173011878</v>
+        <v>-0.0344911100778259</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>21.98448443333333</v>
+        <v>24.21805772916667</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>1.939875844295749</v>
+        <v>4.173449140129083</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46242</v>
+        <v>46243</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46243.29188657407</v>
+        <v>46244.291875</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-11
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 09/08/2026  |  Ultimo aggiornamento: 10/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 10/08/2026  |  Ultimo aggiornamento: 11/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>2322.58064516129</v>
+        <v>2580.645161290322</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>2358.145757</v>
+        <v>2619.282731</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>35.56511183870953</v>
+        <v>38.63756970967734</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.015312756486111</v>
+        <v>0.0149720582624999</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>290.3225806451613</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>288.417943</v>
+        <v>330.648205</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>-1.904637645161301</v>
+        <v>8.067559838709712</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>-0.0065604185555555</v>
+        <v>0.0250094355000001</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>2758.064516129032</v>
+        <v>3064.516129032258</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>2674.78</v>
+        <v>3001.42</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-83.284516129032</v>
+        <v>-63.09612903225798</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0301967251461987</v>
+        <v>-0.0205892631578947</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>124.9062265566392</v>
+        <v>138.7846961740435</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-8.906226556639155</v>
+        <v>-22.78469617404352</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>5370.967741935484</v>
+        <v>5967.741935483871</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>5321.3437</v>
+        <v>5951.350936</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-49.62404193548355</v>
+        <v>-16.39099948387138</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.009239311111111001</v>
+        <v>-0.0027465999135135</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>45.8736525862069</v>
+        <v>51.30474944827586</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>2.873652586206902</v>
+        <v>8.304749448275864</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>18.73048907388137</v>
+        <v>20.81165452653486</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>3.269510926118627</v>
+        <v>1.188345473465141</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>580.6451612903226</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>737.770342</v>
+        <v>789.936725</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>157.1251807096775</v>
+        <v>144.7754346774194</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.270604477888889</v>
+        <v>0.2244019237500001</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>33.53501554545455</v>
+        <v>35.90621477272727</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>2.535015545454549</v>
+        <v>4.906214772727274</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>31.38622493461203</v>
+        <v>34.87358326068004</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-11.38622493461203</v>
+        <v>-14.87358326068004</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>1161.290322580645</v>
+        <v>1290.322580645161</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>1203.648603</v>
+        <v>1334.840728</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>42.35828041935497</v>
+        <v>44.51814735483868</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>0.0364751859166667</v>
+        <v>0.0345015641999999</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>60.18243015</v>
+        <v>66.74203639999999</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>23.18243015</v>
+        <v>29.74203639999999</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>2.502780867630701</v>
+        <v>2.780867630700779</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-0.5027808676307011</v>
+        <v>-0.7808676307007789</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>145.1612903225806</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>152.627791</v>
+        <v>169.607791</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>7.466500677419361</v>
+        <v>8.317468419354839</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0514358935555556</v>
+        <v>0.0515683042</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>76.3138955</v>
+        <v>84.8038955</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>18.3138955</v>
+        <v>26.8038955</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,34 +1540,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>0.907258064516129</v>
+        <v>1.008064516129032</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>0.092741935483871</v>
+        <v>-0.008064516129032201</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>145.1612903225806</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>19.26</v>
+        <v>47.27</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-125.9012903225806</v>
+        <v>-114.0203225806451</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.86732</v>
+        <v>-0.7069259999999999</v>
       </c>
       <c r="U12" s="117" t="n">
-        <v>19.26</v>
+        <v>47.27</v>
       </c>
       <c r="V12" s="117" t="n">
-        <v>-140.74</v>
+        <v>-112.73</v>
       </c>
       <c r="W12" s="120" t="inlineStr"/>
     </row>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>84.04074702886248</v>
+        <v>93.3786078098472</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>7.959252971137516</v>
+        <v>-1.378607809847196</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>1596.774193548387</v>
+        <v>1774.193548387097</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>1622.82</v>
+        <v>1820.29</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>26.04580645161286</v>
+        <v>46.09645161290337</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.0163115151515151</v>
+        <v>0.0259816363636364</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>17.63934782608695</v>
+        <v>19.78576086956522</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>-1.360652173913045</v>
+        <v>0.7857608695652161</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>4.838709677419356</v>
+        <v>5.376344086021506</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>2.161290322580644</v>
+        <v>1.623655913978494</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>145.1612903225806</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>92.20999999999999</v>
+        <v>103.51</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-52.95129032258065</v>
+        <v>-57.78032258064515</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3647755555555556</v>
+        <v>-0.3582379999999999</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>13.17285714285714</v>
+        <v>14.78714285714286</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-16.82714285714286</v>
+        <v>-15.21285714285714</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>1.612903225806452</v>
+        <v>1.792114695340502</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-1.612903225806452</v>
+        <v>-1.792114695340502</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>145.1612903225806</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>93</v>
+        <v>102.45</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-52.16129032258064</v>
+        <v>-58.84032258064515</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3593333333333333</v>
+        <v>-0.3648099999999999</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>36.29032258064516</v>
+        <v>40.32258064516129</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-17.29032258064516</v>
+        <v>-21.32258064516129</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>435.483870967742</v>
+        <v>483.8709677419355</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>527.797274</v>
+        <v>566.95176</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>92.31340303225808</v>
+        <v>83.08079225806455</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.2119789254814814</v>
+        <v>0.171700304</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>27.77880389473684</v>
+        <v>29.83956631578948</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>15.77880389473684</v>
+        <v>17.83956631578948</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>12.62272089761571</v>
+        <v>14.02524544179523</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-9.622720897615707</v>
+        <v>-11.02524544179523</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>290.3225806451613</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>247.39</v>
+        <v>282.35</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-42.93258064516129</v>
+        <v>-40.23064516129028</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.1478788888888889</v>
+        <v>-0.1247149999999998</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>82.46333333333332</v>
+        <v>94.11666666666667</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>59.46333333333333</v>
+        <v>71.11666666666667</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>192.9321563509894</v>
+        <v>214.3690626122104</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-26.9321563509894</v>
+        <v>-48.36906261221043</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>4645.16129032258</v>
+        <v>5161.290322580645</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>4696.52401</v>
+        <v>5217.207004</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>51.36271967741959</v>
+        <v>55.91668141935497</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>0.0110572521527778</v>
+        <v>0.010833857025</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>28.29231331325301</v>
+        <v>31.42895785542169</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>4.21565663673751</v>
+        <v>7.352301178906185</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2063,28 +2063,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>140.9774436090226</v>
+        <v>169.1729323308271</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>93</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-47.97744360902257</v>
+        <v>-76.17293233082711</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>1071.428571428571</v>
+        <v>1285.714285714286</v>
       </c>
       <c r="R19" s="117" t="n">
         <v>706.8</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-364.6285714285714</v>
+        <v>-578.9142857142858</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.3403199999999999</v>
+        <v>-0.4502666666666667</v>
       </c>
       <c r="U19" s="117" t="n">
         <v>7.6</v>
@@ -2138,28 +2138,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>79.36507936507935</v>
+        <v>95.23809523809524</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>60</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-19.36507936507936</v>
+        <v>-35.23809523809523</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>714.2857142857143</v>
+        <v>857.1428571428571</v>
       </c>
       <c r="R20" s="117" t="n">
         <v>540</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-174.2857142857143</v>
+        <v>-317.1428571428571</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.244</v>
+        <v>-0.37</v>
       </c>
       <c r="U20" s="117" t="n">
         <v>9</v>
@@ -2213,28 +2213,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>29.76190476190476</v>
+        <v>35.71428571428572</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>15.23809523809524</v>
+        <v>9.285714285714285</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>238.0952380952381</v>
+        <v>285.7142857142857</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>360</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>121.9047619047619</v>
+        <v>74.28571428571428</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>0.512</v>
+        <v>0.2599999999999999</v>
       </c>
       <c r="U21" s="117" t="n">
         <v>8</v>
@@ -2276,28 +2276,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>250.1044277360067</v>
+        <v>300.125313283208</v>
       </c>
       <c r="N22" s="125" t="n">
         <v>198</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-52.1044277360067</v>
+        <v>-102.1253132832081</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="Q22" s="123" t="n">
-        <v>2023.809523809524</v>
+        <v>2428.571428571428</v>
       </c>
       <c r="R22" s="123" t="n">
         <v>1606.8</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-417.0095238095239</v>
+        <v>-821.7714285714285</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-0.2060517647058823</v>
+        <v>-0.3383764705882353</v>
       </c>
       <c r="U22" s="123" t="n">
         <v>8.115151515151515</v>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>567.9428106436353</v>
+        <v>653.279072069462</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-87.94281064363531</v>
+        <v>-173.279072069462</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>12039.93855606759</v>
+        <v>13557.60368663594</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>11624.66771</v>
+        <v>12775.35794</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-415.2708460675876</v>
+        <v>-782.2457466359447</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.0344911100778259</v>
+        <v>-0.0576979357647858</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>24.21805772916667</v>
+        <v>26.61532904166667</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>4.173449140129083</v>
+        <v>6.570720452629082</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>2322.58064516129</v>
+        <v>2580.645161290322</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>2358.145757</v>
+        <v>2619.282731</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>35.56511183870953</v>
+        <v>38.63756970967734</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.015312756486111</v>
+        <v>0.0149720582624999</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>290.3225806451613</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>288.417943</v>
+        <v>330.648205</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>-1.904637645161301</v>
+        <v>8.067559838709712</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>-0.0065604185555555</v>
+        <v>0.0250094355000001</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>2758.064516129032</v>
+        <v>3064.516129032258</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>2674.78</v>
+        <v>3001.42</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-83.284516129032</v>
+        <v>-63.09612903225798</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0301967251461987</v>
+        <v>-0.0205892631578947</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2933,28 +2933,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>140.9774436090226</v>
+        <v>169.1729323308271</v>
       </c>
       <c r="R5" t="n">
         <v>93</v>
       </c>
       <c r="S5" t="n">
-        <v>-47.97744360902257</v>
+        <v>-76.17293233082711</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="U5" s="135" t="n">
-        <v>1071.428571428571</v>
+        <v>1285.714285714286</v>
       </c>
       <c r="V5" s="135" t="n">
         <v>706.8</v>
       </c>
       <c r="W5" s="135" t="n">
-        <v>-364.6285714285714</v>
+        <v>-578.9142857142858</v>
       </c>
       <c r="X5" s="136" t="n">
-        <v>-0.3403199999999999</v>
+        <v>-0.4502666666666667</v>
       </c>
       <c r="Y5" s="135" t="n">
         <v>7.6</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3036,28 +3036,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>79.36507936507935</v>
+        <v>95.23809523809524</v>
       </c>
       <c r="R6" t="n">
         <v>60</v>
       </c>
       <c r="S6" t="n">
-        <v>-19.36507936507936</v>
+        <v>-35.23809523809523</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>714.2857142857143</v>
+        <v>857.1428571428571</v>
       </c>
       <c r="V6" s="135" t="n">
         <v>540</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-174.2857142857143</v>
+        <v>-317.1428571428571</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.244</v>
+        <v>-0.37</v>
       </c>
       <c r="Y6" s="135" t="n">
         <v>9</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3139,28 +3139,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>29.76190476190476</v>
+        <v>35.71428571428572</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>15.23809523809524</v>
+        <v>9.285714285714285</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>238.0952380952381</v>
+        <v>285.7142857142857</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>360</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>121.9047619047619</v>
+        <v>74.28571428571428</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>0.512</v>
+        <v>0.2599999999999999</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>8</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>18.73048907388137</v>
+        <v>20.81165452653486</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>3.269510926118627</v>
+        <v>1.188345473465141</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>580.6451612903226</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>737.770342</v>
+        <v>789.936725</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>157.1251807096775</v>
+        <v>144.7754346774194</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>0.270604477888889</v>
+        <v>0.2244019237500001</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>33.53501554545455</v>
+        <v>35.90621477272727</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>2.535015545454549</v>
+        <v>4.906214772727274</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>31.38622493461203</v>
+        <v>34.87358326068004</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-11.38622493461203</v>
+        <v>-14.87358326068004</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>1161.290322580645</v>
+        <v>1290.322580645161</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>1203.648603</v>
+        <v>1334.840728</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>42.35828041935497</v>
+        <v>44.51814735483868</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.0364751859166667</v>
+        <v>0.0345015641999999</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>60.18243015</v>
+        <v>66.74203639999999</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>23.18243015</v>
+        <v>29.74203639999999</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>2.502780867630701</v>
+        <v>2.780867630700779</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-0.5027808676307011</v>
+        <v>-0.7808676307007789</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>145.1612903225806</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>152.627791</v>
+        <v>169.607791</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>7.466500677419361</v>
+        <v>8.317468419354839</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0514358935555556</v>
+        <v>0.0515683042</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>76.3138955</v>
+        <v>84.8038955</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>18.3138955</v>
+        <v>26.8038955</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,34 +3563,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.907258064516129</v>
+        <v>1.008064516129032</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>0.092741935483871</v>
+        <v>-0.008064516129032201</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>145.1612903225806</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="V11" s="135" t="n">
-        <v>19.26</v>
+        <v>47.27</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-125.9012903225806</v>
+        <v>-114.0203225806451</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.86732</v>
+        <v>-0.7069259999999999</v>
       </c>
       <c r="Y11" s="135" t="n">
-        <v>19.26</v>
+        <v>47.27</v>
       </c>
       <c r="Z11" s="135" t="n">
-        <v>-140.74</v>
+        <v>-112.73</v>
       </c>
       <c r="AB11" s="137" t="inlineStr">
         <is>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>84.04074702886248</v>
+        <v>93.3786078098472</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>7.959252971137516</v>
+        <v>-1.378607809847196</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>1596.774193548387</v>
+        <v>1774.193548387097</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>1622.82</v>
+        <v>1820.29</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>26.04580645161286</v>
+        <v>46.09645161290337</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.0163115151515151</v>
+        <v>0.0259816363636364</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>17.63934782608695</v>
+        <v>19.78576086956522</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>-1.360652173913045</v>
+        <v>0.7857608695652161</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.838709677419356</v>
+        <v>5.376344086021506</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>2.161290322580644</v>
+        <v>1.623655913978494</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>145.1612903225806</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>92.20999999999999</v>
+        <v>103.51</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-52.95129032258065</v>
+        <v>-57.78032258064515</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3647755555555556</v>
+        <v>-0.3582379999999999</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>13.17285714285714</v>
+        <v>14.78714285714286</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-16.82714285714286</v>
+        <v>-15.21285714285714</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.612903225806452</v>
+        <v>1.792114695340502</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-1.612903225806452</v>
+        <v>-1.792114695340502</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>145.1612903225806</v>
+        <v>161.2903225806452</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>93</v>
+        <v>102.45</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-52.16129032258064</v>
+        <v>-58.84032258064515</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3593333333333333</v>
+        <v>-0.3648099999999999</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>36.29032258064516</v>
+        <v>40.32258064516129</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-17.29032258064516</v>
+        <v>-21.32258064516129</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>435.483870967742</v>
+        <v>483.8709677419355</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>527.797274</v>
+        <v>566.95176</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>92.31340303225808</v>
+        <v>83.08079225806455</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>0.2119789254814814</v>
+        <v>0.171700304</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>27.77880389473684</v>
+        <v>29.83956631578948</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>15.77880389473684</v>
+        <v>17.83956631578948</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>12.62272089761571</v>
+        <v>14.02524544179523</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-9.622720897615707</v>
+        <v>-11.02524544179523</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>290.3225806451613</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>247.39</v>
+        <v>282.35</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-42.93258064516129</v>
+        <v>-40.23064516129028</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.1478788888888889</v>
+        <v>-0.1247149999999998</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>82.46333333333332</v>
+        <v>94.11666666666667</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>59.46333333333333</v>
+        <v>71.11666666666667</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>124.9062265566392</v>
+        <v>138.7846961740435</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-8.906226556639155</v>
+        <v>-22.78469617404352</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>5370.967741935484</v>
+        <v>5967.741935483871</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>5321.3437</v>
+        <v>5951.350936</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-49.62404193548355</v>
+        <v>-16.39099948387138</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.009239311111111001</v>
+        <v>-0.0027465999135135</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>45.8736525862069</v>
+        <v>51.30474944827586</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>2.873652586206902</v>
+        <v>8.304749448275864</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>192.9321563509894</v>
+        <v>214.3690626122104</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-26.9321563509894</v>
+        <v>-48.36906261221043</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>4645.16129032258</v>
+        <v>5161.290322580645</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>4696.52401</v>
+        <v>5217.207004</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>51.36271967741959</v>
+        <v>55.91668141935497</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>0.0110572521527778</v>
+        <v>0.010833857025</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>28.29231331325301</v>
+        <v>31.42895785542169</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>4.21565663673751</v>
+        <v>7.352301178906185</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4350,28 +4350,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>250.1044277360067</v>
+        <v>300.125313283208</v>
       </c>
       <c r="R19" t="n">
         <v>198</v>
       </c>
       <c r="S19" t="n">
-        <v>-52.1044277360067</v>
+        <v>-102.1253132832081</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>2023.809523809524</v>
+        <v>2428.571428571428</v>
       </c>
       <c r="V19" s="135" t="n">
         <v>1606.8</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-417.0095238095239</v>
+        <v>-821.7714285714285</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.2060517647058823</v>
+        <v>-0.3383764705882353</v>
       </c>
       <c r="Y19" s="135" t="n">
         <v>8.115151515151515</v>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>567.9428106436353</v>
+        <v>653.279072069462</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-87.94281064363531</v>
+        <v>-173.279072069462</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>12039.93855606759</v>
+        <v>13557.60368663594</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>11624.66771</v>
+        <v>12775.35794</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-415.2708460675876</v>
+        <v>-782.2457466359447</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.0344911100778259</v>
+        <v>-0.0576979357647858</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>24.21805772916667</v>
+        <v>26.61532904166667</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>4.173449140129083</v>
+        <v>6.570720452629082</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46244.291875</v>
+        <v>46245.291875</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-12
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 10/08/2026  |  Ultimo aggiornamento: 11/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 11/08/2026  |  Ultimo aggiornamento: 12/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>2580.645161290322</v>
+        <v>2838.709677419354</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>2619.282731</v>
+        <v>2903.076808</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>38.63756970967734</v>
+        <v>64.36713058064515</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0149720582624999</v>
+        <v>0.0226747846363636</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>322.5806451612903</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>330.648205</v>
+        <v>369.92827</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>8.067559838709712</v>
+        <v>15.08956032258067</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>0.0250094355000001</v>
+        <v>0.0425251245454546</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>3064.516129032258</v>
+        <v>3370.967741935484</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>3001.42</v>
+        <v>3278.19</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-63.09612903225798</v>
+        <v>-92.77774193548385</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0205892631578947</v>
+        <v>-0.0275225837320574</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>138.7846961740435</v>
+        <v>152.6631657914479</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-22.78469617404352</v>
+        <v>-36.66316579144785</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>5967.741935483871</v>
+        <v>6564.516129032258</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>5951.350936</v>
+        <v>6551.195078</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-16.39099948387138</v>
+        <v>-13.32105103225786</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0027465999135135</v>
+        <v>-0.0020292510171989</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>51.30474944827586</v>
+        <v>56.47581963793103</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>8.304749448275864</v>
+        <v>13.47581963793103</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>20.81165452653486</v>
+        <v>22.89281997918835</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>1.188345473465141</v>
+        <v>-0.8928199791883422</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>645.1612903225806</v>
+        <v>709.6774193548387</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>789.936725</v>
+        <v>843.0790950000001</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>144.7754346774194</v>
+        <v>133.4016756451614</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.2244019237500001</v>
+        <v>0.187975088409091</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>35.90621477272727</v>
+        <v>38.32177704545455</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>4.906214772727274</v>
+        <v>7.321777045454546</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>34.87358326068004</v>
+        <v>38.36094158674804</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-14.87358326068004</v>
+        <v>-18.36094158674804</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>1290.322580645161</v>
+        <v>1419.354838709677</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>1334.840728</v>
+        <v>1462.139115</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>44.51814735483868</v>
+        <v>42.78427629032262</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>0.0345015641999999</v>
+        <v>0.0301434673863636</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>66.74203639999999</v>
+        <v>73.10695575</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>29.74203639999999</v>
+        <v>36.10695575</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>2.780867630700779</v>
+        <v>3.058954393770857</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-0.7808676307007789</v>
+        <v>-1.058954393770857</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>161.2903225806452</v>
+        <v>177.4193548387097</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>169.607791</v>
+        <v>184.640047</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>8.317468419354839</v>
+        <v>7.220692161290344</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0515683042</v>
+        <v>0.0406984467272728</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>84.8038955</v>
+        <v>92.3200235</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>26.8038955</v>
+        <v>34.3200235</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,34 +1540,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>1.008064516129032</v>
+        <v>1.108870967741935</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-0.008064516129032201</v>
+        <v>-0.1088709677419355</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>161.2903225806452</v>
+        <v>177.4193548387097</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>47.27</v>
+        <v>59.204384</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-114.0203225806451</v>
+        <v>-118.2149708387097</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.7069259999999999</v>
+        <v>-0.6663025629090908</v>
       </c>
       <c r="U12" s="117" t="n">
-        <v>47.27</v>
+        <v>59.204384</v>
       </c>
       <c r="V12" s="117" t="n">
-        <v>-112.73</v>
+        <v>-100.795616</v>
       </c>
       <c r="W12" s="120" t="inlineStr"/>
     </row>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>93.3786078098472</v>
+        <v>102.7164685908319</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-1.378607809847196</v>
+        <v>-10.71646859083191</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>1774.193548387097</v>
+        <v>1951.612903225806</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>1820.29</v>
+        <v>1999.25</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>46.09645161290337</v>
+        <v>47.63709677419365</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.0259816363636364</v>
+        <v>0.0244090909090909</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>19.78576086956522</v>
+        <v>21.73097826086957</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>0.7857608695652161</v>
+        <v>2.730978260869566</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>5.376344086021506</v>
+        <v>5.913978494623657</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>1.623655913978494</v>
+        <v>1.086021505376343</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>161.2903225806452</v>
+        <v>177.4193548387097</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>103.51</v>
+        <v>114.02</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-57.78032258064515</v>
+        <v>-63.39935483870967</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3582379999999999</v>
+        <v>-0.3573418181818181</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>14.78714285714286</v>
+        <v>16.28857142857143</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-15.21285714285714</v>
+        <v>-13.71142857142857</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>1.792114695340502</v>
+        <v>1.971326164874552</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-1.792114695340502</v>
+        <v>-1.971326164874552</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>161.2903225806452</v>
+        <v>177.4193548387097</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>102.45</v>
+        <v>112.32</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-58.84032258064515</v>
+        <v>-65.09935483870967</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3648099999999999</v>
+        <v>-0.3669236363636363</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>40.32258064516129</v>
+        <v>44.35483870967742</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-21.32258064516129</v>
+        <v>-25.35483870967742</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>483.8709677419355</v>
+        <v>532.258064516129</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>566.95176</v>
+        <v>609.1047150000001</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>83.08079225806455</v>
+        <v>76.84665048387103</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.171700304</v>
+        <v>0.1443785554545456</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>29.83956631578948</v>
+        <v>32.05814289473685</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>17.83956631578948</v>
+        <v>20.05814289473685</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>14.02524544179523</v>
+        <v>15.42776998597475</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-11.02524544179523</v>
+        <v>-12.42776998597475</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>322.5806451612903</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>282.35</v>
+        <v>316.15</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-40.23064516129028</v>
+        <v>-38.68870967741936</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.1247149999999998</v>
+        <v>-0.1090318181818181</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>94.11666666666667</v>
+        <v>105.3833333333333</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>71.11666666666667</v>
+        <v>82.38333333333333</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>214.3690626122104</v>
+        <v>235.8059688734315</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-48.36906261221043</v>
+        <v>-69.80596887343145</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>5161.290322580645</v>
+        <v>5677.419354838709</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>5217.207004</v>
+        <v>5699.907356</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>55.91668141935497</v>
+        <v>22.48800116129041</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>0.010833857025</v>
+        <v>0.00396095475</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>31.42895785542169</v>
+        <v>34.33679130120482</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>7.352301178906185</v>
+        <v>10.26013462468932</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2063,28 +2063,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>169.1729323308271</v>
+        <v>197.3684210526316</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>93</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-76.17293233082711</v>
+        <v>-104.3684210526316</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>1285.714285714286</v>
+        <v>1500</v>
       </c>
       <c r="R19" s="117" t="n">
         <v>706.8</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-578.9142857142858</v>
+        <v>-793.2</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.4502666666666667</v>
+        <v>-0.5288</v>
       </c>
       <c r="U19" s="117" t="n">
         <v>7.6</v>
@@ -2138,28 +2138,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>95.23809523809524</v>
+        <v>111.1111111111111</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>60</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-35.23809523809523</v>
+        <v>-51.1111111111111</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>857.1428571428571</v>
+        <v>1000</v>
       </c>
       <c r="R20" s="117" t="n">
         <v>540</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-317.1428571428571</v>
+        <v>-460</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.37</v>
+        <v>-0.46</v>
       </c>
       <c r="U20" s="117" t="n">
         <v>9</v>
@@ -2213,28 +2213,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>35.71428571428572</v>
+        <v>41.66666666666667</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>9.285714285714285</v>
+        <v>3.333333333333329</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>285.7142857142857</v>
+        <v>333.3333333333334</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>360</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>74.28571428571428</v>
+        <v>26.66666666666663</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>0.2599999999999999</v>
+        <v>0.07999999999999979</v>
       </c>
       <c r="U21" s="117" t="n">
         <v>8</v>
@@ -2276,28 +2276,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>300.125313283208</v>
+        <v>350.1461988304094</v>
       </c>
       <c r="N22" s="125" t="n">
         <v>198</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-102.1253132832081</v>
+        <v>-152.1461988304094</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="Q22" s="123" t="n">
-        <v>2428.571428571428</v>
+        <v>2833.333333333333</v>
       </c>
       <c r="R22" s="123" t="n">
         <v>1606.8</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-821.7714285714285</v>
+        <v>-1226.533333333334</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-0.3383764705882353</v>
+        <v>-0.4328941176470589</v>
       </c>
       <c r="U22" s="123" t="n">
         <v>8.115151515151515</v>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>653.279072069462</v>
+        <v>738.6153334952887</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-173.279072069462</v>
+        <v>-258.6153334952887</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>13557.60368663594</v>
+        <v>15075.2688172043</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>12775.35794</v>
+        <v>13857.902434</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-782.2457466359447</v>
+        <v>-1217.3663832043</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.0576979357647858</v>
+        <v>-0.08075254895720391</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>26.61532904166667</v>
+        <v>28.87063007083333</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>6.570720452629082</v>
+        <v>8.826021481795749</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>2580.645161290322</v>
+        <v>2838.709677419354</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>2619.282731</v>
+        <v>2903.076808</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>38.63756970967734</v>
+        <v>64.36713058064515</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0149720582624999</v>
+        <v>0.0226747846363636</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>322.5806451612903</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>330.648205</v>
+        <v>369.92827</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>8.067559838709712</v>
+        <v>15.08956032258067</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>0.0250094355000001</v>
+        <v>0.0425251245454546</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>3064.516129032258</v>
+        <v>3370.967741935484</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>3001.42</v>
+        <v>3278.19</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-63.09612903225798</v>
+        <v>-92.77774193548385</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0205892631578947</v>
+        <v>-0.0275225837320574</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2933,28 +2933,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>169.1729323308271</v>
+        <v>197.3684210526316</v>
       </c>
       <c r="R5" t="n">
         <v>93</v>
       </c>
       <c r="S5" t="n">
-        <v>-76.17293233082711</v>
+        <v>-104.3684210526316</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="U5" s="135" t="n">
-        <v>1285.714285714286</v>
+        <v>1500</v>
       </c>
       <c r="V5" s="135" t="n">
         <v>706.8</v>
       </c>
       <c r="W5" s="135" t="n">
-        <v>-578.9142857142858</v>
+        <v>-793.2</v>
       </c>
       <c r="X5" s="136" t="n">
-        <v>-0.4502666666666667</v>
+        <v>-0.5288</v>
       </c>
       <c r="Y5" s="135" t="n">
         <v>7.6</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3036,28 +3036,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>95.23809523809524</v>
+        <v>111.1111111111111</v>
       </c>
       <c r="R6" t="n">
         <v>60</v>
       </c>
       <c r="S6" t="n">
-        <v>-35.23809523809523</v>
+        <v>-51.1111111111111</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>857.1428571428571</v>
+        <v>1000</v>
       </c>
       <c r="V6" s="135" t="n">
         <v>540</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-317.1428571428571</v>
+        <v>-460</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.37</v>
+        <v>-0.46</v>
       </c>
       <c r="Y6" s="135" t="n">
         <v>9</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3139,28 +3139,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>35.71428571428572</v>
+        <v>41.66666666666667</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>9.285714285714285</v>
+        <v>3.333333333333329</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>285.7142857142857</v>
+        <v>333.3333333333334</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>360</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>74.28571428571428</v>
+        <v>26.66666666666663</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>0.2599999999999999</v>
+        <v>0.07999999999999979</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>8</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>20.81165452653486</v>
+        <v>22.89281997918835</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>1.188345473465141</v>
+        <v>-0.8928199791883422</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>645.1612903225806</v>
+        <v>709.6774193548387</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>789.936725</v>
+        <v>843.0790950000001</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>144.7754346774194</v>
+        <v>133.4016756451614</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>0.2244019237500001</v>
+        <v>0.187975088409091</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>35.90621477272727</v>
+        <v>38.32177704545455</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>4.906214772727274</v>
+        <v>7.321777045454546</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>34.87358326068004</v>
+        <v>38.36094158674804</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-14.87358326068004</v>
+        <v>-18.36094158674804</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>1290.322580645161</v>
+        <v>1419.354838709677</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>1334.840728</v>
+        <v>1462.139115</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>44.51814735483868</v>
+        <v>42.78427629032262</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.0345015641999999</v>
+        <v>0.0301434673863636</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>66.74203639999999</v>
+        <v>73.10695575</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>29.74203639999999</v>
+        <v>36.10695575</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>2.780867630700779</v>
+        <v>3.058954393770857</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-0.7808676307007789</v>
+        <v>-1.058954393770857</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>161.2903225806452</v>
+        <v>177.4193548387097</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>169.607791</v>
+        <v>184.640047</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>8.317468419354839</v>
+        <v>7.220692161290344</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0515683042</v>
+        <v>0.0406984467272728</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>84.8038955</v>
+        <v>92.3200235</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>26.8038955</v>
+        <v>34.3200235</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,34 +3563,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.008064516129032</v>
+        <v>1.108870967741935</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.008064516129032201</v>
+        <v>-0.1088709677419355</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>161.2903225806452</v>
+        <v>177.4193548387097</v>
       </c>
       <c r="V11" s="135" t="n">
-        <v>47.27</v>
+        <v>59.204384</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-114.0203225806451</v>
+        <v>-118.2149708387097</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.7069259999999999</v>
+        <v>-0.6663025629090908</v>
       </c>
       <c r="Y11" s="135" t="n">
-        <v>47.27</v>
+        <v>59.204384</v>
       </c>
       <c r="Z11" s="135" t="n">
-        <v>-112.73</v>
+        <v>-100.795616</v>
       </c>
       <c r="AB11" s="137" t="inlineStr">
         <is>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>93.3786078098472</v>
+        <v>102.7164685908319</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-1.378607809847196</v>
+        <v>-10.71646859083191</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>1774.193548387097</v>
+        <v>1951.612903225806</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>1820.29</v>
+        <v>1999.25</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>46.09645161290337</v>
+        <v>47.63709677419365</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.0259816363636364</v>
+        <v>0.0244090909090909</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>19.78576086956522</v>
+        <v>21.73097826086957</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>0.7857608695652161</v>
+        <v>2.730978260869566</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.376344086021506</v>
+        <v>5.913978494623657</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>1.623655913978494</v>
+        <v>1.086021505376343</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>161.2903225806452</v>
+        <v>177.4193548387097</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>103.51</v>
+        <v>114.02</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-57.78032258064515</v>
+        <v>-63.39935483870967</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3582379999999999</v>
+        <v>-0.3573418181818181</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>14.78714285714286</v>
+        <v>16.28857142857143</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-15.21285714285714</v>
+        <v>-13.71142857142857</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.792114695340502</v>
+        <v>1.971326164874552</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-1.792114695340502</v>
+        <v>-1.971326164874552</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>161.2903225806452</v>
+        <v>177.4193548387097</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>102.45</v>
+        <v>112.32</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-58.84032258064515</v>
+        <v>-65.09935483870967</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3648099999999999</v>
+        <v>-0.3669236363636363</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>40.32258064516129</v>
+        <v>44.35483870967742</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-21.32258064516129</v>
+        <v>-25.35483870967742</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>483.8709677419355</v>
+        <v>532.258064516129</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>566.95176</v>
+        <v>609.1047150000001</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>83.08079225806455</v>
+        <v>76.84665048387103</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>0.171700304</v>
+        <v>0.1443785554545456</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>29.83956631578948</v>
+        <v>32.05814289473685</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>17.83956631578948</v>
+        <v>20.05814289473685</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>14.02524544179523</v>
+        <v>15.42776998597475</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-11.02524544179523</v>
+        <v>-12.42776998597475</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>322.5806451612903</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>282.35</v>
+        <v>316.15</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-40.23064516129028</v>
+        <v>-38.68870967741936</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.1247149999999998</v>
+        <v>-0.1090318181818181</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>94.11666666666667</v>
+        <v>105.3833333333333</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>71.11666666666667</v>
+        <v>82.38333333333333</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>138.7846961740435</v>
+        <v>152.6631657914479</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-22.78469617404352</v>
+        <v>-36.66316579144785</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>5967.741935483871</v>
+        <v>6564.516129032258</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>5951.350936</v>
+        <v>6551.195078</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-16.39099948387138</v>
+        <v>-13.32105103225786</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0027465999135135</v>
+        <v>-0.0020292510171989</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>51.30474944827586</v>
+        <v>56.47581963793103</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>8.304749448275864</v>
+        <v>13.47581963793103</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>214.3690626122104</v>
+        <v>235.8059688734315</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-48.36906261221043</v>
+        <v>-69.80596887343145</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>5161.290322580645</v>
+        <v>5677.419354838709</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>5217.207004</v>
+        <v>5699.907356</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>55.91668141935497</v>
+        <v>22.48800116129041</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>0.010833857025</v>
+        <v>0.00396095475</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>31.42895785542169</v>
+        <v>34.33679130120482</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>7.352301178906185</v>
+        <v>10.26013462468932</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4350,28 +4350,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>300.125313283208</v>
+        <v>350.1461988304094</v>
       </c>
       <c r="R19" t="n">
         <v>198</v>
       </c>
       <c r="S19" t="n">
-        <v>-102.1253132832081</v>
+        <v>-152.1461988304094</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>2428.571428571428</v>
+        <v>2833.333333333333</v>
       </c>
       <c r="V19" s="135" t="n">
         <v>1606.8</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-821.7714285714285</v>
+        <v>-1226.533333333334</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.3383764705882353</v>
+        <v>-0.4328941176470589</v>
       </c>
       <c r="Y19" s="135" t="n">
         <v>8.115151515151515</v>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>653.279072069462</v>
+        <v>738.6153334952887</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-173.279072069462</v>
+        <v>-258.6153334952887</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>13557.60368663594</v>
+        <v>15075.2688172043</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>12775.35794</v>
+        <v>13857.902434</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-782.2457466359447</v>
+        <v>-1217.3663832043</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.0576979357647858</v>
+        <v>-0.08075254895720391</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>26.61532904166667</v>
+        <v>28.87063007083333</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>6.570720452629082</v>
+        <v>8.826021481795749</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46245.291875</v>
+        <v>46246.29199074074</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-13
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 11/08/2026  |  Ultimo aggiornamento: 12/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 12/08/2026  |  Ultimo aggiornamento: 13/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>2838.709677419354</v>
+        <v>3096.774193548388</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>2903.076808</v>
+        <v>3174.420014</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>64.36713058064515</v>
+        <v>77.64582045161251</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0226747846363636</v>
+        <v>0.0250731295208332</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>354.8387096774193</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>369.92827</v>
+        <v>406.074798</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>15.08956032258067</v>
+        <v>18.97802380645157</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>0.0425251245454546</v>
+        <v>0.0490265614999999</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>3370.967741935484</v>
+        <v>3677.419354838709</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>3278.19</v>
+        <v>3552.18</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-92.77774193548385</v>
+        <v>-125.2393548387095</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0275225837320574</v>
+        <v>-0.0340563157894736</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>152.6631657914479</v>
+        <v>166.5416354088522</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-36.66316579144785</v>
+        <v>-50.54163540885222</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>6564.516129032258</v>
+        <v>7161.290322580645</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>6551.195078</v>
+        <v>7132.674811999999</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-13.32105103225786</v>
+        <v>-28.6155105806456</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0020292510171989</v>
+        <v>-0.0039958595855856</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>56.47581963793103</v>
+        <v>61.48857596551724</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>13.47581963793103</v>
+        <v>18.48857596551724</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>22.89281997918835</v>
+        <v>24.97398543184183</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-0.8928199791883422</v>
+        <v>-2.973985431841829</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>709.6774193548387</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>843.0790950000001</v>
+        <v>903.203061</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>133.4016756451614</v>
+        <v>129.0095126129032</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.187975088409091</v>
+        <v>0.1666372871249999</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>38.32177704545455</v>
+        <v>41.05468459090909</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>7.321777045454546</v>
+        <v>10.05468459090909</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>38.36094158674804</v>
+        <v>41.84829991281605</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-18.36094158674804</v>
+        <v>-21.84829991281605</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>1419.354838709677</v>
+        <v>1548.387096774194</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>1462.139115</v>
+        <v>1589.226636</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>42.78427629032262</v>
+        <v>40.83953922580645</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>0.0301434673863636</v>
+        <v>0.0263755357499999</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>73.10695575</v>
+        <v>79.46133180000001</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>36.10695575</v>
+        <v>42.46133180000001</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>3.058954393770857</v>
+        <v>3.337041156840935</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-1.058954393770857</v>
+        <v>-1.337041156840935</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>177.4193548387097</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>184.640047</v>
+        <v>200.062156</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>7.220692161290344</v>
+        <v>6.513768903225781</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0406984467272728</v>
+        <v>0.0336544726666665</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>92.3200235</v>
+        <v>100.031078</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>34.3200235</v>
+        <v>42.031078</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,34 +1540,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>1.108870967741935</v>
+        <v>1.209677419354838</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-0.1088709677419355</v>
+        <v>-0.2096774193548385</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>177.4193548387097</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>59.204384</v>
+        <v>67.254384</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-118.2149708387097</v>
+        <v>-126.2940030967742</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.6663025629090908</v>
+        <v>-0.6525190160000001</v>
       </c>
       <c r="U12" s="117" t="n">
-        <v>59.204384</v>
+        <v>67.254384</v>
       </c>
       <c r="V12" s="117" t="n">
-        <v>-100.795616</v>
+        <v>-92.745616</v>
       </c>
       <c r="W12" s="120" t="inlineStr"/>
     </row>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>102.7164685908319</v>
+        <v>112.0543293718166</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-10.71646859083191</v>
+        <v>-20.05432937181664</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>1951.612903225806</v>
+        <v>2129.032258064516</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>1999.25</v>
+        <v>2170.12</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>47.63709677419365</v>
+        <v>41.08774193548379</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.0244090909090909</v>
+        <v>0.0192987878787878</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>21.73097826086957</v>
+        <v>23.58826086956521</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>2.730978260869566</v>
+        <v>4.588260869565215</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>5.913978494623657</v>
+        <v>6.451612903225808</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>1.086021505376343</v>
+        <v>0.5483870967741922</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>177.4193548387097</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>114.02</v>
+        <v>122.45</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-63.39935483870967</v>
+        <v>-71.0983870967742</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3573418181818181</v>
+        <v>-0.3673416666666667</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>16.28857142857143</v>
+        <v>17.49285714285714</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-13.71142857142857</v>
+        <v>-12.50714285714286</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>1.971326164874552</v>
+        <v>2.150537634408602</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-1.971326164874552</v>
+        <v>-2.150537634408602</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>177.4193548387097</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>112.32</v>
+        <v>121.57</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-65.09935483870967</v>
+        <v>-71.97838709677421</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3669236363636363</v>
+        <v>-0.3718883333333334</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>44.35483870967742</v>
+        <v>48.38709677419355</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-25.35483870967742</v>
+        <v>-29.38709677419355</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>532.258064516129</v>
+        <v>580.6451612903227</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>609.1047150000001</v>
+        <v>649.063071</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>76.84665048387103</v>
+        <v>68.41790970967736</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.1443785554545456</v>
+        <v>0.1178308444999998</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>32.05814289473685</v>
+        <v>34.16121426315789</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>20.05814289473685</v>
+        <v>22.16121426315789</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>15.42776998597475</v>
+        <v>16.83029453015428</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-12.42776998597475</v>
+        <v>-13.83029453015428</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>354.8387096774193</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>316.15</v>
+        <v>345.44</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-38.68870967741936</v>
+        <v>-41.65677419354842</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.1090318181818181</v>
+        <v>-0.1076133333333334</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>105.3833333333333</v>
+        <v>115.1466666666667</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>82.38333333333333</v>
+        <v>92.14666666666666</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>235.8059688734315</v>
+        <v>257.2428751346525</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-69.80596887343145</v>
+        <v>-91.24287513465254</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>5677.419354838709</v>
+        <v>6193.548387096775</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>5699.907356</v>
+        <v>6168.389308</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>22.48800116129041</v>
+        <v>-25.1590790967748</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>0.00396095475</v>
+        <v>-0.0040621429791667</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>34.33679130120482</v>
+        <v>37.15897173493976</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>10.26013462468932</v>
+        <v>13.08231505842425</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2063,28 +2063,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>197.3684210526316</v>
+        <v>225.5639097744361</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>93</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-104.3684210526316</v>
+        <v>-132.5639097744361</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>1500</v>
+        <v>1714.285714285714</v>
       </c>
       <c r="R19" s="117" t="n">
         <v>706.8</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-793.2</v>
+        <v>-1007.485714285714</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.5288</v>
+        <v>-0.5877</v>
       </c>
       <c r="U19" s="117" t="n">
         <v>7.6</v>
@@ -2138,28 +2138,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>111.1111111111111</v>
+        <v>126.984126984127</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>60</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-51.1111111111111</v>
+        <v>-66.98412698412697</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>1000</v>
+        <v>1142.857142857143</v>
       </c>
       <c r="R20" s="117" t="n">
         <v>540</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-460</v>
+        <v>-602.8571428571429</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.46</v>
+        <v>-0.5275</v>
       </c>
       <c r="U20" s="117" t="n">
         <v>9</v>
@@ -2213,28 +2213,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>41.66666666666667</v>
+        <v>47.61904761904762</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>3.333333333333329</v>
+        <v>-2.61904761904762</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>333.3333333333334</v>
+        <v>380.952380952381</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>360</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>26.66666666666663</v>
+        <v>-20.95238095238096</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>0.07999999999999979</v>
+        <v>-0.055</v>
       </c>
       <c r="U21" s="117" t="n">
         <v>8</v>
@@ -2276,28 +2276,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>350.1461988304094</v>
+        <v>400.1670843776107</v>
       </c>
       <c r="N22" s="125" t="n">
         <v>198</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-152.1461988304094</v>
+        <v>-202.1670843776107</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="Q22" s="123" t="n">
-        <v>2833.333333333333</v>
+        <v>3238.095238095238</v>
       </c>
       <c r="R22" s="123" t="n">
         <v>1606.8</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-1226.533333333334</v>
+        <v>-1631.295238095238</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-0.4328941176470589</v>
+        <v>-0.5037823529411765</v>
       </c>
       <c r="U22" s="123" t="n">
         <v>8.115151515151515</v>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>738.6153334952887</v>
+        <v>823.9515949211154</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-258.6153334952887</v>
+        <v>-343.9515949211154</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>15075.2688172043</v>
+        <v>16592.93394777266</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>13857.902434</v>
+        <v>14907.86412</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-1217.3663832043</v>
+        <v>-1685.069827772657</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.08075254895720391</v>
+        <v>-0.1015534584225143</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>28.87063007083333</v>
+        <v>31.05805025</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>8.826021481795749</v>
+        <v>11.01344166096242</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>2838.709677419354</v>
+        <v>3096.774193548388</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>2903.076808</v>
+        <v>3174.420014</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>64.36713058064515</v>
+        <v>77.64582045161251</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0226747846363636</v>
+        <v>0.0250731295208332</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>354.8387096774193</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>369.92827</v>
+        <v>406.074798</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>15.08956032258067</v>
+        <v>18.97802380645157</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>0.0425251245454546</v>
+        <v>0.0490265614999999</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>3370.967741935484</v>
+        <v>3677.419354838709</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>3278.19</v>
+        <v>3552.18</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-92.77774193548385</v>
+        <v>-125.2393548387095</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0275225837320574</v>
+        <v>-0.0340563157894736</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2933,28 +2933,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>197.3684210526316</v>
+        <v>225.5639097744361</v>
       </c>
       <c r="R5" t="n">
         <v>93</v>
       </c>
       <c r="S5" t="n">
-        <v>-104.3684210526316</v>
+        <v>-132.5639097744361</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="U5" s="135" t="n">
-        <v>1500</v>
+        <v>1714.285714285714</v>
       </c>
       <c r="V5" s="135" t="n">
         <v>706.8</v>
       </c>
       <c r="W5" s="135" t="n">
-        <v>-793.2</v>
+        <v>-1007.485714285714</v>
       </c>
       <c r="X5" s="136" t="n">
-        <v>-0.5288</v>
+        <v>-0.5877</v>
       </c>
       <c r="Y5" s="135" t="n">
         <v>7.6</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3036,28 +3036,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>111.1111111111111</v>
+        <v>126.984126984127</v>
       </c>
       <c r="R6" t="n">
         <v>60</v>
       </c>
       <c r="S6" t="n">
-        <v>-51.1111111111111</v>
+        <v>-66.98412698412697</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>1000</v>
+        <v>1142.857142857143</v>
       </c>
       <c r="V6" s="135" t="n">
         <v>540</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-460</v>
+        <v>-602.8571428571429</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.46</v>
+        <v>-0.5275</v>
       </c>
       <c r="Y6" s="135" t="n">
         <v>9</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3139,28 +3139,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>41.66666666666667</v>
+        <v>47.61904761904762</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>3.333333333333329</v>
+        <v>-2.61904761904762</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>333.3333333333334</v>
+        <v>380.952380952381</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>360</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>26.66666666666663</v>
+        <v>-20.95238095238096</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>0.07999999999999979</v>
+        <v>-0.055</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>8</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>22.89281997918835</v>
+        <v>24.97398543184183</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-0.8928199791883422</v>
+        <v>-2.973985431841829</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>709.6774193548387</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>843.0790950000001</v>
+        <v>903.203061</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>133.4016756451614</v>
+        <v>129.0095126129032</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>0.187975088409091</v>
+        <v>0.1666372871249999</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>38.32177704545455</v>
+        <v>41.05468459090909</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>7.321777045454546</v>
+        <v>10.05468459090909</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>38.36094158674804</v>
+        <v>41.84829991281605</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-18.36094158674804</v>
+        <v>-21.84829991281605</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>1419.354838709677</v>
+        <v>1548.387096774194</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>1462.139115</v>
+        <v>1589.226636</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>42.78427629032262</v>
+        <v>40.83953922580645</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.0301434673863636</v>
+        <v>0.0263755357499999</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>73.10695575</v>
+        <v>79.46133180000001</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>36.10695575</v>
+        <v>42.46133180000001</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>3.058954393770857</v>
+        <v>3.337041156840935</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-1.058954393770857</v>
+        <v>-1.337041156840935</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>177.4193548387097</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>184.640047</v>
+        <v>200.062156</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>7.220692161290344</v>
+        <v>6.513768903225781</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0406984467272728</v>
+        <v>0.0336544726666665</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>92.3200235</v>
+        <v>100.031078</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>34.3200235</v>
+        <v>42.031078</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,34 +3563,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.108870967741935</v>
+        <v>1.209677419354838</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.1088709677419355</v>
+        <v>-0.2096774193548385</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>177.4193548387097</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="V11" s="135" t="n">
-        <v>59.204384</v>
+        <v>67.254384</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-118.2149708387097</v>
+        <v>-126.2940030967742</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.6663025629090908</v>
+        <v>-0.6525190160000001</v>
       </c>
       <c r="Y11" s="135" t="n">
-        <v>59.204384</v>
+        <v>67.254384</v>
       </c>
       <c r="Z11" s="135" t="n">
-        <v>-100.795616</v>
+        <v>-92.745616</v>
       </c>
       <c r="AB11" s="137" t="inlineStr">
         <is>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>102.7164685908319</v>
+        <v>112.0543293718166</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-10.71646859083191</v>
+        <v>-20.05432937181664</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>1951.612903225806</v>
+        <v>2129.032258064516</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>1999.25</v>
+        <v>2170.12</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>47.63709677419365</v>
+        <v>41.08774193548379</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.0244090909090909</v>
+        <v>0.0192987878787878</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>21.73097826086957</v>
+        <v>23.58826086956521</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>2.730978260869566</v>
+        <v>4.588260869565215</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.913978494623657</v>
+        <v>6.451612903225808</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>1.086021505376343</v>
+        <v>0.5483870967741922</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>177.4193548387097</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>114.02</v>
+        <v>122.45</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-63.39935483870967</v>
+        <v>-71.0983870967742</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3573418181818181</v>
+        <v>-0.3673416666666667</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>16.28857142857143</v>
+        <v>17.49285714285714</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-13.71142857142857</v>
+        <v>-12.50714285714286</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>1.971326164874552</v>
+        <v>2.150537634408602</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-1.971326164874552</v>
+        <v>-2.150537634408602</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>177.4193548387097</v>
+        <v>193.5483870967742</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>112.32</v>
+        <v>121.57</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-65.09935483870967</v>
+        <v>-71.97838709677421</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3669236363636363</v>
+        <v>-0.3718883333333334</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>44.35483870967742</v>
+        <v>48.38709677419355</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-25.35483870967742</v>
+        <v>-29.38709677419355</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>532.258064516129</v>
+        <v>580.6451612903227</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>609.1047150000001</v>
+        <v>649.063071</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>76.84665048387103</v>
+        <v>68.41790970967736</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>0.1443785554545456</v>
+        <v>0.1178308444999998</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>32.05814289473685</v>
+        <v>34.16121426315789</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>20.05814289473685</v>
+        <v>22.16121426315789</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>15.42776998597475</v>
+        <v>16.83029453015428</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-12.42776998597475</v>
+        <v>-13.83029453015428</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>354.8387096774193</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>316.15</v>
+        <v>345.44</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-38.68870967741936</v>
+        <v>-41.65677419354842</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.1090318181818181</v>
+        <v>-0.1076133333333334</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>105.3833333333333</v>
+        <v>115.1466666666667</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>82.38333333333333</v>
+        <v>92.14666666666666</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>152.6631657914479</v>
+        <v>166.5416354088522</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-36.66316579144785</v>
+        <v>-50.54163540885222</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>6564.516129032258</v>
+        <v>7161.290322580645</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>6551.195078</v>
+        <v>7132.674811999999</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-13.32105103225786</v>
+        <v>-28.6155105806456</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0020292510171989</v>
+        <v>-0.0039958595855856</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>56.47581963793103</v>
+        <v>61.48857596551724</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>13.47581963793103</v>
+        <v>18.48857596551724</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>235.8059688734315</v>
+        <v>257.2428751346525</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-69.80596887343145</v>
+        <v>-91.24287513465254</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>5677.419354838709</v>
+        <v>6193.548387096775</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>5699.907356</v>
+        <v>6168.389308</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>22.48800116129041</v>
+        <v>-25.1590790967748</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>0.00396095475</v>
+        <v>-0.0040621429791667</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>34.33679130120482</v>
+        <v>37.15897173493976</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>10.26013462468932</v>
+        <v>13.08231505842425</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4350,28 +4350,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>350.1461988304094</v>
+        <v>400.1670843776107</v>
       </c>
       <c r="R19" t="n">
         <v>198</v>
       </c>
       <c r="S19" t="n">
-        <v>-152.1461988304094</v>
+        <v>-202.1670843776107</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>2833.333333333333</v>
+        <v>3238.095238095238</v>
       </c>
       <c r="V19" s="135" t="n">
         <v>1606.8</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-1226.533333333334</v>
+        <v>-1631.295238095238</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.4328941176470589</v>
+        <v>-0.5037823529411765</v>
       </c>
       <c r="Y19" s="135" t="n">
         <v>8.115151515151515</v>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>738.6153334952887</v>
+        <v>823.9515949211154</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-258.6153334952887</v>
+        <v>-343.9515949211154</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>15075.2688172043</v>
+        <v>16592.93394777266</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>13857.902434</v>
+        <v>14907.86412</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-1217.3663832043</v>
+        <v>-1685.069827772657</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.08075254895720391</v>
+        <v>-0.1015534584225143</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>28.87063007083333</v>
+        <v>31.05805025</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>8.826021481795749</v>
+        <v>11.01344166096242</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46246.29199074074</v>
+        <v>46247.29190972223</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-14
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 12/08/2026  |  Ultimo aggiornamento: 13/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 13/08/2026  |  Ultimo aggiornamento: 14/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>3096.774193548388</v>
+        <v>3354.83870967742</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>3174.420014</v>
+        <v>3431.964539</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>77.64582045161251</v>
+        <v>77.12582932258056</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0250731295208332</v>
+        <v>0.0229894298942307</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>387.0967741935484</v>
+        <v>419.3548387096774</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>406.074798</v>
+        <v>438.314513</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>18.97802380645157</v>
+        <v>18.95967429032254</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>0.0490265614999999</v>
+        <v>0.0452115309999999</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>3677.419354838709</v>
+        <v>3983.870967741935</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>3552.18</v>
+        <v>3799.54</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-125.2393548387095</v>
+        <v>-184.3309677419352</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0340563157894736</v>
+        <v>-0.0462693117408906</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>166.5416354088522</v>
+        <v>180.4201050262565</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-50.54163540885222</v>
+        <v>-64.42010502625655</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>7161.290322580645</v>
+        <v>7758.064516129032</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>7132.674811999999</v>
+        <v>7669.819052</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-28.6155105806456</v>
+        <v>-88.24546412903237</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0039958595855856</v>
+        <v>-0.0113746752099792</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>61.48857596551724</v>
+        <v>66.11912975862069</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>18.48857596551724</v>
+        <v>23.11912975862069</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>24.97398543184183</v>
+        <v>27.05515088449532</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-2.973985431841829</v>
+        <v>-5.055150884495316</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>774.1935483870968</v>
+        <v>838.7096774193549</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>903.203061</v>
+        <v>956.308552</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>129.0095126129032</v>
+        <v>117.5988745806451</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.1666372871249999</v>
+        <v>0.1402140427692306</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>41.05468459090909</v>
+        <v>43.46857054545455</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>10.05468459090909</v>
+        <v>12.46857054545455</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>41.84829991281605</v>
+        <v>45.33565823888405</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-21.84829991281605</v>
+        <v>-25.33565823888405</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>1548.387096774194</v>
+        <v>1677.41935483871</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>1589.226636</v>
+        <v>1715.041703</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>40.83953922580645</v>
+        <v>37.62234816129035</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>0.0263755357499999</v>
+        <v>0.0224287075576923</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>79.46133180000001</v>
+        <v>85.75208515</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>42.46133180000001</v>
+        <v>48.75208515</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>3.337041156840935</v>
+        <v>3.615127919911013</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-1.337041156840935</v>
+        <v>-1.615127919911013</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>193.5483870967742</v>
+        <v>209.6774193548387</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>200.062156</v>
+        <v>216.72541</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>6.513768903225781</v>
+        <v>7.047990645161292</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0336544726666665</v>
+        <v>0.0336134938461538</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>100.031078</v>
+        <v>108.362705</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>42.031078</v>
+        <v>50.36270500000001</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,34 +1540,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>1.209677419354838</v>
+        <v>1.310483870967742</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-0.2096774193548385</v>
+        <v>-0.3104838709677417</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>193.5483870967742</v>
+        <v>209.6774193548387</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>67.254384</v>
+        <v>89.656346</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-126.2940030967742</v>
+        <v>-120.0210733548387</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.6525190160000001</v>
+        <v>-0.572408196</v>
       </c>
       <c r="U12" s="117" t="n">
-        <v>67.254384</v>
+        <v>89.656346</v>
       </c>
       <c r="V12" s="117" t="n">
-        <v>-92.745616</v>
+        <v>-70.343654</v>
       </c>
       <c r="W12" s="120" t="inlineStr"/>
     </row>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>112.0543293718166</v>
+        <v>121.3921901528014</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-20.05432937181664</v>
+        <v>-29.39219015280136</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>2129.032258064516</v>
+        <v>2306.451612903226</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>2170.12</v>
+        <v>2335.44</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>41.08774193548379</v>
+        <v>28.9883870967742</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.0192987878787878</v>
+        <v>0.0125683916083916</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>23.58826086956521</v>
+        <v>25.38521739130435</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>4.588260869565215</v>
+        <v>6.385217391304348</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>6.451612903225808</v>
+        <v>6.989247311827958</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>0.5483870967741922</v>
+        <v>0.0107526881720421</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>193.5483870967742</v>
+        <v>209.6774193548387</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>122.45</v>
+        <v>131.32</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-71.0983870967742</v>
+        <v>-78.35741935483873</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3673416666666667</v>
+        <v>-0.3737046153846154</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>17.49285714285714</v>
+        <v>18.76</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-12.50714285714286</v>
+        <v>-11.24</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>2.150537634408602</v>
+        <v>2.329749103942652</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-2.150537634408602</v>
+        <v>-2.329749103942652</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>193.5483870967742</v>
+        <v>209.6774193548387</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>121.57</v>
+        <v>132.2</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-71.97838709677421</v>
+        <v>-77.47741935483873</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3718883333333334</v>
+        <v>-0.3695076923076923</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>48.38709677419355</v>
+        <v>52.41935483870968</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-29.38709677419355</v>
+        <v>-33.41935483870968</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>580.6451612903227</v>
+        <v>629.0322580645162</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>649.063071</v>
+        <v>701.670927</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>68.41790970967736</v>
+        <v>72.63866893548379</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.1178308444999998</v>
+        <v>0.1154768583076921</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>34.16121426315789</v>
+        <v>36.93004878947369</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>22.16121426315789</v>
+        <v>24.93004878947369</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>16.83029453015428</v>
+        <v>18.2328190743338</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-13.83029453015428</v>
+        <v>-15.2328190743338</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>387.0967741935484</v>
+        <v>419.3548387096774</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>345.44</v>
+        <v>373.86</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-41.65677419354842</v>
+        <v>-45.49483870967742</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.1076133333333334</v>
+        <v>-0.1084876923076923</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>115.1466666666667</v>
+        <v>124.62</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>92.14666666666666</v>
+        <v>101.62</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>257.2428751346525</v>
+        <v>278.6797813958736</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-91.24287513465254</v>
+        <v>-112.6797813958736</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>6193.548387096775</v>
+        <v>6709.677419354839</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>6168.389308</v>
+        <v>6652.222938</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>-25.1590790967748</v>
+        <v>-57.45448135483912</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>-0.0040621429791667</v>
+        <v>-0.0085629275096154</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>37.15897173493976</v>
+        <v>40.0736321566265</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>13.08231505842425</v>
+        <v>15.996975480111</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2063,28 +2063,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>225.5639097744361</v>
+        <v>253.7593984962406</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>93</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-132.5639097744361</v>
+        <v>-160.7593984962406</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>1714.285714285714</v>
+        <v>1928.571428571428</v>
       </c>
       <c r="R19" s="117" t="n">
         <v>706.8</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-1007.485714285714</v>
+        <v>-1221.771428571428</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.5877</v>
+        <v>-0.6335111111111111</v>
       </c>
       <c r="U19" s="117" t="n">
         <v>7.6</v>
@@ -2138,28 +2138,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>126.984126984127</v>
+        <v>142.8571428571428</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>60</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-66.98412698412697</v>
+        <v>-82.85714285714283</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>1142.857142857143</v>
+        <v>1285.714285714286</v>
       </c>
       <c r="R20" s="117" t="n">
         <v>540</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-602.8571428571429</v>
+        <v>-745.7142857142858</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.5275</v>
+        <v>-0.5800000000000001</v>
       </c>
       <c r="U20" s="117" t="n">
         <v>9</v>
@@ -2213,28 +2213,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>47.61904761904762</v>
+        <v>53.57142857142857</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-2.61904761904762</v>
+        <v>-8.571428571428569</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>380.952380952381</v>
+        <v>428.5714285714286</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>360</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-20.95238095238096</v>
+        <v>-68.57142857142856</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.055</v>
+        <v>-0.1599999999999999</v>
       </c>
       <c r="U21" s="117" t="n">
         <v>8</v>
@@ -2276,28 +2276,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>400.1670843776107</v>
+        <v>450.187969924812</v>
       </c>
       <c r="N22" s="125" t="n">
         <v>198</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-202.1670843776107</v>
+        <v>-252.187969924812</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="Q22" s="123" t="n">
-        <v>3238.095238095238</v>
+        <v>3642.857142857143</v>
       </c>
       <c r="R22" s="123" t="n">
         <v>1606.8</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-1631.295238095238</v>
+        <v>-2036.057142857143</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-0.5037823529411765</v>
+        <v>-0.5589176470588235</v>
       </c>
       <c r="U22" s="123" t="n">
         <v>8.115151515151515</v>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>823.9515949211154</v>
+        <v>909.287856346942</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-343.9515949211154</v>
+        <v>-429.2878563469421</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>16592.93394777266</v>
+        <v>18110.59907834101</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>14907.86412</v>
+        <v>15928.84199</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-1685.069827772657</v>
+        <v>-2181.757088341012</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1015534584225143</v>
+        <v>-0.1204685211628497</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>31.05805025</v>
+        <v>33.18508747916667</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>11.01344166096242</v>
+        <v>13.14047889012908</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>3096.774193548388</v>
+        <v>3354.83870967742</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>3174.420014</v>
+        <v>3431.964539</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>77.64582045161251</v>
+        <v>77.12582932258056</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0250731295208332</v>
+        <v>0.0229894298942307</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>387.0967741935484</v>
+        <v>419.3548387096774</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>406.074798</v>
+        <v>438.314513</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>18.97802380645157</v>
+        <v>18.95967429032254</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>0.0490265614999999</v>
+        <v>0.0452115309999999</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>3677.419354838709</v>
+        <v>3983.870967741935</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>3552.18</v>
+        <v>3799.54</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-125.2393548387095</v>
+        <v>-184.3309677419352</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0340563157894736</v>
+        <v>-0.0462693117408906</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2933,28 +2933,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>225.5639097744361</v>
+        <v>253.7593984962406</v>
       </c>
       <c r="R5" t="n">
         <v>93</v>
       </c>
       <c r="S5" t="n">
-        <v>-132.5639097744361</v>
+        <v>-160.7593984962406</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="U5" s="135" t="n">
-        <v>1714.285714285714</v>
+        <v>1928.571428571428</v>
       </c>
       <c r="V5" s="135" t="n">
         <v>706.8</v>
       </c>
       <c r="W5" s="135" t="n">
-        <v>-1007.485714285714</v>
+        <v>-1221.771428571428</v>
       </c>
       <c r="X5" s="136" t="n">
-        <v>-0.5877</v>
+        <v>-0.6335111111111111</v>
       </c>
       <c r="Y5" s="135" t="n">
         <v>7.6</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3036,28 +3036,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>126.984126984127</v>
+        <v>142.8571428571428</v>
       </c>
       <c r="R6" t="n">
         <v>60</v>
       </c>
       <c r="S6" t="n">
-        <v>-66.98412698412697</v>
+        <v>-82.85714285714283</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>1142.857142857143</v>
+        <v>1285.714285714286</v>
       </c>
       <c r="V6" s="135" t="n">
         <v>540</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-602.8571428571429</v>
+        <v>-745.7142857142858</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.5275</v>
+        <v>-0.5800000000000001</v>
       </c>
       <c r="Y6" s="135" t="n">
         <v>9</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3139,28 +3139,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>47.61904761904762</v>
+        <v>53.57142857142857</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>-2.61904761904762</v>
+        <v>-8.571428571428569</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>380.952380952381</v>
+        <v>428.5714285714286</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>360</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>-20.95238095238096</v>
+        <v>-68.57142857142856</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>-0.055</v>
+        <v>-0.1599999999999999</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>8</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>24.97398543184183</v>
+        <v>27.05515088449532</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-2.973985431841829</v>
+        <v>-5.055150884495316</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>774.1935483870968</v>
+        <v>838.7096774193549</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>903.203061</v>
+        <v>956.308552</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>129.0095126129032</v>
+        <v>117.5988745806451</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>0.1666372871249999</v>
+        <v>0.1402140427692306</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>41.05468459090909</v>
+        <v>43.46857054545455</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>10.05468459090909</v>
+        <v>12.46857054545455</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>41.84829991281605</v>
+        <v>45.33565823888405</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-21.84829991281605</v>
+        <v>-25.33565823888405</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>1548.387096774194</v>
+        <v>1677.41935483871</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>1589.226636</v>
+        <v>1715.041703</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>40.83953922580645</v>
+        <v>37.62234816129035</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.0263755357499999</v>
+        <v>0.0224287075576923</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>79.46133180000001</v>
+        <v>85.75208515</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>42.46133180000001</v>
+        <v>48.75208515</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>3.337041156840935</v>
+        <v>3.615127919911013</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-1.337041156840935</v>
+        <v>-1.615127919911013</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>193.5483870967742</v>
+        <v>209.6774193548387</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>200.062156</v>
+        <v>216.72541</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>6.513768903225781</v>
+        <v>7.047990645161292</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0336544726666665</v>
+        <v>0.0336134938461538</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>100.031078</v>
+        <v>108.362705</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>42.031078</v>
+        <v>50.36270500000001</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,34 +3563,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.209677419354838</v>
+        <v>1.310483870967742</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.2096774193548385</v>
+        <v>-0.3104838709677417</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>193.5483870967742</v>
+        <v>209.6774193548387</v>
       </c>
       <c r="V11" s="135" t="n">
-        <v>67.254384</v>
+        <v>89.656346</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-126.2940030967742</v>
+        <v>-120.0210733548387</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.6525190160000001</v>
+        <v>-0.572408196</v>
       </c>
       <c r="Y11" s="135" t="n">
-        <v>67.254384</v>
+        <v>89.656346</v>
       </c>
       <c r="Z11" s="135" t="n">
-        <v>-92.745616</v>
+        <v>-70.343654</v>
       </c>
       <c r="AB11" s="137" t="inlineStr">
         <is>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>112.0543293718166</v>
+        <v>121.3921901528014</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-20.05432937181664</v>
+        <v>-29.39219015280136</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>2129.032258064516</v>
+        <v>2306.451612903226</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>2170.12</v>
+        <v>2335.44</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>41.08774193548379</v>
+        <v>28.9883870967742</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.0192987878787878</v>
+        <v>0.0125683916083916</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>23.58826086956521</v>
+        <v>25.38521739130435</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>4.588260869565215</v>
+        <v>6.385217391304348</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>6.451612903225808</v>
+        <v>6.989247311827958</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>0.5483870967741922</v>
+        <v>0.0107526881720421</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>193.5483870967742</v>
+        <v>209.6774193548387</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>122.45</v>
+        <v>131.32</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-71.0983870967742</v>
+        <v>-78.35741935483873</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3673416666666667</v>
+        <v>-0.3737046153846154</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>17.49285714285714</v>
+        <v>18.76</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-12.50714285714286</v>
+        <v>-11.24</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>2.150537634408602</v>
+        <v>2.329749103942652</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-2.150537634408602</v>
+        <v>-2.329749103942652</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>193.5483870967742</v>
+        <v>209.6774193548387</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>121.57</v>
+        <v>132.2</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-71.97838709677421</v>
+        <v>-77.47741935483873</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3718883333333334</v>
+        <v>-0.3695076923076923</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>48.38709677419355</v>
+        <v>52.41935483870968</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-29.38709677419355</v>
+        <v>-33.41935483870968</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>580.6451612903227</v>
+        <v>629.0322580645162</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>649.063071</v>
+        <v>701.670927</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>68.41790970967736</v>
+        <v>72.63866893548379</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>0.1178308444999998</v>
+        <v>0.1154768583076921</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>34.16121426315789</v>
+        <v>36.93004878947369</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>22.16121426315789</v>
+        <v>24.93004878947369</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>16.83029453015428</v>
+        <v>18.2328190743338</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-13.83029453015428</v>
+        <v>-15.2328190743338</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>387.0967741935484</v>
+        <v>419.3548387096774</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>345.44</v>
+        <v>373.86</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-41.65677419354842</v>
+        <v>-45.49483870967742</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.1076133333333334</v>
+        <v>-0.1084876923076923</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>115.1466666666667</v>
+        <v>124.62</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>92.14666666666666</v>
+        <v>101.62</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>166.5416354088522</v>
+        <v>180.4201050262565</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-50.54163540885222</v>
+        <v>-64.42010502625655</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>7161.290322580645</v>
+        <v>7758.064516129032</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>7132.674811999999</v>
+        <v>7669.819052</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-28.6155105806456</v>
+        <v>-88.24546412903237</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0039958595855856</v>
+        <v>-0.0113746752099792</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>61.48857596551724</v>
+        <v>66.11912975862069</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>18.48857596551724</v>
+        <v>23.11912975862069</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>257.2428751346525</v>
+        <v>278.6797813958736</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-91.24287513465254</v>
+        <v>-112.6797813958736</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>6193.548387096775</v>
+        <v>6709.677419354839</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>6168.389308</v>
+        <v>6652.222938</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>-25.1590790967748</v>
+        <v>-57.45448135483912</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>-0.0040621429791667</v>
+        <v>-0.0085629275096154</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>37.15897173493976</v>
+        <v>40.0736321566265</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>13.08231505842425</v>
+        <v>15.996975480111</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4350,28 +4350,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>400.1670843776107</v>
+        <v>450.187969924812</v>
       </c>
       <c r="R19" t="n">
         <v>198</v>
       </c>
       <c r="S19" t="n">
-        <v>-202.1670843776107</v>
+        <v>-252.187969924812</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>3238.095238095238</v>
+        <v>3642.857142857143</v>
       </c>
       <c r="V19" s="135" t="n">
         <v>1606.8</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-1631.295238095238</v>
+        <v>-2036.057142857143</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.5037823529411765</v>
+        <v>-0.5589176470588235</v>
       </c>
       <c r="Y19" s="135" t="n">
         <v>8.115151515151515</v>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>823.9515949211154</v>
+        <v>909.287856346942</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-343.9515949211154</v>
+        <v>-429.2878563469421</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>16592.93394777266</v>
+        <v>18110.59907834101</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>14907.86412</v>
+        <v>15928.84199</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-1685.069827772657</v>
+        <v>-2181.757088341012</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1015534584225143</v>
+        <v>-0.1204685211628497</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>31.05805025</v>
+        <v>33.18508747916667</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>11.01344166096242</v>
+        <v>13.14047889012908</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46247.29190972223</v>
+        <v>46248.29186342593</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-15
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 13/08/2026  |  Ultimo aggiornamento: 14/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 14/08/2026  |  Ultimo aggiornamento: 15/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>3354.83870967742</v>
+        <v>3612.903225806452</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>3431.964539</v>
+        <v>3685.611495</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>77.12582932258056</v>
+        <v>72.7082691935484</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0229894298942307</v>
+        <v>0.0201246102232142</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>419.3548387096774</v>
+        <v>451.6129032258065</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>438.314513</v>
+        <v>469.206465</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>18.95967429032254</v>
+        <v>17.59356177419352</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>0.0452115309999999</v>
+        <v>0.0389571724999999</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>3983.870967741935</v>
+        <v>4290.322580645161</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>3799.54</v>
+        <v>4029.76</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-184.3309677419352</v>
+        <v>-260.5625806451608</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0462693117408906</v>
+        <v>-0.0607326315789472</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>180.4201050262565</v>
+        <v>194.2985746436609</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-64.42010502625655</v>
+        <v>-78.29857464366091</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>7758.064516129032</v>
+        <v>8354.838709677419</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>7669.819052</v>
+        <v>8184.57796</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-88.24546412903237</v>
+        <v>-170.2607496774181</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0113746752099792</v>
+        <v>-0.0203786997683396</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>66.11912975862069</v>
+        <v>70.55670655172415</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>23.11912975862069</v>
+        <v>27.55670655172415</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>27.05515088449532</v>
+        <v>29.1363163371488</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-5.055150884495316</v>
+        <v>-7.136316337148799</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>838.7096774193549</v>
+        <v>903.2258064516128</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>956.308552</v>
+        <v>1014.072829</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>117.5988745806451</v>
+        <v>110.847022548387</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.1402140427692306</v>
+        <v>0.1227234892499999</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>43.46857054545455</v>
+        <v>46.0942195</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>12.46857054545455</v>
+        <v>15.0942195</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>45.33565823888405</v>
+        <v>48.82301656495205</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-25.33565823888405</v>
+        <v>-28.82301656495205</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>1677.41935483871</v>
+        <v>1806.451612903226</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>1715.041703</v>
+        <v>1838.972885</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>37.62234816129035</v>
+        <v>32.52127209677406</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>0.0224287075576923</v>
+        <v>0.0180028470535713</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>85.75208515</v>
+        <v>91.94864425</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>48.75208515</v>
+        <v>54.94864425</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>3.615127919911013</v>
+        <v>3.89321468298109</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-1.615127919911013</v>
+        <v>-1.893214682981091</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>209.6774193548387</v>
+        <v>225.8064516129032</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>216.72541</v>
+        <v>232.31417</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>7.047990645161292</v>
+        <v>6.507718387096759</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0336134938461538</v>
+        <v>0.0288198957142856</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>108.362705</v>
+        <v>116.157085</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>50.36270500000001</v>
+        <v>58.157085</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,28 +1540,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>1.310483870967742</v>
+        <v>1.411290322580645</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-0.3104838709677417</v>
+        <v>-0.411290322580645</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>209.6774193548387</v>
+        <v>225.8064516129032</v>
       </c>
       <c r="R12" s="117" t="n">
         <v>89.656346</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-120.0210733548387</v>
+        <v>-136.1501056129032</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.572408196</v>
+        <v>-0.6029504677142858</v>
       </c>
       <c r="U12" s="117" t="n">
         <v>89.656346</v>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>121.3921901528014</v>
+        <v>130.7300509337861</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-29.39219015280136</v>
+        <v>-38.73005093378606</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>2306.451612903226</v>
+        <v>2483.870967741935</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>2335.44</v>
+        <v>2496.76</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>28.9883870967742</v>
+        <v>12.88903225806507</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.0125683916083916</v>
+        <v>0.0051890909090911</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>25.38521739130435</v>
+        <v>27.13869565217392</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>6.385217391304348</v>
+        <v>8.138695652173915</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>6.989247311827958</v>
+        <v>7.526881720430109</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>0.0107526881720421</v>
+        <v>-0.5268817204301088</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>209.6774193548387</v>
+        <v>225.8064516129032</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>131.32</v>
+        <v>139.96</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-78.35741935483873</v>
+        <v>-85.84645161290322</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3737046153846154</v>
+        <v>-0.3801771428571428</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>18.76</v>
+        <v>19.99428571428572</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-11.24</v>
+        <v>-10.00571428571428</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>2.329749103942652</v>
+        <v>2.508960573476702</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-2.329749103942652</v>
+        <v>-2.508960573476702</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>209.6774193548387</v>
+        <v>225.8064516129032</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>132.2</v>
+        <v>139.91</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-77.47741935483873</v>
+        <v>-85.89645161290323</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3695076923076923</v>
+        <v>-0.3803985714285715</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>52.41935483870968</v>
+        <v>56.45161290322581</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-33.41935483870968</v>
+        <v>-37.45161290322581</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>629.0322580645162</v>
+        <v>677.4193548387098</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>701.670927</v>
+        <v>755.488914</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>72.63866893548379</v>
+        <v>78.06955916129027</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.1154768583076921</v>
+        <v>0.1152455397142856</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>36.93004878947369</v>
+        <v>39.76257442105263</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>24.93004878947369</v>
+        <v>27.76257442105264</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>18.2328190743338</v>
+        <v>19.63534361851332</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-15.2328190743338</v>
+        <v>-16.63534361851332</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>419.3548387096774</v>
+        <v>451.6129032258065</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>373.86</v>
+        <v>401.93</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-45.49483870967742</v>
+        <v>-49.68290322580646</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.1084876923076923</v>
+        <v>-0.1100121428571428</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>124.62</v>
+        <v>133.9766666666667</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>101.62</v>
+        <v>110.9766666666667</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>278.6797813958736</v>
+        <v>300.1166876570946</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-112.6797813958736</v>
+        <v>-134.1166876570946</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>6709.677419354839</v>
+        <v>7225.806451612903</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>6652.222938</v>
+        <v>7109.065144</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>-57.45448135483912</v>
+        <v>-116.7413076129033</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>-0.0085629275096154</v>
+        <v>-0.0161561631071428</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>40.0736321566265</v>
+        <v>42.82569363855422</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>15.996975480111</v>
+        <v>18.74903696203872</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2063,28 +2063,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>253.7593984962406</v>
+        <v>281.9548872180451</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>93</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-160.7593984962406</v>
+        <v>-188.9548872180452</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>1928.571428571428</v>
+        <v>2142.857142857143</v>
       </c>
       <c r="R19" s="117" t="n">
         <v>706.8</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-1221.771428571428</v>
+        <v>-1436.057142857143</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.6335111111111111</v>
+        <v>-0.67016</v>
       </c>
       <c r="U19" s="117" t="n">
         <v>7.6</v>
@@ -2138,28 +2138,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>142.8571428571428</v>
+        <v>158.7301587301587</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>60</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-82.85714285714283</v>
+        <v>-98.73015873015871</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>1285.714285714286</v>
+        <v>1428.571428571429</v>
       </c>
       <c r="R20" s="117" t="n">
         <v>540</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-745.7142857142858</v>
+        <v>-888.5714285714287</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.5800000000000001</v>
+        <v>-0.622</v>
       </c>
       <c r="U20" s="117" t="n">
         <v>9</v>
@@ -2213,28 +2213,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>53.57142857142857</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-8.571428571428569</v>
+        <v>-14.52380952380953</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>428.5714285714286</v>
+        <v>476.1904761904762</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>360</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-68.57142857142856</v>
+        <v>-116.1904761904762</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.1599999999999999</v>
+        <v>-0.244</v>
       </c>
       <c r="U21" s="117" t="n">
         <v>8</v>
@@ -2276,28 +2276,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>450.187969924812</v>
+        <v>500.2088554720134</v>
       </c>
       <c r="N22" s="125" t="n">
         <v>198</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-252.187969924812</v>
+        <v>-302.2088554720134</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="Q22" s="123" t="n">
-        <v>3642.857142857143</v>
+        <v>4047.619047619048</v>
       </c>
       <c r="R22" s="123" t="n">
         <v>1606.8</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-2036.057142857143</v>
+        <v>-2440.819047619048</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-0.5589176470588235</v>
+        <v>-0.6030258823529412</v>
       </c>
       <c r="U22" s="123" t="n">
         <v>8.115151515151515</v>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>909.287856346942</v>
+        <v>994.6241177727688</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-429.2878563469421</v>
+        <v>-514.6241177727688</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>18110.59907834101</v>
+        <v>19628.26420890937</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>15928.84199</v>
+        <v>16900.443104</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-2181.757088341012</v>
+        <v>-2727.82110490937</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1204685211628497</v>
+        <v>-0.1389741383077163</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>33.18508747916667</v>
+        <v>35.20925646666667</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>13.14047889012908</v>
+        <v>15.16464787762909</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>3354.83870967742</v>
+        <v>3612.903225806452</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>3431.964539</v>
+        <v>3685.611495</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>77.12582932258056</v>
+        <v>72.7082691935484</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0229894298942307</v>
+        <v>0.0201246102232142</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>419.3548387096774</v>
+        <v>451.6129032258065</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>438.314513</v>
+        <v>469.206465</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>18.95967429032254</v>
+        <v>17.59356177419352</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>0.0452115309999999</v>
+        <v>0.0389571724999999</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>3983.870967741935</v>
+        <v>4290.322580645161</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>3799.54</v>
+        <v>4029.76</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-184.3309677419352</v>
+        <v>-260.5625806451608</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0462693117408906</v>
+        <v>-0.0607326315789472</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2933,28 +2933,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>253.7593984962406</v>
+        <v>281.9548872180451</v>
       </c>
       <c r="R5" t="n">
         <v>93</v>
       </c>
       <c r="S5" t="n">
-        <v>-160.7593984962406</v>
+        <v>-188.9548872180452</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="U5" s="135" t="n">
-        <v>1928.571428571428</v>
+        <v>2142.857142857143</v>
       </c>
       <c r="V5" s="135" t="n">
         <v>706.8</v>
       </c>
       <c r="W5" s="135" t="n">
-        <v>-1221.771428571428</v>
+        <v>-1436.057142857143</v>
       </c>
       <c r="X5" s="136" t="n">
-        <v>-0.6335111111111111</v>
+        <v>-0.67016</v>
       </c>
       <c r="Y5" s="135" t="n">
         <v>7.6</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3036,28 +3036,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>142.8571428571428</v>
+        <v>158.7301587301587</v>
       </c>
       <c r="R6" t="n">
         <v>60</v>
       </c>
       <c r="S6" t="n">
-        <v>-82.85714285714283</v>
+        <v>-98.73015873015871</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>1285.714285714286</v>
+        <v>1428.571428571429</v>
       </c>
       <c r="V6" s="135" t="n">
         <v>540</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-745.7142857142858</v>
+        <v>-888.5714285714287</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.5800000000000001</v>
+        <v>-0.622</v>
       </c>
       <c r="Y6" s="135" t="n">
         <v>9</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3139,28 +3139,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>53.57142857142857</v>
+        <v>59.52380952380953</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>-8.571428571428569</v>
+        <v>-14.52380952380953</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>428.5714285714286</v>
+        <v>476.1904761904762</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>360</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>-68.57142857142856</v>
+        <v>-116.1904761904762</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>-0.1599999999999999</v>
+        <v>-0.244</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>8</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>27.05515088449532</v>
+        <v>29.1363163371488</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-5.055150884495316</v>
+        <v>-7.136316337148799</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>838.7096774193549</v>
+        <v>903.2258064516128</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>956.308552</v>
+        <v>1014.072829</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>117.5988745806451</v>
+        <v>110.847022548387</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>0.1402140427692306</v>
+        <v>0.1227234892499999</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>43.46857054545455</v>
+        <v>46.0942195</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>12.46857054545455</v>
+        <v>15.0942195</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>45.33565823888405</v>
+        <v>48.82301656495205</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-25.33565823888405</v>
+        <v>-28.82301656495205</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>1677.41935483871</v>
+        <v>1806.451612903226</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>1715.041703</v>
+        <v>1838.972885</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>37.62234816129035</v>
+        <v>32.52127209677406</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.0224287075576923</v>
+        <v>0.0180028470535713</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>85.75208515</v>
+        <v>91.94864425</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>48.75208515</v>
+        <v>54.94864425</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>3.615127919911013</v>
+        <v>3.89321468298109</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-1.615127919911013</v>
+        <v>-1.893214682981091</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>209.6774193548387</v>
+        <v>225.8064516129032</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>216.72541</v>
+        <v>232.31417</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>7.047990645161292</v>
+        <v>6.507718387096759</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0336134938461538</v>
+        <v>0.0288198957142856</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>108.362705</v>
+        <v>116.157085</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>50.36270500000001</v>
+        <v>58.157085</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,28 +3563,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.310483870967742</v>
+        <v>1.411290322580645</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.3104838709677417</v>
+        <v>-0.411290322580645</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>209.6774193548387</v>
+        <v>225.8064516129032</v>
       </c>
       <c r="V11" s="135" t="n">
         <v>89.656346</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-120.0210733548387</v>
+        <v>-136.1501056129032</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.572408196</v>
+        <v>-0.6029504677142858</v>
       </c>
       <c r="Y11" s="135" t="n">
         <v>89.656346</v>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>121.3921901528014</v>
+        <v>130.7300509337861</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-29.39219015280136</v>
+        <v>-38.73005093378606</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>2306.451612903226</v>
+        <v>2483.870967741935</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>2335.44</v>
+        <v>2496.76</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>28.9883870967742</v>
+        <v>12.88903225806507</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.0125683916083916</v>
+        <v>0.0051890909090911</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>25.38521739130435</v>
+        <v>27.13869565217392</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>6.385217391304348</v>
+        <v>8.138695652173915</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>6.989247311827958</v>
+        <v>7.526881720430109</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>0.0107526881720421</v>
+        <v>-0.5268817204301088</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>209.6774193548387</v>
+        <v>225.8064516129032</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>131.32</v>
+        <v>139.96</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-78.35741935483873</v>
+        <v>-85.84645161290322</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3737046153846154</v>
+        <v>-0.3801771428571428</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>18.76</v>
+        <v>19.99428571428572</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-11.24</v>
+        <v>-10.00571428571428</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>2.329749103942652</v>
+        <v>2.508960573476702</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-2.329749103942652</v>
+        <v>-2.508960573476702</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>209.6774193548387</v>
+        <v>225.8064516129032</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>132.2</v>
+        <v>139.91</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-77.47741935483873</v>
+        <v>-85.89645161290323</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3695076923076923</v>
+        <v>-0.3803985714285715</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>52.41935483870968</v>
+        <v>56.45161290322581</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-33.41935483870968</v>
+        <v>-37.45161290322581</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>629.0322580645162</v>
+        <v>677.4193548387098</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>701.670927</v>
+        <v>755.488914</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>72.63866893548379</v>
+        <v>78.06955916129027</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>0.1154768583076921</v>
+        <v>0.1152455397142856</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>36.93004878947369</v>
+        <v>39.76257442105263</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>24.93004878947369</v>
+        <v>27.76257442105264</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>18.2328190743338</v>
+        <v>19.63534361851332</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-15.2328190743338</v>
+        <v>-16.63534361851332</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>419.3548387096774</v>
+        <v>451.6129032258065</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>373.86</v>
+        <v>401.93</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-45.49483870967742</v>
+        <v>-49.68290322580646</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.1084876923076923</v>
+        <v>-0.1100121428571428</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>124.62</v>
+        <v>133.9766666666667</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>101.62</v>
+        <v>110.9766666666667</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>180.4201050262565</v>
+        <v>194.2985746436609</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-64.42010502625655</v>
+        <v>-78.29857464366091</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>7758.064516129032</v>
+        <v>8354.838709677419</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>7669.819052</v>
+        <v>8184.57796</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-88.24546412903237</v>
+        <v>-170.2607496774181</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0113746752099792</v>
+        <v>-0.0203786997683396</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>66.11912975862069</v>
+        <v>70.55670655172415</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>23.11912975862069</v>
+        <v>27.55670655172415</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>278.6797813958736</v>
+        <v>300.1166876570946</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-112.6797813958736</v>
+        <v>-134.1166876570946</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>6709.677419354839</v>
+        <v>7225.806451612903</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>6652.222938</v>
+        <v>7109.065144</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>-57.45448135483912</v>
+        <v>-116.7413076129033</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>-0.0085629275096154</v>
+        <v>-0.0161561631071428</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>40.0736321566265</v>
+        <v>42.82569363855422</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>15.996975480111</v>
+        <v>18.74903696203872</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4350,28 +4350,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>450.187969924812</v>
+        <v>500.2088554720134</v>
       </c>
       <c r="R19" t="n">
         <v>198</v>
       </c>
       <c r="S19" t="n">
-        <v>-252.187969924812</v>
+        <v>-302.2088554720134</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>3642.857142857143</v>
+        <v>4047.619047619048</v>
       </c>
       <c r="V19" s="135" t="n">
         <v>1606.8</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-2036.057142857143</v>
+        <v>-2440.819047619048</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.5589176470588235</v>
+        <v>-0.6030258823529412</v>
       </c>
       <c r="Y19" s="135" t="n">
         <v>8.115151515151515</v>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>909.287856346942</v>
+        <v>994.6241177727688</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-429.2878563469421</v>
+        <v>-514.6241177727688</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>18110.59907834101</v>
+        <v>19628.26420890937</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>15928.84199</v>
+        <v>16900.443104</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-2181.757088341012</v>
+        <v>-2727.82110490937</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1204685211628497</v>
+        <v>-0.1389741383077163</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>33.18508747916667</v>
+        <v>35.20925646666667</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>13.14047889012908</v>
+        <v>15.16464787762909</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46248.29186342593</v>
+        <v>46249.29186342593</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-16
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 14/08/2026  |  Ultimo aggiornamento: 15/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 15/08/2026  |  Ultimo aggiornamento: 16/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>3612.903225806452</v>
+        <v>3870.967741935484</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>3685.611495</v>
+        <v>3932.884809</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>72.7082691935484</v>
+        <v>61.91706706451623</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0201246102232142</v>
+        <v>0.015995242325</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>451.6129032258065</v>
+        <v>483.8709677419355</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>469.206465</v>
+        <v>500.43121</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>17.59356177419352</v>
+        <v>16.56024225806453</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>0.0389571724999999</v>
+        <v>0.0342245006666667</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>4290.322580645161</v>
+        <v>4596.774193548387</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>4029.76</v>
+        <v>4255.02</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-260.5625806451608</v>
+        <v>-341.7541935483869</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0607326315789472</v>
+        <v>-0.0743465263157894</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>194.2985746436609</v>
+        <v>208.1770442610652</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-78.29857464366091</v>
+        <v>-92.17704426106523</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>8354.838709677419</v>
+        <v>8951.612903225807</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>8184.57796</v>
+        <v>8688.336019</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-170.2607496774181</v>
+        <v>-263.2768842258065</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0203786997683396</v>
+        <v>-0.0294111113909909</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>70.55670655172415</v>
+        <v>74.89944843965517</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>27.55670655172415</v>
+        <v>31.89944843965517</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>29.1363163371488</v>
+        <v>31.21748178980229</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-7.136316337148799</v>
+        <v>-9.217481789802283</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>903.2258064516128</v>
+        <v>967.741935483871</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>1014.072829</v>
+        <v>1059.685689</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>110.847022548387</v>
+        <v>91.94375351612894</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.1227234892499999</v>
+        <v>0.0950085452999999</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>46.0942195</v>
+        <v>48.16753131818182</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>15.0942195</v>
+        <v>17.16753131818182</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>48.82301656495205</v>
+        <v>52.31037489102005</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-28.82301656495205</v>
+        <v>-32.31037489102005</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>1806.451612903226</v>
+        <v>1935.483870967742</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>1838.972885</v>
+        <v>1965.460184</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>32.52127209677406</v>
+        <v>29.97631303225808</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>0.0180028470535713</v>
+        <v>0.0154877617333333</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>91.94864425</v>
+        <v>98.2730092</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>54.94864425</v>
+        <v>61.2730092</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>3.89321468298109</v>
+        <v>4.171301446051168</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-1.893214682981091</v>
+        <v>-2.171301446051168</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>225.8064516129032</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>232.31417</v>
+        <v>247.463069</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>6.507718387096759</v>
+        <v>5.527585129032246</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0288198957142856</v>
+        <v>0.0228473518666666</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>116.157085</v>
+        <v>123.7315345</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>58.157085</v>
+        <v>65.7315345</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,28 +1540,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>1.411290322580645</v>
+        <v>1.512096774193548</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-0.411290322580645</v>
+        <v>-0.5120967741935483</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>225.8064516129032</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="R12" s="117" t="n">
         <v>89.656346</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-136.1501056129032</v>
+        <v>-152.2791378709678</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.6029504677142858</v>
+        <v>-0.6294204365333333</v>
       </c>
       <c r="U12" s="117" t="n">
         <v>89.656346</v>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>130.7300509337861</v>
+        <v>140.0679117147708</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-38.73005093378606</v>
+        <v>-48.06791171477079</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>2483.870967741935</v>
+        <v>2661.290322580645</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>2496.76</v>
+        <v>2615.47</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>12.88903225806507</v>
+        <v>-45.8203225806451</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.0051890909090911</v>
+        <v>-0.0172173333333333</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>27.13869565217392</v>
+        <v>28.42902173913044</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>8.138695652173915</v>
+        <v>9.429021739130434</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>7.526881720430109</v>
+        <v>8.06451612903226</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-0.5268817204301088</v>
+        <v>-1.06451612903226</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>225.8064516129032</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>139.96</v>
+        <v>149.64</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-85.84645161290322</v>
+        <v>-92.29548387096776</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3801771428571428</v>
+        <v>-0.381488</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>19.99428571428572</v>
+        <v>21.37714285714285</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-10.00571428571428</v>
+        <v>-8.622857142857146</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>2.508960573476702</v>
+        <v>2.688172043010753</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-2.508960573476702</v>
+        <v>-2.688172043010753</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>225.8064516129032</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>139.91</v>
+        <v>150.42</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-85.89645161290323</v>
+        <v>-91.51548387096776</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3803985714285715</v>
+        <v>-0.378264</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>56.45161290322581</v>
+        <v>60.48387096774194</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-37.45161290322581</v>
+        <v>-41.48387096774194</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>677.4193548387098</v>
+        <v>725.8064516129033</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>755.488914</v>
+        <v>789.344701</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>78.06955916129027</v>
+        <v>63.5382493870967</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.1152455397142856</v>
+        <v>0.0875415880444443</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>39.76257442105263</v>
+        <v>41.54445794736842</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>27.76257442105264</v>
+        <v>29.54445794736842</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>19.63534361851332</v>
+        <v>21.03786816269285</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-16.63534361851332</v>
+        <v>-18.03786816269285</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>451.6129032258065</v>
+        <v>483.8709677419355</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>401.93</v>
+        <v>427.36</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-49.68290322580646</v>
+        <v>-56.51096774193547</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.1100121428571428</v>
+        <v>-0.1167893333333333</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>133.9766666666667</v>
+        <v>142.4533333333333</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>110.9766666666667</v>
+        <v>119.4533333333334</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>300.1166876570946</v>
+        <v>321.5535939183156</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-134.1166876570946</v>
+        <v>-155.5535939183156</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>7225.806451612903</v>
+        <v>7741.935483870968</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>7109.065144</v>
+        <v>7494.499989</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>-116.7413076129033</v>
+        <v>-247.4354948709679</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>-0.0161561631071428</v>
+        <v>-0.0319604180875</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>42.82569363855422</v>
+        <v>45.14759029518072</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>18.74903696203872</v>
+        <v>21.07093361866522</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>994.6241177727688</v>
+        <v>1029.939493651394</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-514.6241177727688</v>
+        <v>-549.9394936513943</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>19628.26420890937</v>
+        <v>20741.16743471582</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>16900.443104</v>
+        <v>17789.636008</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-2727.82110490937</v>
+        <v>-2951.531426715821</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1389741383077163</v>
+        <v>-0.1423030519379373</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>35.20925646666667</v>
+        <v>37.06174168333334</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>15.16464787762909</v>
+        <v>17.01713309429575</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>3612.903225806452</v>
+        <v>3870.967741935484</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>3685.611495</v>
+        <v>3932.884809</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>72.7082691935484</v>
+        <v>61.91706706451623</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0201246102232142</v>
+        <v>0.015995242325</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>451.6129032258065</v>
+        <v>483.8709677419355</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>469.206465</v>
+        <v>500.43121</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>17.59356177419352</v>
+        <v>16.56024225806453</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>0.0389571724999999</v>
+        <v>0.0342245006666667</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>4290.322580645161</v>
+        <v>4596.774193548387</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>4029.76</v>
+        <v>4255.02</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-260.5625806451608</v>
+        <v>-341.7541935483869</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0607326315789472</v>
+        <v>-0.0743465263157894</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>29.1363163371488</v>
+        <v>31.21748178980229</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-7.136316337148799</v>
+        <v>-9.217481789802283</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>903.2258064516128</v>
+        <v>967.741935483871</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>1014.072829</v>
+        <v>1059.685689</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>110.847022548387</v>
+        <v>91.94375351612894</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>0.1227234892499999</v>
+        <v>0.0950085452999999</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>46.0942195</v>
+        <v>48.16753131818182</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>15.0942195</v>
+        <v>17.16753131818182</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>48.82301656495205</v>
+        <v>52.31037489102005</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-28.82301656495205</v>
+        <v>-32.31037489102005</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>1806.451612903226</v>
+        <v>1935.483870967742</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>1838.972885</v>
+        <v>1965.460184</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>32.52127209677406</v>
+        <v>29.97631303225808</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.0180028470535713</v>
+        <v>0.0154877617333333</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>91.94864425</v>
+        <v>98.2730092</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>54.94864425</v>
+        <v>61.2730092</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>3.89321468298109</v>
+        <v>4.171301446051168</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-1.893214682981091</v>
+        <v>-2.171301446051168</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>225.8064516129032</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>232.31417</v>
+        <v>247.463069</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>6.507718387096759</v>
+        <v>5.527585129032246</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0288198957142856</v>
+        <v>0.0228473518666666</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>116.157085</v>
+        <v>123.7315345</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>58.157085</v>
+        <v>65.7315345</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,28 +3563,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.411290322580645</v>
+        <v>1.512096774193548</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.411290322580645</v>
+        <v>-0.5120967741935483</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>225.8064516129032</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="V11" s="135" t="n">
         <v>89.656346</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-136.1501056129032</v>
+        <v>-152.2791378709678</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.6029504677142858</v>
+        <v>-0.6294204365333333</v>
       </c>
       <c r="Y11" s="135" t="n">
         <v>89.656346</v>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>130.7300509337861</v>
+        <v>140.0679117147708</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-38.73005093378606</v>
+        <v>-48.06791171477079</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>2483.870967741935</v>
+        <v>2661.290322580645</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>2496.76</v>
+        <v>2615.47</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>12.88903225806507</v>
+        <v>-45.8203225806451</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.0051890909090911</v>
+        <v>-0.0172173333333333</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>27.13869565217392</v>
+        <v>28.42902173913044</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>8.138695652173915</v>
+        <v>9.429021739130434</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>7.526881720430109</v>
+        <v>8.06451612903226</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>-0.5268817204301088</v>
+        <v>-1.06451612903226</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>225.8064516129032</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>139.96</v>
+        <v>149.64</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-85.84645161290322</v>
+        <v>-92.29548387096776</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3801771428571428</v>
+        <v>-0.381488</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>19.99428571428572</v>
+        <v>21.37714285714285</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-10.00571428571428</v>
+        <v>-8.622857142857146</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>2.508960573476702</v>
+        <v>2.688172043010753</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-2.508960573476702</v>
+        <v>-2.688172043010753</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>225.8064516129032</v>
+        <v>241.9354838709677</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>139.91</v>
+        <v>150.42</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-85.89645161290323</v>
+        <v>-91.51548387096776</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3803985714285715</v>
+        <v>-0.378264</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>56.45161290322581</v>
+        <v>60.48387096774194</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-37.45161290322581</v>
+        <v>-41.48387096774194</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>677.4193548387098</v>
+        <v>725.8064516129033</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>755.488914</v>
+        <v>789.344701</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>78.06955916129027</v>
+        <v>63.5382493870967</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>0.1152455397142856</v>
+        <v>0.0875415880444443</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>39.76257442105263</v>
+        <v>41.54445794736842</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>27.76257442105264</v>
+        <v>29.54445794736842</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>19.63534361851332</v>
+        <v>21.03786816269285</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-16.63534361851332</v>
+        <v>-18.03786816269285</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>451.6129032258065</v>
+        <v>483.8709677419355</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>401.93</v>
+        <v>427.36</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-49.68290322580646</v>
+        <v>-56.51096774193547</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.1100121428571428</v>
+        <v>-0.1167893333333333</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>133.9766666666667</v>
+        <v>142.4533333333333</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>110.9766666666667</v>
+        <v>119.4533333333334</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>194.2985746436609</v>
+        <v>208.1770442610652</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-78.29857464366091</v>
+        <v>-92.17704426106523</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>8354.838709677419</v>
+        <v>8951.612903225807</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>8184.57796</v>
+        <v>8688.336019</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-170.2607496774181</v>
+        <v>-263.2768842258065</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0203786997683396</v>
+        <v>-0.0294111113909909</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>70.55670655172415</v>
+        <v>74.89944843965517</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>27.55670655172415</v>
+        <v>31.89944843965517</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>300.1166876570946</v>
+        <v>321.5535939183156</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-134.1166876570946</v>
+        <v>-155.5535939183156</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>7225.806451612903</v>
+        <v>7741.935483870968</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>7109.065144</v>
+        <v>7494.499989</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>-116.7413076129033</v>
+        <v>-247.4354948709679</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>-0.0161561631071428</v>
+        <v>-0.0319604180875</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>42.82569363855422</v>
+        <v>45.14759029518072</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>18.74903696203872</v>
+        <v>21.07093361866522</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>994.6241177727688</v>
+        <v>1029.939493651394</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-514.6241177727688</v>
+        <v>-549.9394936513943</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>19628.26420890937</v>
+        <v>20741.16743471582</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>16900.443104</v>
+        <v>17789.636008</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-2727.82110490937</v>
+        <v>-2951.531426715821</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1389741383077163</v>
+        <v>-0.1423030519379373</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>35.20925646666667</v>
+        <v>37.06174168333334</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>15.16464787762909</v>
+        <v>17.01713309429575</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46248</v>
+        <v>46249</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46249.29186342593</v>
+        <v>46250.29188657407</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-17
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 15/08/2026  |  Ultimo aggiornamento: 16/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 16/08/2026  |  Ultimo aggiornamento: 17/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>3870.967741935484</v>
+        <v>4129.032258064516</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>3932.884809</v>
+        <v>4155.458576</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>61.91706706451623</v>
+        <v>26.42631793548389</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.015995242325</v>
+        <v>0.006400123875</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>483.8709677419355</v>
+        <v>516.1290322580645</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>500.43121</v>
+        <v>525.645997</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>16.56024225806453</v>
+        <v>9.516964741935451</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>0.0342245006666667</v>
+        <v>0.0184391191874999</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>4596.774193548387</v>
+        <v>4903.225806451613</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>4255.02</v>
+        <v>4577.85</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-341.7541935483869</v>
+        <v>-325.3758064516123</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0743465263157894</v>
+        <v>-0.0663595394736841</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>208.1770442610652</v>
+        <v>222.0555138784696</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-92.17704426106523</v>
+        <v>-106.0555138784696</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>8951.612903225807</v>
+        <v>9548.387096774191</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>8688.336019</v>
+        <v>9258.954573000001</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-263.2768842258065</v>
+        <v>-289.4325237741923</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0294111113909909</v>
+        <v>-0.0303121899898647</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>74.89944843965517</v>
+        <v>79.81857390517243</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>31.89944843965517</v>
+        <v>36.81857390517243</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>31.21748178980229</v>
+        <v>33.29864724245577</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-9.217481789802283</v>
+        <v>-11.29864724245577</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>967.741935483871</v>
+        <v>1032.258064516129</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>1059.685689</v>
+        <v>1109.485964</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>91.94375351612894</v>
+        <v>77.22789948387094</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.0950085452999999</v>
+        <v>0.0748145276249999</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>48.16753131818182</v>
+        <v>50.43118018181818</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>17.16753131818182</v>
+        <v>19.43118018181818</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>52.31037489102005</v>
+        <v>55.79773321708806</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-32.31037489102005</v>
+        <v>-35.79773321708806</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>1935.483870967742</v>
+        <v>2064.516129032258</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>1965.460184</v>
+        <v>2066.795089</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>29.97631303225808</v>
+        <v>2.27895996774214</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>0.0154877617333333</v>
+        <v>0.001103871234375</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>98.2730092</v>
+        <v>103.33975445</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>61.2730092</v>
+        <v>66.33975445000002</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>4.171301446051168</v>
+        <v>4.449388209121246</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-2.171301446051168</v>
+        <v>-2.449388209121246</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>241.9354838709677</v>
+        <v>258.0645161290323</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>247.463069</v>
+        <v>264.212647</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>5.527585129032246</v>
+        <v>6.148130870967748</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0228473518666666</v>
+        <v>0.023824007125</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>123.7315345</v>
+        <v>132.1063235</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>65.7315345</v>
+        <v>74.1063235</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,28 +1540,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>1.512096774193548</v>
+        <v>1.612903225806452</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-0.5120967741935483</v>
+        <v>-0.6129032258064515</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>241.9354838709677</v>
+        <v>258.0645161290323</v>
       </c>
       <c r="R12" s="117" t="n">
         <v>89.656346</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-152.2791378709678</v>
+        <v>-168.4081701290323</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.6294204365333333</v>
+        <v>-0.65258165925</v>
       </c>
       <c r="U12" s="117" t="n">
         <v>89.656346</v>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>140.0679117147708</v>
+        <v>149.4057724957555</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-48.06791171477079</v>
+        <v>-57.40577249575552</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>2661.290322580645</v>
+        <v>2838.709677419354</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>2615.47</v>
+        <v>2819.47</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>-45.8203225806451</v>
+        <v>-19.23967741935485</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>-0.0172173333333333</v>
+        <v>-0.0067776136363636</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>28.42902173913044</v>
+        <v>30.64641304347826</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>9.429021739130434</v>
+        <v>11.64641304347826</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>8.06451612903226</v>
+        <v>8.60215053763441</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-1.06451612903226</v>
+        <v>-1.60215053763441</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>241.9354838709677</v>
+        <v>258.0645161290323</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>149.64</v>
+        <v>161.85</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-92.29548387096776</v>
+        <v>-96.21451612903226</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.381488</v>
+        <v>-0.37283125</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>21.37714285714285</v>
+        <v>23.12142857142857</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-8.622857142857146</v>
+        <v>-6.87857142857143</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>2.688172043010753</v>
+        <v>2.867383512544803</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-2.688172043010753</v>
+        <v>-2.867383512544803</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>241.9354838709677</v>
+        <v>258.0645161290323</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>150.42</v>
+        <v>163.16</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-91.51548387096776</v>
+        <v>-94.90451612903226</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.378264</v>
+        <v>-0.367755</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>60.48387096774194</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-41.48387096774194</v>
+        <v>-45.51612903225806</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>725.8064516129033</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>789.344701</v>
+        <v>823.406868</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>63.5382493870967</v>
+        <v>49.21331961290321</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.0875415880444443</v>
+        <v>0.0635672044999999</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>41.54445794736842</v>
+        <v>43.33720357894737</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>29.54445794736842</v>
+        <v>31.33720357894737</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>21.03786816269285</v>
+        <v>22.44039270687237</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-18.03786816269285</v>
+        <v>-19.44039270687237</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>483.8709677419355</v>
+        <v>516.1290322580645</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>427.36</v>
+        <v>461.74</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-56.51096774193547</v>
+        <v>-54.3890322580645</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.1167893333333333</v>
+        <v>-0.1053787499999999</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>142.4533333333333</v>
+        <v>153.9133333333333</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>119.4533333333334</v>
+        <v>130.9133333333333</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>321.5535939183156</v>
+        <v>342.9905001795367</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-155.5535939183156</v>
+        <v>-176.9905001795367</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>7741.935483870968</v>
+        <v>8258.064516129032</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>7494.499989</v>
+        <v>7959.776914</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>-247.4354948709679</v>
+        <v>-298.2876021290322</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>-0.0319604180875</v>
+        <v>-0.0361207643203124</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>45.14759029518072</v>
+        <v>47.9504633373494</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>21.07093361866522</v>
+        <v>23.8738066608339</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>1029.939493651394</v>
+        <v>1065.25486953002</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-549.9394936513943</v>
+        <v>-585.2548695300197</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>20741.16743471582</v>
+        <v>21854.07066052228</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>17789.636008</v>
+        <v>18825.531487</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-2951.531426715821</v>
+        <v>-3028.539173522273</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1423030519379373</v>
+        <v>-0.138580094325086</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>37.06174168333334</v>
+        <v>39.21985726458333</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>17.01713309429575</v>
+        <v>19.17524867554575</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>3870.967741935484</v>
+        <v>4129.032258064516</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>3932.884809</v>
+        <v>4155.458576</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>61.91706706451623</v>
+        <v>26.42631793548389</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.015995242325</v>
+        <v>0.006400123875</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>483.8709677419355</v>
+        <v>516.1290322580645</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>500.43121</v>
+        <v>525.645997</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>16.56024225806453</v>
+        <v>9.516964741935451</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>0.0342245006666667</v>
+        <v>0.0184391191874999</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>4596.774193548387</v>
+        <v>4903.225806451613</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>4255.02</v>
+        <v>4577.85</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-341.7541935483869</v>
+        <v>-325.3758064516123</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0743465263157894</v>
+        <v>-0.0663595394736841</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>31.21748178980229</v>
+        <v>33.29864724245577</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-9.217481789802283</v>
+        <v>-11.29864724245577</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>967.741935483871</v>
+        <v>1032.258064516129</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>1059.685689</v>
+        <v>1109.485964</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>91.94375351612894</v>
+        <v>77.22789948387094</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>0.0950085452999999</v>
+        <v>0.0748145276249999</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>48.16753131818182</v>
+        <v>50.43118018181818</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>17.16753131818182</v>
+        <v>19.43118018181818</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>52.31037489102005</v>
+        <v>55.79773321708806</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-32.31037489102005</v>
+        <v>-35.79773321708806</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>1935.483870967742</v>
+        <v>2064.516129032258</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>1965.460184</v>
+        <v>2066.795089</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>29.97631303225808</v>
+        <v>2.27895996774214</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.0154877617333333</v>
+        <v>0.001103871234375</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>98.2730092</v>
+        <v>103.33975445</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>61.2730092</v>
+        <v>66.33975445000002</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>4.171301446051168</v>
+        <v>4.449388209121246</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-2.171301446051168</v>
+        <v>-2.449388209121246</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>241.9354838709677</v>
+        <v>258.0645161290323</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>247.463069</v>
+        <v>264.212647</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>5.527585129032246</v>
+        <v>6.148130870967748</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0228473518666666</v>
+        <v>0.023824007125</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>123.7315345</v>
+        <v>132.1063235</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>65.7315345</v>
+        <v>74.1063235</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,28 +3563,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.512096774193548</v>
+        <v>1.612903225806452</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.5120967741935483</v>
+        <v>-0.6129032258064515</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>241.9354838709677</v>
+        <v>258.0645161290323</v>
       </c>
       <c r="V11" s="135" t="n">
         <v>89.656346</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-152.2791378709678</v>
+        <v>-168.4081701290323</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.6294204365333333</v>
+        <v>-0.65258165925</v>
       </c>
       <c r="Y11" s="135" t="n">
         <v>89.656346</v>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>140.0679117147708</v>
+        <v>149.4057724957555</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-48.06791171477079</v>
+        <v>-57.40577249575552</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>2661.290322580645</v>
+        <v>2838.709677419354</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>2615.47</v>
+        <v>2819.47</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>-45.8203225806451</v>
+        <v>-19.23967741935485</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>-0.0172173333333333</v>
+        <v>-0.0067776136363636</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>28.42902173913044</v>
+        <v>30.64641304347826</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>9.429021739130434</v>
+        <v>11.64641304347826</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>8.06451612903226</v>
+        <v>8.60215053763441</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>-1.06451612903226</v>
+        <v>-1.60215053763441</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>241.9354838709677</v>
+        <v>258.0645161290323</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>149.64</v>
+        <v>161.85</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-92.29548387096776</v>
+        <v>-96.21451612903226</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.381488</v>
+        <v>-0.37283125</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>21.37714285714285</v>
+        <v>23.12142857142857</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-8.622857142857146</v>
+        <v>-6.87857142857143</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>2.688172043010753</v>
+        <v>2.867383512544803</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-2.688172043010753</v>
+        <v>-2.867383512544803</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>241.9354838709677</v>
+        <v>258.0645161290323</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>150.42</v>
+        <v>163.16</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-91.51548387096776</v>
+        <v>-94.90451612903226</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.378264</v>
+        <v>-0.367755</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>60.48387096774194</v>
+        <v>64.51612903225806</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-41.48387096774194</v>
+        <v>-45.51612903225806</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>725.8064516129033</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>789.344701</v>
+        <v>823.406868</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>63.5382493870967</v>
+        <v>49.21331961290321</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>0.0875415880444443</v>
+        <v>0.0635672044999999</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>41.54445794736842</v>
+        <v>43.33720357894737</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>29.54445794736842</v>
+        <v>31.33720357894737</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>21.03786816269285</v>
+        <v>22.44039270687237</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-18.03786816269285</v>
+        <v>-19.44039270687237</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>483.8709677419355</v>
+        <v>516.1290322580645</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>427.36</v>
+        <v>461.74</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-56.51096774193547</v>
+        <v>-54.3890322580645</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.1167893333333333</v>
+        <v>-0.1053787499999999</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>142.4533333333333</v>
+        <v>153.9133333333333</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>119.4533333333334</v>
+        <v>130.9133333333333</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>208.1770442610652</v>
+        <v>222.0555138784696</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-92.17704426106523</v>
+        <v>-106.0555138784696</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>8951.612903225807</v>
+        <v>9548.387096774191</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>8688.336019</v>
+        <v>9258.954573000001</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-263.2768842258065</v>
+        <v>-289.4325237741923</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0294111113909909</v>
+        <v>-0.0303121899898647</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>74.89944843965517</v>
+        <v>79.81857390517243</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>31.89944843965517</v>
+        <v>36.81857390517243</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>321.5535939183156</v>
+        <v>342.9905001795367</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-155.5535939183156</v>
+        <v>-176.9905001795367</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>7741.935483870968</v>
+        <v>8258.064516129032</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>7494.499989</v>
+        <v>7959.776914</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>-247.4354948709679</v>
+        <v>-298.2876021290322</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>-0.0319604180875</v>
+        <v>-0.0361207643203124</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>45.14759029518072</v>
+        <v>47.9504633373494</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>21.07093361866522</v>
+        <v>23.8738066608339</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>1029.939493651394</v>
+        <v>1065.25486953002</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-549.9394936513943</v>
+        <v>-585.2548695300197</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>20741.16743471582</v>
+        <v>21854.07066052228</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>17789.636008</v>
+        <v>18825.531487</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-2951.531426715821</v>
+        <v>-3028.539173522273</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1423030519379373</v>
+        <v>-0.138580094325086</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>37.06174168333334</v>
+        <v>39.21985726458333</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>17.01713309429575</v>
+        <v>19.17524867554575</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46250.29188657407</v>
+        <v>46251.29186342593</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-18
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 16/08/2026  |  Ultimo aggiornamento: 17/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 17/08/2026  |  Ultimo aggiornamento: 18/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>4129.032258064516</v>
+        <v>4387.096774193548</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>4155.458576</v>
+        <v>4412.23302</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>26.42631793548389</v>
+        <v>25.13624580645137</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.006400123875</v>
+        <v>0.0057295854411764</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>516.1290322580645</v>
+        <v>548.3870967741935</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>525.645997</v>
+        <v>553.671743</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>9.516964741935451</v>
+        <v>5.284646225806455</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>0.0184391191874999</v>
+        <v>0.0096367078235294</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>4903.225806451613</v>
+        <v>5209.677419354838</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>4577.85</v>
+        <v>4905.29</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-325.3758064516123</v>
+        <v>-304.3874193548381</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0663595394736841</v>
+        <v>-0.0584273065015478</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>222.0555138784696</v>
+        <v>235.933983495874</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-106.0555138784696</v>
+        <v>-119.933983495874</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>9548.387096774191</v>
+        <v>10145.16129032258</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>9258.954573000001</v>
+        <v>9871.194763</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-289.4325237741923</v>
+        <v>-273.9665273225801</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0303121899898647</v>
+        <v>-0.0270046497519872</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>79.81857390517243</v>
+        <v>85.0965065775862</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>36.81857390517243</v>
+        <v>42.0965065775862</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>33.29864724245577</v>
+        <v>35.37981269510926</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-11.29864724245577</v>
+        <v>-13.37981269510926</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>1032.258064516129</v>
+        <v>1096.774193548387</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>1109.485964</v>
+        <v>1151.519237</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>77.22789948387094</v>
+        <v>54.7450434516129</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.0748145276249999</v>
+        <v>0.0499145984411764</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>50.43118018181818</v>
+        <v>52.3417835</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>19.43118018181818</v>
+        <v>21.3417835</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>55.79773321708806</v>
+        <v>59.28509154315606</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-35.79773321708806</v>
+        <v>-39.28509154315606</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>2064.516129032258</v>
+        <v>2193.548387096774</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>2066.795089</v>
+        <v>2194.825089</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>2.27895996774214</v>
+        <v>1.276701903225785</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>0.001103871234375</v>
+        <v>0.000582025867647</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>103.33975445</v>
+        <v>109.74125445</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>66.33975445000002</v>
+        <v>72.74125445</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>4.449388209121246</v>
+        <v>4.727474972191325</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-2.449388209121246</v>
+        <v>-2.727474972191325</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>258.0645161290323</v>
+        <v>274.1935483870968</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>264.212647</v>
+        <v>279.660959</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>6.148130870967748</v>
+        <v>5.467410612903223</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.023824007125</v>
+        <v>0.019939968117647</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>132.1063235</v>
+        <v>139.8304795</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>74.1063235</v>
+        <v>81.8304795</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,34 +1540,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>1.612903225806452</v>
+        <v>1.713709677419355</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-0.6129032258064515</v>
+        <v>-0.7137096774193548</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>258.0645161290323</v>
+        <v>274.1935483870968</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>89.656346</v>
+        <v>97.33634600000001</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-168.4081701290323</v>
+        <v>-176.8572023870968</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.65258165925</v>
+        <v>-0.6450086204705883</v>
       </c>
       <c r="U12" s="117" t="n">
-        <v>89.656346</v>
+        <v>97.33634600000001</v>
       </c>
       <c r="V12" s="117" t="n">
-        <v>-70.343654</v>
+        <v>-62.663654</v>
       </c>
       <c r="W12" s="120" t="inlineStr"/>
     </row>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>149.4057724957555</v>
+        <v>158.7436332767402</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-57.40577249575552</v>
+        <v>-66.74363327674024</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>2838.709677419354</v>
+        <v>3016.129032258064</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>2819.47</v>
+        <v>3009.96</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>-19.23967741935485</v>
+        <v>-6.169032258064362</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>-0.0067776136363636</v>
+        <v>-0.0020453475935828</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>30.64641304347826</v>
+        <v>32.71695652173913</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>11.64641304347826</v>
+        <v>13.71695652173913</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>8.60215053763441</v>
+        <v>9.13978494623656</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-1.60215053763441</v>
+        <v>-2.13978494623656</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>258.0645161290323</v>
+        <v>274.1935483870968</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>161.85</v>
+        <v>174.17</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-96.21451612903226</v>
+        <v>-100.0235483870968</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.37283125</v>
+        <v>-0.3647917647058823</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>23.12142857142857</v>
+        <v>24.88142857142857</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-6.87857142857143</v>
+        <v>-5.118571428571432</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>2.867383512544803</v>
+        <v>3.046594982078853</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-2.867383512544803</v>
+        <v>-3.046594982078853</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>258.0645161290323</v>
+        <v>274.1935483870968</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>163.16</v>
+        <v>171.67</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-94.90451612903226</v>
+        <v>-102.5235483870968</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.367755</v>
+        <v>-0.3739094117647059</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>64.51612903225806</v>
+        <v>68.54838709677419</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-45.51612903225806</v>
+        <v>-49.54838709677419</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>774.1935483870968</v>
+        <v>822.5806451612904</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>823.406868</v>
+        <v>858.955881</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>49.21331961290321</v>
+        <v>36.37523583870961</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.0635672044999999</v>
+        <v>0.0442208749411763</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>43.33720357894737</v>
+        <v>45.2082042631579</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>31.33720357894737</v>
+        <v>33.2082042631579</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>22.44039270687237</v>
+        <v>23.84291725105189</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-19.44039270687237</v>
+        <v>-20.84291725105189</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>516.1290322580645</v>
+        <v>548.3870967741935</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>461.74</v>
+        <v>496.81</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-54.3890322580645</v>
+        <v>-51.57709677419354</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.1053787499999999</v>
+        <v>-0.09405235294117641</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>153.9133333333333</v>
+        <v>165.6033333333333</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>130.9133333333333</v>
+        <v>142.6033333333333</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>342.9905001795367</v>
+        <v>364.4274064407577</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-176.9905001795367</v>
+        <v>-198.4274064407577</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>8258.064516129032</v>
+        <v>8774.193548387097</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>7959.776914</v>
+        <v>8434.907512</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>-298.2876021290322</v>
+        <v>-339.2860363870968</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>-0.0361207643203124</v>
+        <v>-0.0386686291470588</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>47.9504633373494</v>
+        <v>50.81269585542169</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>23.8738066608339</v>
+        <v>26.73603917890619</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2063,28 +2063,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>281.9548872180451</v>
+        <v>310.1503759398497</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>93</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-188.9548872180452</v>
+        <v>-217.1503759398497</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>2142.857142857143</v>
+        <v>2357.142857142857</v>
       </c>
       <c r="R19" s="117" t="n">
         <v>706.8</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-1436.057142857143</v>
+        <v>-1650.342857142857</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.67016</v>
+        <v>-0.7001454545454545</v>
       </c>
       <c r="U19" s="117" t="n">
         <v>7.6</v>
@@ -2138,28 +2138,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>158.7301587301587</v>
+        <v>174.6031746031746</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>60</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-98.73015873015871</v>
+        <v>-114.6031746031746</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>1428.571428571429</v>
+        <v>1571.428571428572</v>
       </c>
       <c r="R20" s="117" t="n">
         <v>540</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-888.5714285714287</v>
+        <v>-1031.428571428572</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.622</v>
+        <v>-0.6563636363636364</v>
       </c>
       <c r="U20" s="117" t="n">
         <v>9</v>
@@ -2213,28 +2213,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>59.52380952380953</v>
+        <v>65.47619047619048</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-14.52380952380953</v>
+        <v>-20.47619047619048</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>476.1904761904762</v>
+        <v>523.8095238095239</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>360</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-116.1904761904762</v>
+        <v>-163.8095238095239</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.244</v>
+        <v>-0.3127272727272728</v>
       </c>
       <c r="U21" s="117" t="n">
         <v>8</v>
@@ -2276,28 +2276,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>500.2088554720134</v>
+        <v>550.2297410192148</v>
       </c>
       <c r="N22" s="125" t="n">
         <v>198</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-302.2088554720134</v>
+        <v>-352.2297410192148</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="Q22" s="123" t="n">
-        <v>4047.619047619048</v>
+        <v>4452.380952380952</v>
       </c>
       <c r="R22" s="123" t="n">
         <v>1606.8</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-2440.819047619048</v>
+        <v>-2845.580952380952</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-0.6030258823529412</v>
+        <v>-0.6391144385026738</v>
       </c>
       <c r="U22" s="123" t="n">
         <v>8.115151515151515</v>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>1065.25486953002</v>
+        <v>1150.591130955846</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-585.2548695300197</v>
+        <v>-670.5911309558464</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>21854.07066052228</v>
+        <v>23371.73579109063</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>18825.531487</v>
+        <v>19912.902275</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-3028.539173522273</v>
+        <v>-3458.833516090628</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.138580094325086</v>
+        <v>-0.1479921537282286</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>39.21985726458333</v>
+        <v>41.48521307291666</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>19.17524867554575</v>
+        <v>21.44060448387908</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>4129.032258064516</v>
+        <v>4387.096774193548</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>4155.458576</v>
+        <v>4412.23302</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>26.42631793548389</v>
+        <v>25.13624580645137</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.006400123875</v>
+        <v>0.0057295854411764</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>516.1290322580645</v>
+        <v>548.3870967741935</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>525.645997</v>
+        <v>553.671743</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>9.516964741935451</v>
+        <v>5.284646225806455</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>0.0184391191874999</v>
+        <v>0.0096367078235294</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>4903.225806451613</v>
+        <v>5209.677419354838</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>4577.85</v>
+        <v>4905.29</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-325.3758064516123</v>
+        <v>-304.3874193548381</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0663595394736841</v>
+        <v>-0.0584273065015478</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2933,28 +2933,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>281.9548872180451</v>
+        <v>310.1503759398497</v>
       </c>
       <c r="R5" t="n">
         <v>93</v>
       </c>
       <c r="S5" t="n">
-        <v>-188.9548872180452</v>
+        <v>-217.1503759398497</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="U5" s="135" t="n">
-        <v>2142.857142857143</v>
+        <v>2357.142857142857</v>
       </c>
       <c r="V5" s="135" t="n">
         <v>706.8</v>
       </c>
       <c r="W5" s="135" t="n">
-        <v>-1436.057142857143</v>
+        <v>-1650.342857142857</v>
       </c>
       <c r="X5" s="136" t="n">
-        <v>-0.67016</v>
+        <v>-0.7001454545454545</v>
       </c>
       <c r="Y5" s="135" t="n">
         <v>7.6</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3036,28 +3036,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>158.7301587301587</v>
+        <v>174.6031746031746</v>
       </c>
       <c r="R6" t="n">
         <v>60</v>
       </c>
       <c r="S6" t="n">
-        <v>-98.73015873015871</v>
+        <v>-114.6031746031746</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>1428.571428571429</v>
+        <v>1571.428571428572</v>
       </c>
       <c r="V6" s="135" t="n">
         <v>540</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-888.5714285714287</v>
+        <v>-1031.428571428572</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.622</v>
+        <v>-0.6563636363636364</v>
       </c>
       <c r="Y6" s="135" t="n">
         <v>9</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3139,28 +3139,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>59.52380952380953</v>
+        <v>65.47619047619048</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>-14.52380952380953</v>
+        <v>-20.47619047619048</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>476.1904761904762</v>
+        <v>523.8095238095239</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>360</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>-116.1904761904762</v>
+        <v>-163.8095238095239</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>-0.244</v>
+        <v>-0.3127272727272728</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>8</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>33.29864724245577</v>
+        <v>35.37981269510926</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-11.29864724245577</v>
+        <v>-13.37981269510926</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>1032.258064516129</v>
+        <v>1096.774193548387</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>1109.485964</v>
+        <v>1151.519237</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>77.22789948387094</v>
+        <v>54.7450434516129</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>0.0748145276249999</v>
+        <v>0.0499145984411764</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>50.43118018181818</v>
+        <v>52.3417835</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>19.43118018181818</v>
+        <v>21.3417835</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>55.79773321708806</v>
+        <v>59.28509154315606</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-35.79773321708806</v>
+        <v>-39.28509154315606</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>2064.516129032258</v>
+        <v>2193.548387096774</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>2066.795089</v>
+        <v>2194.825089</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>2.27895996774214</v>
+        <v>1.276701903225785</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.001103871234375</v>
+        <v>0.000582025867647</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>103.33975445</v>
+        <v>109.74125445</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>66.33975445000002</v>
+        <v>72.74125445</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>4.449388209121246</v>
+        <v>4.727474972191325</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-2.449388209121246</v>
+        <v>-2.727474972191325</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>258.0645161290323</v>
+        <v>274.1935483870968</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>264.212647</v>
+        <v>279.660959</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>6.148130870967748</v>
+        <v>5.467410612903223</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.023824007125</v>
+        <v>0.019939968117647</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>132.1063235</v>
+        <v>139.8304795</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>74.1063235</v>
+        <v>81.8304795</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,34 +3563,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.612903225806452</v>
+        <v>1.713709677419355</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.6129032258064515</v>
+        <v>-0.7137096774193548</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>258.0645161290323</v>
+        <v>274.1935483870968</v>
       </c>
       <c r="V11" s="135" t="n">
-        <v>89.656346</v>
+        <v>97.33634600000001</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-168.4081701290323</v>
+        <v>-176.8572023870968</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.65258165925</v>
+        <v>-0.6450086204705883</v>
       </c>
       <c r="Y11" s="135" t="n">
-        <v>89.656346</v>
+        <v>97.33634600000001</v>
       </c>
       <c r="Z11" s="135" t="n">
-        <v>-70.343654</v>
+        <v>-62.663654</v>
       </c>
       <c r="AB11" s="137" t="inlineStr">
         <is>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>149.4057724957555</v>
+        <v>158.7436332767402</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-57.40577249575552</v>
+        <v>-66.74363327674024</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>2838.709677419354</v>
+        <v>3016.129032258064</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>2819.47</v>
+        <v>3009.96</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>-19.23967741935485</v>
+        <v>-6.169032258064362</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>-0.0067776136363636</v>
+        <v>-0.0020453475935828</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>30.64641304347826</v>
+        <v>32.71695652173913</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>11.64641304347826</v>
+        <v>13.71695652173913</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>8.60215053763441</v>
+        <v>9.13978494623656</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>-1.60215053763441</v>
+        <v>-2.13978494623656</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>258.0645161290323</v>
+        <v>274.1935483870968</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>161.85</v>
+        <v>174.17</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-96.21451612903226</v>
+        <v>-100.0235483870968</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.37283125</v>
+        <v>-0.3647917647058823</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>23.12142857142857</v>
+        <v>24.88142857142857</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-6.87857142857143</v>
+        <v>-5.118571428571432</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>2.867383512544803</v>
+        <v>3.046594982078853</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-2.867383512544803</v>
+        <v>-3.046594982078853</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>258.0645161290323</v>
+        <v>274.1935483870968</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>163.16</v>
+        <v>171.67</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-94.90451612903226</v>
+        <v>-102.5235483870968</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.367755</v>
+        <v>-0.3739094117647059</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>64.51612903225806</v>
+        <v>68.54838709677419</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-45.51612903225806</v>
+        <v>-49.54838709677419</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>774.1935483870968</v>
+        <v>822.5806451612904</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>823.406868</v>
+        <v>858.955881</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>49.21331961290321</v>
+        <v>36.37523583870961</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>0.0635672044999999</v>
+        <v>0.0442208749411763</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>43.33720357894737</v>
+        <v>45.2082042631579</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>31.33720357894737</v>
+        <v>33.2082042631579</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>22.44039270687237</v>
+        <v>23.84291725105189</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-19.44039270687237</v>
+        <v>-20.84291725105189</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>516.1290322580645</v>
+        <v>548.3870967741935</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>461.74</v>
+        <v>496.81</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-54.3890322580645</v>
+        <v>-51.57709677419354</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.1053787499999999</v>
+        <v>-0.09405235294117641</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>153.9133333333333</v>
+        <v>165.6033333333333</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>130.9133333333333</v>
+        <v>142.6033333333333</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>222.0555138784696</v>
+        <v>235.933983495874</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-106.0555138784696</v>
+        <v>-119.933983495874</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>9548.387096774191</v>
+        <v>10145.16129032258</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>9258.954573000001</v>
+        <v>9871.194763</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-289.4325237741923</v>
+        <v>-273.9665273225801</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0303121899898647</v>
+        <v>-0.0270046497519872</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>79.81857390517243</v>
+        <v>85.0965065775862</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>36.81857390517243</v>
+        <v>42.0965065775862</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>342.9905001795367</v>
+        <v>364.4274064407577</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-176.9905001795367</v>
+        <v>-198.4274064407577</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>8258.064516129032</v>
+        <v>8774.193548387097</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>7959.776914</v>
+        <v>8434.907512</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>-298.2876021290322</v>
+        <v>-339.2860363870968</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>-0.0361207643203124</v>
+        <v>-0.0386686291470588</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>47.9504633373494</v>
+        <v>50.81269585542169</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>23.8738066608339</v>
+        <v>26.73603917890619</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4350,28 +4350,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>500.2088554720134</v>
+        <v>550.2297410192148</v>
       </c>
       <c r="R19" t="n">
         <v>198</v>
       </c>
       <c r="S19" t="n">
-        <v>-302.2088554720134</v>
+        <v>-352.2297410192148</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>4047.619047619048</v>
+        <v>4452.380952380952</v>
       </c>
       <c r="V19" s="135" t="n">
         <v>1606.8</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-2440.819047619048</v>
+        <v>-2845.580952380952</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.6030258823529412</v>
+        <v>-0.6391144385026738</v>
       </c>
       <c r="Y19" s="135" t="n">
         <v>8.115151515151515</v>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>1065.25486953002</v>
+        <v>1150.591130955846</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-585.2548695300197</v>
+        <v>-670.5911309558464</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>21854.07066052228</v>
+        <v>23371.73579109063</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>18825.531487</v>
+        <v>19912.902275</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-3028.539173522273</v>
+        <v>-3458.833516090628</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.138580094325086</v>
+        <v>-0.1479921537282286</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>39.21985726458333</v>
+        <v>41.48521307291666</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>19.17524867554575</v>
+        <v>21.44060448387908</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46250</v>
+        <v>46251</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46251.29186342593</v>
+        <v>46252.29188657407</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-19
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 17/08/2026  |  Ultimo aggiornamento: 18/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 18/08/2026  |  Ultimo aggiornamento: 19/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>4387.096774193548</v>
+        <v>4645.16129032258</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>4412.23302</v>
+        <v>4708.950705</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>25.13624580645137</v>
+        <v>63.7894146774197</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0057295854411764</v>
+        <v>0.0137324434375</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>548.3870967741935</v>
+        <v>580.6451612903226</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>553.671743</v>
+        <v>580.421743</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>5.284646225806455</v>
+        <v>-0.2234182903225701</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>0.0096367078235294</v>
+        <v>-0.0003847759444444</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>5209.677419354838</v>
+        <v>5516.129032258064</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>4905.29</v>
+        <v>5186.18</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-304.3874193548381</v>
+        <v>-329.9490322580641</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0584273065015478</v>
+        <v>-0.0598153216374268</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>235.933983495874</v>
+        <v>249.8124531132783</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-119.933983495874</v>
+        <v>-133.8124531132783</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>10145.16129032258</v>
+        <v>10741.93548387097</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>9871.194763</v>
+        <v>10475.552448</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-273.9665273225801</v>
+        <v>-266.3830358709674</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0270046497519872</v>
+        <v>-0.0247984207567567</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>85.0965065775862</v>
+        <v>90.30648662068964</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>42.0965065775862</v>
+        <v>47.30648662068965</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>35.37981269510926</v>
+        <v>37.46097814776275</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-13.37981269510926</v>
+        <v>-15.46097814776274</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>1096.774193548387</v>
+        <v>1161.290322580645</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>1151.519237</v>
+        <v>1197.994656</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>54.7450434516129</v>
+        <v>36.70433341935495</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.0499145984411764</v>
+        <v>0.0316065093333334</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>52.3417835</v>
+        <v>54.45430254545455</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>21.3417835</v>
+        <v>23.45430254545455</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>59.28509154315606</v>
+        <v>62.77244986922407</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-39.28509154315606</v>
+        <v>-42.77244986922407</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>2193.548387096774</v>
+        <v>2322.58064516129</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>2194.825089</v>
+        <v>2317.398099</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>1.276701903225785</v>
+        <v>-5.182546161290247</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>0.000582025867647</v>
+        <v>-0.0022313740416666</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>109.74125445</v>
+        <v>115.86990495</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>72.74125445</v>
+        <v>78.86990495000001</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>4.727474972191325</v>
+        <v>5.005561735261402</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-2.727474972191325</v>
+        <v>-3.005561735261402</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>274.1935483870968</v>
+        <v>290.3225806451613</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>279.660959</v>
+        <v>297.330959</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>5.467410612903223</v>
+        <v>7.008378354838726</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.019939968117647</v>
+        <v>0.0241399698888889</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>139.8304795</v>
+        <v>148.6654795</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>81.8304795</v>
+        <v>90.6654795</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,34 +1540,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>1.713709677419355</v>
+        <v>1.814516129032258</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-0.7137096774193548</v>
+        <v>-0.814516129032258</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>274.1935483870968</v>
+        <v>290.3225806451613</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>97.33634600000001</v>
+        <v>123.536346</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-176.8572023870968</v>
+        <v>-166.7862346451613</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.6450086204705883</v>
+        <v>-0.5744859193333334</v>
       </c>
       <c r="U12" s="117" t="n">
-        <v>97.33634600000001</v>
+        <v>123.536346</v>
       </c>
       <c r="V12" s="117" t="n">
-        <v>-62.663654</v>
+        <v>-36.46365400000001</v>
       </c>
       <c r="W12" s="120" t="inlineStr"/>
     </row>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>158.7436332767402</v>
+        <v>168.081494057725</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-66.74363327674024</v>
+        <v>-76.08149405772497</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>3016.129032258064</v>
+        <v>3193.548387096774</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>3009.96</v>
+        <v>3195.09</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>-6.169032258064362</v>
+        <v>1.541612903225996</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>-0.0020453475935828</v>
+        <v>0.0004827272727273</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>32.71695652173913</v>
+        <v>34.72923913043478</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>13.71695652173913</v>
+        <v>15.72923913043478</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>9.13978494623656</v>
+        <v>9.677419354838712</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-2.13978494623656</v>
+        <v>-2.677419354838712</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>274.1935483870968</v>
+        <v>290.3225806451613</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>174.17</v>
+        <v>184.54</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-100.0235483870968</v>
+        <v>-105.7825806451613</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3647917647058823</v>
+        <v>-0.3643622222222222</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>24.88142857142857</v>
+        <v>26.36285714285714</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-5.118571428571432</v>
+        <v>-3.637142857142859</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>3.046594982078853</v>
+        <v>3.225806451612903</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-3.046594982078853</v>
+        <v>-3.225806451612903</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>274.1935483870968</v>
+        <v>290.3225806451613</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>171.67</v>
+        <v>181.11</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-102.5235483870968</v>
+        <v>-109.2125806451613</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3739094117647059</v>
+        <v>-0.3761766666666666</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>68.54838709677419</v>
+        <v>72.58064516129032</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-49.54838709677419</v>
+        <v>-53.58064516129032</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>822.5806451612904</v>
+        <v>870.9677419354839</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>858.955881</v>
+        <v>887.5860730000001</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>36.37523583870961</v>
+        <v>16.61833106451616</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.0442208749411763</v>
+        <v>0.019080306037037</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>45.2082042631579</v>
+        <v>46.71505647368421</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>33.2082042631579</v>
+        <v>34.71505647368421</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>23.84291725105189</v>
+        <v>25.24544179523141</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-20.84291725105189</v>
+        <v>-22.24544179523141</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>548.3870967741935</v>
+        <v>580.6451612903226</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>496.81</v>
+        <v>529.86</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-51.57709677419354</v>
+        <v>-50.78516129032255</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.09405235294117641</v>
+        <v>-0.0874633333333332</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>165.6033333333333</v>
+        <v>176.62</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>142.6033333333333</v>
+        <v>153.62</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>364.4274064407577</v>
+        <v>385.8643127019788</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-198.4274064407577</v>
+        <v>-219.8643127019788</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>8774.193548387097</v>
+        <v>9290.322580645159</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>8434.907512</v>
+        <v>8914.446132999999</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>-339.2860363870968</v>
+        <v>-375.8764476451615</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>-0.0386686291470588</v>
+        <v>-0.0404589231840278</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>50.81269585542169</v>
+        <v>53.70148272891566</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>26.73603917890619</v>
+        <v>29.62482605240016</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2063,28 +2063,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>310.1503759398497</v>
+        <v>338.3458646616542</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>93</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-217.1503759398497</v>
+        <v>-245.3458646616542</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>2357.142857142857</v>
+        <v>2571.428571428572</v>
       </c>
       <c r="R19" s="117" t="n">
         <v>706.8</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-1650.342857142857</v>
+        <v>-1864.628571428572</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.7001454545454545</v>
+        <v>-0.7251333333333334</v>
       </c>
       <c r="U19" s="117" t="n">
         <v>7.6</v>
@@ -2138,28 +2138,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>174.6031746031746</v>
+        <v>190.4761904761905</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>60</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-114.6031746031746</v>
+        <v>-130.4761904761905</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>1571.428571428572</v>
+        <v>1714.285714285714</v>
       </c>
       <c r="R20" s="117" t="n">
         <v>540</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-1031.428571428572</v>
+        <v>-1174.285714285714</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.6563636363636364</v>
+        <v>-0.6849999999999999</v>
       </c>
       <c r="U20" s="117" t="n">
         <v>9</v>
@@ -2213,28 +2213,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>65.47619047619048</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-20.47619047619048</v>
+        <v>-26.42857142857143</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>523.8095238095239</v>
+        <v>571.4285714285714</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>360</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-163.8095238095239</v>
+        <v>-211.4285714285714</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.3127272727272728</v>
+        <v>-0.37</v>
       </c>
       <c r="U21" s="117" t="n">
         <v>8</v>
@@ -2276,28 +2276,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>550.2297410192148</v>
+        <v>600.250626566416</v>
       </c>
       <c r="N22" s="125" t="n">
         <v>198</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-352.2297410192148</v>
+        <v>-402.2506265664161</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="Q22" s="123" t="n">
-        <v>4452.380952380952</v>
+        <v>4857.142857142857</v>
       </c>
       <c r="R22" s="123" t="n">
         <v>1606.8</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-2845.580952380952</v>
+        <v>-3250.342857142857</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-0.6391144385026738</v>
+        <v>-0.6691882352941176</v>
       </c>
       <c r="U22" s="123" t="n">
         <v>8.115151515151515</v>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>1150.591130955846</v>
+        <v>1235.927392381673</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-670.5911309558464</v>
+        <v>-755.9273923816731</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>23371.73579109063</v>
+        <v>24889.40092165899</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>19912.902275</v>
+        <v>20996.798581</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-3458.833516090628</v>
+        <v>-3892.602340658989</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1479921537282286</v>
+        <v>-0.1563959836924644</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>41.48521307291666</v>
+        <v>43.74333037708333</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>21.44060448387908</v>
+        <v>23.69872178804575</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>4387.096774193548</v>
+        <v>4645.16129032258</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>4412.23302</v>
+        <v>4708.950705</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>25.13624580645137</v>
+        <v>63.7894146774197</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0057295854411764</v>
+        <v>0.0137324434375</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>548.3870967741935</v>
+        <v>580.6451612903226</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>553.671743</v>
+        <v>580.421743</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>5.284646225806455</v>
+        <v>-0.2234182903225701</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>0.0096367078235294</v>
+        <v>-0.0003847759444444</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>5209.677419354838</v>
+        <v>5516.129032258064</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>4905.29</v>
+        <v>5186.18</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-304.3874193548381</v>
+        <v>-329.9490322580641</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0584273065015478</v>
+        <v>-0.0598153216374268</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2933,28 +2933,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>310.1503759398497</v>
+        <v>338.3458646616542</v>
       </c>
       <c r="R5" t="n">
         <v>93</v>
       </c>
       <c r="S5" t="n">
-        <v>-217.1503759398497</v>
+        <v>-245.3458646616542</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="U5" s="135" t="n">
-        <v>2357.142857142857</v>
+        <v>2571.428571428572</v>
       </c>
       <c r="V5" s="135" t="n">
         <v>706.8</v>
       </c>
       <c r="W5" s="135" t="n">
-        <v>-1650.342857142857</v>
+        <v>-1864.628571428572</v>
       </c>
       <c r="X5" s="136" t="n">
-        <v>-0.7001454545454545</v>
+        <v>-0.7251333333333334</v>
       </c>
       <c r="Y5" s="135" t="n">
         <v>7.6</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3036,28 +3036,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>174.6031746031746</v>
+        <v>190.4761904761905</v>
       </c>
       <c r="R6" t="n">
         <v>60</v>
       </c>
       <c r="S6" t="n">
-        <v>-114.6031746031746</v>
+        <v>-130.4761904761905</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>1571.428571428572</v>
+        <v>1714.285714285714</v>
       </c>
       <c r="V6" s="135" t="n">
         <v>540</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-1031.428571428572</v>
+        <v>-1174.285714285714</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.6563636363636364</v>
+        <v>-0.6849999999999999</v>
       </c>
       <c r="Y6" s="135" t="n">
         <v>9</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3139,28 +3139,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>65.47619047619048</v>
+        <v>71.42857142857143</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>-20.47619047619048</v>
+        <v>-26.42857142857143</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>523.8095238095239</v>
+        <v>571.4285714285714</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>360</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>-163.8095238095239</v>
+        <v>-211.4285714285714</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>-0.3127272727272728</v>
+        <v>-0.37</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>8</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>35.37981269510926</v>
+        <v>37.46097814776275</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-13.37981269510926</v>
+        <v>-15.46097814776274</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>1096.774193548387</v>
+        <v>1161.290322580645</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>1151.519237</v>
+        <v>1197.994656</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>54.7450434516129</v>
+        <v>36.70433341935495</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>0.0499145984411764</v>
+        <v>0.0316065093333334</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>52.3417835</v>
+        <v>54.45430254545455</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>21.3417835</v>
+        <v>23.45430254545455</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>59.28509154315606</v>
+        <v>62.77244986922407</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-39.28509154315606</v>
+        <v>-42.77244986922407</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>2193.548387096774</v>
+        <v>2322.58064516129</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>2194.825089</v>
+        <v>2317.398099</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>1.276701903225785</v>
+        <v>-5.182546161290247</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.000582025867647</v>
+        <v>-0.0022313740416666</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>109.74125445</v>
+        <v>115.86990495</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>72.74125445</v>
+        <v>78.86990495000001</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>4.727474972191325</v>
+        <v>5.005561735261402</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-2.727474972191325</v>
+        <v>-3.005561735261402</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>274.1935483870968</v>
+        <v>290.3225806451613</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>279.660959</v>
+        <v>297.330959</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>5.467410612903223</v>
+        <v>7.008378354838726</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.019939968117647</v>
+        <v>0.0241399698888889</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>139.8304795</v>
+        <v>148.6654795</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>81.8304795</v>
+        <v>90.6654795</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,34 +3563,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.713709677419355</v>
+        <v>1.814516129032258</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.7137096774193548</v>
+        <v>-0.814516129032258</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>274.1935483870968</v>
+        <v>290.3225806451613</v>
       </c>
       <c r="V11" s="135" t="n">
-        <v>97.33634600000001</v>
+        <v>123.536346</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-176.8572023870968</v>
+        <v>-166.7862346451613</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.6450086204705883</v>
+        <v>-0.5744859193333334</v>
       </c>
       <c r="Y11" s="135" t="n">
-        <v>97.33634600000001</v>
+        <v>123.536346</v>
       </c>
       <c r="Z11" s="135" t="n">
-        <v>-62.663654</v>
+        <v>-36.46365400000001</v>
       </c>
       <c r="AB11" s="137" t="inlineStr">
         <is>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>158.7436332767402</v>
+        <v>168.081494057725</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-66.74363327674024</v>
+        <v>-76.08149405772497</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>3016.129032258064</v>
+        <v>3193.548387096774</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>3009.96</v>
+        <v>3195.09</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>-6.169032258064362</v>
+        <v>1.541612903225996</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>-0.0020453475935828</v>
+        <v>0.0004827272727273</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>32.71695652173913</v>
+        <v>34.72923913043478</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>13.71695652173913</v>
+        <v>15.72923913043478</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>9.13978494623656</v>
+        <v>9.677419354838712</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>-2.13978494623656</v>
+        <v>-2.677419354838712</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>274.1935483870968</v>
+        <v>290.3225806451613</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>174.17</v>
+        <v>184.54</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-100.0235483870968</v>
+        <v>-105.7825806451613</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3647917647058823</v>
+        <v>-0.3643622222222222</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>24.88142857142857</v>
+        <v>26.36285714285714</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-5.118571428571432</v>
+        <v>-3.637142857142859</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>3.046594982078853</v>
+        <v>3.225806451612903</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-3.046594982078853</v>
+        <v>-3.225806451612903</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>274.1935483870968</v>
+        <v>290.3225806451613</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>171.67</v>
+        <v>181.11</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-102.5235483870968</v>
+        <v>-109.2125806451613</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3739094117647059</v>
+        <v>-0.3761766666666666</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>68.54838709677419</v>
+        <v>72.58064516129032</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-49.54838709677419</v>
+        <v>-53.58064516129032</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>822.5806451612904</v>
+        <v>870.9677419354839</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>858.955881</v>
+        <v>887.5860730000001</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>36.37523583870961</v>
+        <v>16.61833106451616</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>0.0442208749411763</v>
+        <v>0.019080306037037</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>45.2082042631579</v>
+        <v>46.71505647368421</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>33.2082042631579</v>
+        <v>34.71505647368421</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>23.84291725105189</v>
+        <v>25.24544179523141</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-20.84291725105189</v>
+        <v>-22.24544179523141</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>548.3870967741935</v>
+        <v>580.6451612903226</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>496.81</v>
+        <v>529.86</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-51.57709677419354</v>
+        <v>-50.78516129032255</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.09405235294117641</v>
+        <v>-0.0874633333333332</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>165.6033333333333</v>
+        <v>176.62</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>142.6033333333333</v>
+        <v>153.62</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>235.933983495874</v>
+        <v>249.8124531132783</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-119.933983495874</v>
+        <v>-133.8124531132783</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>10145.16129032258</v>
+        <v>10741.93548387097</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>9871.194763</v>
+        <v>10475.552448</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-273.9665273225801</v>
+        <v>-266.3830358709674</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0270046497519872</v>
+        <v>-0.0247984207567567</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>85.0965065775862</v>
+        <v>90.30648662068964</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>42.0965065775862</v>
+        <v>47.30648662068965</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>364.4274064407577</v>
+        <v>385.8643127019788</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-198.4274064407577</v>
+        <v>-219.8643127019788</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>8774.193548387097</v>
+        <v>9290.322580645159</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>8434.907512</v>
+        <v>8914.446132999999</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>-339.2860363870968</v>
+        <v>-375.8764476451615</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>-0.0386686291470588</v>
+        <v>-0.0404589231840278</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>50.81269585542169</v>
+        <v>53.70148272891566</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>26.73603917890619</v>
+        <v>29.62482605240016</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4350,28 +4350,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>550.2297410192148</v>
+        <v>600.250626566416</v>
       </c>
       <c r="R19" t="n">
         <v>198</v>
       </c>
       <c r="S19" t="n">
-        <v>-352.2297410192148</v>
+        <v>-402.2506265664161</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>4452.380952380952</v>
+        <v>4857.142857142857</v>
       </c>
       <c r="V19" s="135" t="n">
         <v>1606.8</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-2845.580952380952</v>
+        <v>-3250.342857142857</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.6391144385026738</v>
+        <v>-0.6691882352941176</v>
       </c>
       <c r="Y19" s="135" t="n">
         <v>8.115151515151515</v>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>1150.591130955846</v>
+        <v>1235.927392381673</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-670.5911309558464</v>
+        <v>-755.9273923816731</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>23371.73579109063</v>
+        <v>24889.40092165899</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>19912.902275</v>
+        <v>20996.798581</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-3458.833516090628</v>
+        <v>-3892.602340658989</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1479921537282286</v>
+        <v>-0.1563959836924644</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>41.48521307291666</v>
+        <v>43.74333037708333</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>21.44060448387908</v>
+        <v>23.69872178804575</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46252.29188657407</v>
+        <v>46253.291875</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-20
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 18/08/2026  |  Ultimo aggiornamento: 19/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 19/08/2026  |  Ultimo aggiornamento: 20/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>4645.16129032258</v>
+        <v>4903.225806451613</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>4708.950705</v>
+        <v>4963.575197</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>63.7894146774197</v>
+        <v>60.34939054838742</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0137324434375</v>
+        <v>0.0123080993881579</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>580.6451612903226</v>
+        <v>612.9032258064516</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>580.421743</v>
+        <v>607.7787070000001</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>-0.2234182903225701</v>
+        <v>-5.124518806451533</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>-0.0003847759444444</v>
+        <v>-0.0083610569999998</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>5516.129032258064</v>
+        <v>5822.58064516129</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>5186.18</v>
+        <v>5438.54</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-329.9490322580641</v>
+        <v>-384.0406451612898</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0598153216374268</v>
+        <v>-0.0659571191135733</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>249.8124531132783</v>
+        <v>263.6909227306826</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-133.8124531132783</v>
+        <v>-147.6909227306826</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>10741.93548387097</v>
+        <v>11338.70967741935</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>10475.552448</v>
+        <v>11009.893904</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-266.3830358709674</v>
+        <v>-328.8157734193537</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0247984207567567</v>
+        <v>-0.028999399647226</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>90.30648662068964</v>
+        <v>94.91287848275864</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>47.30648662068965</v>
+        <v>51.91287848275863</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>37.46097814776275</v>
+        <v>39.54214360041623</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-15.46097814776274</v>
+        <v>-17.54214360041623</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>1161.290322580645</v>
+        <v>1225.806451612903</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>1197.994656</v>
+        <v>1242.347785</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>36.70433341935495</v>
+        <v>16.54133338709676</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.0316065093333334</v>
+        <v>0.0134942456578947</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>54.45430254545455</v>
+        <v>56.47035386363636</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>23.45430254545455</v>
+        <v>25.47035386363636</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>62.77244986922407</v>
+        <v>66.25980819529207</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-42.77244986922407</v>
+        <v>-46.25980819529207</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>2322.58064516129</v>
+        <v>2451.612903225806</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>2317.398099</v>
+        <v>2449.310856</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>-5.182546161290247</v>
+        <v>-2.302047225806291</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>-0.0022313740416666</v>
+        <v>-0.0009389929473682999</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>115.86990495</v>
+        <v>122.4655428</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>78.86990495000001</v>
+        <v>85.46554280000001</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>5.005561735261402</v>
+        <v>5.28364849833148</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-3.005561735261402</v>
+        <v>-3.28364849833148</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>290.3225806451613</v>
+        <v>306.4516129032258</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>297.330959</v>
+        <v>314.050885</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>7.008378354838726</v>
+        <v>7.5992720967742</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0241399698888889</v>
+        <v>0.0247976247368421</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>148.6654795</v>
+        <v>157.0254425</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>90.6654795</v>
+        <v>99.0254425</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,34 +1540,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>1.814516129032258</v>
+        <v>1.915322580645161</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-0.814516129032258</v>
+        <v>-0.9153225806451613</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>290.3225806451613</v>
+        <v>306.4516129032258</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>123.536346</v>
+        <v>128.836346</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-166.7862346451613</v>
+        <v>-177.6152669032258</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.5744859193333334</v>
+        <v>-0.5795866604210527</v>
       </c>
       <c r="U12" s="117" t="n">
-        <v>123.536346</v>
+        <v>128.836346</v>
       </c>
       <c r="V12" s="117" t="n">
-        <v>-36.46365400000001</v>
+        <v>-31.16365400000001</v>
       </c>
       <c r="W12" s="120" t="inlineStr"/>
     </row>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>168.081494057725</v>
+        <v>177.4193548387097</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-76.08149405772497</v>
+        <v>-85.41935483870967</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>3193.548387096774</v>
+        <v>3370.967741935483</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>3195.09</v>
+        <v>3373.31</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>1.541612903225996</v>
+        <v>2.3422580645165</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.0004827272727273</v>
+        <v>0.0006948325358852</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>34.72923913043478</v>
+        <v>36.66641304347826</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>15.72923913043478</v>
+        <v>17.66641304347826</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>9.677419354838712</v>
+        <v>10.21505376344086</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-2.677419354838712</v>
+        <v>-3.215053763440862</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>290.3225806451613</v>
+        <v>306.4516129032258</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>184.54</v>
+        <v>193.58</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-105.7825806451613</v>
+        <v>-112.8716129032258</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3643622222222222</v>
+        <v>-0.368317894736842</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>26.36285714285714</v>
+        <v>27.65428571428572</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-3.637142857142859</v>
+        <v>-2.345714285714283</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>3.225806451612903</v>
+        <v>3.405017921146953</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-3.225806451612903</v>
+        <v>-3.405017921146953</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>290.3225806451613</v>
+        <v>306.4516129032258</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>181.11</v>
+        <v>189.94</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-109.2125806451613</v>
+        <v>-116.5116129032258</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3761766666666666</v>
+        <v>-0.3801957894736842</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>72.58064516129032</v>
+        <v>76.61290322580645</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-53.58064516129032</v>
+        <v>-57.61290322580645</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>870.9677419354839</v>
+        <v>919.3548387096774</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>887.5860730000001</v>
+        <v>920.708138</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>16.61833106451616</v>
+        <v>1.353299290322525</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.019080306037037</v>
+        <v>0.0014720097543859</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>46.71505647368421</v>
+        <v>48.45832305263158</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>34.71505647368421</v>
+        <v>36.45832305263158</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>25.24544179523141</v>
+        <v>26.64796633941094</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-22.24544179523141</v>
+        <v>-23.64796633941094</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>580.6451612903226</v>
+        <v>612.9032258064516</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>529.86</v>
+        <v>559.75</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-50.78516129032255</v>
+        <v>-53.15322580645159</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.0874633333333332</v>
+        <v>-0.0867236842105262</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>176.62</v>
+        <v>186.5833333333333</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>153.62</v>
+        <v>163.5833333333333</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>385.8643127019788</v>
+        <v>407.3012189631998</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-219.8643127019788</v>
+        <v>-241.3012189631998</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>9290.322580645159</v>
+        <v>9806.451612903224</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>8914.446132999999</v>
+        <v>9371.83401</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>-375.8764476451615</v>
+        <v>-434.6176029032249</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>-0.0404589231840278</v>
+        <v>-0.0443195581907893</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>53.70148272891566</v>
+        <v>56.45683138554217</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>29.62482605240016</v>
+        <v>32.38017470902668</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2063,28 +2063,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>338.3458646616542</v>
+        <v>366.5413533834587</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>93</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-245.3458646616542</v>
+        <v>-273.5413533834587</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>2571.428571428572</v>
+        <v>2785.714285714286</v>
       </c>
       <c r="R19" s="117" t="n">
         <v>706.8</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-1864.628571428572</v>
+        <v>-2078.914285714286</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.7251333333333334</v>
+        <v>-0.7462769230769232</v>
       </c>
       <c r="U19" s="117" t="n">
         <v>7.6</v>
@@ -2138,28 +2138,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>190.4761904761905</v>
+        <v>206.3492063492064</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>60</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-130.4761904761905</v>
+        <v>-146.3492063492063</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>1714.285714285714</v>
+        <v>1857.142857142857</v>
       </c>
       <c r="R20" s="117" t="n">
         <v>540</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-1174.285714285714</v>
+        <v>-1317.142857142857</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.6849999999999999</v>
+        <v>-0.7092307692307692</v>
       </c>
       <c r="U20" s="117" t="n">
         <v>9</v>
@@ -2213,28 +2213,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>71.42857142857143</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-26.42857142857143</v>
+        <v>-32.38095238095238</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>571.4285714285714</v>
+        <v>619.047619047619</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>360</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-211.4285714285714</v>
+        <v>-259.047619047619</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.37</v>
+        <v>-0.4184615384615384</v>
       </c>
       <c r="U21" s="117" t="n">
         <v>8</v>
@@ -2276,28 +2276,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>600.250626566416</v>
+        <v>650.2715121136174</v>
       </c>
       <c r="N22" s="125" t="n">
         <v>198</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-402.2506265664161</v>
+        <v>-452.2715121136174</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="Q22" s="123" t="n">
-        <v>4857.142857142857</v>
+        <v>5261.904761904761</v>
       </c>
       <c r="R22" s="123" t="n">
         <v>1606.8</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-3250.342857142857</v>
+        <v>-3655.104761904761</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-0.6691882352941176</v>
+        <v>-0.694635294117647</v>
       </c>
       <c r="U22" s="123" t="n">
         <v>8.115151515151515</v>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>1235.927392381673</v>
+        <v>1321.2636538075</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-755.9273923816731</v>
+        <v>-841.2636538074998</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>24889.40092165899</v>
+        <v>26407.06605222734</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>20996.798581</v>
+        <v>21988.527914</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-3892.602340658989</v>
+        <v>-4418.538138227344</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1563959836924644</v>
+        <v>-0.1673240839966262</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>43.74333037708333</v>
+        <v>45.80943315416666</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>23.69872178804575</v>
+        <v>25.76482456512908</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>4645.16129032258</v>
+        <v>4903.225806451613</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>4708.950705</v>
+        <v>4963.575197</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>63.7894146774197</v>
+        <v>60.34939054838742</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0137324434375</v>
+        <v>0.0123080993881579</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>580.6451612903226</v>
+        <v>612.9032258064516</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>580.421743</v>
+        <v>607.7787070000001</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>-0.2234182903225701</v>
+        <v>-5.124518806451533</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>-0.0003847759444444</v>
+        <v>-0.0083610569999998</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>5516.129032258064</v>
+        <v>5822.58064516129</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>5186.18</v>
+        <v>5438.54</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-329.9490322580641</v>
+        <v>-384.0406451612898</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0598153216374268</v>
+        <v>-0.0659571191135733</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2933,28 +2933,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>338.3458646616542</v>
+        <v>366.5413533834587</v>
       </c>
       <c r="R5" t="n">
         <v>93</v>
       </c>
       <c r="S5" t="n">
-        <v>-245.3458646616542</v>
+        <v>-273.5413533834587</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="U5" s="135" t="n">
-        <v>2571.428571428572</v>
+        <v>2785.714285714286</v>
       </c>
       <c r="V5" s="135" t="n">
         <v>706.8</v>
       </c>
       <c r="W5" s="135" t="n">
-        <v>-1864.628571428572</v>
+        <v>-2078.914285714286</v>
       </c>
       <c r="X5" s="136" t="n">
-        <v>-0.7251333333333334</v>
+        <v>-0.7462769230769232</v>
       </c>
       <c r="Y5" s="135" t="n">
         <v>7.6</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3036,28 +3036,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>190.4761904761905</v>
+        <v>206.3492063492064</v>
       </c>
       <c r="R6" t="n">
         <v>60</v>
       </c>
       <c r="S6" t="n">
-        <v>-130.4761904761905</v>
+        <v>-146.3492063492063</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>1714.285714285714</v>
+        <v>1857.142857142857</v>
       </c>
       <c r="V6" s="135" t="n">
         <v>540</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-1174.285714285714</v>
+        <v>-1317.142857142857</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.6849999999999999</v>
+        <v>-0.7092307692307692</v>
       </c>
       <c r="Y6" s="135" t="n">
         <v>9</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3139,28 +3139,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>71.42857142857143</v>
+        <v>77.38095238095238</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>-26.42857142857143</v>
+        <v>-32.38095238095238</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>571.4285714285714</v>
+        <v>619.047619047619</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>360</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>-211.4285714285714</v>
+        <v>-259.047619047619</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>-0.37</v>
+        <v>-0.4184615384615384</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>8</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>37.46097814776275</v>
+        <v>39.54214360041623</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-15.46097814776274</v>
+        <v>-17.54214360041623</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>1161.290322580645</v>
+        <v>1225.806451612903</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>1197.994656</v>
+        <v>1242.347785</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>36.70433341935495</v>
+        <v>16.54133338709676</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>0.0316065093333334</v>
+        <v>0.0134942456578947</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>54.45430254545455</v>
+        <v>56.47035386363636</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>23.45430254545455</v>
+        <v>25.47035386363636</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>62.77244986922407</v>
+        <v>66.25980819529207</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-42.77244986922407</v>
+        <v>-46.25980819529207</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>2322.58064516129</v>
+        <v>2451.612903225806</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>2317.398099</v>
+        <v>2449.310856</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>-5.182546161290247</v>
+        <v>-2.302047225806291</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>-0.0022313740416666</v>
+        <v>-0.0009389929473682999</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>115.86990495</v>
+        <v>122.4655428</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>78.86990495000001</v>
+        <v>85.46554280000001</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>5.005561735261402</v>
+        <v>5.28364849833148</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-3.005561735261402</v>
+        <v>-3.28364849833148</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>290.3225806451613</v>
+        <v>306.4516129032258</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>297.330959</v>
+        <v>314.050885</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>7.008378354838726</v>
+        <v>7.5992720967742</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0241399698888889</v>
+        <v>0.0247976247368421</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>148.6654795</v>
+        <v>157.0254425</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>90.6654795</v>
+        <v>99.0254425</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,34 +3563,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.814516129032258</v>
+        <v>1.915322580645161</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.814516129032258</v>
+        <v>-0.9153225806451613</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>290.3225806451613</v>
+        <v>306.4516129032258</v>
       </c>
       <c r="V11" s="135" t="n">
-        <v>123.536346</v>
+        <v>128.836346</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-166.7862346451613</v>
+        <v>-177.6152669032258</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.5744859193333334</v>
+        <v>-0.5795866604210527</v>
       </c>
       <c r="Y11" s="135" t="n">
-        <v>123.536346</v>
+        <v>128.836346</v>
       </c>
       <c r="Z11" s="135" t="n">
-        <v>-36.46365400000001</v>
+        <v>-31.16365400000001</v>
       </c>
       <c r="AB11" s="137" t="inlineStr">
         <is>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>168.081494057725</v>
+        <v>177.4193548387097</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-76.08149405772497</v>
+        <v>-85.41935483870967</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>3193.548387096774</v>
+        <v>3370.967741935483</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>3195.09</v>
+        <v>3373.31</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>1.541612903225996</v>
+        <v>2.3422580645165</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.0004827272727273</v>
+        <v>0.0006948325358852</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>34.72923913043478</v>
+        <v>36.66641304347826</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>15.72923913043478</v>
+        <v>17.66641304347826</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>9.677419354838712</v>
+        <v>10.21505376344086</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>-2.677419354838712</v>
+        <v>-3.215053763440862</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>290.3225806451613</v>
+        <v>306.4516129032258</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>184.54</v>
+        <v>193.58</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-105.7825806451613</v>
+        <v>-112.8716129032258</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3643622222222222</v>
+        <v>-0.368317894736842</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>26.36285714285714</v>
+        <v>27.65428571428572</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-3.637142857142859</v>
+        <v>-2.345714285714283</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>3.225806451612903</v>
+        <v>3.405017921146953</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-3.225806451612903</v>
+        <v>-3.405017921146953</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>290.3225806451613</v>
+        <v>306.4516129032258</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>181.11</v>
+        <v>189.94</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-109.2125806451613</v>
+        <v>-116.5116129032258</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3761766666666666</v>
+        <v>-0.3801957894736842</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>72.58064516129032</v>
+        <v>76.61290322580645</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-53.58064516129032</v>
+        <v>-57.61290322580645</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>870.9677419354839</v>
+        <v>919.3548387096774</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>887.5860730000001</v>
+        <v>920.708138</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>16.61833106451616</v>
+        <v>1.353299290322525</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>0.019080306037037</v>
+        <v>0.0014720097543859</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>46.71505647368421</v>
+        <v>48.45832305263158</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>34.71505647368421</v>
+        <v>36.45832305263158</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>25.24544179523141</v>
+        <v>26.64796633941094</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-22.24544179523141</v>
+        <v>-23.64796633941094</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>580.6451612903226</v>
+        <v>612.9032258064516</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>529.86</v>
+        <v>559.75</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-50.78516129032255</v>
+        <v>-53.15322580645159</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.0874633333333332</v>
+        <v>-0.0867236842105262</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>176.62</v>
+        <v>186.5833333333333</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>153.62</v>
+        <v>163.5833333333333</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>249.8124531132783</v>
+        <v>263.6909227306826</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-133.8124531132783</v>
+        <v>-147.6909227306826</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>10741.93548387097</v>
+        <v>11338.70967741935</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>10475.552448</v>
+        <v>11009.893904</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-266.3830358709674</v>
+        <v>-328.8157734193537</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0247984207567567</v>
+        <v>-0.028999399647226</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>90.30648662068964</v>
+        <v>94.91287848275864</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>47.30648662068965</v>
+        <v>51.91287848275863</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>385.8643127019788</v>
+        <v>407.3012189631998</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-219.8643127019788</v>
+        <v>-241.3012189631998</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>9290.322580645159</v>
+        <v>9806.451612903224</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>8914.446132999999</v>
+        <v>9371.83401</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>-375.8764476451615</v>
+        <v>-434.6176029032249</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>-0.0404589231840278</v>
+        <v>-0.0443195581907893</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>53.70148272891566</v>
+        <v>56.45683138554217</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>29.62482605240016</v>
+        <v>32.38017470902668</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4350,28 +4350,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>600.250626566416</v>
+        <v>650.2715121136174</v>
       </c>
       <c r="R19" t="n">
         <v>198</v>
       </c>
       <c r="S19" t="n">
-        <v>-402.2506265664161</v>
+        <v>-452.2715121136174</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>4857.142857142857</v>
+        <v>5261.904761904761</v>
       </c>
       <c r="V19" s="135" t="n">
         <v>1606.8</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-3250.342857142857</v>
+        <v>-3655.104761904761</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.6691882352941176</v>
+        <v>-0.694635294117647</v>
       </c>
       <c r="Y19" s="135" t="n">
         <v>8.115151515151515</v>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>1235.927392381673</v>
+        <v>1321.2636538075</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-755.9273923816731</v>
+        <v>-841.2636538074998</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>24889.40092165899</v>
+        <v>26407.06605222734</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>20996.798581</v>
+        <v>21988.527914</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-3892.602340658989</v>
+        <v>-4418.538138227344</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1563959836924644</v>
+        <v>-0.1673240839966262</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>43.74333037708333</v>
+        <v>45.80943315416666</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>23.69872178804575</v>
+        <v>25.76482456512908</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46252</v>
+        <v>46253</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46253.291875</v>
+        <v>46254.2919212963</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-21
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 19/08/2026  |  Ultimo aggiornamento: 20/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 20/08/2026  |  Ultimo aggiornamento: 21/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>4903.225806451613</v>
+        <v>5161.290322580645</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>4963.575197</v>
+        <v>5225.023895</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>60.34939054838742</v>
+        <v>63.73357241935537</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0123080993881579</v>
+        <v>0.0123483796562501</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>612.9032258064516</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>607.7787070000001</v>
+        <v>632.346542</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>-5.124518806451533</v>
+        <v>-12.81474832258061</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>-0.0083610569999998</v>
+        <v>-0.0198628598999999</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>5822.58064516129</v>
+        <v>6129.032258064516</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>5438.54</v>
+        <v>5644.82</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-384.0406451612898</v>
+        <v>-484.2122580645164</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0659571191135733</v>
+        <v>-0.0790030526315789</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>263.6909227306826</v>
+        <v>277.569392348087</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-147.6909227306826</v>
+        <v>-161.569392348087</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>11338.70967741935</v>
+        <v>11935.48387096774</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>11009.893904</v>
+        <v>11502.190437</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-328.8157734193537</v>
+        <v>-433.2934339677431</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.028999399647226</v>
+        <v>-0.0363029633864865</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>94.91287848275864</v>
+        <v>99.15681411206896</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>51.91287848275863</v>
+        <v>56.15681411206896</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>39.54214360041623</v>
+        <v>41.62330905306972</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-17.54214360041623</v>
+        <v>-19.62330905306972</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>1225.806451612903</v>
+        <v>1290.322580645161</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>1242.347785</v>
+        <v>1287.967718</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>16.54133338709676</v>
+        <v>-2.35486264516112</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>0.0134942456578947</v>
+        <v>-0.0018250185499998</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>56.47035386363636</v>
+        <v>58.54398718181819</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>25.47035386363636</v>
+        <v>27.54398718181819</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>66.25980819529207</v>
+        <v>69.74716652136007</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-46.25980819529207</v>
+        <v>-49.74716652136007</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>2451.612903225806</v>
+        <v>2580.645161290322</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>2449.310856</v>
+        <v>2565.755958</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>-2.302047225806291</v>
+        <v>-14.88920329032226</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>-0.0009389929473682999</v>
+        <v>-0.0057695662749998</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>122.4655428</v>
+        <v>128.2877979</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>85.46554280000001</v>
+        <v>91.28779790000002</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>5.28364849833148</v>
+        <v>5.561735261401558</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-3.28364849833148</v>
+        <v>-3.561735261401558</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>306.4516129032258</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>314.050885</v>
+        <v>330.470885</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>7.5992720967742</v>
+        <v>7.890239838709704</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0247976247368421</v>
+        <v>0.0244597435</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>157.0254425</v>
+        <v>165.2354425</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>99.0254425</v>
+        <v>107.2354425</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,34 +1540,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>1.915322580645161</v>
+        <v>2.016129032258065</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-0.9153225806451613</v>
+        <v>-1.016129032258065</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>306.4516129032258</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>128.836346</v>
+        <v>157.606346</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-177.6152669032258</v>
+        <v>-164.9742991612903</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.5795866604210527</v>
+        <v>-0.5114203274</v>
       </c>
       <c r="U12" s="117" t="n">
-        <v>128.836346</v>
+        <v>157.606346</v>
       </c>
       <c r="V12" s="117" t="n">
-        <v>-31.16365400000001</v>
+        <v>-2.393653999999998</v>
       </c>
       <c r="W12" s="120" t="inlineStr"/>
     </row>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>177.4193548387097</v>
+        <v>186.7572156196944</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-85.41935483870967</v>
+        <v>-94.75721561969441</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>3370.967741935483</v>
+        <v>3548.387096774193</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>3373.31</v>
+        <v>3542.01</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>2.3422580645165</v>
+        <v>-6.377096774192978</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>0.0006948325358852</v>
+        <v>-0.0017971818181816</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>36.66641304347826</v>
+        <v>38.50010869565217</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>17.66641304347826</v>
+        <v>19.50010869565217</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>10.21505376344086</v>
+        <v>10.75268817204301</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-3.215053763440862</v>
+        <v>-3.752688172043012</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>306.4516129032258</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>193.58</v>
+        <v>201.47</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-112.8716129032258</v>
+        <v>-121.1106451612903</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.368317894736842</v>
+        <v>-0.3754429999999999</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>27.65428571428572</v>
+        <v>28.78142857142857</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-2.345714285714283</v>
+        <v>-1.21857142857143</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>3.405017921146953</v>
+        <v>3.584229390681004</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-3.405017921146953</v>
+        <v>-3.584229390681004</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>306.4516129032258</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>189.94</v>
+        <v>198.67</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-116.5116129032258</v>
+        <v>-123.9106451612903</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3801957894736842</v>
+        <v>-0.384123</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>76.61290322580645</v>
+        <v>80.64516129032258</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-57.61290322580645</v>
+        <v>-61.64516129032258</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>919.3548387096774</v>
+        <v>967.741935483871</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>920.708138</v>
+        <v>956.753649</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>1.353299290322525</v>
+        <v>-10.98828648387098</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>0.0014720097543859</v>
+        <v>-0.0113545627</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>48.45832305263158</v>
+        <v>50.35545521052632</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>36.45832305263158</v>
+        <v>38.35545521052632</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>26.64796633941094</v>
+        <v>28.05049088359046</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-23.64796633941094</v>
+        <v>-25.05049088359046</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>612.9032258064516</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>559.75</v>
+        <v>589.52</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-53.15322580645159</v>
+        <v>-55.64129032258063</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.0867236842105262</v>
+        <v>-0.0862439999999999</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>186.5833333333333</v>
+        <v>196.5066666666666</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>163.5833333333333</v>
+        <v>173.5066666666667</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>407.3012189631998</v>
+        <v>428.7381252244209</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-241.3012189631998</v>
+        <v>-262.7381252244209</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>9806.451612903224</v>
+        <v>10322.58064516129</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>9371.83401</v>
+        <v>9830.224555999999</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>-434.6176029032249</v>
+        <v>-492.3560891612888</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>-0.0443195581907893</v>
+        <v>-0.0476969961374998</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>56.45683138554217</v>
+        <v>59.21822021686748</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>32.38017470902668</v>
+        <v>35.14156354035198</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2063,28 +2063,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>366.5413533834587</v>
+        <v>394.7368421052632</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>93</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-273.5413533834587</v>
+        <v>-301.7368421052632</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>2785.714285714286</v>
+        <v>3000</v>
       </c>
       <c r="R19" s="117" t="n">
         <v>706.8</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-2078.914285714286</v>
+        <v>-2293.2</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.7462769230769232</v>
+        <v>-0.7644</v>
       </c>
       <c r="U19" s="117" t="n">
         <v>7.6</v>
@@ -2138,28 +2138,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>206.3492063492064</v>
+        <v>222.2222222222222</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>60</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-146.3492063492063</v>
+        <v>-162.2222222222222</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>1857.142857142857</v>
+        <v>2000</v>
       </c>
       <c r="R20" s="117" t="n">
         <v>540</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-1317.142857142857</v>
+        <v>-1460</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.7092307692307692</v>
+        <v>-0.73</v>
       </c>
       <c r="U20" s="117" t="n">
         <v>9</v>
@@ -2213,28 +2213,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>77.38095238095238</v>
+        <v>83.33333333333334</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-32.38095238095238</v>
+        <v>-38.33333333333334</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>619.047619047619</v>
+        <v>666.6666666666667</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>360</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-259.047619047619</v>
+        <v>-306.6666666666667</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.4184615384615384</v>
+        <v>-0.4600000000000001</v>
       </c>
       <c r="U21" s="117" t="n">
         <v>8</v>
@@ -2276,28 +2276,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>650.2715121136174</v>
+        <v>700.2923976608188</v>
       </c>
       <c r="N22" s="125" t="n">
         <v>198</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-452.2715121136174</v>
+        <v>-502.2923976608188</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="Q22" s="123" t="n">
-        <v>5261.904761904761</v>
+        <v>5666.666666666667</v>
       </c>
       <c r="R22" s="123" t="n">
         <v>1606.8</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-3655.104761904761</v>
+        <v>-4059.866666666667</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-0.694635294117647</v>
+        <v>-0.7164470588235294</v>
       </c>
       <c r="U22" s="123" t="n">
         <v>8.115151515151515</v>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>1321.2636538075</v>
+        <v>1406.599915233327</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-841.2636538074998</v>
+        <v>-926.5999152333266</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>26407.06605222734</v>
+        <v>27924.7311827957</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>21988.527914</v>
+        <v>22939.214993</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-4418.538138227344</v>
+        <v>-4985.516189795697</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1673240839966262</v>
+        <v>-0.1785340799580284</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>45.80943315416666</v>
+        <v>47.79003123541667</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>25.76482456512908</v>
+        <v>27.74542264637909</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>4903.225806451613</v>
+        <v>5161.290322580645</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>4963.575197</v>
+        <v>5225.023895</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>60.34939054838742</v>
+        <v>63.73357241935537</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0123080993881579</v>
+        <v>0.0123483796562501</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>612.9032258064516</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>607.7787070000001</v>
+        <v>632.346542</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>-5.124518806451533</v>
+        <v>-12.81474832258061</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>-0.0083610569999998</v>
+        <v>-0.0198628598999999</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>5822.58064516129</v>
+        <v>6129.032258064516</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>5438.54</v>
+        <v>5644.82</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-384.0406451612898</v>
+        <v>-484.2122580645164</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0659571191135733</v>
+        <v>-0.0790030526315789</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2933,28 +2933,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>366.5413533834587</v>
+        <v>394.7368421052632</v>
       </c>
       <c r="R5" t="n">
         <v>93</v>
       </c>
       <c r="S5" t="n">
-        <v>-273.5413533834587</v>
+        <v>-301.7368421052632</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="U5" s="135" t="n">
-        <v>2785.714285714286</v>
+        <v>3000</v>
       </c>
       <c r="V5" s="135" t="n">
         <v>706.8</v>
       </c>
       <c r="W5" s="135" t="n">
-        <v>-2078.914285714286</v>
+        <v>-2293.2</v>
       </c>
       <c r="X5" s="136" t="n">
-        <v>-0.7462769230769232</v>
+        <v>-0.7644</v>
       </c>
       <c r="Y5" s="135" t="n">
         <v>7.6</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3036,28 +3036,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>206.3492063492064</v>
+        <v>222.2222222222222</v>
       </c>
       <c r="R6" t="n">
         <v>60</v>
       </c>
       <c r="S6" t="n">
-        <v>-146.3492063492063</v>
+        <v>-162.2222222222222</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>1857.142857142857</v>
+        <v>2000</v>
       </c>
       <c r="V6" s="135" t="n">
         <v>540</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-1317.142857142857</v>
+        <v>-1460</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.7092307692307692</v>
+        <v>-0.73</v>
       </c>
       <c r="Y6" s="135" t="n">
         <v>9</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3139,28 +3139,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>77.38095238095238</v>
+        <v>83.33333333333334</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>-32.38095238095238</v>
+        <v>-38.33333333333334</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>619.047619047619</v>
+        <v>666.6666666666667</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>360</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>-259.047619047619</v>
+        <v>-306.6666666666667</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>-0.4184615384615384</v>
+        <v>-0.4600000000000001</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>8</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>39.54214360041623</v>
+        <v>41.62330905306972</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-17.54214360041623</v>
+        <v>-19.62330905306972</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>1225.806451612903</v>
+        <v>1290.322580645161</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>1242.347785</v>
+        <v>1287.967718</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>16.54133338709676</v>
+        <v>-2.35486264516112</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>0.0134942456578947</v>
+        <v>-0.0018250185499998</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>56.47035386363636</v>
+        <v>58.54398718181819</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>25.47035386363636</v>
+        <v>27.54398718181819</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>66.25980819529207</v>
+        <v>69.74716652136007</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-46.25980819529207</v>
+        <v>-49.74716652136007</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>2451.612903225806</v>
+        <v>2580.645161290322</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>2449.310856</v>
+        <v>2565.755958</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>-2.302047225806291</v>
+        <v>-14.88920329032226</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>-0.0009389929473682999</v>
+        <v>-0.0057695662749998</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>122.4655428</v>
+        <v>128.2877979</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>85.46554280000001</v>
+        <v>91.28779790000002</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>5.28364849833148</v>
+        <v>5.561735261401558</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-3.28364849833148</v>
+        <v>-3.561735261401558</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>306.4516129032258</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>314.050885</v>
+        <v>330.470885</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>7.5992720967742</v>
+        <v>7.890239838709704</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0247976247368421</v>
+        <v>0.0244597435</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>157.0254425</v>
+        <v>165.2354425</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>99.0254425</v>
+        <v>107.2354425</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,34 +3563,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>1.915322580645161</v>
+        <v>2.016129032258065</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.9153225806451613</v>
+        <v>-1.016129032258065</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>306.4516129032258</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="V11" s="135" t="n">
-        <v>128.836346</v>
+        <v>157.606346</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-177.6152669032258</v>
+        <v>-164.9742991612903</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.5795866604210527</v>
+        <v>-0.5114203274</v>
       </c>
       <c r="Y11" s="135" t="n">
-        <v>128.836346</v>
+        <v>157.606346</v>
       </c>
       <c r="Z11" s="135" t="n">
-        <v>-31.16365400000001</v>
+        <v>-2.393653999999998</v>
       </c>
       <c r="AB11" s="137" t="inlineStr">
         <is>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>177.4193548387097</v>
+        <v>186.7572156196944</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-85.41935483870967</v>
+        <v>-94.75721561969441</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>3370.967741935483</v>
+        <v>3548.387096774193</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>3373.31</v>
+        <v>3542.01</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>2.3422580645165</v>
+        <v>-6.377096774192978</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>0.0006948325358852</v>
+        <v>-0.0017971818181816</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>36.66641304347826</v>
+        <v>38.50010869565217</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>17.66641304347826</v>
+        <v>19.50010869565217</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>10.21505376344086</v>
+        <v>10.75268817204301</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>-3.215053763440862</v>
+        <v>-3.752688172043012</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>306.4516129032258</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>193.58</v>
+        <v>201.47</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-112.8716129032258</v>
+        <v>-121.1106451612903</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.368317894736842</v>
+        <v>-0.3754429999999999</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>27.65428571428572</v>
+        <v>28.78142857142857</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-2.345714285714283</v>
+        <v>-1.21857142857143</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>3.405017921146953</v>
+        <v>3.584229390681004</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-3.405017921146953</v>
+        <v>-3.584229390681004</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>306.4516129032258</v>
+        <v>322.5806451612903</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>189.94</v>
+        <v>198.67</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-116.5116129032258</v>
+        <v>-123.9106451612903</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3801957894736842</v>
+        <v>-0.384123</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>76.61290322580645</v>
+        <v>80.64516129032258</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-57.61290322580645</v>
+        <v>-61.64516129032258</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>919.3548387096774</v>
+        <v>967.741935483871</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>920.708138</v>
+        <v>956.753649</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>1.353299290322525</v>
+        <v>-10.98828648387098</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>0.0014720097543859</v>
+        <v>-0.0113545627</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>48.45832305263158</v>
+        <v>50.35545521052632</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>36.45832305263158</v>
+        <v>38.35545521052632</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>26.64796633941094</v>
+        <v>28.05049088359046</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-23.64796633941094</v>
+        <v>-25.05049088359046</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>612.9032258064516</v>
+        <v>645.1612903225806</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>559.75</v>
+        <v>589.52</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-53.15322580645159</v>
+        <v>-55.64129032258063</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.0867236842105262</v>
+        <v>-0.0862439999999999</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>186.5833333333333</v>
+        <v>196.5066666666666</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>163.5833333333333</v>
+        <v>173.5066666666667</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>263.6909227306826</v>
+        <v>277.569392348087</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-147.6909227306826</v>
+        <v>-161.569392348087</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>11338.70967741935</v>
+        <v>11935.48387096774</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>11009.893904</v>
+        <v>11502.190437</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-328.8157734193537</v>
+        <v>-433.2934339677431</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.028999399647226</v>
+        <v>-0.0363029633864865</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>94.91287848275864</v>
+        <v>99.15681411206896</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>51.91287848275863</v>
+        <v>56.15681411206896</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>407.3012189631998</v>
+        <v>428.7381252244209</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-241.3012189631998</v>
+        <v>-262.7381252244209</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>9806.451612903224</v>
+        <v>10322.58064516129</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>9371.83401</v>
+        <v>9830.224555999999</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>-434.6176029032249</v>
+        <v>-492.3560891612888</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>-0.0443195581907893</v>
+        <v>-0.0476969961374998</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>56.45683138554217</v>
+        <v>59.21822021686748</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>32.38017470902668</v>
+        <v>35.14156354035198</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4350,28 +4350,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>650.2715121136174</v>
+        <v>700.2923976608188</v>
       </c>
       <c r="R19" t="n">
         <v>198</v>
       </c>
       <c r="S19" t="n">
-        <v>-452.2715121136174</v>
+        <v>-502.2923976608188</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>5261.904761904761</v>
+        <v>5666.666666666667</v>
       </c>
       <c r="V19" s="135" t="n">
         <v>1606.8</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-3655.104761904761</v>
+        <v>-4059.866666666667</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.694635294117647</v>
+        <v>-0.7164470588235294</v>
       </c>
       <c r="Y19" s="135" t="n">
         <v>8.115151515151515</v>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>1321.2636538075</v>
+        <v>1406.599915233327</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-841.2636538074998</v>
+        <v>-926.5999152333266</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>26407.06605222734</v>
+        <v>27924.7311827957</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>21988.527914</v>
+        <v>22939.214993</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-4418.538138227344</v>
+        <v>-4985.516189795697</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1673240839966262</v>
+        <v>-0.1785340799580284</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>45.80943315416666</v>
+        <v>47.79003123541667</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>25.76482456512908</v>
+        <v>27.74542264637909</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46254.2919212963</v>
+        <v>46255.29188657407</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-22
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 20/08/2026  |  Ultimo aggiornamento: 21/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 21/08/2026  |  Ultimo aggiornamento: 22/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>5161.290322580645</v>
+        <v>5419.354838709677</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>5225.023895</v>
+        <v>5491.980911</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>63.73357241935537</v>
+        <v>72.62607229032255</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0123483796562501</v>
+        <v>0.0134012395297619</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>645.1612903225806</v>
+        <v>677.4193548387096</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>632.346542</v>
+        <v>658.335365</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>-12.81474832258061</v>
+        <v>-19.08398983870961</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>-0.0198628598999999</v>
+        <v>-0.0281716040476189</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>6129.032258064516</v>
+        <v>6435.483870967741</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>5644.82</v>
+        <v>5864.3</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-484.2122580645164</v>
+        <v>-571.1838709677413</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0790030526315789</v>
+        <v>-0.0887553884711778</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>277.569392348087</v>
+        <v>291.4478619654914</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-161.569392348087</v>
+        <v>-175.4478619654914</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>11935.48387096774</v>
+        <v>12532.25806451613</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>11502.190437</v>
+        <v>12014.616276</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-433.2934339677431</v>
+        <v>-517.6417885161281</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0363029633864865</v>
+        <v>-0.0413047501776061</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>99.15681411206896</v>
+        <v>103.5742782413793</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>56.15681411206896</v>
+        <v>60.57427824137932</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>41.62330905306972</v>
+        <v>43.7044745057232</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-19.62330905306972</v>
+        <v>-21.7044745057232</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>1290.322580645161</v>
+        <v>1354.838709677419</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>1287.967718</v>
+        <v>1333.238648</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-2.35486264516112</v>
+        <v>-21.60006167741927</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.0018250185499998</v>
+        <v>-0.0159429026666666</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>58.54398718181819</v>
+        <v>60.60175672727273</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>27.54398718181819</v>
+        <v>29.60175672727273</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>69.74716652136007</v>
+        <v>73.23452484742808</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-49.74716652136007</v>
+        <v>-53.23452484742808</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>2580.645161290322</v>
+        <v>2709.677419354839</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>2565.755958</v>
+        <v>2689.186545</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>-14.88920329032226</v>
+        <v>-20.49087435483852</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>-0.0057695662749998</v>
+        <v>-0.007562108392857</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>128.2877979</v>
+        <v>134.45932725</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>91.28779790000002</v>
+        <v>97.45932725</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>5.561735261401558</v>
+        <v>5.839822024471636</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-3.561735261401558</v>
+        <v>-3.839822024471636</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>322.5806451612903</v>
+        <v>338.7096774193548</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>330.470885</v>
+        <v>344.699345</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>7.890239838709704</v>
+        <v>5.989667580645175</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0244597435</v>
+        <v>0.0176837804761905</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>165.2354425</v>
+        <v>172.3496725</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>107.2354425</v>
+        <v>114.3496725</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,28 +1540,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>2.016129032258065</v>
+        <v>2.116935483870968</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-1.016129032258065</v>
+        <v>-1.116935483870968</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>322.5806451612903</v>
+        <v>338.7096774193548</v>
       </c>
       <c r="R12" s="117" t="n">
         <v>157.606346</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-164.9742991612903</v>
+        <v>-181.1033314193548</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.5114203274</v>
+        <v>-0.5346860260952381</v>
       </c>
       <c r="U12" s="117" t="n">
         <v>157.606346</v>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>186.7572156196944</v>
+        <v>196.0950764006791</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-94.75721561969441</v>
+        <v>-104.0950764006791</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>3548.387096774193</v>
+        <v>3725.806451612903</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>3542.01</v>
+        <v>3694.98</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>-6.377096774192978</v>
+        <v>-30.82645161290293</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>-0.0017971818181816</v>
+        <v>-0.0082737662337661</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>38.50010869565217</v>
+        <v>40.16282608695652</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>19.50010869565217</v>
+        <v>21.16282608695652</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>10.75268817204301</v>
+        <v>11.29032258064516</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-3.752688172043012</v>
+        <v>-4.290322580645164</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>322.5806451612903</v>
+        <v>338.7096774193548</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>201.47</v>
+        <v>209.2</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-121.1106451612903</v>
+        <v>-129.5096774193548</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3754429999999999</v>
+        <v>-0.3823619047619047</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>28.78142857142857</v>
+        <v>29.88571428571428</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-1.21857142857143</v>
+        <v>-0.1142857142857174</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>3.584229390681004</v>
+        <v>3.763440860215054</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-3.584229390681004</v>
+        <v>-3.763440860215054</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>322.5806451612903</v>
+        <v>338.7096774193548</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>198.67</v>
+        <v>207.53</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-123.9106451612903</v>
+        <v>-131.1796774193548</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.384123</v>
+        <v>-0.3872923809523809</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>80.64516129032258</v>
+        <v>84.6774193548387</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-61.64516129032258</v>
+        <v>-65.6774193548387</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>967.741935483871</v>
+        <v>1016.129032258065</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>956.753649</v>
+        <v>988.236982</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>-10.98828648387098</v>
+        <v>-27.89205025806461</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>-0.0113545627</v>
+        <v>-0.0274493193015873</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>50.35545521052632</v>
+        <v>52.01247273684211</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>38.35545521052632</v>
+        <v>40.01247273684211</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>28.05049088359046</v>
+        <v>29.45301542776998</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-25.05049088359046</v>
+        <v>-26.45301542776998</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>645.1612903225806</v>
+        <v>677.4193548387096</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>589.52</v>
+        <v>615.77</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-55.64129032258063</v>
+        <v>-61.64935483870966</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.0862439999999999</v>
+        <v>-0.09100619047619039</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>196.5066666666666</v>
+        <v>205.2566666666666</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>173.5066666666667</v>
+        <v>182.2566666666666</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>428.7381252244209</v>
+        <v>450.1750314856419</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-262.7381252244209</v>
+        <v>-284.1750314856419</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>10322.58064516129</v>
+        <v>10838.70967741935</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>9830.224555999999</v>
+        <v>10240.447866</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>-492.3560891612888</v>
+        <v>-598.2618114193538</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>-0.0476969961374998</v>
+        <v>-0.055196774267857</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>59.21822021686748</v>
+        <v>61.68944497590362</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>35.14156354035198</v>
+        <v>37.61278829938811</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2063,28 +2063,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>394.7368421052632</v>
+        <v>422.9323308270677</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>93</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-301.7368421052632</v>
+        <v>-329.9323308270677</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>3000</v>
+        <v>3214.285714285714</v>
       </c>
       <c r="R19" s="117" t="n">
         <v>706.8</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-2293.2</v>
+        <v>-2507.485714285714</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.7644</v>
+        <v>-0.7801066666666667</v>
       </c>
       <c r="U19" s="117" t="n">
         <v>7.6</v>
@@ -2138,28 +2138,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>222.2222222222222</v>
+        <v>238.0952380952381</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>60</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-162.2222222222222</v>
+        <v>-178.0952380952381</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>2000</v>
+        <v>2142.857142857143</v>
       </c>
       <c r="R20" s="117" t="n">
         <v>540</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-1460</v>
+        <v>-1602.857142857143</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.73</v>
+        <v>-0.748</v>
       </c>
       <c r="U20" s="117" t="n">
         <v>9</v>
@@ -2213,28 +2213,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>83.33333333333334</v>
+        <v>89.28571428571429</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-38.33333333333334</v>
+        <v>-44.28571428571429</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>666.6666666666667</v>
+        <v>714.2857142857143</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>360</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-306.6666666666667</v>
+        <v>-354.2857142857143</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.4600000000000001</v>
+        <v>-0.496</v>
       </c>
       <c r="U21" s="117" t="n">
         <v>8</v>
@@ -2276,28 +2276,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>700.2923976608188</v>
+        <v>750.31328320802</v>
       </c>
       <c r="N22" s="125" t="n">
         <v>198</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-502.2923976608188</v>
+        <v>-552.3132832080202</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="Q22" s="123" t="n">
-        <v>5666.666666666667</v>
+        <v>6071.428571428572</v>
       </c>
       <c r="R22" s="123" t="n">
         <v>1606.8</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-4059.866666666667</v>
+        <v>-4464.628571428571</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-0.7164470588235294</v>
+        <v>-0.7353505882352941</v>
       </c>
       <c r="U22" s="123" t="n">
         <v>8.115151515151515</v>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>1406.599915233327</v>
+        <v>1491.936176659153</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-926.5999152333266</v>
+        <v>-1011.936176659153</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>27924.7311827957</v>
+        <v>29442.39631336405</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>22939.214993</v>
+        <v>23861.864142</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-4985.516189795697</v>
+        <v>-5580.532171364055</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1785340799580284</v>
+        <v>-0.1895406919996869</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>47.79003123541667</v>
+        <v>49.7122169625</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>27.74542264637909</v>
+        <v>29.66760837346241</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>5161.290322580645</v>
+        <v>5419.354838709677</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>5225.023895</v>
+        <v>5491.980911</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>63.73357241935537</v>
+        <v>72.62607229032255</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0123483796562501</v>
+        <v>0.0134012395297619</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>645.1612903225806</v>
+        <v>677.4193548387096</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>632.346542</v>
+        <v>658.335365</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>-12.81474832258061</v>
+        <v>-19.08398983870961</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>-0.0198628598999999</v>
+        <v>-0.0281716040476189</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>6129.032258064516</v>
+        <v>6435.483870967741</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>5644.82</v>
+        <v>5864.3</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-484.2122580645164</v>
+        <v>-571.1838709677413</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0790030526315789</v>
+        <v>-0.0887553884711778</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2933,28 +2933,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>394.7368421052632</v>
+        <v>422.9323308270677</v>
       </c>
       <c r="R5" t="n">
         <v>93</v>
       </c>
       <c r="S5" t="n">
-        <v>-301.7368421052632</v>
+        <v>-329.9323308270677</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="U5" s="135" t="n">
-        <v>3000</v>
+        <v>3214.285714285714</v>
       </c>
       <c r="V5" s="135" t="n">
         <v>706.8</v>
       </c>
       <c r="W5" s="135" t="n">
-        <v>-2293.2</v>
+        <v>-2507.485714285714</v>
       </c>
       <c r="X5" s="136" t="n">
-        <v>-0.7644</v>
+        <v>-0.7801066666666667</v>
       </c>
       <c r="Y5" s="135" t="n">
         <v>7.6</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3036,28 +3036,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>222.2222222222222</v>
+        <v>238.0952380952381</v>
       </c>
       <c r="R6" t="n">
         <v>60</v>
       </c>
       <c r="S6" t="n">
-        <v>-162.2222222222222</v>
+        <v>-178.0952380952381</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>2000</v>
+        <v>2142.857142857143</v>
       </c>
       <c r="V6" s="135" t="n">
         <v>540</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-1460</v>
+        <v>-1602.857142857143</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.73</v>
+        <v>-0.748</v>
       </c>
       <c r="Y6" s="135" t="n">
         <v>9</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3139,28 +3139,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>83.33333333333334</v>
+        <v>89.28571428571429</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>-38.33333333333334</v>
+        <v>-44.28571428571429</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>666.6666666666667</v>
+        <v>714.2857142857143</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>360</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>-306.6666666666667</v>
+        <v>-354.2857142857143</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>-0.4600000000000001</v>
+        <v>-0.496</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>8</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>41.62330905306972</v>
+        <v>43.7044745057232</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-19.62330905306972</v>
+        <v>-21.7044745057232</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>1290.322580645161</v>
+        <v>1354.838709677419</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>1287.967718</v>
+        <v>1333.238648</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>-2.35486264516112</v>
+        <v>-21.60006167741927</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>-0.0018250185499998</v>
+        <v>-0.0159429026666666</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>58.54398718181819</v>
+        <v>60.60175672727273</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>27.54398718181819</v>
+        <v>29.60175672727273</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>69.74716652136007</v>
+        <v>73.23452484742808</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-49.74716652136007</v>
+        <v>-53.23452484742808</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>2580.645161290322</v>
+        <v>2709.677419354839</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>2565.755958</v>
+        <v>2689.186545</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>-14.88920329032226</v>
+        <v>-20.49087435483852</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>-0.0057695662749998</v>
+        <v>-0.007562108392857</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>128.2877979</v>
+        <v>134.45932725</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>91.28779790000002</v>
+        <v>97.45932725</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>5.561735261401558</v>
+        <v>5.839822024471636</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-3.561735261401558</v>
+        <v>-3.839822024471636</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>322.5806451612903</v>
+        <v>338.7096774193548</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>330.470885</v>
+        <v>344.699345</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>7.890239838709704</v>
+        <v>5.989667580645175</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0244597435</v>
+        <v>0.0176837804761905</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>165.2354425</v>
+        <v>172.3496725</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>107.2354425</v>
+        <v>114.3496725</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,28 +3563,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>2.016129032258065</v>
+        <v>2.116935483870968</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-1.016129032258065</v>
+        <v>-1.116935483870968</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>322.5806451612903</v>
+        <v>338.7096774193548</v>
       </c>
       <c r="V11" s="135" t="n">
         <v>157.606346</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-164.9742991612903</v>
+        <v>-181.1033314193548</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.5114203274</v>
+        <v>-0.5346860260952381</v>
       </c>
       <c r="Y11" s="135" t="n">
         <v>157.606346</v>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>186.7572156196944</v>
+        <v>196.0950764006791</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-94.75721561969441</v>
+        <v>-104.0950764006791</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>3548.387096774193</v>
+        <v>3725.806451612903</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>3542.01</v>
+        <v>3694.98</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>-6.377096774192978</v>
+        <v>-30.82645161290293</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>-0.0017971818181816</v>
+        <v>-0.0082737662337661</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>38.50010869565217</v>
+        <v>40.16282608695652</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>19.50010869565217</v>
+        <v>21.16282608695652</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>10.75268817204301</v>
+        <v>11.29032258064516</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>-3.752688172043012</v>
+        <v>-4.290322580645164</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>322.5806451612903</v>
+        <v>338.7096774193548</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>201.47</v>
+        <v>209.2</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-121.1106451612903</v>
+        <v>-129.5096774193548</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3754429999999999</v>
+        <v>-0.3823619047619047</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>28.78142857142857</v>
+        <v>29.88571428571428</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-1.21857142857143</v>
+        <v>-0.1142857142857174</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>3.584229390681004</v>
+        <v>3.763440860215054</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-3.584229390681004</v>
+        <v>-3.763440860215054</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>322.5806451612903</v>
+        <v>338.7096774193548</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>198.67</v>
+        <v>207.53</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-123.9106451612903</v>
+        <v>-131.1796774193548</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.384123</v>
+        <v>-0.3872923809523809</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>80.64516129032258</v>
+        <v>84.6774193548387</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-61.64516129032258</v>
+        <v>-65.6774193548387</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>967.741935483871</v>
+        <v>1016.129032258065</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>956.753649</v>
+        <v>988.236982</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>-10.98828648387098</v>
+        <v>-27.89205025806461</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>-0.0113545627</v>
+        <v>-0.0274493193015873</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>50.35545521052632</v>
+        <v>52.01247273684211</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>38.35545521052632</v>
+        <v>40.01247273684211</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>28.05049088359046</v>
+        <v>29.45301542776998</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-25.05049088359046</v>
+        <v>-26.45301542776998</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>645.1612903225806</v>
+        <v>677.4193548387096</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>589.52</v>
+        <v>615.77</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-55.64129032258063</v>
+        <v>-61.64935483870966</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.0862439999999999</v>
+        <v>-0.09100619047619039</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>196.5066666666666</v>
+        <v>205.2566666666666</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>173.5066666666667</v>
+        <v>182.2566666666666</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>277.569392348087</v>
+        <v>291.4478619654914</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-161.569392348087</v>
+        <v>-175.4478619654914</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>11935.48387096774</v>
+        <v>12532.25806451613</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>11502.190437</v>
+        <v>12014.616276</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-433.2934339677431</v>
+        <v>-517.6417885161281</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0363029633864865</v>
+        <v>-0.0413047501776061</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>99.15681411206896</v>
+        <v>103.5742782413793</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>56.15681411206896</v>
+        <v>60.57427824137932</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>428.7381252244209</v>
+        <v>450.1750314856419</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-262.7381252244209</v>
+        <v>-284.1750314856419</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>10322.58064516129</v>
+        <v>10838.70967741935</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>9830.224555999999</v>
+        <v>10240.447866</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>-492.3560891612888</v>
+        <v>-598.2618114193538</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>-0.0476969961374998</v>
+        <v>-0.055196774267857</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>59.21822021686748</v>
+        <v>61.68944497590362</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>35.14156354035198</v>
+        <v>37.61278829938811</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4350,28 +4350,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>700.2923976608188</v>
+        <v>750.31328320802</v>
       </c>
       <c r="R19" t="n">
         <v>198</v>
       </c>
       <c r="S19" t="n">
-        <v>-502.2923976608188</v>
+        <v>-552.3132832080202</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>5666.666666666667</v>
+        <v>6071.428571428572</v>
       </c>
       <c r="V19" s="135" t="n">
         <v>1606.8</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-4059.866666666667</v>
+        <v>-4464.628571428571</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.7164470588235294</v>
+        <v>-0.7353505882352941</v>
       </c>
       <c r="Y19" s="135" t="n">
         <v>8.115151515151515</v>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>1406.599915233327</v>
+        <v>1491.936176659153</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-926.5999152333266</v>
+        <v>-1011.936176659153</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>27924.7311827957</v>
+        <v>29442.39631336405</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>22939.214993</v>
+        <v>23861.864142</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-4985.516189795697</v>
+        <v>-5580.532171364055</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1785340799580284</v>
+        <v>-0.1895406919996869</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>47.79003123541667</v>
+        <v>49.7122169625</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>27.74542264637909</v>
+        <v>29.66760837346241</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46255.29188657407</v>
+        <v>46256.291875</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-23
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 21/08/2026  |  Ultimo aggiornamento: 22/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 22/08/2026  |  Ultimo aggiornamento: 23/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>5419.354838709677</v>
+        <v>5677.419354838709</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>5491.980911</v>
+        <v>5737.982127</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>72.62607229032255</v>
+        <v>60.56277216129092</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0134012395297619</v>
+        <v>0.0106673064602273</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>677.4193548387096</v>
+        <v>709.6774193548387</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>658.335365</v>
+        <v>687.605365</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>-19.08398983870961</v>
+        <v>-22.07205435483866</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>-0.0281716040476189</v>
+        <v>-0.0311015311363635</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>6435.483870967741</v>
+        <v>6741.935483870968</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>5864.3</v>
+        <v>0</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-571.1838709677413</v>
+        <v>-6741.935483870968</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0887553884711778</v>
+        <v>-1</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>291.4478619654914</v>
+        <v>305.3263315828957</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-175.4478619654914</v>
+        <v>-189.3263315828957</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>12532.25806451613</v>
+        <v>13129.03225806452</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>12014.616276</v>
+        <v>6425.587492000001</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-517.6417885161281</v>
+        <v>-6703.444766064515</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0413047501776061</v>
+        <v>-0.510581788078624</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>103.5742782413793</v>
+        <v>55.39299562068966</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>60.57427824137932</v>
+        <v>12.39299562068966</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>43.7044745057232</v>
+        <v>45.78563995837669</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-21.7044745057232</v>
+        <v>-23.78563995837668</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>1354.838709677419</v>
+        <v>1419.354838709677</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>1333.238648</v>
+        <v>1379.090182</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-21.60006167741927</v>
+        <v>-40.26465670967741</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.0159429026666666</v>
+        <v>-0.0283682808636363</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>60.60175672727273</v>
+        <v>62.68591736363636</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>29.60175672727273</v>
+        <v>31.68591736363636</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>73.23452484742808</v>
+        <v>76.72188317349608</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-53.23452484742808</v>
+        <v>-56.72188317349608</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>2709.677419354839</v>
+        <v>2838.709677419354</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>2689.186545</v>
+        <v>2824.039492</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>-20.49087435483852</v>
+        <v>-14.67018541935477</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>-0.007562108392857</v>
+        <v>-0.0051679062272727</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>134.45932725</v>
+        <v>141.2019746</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>97.45932725</v>
+        <v>104.2019746</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>5.839822024471636</v>
+        <v>6.117908787541714</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-3.839822024471636</v>
+        <v>-4.117908787541714</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>338.7096774193548</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>344.699345</v>
+        <v>363.075511</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>5.989667580645175</v>
+        <v>8.236801322580675</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0176837804761905</v>
+        <v>0.0232128037272728</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>172.3496725</v>
+        <v>181.5377555</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>114.3496725</v>
+        <v>123.5377555</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,28 +1540,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>2.116935483870968</v>
+        <v>2.217741935483871</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-1.116935483870968</v>
+        <v>-1.217741935483871</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>338.7096774193548</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="R12" s="117" t="n">
         <v>157.606346</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-181.1033314193548</v>
+        <v>-197.2323636774193</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.5346860260952381</v>
+        <v>-0.5558366612727272</v>
       </c>
       <c r="U12" s="117" t="n">
         <v>157.606346</v>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>196.0950764006791</v>
+        <v>205.4329371816638</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-104.0950764006791</v>
+        <v>-113.4329371816638</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>3725.806451612903</v>
+        <v>3903.225806451613</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>3694.98</v>
+        <v>0</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>-30.82645161290293</v>
+        <v>-3903.225806451613</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>-0.0082737662337661</v>
+        <v>-1</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>40.16282608695652</v>
+        <v>0</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>21.16282608695652</v>
+        <v>-19</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>11.29032258064516</v>
+        <v>11.82795698924731</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-4.290322580645164</v>
+        <v>-4.827956989247314</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>338.7096774193548</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>209.2</v>
+        <v>0</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-129.5096774193548</v>
+        <v>-354.8387096774193</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3823619047619047</v>
+        <v>-1</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>29.88571428571428</v>
+        <v>0</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-0.1142857142857174</v>
+        <v>-30</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>3.763440860215054</v>
+        <v>3.942652329749104</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-3.763440860215054</v>
+        <v>-3.942652329749104</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>338.7096774193548</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-131.1796774193548</v>
+        <v>-354.8387096774193</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3872923809523809</v>
+        <v>-1</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>84.6774193548387</v>
+        <v>88.70967741935483</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-65.6774193548387</v>
+        <v>-69.70967741935483</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>1016.129032258065</v>
+        <v>1064.516129032258</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>988.236982</v>
+        <v>1018.620695</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>-27.89205025806461</v>
+        <v>-45.89543403225809</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>-0.0274493193015873</v>
+        <v>-0.0431138925757576</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>52.01247273684211</v>
+        <v>53.61161552631579</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>40.01247273684211</v>
+        <v>41.61161552631579</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>29.45301542776998</v>
+        <v>30.85553997194951</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-26.45301542776998</v>
+        <v>-27.85553997194951</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>677.4193548387096</v>
+        <v>709.6774193548387</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>615.77</v>
+        <v>0</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-61.64935483870966</v>
+        <v>-709.6774193548387</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.09100619047619039</v>
+        <v>-1</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>205.2566666666666</v>
+        <v>0</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>182.2566666666666</v>
+        <v>-23</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>450.1750314856419</v>
+        <v>471.611937746863</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-284.1750314856419</v>
+        <v>-305.6119377468629</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>10838.70967741935</v>
+        <v>11354.83870967742</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>10240.447866</v>
+        <v>5742.432226</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>-598.2618114193538</v>
+        <v>-5612.406483677419</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>-0.055196774267857</v>
+        <v>-0.4942744346420454</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>61.68944497590362</v>
+        <v>34.59296521686747</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>37.61278829938811</v>
+        <v>10.51630854035197</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>1491.936176659153</v>
+        <v>1527.251552537779</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-1011.936176659153</v>
+        <v>-1047.251552537779</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>29442.39631336405</v>
+        <v>30555.2995391705</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>23861.864142</v>
+        <v>13774.819718</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-5580.532171364055</v>
+        <v>-16780.47982117051</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1895406919996869</v>
+        <v>-0.549183941059347</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>49.7122169625</v>
+        <v>28.69754107916667</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>29.66760837346241</v>
+        <v>8.652932490129086</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>5419.354838709677</v>
+        <v>5677.419354838709</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>5491.980911</v>
+        <v>5737.982127</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>72.62607229032255</v>
+        <v>60.56277216129092</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0134012395297619</v>
+        <v>0.0106673064602273</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>677.4193548387096</v>
+        <v>709.6774193548387</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>658.335365</v>
+        <v>687.605365</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>-19.08398983870961</v>
+        <v>-22.07205435483866</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>-0.0281716040476189</v>
+        <v>-0.0311015311363635</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>6435.483870967741</v>
+        <v>6741.935483870968</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>5864.3</v>
+        <v>0</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-571.1838709677413</v>
+        <v>-6741.935483870968</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0887553884711778</v>
+        <v>-1</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2864,7 +2864,7 @@
       <c r="AD4" s="137" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:no_delivery;crm:stale</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>43.7044745057232</v>
+        <v>45.78563995837669</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-21.7044745057232</v>
+        <v>-23.78563995837668</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>1354.838709677419</v>
+        <v>1419.354838709677</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>1333.238648</v>
+        <v>1379.090182</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>-21.60006167741927</v>
+        <v>-40.26465670967741</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>-0.0159429026666666</v>
+        <v>-0.0283682808636363</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>60.60175672727273</v>
+        <v>62.68591736363636</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>29.60175672727273</v>
+        <v>31.68591736363636</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>73.23452484742808</v>
+        <v>76.72188317349608</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-53.23452484742808</v>
+        <v>-56.72188317349608</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>2709.677419354839</v>
+        <v>2838.709677419354</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>2689.186545</v>
+        <v>2824.039492</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>-20.49087435483852</v>
+        <v>-14.67018541935477</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>-0.007562108392857</v>
+        <v>-0.0051679062272727</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>134.45932725</v>
+        <v>141.2019746</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>97.45932725</v>
+        <v>104.2019746</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>5.839822024471636</v>
+        <v>6.117908787541714</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-3.839822024471636</v>
+        <v>-4.117908787541714</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>338.7096774193548</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>344.699345</v>
+        <v>363.075511</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>5.989667580645175</v>
+        <v>8.236801322580675</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0176837804761905</v>
+        <v>0.0232128037272728</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>172.3496725</v>
+        <v>181.5377555</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>114.3496725</v>
+        <v>123.5377555</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,28 +3563,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>2.116935483870968</v>
+        <v>2.217741935483871</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-1.116935483870968</v>
+        <v>-1.217741935483871</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>338.7096774193548</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="V11" s="135" t="n">
         <v>157.606346</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-181.1033314193548</v>
+        <v>-197.2323636774193</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.5346860260952381</v>
+        <v>-0.5558366612727272</v>
       </c>
       <c r="Y11" s="135" t="n">
         <v>157.606346</v>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>196.0950764006791</v>
+        <v>205.4329371816638</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-104.0950764006791</v>
+        <v>-113.4329371816638</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>3725.806451612903</v>
+        <v>3903.225806451613</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>3694.98</v>
+        <v>0</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>-30.82645161290293</v>
+        <v>-3903.225806451613</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>-0.0082737662337661</v>
+        <v>-1</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>40.16282608695652</v>
+        <v>0</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>21.16282608695652</v>
+        <v>-19</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3708,7 +3708,7 @@
       <c r="AD12" s="137" t="inlineStr"/>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:no_delivery;crm:stale</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>11.29032258064516</v>
+        <v>11.82795698924731</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>-4.290322580645164</v>
+        <v>-4.827956989247314</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>338.7096774193548</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>209.2</v>
+        <v>0</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-129.5096774193548</v>
+        <v>-354.8387096774193</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3823619047619047</v>
+        <v>-1</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>29.88571428571428</v>
+        <v>0</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-0.1142857142857174</v>
+        <v>-30</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3815,7 +3815,7 @@
       <c r="AD13" s="137" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:no_delivery;crm:stale</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>3.763440860215054</v>
+        <v>3.942652329749104</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-3.763440860215054</v>
+        <v>-3.942652329749104</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>338.7096774193548</v>
+        <v>354.8387096774193</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>207.53</v>
+        <v>0</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-131.1796774193548</v>
+        <v>-354.8387096774193</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3872923809523809</v>
+        <v>-1</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3915,7 +3915,7 @@
       <c r="AD14" s="137" t="inlineStr"/>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:no_delivery;crm:stale</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>84.6774193548387</v>
+        <v>88.70967741935483</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-65.6774193548387</v>
+        <v>-69.70967741935483</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>1016.129032258065</v>
+        <v>1064.516129032258</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>988.236982</v>
+        <v>1018.620695</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>-27.89205025806461</v>
+        <v>-45.89543403225809</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>-0.0274493193015873</v>
+        <v>-0.0431138925757576</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>52.01247273684211</v>
+        <v>53.61161552631579</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>40.01247273684211</v>
+        <v>41.61161552631579</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>29.45301542776998</v>
+        <v>30.85553997194951</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-26.45301542776998</v>
+        <v>-27.85553997194951</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>677.4193548387096</v>
+        <v>709.6774193548387</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>615.77</v>
+        <v>0</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-61.64935483870966</v>
+        <v>-709.6774193548387</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.09100619047619039</v>
+        <v>-1</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>205.2566666666666</v>
+        <v>0</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>182.2566666666666</v>
+        <v>-23</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4124,7 +4124,7 @@
       <c r="AD16" s="137" t="inlineStr"/>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>meta:ok;crm:stale</t>
+          <t>meta:no_delivery;crm:stale</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>291.4478619654914</v>
+        <v>305.3263315828957</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-175.4478619654914</v>
+        <v>-189.3263315828957</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>12532.25806451613</v>
+        <v>13129.03225806452</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>12014.616276</v>
+        <v>6425.587492000001</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-517.6417885161281</v>
+        <v>-6703.444766064515</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0413047501776061</v>
+        <v>-0.510581788078624</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>103.5742782413793</v>
+        <v>55.39299562068966</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>60.57427824137932</v>
+        <v>12.39299562068966</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>450.1750314856419</v>
+        <v>471.611937746863</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-284.1750314856419</v>
+        <v>-305.6119377468629</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>10838.70967741935</v>
+        <v>11354.83870967742</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>10240.447866</v>
+        <v>5742.432226</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>-598.2618114193538</v>
+        <v>-5612.406483677419</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>-0.055196774267857</v>
+        <v>-0.4942744346420454</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>61.68944497590362</v>
+        <v>34.59296521686747</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>37.61278829938811</v>
+        <v>10.51630854035197</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>1491.936176659153</v>
+        <v>1527.251552537779</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-1011.936176659153</v>
+        <v>-1047.251552537779</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>29442.39631336405</v>
+        <v>30555.2995391705</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>23861.864142</v>
+        <v>13774.819718</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-5580.532171364055</v>
+        <v>-16780.47982117051</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1895406919996869</v>
+        <v>-0.549183941059347</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>49.7122169625</v>
+        <v>28.69754107916667</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>29.66760837346241</v>
+        <v>8.652932490129086</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46256.291875</v>
+        <v>46257.29188657407</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-24
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 22/08/2026  |  Ultimo aggiornamento: 23/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 23/08/2026  |  Ultimo aggiornamento: 24/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>5677.419354838709</v>
+        <v>5935.483870967741</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>5737.982127</v>
+        <v>6001.442184</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>60.56277216129092</v>
+        <v>65.95831303225896</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0106673064602273</v>
+        <v>0.0111125418695653</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>709.6774193548387</v>
+        <v>741.9354838709677</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>687.605365</v>
+        <v>718.411614</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>-22.07205435483866</v>
+        <v>-23.5238698709677</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>-0.0311015311363635</v>
+        <v>-0.0317060854782608</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>6741.935483870968</v>
+        <v>7048.387096774193</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>0</v>
+        <v>6415.15</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-6741.935483870968</v>
+        <v>-633.2370967741936</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-1</v>
+        <v>-0.089841418764302</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>305.3263315828957</v>
+        <v>319.2048012003</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-189.3263315828957</v>
+        <v>-203.2048012003</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>13129.03225806452</v>
+        <v>13725.8064516129</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>6425.587492000001</v>
+        <v>13135.003798</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-6703.444766064515</v>
+        <v>-590.8026536129018</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.510581788078624</v>
+        <v>-0.0430432015558165</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>55.39299562068966</v>
+        <v>113.232791362069</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>12.39299562068966</v>
+        <v>70.23279136206897</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>45.78563995837669</v>
+        <v>47.86680541103017</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-23.78563995837668</v>
+        <v>-25.86680541103017</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>1419.354838709677</v>
+        <v>1483.870967741935</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>1379.090182</v>
+        <v>1424.034157</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-40.26465670967741</v>
+        <v>-59.83681074193533</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.0283682808636363</v>
+        <v>-0.0403248072391303</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>62.68591736363636</v>
+        <v>64.72882531818182</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>31.68591736363636</v>
+        <v>33.72882531818182</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>76.72188317349608</v>
+        <v>80.20924149956409</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-56.72188317349608</v>
+        <v>-60.20924149956409</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>2838.709677419354</v>
+        <v>2967.741935483871</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>2824.039492</v>
+        <v>2947.733182</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>-14.67018541935477</v>
+        <v>-20.00875348387081</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>-0.0051679062272727</v>
+        <v>-0.0067420799782608</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>141.2019746</v>
+        <v>147.3866591</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>104.2019746</v>
+        <v>110.3866591</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>6.117908787541714</v>
+        <v>6.395995550611792</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-4.117908787541714</v>
+        <v>-4.395995550611792</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>354.8387096774193</v>
+        <v>370.9677419354838</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>363.075511</v>
+        <v>374.253321</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>8.236801322580675</v>
+        <v>3.285579064516185</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0232128037272728</v>
+        <v>0.008856778347826199</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>181.5377555</v>
+        <v>187.1266605</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>123.5377555</v>
+        <v>129.1266605</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,28 +1540,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>2.217741935483871</v>
+        <v>2.318548387096774</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-1.217741935483871</v>
+        <v>-1.318548387096774</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>354.8387096774193</v>
+        <v>370.9677419354838</v>
       </c>
       <c r="R12" s="117" t="n">
         <v>157.606346</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-197.2323636774193</v>
+        <v>-213.3613959354838</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.5558366612727272</v>
+        <v>-0.5751481107826086</v>
       </c>
       <c r="U12" s="117" t="n">
         <v>157.606346</v>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>205.4329371816638</v>
+        <v>214.7707979626485</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-113.4329371816638</v>
+        <v>-122.7707979626485</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>3903.225806451613</v>
+        <v>4080.645161290322</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>0</v>
+        <v>4001.21</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>-3903.225806451613</v>
+        <v>-79.43516129032241</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>-1</v>
+        <v>-0.0194663241106718</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>0</v>
+        <v>43.49141304347826</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>-19</v>
+        <v>24.49141304347826</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>11.82795698924731</v>
+        <v>12.36559139784946</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-4.827956989247314</v>
+        <v>-5.365591397849464</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>354.8387096774193</v>
+        <v>370.9677419354838</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>0</v>
+        <v>231.44</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-354.8387096774193</v>
+        <v>-139.5277419354838</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-1</v>
+        <v>-0.3761182608695652</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>0</v>
+        <v>33.06285714285714</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>-30</v>
+        <v>3.062857142857141</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>3.942652329749104</v>
+        <v>4.121863799283154</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-3.942652329749104</v>
+        <v>-4.121863799283154</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>354.8387096774193</v>
+        <v>370.9677419354838</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>0</v>
+        <v>231.15</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-354.8387096774193</v>
+        <v>-139.8177419354838</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-1</v>
+        <v>-0.3768999999999999</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>88.70967741935483</v>
+        <v>92.74193548387096</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-69.70967741935483</v>
+        <v>-73.74193548387096</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>1064.516129032258</v>
+        <v>1112.903225806452</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>1018.620695</v>
+        <v>1047.421456</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>-45.89543403225809</v>
+        <v>-65.48176980645167</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>-0.0431138925757576</v>
+        <v>-0.0588386917101449</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>53.61161552631579</v>
+        <v>55.12744505263158</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>41.61161552631579</v>
+        <v>43.12744505263158</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>30.85553997194951</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-27.85553997194951</v>
+        <v>-29.25806451612903</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>709.6774193548387</v>
+        <v>741.9354838709677</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>0</v>
+        <v>674.39</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-709.6774193548387</v>
+        <v>-67.5454838709677</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-1</v>
+        <v>-0.09103956521739121</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>0</v>
+        <v>224.7966666666667</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>-23</v>
+        <v>201.7966666666667</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>471.611937746863</v>
+        <v>493.048844008084</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-305.6119377468629</v>
+        <v>-327.048844008084</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>11354.83870967742</v>
+        <v>11870.96774193548</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>5742.432226</v>
+        <v>11089.238462</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>-5612.406483677419</v>
+        <v>-781.7292799354836</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>-0.4942744346420454</v>
+        <v>-0.0658521947771739</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>34.59296521686747</v>
+        <v>66.8026413373494</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>10.51630854035197</v>
+        <v>42.7259846608339</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>1527.251552537779</v>
+        <v>1562.566928416404</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-1047.251552537779</v>
+        <v>-1082.566928416404</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>30555.2995391705</v>
+        <v>31668.20276497696</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>13774.819718</v>
+        <v>25831.04226</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-16780.47982117051</v>
+        <v>-5837.160504976961</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.549183941059347</v>
+        <v>-0.1843224431868452</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>28.69754107916667</v>
+        <v>53.814671375</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>8.652932490129086</v>
+        <v>33.77006278596241</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>5677.419354838709</v>
+        <v>5935.483870967741</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>5737.982127</v>
+        <v>6001.442184</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>60.56277216129092</v>
+        <v>65.95831303225896</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0106673064602273</v>
+        <v>0.0111125418695653</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>709.6774193548387</v>
+        <v>741.9354838709677</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>687.605365</v>
+        <v>718.411614</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>-22.07205435483866</v>
+        <v>-23.5238698709677</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>-0.0311015311363635</v>
+        <v>-0.0317060854782608</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>6741.935483870968</v>
+        <v>7048.387096774193</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>0</v>
+        <v>6415.15</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-6741.935483870968</v>
+        <v>-633.2370967741936</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-1</v>
+        <v>-0.089841418764302</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2864,7 +2864,7 @@
       <c r="AD4" s="137" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>meta:no_delivery;crm:stale</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>45.78563995837669</v>
+        <v>47.86680541103017</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-23.78563995837668</v>
+        <v>-25.86680541103017</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>1419.354838709677</v>
+        <v>1483.870967741935</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>1379.090182</v>
+        <v>1424.034157</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>-40.26465670967741</v>
+        <v>-59.83681074193533</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>-0.0283682808636363</v>
+        <v>-0.0403248072391303</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>62.68591736363636</v>
+        <v>64.72882531818182</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>31.68591736363636</v>
+        <v>33.72882531818182</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>76.72188317349608</v>
+        <v>80.20924149956409</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-56.72188317349608</v>
+        <v>-60.20924149956409</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>2838.709677419354</v>
+        <v>2967.741935483871</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>2824.039492</v>
+        <v>2947.733182</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>-14.67018541935477</v>
+        <v>-20.00875348387081</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>-0.0051679062272727</v>
+        <v>-0.0067420799782608</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>141.2019746</v>
+        <v>147.3866591</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>104.2019746</v>
+        <v>110.3866591</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>6.117908787541714</v>
+        <v>6.395995550611792</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-4.117908787541714</v>
+        <v>-4.395995550611792</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>354.8387096774193</v>
+        <v>370.9677419354838</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>363.075511</v>
+        <v>374.253321</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>8.236801322580675</v>
+        <v>3.285579064516185</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0232128037272728</v>
+        <v>0.008856778347826199</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>181.5377555</v>
+        <v>187.1266605</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>123.5377555</v>
+        <v>129.1266605</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,28 +3563,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>2.217741935483871</v>
+        <v>2.318548387096774</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-1.217741935483871</v>
+        <v>-1.318548387096774</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>354.8387096774193</v>
+        <v>370.9677419354838</v>
       </c>
       <c r="V11" s="135" t="n">
         <v>157.606346</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-197.2323636774193</v>
+        <v>-213.3613959354838</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.5558366612727272</v>
+        <v>-0.5751481107826086</v>
       </c>
       <c r="Y11" s="135" t="n">
         <v>157.606346</v>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>205.4329371816638</v>
+        <v>214.7707979626485</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-113.4329371816638</v>
+        <v>-122.7707979626485</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>3903.225806451613</v>
+        <v>4080.645161290322</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>0</v>
+        <v>4001.21</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>-3903.225806451613</v>
+        <v>-79.43516129032241</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>-1</v>
+        <v>-0.0194663241106718</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>0</v>
+        <v>43.49141304347826</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>-19</v>
+        <v>24.49141304347826</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3708,7 +3708,7 @@
       <c r="AD12" s="137" t="inlineStr"/>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>meta:no_delivery;crm:stale</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>11.82795698924731</v>
+        <v>12.36559139784946</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>-4.827956989247314</v>
+        <v>-5.365591397849464</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>354.8387096774193</v>
+        <v>370.9677419354838</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>0</v>
+        <v>231.44</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-354.8387096774193</v>
+        <v>-139.5277419354838</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-1</v>
+        <v>-0.3761182608695652</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>0</v>
+        <v>33.06285714285714</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>-30</v>
+        <v>3.062857142857141</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3815,7 +3815,7 @@
       <c r="AD13" s="137" t="inlineStr"/>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>meta:no_delivery;crm:stale</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>3.942652329749104</v>
+        <v>4.121863799283154</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-3.942652329749104</v>
+        <v>-4.121863799283154</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>354.8387096774193</v>
+        <v>370.9677419354838</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>0</v>
+        <v>231.15</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-354.8387096774193</v>
+        <v>-139.8177419354838</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-1</v>
+        <v>-0.3768999999999999</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3915,7 +3915,7 @@
       <c r="AD14" s="137" t="inlineStr"/>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>meta:no_delivery;crm:stale</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>88.70967741935483</v>
+        <v>92.74193548387096</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-69.70967741935483</v>
+        <v>-73.74193548387096</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>1064.516129032258</v>
+        <v>1112.903225806452</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>1018.620695</v>
+        <v>1047.421456</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>-45.89543403225809</v>
+        <v>-65.48176980645167</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>-0.0431138925757576</v>
+        <v>-0.0588386917101449</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>53.61161552631579</v>
+        <v>55.12744505263158</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>41.61161552631579</v>
+        <v>43.12744505263158</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>30.85553997194951</v>
+        <v>32.25806451612903</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-27.85553997194951</v>
+        <v>-29.25806451612903</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>709.6774193548387</v>
+        <v>741.9354838709677</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>0</v>
+        <v>674.39</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-709.6774193548387</v>
+        <v>-67.5454838709677</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-1</v>
+        <v>-0.09103956521739121</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>0</v>
+        <v>224.7966666666667</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>-23</v>
+        <v>201.7966666666667</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4124,7 +4124,7 @@
       <c r="AD16" s="137" t="inlineStr"/>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>meta:no_delivery;crm:stale</t>
+          <t>meta:ok;crm:stale</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>305.3263315828957</v>
+        <v>319.2048012003</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-189.3263315828957</v>
+        <v>-203.2048012003</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>13129.03225806452</v>
+        <v>13725.8064516129</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>6425.587492000001</v>
+        <v>13135.003798</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-6703.444766064515</v>
+        <v>-590.8026536129018</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.510581788078624</v>
+        <v>-0.0430432015558165</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>55.39299562068966</v>
+        <v>113.232791362069</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>12.39299562068966</v>
+        <v>70.23279136206897</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>471.611937746863</v>
+        <v>493.048844008084</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-305.6119377468629</v>
+        <v>-327.048844008084</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>11354.83870967742</v>
+        <v>11870.96774193548</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>5742.432226</v>
+        <v>11089.238462</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>-5612.406483677419</v>
+        <v>-781.7292799354836</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>-0.4942744346420454</v>
+        <v>-0.0658521947771739</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>34.59296521686747</v>
+        <v>66.8026413373494</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>10.51630854035197</v>
+        <v>42.7259846608339</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>1527.251552537779</v>
+        <v>1562.566928416404</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-1047.251552537779</v>
+        <v>-1082.566928416404</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>30555.2995391705</v>
+        <v>31668.20276497696</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>13774.819718</v>
+        <v>25831.04226</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-16780.47982117051</v>
+        <v>-5837.160504976961</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.549183941059347</v>
+        <v>-0.1843224431868452</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>28.69754107916667</v>
+        <v>53.814671375</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>8.652932490129086</v>
+        <v>33.77006278596241</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46257.29188657407</v>
+        <v>46258.29190972223</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-25
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 23/08/2026  |  Ultimo aggiornamento: 24/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 24/08/2026  |  Ultimo aggiornamento: 25/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>5935.483870967741</v>
+        <v>6193.548387096775</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>6001.442184</v>
+        <v>6256.285785</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>65.95831303225896</v>
+        <v>62.73739790322543</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0111125418695653</v>
+        <v>0.0101294757031249</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>741.9354838709677</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>718.411614</v>
+        <v>747.771898</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>-23.5238698709677</v>
+        <v>-26.42165038709686</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>-0.0317060854782608</v>
+        <v>-0.0341279650833334</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>7048.387096774193</v>
+        <v>7354.838709677419</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>6415.15</v>
+        <v>6708.89</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-633.2370967741936</v>
+        <v>-645.9487096774183</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.089841418764302</v>
+        <v>-0.0878263596491226</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>319.2048012003</v>
+        <v>333.0832708177044</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-203.2048012003</v>
+        <v>-217.0832708177044</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>13725.8064516129</v>
+        <v>14322.58064516129</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>13135.003798</v>
+        <v>13712.947683</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-590.8026536129018</v>
+        <v>-609.6329621612895</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0430432015558165</v>
+        <v>-0.0425644635743242</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>113.232791362069</v>
+        <v>118.2150662327586</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>70.23279136206897</v>
+        <v>75.21506623275863</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>47.86680541103017</v>
+        <v>49.94797086368366</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-25.86680541103017</v>
+        <v>-27.94797086368366</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>1483.870967741935</v>
+        <v>1548.387096774194</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>1424.034157</v>
+        <v>1470.519531</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-59.83681074193533</v>
+        <v>-77.86756577419374</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.0403248072391303</v>
+        <v>-0.0502894695625001</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>64.72882531818182</v>
+        <v>66.84179686363636</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>33.72882531818182</v>
+        <v>35.84179686363636</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>80.20924149956409</v>
+        <v>83.69659982563209</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-60.20924149956409</v>
+        <v>-63.69659982563209</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>2967.741935483871</v>
+        <v>3096.774193548388</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>2947.733182</v>
+        <v>3079.972742</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>-20.00875348387081</v>
+        <v>-16.80145154838738</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>-0.0067420799782608</v>
+        <v>-0.0054254687291667</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>147.3866591</v>
+        <v>153.9986371</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>110.3866591</v>
+        <v>116.9986371</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>6.395995550611792</v>
+        <v>6.67408231368187</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-4.395995550611792</v>
+        <v>-4.67408231368187</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>370.9677419354838</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>374.253321</v>
+        <v>408.723321</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>3.285579064516185</v>
+        <v>21.62654680645158</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.008856778347826199</v>
+        <v>0.0558685792499999</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>187.1266605</v>
+        <v>204.3616605</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>129.1266605</v>
+        <v>146.3616605</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,28 +1540,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>2.318548387096774</v>
+        <v>2.419354838709677</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-1.318548387096774</v>
+        <v>-1.419354838709677</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>370.9677419354838</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="R12" s="117" t="n">
         <v>157.606346</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-213.3613959354838</v>
+        <v>-229.4904281935484</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.5751481107826086</v>
+        <v>-0.5928502728333334</v>
       </c>
       <c r="U12" s="117" t="n">
         <v>157.606346</v>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>214.7707979626485</v>
+        <v>224.1086587436333</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-122.7707979626485</v>
+        <v>-132.1086587436333</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>4080.645161290322</v>
+        <v>4258.064516129032</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>4001.21</v>
+        <v>4191.87</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>-79.43516129032241</v>
+        <v>-66.19451612903231</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>-0.0194663241106718</v>
+        <v>-0.0155456818181818</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>43.49141304347826</v>
+        <v>45.56380434782609</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>24.49141304347826</v>
+        <v>26.56380434782609</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>12.36559139784946</v>
+        <v>12.90322580645162</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-5.365591397849464</v>
+        <v>-5.903225806451616</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>370.9677419354838</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>231.44</v>
+        <v>241.84</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-139.5277419354838</v>
+        <v>-145.2567741935484</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3761182608695652</v>
+        <v>-0.3752466666666667</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>33.06285714285714</v>
+        <v>34.54857142857143</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>3.062857142857141</v>
+        <v>4.548571428571428</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>4.121863799283154</v>
+        <v>4.301075268817204</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-4.121863799283154</v>
+        <v>-4.301075268817204</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>370.9677419354838</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>231.15</v>
+        <v>240.37</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-139.8177419354838</v>
+        <v>-146.7267741935484</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3768999999999999</v>
+        <v>-0.3790441666666667</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>92.74193548387096</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-73.74193548387096</v>
+        <v>-77.7741935483871</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>1112.903225806452</v>
+        <v>1161.290322580645</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>1047.421456</v>
+        <v>1074.657643</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>-65.48176980645167</v>
+        <v>-86.63267958064534</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>-0.0588386917101449</v>
+        <v>-0.07460036297222231</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>55.12744505263158</v>
+        <v>56.56092857894737</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>43.12744505263158</v>
+        <v>44.56092857894737</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>32.25806451612903</v>
+        <v>33.66058906030855</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-29.25806451612903</v>
+        <v>-30.66058906030856</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>741.9354838709677</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>674.39</v>
+        <v>708.86</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-67.5454838709677</v>
+        <v>-65.33354838709681</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.09103956521739121</v>
+        <v>-0.0843891666666667</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>224.7966666666667</v>
+        <v>236.2866666666666</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>201.7966666666667</v>
+        <v>213.2866666666666</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>493.048844008084</v>
+        <v>514.4857502693051</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-327.048844008084</v>
+        <v>-348.4857502693051</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>11870.96774193548</v>
+        <v>12387.09677419355</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>11089.238462</v>
+        <v>11574.419583</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>-781.7292799354836</v>
+        <v>-812.6771911935502</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>-0.0658521947771739</v>
+        <v>-0.06560675241406259</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>66.8026413373494</v>
+        <v>69.72541917469879</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>42.7259846608339</v>
+        <v>45.64876249818329</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2063,28 +2063,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>422.9323308270677</v>
+        <v>451.1278195488723</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>93</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-329.9323308270677</v>
+        <v>-358.1278195488723</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>3214.285714285714</v>
+        <v>3428.571428571428</v>
       </c>
       <c r="R19" s="117" t="n">
         <v>706.8</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-2507.485714285714</v>
+        <v>-2721.771428571428</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.7801066666666667</v>
+        <v>-0.7938499999999999</v>
       </c>
       <c r="U19" s="117" t="n">
         <v>7.6</v>
@@ -2138,28 +2138,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>238.0952380952381</v>
+        <v>253.9682539682539</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>60</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-178.0952380952381</v>
+        <v>-193.9682539682539</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>2142.857142857143</v>
+        <v>2285.714285714286</v>
       </c>
       <c r="R20" s="117" t="n">
         <v>540</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-1602.857142857143</v>
+        <v>-1745.714285714286</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.748</v>
+        <v>-0.76375</v>
       </c>
       <c r="U20" s="117" t="n">
         <v>9</v>
@@ -2213,28 +2213,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>89.28571428571429</v>
+        <v>95.23809523809524</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-44.28571428571429</v>
+        <v>-50.23809523809524</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>714.2857142857143</v>
+        <v>761.9047619047619</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>360</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-354.2857142857143</v>
+        <v>-401.9047619047619</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.496</v>
+        <v>-0.5275</v>
       </c>
       <c r="U21" s="117" t="n">
         <v>8</v>
@@ -2276,28 +2276,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>750.31328320802</v>
+        <v>800.3341687552214</v>
       </c>
       <c r="N22" s="125" t="n">
         <v>198</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-552.3132832080202</v>
+        <v>-602.3341687552214</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="Q22" s="123" t="n">
-        <v>6071.428571428572</v>
+        <v>6476.190476190476</v>
       </c>
       <c r="R22" s="123" t="n">
         <v>1606.8</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-4464.628571428571</v>
+        <v>-4869.390476190476</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-0.7353505882352941</v>
+        <v>-0.7518911764705882</v>
       </c>
       <c r="U22" s="123" t="n">
         <v>8.115151515151515</v>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>1562.566928416404</v>
+        <v>1647.903189842231</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-1082.566928416404</v>
+        <v>-1167.903189842231</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>31668.20276497696</v>
+        <v>33185.86789554531</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>25831.04226</v>
+        <v>26894.167266</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-5837.160504976961</v>
+        <v>-6291.700629545314</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1843224431868452</v>
+        <v>-0.1895897569817626</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>53.814671375</v>
+        <v>56.0295151375</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>33.77006278596241</v>
+        <v>35.98490654846242</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>5935.483870967741</v>
+        <v>6193.548387096775</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>6001.442184</v>
+        <v>6256.285785</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>65.95831303225896</v>
+        <v>62.73739790322543</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0111125418695653</v>
+        <v>0.0101294757031249</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>741.9354838709677</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>718.411614</v>
+        <v>747.771898</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>-23.5238698709677</v>
+        <v>-26.42165038709686</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>-0.0317060854782608</v>
+        <v>-0.0341279650833334</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>7048.387096774193</v>
+        <v>7354.838709677419</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>6415.15</v>
+        <v>6708.89</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-633.2370967741936</v>
+        <v>-645.9487096774183</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.089841418764302</v>
+        <v>-0.0878263596491226</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2933,28 +2933,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>422.9323308270677</v>
+        <v>451.1278195488723</v>
       </c>
       <c r="R5" t="n">
         <v>93</v>
       </c>
       <c r="S5" t="n">
-        <v>-329.9323308270677</v>
+        <v>-358.1278195488723</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="U5" s="135" t="n">
-        <v>3214.285714285714</v>
+        <v>3428.571428571428</v>
       </c>
       <c r="V5" s="135" t="n">
         <v>706.8</v>
       </c>
       <c r="W5" s="135" t="n">
-        <v>-2507.485714285714</v>
+        <v>-2721.771428571428</v>
       </c>
       <c r="X5" s="136" t="n">
-        <v>-0.7801066666666667</v>
+        <v>-0.7938499999999999</v>
       </c>
       <c r="Y5" s="135" t="n">
         <v>7.6</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3036,28 +3036,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>238.0952380952381</v>
+        <v>253.9682539682539</v>
       </c>
       <c r="R6" t="n">
         <v>60</v>
       </c>
       <c r="S6" t="n">
-        <v>-178.0952380952381</v>
+        <v>-193.9682539682539</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>2142.857142857143</v>
+        <v>2285.714285714286</v>
       </c>
       <c r="V6" s="135" t="n">
         <v>540</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-1602.857142857143</v>
+        <v>-1745.714285714286</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.748</v>
+        <v>-0.76375</v>
       </c>
       <c r="Y6" s="135" t="n">
         <v>9</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3139,28 +3139,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>89.28571428571429</v>
+        <v>95.23809523809524</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>-44.28571428571429</v>
+        <v>-50.23809523809524</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>714.2857142857143</v>
+        <v>761.9047619047619</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>360</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>-354.2857142857143</v>
+        <v>-401.9047619047619</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>-0.496</v>
+        <v>-0.5275</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>8</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>47.86680541103017</v>
+        <v>49.94797086368366</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-25.86680541103017</v>
+        <v>-27.94797086368366</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>1483.870967741935</v>
+        <v>1548.387096774194</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>1424.034157</v>
+        <v>1470.519531</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>-59.83681074193533</v>
+        <v>-77.86756577419374</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>-0.0403248072391303</v>
+        <v>-0.0502894695625001</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>64.72882531818182</v>
+        <v>66.84179686363636</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>33.72882531818182</v>
+        <v>35.84179686363636</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>80.20924149956409</v>
+        <v>83.69659982563209</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-60.20924149956409</v>
+        <v>-63.69659982563209</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>2967.741935483871</v>
+        <v>3096.774193548388</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>2947.733182</v>
+        <v>3079.972742</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>-20.00875348387081</v>
+        <v>-16.80145154838738</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>-0.0067420799782608</v>
+        <v>-0.0054254687291667</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>147.3866591</v>
+        <v>153.9986371</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>110.3866591</v>
+        <v>116.9986371</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>6.395995550611792</v>
+        <v>6.67408231368187</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-4.395995550611792</v>
+        <v>-4.67408231368187</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>370.9677419354838</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>374.253321</v>
+        <v>408.723321</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>3.285579064516185</v>
+        <v>21.62654680645158</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.008856778347826199</v>
+        <v>0.0558685792499999</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>187.1266605</v>
+        <v>204.3616605</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>129.1266605</v>
+        <v>146.3616605</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,28 +3563,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>2.318548387096774</v>
+        <v>2.419354838709677</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-1.318548387096774</v>
+        <v>-1.419354838709677</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>370.9677419354838</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="V11" s="135" t="n">
         <v>157.606346</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-213.3613959354838</v>
+        <v>-229.4904281935484</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.5751481107826086</v>
+        <v>-0.5928502728333334</v>
       </c>
       <c r="Y11" s="135" t="n">
         <v>157.606346</v>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>214.7707979626485</v>
+        <v>224.1086587436333</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-122.7707979626485</v>
+        <v>-132.1086587436333</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>4080.645161290322</v>
+        <v>4258.064516129032</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>4001.21</v>
+        <v>4191.87</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>-79.43516129032241</v>
+        <v>-66.19451612903231</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>-0.0194663241106718</v>
+        <v>-0.0155456818181818</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>43.49141304347826</v>
+        <v>45.56380434782609</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>24.49141304347826</v>
+        <v>26.56380434782609</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>12.36559139784946</v>
+        <v>12.90322580645162</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>-5.365591397849464</v>
+        <v>-5.903225806451616</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>370.9677419354838</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>231.44</v>
+        <v>241.84</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-139.5277419354838</v>
+        <v>-145.2567741935484</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3761182608695652</v>
+        <v>-0.3752466666666667</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>33.06285714285714</v>
+        <v>34.54857142857143</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>3.062857142857141</v>
+        <v>4.548571428571428</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.121863799283154</v>
+        <v>4.301075268817204</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-4.121863799283154</v>
+        <v>-4.301075268817204</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>370.9677419354838</v>
+        <v>387.0967741935484</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>231.15</v>
+        <v>240.37</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-139.8177419354838</v>
+        <v>-146.7267741935484</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3768999999999999</v>
+        <v>-0.3790441666666667</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>92.74193548387096</v>
+        <v>96.7741935483871</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-73.74193548387096</v>
+        <v>-77.7741935483871</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>1112.903225806452</v>
+        <v>1161.290322580645</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>1047.421456</v>
+        <v>1074.657643</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>-65.48176980645167</v>
+        <v>-86.63267958064534</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>-0.0588386917101449</v>
+        <v>-0.07460036297222231</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>55.12744505263158</v>
+        <v>56.56092857894737</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>43.12744505263158</v>
+        <v>44.56092857894737</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>32.25806451612903</v>
+        <v>33.66058906030855</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-29.25806451612903</v>
+        <v>-30.66058906030856</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>741.9354838709677</v>
+        <v>774.1935483870968</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>674.39</v>
+        <v>708.86</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-67.5454838709677</v>
+        <v>-65.33354838709681</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.09103956521739121</v>
+        <v>-0.0843891666666667</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>224.7966666666667</v>
+        <v>236.2866666666666</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>201.7966666666667</v>
+        <v>213.2866666666666</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>319.2048012003</v>
+        <v>333.0832708177044</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-203.2048012003</v>
+        <v>-217.0832708177044</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>13725.8064516129</v>
+        <v>14322.58064516129</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>13135.003798</v>
+        <v>13712.947683</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-590.8026536129018</v>
+        <v>-609.6329621612895</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0430432015558165</v>
+        <v>-0.0425644635743242</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>113.232791362069</v>
+        <v>118.2150662327586</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>70.23279136206897</v>
+        <v>75.21506623275863</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>493.048844008084</v>
+        <v>514.4857502693051</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-327.048844008084</v>
+        <v>-348.4857502693051</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>11870.96774193548</v>
+        <v>12387.09677419355</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>11089.238462</v>
+        <v>11574.419583</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>-781.7292799354836</v>
+        <v>-812.6771911935502</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>-0.0658521947771739</v>
+        <v>-0.06560675241406259</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>66.8026413373494</v>
+        <v>69.72541917469879</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>42.7259846608339</v>
+        <v>45.64876249818329</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4350,28 +4350,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>750.31328320802</v>
+        <v>800.3341687552214</v>
       </c>
       <c r="R19" t="n">
         <v>198</v>
       </c>
       <c r="S19" t="n">
-        <v>-552.3132832080202</v>
+        <v>-602.3341687552214</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>6071.428571428572</v>
+        <v>6476.190476190476</v>
       </c>
       <c r="V19" s="135" t="n">
         <v>1606.8</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-4464.628571428571</v>
+        <v>-4869.390476190476</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.7353505882352941</v>
+        <v>-0.7518911764705882</v>
       </c>
       <c r="Y19" s="135" t="n">
         <v>8.115151515151515</v>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>1562.566928416404</v>
+        <v>1647.903189842231</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-1082.566928416404</v>
+        <v>-1167.903189842231</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>31668.20276497696</v>
+        <v>33185.86789554531</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>25831.04226</v>
+        <v>26894.167266</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-5837.160504976961</v>
+        <v>-6291.700629545314</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1843224431868452</v>
+        <v>-0.1895897569817626</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>53.814671375</v>
+        <v>56.0295151375</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>33.77006278596241</v>
+        <v>35.98490654846242</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46258.29190972223</v>
+        <v>46259.291875</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-26
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 24/08/2026  |  Ultimo aggiornamento: 25/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 25/08/2026  |  Ultimo aggiornamento: 26/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>6193.548387096775</v>
+        <v>6451.612903225807</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>6256.285785</v>
+        <v>6551.493881</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>62.73739790322543</v>
+        <v>99.88097777419352</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0101294757031249</v>
+        <v>0.0154815515549999</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>774.1935483870968</v>
+        <v>806.4516129032259</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>747.771898</v>
+        <v>801.896588</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>-26.42165038709686</v>
+        <v>-4.555024903225899</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>-0.0341279650833334</v>
+        <v>-0.0056482308800001</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>7354.838709677419</v>
+        <v>7661.290322580645</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>6708.89</v>
+        <v>7066.75</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-645.9487096774183</v>
+        <v>-594.5403225806449</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0878263596491226</v>
+        <v>-0.0776031578947368</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>333.0832708177044</v>
+        <v>346.9617404351088</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-217.0832708177044</v>
+        <v>-230.9617404351088</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>14322.58064516129</v>
+        <v>14919.35483870968</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>13712.947683</v>
+        <v>14420.140469</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-609.6329621612895</v>
+        <v>-499.2143697096781</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0425644635743242</v>
+        <v>-0.0334608550508108</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>118.2150662327586</v>
+        <v>124.3115557672414</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>75.21506623275863</v>
+        <v>81.31155576724137</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>49.94797086368366</v>
+        <v>52.02913631633714</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-27.94797086368366</v>
+        <v>-30.02913631633714</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>1548.387096774194</v>
+        <v>1612.903225806452</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>1470.519531</v>
+        <v>1525.409531</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-77.86756577419374</v>
+        <v>-87.49369480645169</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.0502894695625001</v>
+        <v>-0.05424609078</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>66.84179686363636</v>
+        <v>69.33679686363637</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>35.84179686363636</v>
+        <v>38.33679686363637</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>83.69659982563209</v>
+        <v>87.1839581517001</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-63.69659982563209</v>
+        <v>-67.1839581517001</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>3096.774193548388</v>
+        <v>3225.806451612903</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>3079.972742</v>
+        <v>3248.620991</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>-16.80145154838738</v>
+        <v>22.81453938709637</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>-0.0054254687291667</v>
+        <v>0.0070725072099998</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>153.9986371</v>
+        <v>162.43104955</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>116.9986371</v>
+        <v>125.43104955</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>6.67408231368187</v>
+        <v>6.952169076751948</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-4.67408231368187</v>
+        <v>-4.952169076751948</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>387.0967741935484</v>
+        <v>403.2258064516129</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>408.723321</v>
+        <v>415.854922</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>21.62654680645158</v>
+        <v>12.62911554838706</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0558685792499999</v>
+        <v>0.0313202065599999</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>204.3616605</v>
+        <v>207.927461</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>146.3616605</v>
+        <v>149.927461</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,34 +1540,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>2.419354838709677</v>
+        <v>2.520161290322581</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-1.419354838709677</v>
+        <v>-1.52016129032258</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>387.0967741935484</v>
+        <v>403.2258064516129</v>
       </c>
       <c r="R12" s="117" t="n">
-        <v>157.606346</v>
+        <v>162.246346</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-229.4904281935484</v>
+        <v>-240.9794604516129</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.5928502728333334</v>
+        <v>-0.5976290619200001</v>
       </c>
       <c r="U12" s="117" t="n">
-        <v>157.606346</v>
+        <v>162.246346</v>
       </c>
       <c r="V12" s="117" t="n">
-        <v>-2.393653999999998</v>
+        <v>2.246345999999988</v>
       </c>
       <c r="W12" s="120" t="inlineStr"/>
     </row>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>224.1086587436333</v>
+        <v>233.446519524618</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-132.1086587436333</v>
+        <v>-141.446519524618</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>4258.064516129032</v>
+        <v>4435.483870967741</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>4191.87</v>
+        <v>4374.49</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>-66.19451612903231</v>
+        <v>-60.99387096774171</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>-0.0155456818181818</v>
+        <v>-0.0137513454545454</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>45.56380434782609</v>
+        <v>47.54880434782608</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>26.56380434782609</v>
+        <v>28.54880434782608</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>12.90322580645162</v>
+        <v>13.44086021505377</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-5.903225806451616</v>
+        <v>-6.440860215053766</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>387.0967741935484</v>
+        <v>403.2258064516129</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>241.84</v>
+        <v>257.34</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-145.2567741935484</v>
+        <v>-145.885806451613</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3752466666666667</v>
+        <v>-0.3617968000000001</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>34.54857142857143</v>
+        <v>36.76285714285714</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>4.548571428571428</v>
+        <v>6.762857142857136</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>4.301075268817204</v>
+        <v>4.480286738351254</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-4.301075268817204</v>
+        <v>-4.480286738351254</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>387.0967741935484</v>
+        <v>403.2258064516129</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>240.37</v>
+        <v>253.32</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-146.7267741935484</v>
+        <v>-149.9058064516129</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3790441666666667</v>
+        <v>-0.3717664</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>96.7741935483871</v>
+        <v>100.8064516129032</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-77.7741935483871</v>
+        <v>-81.80645161290323</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>1161.290322580645</v>
+        <v>1209.677419354839</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>1074.657643</v>
+        <v>1118.466974</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>-86.63267958064534</v>
+        <v>-91.21044535483884</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>-0.07460036297222231</v>
+        <v>-0.0754006348266667</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>56.56092857894737</v>
+        <v>58.86668284210526</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>44.56092857894737</v>
+        <v>46.86668284210526</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>33.66058906030855</v>
+        <v>35.06311360448808</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-30.66058906030856</v>
+        <v>-32.06311360448808</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>774.1935483870968</v>
+        <v>806.4516129032259</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>708.86</v>
+        <v>742.35</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-65.33354838709681</v>
+        <v>-64.10161290322583</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.0843891666666667</v>
+        <v>-0.079486</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>236.2866666666666</v>
+        <v>247.45</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>213.2866666666666</v>
+        <v>224.45</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>514.4857502693051</v>
+        <v>535.9226565305261</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-348.4857502693051</v>
+        <v>-369.9226565305261</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>12387.09677419355</v>
+        <v>12903.22580645161</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>11574.419583</v>
+        <v>12098.098764</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>-812.6771911935502</v>
+        <v>-805.1270424516133</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>-0.06560675241406259</v>
+        <v>-0.06239734579</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>69.72541917469879</v>
+        <v>72.88011303614458</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>45.64876249818329</v>
+        <v>48.80345635962908</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2063,28 +2063,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>451.1278195488723</v>
+        <v>479.3233082706768</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>93</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-358.1278195488723</v>
+        <v>-386.3233082706768</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>3428.571428571428</v>
+        <v>3642.857142857143</v>
       </c>
       <c r="R19" s="117" t="n">
         <v>706.8</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-2721.771428571428</v>
+        <v>-2936.057142857143</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.7938499999999999</v>
+        <v>-0.8059764705882354</v>
       </c>
       <c r="U19" s="117" t="n">
         <v>7.6</v>
@@ -2138,28 +2138,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>253.9682539682539</v>
+        <v>269.8412698412698</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>60</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-193.9682539682539</v>
+        <v>-209.8412698412698</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>2285.714285714286</v>
+        <v>2428.571428571428</v>
       </c>
       <c r="R20" s="117" t="n">
         <v>540</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-1745.714285714286</v>
+        <v>-1888.571428571428</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.76375</v>
+        <v>-0.7776470588235294</v>
       </c>
       <c r="U20" s="117" t="n">
         <v>9</v>
@@ -2213,28 +2213,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>95.23809523809524</v>
+        <v>101.1904761904762</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-50.23809523809524</v>
+        <v>-56.19047619047619</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>761.9047619047619</v>
+        <v>809.5238095238095</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>360</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-401.9047619047619</v>
+        <v>-449.5238095238095</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.5275</v>
+        <v>-0.5552941176470588</v>
       </c>
       <c r="U21" s="117" t="n">
         <v>8</v>
@@ -2276,28 +2276,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>800.3341687552214</v>
+        <v>850.3550543024228</v>
       </c>
       <c r="N22" s="125" t="n">
         <v>198</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-602.3341687552214</v>
+        <v>-652.3550543024228</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="Q22" s="123" t="n">
-        <v>6476.190476190476</v>
+        <v>6880.952380952381</v>
       </c>
       <c r="R22" s="123" t="n">
         <v>1606.8</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-4869.390476190476</v>
+        <v>-5274.152380952381</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-0.7518911764705882</v>
+        <v>-0.7664858131487889</v>
       </c>
       <c r="U22" s="123" t="n">
         <v>8.115151515151515</v>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>1647.903189842231</v>
+        <v>1733.239451268058</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-1167.903189842231</v>
+        <v>-1253.239451268058</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>33185.86789554531</v>
+        <v>34703.53302611367</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>26894.167266</v>
+        <v>28125.039233</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-6291.700629545314</v>
+        <v>-6578.49379311367</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1895897569817626</v>
+        <v>-0.1895626531213261</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>56.0295151375</v>
+        <v>58.59383173541666</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>35.98490654846242</v>
+        <v>38.54922314637908</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>6193.548387096775</v>
+        <v>6451.612903225807</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>6256.285785</v>
+        <v>6551.493881</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>62.73739790322543</v>
+        <v>99.88097777419352</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0101294757031249</v>
+        <v>0.0154815515549999</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>774.1935483870968</v>
+        <v>806.4516129032259</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>747.771898</v>
+        <v>801.896588</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>-26.42165038709686</v>
+        <v>-4.555024903225899</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>-0.0341279650833334</v>
+        <v>-0.0056482308800001</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>7354.838709677419</v>
+        <v>7661.290322580645</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>6708.89</v>
+        <v>7066.75</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-645.9487096774183</v>
+        <v>-594.5403225806449</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0878263596491226</v>
+        <v>-0.0776031578947368</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2933,28 +2933,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>451.1278195488723</v>
+        <v>479.3233082706768</v>
       </c>
       <c r="R5" t="n">
         <v>93</v>
       </c>
       <c r="S5" t="n">
-        <v>-358.1278195488723</v>
+        <v>-386.3233082706768</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="U5" s="135" t="n">
-        <v>3428.571428571428</v>
+        <v>3642.857142857143</v>
       </c>
       <c r="V5" s="135" t="n">
         <v>706.8</v>
       </c>
       <c r="W5" s="135" t="n">
-        <v>-2721.771428571428</v>
+        <v>-2936.057142857143</v>
       </c>
       <c r="X5" s="136" t="n">
-        <v>-0.7938499999999999</v>
+        <v>-0.8059764705882354</v>
       </c>
       <c r="Y5" s="135" t="n">
         <v>7.6</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3036,28 +3036,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>253.9682539682539</v>
+        <v>269.8412698412698</v>
       </c>
       <c r="R6" t="n">
         <v>60</v>
       </c>
       <c r="S6" t="n">
-        <v>-193.9682539682539</v>
+        <v>-209.8412698412698</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>2285.714285714286</v>
+        <v>2428.571428571428</v>
       </c>
       <c r="V6" s="135" t="n">
         <v>540</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-1745.714285714286</v>
+        <v>-1888.571428571428</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.76375</v>
+        <v>-0.7776470588235294</v>
       </c>
       <c r="Y6" s="135" t="n">
         <v>9</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3139,28 +3139,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>95.23809523809524</v>
+        <v>101.1904761904762</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>-50.23809523809524</v>
+        <v>-56.19047619047619</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>761.9047619047619</v>
+        <v>809.5238095238095</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>360</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>-401.9047619047619</v>
+        <v>-449.5238095238095</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>-0.5275</v>
+        <v>-0.5552941176470588</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>8</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>49.94797086368366</v>
+        <v>52.02913631633714</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-27.94797086368366</v>
+        <v>-30.02913631633714</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>1548.387096774194</v>
+        <v>1612.903225806452</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>1470.519531</v>
+        <v>1525.409531</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>-77.86756577419374</v>
+        <v>-87.49369480645169</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>-0.0502894695625001</v>
+        <v>-0.05424609078</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>66.84179686363636</v>
+        <v>69.33679686363637</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>35.84179686363636</v>
+        <v>38.33679686363637</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>83.69659982563209</v>
+        <v>87.1839581517001</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-63.69659982563209</v>
+        <v>-67.1839581517001</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>3096.774193548388</v>
+        <v>3225.806451612903</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>3079.972742</v>
+        <v>3248.620991</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>-16.80145154838738</v>
+        <v>22.81453938709637</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>-0.0054254687291667</v>
+        <v>0.0070725072099998</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>153.9986371</v>
+        <v>162.43104955</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>116.9986371</v>
+        <v>125.43104955</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>6.67408231368187</v>
+        <v>6.952169076751948</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-4.67408231368187</v>
+        <v>-4.952169076751948</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>387.0967741935484</v>
+        <v>403.2258064516129</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>408.723321</v>
+        <v>415.854922</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>21.62654680645158</v>
+        <v>12.62911554838706</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0558685792499999</v>
+        <v>0.0313202065599999</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>204.3616605</v>
+        <v>207.927461</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>146.3616605</v>
+        <v>149.927461</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,34 +3563,34 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>2.419354838709677</v>
+        <v>2.520161290322581</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-1.419354838709677</v>
+        <v>-1.52016129032258</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>387.0967741935484</v>
+        <v>403.2258064516129</v>
       </c>
       <c r="V11" s="135" t="n">
-        <v>157.606346</v>
+        <v>162.246346</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-229.4904281935484</v>
+        <v>-240.9794604516129</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.5928502728333334</v>
+        <v>-0.5976290619200001</v>
       </c>
       <c r="Y11" s="135" t="n">
-        <v>157.606346</v>
+        <v>162.246346</v>
       </c>
       <c r="Z11" s="135" t="n">
-        <v>-2.393653999999998</v>
+        <v>2.246345999999988</v>
       </c>
       <c r="AB11" s="137" t="inlineStr">
         <is>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>224.1086587436333</v>
+        <v>233.446519524618</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-132.1086587436333</v>
+        <v>-141.446519524618</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>4258.064516129032</v>
+        <v>4435.483870967741</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>4191.87</v>
+        <v>4374.49</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>-66.19451612903231</v>
+        <v>-60.99387096774171</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>-0.0155456818181818</v>
+        <v>-0.0137513454545454</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>45.56380434782609</v>
+        <v>47.54880434782608</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>26.56380434782609</v>
+        <v>28.54880434782608</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>12.90322580645162</v>
+        <v>13.44086021505377</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>-5.903225806451616</v>
+        <v>-6.440860215053766</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>387.0967741935484</v>
+        <v>403.2258064516129</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>241.84</v>
+        <v>257.34</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-145.2567741935484</v>
+        <v>-145.885806451613</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3752466666666667</v>
+        <v>-0.3617968000000001</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>34.54857142857143</v>
+        <v>36.76285714285714</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>4.548571428571428</v>
+        <v>6.762857142857136</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.301075268817204</v>
+        <v>4.480286738351254</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-4.301075268817204</v>
+        <v>-4.480286738351254</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>387.0967741935484</v>
+        <v>403.2258064516129</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>240.37</v>
+        <v>253.32</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-146.7267741935484</v>
+        <v>-149.9058064516129</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3790441666666667</v>
+        <v>-0.3717664</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>96.7741935483871</v>
+        <v>100.8064516129032</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-77.7741935483871</v>
+        <v>-81.80645161290323</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>1161.290322580645</v>
+        <v>1209.677419354839</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>1074.657643</v>
+        <v>1118.466974</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>-86.63267958064534</v>
+        <v>-91.21044535483884</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>-0.07460036297222231</v>
+        <v>-0.0754006348266667</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>56.56092857894737</v>
+        <v>58.86668284210526</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>44.56092857894737</v>
+        <v>46.86668284210526</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>33.66058906030855</v>
+        <v>35.06311360448808</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-30.66058906030856</v>
+        <v>-32.06311360448808</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>774.1935483870968</v>
+        <v>806.4516129032259</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>708.86</v>
+        <v>742.35</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-65.33354838709681</v>
+        <v>-64.10161290322583</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.0843891666666667</v>
+        <v>-0.079486</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>236.2866666666666</v>
+        <v>247.45</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>213.2866666666666</v>
+        <v>224.45</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>333.0832708177044</v>
+        <v>346.9617404351088</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-217.0832708177044</v>
+        <v>-230.9617404351088</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>14322.58064516129</v>
+        <v>14919.35483870968</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>13712.947683</v>
+        <v>14420.140469</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-609.6329621612895</v>
+        <v>-499.2143697096781</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0425644635743242</v>
+        <v>-0.0334608550508108</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>118.2150662327586</v>
+        <v>124.3115557672414</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>75.21506623275863</v>
+        <v>81.31155576724137</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>514.4857502693051</v>
+        <v>535.9226565305261</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-348.4857502693051</v>
+        <v>-369.9226565305261</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>12387.09677419355</v>
+        <v>12903.22580645161</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>11574.419583</v>
+        <v>12098.098764</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>-812.6771911935502</v>
+        <v>-805.1270424516133</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>-0.06560675241406259</v>
+        <v>-0.06239734579</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>69.72541917469879</v>
+        <v>72.88011303614458</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>45.64876249818329</v>
+        <v>48.80345635962908</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4350,28 +4350,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>800.3341687552214</v>
+        <v>850.3550543024228</v>
       </c>
       <c r="R19" t="n">
         <v>198</v>
       </c>
       <c r="S19" t="n">
-        <v>-602.3341687552214</v>
+        <v>-652.3550543024228</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>6476.190476190476</v>
+        <v>6880.952380952381</v>
       </c>
       <c r="V19" s="135" t="n">
         <v>1606.8</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-4869.390476190476</v>
+        <v>-5274.152380952381</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.7518911764705882</v>
+        <v>-0.7664858131487889</v>
       </c>
       <c r="Y19" s="135" t="n">
         <v>8.115151515151515</v>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>1647.903189842231</v>
+        <v>1733.239451268058</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-1167.903189842231</v>
+        <v>-1253.239451268058</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>33185.86789554531</v>
+        <v>34703.53302611367</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>26894.167266</v>
+        <v>28125.039233</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-6291.700629545314</v>
+        <v>-6578.49379311367</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1895897569817626</v>
+        <v>-0.1895626531213261</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>56.0295151375</v>
+        <v>58.59383173541666</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>35.98490654846242</v>
+        <v>38.54922314637908</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46259.291875</v>
+        <v>46260.29199074074</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-27
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 25/08/2026  |  Ultimo aggiornamento: 26/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 26/08/2026  |  Ultimo aggiornamento: 27/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>6451.612903225807</v>
+        <v>6709.677419354839</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>6551.493881</v>
+        <v>6829.212182</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>99.88097777419352</v>
+        <v>119.5347626451612</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0154815515549999</v>
+        <v>0.0178152771249999</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>806.4516129032259</v>
+        <v>838.7096774193549</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>801.896588</v>
+        <v>827.4065880000001</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>-4.555024903225899</v>
+        <v>-11.30308941935482</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>-0.0056482308800001</v>
+        <v>-0.0134767604615384</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>7661.290322580645</v>
+        <v>7967.74193548387</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>7066.75</v>
+        <v>7373.94</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-594.5403225806449</v>
+        <v>-593.8019354838707</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0776031578947368</v>
+        <v>-0.0745257489878542</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>346.9617404351088</v>
+        <v>360.8402100525131</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-230.9617404351088</v>
+        <v>-244.8402100525131</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>14919.35483870968</v>
+        <v>15516.12903225806</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>14420.140469</v>
+        <v>15030.55877</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-499.2143697096781</v>
+        <v>-485.5702622580648</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0334608550508108</v>
+        <v>-0.0312945491268191</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>124.3115557672414</v>
+        <v>129.5737825</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>81.31155576724137</v>
+        <v>86.57378249999999</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>52.02913631633714</v>
+        <v>54.11030176899063</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-30.02913631633714</v>
+        <v>-32.11030176899063</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>1612.903225806452</v>
+        <v>1677.41935483871</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>1525.409531</v>
+        <v>1587.540775</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-87.49369480645169</v>
+        <v>-89.87857983870981</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.05424609078</v>
+        <v>-0.0535814610576923</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>69.33679686363637</v>
+        <v>72.16094431818182</v>
       </c>
       <c r="V9" s="117" t="n">
-        <v>38.33679686363637</v>
+        <v>41.16094431818182</v>
       </c>
       <c r="W9" s="120" t="inlineStr"/>
     </row>
@@ -1382,34 +1382,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="M10" s="119" t="n">
-        <v>87.1839581517001</v>
+        <v>90.6713164777681</v>
       </c>
       <c r="N10" s="119" t="n">
         <v>20</v>
       </c>
       <c r="O10" s="119" t="n">
-        <v>-67.1839581517001</v>
+        <v>-70.6713164777681</v>
       </c>
       <c r="P10" s="117" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="Q10" s="117" t="n">
-        <v>3225.806451612903</v>
+        <v>3354.83870967742</v>
       </c>
       <c r="R10" s="117" t="n">
-        <v>3248.620991</v>
+        <v>3370.446577</v>
       </c>
       <c r="S10" s="117" t="n">
-        <v>22.81453938709637</v>
+        <v>15.60786732258066</v>
       </c>
       <c r="T10" s="118" t="n">
-        <v>0.0070725072099998</v>
+        <v>0.0046523450673076</v>
       </c>
       <c r="U10" s="117" t="n">
-        <v>162.43104955</v>
+        <v>168.52232885</v>
       </c>
       <c r="V10" s="117" t="n">
-        <v>125.43104955</v>
+        <v>131.52232885</v>
       </c>
       <c r="W10" s="120" t="inlineStr"/>
     </row>
@@ -1461,34 +1461,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="M11" s="119" t="n">
-        <v>6.952169076751948</v>
+        <v>7.230255839822026</v>
       </c>
       <c r="N11" s="119" t="n">
         <v>2</v>
       </c>
       <c r="O11" s="119" t="n">
-        <v>-4.952169076751948</v>
+        <v>-5.230255839822026</v>
       </c>
       <c r="P11" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q11" s="117" t="n">
-        <v>403.2258064516129</v>
+        <v>419.3548387096774</v>
       </c>
       <c r="R11" s="117" t="n">
-        <v>415.854922</v>
+        <v>424.445841</v>
       </c>
       <c r="S11" s="117" t="n">
-        <v>12.62911554838706</v>
+        <v>5.091002290322535</v>
       </c>
       <c r="T11" s="118" t="n">
-        <v>0.0313202065599999</v>
+        <v>0.0121400823846152</v>
       </c>
       <c r="U11" s="117" t="n">
-        <v>207.927461</v>
+        <v>212.2229205</v>
       </c>
       <c r="V11" s="117" t="n">
-        <v>149.927461</v>
+        <v>154.2229205</v>
       </c>
       <c r="W11" s="120" t="inlineStr"/>
     </row>
@@ -1540,28 +1540,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="M12" s="119" t="n">
-        <v>2.520161290322581</v>
+        <v>2.620967741935484</v>
       </c>
       <c r="N12" s="119" t="n">
         <v>1</v>
       </c>
       <c r="O12" s="119" t="n">
-        <v>-1.52016129032258</v>
+        <v>-1.620967741935484</v>
       </c>
       <c r="P12" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q12" s="117" t="n">
-        <v>403.2258064516129</v>
+        <v>419.3548387096774</v>
       </c>
       <c r="R12" s="117" t="n">
         <v>162.246346</v>
       </c>
       <c r="S12" s="117" t="n">
-        <v>-240.9794604516129</v>
+        <v>-257.1084927096774</v>
       </c>
       <c r="T12" s="118" t="n">
-        <v>-0.5976290619200001</v>
+        <v>-0.6131048672307692</v>
       </c>
       <c r="U12" s="117" t="n">
         <v>162.246346</v>
@@ -1619,34 +1619,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="M13" s="119" t="n">
-        <v>233.446519524618</v>
+        <v>242.7843803056027</v>
       </c>
       <c r="N13" s="119" t="n">
         <v>92</v>
       </c>
       <c r="O13" s="119" t="n">
-        <v>-141.446519524618</v>
+        <v>-150.7843803056027</v>
       </c>
       <c r="P13" s="117" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="Q13" s="117" t="n">
-        <v>4435.483870967741</v>
+        <v>4612.903225806452</v>
       </c>
       <c r="R13" s="117" t="n">
-        <v>4374.49</v>
+        <v>4548.58</v>
       </c>
       <c r="S13" s="117" t="n">
-        <v>-60.99387096774171</v>
+        <v>-64.32322580645177</v>
       </c>
       <c r="T13" s="118" t="n">
-        <v>-0.0137513454545454</v>
+        <v>-0.0139441958041958</v>
       </c>
       <c r="U13" s="117" t="n">
-        <v>47.54880434782608</v>
+        <v>49.44108695652174</v>
       </c>
       <c r="V13" s="117" t="n">
-        <v>28.54880434782608</v>
+        <v>30.44108695652174</v>
       </c>
       <c r="W13" s="120" t="inlineStr"/>
     </row>
@@ -1698,34 +1698,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="M14" s="119" t="n">
-        <v>13.44086021505377</v>
+        <v>13.97849462365592</v>
       </c>
       <c r="N14" s="119" t="n">
         <v>7</v>
       </c>
       <c r="O14" s="119" t="n">
-        <v>-6.440860215053766</v>
+        <v>-6.978494623655916</v>
       </c>
       <c r="P14" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q14" s="117" t="n">
-        <v>403.2258064516129</v>
+        <v>419.3548387096774</v>
       </c>
       <c r="R14" s="117" t="n">
-        <v>257.34</v>
+        <v>273.62</v>
       </c>
       <c r="S14" s="117" t="n">
-        <v>-145.885806451613</v>
+        <v>-145.7348387096774</v>
       </c>
       <c r="T14" s="118" t="n">
-        <v>-0.3617968000000001</v>
+        <v>-0.3475215384615385</v>
       </c>
       <c r="U14" s="117" t="n">
-        <v>36.76285714285714</v>
+        <v>39.08857142857143</v>
       </c>
       <c r="V14" s="117" t="n">
-        <v>6.762857142857136</v>
+        <v>9.088571428571427</v>
       </c>
       <c r="W14" s="120" t="inlineStr"/>
     </row>
@@ -1775,28 +1775,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="M15" s="119" t="n">
-        <v>4.480286738351254</v>
+        <v>4.659498207885305</v>
       </c>
       <c r="N15" s="119" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="119" t="n">
-        <v>-4.480286738351254</v>
+        <v>-4.659498207885305</v>
       </c>
       <c r="P15" s="117" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="Q15" s="117" t="n">
-        <v>403.2258064516129</v>
+        <v>419.3548387096774</v>
       </c>
       <c r="R15" s="117" t="n">
-        <v>253.32</v>
+        <v>267.62</v>
       </c>
       <c r="S15" s="117" t="n">
-        <v>-149.9058064516129</v>
+        <v>-151.7348387096774</v>
       </c>
       <c r="T15" s="118" t="n">
-        <v>-0.3717664</v>
+        <v>-0.3618292307692308</v>
       </c>
       <c r="U15" s="117" t="n"/>
       <c r="V15" s="117" t="n"/>
@@ -1850,34 +1850,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="M16" s="119" t="n">
-        <v>100.8064516129032</v>
+        <v>104.8387096774194</v>
       </c>
       <c r="N16" s="119" t="n">
         <v>19</v>
       </c>
       <c r="O16" s="119" t="n">
-        <v>-81.80645161290323</v>
+        <v>-85.83870967741936</v>
       </c>
       <c r="P16" s="117" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="Q16" s="117" t="n">
-        <v>1209.677419354839</v>
+        <v>1258.064516129032</v>
       </c>
       <c r="R16" s="117" t="n">
-        <v>1118.466974</v>
+        <v>1157.024833</v>
       </c>
       <c r="S16" s="117" t="n">
-        <v>-91.21044535483884</v>
+        <v>-101.0396831290325</v>
       </c>
       <c r="T16" s="118" t="n">
-        <v>-0.0754006348266667</v>
+        <v>-0.0803135942820514</v>
       </c>
       <c r="U16" s="117" t="n">
-        <v>58.86668284210526</v>
+        <v>60.89604384210526</v>
       </c>
       <c r="V16" s="117" t="n">
-        <v>46.86668284210526</v>
+        <v>48.89604384210526</v>
       </c>
       <c r="W16" s="120" t="inlineStr"/>
     </row>
@@ -1925,34 +1925,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="M17" s="119" t="n">
-        <v>35.06311360448808</v>
+        <v>36.4656381486676</v>
       </c>
       <c r="N17" s="119" t="n">
         <v>3</v>
       </c>
       <c r="O17" s="119" t="n">
-        <v>-32.06311360448808</v>
+        <v>-33.4656381486676</v>
       </c>
       <c r="P17" s="117" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="Q17" s="117" t="n">
-        <v>806.4516129032259</v>
+        <v>838.7096774193549</v>
       </c>
       <c r="R17" s="117" t="n">
-        <v>742.35</v>
+        <v>772.61</v>
       </c>
       <c r="S17" s="117" t="n">
-        <v>-64.10161290322583</v>
+        <v>-66.09967741935486</v>
       </c>
       <c r="T17" s="118" t="n">
-        <v>-0.079486</v>
+        <v>-0.07881115384615379</v>
       </c>
       <c r="U17" s="117" t="n">
-        <v>247.45</v>
+        <v>257.5366666666667</v>
       </c>
       <c r="V17" s="117" t="n">
-        <v>224.45</v>
+        <v>234.5366666666667</v>
       </c>
       <c r="W17" s="120" t="inlineStr"/>
     </row>
@@ -1988,34 +1988,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="M18" s="125" t="n">
-        <v>535.9226565305261</v>
+        <v>557.3595627917472</v>
       </c>
       <c r="N18" s="125" t="n">
         <v>166</v>
       </c>
       <c r="O18" s="125" t="n">
-        <v>-369.9226565305261</v>
+        <v>-391.3595627917472</v>
       </c>
       <c r="P18" s="123" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="Q18" s="123" t="n">
-        <v>12903.22580645161</v>
+        <v>13419.35483870968</v>
       </c>
       <c r="R18" s="123" t="n">
-        <v>12098.098764</v>
+        <v>12564.134372</v>
       </c>
       <c r="S18" s="123" t="n">
-        <v>-805.1270424516133</v>
+        <v>-855.2204667096776</v>
       </c>
       <c r="T18" s="124" t="n">
-        <v>-0.06239734579</v>
+        <v>-0.0637303713173077</v>
       </c>
       <c r="U18" s="123" t="n">
-        <v>72.88011303614458</v>
+        <v>75.68755645783133</v>
       </c>
       <c r="V18" s="123" t="n">
-        <v>48.80345635962908</v>
+        <v>51.61089978131584</v>
       </c>
       <c r="W18" s="126" t="n"/>
     </row>
@@ -2063,28 +2063,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="M19" s="119" t="n">
-        <v>479.3233082706768</v>
+        <v>507.5187969924813</v>
       </c>
       <c r="N19" s="119" t="n">
         <v>93</v>
       </c>
       <c r="O19" s="119" t="n">
-        <v>-386.3233082706768</v>
+        <v>-414.5187969924813</v>
       </c>
       <c r="P19" s="117" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="Q19" s="117" t="n">
-        <v>3642.857142857143</v>
+        <v>3857.142857142857</v>
       </c>
       <c r="R19" s="117" t="n">
         <v>706.8</v>
       </c>
       <c r="S19" s="117" t="n">
-        <v>-2936.057142857143</v>
+        <v>-3150.342857142857</v>
       </c>
       <c r="T19" s="118" t="n">
-        <v>-0.8059764705882354</v>
+        <v>-0.8167555555555555</v>
       </c>
       <c r="U19" s="117" t="n">
         <v>7.6</v>
@@ -2138,28 +2138,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="M20" s="119" t="n">
-        <v>269.8412698412698</v>
+        <v>285.7142857142857</v>
       </c>
       <c r="N20" s="119" t="n">
         <v>60</v>
       </c>
       <c r="O20" s="119" t="n">
-        <v>-209.8412698412698</v>
+        <v>-225.7142857142857</v>
       </c>
       <c r="P20" s="117" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="Q20" s="117" t="n">
-        <v>2428.571428571428</v>
+        <v>2571.428571428572</v>
       </c>
       <c r="R20" s="117" t="n">
         <v>540</v>
       </c>
       <c r="S20" s="117" t="n">
-        <v>-1888.571428571428</v>
+        <v>-2031.428571428572</v>
       </c>
       <c r="T20" s="118" t="n">
-        <v>-0.7776470588235294</v>
+        <v>-0.79</v>
       </c>
       <c r="U20" s="117" t="n">
         <v>9</v>
@@ -2213,28 +2213,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="M21" s="119" t="n">
-        <v>101.1904761904762</v>
+        <v>107.1428571428571</v>
       </c>
       <c r="N21" s="119" t="n">
         <v>45</v>
       </c>
       <c r="O21" s="119" t="n">
-        <v>-56.19047619047619</v>
+        <v>-62.14285714285714</v>
       </c>
       <c r="P21" s="117" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="Q21" s="117" t="n">
-        <v>809.5238095238095</v>
+        <v>857.1428571428571</v>
       </c>
       <c r="R21" s="117" t="n">
         <v>360</v>
       </c>
       <c r="S21" s="117" t="n">
-        <v>-449.5238095238095</v>
+        <v>-497.1428571428571</v>
       </c>
       <c r="T21" s="118" t="n">
-        <v>-0.5552941176470588</v>
+        <v>-0.58</v>
       </c>
       <c r="U21" s="117" t="n">
         <v>8</v>
@@ -2276,28 +2276,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="M22" s="125" t="n">
-        <v>850.3550543024228</v>
+        <v>900.375939849624</v>
       </c>
       <c r="N22" s="125" t="n">
         <v>198</v>
       </c>
       <c r="O22" s="125" t="n">
-        <v>-652.3550543024228</v>
+        <v>-702.375939849624</v>
       </c>
       <c r="P22" s="123" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="Q22" s="123" t="n">
-        <v>6880.952380952381</v>
+        <v>7285.714285714285</v>
       </c>
       <c r="R22" s="123" t="n">
         <v>1606.8</v>
       </c>
       <c r="S22" s="123" t="n">
-        <v>-5274.152380952381</v>
+        <v>-5678.914285714285</v>
       </c>
       <c r="T22" s="124" t="n">
-        <v>-0.7664858131487889</v>
+        <v>-0.7794588235294118</v>
       </c>
       <c r="U22" s="123" t="n">
         <v>8.115151515151515</v>
@@ -2339,34 +2339,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="M23" s="131" t="n">
-        <v>1733.239451268058</v>
+        <v>1818.575712693884</v>
       </c>
       <c r="N23" s="131" t="n">
         <v>480</v>
       </c>
       <c r="O23" s="131" t="n">
-        <v>-1253.239451268058</v>
+        <v>-1338.575712693884</v>
       </c>
       <c r="P23" s="129" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="Q23" s="129" t="n">
-        <v>34703.53302611367</v>
+        <v>36221.19815668203</v>
       </c>
       <c r="R23" s="129" t="n">
-        <v>28125.039233</v>
+        <v>29201.493142</v>
       </c>
       <c r="S23" s="129" t="n">
-        <v>-6578.49379311367</v>
+        <v>-7019.705014682026</v>
       </c>
       <c r="T23" s="130" t="n">
-        <v>-0.1895626531213261</v>
+        <v>-0.1938010163086513</v>
       </c>
       <c r="U23" s="129" t="n">
-        <v>58.59383173541666</v>
+        <v>60.83644404583333</v>
       </c>
       <c r="V23" s="129" t="n">
-        <v>38.54922314637908</v>
+        <v>40.79183545679575</v>
       </c>
       <c r="W23" s="132" t="n"/>
     </row>
@@ -2637,13 +2637,13 @@
         </is>
       </c>
       <c r="B2" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C2" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D2" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -2680,16 +2680,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="U2" s="135" t="n">
-        <v>6451.612903225807</v>
+        <v>6709.677419354839</v>
       </c>
       <c r="V2" s="135" t="n">
-        <v>6551.493881</v>
+        <v>6829.212182</v>
       </c>
       <c r="W2" s="135" t="n">
-        <v>99.88097777419352</v>
+        <v>119.5347626451612</v>
       </c>
       <c r="X2" s="136" t="n">
-        <v>0.0154815515549999</v>
+        <v>0.0178152771249999</v>
       </c>
       <c r="Y2" s="135" t="n"/>
       <c r="Z2" s="135" t="n"/>
@@ -2718,13 +2718,13 @@
         </is>
       </c>
       <c r="B3" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C3" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D3" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E3" t="n">
         <v>3</v>
@@ -2761,16 +2761,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="U3" s="135" t="n">
-        <v>806.4516129032259</v>
+        <v>838.7096774193549</v>
       </c>
       <c r="V3" s="135" t="n">
-        <v>801.896588</v>
+        <v>827.4065880000001</v>
       </c>
       <c r="W3" s="135" t="n">
-        <v>-4.555024903225899</v>
+        <v>-11.30308941935482</v>
       </c>
       <c r="X3" s="136" t="n">
-        <v>-0.0056482308800001</v>
+        <v>-0.0134767604615384</v>
       </c>
       <c r="Y3" s="135" t="n"/>
       <c r="Z3" s="135" t="n"/>
@@ -2799,13 +2799,13 @@
         </is>
       </c>
       <c r="B4" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C4" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D4" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E4" t="n">
         <v>4</v>
@@ -2842,16 +2842,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="U4" s="135" t="n">
-        <v>7661.290322580645</v>
+        <v>7967.74193548387</v>
       </c>
       <c r="V4" s="135" t="n">
-        <v>7066.75</v>
+        <v>7373.94</v>
       </c>
       <c r="W4" s="135" t="n">
-        <v>-594.5403225806449</v>
+        <v>-593.8019354838707</v>
       </c>
       <c r="X4" s="136" t="n">
-        <v>-0.0776031578947368</v>
+        <v>-0.0745257489878542</v>
       </c>
       <c r="Y4" s="135" t="n"/>
       <c r="Z4" s="135" t="n"/>
@@ -2880,13 +2880,13 @@
         </is>
       </c>
       <c r="B5" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C5" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D5" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E5" t="n">
         <v>16</v>
@@ -2933,28 +2933,28 @@
         <v>28.19548872180452</v>
       </c>
       <c r="Q5" t="n">
-        <v>479.3233082706768</v>
+        <v>507.5187969924813</v>
       </c>
       <c r="R5" t="n">
         <v>93</v>
       </c>
       <c r="S5" t="n">
-        <v>-386.3233082706768</v>
+        <v>-414.5187969924813</v>
       </c>
       <c r="T5" s="135" t="n">
         <v>214.2857142857143</v>
       </c>
       <c r="U5" s="135" t="n">
-        <v>3642.857142857143</v>
+        <v>3857.142857142857</v>
       </c>
       <c r="V5" s="135" t="n">
         <v>706.8</v>
       </c>
       <c r="W5" s="135" t="n">
-        <v>-2936.057142857143</v>
+        <v>-3150.342857142857</v>
       </c>
       <c r="X5" s="136" t="n">
-        <v>-0.8059764705882354</v>
+        <v>-0.8167555555555555</v>
       </c>
       <c r="Y5" s="135" t="n">
         <v>7.6</v>
@@ -2983,13 +2983,13 @@
         </is>
       </c>
       <c r="B6" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C6" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D6" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E6" t="n">
         <v>17</v>
@@ -3036,28 +3036,28 @@
         <v>15.87301587301587</v>
       </c>
       <c r="Q6" t="n">
-        <v>269.8412698412698</v>
+        <v>285.7142857142857</v>
       </c>
       <c r="R6" t="n">
         <v>60</v>
       </c>
       <c r="S6" t="n">
-        <v>-209.8412698412698</v>
+        <v>-225.7142857142857</v>
       </c>
       <c r="T6" s="135" t="n">
         <v>142.8571428571429</v>
       </c>
       <c r="U6" s="135" t="n">
-        <v>2428.571428571428</v>
+        <v>2571.428571428572</v>
       </c>
       <c r="V6" s="135" t="n">
         <v>540</v>
       </c>
       <c r="W6" s="135" t="n">
-        <v>-1888.571428571428</v>
+        <v>-2031.428571428572</v>
       </c>
       <c r="X6" s="136" t="n">
-        <v>-0.7776470588235294</v>
+        <v>-0.79</v>
       </c>
       <c r="Y6" s="135" t="n">
         <v>9</v>
@@ -3086,13 +3086,13 @@
         </is>
       </c>
       <c r="B7" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C7" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D7" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
@@ -3139,28 +3139,28 @@
         <v>5.952380952380953</v>
       </c>
       <c r="Q7" t="n">
-        <v>101.1904761904762</v>
+        <v>107.1428571428571</v>
       </c>
       <c r="R7" t="n">
         <v>45</v>
       </c>
       <c r="S7" t="n">
-        <v>-56.19047619047619</v>
+        <v>-62.14285714285714</v>
       </c>
       <c r="T7" s="135" t="n">
         <v>47.61904761904762</v>
       </c>
       <c r="U7" s="135" t="n">
-        <v>809.5238095238095</v>
+        <v>857.1428571428571</v>
       </c>
       <c r="V7" s="135" t="n">
         <v>360</v>
       </c>
       <c r="W7" s="135" t="n">
-        <v>-449.5238095238095</v>
+        <v>-497.1428571428571</v>
       </c>
       <c r="X7" s="136" t="n">
-        <v>-0.5552941176470588</v>
+        <v>-0.58</v>
       </c>
       <c r="Y7" s="135" t="n">
         <v>8</v>
@@ -3189,13 +3189,13 @@
         </is>
       </c>
       <c r="B8" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C8" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D8" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -3242,34 +3242,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="Q8" t="n">
-        <v>52.02913631633714</v>
+        <v>54.11030176899063</v>
       </c>
       <c r="R8" t="n">
         <v>22</v>
       </c>
       <c r="S8" t="n">
-        <v>-30.02913631633714</v>
+        <v>-32.11030176899063</v>
       </c>
       <c r="T8" s="135" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="U8" s="135" t="n">
-        <v>1612.903225806452</v>
+        <v>1677.41935483871</v>
       </c>
       <c r="V8" s="135" t="n">
-        <v>1525.409531</v>
+        <v>1587.540775</v>
       </c>
       <c r="W8" s="135" t="n">
-        <v>-87.49369480645169</v>
+        <v>-89.87857983870981</v>
       </c>
       <c r="X8" s="136" t="n">
-        <v>-0.05424609078</v>
+        <v>-0.0535814610576923</v>
       </c>
       <c r="Y8" s="135" t="n">
-        <v>69.33679686363637</v>
+        <v>72.16094431818182</v>
       </c>
       <c r="Z8" s="135" t="n">
-        <v>38.33679686363637</v>
+        <v>41.16094431818182</v>
       </c>
       <c r="AB8" s="137" t="inlineStr">
         <is>
@@ -3296,13 +3296,13 @@
         </is>
       </c>
       <c r="B9" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C9" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D9" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -3349,34 +3349,34 @@
         <v>3.487358326068004</v>
       </c>
       <c r="Q9" t="n">
-        <v>87.1839581517001</v>
+        <v>90.6713164777681</v>
       </c>
       <c r="R9" t="n">
         <v>20</v>
       </c>
       <c r="S9" t="n">
-        <v>-67.1839581517001</v>
+        <v>-70.6713164777681</v>
       </c>
       <c r="T9" s="135" t="n">
         <v>129.0322580645161</v>
       </c>
       <c r="U9" s="135" t="n">
-        <v>3225.806451612903</v>
+        <v>3354.83870967742</v>
       </c>
       <c r="V9" s="135" t="n">
-        <v>3248.620991</v>
+        <v>3370.446577</v>
       </c>
       <c r="W9" s="135" t="n">
-        <v>22.81453938709637</v>
+        <v>15.60786732258066</v>
       </c>
       <c r="X9" s="136" t="n">
-        <v>0.0070725072099998</v>
+        <v>0.0046523450673076</v>
       </c>
       <c r="Y9" s="135" t="n">
-        <v>162.43104955</v>
+        <v>168.52232885</v>
       </c>
       <c r="Z9" s="135" t="n">
-        <v>125.43104955</v>
+        <v>131.52232885</v>
       </c>
       <c r="AB9" s="137" t="inlineStr">
         <is>
@@ -3403,13 +3403,13 @@
         </is>
       </c>
       <c r="B10" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C10" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D10" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -3456,34 +3456,34 @@
         <v>0.2780867630700779</v>
       </c>
       <c r="Q10" t="n">
-        <v>6.952169076751948</v>
+        <v>7.230255839822026</v>
       </c>
       <c r="R10" t="n">
         <v>2</v>
       </c>
       <c r="S10" t="n">
-        <v>-4.952169076751948</v>
+        <v>-5.230255839822026</v>
       </c>
       <c r="T10" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U10" s="135" t="n">
-        <v>403.2258064516129</v>
+        <v>419.3548387096774</v>
       </c>
       <c r="V10" s="135" t="n">
-        <v>415.854922</v>
+        <v>424.445841</v>
       </c>
       <c r="W10" s="135" t="n">
-        <v>12.62911554838706</v>
+        <v>5.091002290322535</v>
       </c>
       <c r="X10" s="136" t="n">
-        <v>0.0313202065599999</v>
+        <v>0.0121400823846152</v>
       </c>
       <c r="Y10" s="135" t="n">
-        <v>207.927461</v>
+        <v>212.2229205</v>
       </c>
       <c r="Z10" s="135" t="n">
-        <v>149.927461</v>
+        <v>154.2229205</v>
       </c>
       <c r="AB10" s="137" t="inlineStr">
         <is>
@@ -3510,13 +3510,13 @@
         </is>
       </c>
       <c r="B11" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C11" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D11" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -3563,28 +3563,28 @@
         <v>0.1008064516129032</v>
       </c>
       <c r="Q11" t="n">
-        <v>2.520161290322581</v>
+        <v>2.620967741935484</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>-1.52016129032258</v>
+        <v>-1.620967741935484</v>
       </c>
       <c r="T11" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U11" s="135" t="n">
-        <v>403.2258064516129</v>
+        <v>419.3548387096774</v>
       </c>
       <c r="V11" s="135" t="n">
         <v>162.246346</v>
       </c>
       <c r="W11" s="135" t="n">
-        <v>-240.9794604516129</v>
+        <v>-257.1084927096774</v>
       </c>
       <c r="X11" s="136" t="n">
-        <v>-0.5976290619200001</v>
+        <v>-0.6131048672307692</v>
       </c>
       <c r="Y11" s="135" t="n">
         <v>162.246346</v>
@@ -3617,13 +3617,13 @@
         </is>
       </c>
       <c r="B12" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C12" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D12" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E12" t="n">
         <v>11</v>
@@ -3670,34 +3670,34 @@
         <v>9.33786078098472</v>
       </c>
       <c r="Q12" t="n">
-        <v>233.446519524618</v>
+        <v>242.7843803056027</v>
       </c>
       <c r="R12" t="n">
         <v>92</v>
       </c>
       <c r="S12" t="n">
-        <v>-141.446519524618</v>
+        <v>-150.7843803056027</v>
       </c>
       <c r="T12" s="135" t="n">
         <v>177.4193548387097</v>
       </c>
       <c r="U12" s="135" t="n">
-        <v>4435.483870967741</v>
+        <v>4612.903225806452</v>
       </c>
       <c r="V12" s="135" t="n">
-        <v>4374.49</v>
+        <v>4548.58</v>
       </c>
       <c r="W12" s="135" t="n">
-        <v>-60.99387096774171</v>
+        <v>-64.32322580645177</v>
       </c>
       <c r="X12" s="136" t="n">
-        <v>-0.0137513454545454</v>
+        <v>-0.0139441958041958</v>
       </c>
       <c r="Y12" s="135" t="n">
-        <v>47.54880434782608</v>
+        <v>49.44108695652174</v>
       </c>
       <c r="Z12" s="135" t="n">
-        <v>28.54880434782608</v>
+        <v>30.44108695652174</v>
       </c>
       <c r="AB12" s="137" t="inlineStr"/>
       <c r="AC12" s="137" t="inlineStr">
@@ -3724,13 +3724,13 @@
         </is>
       </c>
       <c r="B13" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C13" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D13" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
@@ -3777,34 +3777,34 @@
         <v>0.5376344086021506</v>
       </c>
       <c r="Q13" t="n">
-        <v>13.44086021505377</v>
+        <v>13.97849462365592</v>
       </c>
       <c r="R13" t="n">
         <v>7</v>
       </c>
       <c r="S13" t="n">
-        <v>-6.440860215053766</v>
+        <v>-6.978494623655916</v>
       </c>
       <c r="T13" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U13" s="135" t="n">
-        <v>403.2258064516129</v>
+        <v>419.3548387096774</v>
       </c>
       <c r="V13" s="135" t="n">
-        <v>257.34</v>
+        <v>273.62</v>
       </c>
       <c r="W13" s="135" t="n">
-        <v>-145.885806451613</v>
+        <v>-145.7348387096774</v>
       </c>
       <c r="X13" s="136" t="n">
-        <v>-0.3617968000000001</v>
+        <v>-0.3475215384615385</v>
       </c>
       <c r="Y13" s="135" t="n">
-        <v>36.76285714285714</v>
+        <v>39.08857142857143</v>
       </c>
       <c r="Z13" s="135" t="n">
-        <v>6.762857142857136</v>
+        <v>9.088571428571427</v>
       </c>
       <c r="AB13" s="137" t="inlineStr"/>
       <c r="AC13" s="137" t="inlineStr">
@@ -3831,13 +3831,13 @@
         </is>
       </c>
       <c r="B14" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C14" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D14" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E14" t="n">
         <v>13</v>
@@ -3881,28 +3881,28 @@
         <v>0.1792114695340501</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.480286738351254</v>
+        <v>4.659498207885305</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>-4.480286738351254</v>
+        <v>-4.659498207885305</v>
       </c>
       <c r="T14" s="135" t="n">
         <v>16.12903225806452</v>
       </c>
       <c r="U14" s="135" t="n">
-        <v>403.2258064516129</v>
+        <v>419.3548387096774</v>
       </c>
       <c r="V14" s="135" t="n">
-        <v>253.32</v>
+        <v>267.62</v>
       </c>
       <c r="W14" s="135" t="n">
-        <v>-149.9058064516129</v>
+        <v>-151.7348387096774</v>
       </c>
       <c r="X14" s="136" t="n">
-        <v>-0.3717664</v>
+        <v>-0.3618292307692308</v>
       </c>
       <c r="Y14" s="135" t="n"/>
       <c r="Z14" s="135" t="n"/>
@@ -3931,13 +3931,13 @@
         </is>
       </c>
       <c r="B15" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C15" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D15" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
@@ -3984,34 +3984,34 @@
         <v>4.032258064516129</v>
       </c>
       <c r="Q15" t="n">
-        <v>100.8064516129032</v>
+        <v>104.8387096774194</v>
       </c>
       <c r="R15" t="n">
         <v>19</v>
       </c>
       <c r="S15" t="n">
-        <v>-81.80645161290323</v>
+        <v>-85.83870967741936</v>
       </c>
       <c r="T15" s="135" t="n">
         <v>48.38709677419355</v>
       </c>
       <c r="U15" s="135" t="n">
-        <v>1209.677419354839</v>
+        <v>1258.064516129032</v>
       </c>
       <c r="V15" s="135" t="n">
-        <v>1118.466974</v>
+        <v>1157.024833</v>
       </c>
       <c r="W15" s="135" t="n">
-        <v>-91.21044535483884</v>
+        <v>-101.0396831290325</v>
       </c>
       <c r="X15" s="136" t="n">
-        <v>-0.0754006348266667</v>
+        <v>-0.0803135942820514</v>
       </c>
       <c r="Y15" s="135" t="n">
-        <v>58.86668284210526</v>
+        <v>60.89604384210526</v>
       </c>
       <c r="Z15" s="135" t="n">
-        <v>46.86668284210526</v>
+        <v>48.89604384210526</v>
       </c>
       <c r="AB15" s="137" t="inlineStr">
         <is>
@@ -4038,13 +4038,13 @@
         </is>
       </c>
       <c r="B16" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C16" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D16" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="E16" t="n">
         <v>14</v>
@@ -4086,34 +4086,34 @@
         <v>1.402524544179523</v>
       </c>
       <c r="Q16" t="n">
-        <v>35.06311360448808</v>
+        <v>36.4656381486676</v>
       </c>
       <c r="R16" t="n">
         <v>3</v>
       </c>
       <c r="S16" t="n">
-        <v>-32.06311360448808</v>
+        <v>-33.4656381486676</v>
       </c>
       <c r="T16" s="135" t="n">
         <v>32.25806451612903</v>
       </c>
       <c r="U16" s="135" t="n">
-        <v>806.4516129032259</v>
+        <v>838.7096774193549</v>
       </c>
       <c r="V16" s="135" t="n">
-        <v>742.35</v>
+        <v>772.61</v>
       </c>
       <c r="W16" s="135" t="n">
-        <v>-64.10161290322583</v>
+        <v>-66.09967741935486</v>
       </c>
       <c r="X16" s="136" t="n">
-        <v>-0.079486</v>
+        <v>-0.07881115384615379</v>
       </c>
       <c r="Y16" s="135" t="n">
-        <v>247.45</v>
+        <v>257.5366666666667</v>
       </c>
       <c r="Z16" s="135" t="n">
-        <v>224.45</v>
+        <v>234.5366666666667</v>
       </c>
       <c r="AB16" s="137" t="inlineStr"/>
       <c r="AC16" s="137" t="inlineStr">
@@ -4140,13 +4140,13 @@
         </is>
       </c>
       <c r="B17" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C17" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D17" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -4180,34 +4180,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="Q17" t="n">
-        <v>346.9617404351088</v>
+        <v>360.8402100525131</v>
       </c>
       <c r="R17" t="n">
         <v>116</v>
       </c>
       <c r="S17" t="n">
-        <v>-230.9617404351088</v>
+        <v>-244.8402100525131</v>
       </c>
       <c r="T17" s="135" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="U17" s="135" t="n">
-        <v>14919.35483870968</v>
+        <v>15516.12903225806</v>
       </c>
       <c r="V17" s="135" t="n">
-        <v>14420.140469</v>
+        <v>15030.55877</v>
       </c>
       <c r="W17" s="135" t="n">
-        <v>-499.2143697096781</v>
+        <v>-485.5702622580648</v>
       </c>
       <c r="X17" s="136" t="n">
-        <v>-0.0334608550508108</v>
+        <v>-0.0312945491268191</v>
       </c>
       <c r="Y17" s="135" t="n">
-        <v>124.3115557672414</v>
+        <v>129.5737825</v>
       </c>
       <c r="Z17" s="135" t="n">
-        <v>81.31155576724137</v>
+        <v>86.57378249999999</v>
       </c>
       <c r="AB17" s="137" t="inlineStr"/>
       <c r="AC17" s="137" t="inlineStr"/>
@@ -4225,13 +4225,13 @@
         </is>
       </c>
       <c r="B18" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C18" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D18" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -4265,34 +4265,34 @@
         <v>21.43690626122104</v>
       </c>
       <c r="Q18" t="n">
-        <v>535.9226565305261</v>
+        <v>557.3595627917472</v>
       </c>
       <c r="R18" t="n">
         <v>166</v>
       </c>
       <c r="S18" t="n">
-        <v>-369.9226565305261</v>
+        <v>-391.3595627917472</v>
       </c>
       <c r="T18" s="135" t="n">
         <v>516.1290322580645</v>
       </c>
       <c r="U18" s="135" t="n">
-        <v>12903.22580645161</v>
+        <v>13419.35483870968</v>
       </c>
       <c r="V18" s="135" t="n">
-        <v>12098.098764</v>
+        <v>12564.134372</v>
       </c>
       <c r="W18" s="135" t="n">
-        <v>-805.1270424516133</v>
+        <v>-855.2204667096776</v>
       </c>
       <c r="X18" s="136" t="n">
-        <v>-0.06239734579</v>
+        <v>-0.0637303713173077</v>
       </c>
       <c r="Y18" s="135" t="n">
-        <v>72.88011303614458</v>
+        <v>75.68755645783133</v>
       </c>
       <c r="Z18" s="135" t="n">
-        <v>48.80345635962908</v>
+        <v>51.61089978131584</v>
       </c>
       <c r="AB18" s="137" t="inlineStr"/>
       <c r="AC18" s="137" t="inlineStr"/>
@@ -4310,13 +4310,13 @@
         </is>
       </c>
       <c r="B19" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C19" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D19" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -4350,28 +4350,28 @@
         <v>50.02088554720134</v>
       </c>
       <c r="Q19" t="n">
-        <v>850.3550543024228</v>
+        <v>900.375939849624</v>
       </c>
       <c r="R19" t="n">
         <v>198</v>
       </c>
       <c r="S19" t="n">
-        <v>-652.3550543024228</v>
+        <v>-702.375939849624</v>
       </c>
       <c r="T19" s="135" t="n">
         <v>404.7619047619048</v>
       </c>
       <c r="U19" s="135" t="n">
-        <v>6880.952380952381</v>
+        <v>7285.714285714285</v>
       </c>
       <c r="V19" s="135" t="n">
         <v>1606.8</v>
       </c>
       <c r="W19" s="135" t="n">
-        <v>-5274.152380952381</v>
+        <v>-5678.914285714285</v>
       </c>
       <c r="X19" s="136" t="n">
-        <v>-0.7664858131487889</v>
+        <v>-0.7794588235294118</v>
       </c>
       <c r="Y19" s="135" t="n">
         <v>8.115151515151515</v>
@@ -4395,13 +4395,13 @@
         </is>
       </c>
       <c r="B20" s="134" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="C20" s="134" t="n">
         <v>46235</v>
       </c>
       <c r="D20" s="134" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -4435,34 +4435,34 @@
         <v>85.33626142582673</v>
       </c>
       <c r="Q20" t="n">
-        <v>1733.239451268058</v>
+        <v>1818.575712693884</v>
       </c>
       <c r="R20" t="n">
         <v>480</v>
       </c>
       <c r="S20" t="n">
-        <v>-1253.239451268058</v>
+        <v>-1338.575712693884</v>
       </c>
       <c r="T20" s="135" t="n">
         <v>1517.665130568356</v>
       </c>
       <c r="U20" s="135" t="n">
-        <v>34703.53302611367</v>
+        <v>36221.19815668203</v>
       </c>
       <c r="V20" s="135" t="n">
-        <v>28125.039233</v>
+        <v>29201.493142</v>
       </c>
       <c r="W20" s="135" t="n">
-        <v>-6578.49379311367</v>
+        <v>-7019.705014682026</v>
       </c>
       <c r="X20" s="136" t="n">
-        <v>-0.1895626531213261</v>
+        <v>-0.1938010163086513</v>
       </c>
       <c r="Y20" s="135" t="n">
-        <v>58.59383173541666</v>
+        <v>60.83644404583333</v>
       </c>
       <c r="Z20" s="135" t="n">
-        <v>38.54922314637908</v>
+        <v>40.79183545679575</v>
       </c>
       <c r="AB20" s="137" t="inlineStr"/>
       <c r="AC20" s="137" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
         </is>
       </c>
       <c r="B4" s="138" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="D4" s="33" t="inlineStr">
         <is>
@@ -4605,7 +4605,7 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -4625,7 +4625,7 @@
         </is>
       </c>
       <c r="B7" s="139" t="n">
-        <v>46260.29199074074</v>
+        <v>46261.2919212963</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Aggiornamento dati Dynamica 2026-08-28
</commit_message>
<xml_diff>
--- a/exports/report_dynamica_updated.xlsx
+++ b/exports/report_dynamica_updated.xlsx
@@ -872,7 +872,7 @@
     <row r="2" ht="22" customHeight="1" s="74">
       <c r="A2" s="114" t="inlineStr">
         <is>
-          <t>Periodo: 01/08/2026 - 26/08/2026  |  Ultimo aggiornamento: 27/08/2026 07:00</t>
+          <t>Periodo: 01/08/2026 - 27/08/2026  |  Ultimo aggiornamento: 28/08/2026 07:00</t>
         </is>
       </c>
       <c r="B2" s="113" t="n"/>
@@ -1059,16 +1059,16 @@
         <v>258.0645161290323</v>
       </c>
       <c r="Q5" s="117" t="n">
-        <v>6709.677419354839</v>
+        <v>6967.741935483871</v>
       </c>
       <c r="R5" s="117" t="n">
-        <v>6829.212182</v>
+        <v>7081.263787</v>
       </c>
       <c r="S5" s="117" t="n">
-        <v>119.5347626451612</v>
+        <v>113.5218515161287</v>
       </c>
       <c r="T5" s="118" t="n">
-        <v>0.0178152771249999</v>
+        <v>0.016292487949074</v>
       </c>
       <c r="U5" s="117" t="n"/>
       <c r="V5" s="117" t="n"/>
@@ -1118,16 +1118,16 @@
         <v>32.25806451612903</v>
       </c>
       <c r="Q6" s="117" t="n">
-        <v>838.7096774193549</v>
+        <v>870.9677419354839</v>
       </c>
       <c r="R6" s="117" t="n">
-        <v>827.4065880000001</v>
+        <v>850.676588</v>
       </c>
       <c r="S6" s="117" t="n">
-        <v>-11.30308941935482</v>
+        <v>-20.29115393548386</v>
       </c>
       <c r="T6" s="118" t="n">
-        <v>-0.0134767604615384</v>
+        <v>-0.0232972508148148</v>
       </c>
       <c r="U6" s="117" t="n"/>
       <c r="V6" s="117" t="n"/>
@@ -1177,16 +1177,16 @@
         <v>306.4516129032258</v>
       </c>
       <c r="Q7" s="117" t="n">
-        <v>7967.74193548387</v>
+        <v>8274.193548387097</v>
       </c>
       <c r="R7" s="117" t="n">
-        <v>7373.94</v>
+        <v>7663.14</v>
       </c>
       <c r="S7" s="117" t="n">
-        <v>-593.8019354838707</v>
+        <v>-611.0535483870963</v>
       </c>
       <c r="T7" s="118" t="n">
-        <v>-0.0745257489878542</v>
+        <v>-0.07385052631578939</v>
       </c>
       <c r="U7" s="117" t="n"/>
       <c r="V7" s="117" t="n"/>
@@ -1224,34 +1224,34 @@
         <v>13.87846961740435</v>
       </c>
       <c r="M8" s="125" t="n">
-        <v>360.8402100525131</v>
+        <v>374.7186796699175</v>
       </c>
       <c r="N8" s="125" t="n">
         <v>116</v>
       </c>
       <c r="O8" s="125" t="n">
-        <v>-244.8402100525131</v>
+        <v>-258.7186796699175</v>
       </c>
       <c r="P8" s="123" t="n">
         <v>596.7741935483871</v>
       </c>
       <c r="Q8" s="123" t="n">
-        <v>15516.12903225806</v>
+        <v>16112.90322580645</v>
       </c>
       <c r="R8" s="123" t="n">
-        <v>15030.55877</v>
+        <v>15595.080375</v>
       </c>
       <c r="S8" s="123" t="n">
-        <v>-485.5702622580648</v>
+        <v>-517.8228508064512</v>
       </c>
       <c r="T8" s="124" t="n">
-        <v>-0.0312945491268191</v>
+        <v>-0.0321371539039038</v>
       </c>
       <c r="U8" s="123" t="n">
-        <v>129.5737825</v>
+        <v>134.4403480603448</v>
       </c>
       <c r="V8" s="123" t="n">
-        <v>86.57378249999999</v>
+        <v>91.44034806034485</v>
       </c>
       <c r="W8" s="126" t="n"/>
     </row>
@@ -1303,34 +1303,34 @@
         <v>2.081165452653486</v>
       </c>
       <c r="M9" s="119" t="n">
-        <v>54.11030176899063</v>
+        <v>56.19146722164412</v>
       </c>
       <c r="N9" s="119" t="n">
         <v>22</v>
       </c>
       <c r="O9" s="119" t="n">
-        <v>-32.11030176899063</v>
+        <v>-34.19146722164412</v>
       </c>
       <c r="P9" s="117" t="n">
         <v>64.51612903225806</v>
       </c>
       <c r="Q9" s="117" t="n">
-        <v>1677.41935483871</v>
+        <v>1741.935483870968</v>
       </c>
       <c r="R9" s="117" t="n">
-        <v>1587.540775</v>
+        <v>1634.430434</v>
       </c>
       <c r="S9" s="117" t="n">
-        <v>-89.87857983870981</v>
+        <v>-107.5050498709677</v>
       </c>
       <c r="T9" s="118" t="n">
-        <v>-0.0535814610576923</v>
+        <v>-0.0617158619629629</v>
       </c>
       <c r="U9" s="117" t="n">
-        <v>72.16094431818182</v>